<commit_message>
Atualização automática: reparaveis (10/07/2026 18:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2250,7 +2250,7 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -3114,7 +3114,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -3178,7 +3178,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -3238,7 +3238,7 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -3304,7 +3304,7 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -3414,7 +3414,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3592,7 +3592,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -4150,7 +4150,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -4216,7 +4216,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -4568,7 +4568,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -4860,7 +4860,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -5092,7 +5092,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -5266,7 +5266,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -5568,7 +5568,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -5920,7 +5920,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -5980,7 +5980,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
@@ -6040,7 +6040,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -6100,7 +6100,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -6166,7 +6166,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="I104" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
@@ -6670,7 +6670,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -6732,7 +6732,7 @@
         </is>
       </c>
       <c r="I107" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J107" t="inlineStr">
         <is>
@@ -6794,7 +6794,7 @@
         </is>
       </c>
       <c r="I108" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -6854,7 +6854,7 @@
         </is>
       </c>
       <c r="I109" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -7196,7 +7196,7 @@
         </is>
       </c>
       <c r="I115" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -7256,7 +7256,7 @@
         </is>
       </c>
       <c r="I116" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J116" t="inlineStr">
         <is>
@@ -7316,7 +7316,7 @@
         </is>
       </c>
       <c r="I117" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J117" t="inlineStr">
         <is>
@@ -7376,7 +7376,7 @@
         </is>
       </c>
       <c r="I118" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -7436,7 +7436,7 @@
         </is>
       </c>
       <c r="I119" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
@@ -7496,7 +7496,7 @@
         </is>
       </c>
       <c r="I120" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -7556,7 +7556,7 @@
         </is>
       </c>
       <c r="I121" t="n">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -7620,7 +7620,7 @@
         </is>
       </c>
       <c r="I122" t="n">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="I124" t="n">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -7790,7 +7790,7 @@
         </is>
       </c>
       <c r="I125" t="n">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
         </is>
       </c>
       <c r="I128" t="n">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -8018,7 +8018,7 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -8078,7 +8078,7 @@
         </is>
       </c>
       <c r="I130" t="n">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -8200,7 +8200,7 @@
         </is>
       </c>
       <c r="I132" t="n">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="J132" t="inlineStr">
         <is>
@@ -8314,7 +8314,7 @@
         </is>
       </c>
       <c r="I134" t="n">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="J134" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
         </is>
       </c>
       <c r="I138" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J138" t="inlineStr">
         <is>
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="I148" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
@@ -9118,7 +9118,7 @@
         </is>
       </c>
       <c r="I149" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J149" t="inlineStr">
         <is>
@@ -9174,7 +9174,7 @@
         </is>
       </c>
       <c r="I150" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
         </is>
       </c>
       <c r="I152" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J152" t="inlineStr">
         <is>
@@ -9360,7 +9360,7 @@
         </is>
       </c>
       <c r="I153" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
@@ -9478,7 +9478,7 @@
         </is>
       </c>
       <c r="I155" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J155" t="inlineStr">
         <is>
@@ -9534,7 +9534,7 @@
         </is>
       </c>
       <c r="I156" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J156" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
         </is>
       </c>
       <c r="I157" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J157" t="inlineStr">
         <is>
@@ -9654,7 +9654,7 @@
         </is>
       </c>
       <c r="I158" t="n">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="J158" t="inlineStr">
         <is>
@@ -9716,7 +9716,7 @@
         </is>
       </c>
       <c r="I159" t="n">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="J159" t="inlineStr">
         <is>
@@ -9776,7 +9776,7 @@
         </is>
       </c>
       <c r="I160" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="J160" t="inlineStr">
         <is>
@@ -9836,7 +9836,7 @@
         </is>
       </c>
       <c r="I161" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="J161" t="inlineStr">
         <is>
@@ -9902,7 +9902,7 @@
         </is>
       </c>
       <c r="I162" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="J162" t="inlineStr">
         <is>
@@ -9964,7 +9964,7 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="J163" t="inlineStr">
         <is>
@@ -10026,7 +10026,7 @@
         </is>
       </c>
       <c r="I164" t="n">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="J164" t="inlineStr">
         <is>
@@ -10082,7 +10082,7 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J165" t="inlineStr">
         <is>
@@ -10250,7 +10250,7 @@
         </is>
       </c>
       <c r="I168" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J168" t="inlineStr">
         <is>
@@ -10314,7 +10314,7 @@
         </is>
       </c>
       <c r="I169" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>
@@ -10434,7 +10434,7 @@
         </is>
       </c>
       <c r="I171" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J171" t="inlineStr">
         <is>
@@ -10668,7 +10668,7 @@
         </is>
       </c>
       <c r="I175" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
@@ -10734,7 +10734,7 @@
         </is>
       </c>
       <c r="I176" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J176" t="inlineStr">
         <is>
@@ -10794,7 +10794,7 @@
         </is>
       </c>
       <c r="I177" t="n">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
         </is>
       </c>
       <c r="I178" t="n">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
@@ -10970,7 +10970,7 @@
         </is>
       </c>
       <c r="I180" t="n">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
@@ -11138,7 +11138,7 @@
         </is>
       </c>
       <c r="I183" t="n">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="I184" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
@@ -11250,7 +11250,7 @@
         </is>
       </c>
       <c r="I185" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="I186" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
@@ -11370,7 +11370,7 @@
         </is>
       </c>
       <c r="I187" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
@@ -11434,7 +11434,7 @@
         </is>
       </c>
       <c r="I188" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -11500,7 +11500,7 @@
         </is>
       </c>
       <c r="I189" t="n">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
@@ -11562,7 +11562,7 @@
         </is>
       </c>
       <c r="I190" t="n">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
@@ -11622,7 +11622,7 @@
         </is>
       </c>
       <c r="I191" t="n">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
@@ -11684,7 +11684,7 @@
         </is>
       </c>
       <c r="I192" t="n">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
@@ -11744,7 +11744,7 @@
         </is>
       </c>
       <c r="I193" t="n">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="I195" t="n">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="I199" t="n">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
@@ -12126,7 +12126,7 @@
         </is>
       </c>
       <c r="I200" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J200" t="inlineStr">
         <is>
@@ -12186,7 +12186,7 @@
         </is>
       </c>
       <c r="I201" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J201" t="inlineStr">
         <is>
@@ -12246,7 +12246,7 @@
         </is>
       </c>
       <c r="I202" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J202" t="inlineStr">
         <is>
@@ -12306,7 +12306,7 @@
         </is>
       </c>
       <c r="I203" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J203" t="inlineStr">
         <is>
@@ -12366,7 +12366,7 @@
         </is>
       </c>
       <c r="I204" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J204" t="inlineStr">
         <is>
@@ -12426,7 +12426,7 @@
         </is>
       </c>
       <c r="I205" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J205" t="inlineStr">
         <is>
@@ -12544,7 +12544,7 @@
         </is>
       </c>
       <c r="I207" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J207" t="inlineStr">
         <is>
@@ -12606,7 +12606,7 @@
         </is>
       </c>
       <c r="I208" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="J208" t="inlineStr">
         <is>
@@ -12668,7 +12668,7 @@
         </is>
       </c>
       <c r="I209" t="n">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="J209" t="inlineStr">
         <is>
@@ -12730,7 +12730,7 @@
         </is>
       </c>
       <c r="I210" t="n">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="J210" t="inlineStr">
         <is>
@@ -12906,7 +12906,7 @@
         </is>
       </c>
       <c r="I213" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="J213" t="inlineStr">
         <is>
@@ -12966,7 +12966,7 @@
         </is>
       </c>
       <c r="I214" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="J214" t="inlineStr">
         <is>
@@ -13030,7 +13030,7 @@
         </is>
       </c>
       <c r="I215" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="J215" t="inlineStr">
         <is>
@@ -13140,7 +13140,7 @@
         </is>
       </c>
       <c r="I217" t="n">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="J217" t="inlineStr">
         <is>
@@ -13202,7 +13202,7 @@
         </is>
       </c>
       <c r="I218" t="n">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="J218" t="inlineStr">
         <is>
@@ -13262,7 +13262,7 @@
         </is>
       </c>
       <c r="I219" t="n">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="J219" t="inlineStr">
         <is>
@@ -13322,7 +13322,7 @@
         </is>
       </c>
       <c r="I220" t="n">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="J220" t="inlineStr">
         <is>
@@ -13440,7 +13440,7 @@
         </is>
       </c>
       <c r="I222" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J222" t="inlineStr">
         <is>
@@ -13500,7 +13500,7 @@
         </is>
       </c>
       <c r="I223" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J223" t="inlineStr">
         <is>
@@ -13560,7 +13560,7 @@
         </is>
       </c>
       <c r="I224" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J224" t="inlineStr">
         <is>
@@ -13620,7 +13620,7 @@
         </is>
       </c>
       <c r="I225" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J225" t="inlineStr">
         <is>
@@ -13680,7 +13680,7 @@
         </is>
       </c>
       <c r="I226" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J226" t="inlineStr">
         <is>
@@ -13740,7 +13740,7 @@
         </is>
       </c>
       <c r="I227" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J227" t="inlineStr">
         <is>
@@ -13800,7 +13800,7 @@
         </is>
       </c>
       <c r="I228" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
@@ -13918,7 +13918,7 @@
         </is>
       </c>
       <c r="I230" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J230" t="inlineStr">
         <is>
@@ -13978,7 +13978,7 @@
         </is>
       </c>
       <c r="I231" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J231" t="inlineStr">
         <is>
@@ -14156,7 +14156,7 @@
         </is>
       </c>
       <c r="I234" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
@@ -14222,7 +14222,7 @@
         </is>
       </c>
       <c r="I235" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J235" t="inlineStr">
         <is>
@@ -14288,7 +14288,7 @@
         </is>
       </c>
       <c r="I236" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J236" t="inlineStr">
         <is>
@@ -14350,7 +14350,7 @@
         </is>
       </c>
       <c r="I237" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
@@ -14460,7 +14460,7 @@
         </is>
       </c>
       <c r="I239" t="n">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="J239" t="inlineStr">
         <is>
@@ -14638,7 +14638,7 @@
         </is>
       </c>
       <c r="I242" t="n">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="J242" t="inlineStr">
         <is>
@@ -14752,7 +14752,7 @@
         </is>
       </c>
       <c r="I244" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="J244" t="inlineStr">
         <is>
@@ -14812,7 +14812,7 @@
         </is>
       </c>
       <c r="I245" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="J245" t="inlineStr">
         <is>
@@ -14872,7 +14872,7 @@
         </is>
       </c>
       <c r="I246" t="n">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="I249" t="n">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="J249" t="inlineStr">
         <is>
@@ -15094,7 +15094,7 @@
         </is>
       </c>
       <c r="I250" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J250" t="inlineStr">
         <is>
@@ -15270,7 +15270,7 @@
         </is>
       </c>
       <c r="I253" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J253" t="inlineStr">
         <is>
@@ -15330,7 +15330,7 @@
         </is>
       </c>
       <c r="I254" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J254" t="inlineStr">
         <is>
@@ -15390,7 +15390,7 @@
         </is>
       </c>
       <c r="I255" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J255" t="inlineStr">
         <is>
@@ -15450,7 +15450,7 @@
         </is>
       </c>
       <c r="I256" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J256" t="inlineStr">
         <is>
@@ -15612,7 +15612,7 @@
         </is>
       </c>
       <c r="I259" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J259" t="inlineStr">
         <is>
@@ -15672,7 +15672,7 @@
         </is>
       </c>
       <c r="I260" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J260" t="inlineStr">
         <is>
@@ -15732,7 +15732,7 @@
         </is>
       </c>
       <c r="I261" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J261" t="inlineStr">
         <is>
@@ -15792,7 +15792,7 @@
         </is>
       </c>
       <c r="I262" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J262" t="inlineStr">
         <is>
@@ -15916,7 +15916,7 @@
         </is>
       </c>
       <c r="I264" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J264" t="inlineStr">
         <is>
@@ -15976,7 +15976,7 @@
         </is>
       </c>
       <c r="I265" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J265" t="inlineStr">
         <is>
@@ -16036,7 +16036,7 @@
         </is>
       </c>
       <c r="I266" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J266" t="inlineStr">
         <is>
@@ -16096,7 +16096,7 @@
         </is>
       </c>
       <c r="I267" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J267" t="inlineStr">
         <is>
@@ -16156,7 +16156,7 @@
         </is>
       </c>
       <c r="I268" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J268" t="inlineStr">
         <is>
@@ -16212,7 +16212,7 @@
         </is>
       </c>
       <c r="I269" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J269" t="inlineStr">
         <is>
@@ -16272,7 +16272,7 @@
         </is>
       </c>
       <c r="I270" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J270" t="inlineStr">
         <is>
@@ -16332,7 +16332,7 @@
         </is>
       </c>
       <c r="I271" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J271" t="inlineStr">
         <is>
@@ -16392,7 +16392,7 @@
         </is>
       </c>
       <c r="I272" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J272" t="inlineStr">
         <is>
@@ -16516,7 +16516,7 @@
         </is>
       </c>
       <c r="I274" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J274" t="inlineStr">
         <is>
@@ -16634,7 +16634,7 @@
         </is>
       </c>
       <c r="I276" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J276" t="inlineStr">
         <is>
@@ -16694,7 +16694,7 @@
         </is>
       </c>
       <c r="I277" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="J277" t="inlineStr">
         <is>
@@ -16754,7 +16754,7 @@
         </is>
       </c>
       <c r="I278" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="J278" t="inlineStr">
         <is>
@@ -16814,7 +16814,7 @@
         </is>
       </c>
       <c r="I279" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="J279" t="inlineStr">
         <is>
@@ -16878,7 +16878,7 @@
         </is>
       </c>
       <c r="I280" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="J280" t="inlineStr">
         <is>
@@ -16938,7 +16938,7 @@
         </is>
       </c>
       <c r="I281" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="J281" t="inlineStr">
         <is>
@@ -16998,7 +16998,7 @@
         </is>
       </c>
       <c r="I282" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="J282" t="inlineStr">
         <is>
@@ -17324,7 +17324,7 @@
         </is>
       </c>
       <c r="I288" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J288" t="inlineStr">
         <is>
@@ -17428,7 +17428,7 @@
         </is>
       </c>
       <c r="I290" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J290" t="inlineStr">
         <is>
@@ -17482,7 +17482,7 @@
         </is>
       </c>
       <c r="I291" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J291" t="inlineStr">
         <is>
@@ -17540,7 +17540,7 @@
         </is>
       </c>
       <c r="I292" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J292" t="inlineStr">
         <is>
@@ -17598,7 +17598,7 @@
         </is>
       </c>
       <c r="I293" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J293" t="inlineStr">
         <is>
@@ -17656,7 +17656,7 @@
         </is>
       </c>
       <c r="I294" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J294" t="inlineStr">
         <is>
@@ -17710,7 +17710,7 @@
         </is>
       </c>
       <c r="I295" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J295" t="inlineStr">
         <is>
@@ -17764,7 +17764,7 @@
         </is>
       </c>
       <c r="I296" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J296" t="inlineStr">
         <is>
@@ -17818,7 +17818,7 @@
         </is>
       </c>
       <c r="I297" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J297" t="inlineStr">
         <is>
@@ -17876,7 +17876,7 @@
         </is>
       </c>
       <c r="I298" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J298" t="inlineStr">
         <is>
@@ -17934,7 +17934,7 @@
         </is>
       </c>
       <c r="I299" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J299" t="inlineStr">
         <is>
@@ -17992,7 +17992,7 @@
         </is>
       </c>
       <c r="I300" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J300" t="inlineStr">
         <is>
@@ -18050,7 +18050,7 @@
         </is>
       </c>
       <c r="I301" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J301" t="inlineStr">
         <is>
@@ -18106,7 +18106,7 @@
         </is>
       </c>
       <c r="I302" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J302" t="inlineStr">
         <is>
@@ -18162,7 +18162,7 @@
         </is>
       </c>
       <c r="I303" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J303" t="inlineStr">
         <is>
@@ -18218,7 +18218,7 @@
         </is>
       </c>
       <c r="I304" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J304" t="inlineStr">
         <is>
@@ -18274,7 +18274,7 @@
         </is>
       </c>
       <c r="I305" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J305" t="inlineStr">
         <is>
@@ -18332,7 +18332,7 @@
         </is>
       </c>
       <c r="I306" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J306" t="inlineStr">
         <is>
@@ -18390,7 +18390,7 @@
         </is>
       </c>
       <c r="I307" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J307" t="inlineStr">
         <is>
@@ -18446,7 +18446,7 @@
         </is>
       </c>
       <c r="I308" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J308" t="inlineStr">
         <is>
@@ -18502,7 +18502,7 @@
         </is>
       </c>
       <c r="I309" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J309" t="inlineStr">
         <is>
@@ -18560,7 +18560,7 @@
         </is>
       </c>
       <c r="I310" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J310" t="inlineStr">
         <is>
@@ -18616,7 +18616,7 @@
         </is>
       </c>
       <c r="I311" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J311" t="inlineStr">
         <is>
@@ -18674,7 +18674,7 @@
         </is>
       </c>
       <c r="I312" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J312" t="inlineStr">
         <is>
@@ -18784,7 +18784,7 @@
         </is>
       </c>
       <c r="I314" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J314" t="inlineStr">
         <is>
@@ -18840,7 +18840,7 @@
         </is>
       </c>
       <c r="I315" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J315" t="inlineStr">
         <is>
@@ -18896,7 +18896,7 @@
         </is>
       </c>
       <c r="I316" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J316" t="inlineStr">
         <is>
@@ -18954,7 +18954,7 @@
         </is>
       </c>
       <c r="I317" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J317" t="inlineStr">
         <is>
@@ -19116,7 +19116,7 @@
         </is>
       </c>
       <c r="I320" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J320" t="inlineStr">
         <is>
@@ -19174,7 +19174,7 @@
         </is>
       </c>
       <c r="I321" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J321" t="inlineStr">
         <is>
@@ -19234,7 +19234,7 @@
         </is>
       </c>
       <c r="I322" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J322" t="inlineStr">
         <is>
@@ -19294,7 +19294,7 @@
         </is>
       </c>
       <c r="I323" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J323" t="inlineStr">
         <is>
@@ -19352,7 +19352,7 @@
         </is>
       </c>
       <c r="I324" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J324" t="inlineStr">
         <is>
@@ -19410,7 +19410,7 @@
         </is>
       </c>
       <c r="I325" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J325" t="inlineStr">
         <is>
@@ -19470,7 +19470,7 @@
         </is>
       </c>
       <c r="I326" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J326" t="inlineStr">
         <is>
@@ -19530,7 +19530,7 @@
         </is>
       </c>
       <c r="I327" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J327" t="inlineStr">
         <is>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="I328" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J328" t="inlineStr">
         <is>
@@ -19650,7 +19650,7 @@
         </is>
       </c>
       <c r="I329" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J329" t="inlineStr">
         <is>
@@ -19710,7 +19710,7 @@
         </is>
       </c>
       <c r="I330" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J330" t="inlineStr">
         <is>
@@ -19770,7 +19770,7 @@
         </is>
       </c>
       <c r="I331" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J331" t="inlineStr">
         <is>
@@ -19828,7 +19828,7 @@
         </is>
       </c>
       <c r="I332" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J332" t="inlineStr">
         <is>
@@ -19884,7 +19884,7 @@
         </is>
       </c>
       <c r="I333" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J333" t="inlineStr">
         <is>
@@ -19940,7 +19940,7 @@
         </is>
       </c>
       <c r="I334" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J334" t="inlineStr">
         <is>
@@ -20060,7 +20060,7 @@
         </is>
       </c>
       <c r="I336" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="J336" t="inlineStr">
         <is>
@@ -20180,7 +20180,7 @@
         </is>
       </c>
       <c r="I338" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="J338" t="inlineStr">
         <is>
@@ -20286,7 +20286,7 @@
         </is>
       </c>
       <c r="I340" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J340" t="inlineStr">
         <is>
@@ -20346,7 +20346,7 @@
         </is>
       </c>
       <c r="I341" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J341" t="inlineStr">
         <is>
@@ -20406,7 +20406,7 @@
         </is>
       </c>
       <c r="I342" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J342" t="inlineStr">
         <is>
@@ -20466,7 +20466,7 @@
         </is>
       </c>
       <c r="I343" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J343" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         </is>
       </c>
       <c r="I344" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J344" t="inlineStr">
         <is>
@@ -20586,7 +20586,7 @@
         </is>
       </c>
       <c r="I345" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J345" t="inlineStr">
         <is>
@@ -20646,7 +20646,7 @@
         </is>
       </c>
       <c r="I346" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J346" t="inlineStr">
         <is>
@@ -20706,7 +20706,7 @@
         </is>
       </c>
       <c r="I347" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J347" t="inlineStr">
         <is>
@@ -20768,7 +20768,7 @@
         </is>
       </c>
       <c r="I348" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J348" t="inlineStr">
         <is>
@@ -20830,7 +20830,7 @@
         </is>
       </c>
       <c r="I349" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J349" t="inlineStr">
         <is>
@@ -20890,7 +20890,7 @@
         </is>
       </c>
       <c r="I350" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J350" t="inlineStr">
         <is>
@@ -20946,7 +20946,7 @@
         </is>
       </c>
       <c r="I351" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J351" t="inlineStr">
         <is>
@@ -21006,7 +21006,7 @@
         </is>
       </c>
       <c r="I352" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J352" t="inlineStr">
         <is>
@@ -21066,7 +21066,7 @@
         </is>
       </c>
       <c r="I353" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J353" t="inlineStr">
         <is>
@@ -21126,7 +21126,7 @@
         </is>
       </c>
       <c r="I354" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J354" t="inlineStr">
         <is>
@@ -21186,7 +21186,7 @@
         </is>
       </c>
       <c r="I355" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J355" t="inlineStr">
         <is>
@@ -21308,7 +21308,7 @@
         </is>
       </c>
       <c r="I357" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J357" t="inlineStr">
         <is>
@@ -21368,7 +21368,7 @@
         </is>
       </c>
       <c r="I358" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J358" t="inlineStr">
         <is>
@@ -21428,7 +21428,7 @@
         </is>
       </c>
       <c r="I359" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J359" t="inlineStr">
         <is>
@@ -21488,7 +21488,7 @@
         </is>
       </c>
       <c r="I360" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J360" t="inlineStr">
         <is>
@@ -21548,7 +21548,7 @@
         </is>
       </c>
       <c r="I361" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J361" t="inlineStr">
         <is>
@@ -21608,7 +21608,7 @@
         </is>
       </c>
       <c r="I362" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J362" t="inlineStr">
         <is>
@@ -21668,7 +21668,7 @@
         </is>
       </c>
       <c r="I363" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J363" t="inlineStr">
         <is>
@@ -21728,7 +21728,7 @@
         </is>
       </c>
       <c r="I364" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J364" t="inlineStr">
         <is>
@@ -21788,7 +21788,7 @@
         </is>
       </c>
       <c r="I365" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J365" t="inlineStr">
         <is>
@@ -21848,7 +21848,7 @@
         </is>
       </c>
       <c r="I366" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J366" t="inlineStr">
         <is>
@@ -21908,7 +21908,7 @@
         </is>
       </c>
       <c r="I367" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J367" t="inlineStr">
         <is>
@@ -21968,7 +21968,7 @@
         </is>
       </c>
       <c r="I368" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J368" t="inlineStr">
         <is>
@@ -22028,7 +22028,7 @@
         </is>
       </c>
       <c r="I369" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J369" t="inlineStr">
         <is>
@@ -22088,7 +22088,7 @@
         </is>
       </c>
       <c r="I370" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J370" t="inlineStr">
         <is>
@@ -22148,7 +22148,7 @@
         </is>
       </c>
       <c r="I371" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J371" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
         </is>
       </c>
       <c r="I372" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="J372" t="inlineStr">
         <is>
@@ -22276,7 +22276,7 @@
         </is>
       </c>
       <c r="I373" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="J373" t="inlineStr">
         <is>
@@ -22336,7 +22336,7 @@
         </is>
       </c>
       <c r="I374" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="J374" t="inlineStr">
         <is>
@@ -22396,7 +22396,7 @@
         </is>
       </c>
       <c r="I375" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J375" t="inlineStr">
         <is>
@@ -22456,7 +22456,7 @@
         </is>
       </c>
       <c r="I376" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J376" t="inlineStr">
         <is>
@@ -22516,7 +22516,7 @@
         </is>
       </c>
       <c r="I377" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J377" t="inlineStr">
         <is>
@@ -22531,7 +22531,11 @@
       </c>
       <c r="M377" t="inlineStr"/>
       <c r="N377" t="inlineStr"/>
-      <c r="O377" t="inlineStr"/>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>024/2026</t>
+        </is>
+      </c>
       <c r="P377" t="b">
         <v>1</v>
       </c>
@@ -22576,7 +22580,7 @@
         </is>
       </c>
       <c r="I378" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J378" t="inlineStr">
         <is>
@@ -22636,7 +22640,7 @@
         </is>
       </c>
       <c r="I379" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J379" t="inlineStr">
         <is>
@@ -22698,7 +22702,7 @@
         </is>
       </c>
       <c r="I380" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J380" t="inlineStr">
         <is>
@@ -22758,7 +22762,7 @@
         </is>
       </c>
       <c r="I381" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J381" t="inlineStr">
         <is>
@@ -22818,7 +22822,7 @@
         </is>
       </c>
       <c r="I382" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J382" t="inlineStr">
         <is>
@@ -22878,7 +22882,7 @@
         </is>
       </c>
       <c r="I383" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J383" t="inlineStr">
         <is>
@@ -22938,7 +22942,7 @@
         </is>
       </c>
       <c r="I384" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="J384" t="inlineStr">
         <is>
@@ -22998,7 +23002,7 @@
         </is>
       </c>
       <c r="I385" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="J385" t="inlineStr">
         <is>
@@ -23058,7 +23062,7 @@
         </is>
       </c>
       <c r="I386" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J386" t="inlineStr">
         <is>
@@ -23118,7 +23122,7 @@
         </is>
       </c>
       <c r="I387" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J387" t="inlineStr">
         <is>
@@ -23178,7 +23182,7 @@
         </is>
       </c>
       <c r="I388" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J388" t="inlineStr">
         <is>
@@ -23238,7 +23242,7 @@
         </is>
       </c>
       <c r="I389" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J389" t="inlineStr">
         <is>
@@ -23298,7 +23302,7 @@
         </is>
       </c>
       <c r="I390" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J390" t="inlineStr">
         <is>
@@ -23360,7 +23364,7 @@
         </is>
       </c>
       <c r="I391" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J391" t="inlineStr">
         <is>
@@ -23375,7 +23379,11 @@
       </c>
       <c r="M391" t="inlineStr"/>
       <c r="N391" t="inlineStr"/>
-      <c r="O391" t="inlineStr"/>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>015/2026</t>
+        </is>
+      </c>
       <c r="P391" t="b">
         <v>1</v>
       </c>
@@ -23480,7 +23488,7 @@
         </is>
       </c>
       <c r="I393" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J393" t="inlineStr">
         <is>
@@ -23540,7 +23548,7 @@
         </is>
       </c>
       <c r="I394" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J394" t="inlineStr">
         <is>
@@ -23600,7 +23608,7 @@
         </is>
       </c>
       <c r="I395" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J395" t="inlineStr">
         <is>
@@ -23660,7 +23668,7 @@
         </is>
       </c>
       <c r="I396" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J396" t="inlineStr">
         <is>
@@ -23720,7 +23728,7 @@
         </is>
       </c>
       <c r="I397" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J397" t="inlineStr">
         <is>
@@ -23780,7 +23788,7 @@
         </is>
       </c>
       <c r="I398" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J398" t="inlineStr">
         <is>
@@ -23900,7 +23908,7 @@
         </is>
       </c>
       <c r="I400" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J400" t="inlineStr">
         <is>
@@ -23960,7 +23968,7 @@
         </is>
       </c>
       <c r="I401" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J401" t="inlineStr">
         <is>
@@ -24020,7 +24028,7 @@
         </is>
       </c>
       <c r="I402" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J402" t="inlineStr">
         <is>
@@ -24080,7 +24088,7 @@
         </is>
       </c>
       <c r="I403" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J403" t="inlineStr">
         <is>
@@ -24136,7 +24144,7 @@
         </is>
       </c>
       <c r="I404" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J404" t="inlineStr">
         <is>
@@ -24188,7 +24196,7 @@
         </is>
       </c>
       <c r="I405" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J405" t="inlineStr"/>
       <c r="K405" t="inlineStr"/>
@@ -24236,7 +24244,7 @@
         </is>
       </c>
       <c r="I406" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J406" t="inlineStr"/>
       <c r="K406" t="inlineStr"/>
@@ -24284,7 +24292,7 @@
         </is>
       </c>
       <c r="I407" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J407" t="inlineStr"/>
       <c r="K407" t="inlineStr"/>
@@ -24332,7 +24340,7 @@
         </is>
       </c>
       <c r="I408" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J408" t="inlineStr"/>
       <c r="K408" t="inlineStr"/>
@@ -24380,7 +24388,7 @@
         </is>
       </c>
       <c r="I409" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J409" t="inlineStr"/>
       <c r="K409" t="inlineStr"/>
@@ -24428,7 +24436,7 @@
         </is>
       </c>
       <c r="I410" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J410" t="inlineStr"/>
       <c r="K410" t="inlineStr"/>
@@ -24480,7 +24488,7 @@
         </is>
       </c>
       <c r="I411" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J411" t="inlineStr"/>
       <c r="K411" t="inlineStr"/>
@@ -24532,7 +24540,7 @@
         </is>
       </c>
       <c r="I412" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J412" t="inlineStr"/>
       <c r="K412" t="inlineStr"/>
@@ -24584,7 +24592,7 @@
         </is>
       </c>
       <c r="I413" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J413" t="inlineStr"/>
       <c r="K413" t="inlineStr"/>
@@ -24636,7 +24644,7 @@
         </is>
       </c>
       <c r="I414" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J414" t="inlineStr"/>
       <c r="K414" t="inlineStr"/>
@@ -24686,7 +24694,7 @@
         </is>
       </c>
       <c r="I415" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J415" t="inlineStr"/>
       <c r="K415" t="inlineStr"/>
@@ -24736,7 +24744,7 @@
         </is>
       </c>
       <c r="I416" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J416" t="inlineStr"/>
       <c r="K416" t="inlineStr"/>
@@ -24786,7 +24794,7 @@
         </is>
       </c>
       <c r="I417" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J417" t="inlineStr"/>
       <c r="K417" t="inlineStr"/>
@@ -24836,7 +24844,7 @@
         </is>
       </c>
       <c r="I418" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J418" t="inlineStr"/>
       <c r="K418" t="inlineStr"/>
@@ -24886,7 +24894,7 @@
         </is>
       </c>
       <c r="I419" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J419" t="inlineStr"/>
       <c r="K419" t="inlineStr"/>
@@ -24936,7 +24944,7 @@
         </is>
       </c>
       <c r="I420" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J420" t="inlineStr"/>
       <c r="K420" t="inlineStr"/>
@@ -24986,7 +24994,7 @@
         </is>
       </c>
       <c r="I421" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J421" t="inlineStr"/>
       <c r="K421" t="inlineStr"/>
@@ -25036,7 +25044,7 @@
         </is>
       </c>
       <c r="I422" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J422" t="inlineStr"/>
       <c r="K422" t="inlineStr"/>
@@ -25086,7 +25094,7 @@
         </is>
       </c>
       <c r="I423" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J423" t="inlineStr"/>
       <c r="K423" t="inlineStr"/>
@@ -25136,7 +25144,7 @@
         </is>
       </c>
       <c r="I424" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J424" t="inlineStr"/>
       <c r="K424" t="inlineStr"/>
@@ -25186,7 +25194,7 @@
         </is>
       </c>
       <c r="I425" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J425" t="inlineStr"/>
       <c r="K425" t="inlineStr"/>
@@ -25238,7 +25246,7 @@
         </is>
       </c>
       <c r="I426" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J426" t="inlineStr"/>
       <c r="K426" t="inlineStr"/>
@@ -25288,7 +25296,7 @@
         </is>
       </c>
       <c r="I427" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J427" t="inlineStr"/>
       <c r="K427" t="inlineStr"/>
@@ -25338,7 +25346,7 @@
         </is>
       </c>
       <c r="I428" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J428" t="inlineStr"/>
       <c r="K428" t="inlineStr"/>
@@ -25388,7 +25396,7 @@
         </is>
       </c>
       <c r="I429" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J429" t="inlineStr"/>
       <c r="K429" t="inlineStr"/>
@@ -25438,7 +25446,7 @@
         </is>
       </c>
       <c r="I430" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J430" t="inlineStr"/>
       <c r="K430" t="inlineStr"/>
@@ -25488,7 +25496,7 @@
         </is>
       </c>
       <c r="I431" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J431" t="inlineStr"/>
       <c r="K431" t="inlineStr"/>
@@ -25538,7 +25546,7 @@
         </is>
       </c>
       <c r="I432" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J432" t="inlineStr"/>
       <c r="K432" t="inlineStr"/>
@@ -25588,7 +25596,7 @@
         </is>
       </c>
       <c r="I433" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J433" t="inlineStr"/>
       <c r="K433" t="inlineStr"/>
@@ -25636,7 +25644,7 @@
         </is>
       </c>
       <c r="I434" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J434" t="inlineStr"/>
       <c r="K434" t="inlineStr"/>
@@ -25684,7 +25692,7 @@
         </is>
       </c>
       <c r="I435" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J435" t="inlineStr"/>
       <c r="K435" t="inlineStr"/>
@@ -25732,7 +25740,7 @@
         </is>
       </c>
       <c r="I436" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J436" t="inlineStr"/>
       <c r="K436" t="inlineStr"/>
@@ -25780,7 +25788,7 @@
         </is>
       </c>
       <c r="I437" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J437" t="inlineStr"/>
       <c r="K437" t="inlineStr"/>
@@ -25830,7 +25838,7 @@
         </is>
       </c>
       <c r="I438" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J438" t="inlineStr"/>
       <c r="K438" t="inlineStr"/>
@@ -25882,7 +25890,7 @@
         </is>
       </c>
       <c r="I439" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J439" t="inlineStr"/>
       <c r="K439" t="inlineStr"/>
@@ -25934,7 +25942,7 @@
         </is>
       </c>
       <c r="I440" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J440" t="inlineStr"/>
       <c r="K440" t="inlineStr"/>
@@ -25984,7 +25992,7 @@
         </is>
       </c>
       <c r="I441" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J441" t="inlineStr"/>
       <c r="K441" t="inlineStr"/>
@@ -26034,7 +26042,7 @@
         </is>
       </c>
       <c r="I442" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J442" t="inlineStr"/>
       <c r="K442" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (10/07/2026 22:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,82 +421,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>os</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>cff</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>data_inicio</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>unidade_solicitante</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tat_siloms</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>onde_se_encontra</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>recibo</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>condicao</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>data_retorno_prevista</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>sn_trocado_exchange</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>termo_recebimento</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -540,7 +528,7 @@
           <t>3859</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="1" t="n">
         <v>45698</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -600,7 +588,7 @@
           <t>382750-016</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="1" t="n">
         <v>45714</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -660,7 +648,7 @@
           <t>382750-023</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
         <v>45714</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -720,7 +708,7 @@
           <t>003342</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="1" t="n">
         <v>45714</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -747,7 +735,7 @@
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="1" t="n">
         <v>45993</v>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -782,7 +770,7 @@
           <t>09450</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -809,7 +797,7 @@
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="1" t="n">
         <v>45889</v>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -844,7 +832,7 @@
           <t>1920</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -871,7 +859,7 @@
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -910,7 +898,7 @@
           <t>96967</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -960,7 +948,7 @@
           <t>2410</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -987,7 +975,7 @@
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="1" t="n">
         <v>46098</v>
       </c>
       <c r="N9" t="n">
@@ -1024,7 +1012,7 @@
           <t>P1916</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -1051,7 +1039,7 @@
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="1" t="n">
         <v>46114</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -1090,7 +1078,7 @@
           <t>2697</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -1117,7 +1105,7 @@
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -1156,7 +1144,7 @@
           <t>1569</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -1183,7 +1171,7 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" s="2" t="n">
+      <c r="M12" s="1" t="n">
         <v>45860</v>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -1218,7 +1206,7 @@
           <t>2706</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1276,7 +1264,7 @@
           <t>0215-217</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -1303,7 +1291,7 @@
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
-      <c r="M14" s="2" t="n">
+      <c r="M14" s="1" t="n">
         <v>45800</v>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -1338,7 +1326,7 @@
           <t>K010158</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1398,7 +1386,7 @@
           <t>9911-257</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1458,7 +1446,7 @@
           <t>791</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F17" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1485,7 +1473,7 @@
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" s="2" t="n">
+      <c r="M17" s="1" t="n">
         <v>45897</v>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -1520,7 +1508,7 @@
           <t>7077</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G18" t="inlineStr">
@@ -1547,7 +1535,7 @@
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
+      <c r="M18" s="1" t="n">
         <v>45802</v>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -1582,7 +1570,7 @@
           <t>3890</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="F19" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G19" t="inlineStr">
@@ -1640,7 +1628,7 @@
           <t>KI256-25711</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G20" t="inlineStr">
@@ -1667,7 +1655,7 @@
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" s="2" t="n">
+      <c r="M20" s="1" t="n">
         <v>46135</v>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -1702,7 +1690,7 @@
           <t>KI256-25707</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="F21" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -1760,7 +1748,7 @@
           <t>3885</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -1820,7 +1808,7 @@
           <t>3861</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="F23" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -1847,7 +1835,7 @@
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
+      <c r="M23" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -1886,7 +1874,7 @@
           <t>17143</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G24" t="inlineStr">
@@ -1944,7 +1932,7 @@
           <t>96782</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G25" t="inlineStr">
@@ -2002,7 +1990,7 @@
           <t>KMD540-10071</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -2029,7 +2017,7 @@
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
+      <c r="M26" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="N26" t="inlineStr"/>
@@ -2068,7 +2056,7 @@
           <t>75123</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="F27" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G27" t="inlineStr">
@@ -2128,7 +2116,7 @@
           <t>00B205C</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="F28" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -2178,7 +2166,7 @@
           <t>277</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="F29" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G29" t="inlineStr">
@@ -2236,7 +2224,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G30" t="inlineStr">
@@ -2263,7 +2251,7 @@
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" s="2" t="n">
+      <c r="M30" s="1" t="n">
         <v>45945</v>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -2298,7 +2286,7 @@
           <t>7951</t>
         </is>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="F31" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G31" t="inlineStr">
@@ -2356,7 +2344,7 @@
           <t>5028A</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G32" t="inlineStr">
@@ -2416,7 +2404,7 @@
           <t>122</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G33" t="inlineStr">
@@ -2474,7 +2462,7 @@
           <t>27</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G34" t="inlineStr">
@@ -2524,7 +2512,7 @@
           <t>02B</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F35" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G35" t="inlineStr">
@@ -2574,7 +2562,7 @@
           <t>291</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G36" t="inlineStr">
@@ -2632,7 +2620,7 @@
           <t>0011</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F37" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G37" t="inlineStr">
@@ -2690,7 +2678,7 @@
           <t>791</t>
         </is>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="F38" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G38" t="inlineStr">
@@ -2744,7 +2732,7 @@
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" s="2" t="n">
+      <c r="F39" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G39" t="inlineStr">
@@ -2800,7 +2788,7 @@
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
-      <c r="F40" s="2" t="n">
+      <c r="F40" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G40" t="inlineStr">
@@ -2860,7 +2848,7 @@
           <t>988</t>
         </is>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="F41" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G41" t="inlineStr">
@@ -2918,7 +2906,7 @@
           <t>994</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F42" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G42" t="inlineStr">
@@ -2976,7 +2964,7 @@
           <t>10603745</t>
         </is>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="F43" s="1" t="n">
         <v>45736</v>
       </c>
       <c r="G43" t="inlineStr">
@@ -3034,7 +3022,7 @@
           <t>LS0414</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="F44" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G44" t="inlineStr">
@@ -3061,7 +3049,7 @@
         </is>
       </c>
       <c r="L44" t="inlineStr"/>
-      <c r="M44" s="2" t="n">
+      <c r="M44" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="N44" t="inlineStr"/>
@@ -3100,7 +3088,7 @@
           <t>86805596</t>
         </is>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="F45" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G45" t="inlineStr">
@@ -3127,7 +3115,7 @@
         </is>
       </c>
       <c r="L45" t="inlineStr"/>
-      <c r="M45" s="2" t="n">
+      <c r="M45" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="N45" t="n">
@@ -3164,7 +3152,7 @@
           <t>R50653</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G46" t="inlineStr">
@@ -3224,7 +3212,7 @@
           <t>53450</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="F47" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G47" t="inlineStr">
@@ -3251,7 +3239,7 @@
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
-      <c r="M47" s="2" t="n">
+      <c r="M47" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="N47" t="inlineStr"/>
@@ -3290,7 +3278,7 @@
           <t>52537</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F48" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G48" t="inlineStr">
@@ -3350,7 +3338,7 @@
           <t>51767</t>
         </is>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="F49" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G49" t="inlineStr">
@@ -3400,7 +3388,7 @@
           <t>28411</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F50" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G50" t="inlineStr">
@@ -3460,7 +3448,7 @@
           <t>36025</t>
         </is>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="F51" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G51" t="inlineStr">
@@ -3518,7 +3506,7 @@
           <t>34257</t>
         </is>
       </c>
-      <c r="F52" s="2" t="n">
+      <c r="F52" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G52" t="inlineStr">
@@ -3578,7 +3566,7 @@
           <t>30865</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n">
+      <c r="F53" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G53" t="inlineStr">
@@ -3638,7 +3626,7 @@
           <t>4355</t>
         </is>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="F54" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G54" t="inlineStr">
@@ -3698,7 +3686,7 @@
           <t>38197</t>
         </is>
       </c>
-      <c r="F55" s="2" t="n">
+      <c r="F55" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G55" t="inlineStr">
@@ -3748,7 +3736,7 @@
           <t>85131</t>
         </is>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="F56" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G56" t="inlineStr">
@@ -3806,7 +3794,7 @@
           <t>86012</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="F57" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G57" t="inlineStr">
@@ -3866,7 +3854,7 @@
           <t>85068</t>
         </is>
       </c>
-      <c r="F58" s="2" t="n">
+      <c r="F58" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G58" t="inlineStr">
@@ -3916,7 +3904,7 @@
           <t>84459</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="F59" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G59" t="inlineStr">
@@ -3974,7 +3962,7 @@
           <t>AAT5599</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="F60" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G60" t="inlineStr">
@@ -4032,7 +4020,7 @@
           <t>AAE3882</t>
         </is>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="F61" s="1" t="n">
         <v>45769</v>
       </c>
       <c r="G61" t="inlineStr">
@@ -4086,7 +4074,7 @@
           <t>22005920</t>
         </is>
       </c>
-      <c r="F62" s="2" t="n">
+      <c r="F62" s="1" t="n">
         <v>45770</v>
       </c>
       <c r="G62" t="inlineStr">
@@ -4136,7 +4124,7 @@
           <t>1882C</t>
         </is>
       </c>
-      <c r="F63" s="2" t="n">
+      <c r="F63" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="G63" t="inlineStr">
@@ -4163,7 +4151,7 @@
         </is>
       </c>
       <c r="L63" t="inlineStr"/>
-      <c r="M63" s="2" t="n">
+      <c r="M63" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="N63" t="inlineStr"/>
@@ -4202,7 +4190,7 @@
           <t>02</t>
         </is>
       </c>
-      <c r="F64" s="2" t="n">
+      <c r="F64" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="G64" t="inlineStr">
@@ -4229,7 +4217,7 @@
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
-      <c r="M64" s="2" t="n">
+      <c r="M64" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="N64" t="inlineStr"/>
@@ -4264,7 +4252,7 @@
           <t>323</t>
         </is>
       </c>
-      <c r="F65" s="2" t="n">
+      <c r="F65" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="G65" t="inlineStr">
@@ -4322,7 +4310,7 @@
           <t>297</t>
         </is>
       </c>
-      <c r="F66" s="2" t="n">
+      <c r="F66" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="G66" t="inlineStr">
@@ -4380,7 +4368,7 @@
           <t>144</t>
         </is>
       </c>
-      <c r="F67" s="2" t="n">
+      <c r="F67" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="G67" t="inlineStr">
@@ -4438,7 +4426,7 @@
           <t>324</t>
         </is>
       </c>
-      <c r="F68" s="2" t="n">
+      <c r="F68" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="G68" t="inlineStr">
@@ -4496,7 +4484,7 @@
           <t>475</t>
         </is>
       </c>
-      <c r="F69" s="2" t="n">
+      <c r="F69" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G69" t="inlineStr">
@@ -4554,7 +4542,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="F70" s="2" t="n">
+      <c r="F70" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G70" t="inlineStr">
@@ -4614,7 +4602,7 @@
           <t>UNK01</t>
         </is>
       </c>
-      <c r="F71" s="2" t="n">
+      <c r="F71" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G71" t="inlineStr">
@@ -4670,7 +4658,7 @@
           <t>278</t>
         </is>
       </c>
-      <c r="F72" s="2" t="n">
+      <c r="F72" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G72" t="inlineStr">
@@ -4728,7 +4716,7 @@
           <t>967</t>
         </is>
       </c>
-      <c r="F73" s="2" t="n">
+      <c r="F73" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G73" t="inlineStr">
@@ -4788,7 +4776,7 @@
           <t>278</t>
         </is>
       </c>
-      <c r="F74" s="2" t="n">
+      <c r="F74" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G74" t="inlineStr">
@@ -4846,7 +4834,7 @@
           <t>772</t>
         </is>
       </c>
-      <c r="F75" s="2" t="n">
+      <c r="F75" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G75" t="inlineStr">
@@ -4906,7 +4894,7 @@
           <t>49</t>
         </is>
       </c>
-      <c r="F76" s="2" t="n">
+      <c r="F76" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G76" t="inlineStr">
@@ -4962,7 +4950,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="F77" s="2" t="n">
+      <c r="F77" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G77" t="inlineStr">
@@ -5020,7 +5008,7 @@
           <t>289</t>
         </is>
       </c>
-      <c r="F78" s="2" t="n">
+      <c r="F78" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G78" t="inlineStr">
@@ -5078,7 +5066,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="F79" s="2" t="n">
+      <c r="F79" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G79" t="inlineStr">
@@ -5134,7 +5122,7 @@
           <t>969</t>
         </is>
       </c>
-      <c r="F80" s="2" t="n">
+      <c r="F80" s="1" t="n">
         <v>45803</v>
       </c>
       <c r="G80" t="inlineStr">
@@ -5194,7 +5182,7 @@
           <t>1311</t>
         </is>
       </c>
-      <c r="F81" s="2" t="n">
+      <c r="F81" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G81" t="inlineStr">
@@ -5252,7 +5240,7 @@
           <t>3945</t>
         </is>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F82" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G82" t="inlineStr">
@@ -5312,7 +5300,7 @@
           <t>35378</t>
         </is>
       </c>
-      <c r="F83" s="2" t="n">
+      <c r="F83" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G83" t="inlineStr">
@@ -5370,7 +5358,7 @@
           <t>2469</t>
         </is>
       </c>
-      <c r="F84" s="2" t="n">
+      <c r="F84" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G84" t="inlineStr">
@@ -5397,7 +5385,7 @@
         </is>
       </c>
       <c r="L84" t="inlineStr"/>
-      <c r="M84" s="2" t="n">
+      <c r="M84" s="1" t="n">
         <v>45853</v>
       </c>
       <c r="N84" t="n">
@@ -5434,7 +5422,7 @@
           <t>292</t>
         </is>
       </c>
-      <c r="F85" s="2" t="n">
+      <c r="F85" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G85" t="inlineStr">
@@ -5494,7 +5482,7 @@
           <t>168394-05</t>
         </is>
       </c>
-      <c r="F86" s="2" t="n">
+      <c r="F86" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G86" t="inlineStr">
@@ -5554,7 +5542,7 @@
           <t>197</t>
         </is>
       </c>
-      <c r="F87" s="2" t="n">
+      <c r="F87" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G87" t="inlineStr">
@@ -5581,7 +5569,7 @@
         </is>
       </c>
       <c r="L87" t="inlineStr"/>
-      <c r="M87" s="2" t="n">
+      <c r="M87" s="1" t="n">
         <v>45797</v>
       </c>
       <c r="N87" t="inlineStr">
@@ -5620,7 +5608,7 @@
           <t>10603744</t>
         </is>
       </c>
-      <c r="F88" s="2" t="n">
+      <c r="F88" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G88" t="inlineStr">
@@ -5678,7 +5666,7 @@
           <t>11200477</t>
         </is>
       </c>
-      <c r="F89" s="2" t="n">
+      <c r="F89" s="1" t="n">
         <v>45813</v>
       </c>
       <c r="G89" t="inlineStr">
@@ -5736,7 +5724,7 @@
           <t>5385</t>
         </is>
       </c>
-      <c r="F90" s="2" t="n">
+      <c r="F90" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G90" t="inlineStr">
@@ -5800,7 +5788,7 @@
           <t>001</t>
         </is>
       </c>
-      <c r="F91" s="2" t="n">
+      <c r="F91" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G91" t="inlineStr">
@@ -5856,7 +5844,7 @@
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
-      <c r="F92" s="2" t="n">
+      <c r="F92" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G92" t="inlineStr">
@@ -5906,7 +5894,7 @@
           <t>CE-11200</t>
         </is>
       </c>
-      <c r="F93" s="2" t="n">
+      <c r="F93" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G93" t="inlineStr">
@@ -5966,7 +5954,7 @@
           <t>CE-09234</t>
         </is>
       </c>
-      <c r="F94" s="2" t="n">
+      <c r="F94" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G94" t="inlineStr">
@@ -6026,7 +6014,7 @@
           <t>CE-08838</t>
         </is>
       </c>
-      <c r="F95" s="2" t="n">
+      <c r="F95" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G95" t="inlineStr">
@@ -6086,7 +6074,7 @@
           <t>908</t>
         </is>
       </c>
-      <c r="F96" s="2" t="n">
+      <c r="F96" s="1" t="n">
         <v>45831</v>
       </c>
       <c r="G96" t="inlineStr">
@@ -6113,7 +6101,7 @@
         </is>
       </c>
       <c r="L96" t="inlineStr"/>
-      <c r="M96" s="2" t="n">
+      <c r="M96" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="N96" t="inlineStr">
@@ -6152,7 +6140,7 @@
           <t>203103</t>
         </is>
       </c>
-      <c r="F97" s="2" t="n">
+      <c r="F97" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G97" t="inlineStr">
@@ -6216,7 +6204,7 @@
           <t>56422</t>
         </is>
       </c>
-      <c r="F98" s="2" t="n">
+      <c r="F98" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G98" t="inlineStr">
@@ -6276,7 +6264,7 @@
           <t>07915</t>
         </is>
       </c>
-      <c r="F99" s="2" t="n">
+      <c r="F99" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G99" t="inlineStr">
@@ -6326,7 +6314,7 @@
           <t>X-330970</t>
         </is>
       </c>
-      <c r="F100" s="2" t="n">
+      <c r="F100" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G100" t="inlineStr">
@@ -6386,7 +6374,7 @@
           <t>X-412785</t>
         </is>
       </c>
-      <c r="F101" s="2" t="n">
+      <c r="F101" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G101" t="inlineStr">
@@ -6436,7 +6424,7 @@
           <t>B10811721</t>
         </is>
       </c>
-      <c r="F102" s="2" t="n">
+      <c r="F102" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G102" t="inlineStr">
@@ -6486,7 +6474,7 @@
           <t>X330978</t>
         </is>
       </c>
-      <c r="F103" s="2" t="n">
+      <c r="F103" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G103" t="inlineStr">
@@ -6536,7 +6524,7 @@
           <t>X-467664</t>
         </is>
       </c>
-      <c r="F104" s="2" t="n">
+      <c r="F104" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G104" t="inlineStr">
@@ -6596,7 +6584,7 @@
           <t>D00397798</t>
         </is>
       </c>
-      <c r="F105" s="2" t="n">
+      <c r="F105" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G105" t="inlineStr">
@@ -6656,7 +6644,7 @@
           <t>6132</t>
         </is>
       </c>
-      <c r="F106" s="2" t="n">
+      <c r="F106" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G106" t="inlineStr">
@@ -6683,7 +6671,7 @@
         </is>
       </c>
       <c r="L106" t="inlineStr"/>
-      <c r="M106" s="2" t="n">
+      <c r="M106" s="1" t="n">
         <v>45889</v>
       </c>
       <c r="N106" t="inlineStr"/>
@@ -6718,7 +6706,7 @@
           <t>030998</t>
         </is>
       </c>
-      <c r="F107" s="2" t="n">
+      <c r="F107" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G107" t="inlineStr">
@@ -6745,7 +6733,7 @@
         </is>
       </c>
       <c r="L107" t="inlineStr"/>
-      <c r="M107" s="2" t="n">
+      <c r="M107" s="1" t="n">
         <v>45876</v>
       </c>
       <c r="N107" t="inlineStr"/>
@@ -6780,7 +6768,7 @@
           <t>5AL</t>
         </is>
       </c>
-      <c r="F108" s="2" t="n">
+      <c r="F108" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G108" t="inlineStr">
@@ -6840,7 +6828,7 @@
           <t>7AC</t>
         </is>
       </c>
-      <c r="F109" s="2" t="n">
+      <c r="F109" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G109" t="inlineStr">
@@ -6900,7 +6888,7 @@
           <t>2668-5</t>
         </is>
       </c>
-      <c r="F110" s="2" t="n">
+      <c r="F110" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G110" t="inlineStr">
@@ -6958,7 +6946,7 @@
           <t>3155-5</t>
         </is>
       </c>
-      <c r="F111" s="2" t="n">
+      <c r="F111" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G111" t="inlineStr">
@@ -7016,7 +7004,7 @@
           <t>3124-5</t>
         </is>
       </c>
-      <c r="F112" s="2" t="n">
+      <c r="F112" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G112" t="inlineStr">
@@ -7066,7 +7054,7 @@
           <t>3275-5</t>
         </is>
       </c>
-      <c r="F113" s="2" t="n">
+      <c r="F113" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G113" t="inlineStr">
@@ -7124,7 +7112,7 @@
           <t>9902509</t>
         </is>
       </c>
-      <c r="F114" s="2" t="n">
+      <c r="F114" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G114" t="inlineStr">
@@ -7182,7 +7170,7 @@
           <t>369783-021</t>
         </is>
       </c>
-      <c r="F115" s="2" t="n">
+      <c r="F115" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G115" t="inlineStr">
@@ -7242,7 +7230,7 @@
           <t>363749-030</t>
         </is>
       </c>
-      <c r="F116" s="2" t="n">
+      <c r="F116" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G116" t="inlineStr">
@@ -7302,7 +7290,7 @@
           <t>376422-005</t>
         </is>
       </c>
-      <c r="F117" s="2" t="n">
+      <c r="F117" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G117" t="inlineStr">
@@ -7362,7 +7350,7 @@
           <t>376415-037</t>
         </is>
       </c>
-      <c r="F118" s="2" t="n">
+      <c r="F118" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G118" t="inlineStr">
@@ -7422,7 +7410,7 @@
           <t>363761-060</t>
         </is>
       </c>
-      <c r="F119" s="2" t="n">
+      <c r="F119" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G119" t="inlineStr">
@@ -7482,7 +7470,7 @@
           <t>363749-085</t>
         </is>
       </c>
-      <c r="F120" s="2" t="n">
+      <c r="F120" s="1" t="n">
         <v>45840</v>
       </c>
       <c r="G120" t="inlineStr">
@@ -7542,7 +7530,7 @@
           <t>86800893</t>
         </is>
       </c>
-      <c r="F121" s="2" t="n">
+      <c r="F121" s="1" t="n">
         <v>45849</v>
       </c>
       <c r="G121" t="inlineStr">
@@ -7569,7 +7557,7 @@
         </is>
       </c>
       <c r="L121" t="inlineStr"/>
-      <c r="M121" s="2" t="n">
+      <c r="M121" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="N121" t="n">
@@ -7606,7 +7594,7 @@
           <t>003614</t>
         </is>
       </c>
-      <c r="F122" s="2" t="n">
+      <c r="F122" s="1" t="n">
         <v>45849</v>
       </c>
       <c r="G122" t="inlineStr">
@@ -7666,7 +7654,7 @@
           <t>15100008</t>
         </is>
       </c>
-      <c r="F123" s="2" t="n">
+      <c r="F123" s="1" t="n">
         <v>45849</v>
       </c>
       <c r="G123" t="inlineStr">
@@ -7716,7 +7704,7 @@
           <t>0235</t>
         </is>
       </c>
-      <c r="F124" s="2" t="n">
+      <c r="F124" s="1" t="n">
         <v>45853</v>
       </c>
       <c r="G124" t="inlineStr">
@@ -7776,7 +7764,7 @@
           <t>5236</t>
         </is>
       </c>
-      <c r="F125" s="2" t="n">
+      <c r="F125" s="1" t="n">
         <v>45855</v>
       </c>
       <c r="G125" t="inlineStr">
@@ -7836,7 +7824,7 @@
           <t>ART2000-13237</t>
         </is>
       </c>
-      <c r="F126" s="2" t="n">
+      <c r="F126" s="1" t="n">
         <v>45855</v>
       </c>
       <c r="G126" t="inlineStr">
@@ -7894,7 +7882,7 @@
           <t>T23740</t>
         </is>
       </c>
-      <c r="F127" s="2" t="n">
+      <c r="F127" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="G127" t="inlineStr">
@@ -7944,7 +7932,7 @@
           <t>5K660</t>
         </is>
       </c>
-      <c r="F128" s="2" t="n">
+      <c r="F128" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="G128" t="inlineStr">
@@ -8004,7 +7992,7 @@
           <t>71306307</t>
         </is>
       </c>
-      <c r="F129" s="2" t="n">
+      <c r="F129" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="G129" t="inlineStr">
@@ -8064,7 +8052,7 @@
           <t>47204432</t>
         </is>
       </c>
-      <c r="F130" s="2" t="n">
+      <c r="F130" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="G130" t="inlineStr">
@@ -8091,7 +8079,7 @@
         </is>
       </c>
       <c r="L130" t="inlineStr"/>
-      <c r="M130" s="2" t="n">
+      <c r="M130" s="1" t="n">
         <v>45916</v>
       </c>
       <c r="N130" t="n">
@@ -8128,7 +8116,7 @@
           <t>409496</t>
         </is>
       </c>
-      <c r="F131" s="2" t="n">
+      <c r="F131" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="G131" t="inlineStr">
@@ -8186,7 +8174,7 @@
           <t>71308676</t>
         </is>
       </c>
-      <c r="F132" s="2" t="n">
+      <c r="F132" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="G132" t="inlineStr">
@@ -8213,7 +8201,7 @@
         </is>
       </c>
       <c r="L132" t="inlineStr"/>
-      <c r="M132" s="2" t="n">
+      <c r="M132" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="N132" t="n">
@@ -8250,7 +8238,7 @@
           <t>86819178</t>
         </is>
       </c>
-      <c r="F133" s="2" t="n">
+      <c r="F133" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="G133" t="inlineStr">
@@ -8300,7 +8288,7 @@
           <t>8259</t>
         </is>
       </c>
-      <c r="F134" s="2" t="n">
+      <c r="F134" s="1" t="n">
         <v>45882</v>
       </c>
       <c r="G134" t="inlineStr">
@@ -8360,7 +8348,7 @@
           <t>22A805</t>
         </is>
       </c>
-      <c r="F135" s="2" t="n">
+      <c r="F135" s="1" t="n">
         <v>45882</v>
       </c>
       <c r="G135" t="inlineStr">
@@ -8410,7 +8398,7 @@
           <t>T22974</t>
         </is>
       </c>
-      <c r="F136" s="2" t="n">
+      <c r="F136" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G136" t="inlineStr">
@@ -8460,7 +8448,7 @@
           <t>15508160</t>
         </is>
       </c>
-      <c r="F137" s="2" t="n">
+      <c r="F137" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G137" t="inlineStr">
@@ -8510,7 +8498,7 @@
           <t>12056029</t>
         </is>
       </c>
-      <c r="F138" s="2" t="n">
+      <c r="F138" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G138" t="inlineStr">
@@ -8570,7 +8558,7 @@
           <t>T20503</t>
         </is>
       </c>
-      <c r="F139" s="2" t="n">
+      <c r="F139" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G139" t="inlineStr">
@@ -8620,7 +8608,7 @@
           <t>T25426</t>
         </is>
       </c>
-      <c r="F140" s="2" t="n">
+      <c r="F140" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G140" t="inlineStr">
@@ -8678,7 +8666,7 @@
           <t>03</t>
         </is>
       </c>
-      <c r="F141" s="2" t="n">
+      <c r="F141" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G141" t="inlineStr">
@@ -8728,7 +8716,7 @@
           <t>778</t>
         </is>
       </c>
-      <c r="F142" s="2" t="n">
+      <c r="F142" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G142" t="inlineStr">
@@ -8778,7 +8766,7 @@
           <t>356</t>
         </is>
       </c>
-      <c r="F143" s="2" t="n">
+      <c r="F143" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G143" t="inlineStr">
@@ -8828,7 +8816,7 @@
           <t>28</t>
         </is>
       </c>
-      <c r="F144" s="2" t="n">
+      <c r="F144" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G144" t="inlineStr">
@@ -8878,7 +8866,7 @@
           <t>048F</t>
         </is>
       </c>
-      <c r="F145" s="2" t="n">
+      <c r="F145" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G145" t="inlineStr">
@@ -8936,7 +8924,7 @@
           <t>3270</t>
         </is>
       </c>
-      <c r="F146" s="2" t="n">
+      <c r="F146" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G146" t="inlineStr">
@@ -8986,7 +8974,7 @@
           <t>LSEAM3250</t>
         </is>
       </c>
-      <c r="F147" s="2" t="n">
+      <c r="F147" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G147" t="inlineStr">
@@ -9044,7 +9032,7 @@
           <t>A4H-106-02</t>
         </is>
       </c>
-      <c r="F148" s="2" t="n">
+      <c r="F148" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G148" t="inlineStr">
@@ -9104,7 +9092,7 @@
           <t>K517</t>
         </is>
       </c>
-      <c r="F149" s="2" t="n">
+      <c r="F149" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G149" t="inlineStr">
@@ -9160,7 +9148,7 @@
           <t>016B</t>
         </is>
       </c>
-      <c r="F150" s="2" t="n">
+      <c r="F150" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G150" t="inlineStr">
@@ -9187,7 +9175,7 @@
         </is>
       </c>
       <c r="L150" t="inlineStr"/>
-      <c r="M150" s="2" t="n">
+      <c r="M150" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="N150" t="inlineStr"/>
@@ -9226,7 +9214,7 @@
           <t>935</t>
         </is>
       </c>
-      <c r="F151" s="2" t="n">
+      <c r="F151" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G151" t="inlineStr">
@@ -9284,7 +9272,7 @@
           <t>03</t>
         </is>
       </c>
-      <c r="F152" s="2" t="n">
+      <c r="F152" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G152" t="inlineStr">
@@ -9311,7 +9299,7 @@
         </is>
       </c>
       <c r="L152" t="inlineStr"/>
-      <c r="M152" s="2" t="n">
+      <c r="M152" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="N152" t="inlineStr"/>
@@ -9346,7 +9334,7 @@
           <t>B4H-018</t>
         </is>
       </c>
-      <c r="F153" s="2" t="n">
+      <c r="F153" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G153" t="inlineStr">
@@ -9406,7 +9394,7 @@
           <t>108</t>
         </is>
       </c>
-      <c r="F154" s="2" t="n">
+      <c r="F154" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G154" t="inlineStr">
@@ -9464,7 +9452,7 @@
           <t>66306636</t>
         </is>
       </c>
-      <c r="F155" s="2" t="n">
+      <c r="F155" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G155" t="inlineStr">
@@ -9520,7 +9508,7 @@
           <t>66305791</t>
         </is>
       </c>
-      <c r="F156" s="2" t="n">
+      <c r="F156" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G156" t="inlineStr">
@@ -9580,7 +9568,7 @@
           <t>47203806</t>
         </is>
       </c>
-      <c r="F157" s="2" t="n">
+      <c r="F157" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="G157" t="inlineStr">
@@ -9640,7 +9628,7 @@
           <t>28A403</t>
         </is>
       </c>
-      <c r="F158" s="2" t="n">
+      <c r="F158" s="1" t="n">
         <v>45894</v>
       </c>
       <c r="G158" t="inlineStr">
@@ -9667,7 +9655,7 @@
         </is>
       </c>
       <c r="L158" t="inlineStr"/>
-      <c r="M158" s="2" t="n">
+      <c r="M158" s="1" t="n">
         <v>45946</v>
       </c>
       <c r="N158" t="inlineStr"/>
@@ -9702,7 +9690,7 @@
           <t>479</t>
         </is>
       </c>
-      <c r="F159" s="2" t="n">
+      <c r="F159" s="1" t="n">
         <v>45894</v>
       </c>
       <c r="G159" t="inlineStr">
@@ -9762,7 +9750,7 @@
           <t>15W008701</t>
         </is>
       </c>
-      <c r="F160" s="2" t="n">
+      <c r="F160" s="1" t="n">
         <v>45898</v>
       </c>
       <c r="G160" t="inlineStr">
@@ -9822,7 +9810,7 @@
           <t>15W006615</t>
         </is>
       </c>
-      <c r="F161" s="2" t="n">
+      <c r="F161" s="1" t="n">
         <v>45898</v>
       </c>
       <c r="G161" t="inlineStr">
@@ -9849,7 +9837,7 @@
         </is>
       </c>
       <c r="L161" t="inlineStr"/>
-      <c r="M161" s="2" t="n">
+      <c r="M161" s="1" t="n">
         <v>45953</v>
       </c>
       <c r="N161" t="inlineStr">
@@ -9888,7 +9876,7 @@
           <t>2953</t>
         </is>
       </c>
-      <c r="F162" s="2" t="n">
+      <c r="F162" s="1" t="n">
         <v>45898</v>
       </c>
       <c r="G162" t="inlineStr">
@@ -9915,7 +9903,7 @@
         </is>
       </c>
       <c r="L162" t="inlineStr"/>
-      <c r="M162" s="2" t="n">
+      <c r="M162" s="1" t="n">
         <v>45940</v>
       </c>
       <c r="N162" t="inlineStr"/>
@@ -9950,7 +9938,7 @@
           <t>2982</t>
         </is>
       </c>
-      <c r="F163" s="2" t="n">
+      <c r="F163" s="1" t="n">
         <v>45898</v>
       </c>
       <c r="G163" t="inlineStr">
@@ -9977,7 +9965,7 @@
         </is>
       </c>
       <c r="L163" t="inlineStr"/>
-      <c r="M163" s="2" t="n">
+      <c r="M163" s="1" t="n">
         <v>45940</v>
       </c>
       <c r="N163" t="inlineStr"/>
@@ -10012,7 +10000,7 @@
           <t>37F</t>
         </is>
       </c>
-      <c r="F164" s="2" t="n">
+      <c r="F164" s="1" t="n">
         <v>45910</v>
       </c>
       <c r="G164" t="inlineStr">
@@ -10068,7 +10056,7 @@
           <t>02LS</t>
         </is>
       </c>
-      <c r="F165" s="2" t="n">
+      <c r="F165" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G165" t="inlineStr">
@@ -10128,7 +10116,7 @@
           <t>B10133</t>
         </is>
       </c>
-      <c r="F166" s="2" t="n">
+      <c r="F166" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G166" t="inlineStr">
@@ -10186,7 +10174,7 @@
           <t>T20874</t>
         </is>
       </c>
-      <c r="F167" s="2" t="n">
+      <c r="F167" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G167" t="inlineStr">
@@ -10236,7 +10224,7 @@
           <t>T20976</t>
         </is>
       </c>
-      <c r="F168" s="2" t="n">
+      <c r="F168" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G168" t="inlineStr">
@@ -10300,7 +10288,7 @@
           <t>C25361</t>
         </is>
       </c>
-      <c r="F169" s="2" t="n">
+      <c r="F169" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G169" t="inlineStr">
@@ -10327,7 +10315,7 @@
         </is>
       </c>
       <c r="L169" t="inlineStr"/>
-      <c r="M169" s="2" t="n">
+      <c r="M169" s="1" t="n">
         <v>45973</v>
       </c>
       <c r="N169" t="inlineStr"/>
@@ -10362,7 +10350,7 @@
           <t>C25208</t>
         </is>
       </c>
-      <c r="F170" s="2" t="n">
+      <c r="F170" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G170" t="inlineStr">
@@ -10420,7 +10408,7 @@
           <t>571</t>
         </is>
       </c>
-      <c r="F171" s="2" t="n">
+      <c r="F171" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G171" t="inlineStr">
@@ -10480,7 +10468,7 @@
           <t>776</t>
         </is>
       </c>
-      <c r="F172" s="2" t="n">
+      <c r="F172" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G172" t="inlineStr">
@@ -10538,7 +10526,7 @@
           <t>LSEAM3239</t>
         </is>
       </c>
-      <c r="F173" s="2" t="n">
+      <c r="F173" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G173" t="inlineStr">
@@ -10596,7 +10584,7 @@
           <t>10603742</t>
         </is>
       </c>
-      <c r="F174" s="2" t="n">
+      <c r="F174" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G174" t="inlineStr">
@@ -10654,7 +10642,7 @@
           <t>015A</t>
         </is>
       </c>
-      <c r="F175" s="2" t="n">
+      <c r="F175" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G175" t="inlineStr">
@@ -10681,7 +10669,7 @@
         </is>
       </c>
       <c r="L175" t="inlineStr"/>
-      <c r="M175" s="2" t="n">
+      <c r="M175" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="N175" t="inlineStr"/>
@@ -10720,7 +10708,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="F176" s="2" t="n">
+      <c r="F176" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G176" t="inlineStr">
@@ -10780,7 +10768,7 @@
           <t>327</t>
         </is>
       </c>
-      <c r="F177" s="2" t="n">
+      <c r="F177" s="1" t="n">
         <v>45917</v>
       </c>
       <c r="G177" t="inlineStr">
@@ -10807,7 +10795,7 @@
         </is>
       </c>
       <c r="L177" t="inlineStr"/>
-      <c r="M177" s="2" t="n">
+      <c r="M177" s="1" t="n">
         <v>45961</v>
       </c>
       <c r="N177" t="inlineStr"/>
@@ -10846,7 +10834,7 @@
           <t>16389901</t>
         </is>
       </c>
-      <c r="F178" s="2" t="n">
+      <c r="F178" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="G178" t="inlineStr">
@@ -10906,7 +10894,7 @@
           <t>18384912</t>
         </is>
       </c>
-      <c r="F179" s="2" t="n">
+      <c r="F179" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="G179" t="inlineStr">
@@ -10956,7 +10944,7 @@
           <t>12253839V</t>
         </is>
       </c>
-      <c r="F180" s="2" t="n">
+      <c r="F180" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="G180" t="inlineStr">
@@ -11016,7 +11004,7 @@
           <t>12245097V</t>
         </is>
       </c>
-      <c r="F181" s="2" t="n">
+      <c r="F181" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="G181" t="inlineStr">
@@ -11074,7 +11062,7 @@
           <t>16940865</t>
         </is>
       </c>
-      <c r="F182" s="2" t="n">
+      <c r="F182" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="G182" t="inlineStr">
@@ -11124,7 +11112,7 @@
           <t>66307595</t>
         </is>
       </c>
-      <c r="F183" s="2" t="n">
+      <c r="F183" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="G183" t="inlineStr">
@@ -11180,7 +11168,7 @@
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
-      <c r="F184" s="2" t="n">
+      <c r="F184" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="G184" t="inlineStr">
@@ -11236,7 +11224,7 @@
           <t>66307562</t>
         </is>
       </c>
-      <c r="F185" s="2" t="n">
+      <c r="F185" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="G185" t="inlineStr">
@@ -11296,7 +11284,7 @@
           <t>66306759</t>
         </is>
       </c>
-      <c r="F186" s="2" t="n">
+      <c r="F186" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="G186" t="inlineStr">
@@ -11356,7 +11344,7 @@
           <t>66307058</t>
         </is>
       </c>
-      <c r="F187" s="2" t="n">
+      <c r="F187" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="G187" t="inlineStr">
@@ -11383,7 +11371,7 @@
         </is>
       </c>
       <c r="L187" t="inlineStr"/>
-      <c r="M187" s="2" t="n">
+      <c r="M187" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="N187" t="n">
@@ -11420,7 +11408,7 @@
           <t>21107</t>
         </is>
       </c>
-      <c r="F188" s="2" t="n">
+      <c r="F188" s="1" t="n">
         <v>45946</v>
       </c>
       <c r="G188" t="inlineStr">
@@ -11447,7 +11435,7 @@
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
-      <c r="M188" s="2" t="n">
+      <c r="M188" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="N188" t="inlineStr"/>
@@ -11486,7 +11474,7 @@
           <t>1318</t>
         </is>
       </c>
-      <c r="F189" s="2" t="n">
+      <c r="F189" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="G189" t="inlineStr">
@@ -11513,7 +11501,7 @@
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
-      <c r="M189" s="2" t="n">
+      <c r="M189" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="N189" t="inlineStr"/>
@@ -11548,7 +11536,7 @@
           <t>1608</t>
         </is>
       </c>
-      <c r="F190" s="2" t="n">
+      <c r="F190" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="G190" t="inlineStr">
@@ -11608,7 +11596,7 @@
           <t>17869</t>
         </is>
       </c>
-      <c r="F191" s="2" t="n">
+      <c r="F191" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="G191" t="inlineStr">
@@ -11635,7 +11623,7 @@
         </is>
       </c>
       <c r="L191" t="inlineStr"/>
-      <c r="M191" s="2" t="n">
+      <c r="M191" s="1" t="n">
         <v>45972</v>
       </c>
       <c r="N191" t="inlineStr"/>
@@ -11670,7 +11658,7 @@
           <t>T97147Q</t>
         </is>
       </c>
-      <c r="F192" s="2" t="n">
+      <c r="F192" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="G192" t="inlineStr">
@@ -11730,7 +11718,7 @@
           <t>07</t>
         </is>
       </c>
-      <c r="F193" s="2" t="n">
+      <c r="F193" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="G193" t="inlineStr">
@@ -11790,7 +11778,7 @@
           <t>6891</t>
         </is>
       </c>
-      <c r="F194" s="2" t="n">
+      <c r="F194" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="G194" t="inlineStr">
@@ -11840,7 +11828,7 @@
           <t>D12-10002</t>
         </is>
       </c>
-      <c r="F195" s="2" t="n">
+      <c r="F195" s="1" t="n">
         <v>45971</v>
       </c>
       <c r="G195" t="inlineStr">
@@ -11900,7 +11888,7 @@
           <t>0709LS</t>
         </is>
       </c>
-      <c r="F196" s="2" t="n">
+      <c r="F196" s="1" t="n">
         <v>45978</v>
       </c>
       <c r="G196" t="inlineStr">
@@ -11950,7 +11938,7 @@
           <t>H9533</t>
         </is>
       </c>
-      <c r="F197" s="2" t="n">
+      <c r="F197" s="1" t="n">
         <v>45978</v>
       </c>
       <c r="G197" t="inlineStr">
@@ -12000,7 +11988,7 @@
           <t>1902269</t>
         </is>
       </c>
-      <c r="F198" s="2" t="n">
+      <c r="F198" s="1" t="n">
         <v>45978</v>
       </c>
       <c r="G198" t="inlineStr">
@@ -12050,7 +12038,7 @@
           <t>1439</t>
         </is>
       </c>
-      <c r="F199" s="2" t="n">
+      <c r="F199" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="G199" t="inlineStr">
@@ -12077,7 +12065,7 @@
         </is>
       </c>
       <c r="L199" t="inlineStr"/>
-      <c r="M199" s="2" t="n">
+      <c r="M199" s="1" t="n">
         <v>46049</v>
       </c>
       <c r="N199" t="inlineStr"/>
@@ -12112,7 +12100,7 @@
           <t>182</t>
         </is>
       </c>
-      <c r="F200" s="2" t="n">
+      <c r="F200" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G200" t="inlineStr">
@@ -12172,7 +12160,7 @@
           <t>0707LS</t>
         </is>
       </c>
-      <c r="F201" s="2" t="n">
+      <c r="F201" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G201" t="inlineStr">
@@ -12232,7 +12220,7 @@
           <t>0801LS</t>
         </is>
       </c>
-      <c r="F202" s="2" t="n">
+      <c r="F202" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G202" t="inlineStr">
@@ -12292,7 +12280,7 @@
           <t>H9817</t>
         </is>
       </c>
-      <c r="F203" s="2" t="n">
+      <c r="F203" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G203" t="inlineStr">
@@ -12352,7 +12340,7 @@
           <t>37940</t>
         </is>
       </c>
-      <c r="F204" s="2" t="n">
+      <c r="F204" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G204" t="inlineStr">
@@ -12412,7 +12400,7 @@
           <t>39816</t>
         </is>
       </c>
-      <c r="F205" s="2" t="n">
+      <c r="F205" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G205" t="inlineStr">
@@ -12472,7 +12460,7 @@
           <t>89292</t>
         </is>
       </c>
-      <c r="F206" s="2" t="n">
+      <c r="F206" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G206" t="inlineStr">
@@ -12530,7 +12518,7 @@
           <t>96293</t>
         </is>
       </c>
-      <c r="F207" s="2" t="n">
+      <c r="F207" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G207" t="inlineStr">
@@ -12557,7 +12545,7 @@
         </is>
       </c>
       <c r="L207" t="inlineStr"/>
-      <c r="M207" s="2" t="n">
+      <c r="M207" s="1" t="n">
         <v>46153</v>
       </c>
       <c r="N207" t="inlineStr"/>
@@ -12592,7 +12580,7 @@
           <t>89287</t>
         </is>
       </c>
-      <c r="F208" s="2" t="n">
+      <c r="F208" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="G208" t="inlineStr">
@@ -12619,7 +12607,7 @@
         </is>
       </c>
       <c r="L208" t="inlineStr"/>
-      <c r="M208" s="2" t="n">
+      <c r="M208" s="1" t="n">
         <v>46031</v>
       </c>
       <c r="N208" t="inlineStr"/>
@@ -12654,7 +12642,7 @@
           <t>86805429</t>
         </is>
       </c>
-      <c r="F209" s="2" t="n">
+      <c r="F209" s="1" t="n">
         <v>46000</v>
       </c>
       <c r="G209" t="inlineStr">
@@ -12681,7 +12669,7 @@
         </is>
       </c>
       <c r="L209" t="inlineStr"/>
-      <c r="M209" s="2" t="n">
+      <c r="M209" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="N209" t="inlineStr"/>
@@ -12716,7 +12704,7 @@
           <t>073200G02170010AE</t>
         </is>
       </c>
-      <c r="F210" s="2" t="n">
+      <c r="F210" s="1" t="n">
         <v>46000</v>
       </c>
       <c r="G210" t="inlineStr">
@@ -12776,7 +12764,7 @@
           <t>073200G71030137AE</t>
         </is>
       </c>
-      <c r="F211" s="2" t="n">
+      <c r="F211" s="1" t="n">
         <v>46000</v>
       </c>
       <c r="G211" t="inlineStr">
@@ -12834,7 +12822,7 @@
           <t>073200G71360003AE</t>
         </is>
       </c>
-      <c r="F212" s="2" t="n">
+      <c r="F212" s="1" t="n">
         <v>46000</v>
       </c>
       <c r="G212" t="inlineStr">
@@ -12892,7 +12880,7 @@
           <t>01381310971</t>
         </is>
       </c>
-      <c r="F213" s="2" t="n">
+      <c r="F213" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="G213" t="inlineStr">
@@ -12952,7 +12940,7 @@
           <t>KC225-3029</t>
         </is>
       </c>
-      <c r="F214" s="2" t="n">
+      <c r="F214" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="G214" t="inlineStr">
@@ -12979,7 +12967,7 @@
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
-      <c r="M214" s="2" t="n">
+      <c r="M214" s="1" t="n">
         <v>46021</v>
       </c>
       <c r="N214" t="n">
@@ -13016,7 +13004,7 @@
           <t>1141111980</t>
         </is>
       </c>
-      <c r="F215" s="2" t="n">
+      <c r="F215" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="G215" t="inlineStr">
@@ -13076,7 +13064,7 @@
           <t>A-184434</t>
         </is>
       </c>
-      <c r="F216" s="2" t="n">
+      <c r="F216" s="1" t="n">
         <v>46010</v>
       </c>
       <c r="G216" t="inlineStr">
@@ -13126,7 +13114,7 @@
           <t>3201</t>
         </is>
       </c>
-      <c r="F217" s="2" t="n">
+      <c r="F217" s="1" t="n">
         <v>46010</v>
       </c>
       <c r="G217" t="inlineStr">
@@ -13153,7 +13141,7 @@
         </is>
       </c>
       <c r="L217" t="inlineStr"/>
-      <c r="M217" s="2" t="n">
+      <c r="M217" s="1" t="n">
         <v>46052</v>
       </c>
       <c r="N217" t="inlineStr"/>
@@ -13188,7 +13176,7 @@
           <t>A-183643</t>
         </is>
       </c>
-      <c r="F218" s="2" t="n">
+      <c r="F218" s="1" t="n">
         <v>46010</v>
       </c>
       <c r="G218" t="inlineStr">
@@ -13248,7 +13236,7 @@
           <t>A-180560</t>
         </is>
       </c>
-      <c r="F219" s="2" t="n">
+      <c r="F219" s="1" t="n">
         <v>46010</v>
       </c>
       <c r="G219" t="inlineStr">
@@ -13308,7 +13296,7 @@
           <t>A-134709</t>
         </is>
       </c>
-      <c r="F220" s="2" t="n">
+      <c r="F220" s="1" t="n">
         <v>46010</v>
       </c>
       <c r="G220" t="inlineStr">
@@ -13368,7 +13356,7 @@
           <t>822</t>
         </is>
       </c>
-      <c r="F221" s="2" t="n">
+      <c r="F221" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G221" t="inlineStr">
@@ -13426,7 +13414,7 @@
           <t>795</t>
         </is>
       </c>
-      <c r="F222" s="2" t="n">
+      <c r="F222" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G222" t="inlineStr">
@@ -13486,7 +13474,7 @@
           <t>784</t>
         </is>
       </c>
-      <c r="F223" s="2" t="n">
+      <c r="F223" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G223" t="inlineStr">
@@ -13546,7 +13534,7 @@
           <t>482</t>
         </is>
       </c>
-      <c r="F224" s="2" t="n">
+      <c r="F224" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G224" t="inlineStr">
@@ -13606,7 +13594,7 @@
           <t>LSEAM3218</t>
         </is>
       </c>
-      <c r="F225" s="2" t="n">
+      <c r="F225" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G225" t="inlineStr">
@@ -13666,7 +13654,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="F226" s="2" t="n">
+      <c r="F226" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G226" t="inlineStr">
@@ -13726,7 +13714,7 @@
           <t>LSEAM3167</t>
         </is>
       </c>
-      <c r="F227" s="2" t="n">
+      <c r="F227" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G227" t="inlineStr">
@@ -13786,7 +13774,7 @@
           <t>01B</t>
         </is>
       </c>
-      <c r="F228" s="2" t="n">
+      <c r="F228" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G228" t="inlineStr">
@@ -13846,7 +13834,7 @@
           <t>392-000003</t>
         </is>
       </c>
-      <c r="F229" s="2" t="n">
+      <c r="F229" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G229" t="inlineStr">
@@ -13904,7 +13892,7 @@
           <t>073200G90080062AE</t>
         </is>
       </c>
-      <c r="F230" s="2" t="n">
+      <c r="F230" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G230" t="inlineStr">
@@ -13964,7 +13952,7 @@
           <t>073200G02170087AE</t>
         </is>
       </c>
-      <c r="F231" s="2" t="n">
+      <c r="F231" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G231" t="inlineStr">
@@ -13991,7 +13979,7 @@
         </is>
       </c>
       <c r="L231" t="inlineStr"/>
-      <c r="M231" s="2" t="n">
+      <c r="M231" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="N231" t="inlineStr"/>
@@ -14026,7 +14014,7 @@
           <t>073200G02170089AE</t>
         </is>
       </c>
-      <c r="F232" s="2" t="n">
+      <c r="F232" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G232" t="inlineStr">
@@ -14084,7 +14072,7 @@
           <t>073200G63200008AE</t>
         </is>
       </c>
-      <c r="F233" s="2" t="n">
+      <c r="F233" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G233" t="inlineStr">
@@ -14142,7 +14130,7 @@
           <t>073200G02170034AE</t>
         </is>
       </c>
-      <c r="F234" s="2" t="n">
+      <c r="F234" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G234" t="inlineStr">
@@ -14169,7 +14157,7 @@
         </is>
       </c>
       <c r="L234" t="inlineStr"/>
-      <c r="M234" s="2" t="n">
+      <c r="M234" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="N234" t="inlineStr"/>
@@ -14208,7 +14196,7 @@
           <t>073200G90080045AE</t>
         </is>
       </c>
-      <c r="F235" s="2" t="n">
+      <c r="F235" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G235" t="inlineStr">
@@ -14235,7 +14223,7 @@
         </is>
       </c>
       <c r="L235" t="inlineStr"/>
-      <c r="M235" s="2" t="n">
+      <c r="M235" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="N235" t="inlineStr"/>
@@ -14274,7 +14262,7 @@
           <t>2165</t>
         </is>
       </c>
-      <c r="F236" s="2" t="n">
+      <c r="F236" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G236" t="inlineStr">
@@ -14301,7 +14289,7 @@
         </is>
       </c>
       <c r="L236" t="inlineStr"/>
-      <c r="M236" s="2" t="n">
+      <c r="M236" s="1" t="n">
         <v>46114</v>
       </c>
       <c r="N236" t="inlineStr"/>
@@ -14336,7 +14324,7 @@
           <t>1270</t>
         </is>
       </c>
-      <c r="F237" s="2" t="n">
+      <c r="F237" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G237" t="inlineStr">
@@ -14396,7 +14384,7 @@
           <t>B10274</t>
         </is>
       </c>
-      <c r="F238" s="2" t="n">
+      <c r="F238" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="G238" t="inlineStr">
@@ -14446,7 +14434,7 @@
           <t>F66933</t>
         </is>
       </c>
-      <c r="F239" s="2" t="n">
+      <c r="F239" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="G239" t="inlineStr">
@@ -14473,7 +14461,7 @@
         </is>
       </c>
       <c r="L239" t="inlineStr"/>
-      <c r="M239" s="2" t="n">
+      <c r="M239" s="1" t="n">
         <v>46052</v>
       </c>
       <c r="N239" t="inlineStr"/>
@@ -14508,7 +14496,7 @@
           <t>C66477</t>
         </is>
       </c>
-      <c r="F240" s="2" t="n">
+      <c r="F240" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="G240" t="inlineStr">
@@ -14566,7 +14554,7 @@
           <t>A76103</t>
         </is>
       </c>
-      <c r="F241" s="2" t="n">
+      <c r="F241" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="G241" t="inlineStr">
@@ -14624,7 +14612,7 @@
           <t>B10380</t>
         </is>
       </c>
-      <c r="F242" s="2" t="n">
+      <c r="F242" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="G242" t="inlineStr">
@@ -14684,7 +14672,7 @@
           <t>6949</t>
         </is>
       </c>
-      <c r="F243" s="2" t="n">
+      <c r="F243" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="G243" t="inlineStr">
@@ -14738,7 +14726,7 @@
           <t>24277</t>
         </is>
       </c>
-      <c r="F244" s="2" t="n">
+      <c r="F244" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="G244" t="inlineStr">
@@ -14798,7 +14786,7 @@
           <t>22102</t>
         </is>
       </c>
-      <c r="F245" s="2" t="n">
+      <c r="F245" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="G245" t="inlineStr">
@@ -14858,7 +14846,7 @@
           <t>002798</t>
         </is>
       </c>
-      <c r="F246" s="2" t="n">
+      <c r="F246" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="G246" t="inlineStr">
@@ -14885,7 +14873,7 @@
         </is>
       </c>
       <c r="L246" t="inlineStr"/>
-      <c r="M246" s="2" t="n">
+      <c r="M246" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="N246" t="inlineStr"/>
@@ -14920,7 +14908,7 @@
           <t>004106</t>
         </is>
       </c>
-      <c r="F247" s="2" t="n">
+      <c r="F247" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="G247" t="inlineStr">
@@ -14970,7 +14958,7 @@
           <t>968</t>
         </is>
       </c>
-      <c r="F248" s="2" t="n">
+      <c r="F248" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="G248" t="inlineStr">
@@ -15020,7 +15008,7 @@
           <t>2L094</t>
         </is>
       </c>
-      <c r="F249" s="2" t="n">
+      <c r="F249" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="G249" t="inlineStr">
@@ -15080,7 +15068,7 @@
           <t>003665</t>
         </is>
       </c>
-      <c r="F250" s="2" t="n">
+      <c r="F250" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G250" t="inlineStr">
@@ -15140,7 +15128,7 @@
           <t>004201</t>
         </is>
       </c>
-      <c r="F251" s="2" t="n">
+      <c r="F251" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G251" t="inlineStr">
@@ -15198,7 +15186,7 @@
           <t>004207</t>
         </is>
       </c>
-      <c r="F252" s="2" t="n">
+      <c r="F252" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G252" t="inlineStr">
@@ -15256,7 +15244,7 @@
           <t>1656</t>
         </is>
       </c>
-      <c r="F253" s="2" t="n">
+      <c r="F253" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G253" t="inlineStr">
@@ -15316,7 +15304,7 @@
           <t>T49314</t>
         </is>
       </c>
-      <c r="F254" s="2" t="n">
+      <c r="F254" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G254" t="inlineStr">
@@ -15376,7 +15364,7 @@
           <t>T49816</t>
         </is>
       </c>
-      <c r="F255" s="2" t="n">
+      <c r="F255" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G255" t="inlineStr">
@@ -15436,7 +15424,7 @@
           <t>46710866</t>
         </is>
       </c>
-      <c r="F256" s="2" t="n">
+      <c r="F256" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G256" t="inlineStr">
@@ -15498,7 +15486,7 @@
           <t>20624851</t>
         </is>
       </c>
-      <c r="F257" s="2" t="n">
+      <c r="F257" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G257" t="inlineStr">
@@ -15548,7 +15536,7 @@
           <t>20625310</t>
         </is>
       </c>
-      <c r="F258" s="2" t="n">
+      <c r="F258" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G258" t="inlineStr">
@@ -15598,7 +15586,7 @@
           <t>2926</t>
         </is>
       </c>
-      <c r="F259" s="2" t="n">
+      <c r="F259" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G259" t="inlineStr">
@@ -15658,7 +15646,7 @@
           <t>12023</t>
         </is>
       </c>
-      <c r="F260" s="2" t="n">
+      <c r="F260" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G260" t="inlineStr">
@@ -15718,7 +15706,7 @@
           <t>KAS297B-A23223</t>
         </is>
       </c>
-      <c r="F261" s="2" t="n">
+      <c r="F261" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G261" t="inlineStr">
@@ -15778,7 +15766,7 @@
           <t>42966</t>
         </is>
       </c>
-      <c r="F262" s="2" t="n">
+      <c r="F262" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G262" t="inlineStr">
@@ -15805,7 +15793,7 @@
         </is>
       </c>
       <c r="L262" t="inlineStr"/>
-      <c r="M262" s="2" t="n">
+      <c r="M262" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="N262" t="inlineStr"/>
@@ -15844,7 +15832,7 @@
           <t>48741</t>
         </is>
       </c>
-      <c r="F263" s="2" t="n">
+      <c r="F263" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G263" t="inlineStr">
@@ -15902,7 +15890,7 @@
           <t>21940</t>
         </is>
       </c>
-      <c r="F264" s="2" t="n">
+      <c r="F264" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G264" t="inlineStr">
@@ -15962,7 +15950,7 @@
           <t>22950</t>
         </is>
       </c>
-      <c r="F265" s="2" t="n">
+      <c r="F265" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G265" t="inlineStr">
@@ -16022,7 +16010,7 @@
           <t>7310</t>
         </is>
       </c>
-      <c r="F266" s="2" t="n">
+      <c r="F266" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G266" t="inlineStr">
@@ -16082,7 +16070,7 @@
           <t>11154</t>
         </is>
       </c>
-      <c r="F267" s="2" t="n">
+      <c r="F267" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G267" t="inlineStr">
@@ -16142,7 +16130,7 @@
           <t>17714</t>
         </is>
       </c>
-      <c r="F268" s="2" t="n">
+      <c r="F268" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G268" t="inlineStr">
@@ -16198,7 +16186,7 @@
         </is>
       </c>
       <c r="E269" t="inlineStr"/>
-      <c r="F269" s="2" t="n">
+      <c r="F269" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G269" t="inlineStr">
@@ -16258,7 +16246,7 @@
           <t>KTA77B-A87365</t>
         </is>
       </c>
-      <c r="F270" s="2" t="n">
+      <c r="F270" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G270" t="inlineStr">
@@ -16318,7 +16306,7 @@
           <t>8306</t>
         </is>
       </c>
-      <c r="F271" s="2" t="n">
+      <c r="F271" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G271" t="inlineStr">
@@ -16378,7 +16366,7 @@
           <t>5BE34</t>
         </is>
       </c>
-      <c r="F272" s="2" t="n">
+      <c r="F272" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G272" t="inlineStr">
@@ -16405,7 +16393,7 @@
         </is>
       </c>
       <c r="L272" t="inlineStr"/>
-      <c r="M272" s="2" t="n">
+      <c r="M272" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="N272" t="inlineStr">
@@ -16444,7 +16432,7 @@
           <t>S4H004</t>
         </is>
       </c>
-      <c r="F273" s="2" t="n">
+      <c r="F273" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G273" t="inlineStr">
@@ -16502,7 +16490,7 @@
           <t>0919</t>
         </is>
       </c>
-      <c r="F274" s="2" t="n">
+      <c r="F274" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G274" t="inlineStr">
@@ -16562,7 +16550,7 @@
           <t>B4H-015</t>
         </is>
       </c>
-      <c r="F275" s="2" t="n">
+      <c r="F275" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G275" t="inlineStr">
@@ -16620,7 +16608,7 @@
           <t>B4H-011</t>
         </is>
       </c>
-      <c r="F276" s="2" t="n">
+      <c r="F276" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G276" t="inlineStr">
@@ -16680,7 +16668,7 @@
           <t>20675473</t>
         </is>
       </c>
-      <c r="F277" s="2" t="n">
+      <c r="F277" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="G277" t="inlineStr">
@@ -16740,7 +16728,7 @@
           <t>470055</t>
         </is>
       </c>
-      <c r="F278" s="2" t="n">
+      <c r="F278" s="1" t="n">
         <v>46077</v>
       </c>
       <c r="G278" t="inlineStr">
@@ -16800,7 +16788,7 @@
           <t>471591</t>
         </is>
       </c>
-      <c r="F279" s="2" t="n">
+      <c r="F279" s="1" t="n">
         <v>46077</v>
       </c>
       <c r="G279" t="inlineStr">
@@ -16864,7 +16852,7 @@
           <t>8868</t>
         </is>
       </c>
-      <c r="F280" s="2" t="n">
+      <c r="F280" s="1" t="n">
         <v>46085</v>
       </c>
       <c r="G280" t="inlineStr">
@@ -16924,7 +16912,7 @@
           <t>4965</t>
         </is>
       </c>
-      <c r="F281" s="2" t="n">
+      <c r="F281" s="1" t="n">
         <v>46085</v>
       </c>
       <c r="G281" t="inlineStr">
@@ -16984,7 +16972,7 @@
           <t>000745</t>
         </is>
       </c>
-      <c r="F282" s="2" t="n">
+      <c r="F282" s="1" t="n">
         <v>46090</v>
       </c>
       <c r="G282" t="inlineStr">
@@ -17042,7 +17030,7 @@
           <t>8459XL2</t>
         </is>
       </c>
-      <c r="F283" s="2" t="n">
+      <c r="F283" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="G283" t="inlineStr">
@@ -17098,7 +17086,7 @@
           <t>S00062XL</t>
         </is>
       </c>
-      <c r="F284" s="2" t="n">
+      <c r="F284" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="G284" t="inlineStr">
@@ -17154,7 +17142,7 @@
           <t>073200G02170082AE</t>
         </is>
       </c>
-      <c r="F285" s="2" t="n">
+      <c r="F285" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="G285" t="inlineStr">
@@ -17210,7 +17198,7 @@
           <t>073200G91260061AE</t>
         </is>
       </c>
-      <c r="F286" s="2" t="n">
+      <c r="F286" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="G286" t="inlineStr">
@@ -17264,7 +17252,7 @@
       <c r="E287" t="n">
         <v>35971</v>
       </c>
-      <c r="F287" s="2" t="n">
+      <c r="F287" s="1" t="n">
         <v>46107</v>
       </c>
       <c r="G287" t="inlineStr">
@@ -17310,7 +17298,7 @@
       <c r="E288" t="n">
         <v>107178</v>
       </c>
-      <c r="F288" s="2" t="n">
+      <c r="F288" s="1" t="n">
         <v>46107</v>
       </c>
       <c r="G288" t="inlineStr">
@@ -17366,7 +17354,7 @@
       <c r="E289" t="n">
         <v>108773</v>
       </c>
-      <c r="F289" s="2" t="n">
+      <c r="F289" s="1" t="n">
         <v>46107</v>
       </c>
       <c r="G289" t="inlineStr">
@@ -17414,7 +17402,7 @@
       <c r="E290" t="n">
         <v>7086</v>
       </c>
-      <c r="F290" s="2" t="n">
+      <c r="F290" s="1" t="n">
         <v>46107</v>
       </c>
       <c r="G290" t="inlineStr">
@@ -17437,7 +17425,7 @@
       </c>
       <c r="K290" t="inlineStr"/>
       <c r="L290" t="inlineStr"/>
-      <c r="M290" s="2" t="n">
+      <c r="M290" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="N290" t="inlineStr"/>
@@ -17468,7 +17456,7 @@
       <c r="E291" t="n">
         <v>99743</v>
       </c>
-      <c r="F291" s="2" t="n">
+      <c r="F291" s="1" t="n">
         <v>46107</v>
       </c>
       <c r="G291" t="inlineStr">
@@ -17526,7 +17514,7 @@
           <t>KS272A-49392</t>
         </is>
       </c>
-      <c r="F292" s="2" t="n">
+      <c r="F292" s="1" t="n">
         <v>46112</v>
       </c>
       <c r="G292" t="inlineStr">
@@ -17584,7 +17572,7 @@
           <t>B-10811222</t>
         </is>
       </c>
-      <c r="F293" s="2" t="n">
+      <c r="F293" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G293" t="inlineStr">
@@ -17642,7 +17630,7 @@
           <t>B10811221</t>
         </is>
       </c>
-      <c r="F294" s="2" t="n">
+      <c r="F294" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G294" t="inlineStr">
@@ -17696,7 +17684,7 @@
           <t>B10811220</t>
         </is>
       </c>
-      <c r="F295" s="2" t="n">
+      <c r="F295" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G295" t="inlineStr">
@@ -17750,7 +17738,7 @@
           <t>B10811724</t>
         </is>
       </c>
-      <c r="F296" s="2" t="n">
+      <c r="F296" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G296" t="inlineStr">
@@ -17804,7 +17792,7 @@
       <c r="E297" t="n">
         <v>47203152</v>
       </c>
-      <c r="F297" s="2" t="n">
+      <c r="F297" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G297" t="inlineStr">
@@ -17862,7 +17850,7 @@
       <c r="E298" t="n">
         <v>47202512</v>
       </c>
-      <c r="F298" s="2" t="n">
+      <c r="F298" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G298" t="inlineStr">
@@ -17920,7 +17908,7 @@
       <c r="E299" t="n">
         <v>22005580</v>
       </c>
-      <c r="F299" s="2" t="n">
+      <c r="F299" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G299" t="inlineStr">
@@ -17978,7 +17966,7 @@
       <c r="E300" t="n">
         <v>22005955</v>
       </c>
-      <c r="F300" s="2" t="n">
+      <c r="F300" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G300" t="inlineStr">
@@ -18036,7 +18024,7 @@
       <c r="E301" t="n">
         <v>22005661</v>
       </c>
-      <c r="F301" s="2" t="n">
+      <c r="F301" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G301" t="inlineStr">
@@ -18092,7 +18080,7 @@
       <c r="E302" t="n">
         <v>32207</v>
       </c>
-      <c r="F302" s="2" t="n">
+      <c r="F302" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G302" t="inlineStr">
@@ -18148,7 +18136,7 @@
       <c r="E303" t="n">
         <v>18156</v>
       </c>
-      <c r="F303" s="2" t="n">
+      <c r="F303" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G303" t="inlineStr">
@@ -18204,7 +18192,7 @@
       <c r="E304" t="n">
         <v>37971</v>
       </c>
-      <c r="F304" s="2" t="n">
+      <c r="F304" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G304" t="inlineStr">
@@ -18260,7 +18248,7 @@
       <c r="E305" t="n">
         <v>84317</v>
       </c>
-      <c r="F305" s="2" t="n">
+      <c r="F305" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G305" t="inlineStr">
@@ -18287,7 +18275,7 @@
         </is>
       </c>
       <c r="L305" t="inlineStr"/>
-      <c r="M305" s="2" t="n">
+      <c r="M305" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="N305" t="inlineStr"/>
@@ -18318,7 +18306,7 @@
       <c r="E306" t="n">
         <v>83773</v>
       </c>
-      <c r="F306" s="2" t="n">
+      <c r="F306" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G306" t="inlineStr">
@@ -18345,7 +18333,7 @@
         </is>
       </c>
       <c r="L306" t="inlineStr"/>
-      <c r="M306" s="2" t="n">
+      <c r="M306" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="N306" t="inlineStr"/>
@@ -18376,7 +18364,7 @@
       <c r="E307" t="n">
         <v>83740</v>
       </c>
-      <c r="F307" s="2" t="n">
+      <c r="F307" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G307" t="inlineStr">
@@ -18432,7 +18420,7 @@
       <c r="E308" t="n">
         <v>84326</v>
       </c>
-      <c r="F308" s="2" t="n">
+      <c r="F308" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G308" t="inlineStr">
@@ -18488,7 +18476,7 @@
       <c r="E309" t="n">
         <v>6708</v>
       </c>
-      <c r="F309" s="2" t="n">
+      <c r="F309" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G309" t="inlineStr">
@@ -18546,7 +18534,7 @@
           <t>LSEAM3269</t>
         </is>
       </c>
-      <c r="F310" s="2" t="n">
+      <c r="F310" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G310" t="inlineStr">
@@ -18602,7 +18590,7 @@
       <c r="E311" t="n">
         <v>9727</v>
       </c>
-      <c r="F311" s="2" t="n">
+      <c r="F311" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G311" t="inlineStr">
@@ -18660,7 +18648,7 @@
           <t>LSEAM3168</t>
         </is>
       </c>
-      <c r="F312" s="2" t="n">
+      <c r="F312" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G312" t="inlineStr">
@@ -18716,7 +18704,7 @@
       <c r="E313" t="n">
         <v>31</v>
       </c>
-      <c r="F313" s="2" t="n">
+      <c r="F313" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G313" t="inlineStr">
@@ -18770,7 +18758,7 @@
       <c r="E314" t="n">
         <v>965</v>
       </c>
-      <c r="F314" s="2" t="n">
+      <c r="F314" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G314" t="inlineStr">
@@ -18826,7 +18814,7 @@
       <c r="E315" t="n">
         <v>2007</v>
       </c>
-      <c r="F315" s="2" t="n">
+      <c r="F315" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G315" t="inlineStr">
@@ -18882,7 +18870,7 @@
       <c r="E316" t="n">
         <v>688</v>
       </c>
-      <c r="F316" s="2" t="n">
+      <c r="F316" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G316" t="inlineStr">
@@ -18940,7 +18928,7 @@
           <t>B4H-038</t>
         </is>
       </c>
-      <c r="F317" s="2" t="n">
+      <c r="F317" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G317" t="inlineStr">
@@ -18998,7 +18986,7 @@
           <t>1938-XL</t>
         </is>
       </c>
-      <c r="F318" s="2" t="n">
+      <c r="F318" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G318" t="inlineStr">
@@ -19046,7 +19034,7 @@
           <t>3711XL</t>
         </is>
       </c>
-      <c r="F319" s="2" t="n">
+      <c r="F319" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G319" t="inlineStr">
@@ -19071,7 +19059,7 @@
         </is>
       </c>
       <c r="L319" t="inlineStr"/>
-      <c r="M319" s="2" t="n">
+      <c r="M319" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="N319" t="inlineStr"/>
@@ -19102,7 +19090,7 @@
       <c r="E320" t="n">
         <v>1391</v>
       </c>
-      <c r="F320" s="2" t="n">
+      <c r="F320" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G320" t="inlineStr">
@@ -19160,7 +19148,7 @@
       <c r="E321" t="n">
         <v>120315</v>
       </c>
-      <c r="F321" s="2" t="n">
+      <c r="F321" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G321" t="inlineStr">
@@ -19220,7 +19208,7 @@
           <t>1588-5</t>
         </is>
       </c>
-      <c r="F322" s="2" t="n">
+      <c r="F322" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G322" t="inlineStr">
@@ -19247,7 +19235,7 @@
         </is>
       </c>
       <c r="L322" t="inlineStr"/>
-      <c r="M322" s="2" t="n">
+      <c r="M322" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="N322" t="inlineStr"/>
@@ -19280,7 +19268,7 @@
       <c r="E323" t="n">
         <v>535933</v>
       </c>
-      <c r="F323" s="2" t="n">
+      <c r="F323" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G323" t="inlineStr">
@@ -19338,7 +19326,7 @@
       <c r="E324" t="n">
         <v>289029</v>
       </c>
-      <c r="F324" s="2" t="n">
+      <c r="F324" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G324" t="inlineStr">
@@ -19396,7 +19384,7 @@
       <c r="E325" t="n">
         <v>3454</v>
       </c>
-      <c r="F325" s="2" t="n">
+      <c r="F325" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G325" t="inlineStr">
@@ -19423,7 +19411,7 @@
         </is>
       </c>
       <c r="L325" t="inlineStr"/>
-      <c r="M325" s="2" t="n">
+      <c r="M325" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="N325" t="inlineStr"/>
@@ -19456,7 +19444,7 @@
       <c r="E326" t="n">
         <v>3493</v>
       </c>
-      <c r="F326" s="2" t="n">
+      <c r="F326" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G326" t="inlineStr">
@@ -19516,7 +19504,7 @@
           <t>1588-5</t>
         </is>
       </c>
-      <c r="F327" s="2" t="n">
+      <c r="F327" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G327" t="inlineStr">
@@ -19543,7 +19531,7 @@
         </is>
       </c>
       <c r="L327" t="inlineStr"/>
-      <c r="M327" s="2" t="n">
+      <c r="M327" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="N327" t="inlineStr"/>
@@ -19576,7 +19564,7 @@
       <c r="E328" t="n">
         <v>3235</v>
       </c>
-      <c r="F328" s="2" t="n">
+      <c r="F328" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G328" t="inlineStr">
@@ -19603,7 +19591,7 @@
         </is>
       </c>
       <c r="L328" t="inlineStr"/>
-      <c r="M328" s="2" t="n">
+      <c r="M328" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="N328" t="inlineStr"/>
@@ -19636,7 +19624,7 @@
       <c r="E329" t="n">
         <v>625052</v>
       </c>
-      <c r="F329" s="2" t="n">
+      <c r="F329" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G329" t="inlineStr">
@@ -19663,7 +19651,7 @@
         </is>
       </c>
       <c r="L329" t="inlineStr"/>
-      <c r="M329" s="2" t="n">
+      <c r="M329" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="N329" t="inlineStr"/>
@@ -19696,7 +19684,7 @@
       <c r="E330" t="n">
         <v>614095</v>
       </c>
-      <c r="F330" s="2" t="n">
+      <c r="F330" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G330" t="inlineStr">
@@ -19723,7 +19711,7 @@
         </is>
       </c>
       <c r="L330" t="inlineStr"/>
-      <c r="M330" s="2" t="n">
+      <c r="M330" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="N330" t="inlineStr"/>
@@ -19756,7 +19744,7 @@
           <t>B10274</t>
         </is>
       </c>
-      <c r="F331" s="2" t="n">
+      <c r="F331" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G331" t="inlineStr">
@@ -19814,7 +19802,7 @@
           <t>9715-096</t>
         </is>
       </c>
-      <c r="F332" s="2" t="n">
+      <c r="F332" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G332" t="inlineStr">
@@ -19870,7 +19858,7 @@
       <c r="E333" t="n">
         <v>197</v>
       </c>
-      <c r="F333" s="2" t="n">
+      <c r="F333" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G333" t="inlineStr">
@@ -19926,7 +19914,7 @@
       <c r="E334" t="n">
         <v>1378</v>
       </c>
-      <c r="F334" s="2" t="n">
+      <c r="F334" s="1" t="n">
         <v>46125</v>
       </c>
       <c r="G334" t="inlineStr">
@@ -19986,7 +19974,7 @@
           <t>ATE2717</t>
         </is>
       </c>
-      <c r="F335" s="2" t="n">
+      <c r="F335" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="G335" t="inlineStr">
@@ -20011,7 +19999,7 @@
         </is>
       </c>
       <c r="L335" t="inlineStr"/>
-      <c r="M335" s="2" t="n">
+      <c r="M335" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="N335" t="inlineStr"/>
@@ -20046,7 +20034,7 @@
           <t>LS005</t>
         </is>
       </c>
-      <c r="F336" s="2" t="n">
+      <c r="F336" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="G336" t="inlineStr">
@@ -20106,7 +20094,7 @@
           <t>ATE2714</t>
         </is>
       </c>
-      <c r="F337" s="2" t="n">
+      <c r="F337" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="G337" t="inlineStr">
@@ -20131,7 +20119,7 @@
         </is>
       </c>
       <c r="L337" t="inlineStr"/>
-      <c r="M337" s="2" t="n">
+      <c r="M337" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="N337" t="inlineStr"/>
@@ -20166,7 +20154,7 @@
           <t>ATE2730</t>
         </is>
       </c>
-      <c r="F338" s="2" t="n">
+      <c r="F338" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="G338" t="inlineStr">
@@ -20222,7 +20210,7 @@
       <c r="E339" t="n">
         <v>6291</v>
       </c>
-      <c r="F339" s="2" t="n">
+      <c r="F339" s="1" t="n">
         <v>46129</v>
       </c>
       <c r="G339" t="inlineStr">
@@ -20272,7 +20260,7 @@
           <t>1062</t>
         </is>
       </c>
-      <c r="F340" s="2" t="n">
+      <c r="F340" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G340" t="inlineStr">
@@ -20332,7 +20320,7 @@
           <t>8619</t>
         </is>
       </c>
-      <c r="F341" s="2" t="n">
+      <c r="F341" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G341" t="inlineStr">
@@ -20392,7 +20380,7 @@
           <t>4136</t>
         </is>
       </c>
-      <c r="F342" s="2" t="n">
+      <c r="F342" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G342" t="inlineStr">
@@ -20452,7 +20440,7 @@
           <t>T35158</t>
         </is>
       </c>
-      <c r="F343" s="2" t="n">
+      <c r="F343" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G343" t="inlineStr">
@@ -20512,7 +20500,7 @@
           <t>T35507</t>
         </is>
       </c>
-      <c r="F344" s="2" t="n">
+      <c r="F344" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G344" t="inlineStr">
@@ -20572,7 +20560,7 @@
           <t>20238</t>
         </is>
       </c>
-      <c r="F345" s="2" t="n">
+      <c r="F345" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G345" t="inlineStr">
@@ -20632,7 +20620,7 @@
           <t>102549</t>
         </is>
       </c>
-      <c r="F346" s="2" t="n">
+      <c r="F346" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G346" t="inlineStr">
@@ -20692,7 +20680,7 @@
           <t>16784</t>
         </is>
       </c>
-      <c r="F347" s="2" t="n">
+      <c r="F347" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G347" t="inlineStr">
@@ -20719,7 +20707,7 @@
         </is>
       </c>
       <c r="L347" t="inlineStr"/>
-      <c r="M347" s="2" t="n">
+      <c r="M347" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="N347" t="inlineStr"/>
@@ -20754,7 +20742,7 @@
           <t>16810</t>
         </is>
       </c>
-      <c r="F348" s="2" t="n">
+      <c r="F348" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G348" t="inlineStr">
@@ -20781,7 +20769,7 @@
         </is>
       </c>
       <c r="L348" t="inlineStr"/>
-      <c r="M348" s="2" t="n">
+      <c r="M348" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="N348" t="inlineStr"/>
@@ -20816,7 +20804,7 @@
           <t>108207</t>
         </is>
       </c>
-      <c r="F349" s="2" t="n">
+      <c r="F349" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G349" t="inlineStr">
@@ -20876,7 +20864,7 @@
           <t>4152</t>
         </is>
       </c>
-      <c r="F350" s="2" t="n">
+      <c r="F350" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G350" t="inlineStr">
@@ -20932,7 +20920,7 @@
           <t>96123</t>
         </is>
       </c>
-      <c r="F351" s="2" t="n">
+      <c r="F351" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G351" t="inlineStr">
@@ -20992,7 +20980,7 @@
           <t>4100932</t>
         </is>
       </c>
-      <c r="F352" s="2" t="n">
+      <c r="F352" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G352" t="inlineStr">
@@ -21052,7 +21040,7 @@
           <t>T36593</t>
         </is>
       </c>
-      <c r="F353" s="2" t="n">
+      <c r="F353" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G353" t="inlineStr">
@@ -21112,7 +21100,7 @@
           <t>30316</t>
         </is>
       </c>
-      <c r="F354" s="2" t="n">
+      <c r="F354" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G354" t="inlineStr">
@@ -21172,7 +21160,7 @@
           <t>4155</t>
         </is>
       </c>
-      <c r="F355" s="2" t="n">
+      <c r="F355" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G355" t="inlineStr">
@@ -21199,7 +21187,7 @@
         </is>
       </c>
       <c r="L355" t="inlineStr"/>
-      <c r="M355" s="2" t="n">
+      <c r="M355" s="1" t="n">
         <v>46150</v>
       </c>
       <c r="N355" t="inlineStr"/>
@@ -21234,7 +21222,7 @@
           <t>18685</t>
         </is>
       </c>
-      <c r="F356" s="2" t="n">
+      <c r="F356" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G356" t="inlineStr">
@@ -21259,7 +21247,7 @@
         </is>
       </c>
       <c r="L356" t="inlineStr"/>
-      <c r="M356" s="2" t="n">
+      <c r="M356" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="N356" t="inlineStr"/>
@@ -21294,7 +21282,7 @@
           <t>86815595</t>
         </is>
       </c>
-      <c r="F357" s="2" t="n">
+      <c r="F357" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G357" t="inlineStr">
@@ -21354,7 +21342,7 @@
           <t>86816588</t>
         </is>
       </c>
-      <c r="F358" s="2" t="n">
+      <c r="F358" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G358" t="inlineStr">
@@ -21414,7 +21402,7 @@
           <t>86815646</t>
         </is>
       </c>
-      <c r="F359" s="2" t="n">
+      <c r="F359" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G359" t="inlineStr">
@@ -21474,7 +21462,7 @@
           <t>T23740</t>
         </is>
       </c>
-      <c r="F360" s="2" t="n">
+      <c r="F360" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G360" t="inlineStr">
@@ -21534,7 +21522,7 @@
           <t>T20503</t>
         </is>
       </c>
-      <c r="F361" s="2" t="n">
+      <c r="F361" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G361" t="inlineStr">
@@ -21594,7 +21582,7 @@
           <t>T23036</t>
         </is>
       </c>
-      <c r="F362" s="2" t="n">
+      <c r="F362" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G362" t="inlineStr">
@@ -21654,7 +21642,7 @@
           <t>T25488</t>
         </is>
       </c>
-      <c r="F363" s="2" t="n">
+      <c r="F363" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G363" t="inlineStr">
@@ -21714,7 +21702,7 @@
           <t>T22974</t>
         </is>
       </c>
-      <c r="F364" s="2" t="n">
+      <c r="F364" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G364" t="inlineStr">
@@ -21774,7 +21762,7 @@
           <t>4112112</t>
         </is>
       </c>
-      <c r="F365" s="2" t="n">
+      <c r="F365" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="G365" t="inlineStr">
@@ -21834,7 +21822,7 @@
           <t>30559</t>
         </is>
       </c>
-      <c r="F366" s="2" t="n">
+      <c r="F366" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G366" t="inlineStr">
@@ -21894,7 +21882,7 @@
           <t>34851</t>
         </is>
       </c>
-      <c r="F367" s="2" t="n">
+      <c r="F367" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G367" t="inlineStr">
@@ -21954,7 +21942,7 @@
           <t>3958</t>
         </is>
       </c>
-      <c r="F368" s="2" t="n">
+      <c r="F368" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G368" t="inlineStr">
@@ -22014,7 +22002,7 @@
           <t>4157</t>
         </is>
       </c>
-      <c r="F369" s="2" t="n">
+      <c r="F369" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G369" t="inlineStr">
@@ -22074,7 +22062,7 @@
           <t>2913</t>
         </is>
       </c>
-      <c r="F370" s="2" t="n">
+      <c r="F370" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G370" t="inlineStr">
@@ -22134,7 +22122,7 @@
           <t>4129</t>
         </is>
       </c>
-      <c r="F371" s="2" t="n">
+      <c r="F371" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G371" t="inlineStr">
@@ -22161,7 +22149,7 @@
         </is>
       </c>
       <c r="L371" t="inlineStr"/>
-      <c r="M371" s="2" t="n">
+      <c r="M371" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="N371" t="inlineStr"/>
@@ -22196,7 +22184,7 @@
           <t>KI525A-B100660</t>
         </is>
       </c>
-      <c r="F372" s="2" t="n">
+      <c r="F372" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="G372" t="inlineStr">
@@ -22223,7 +22211,7 @@
         </is>
       </c>
       <c r="L372" t="inlineStr"/>
-      <c r="M372" s="2" t="n">
+      <c r="M372" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="N372" t="inlineStr"/>
@@ -22262,7 +22250,7 @@
           <t>C66508</t>
         </is>
       </c>
-      <c r="F373" s="2" t="n">
+      <c r="F373" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="G373" t="inlineStr">
@@ -22322,7 +22310,7 @@
           <t>C66698</t>
         </is>
       </c>
-      <c r="F374" s="2" t="n">
+      <c r="F374" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="G374" t="inlineStr">
@@ -22382,7 +22370,7 @@
           <t>35511</t>
         </is>
       </c>
-      <c r="F375" s="2" t="n">
+      <c r="F375" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G375" t="inlineStr">
@@ -22442,7 +22430,7 @@
           <t>85023</t>
         </is>
       </c>
-      <c r="F376" s="2" t="n">
+      <c r="F376" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G376" t="inlineStr">
@@ -22502,7 +22490,7 @@
           <t>64318</t>
         </is>
       </c>
-      <c r="F377" s="2" t="n">
+      <c r="F377" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G377" t="inlineStr">
@@ -22566,7 +22554,7 @@
           <t>83287</t>
         </is>
       </c>
-      <c r="F378" s="2" t="n">
+      <c r="F378" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G378" t="inlineStr">
@@ -22626,7 +22614,7 @@
           <t>25424</t>
         </is>
       </c>
-      <c r="F379" s="2" t="n">
+      <c r="F379" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G379" t="inlineStr">
@@ -22653,7 +22641,7 @@
         </is>
       </c>
       <c r="L379" t="inlineStr"/>
-      <c r="M379" s="2" t="n">
+      <c r="M379" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="N379" t="inlineStr"/>
@@ -22688,7 +22676,7 @@
           <t>24970</t>
         </is>
       </c>
-      <c r="F380" s="2" t="n">
+      <c r="F380" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G380" t="inlineStr">
@@ -22748,7 +22736,7 @@
           <t>21156</t>
         </is>
       </c>
-      <c r="F381" s="2" t="n">
+      <c r="F381" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G381" t="inlineStr">
@@ -22808,7 +22796,7 @@
           <t>1652</t>
         </is>
       </c>
-      <c r="F382" s="2" t="n">
+      <c r="F382" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G382" t="inlineStr">
@@ -22868,7 +22856,7 @@
           <t>1713</t>
         </is>
       </c>
-      <c r="F383" s="2" t="n">
+      <c r="F383" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="G383" t="inlineStr">
@@ -22928,7 +22916,7 @@
           <t>1328-5</t>
         </is>
       </c>
-      <c r="F384" s="2" t="n">
+      <c r="F384" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="G384" t="inlineStr">
@@ -22988,7 +22976,7 @@
           <t>2309-5</t>
         </is>
       </c>
-      <c r="F385" s="2" t="n">
+      <c r="F385" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="G385" t="inlineStr">
@@ -23048,7 +23036,7 @@
           <t>4154</t>
         </is>
       </c>
-      <c r="F386" s="2" t="n">
+      <c r="F386" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G386" t="inlineStr">
@@ -23108,7 +23096,7 @@
           <t>4164</t>
         </is>
       </c>
-      <c r="F387" s="2" t="n">
+      <c r="F387" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G387" t="inlineStr">
@@ -23168,7 +23156,7 @@
           <t>17143</t>
         </is>
       </c>
-      <c r="F388" s="2" t="n">
+      <c r="F388" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G388" t="inlineStr">
@@ -23228,7 +23216,7 @@
           <t>3391XL</t>
         </is>
       </c>
-      <c r="F389" s="2" t="n">
+      <c r="F389" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G389" t="inlineStr">
@@ -23288,7 +23276,7 @@
           <t>S00007XL</t>
         </is>
       </c>
-      <c r="F390" s="2" t="n">
+      <c r="F390" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G390" t="inlineStr">
@@ -23315,7 +23303,7 @@
         </is>
       </c>
       <c r="L390" t="inlineStr"/>
-      <c r="M390" s="2" t="n">
+      <c r="M390" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="N390" t="inlineStr"/>
@@ -23350,7 +23338,7 @@
           <t>C66691</t>
         </is>
       </c>
-      <c r="F391" s="2" t="n">
+      <c r="F391" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G391" t="inlineStr">
@@ -23414,7 +23402,7 @@
           <t>9933-49</t>
         </is>
       </c>
-      <c r="F392" s="2" t="n">
+      <c r="F392" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G392" t="inlineStr">
@@ -23439,7 +23427,7 @@
         </is>
       </c>
       <c r="L392" t="inlineStr"/>
-      <c r="M392" s="2" t="n">
+      <c r="M392" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="N392" t="inlineStr"/>
@@ -23474,7 +23462,7 @@
           <t>0612</t>
         </is>
       </c>
-      <c r="F393" s="2" t="n">
+      <c r="F393" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G393" t="inlineStr">
@@ -23534,7 +23522,7 @@
           <t>070407910680166AE</t>
         </is>
       </c>
-      <c r="F394" s="2" t="n">
+      <c r="F394" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G394" t="inlineStr">
@@ -23594,7 +23582,7 @@
           <t>070407983320094AE</t>
         </is>
       </c>
-      <c r="F395" s="2" t="n">
+      <c r="F395" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G395" t="inlineStr">
@@ -23654,7 +23642,7 @@
           <t>070407983320096AE</t>
         </is>
       </c>
-      <c r="F396" s="2" t="n">
+      <c r="F396" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G396" t="inlineStr">
@@ -23714,7 +23702,7 @@
           <t>070407983320111AE</t>
         </is>
       </c>
-      <c r="F397" s="2" t="n">
+      <c r="F397" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G397" t="inlineStr">
@@ -23774,7 +23762,7 @@
           <t>070407983320130AE</t>
         </is>
       </c>
-      <c r="F398" s="2" t="n">
+      <c r="F398" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G398" t="inlineStr">
@@ -23834,7 +23822,7 @@
           <t>B10133</t>
         </is>
       </c>
-      <c r="F399" s="2" t="n">
+      <c r="F399" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="G399" t="inlineStr">
@@ -23859,7 +23847,7 @@
         </is>
       </c>
       <c r="L399" t="inlineStr"/>
-      <c r="M399" s="2" t="n">
+      <c r="M399" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="N399" t="inlineStr"/>
@@ -23894,7 +23882,7 @@
           <t>89177</t>
         </is>
       </c>
-      <c r="F400" s="2" t="n">
+      <c r="F400" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G400" t="inlineStr">
@@ -23954,7 +23942,7 @@
           <t>25304</t>
         </is>
       </c>
-      <c r="F401" s="2" t="n">
+      <c r="F401" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G401" t="inlineStr">
@@ -24014,7 +24002,7 @@
           <t>94934</t>
         </is>
       </c>
-      <c r="F402" s="2" t="n">
+      <c r="F402" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G402" t="inlineStr">
@@ -24074,7 +24062,7 @@
           <t>5155</t>
         </is>
       </c>
-      <c r="F403" s="2" t="n">
+      <c r="F403" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G403" t="inlineStr">
@@ -24130,7 +24118,7 @@
           <t>2333</t>
         </is>
       </c>
-      <c r="F404" s="2" t="n">
+      <c r="F404" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="G404" t="inlineStr">
@@ -24182,7 +24170,7 @@
       <c r="E405" t="n">
         <v>9599</v>
       </c>
-      <c r="F405" s="2" t="n">
+      <c r="F405" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="G405" t="inlineStr">
@@ -24230,7 +24218,7 @@
       <c r="E406" t="n">
         <v>14251</v>
       </c>
-      <c r="F406" s="2" t="n">
+      <c r="F406" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="G406" t="inlineStr">
@@ -24278,7 +24266,7 @@
       <c r="E407" t="n">
         <v>19945</v>
       </c>
-      <c r="F407" s="2" t="n">
+      <c r="F407" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="G407" t="inlineStr">
@@ -24326,7 +24314,7 @@
       <c r="E408" t="n">
         <v>14396</v>
       </c>
-      <c r="F408" s="2" t="n">
+      <c r="F408" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="G408" t="inlineStr">
@@ -24374,7 +24362,7 @@
       <c r="E409" t="n">
         <v>9920</v>
       </c>
-      <c r="F409" s="2" t="n">
+      <c r="F409" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="G409" t="inlineStr">
@@ -24422,7 +24410,7 @@
       <c r="E410" t="n">
         <v>20528</v>
       </c>
-      <c r="F410" s="2" t="n">
+      <c r="F410" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="G410" t="inlineStr">
@@ -24474,7 +24462,7 @@
           <t>3BF23</t>
         </is>
       </c>
-      <c r="F411" s="2" t="n">
+      <c r="F411" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G411" t="inlineStr">
@@ -24526,7 +24514,7 @@
           <t>10BE80</t>
         </is>
       </c>
-      <c r="F412" s="2" t="n">
+      <c r="F412" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G412" t="inlineStr">
@@ -24578,7 +24566,7 @@
           <t>2BC10</t>
         </is>
       </c>
-      <c r="F413" s="2" t="n">
+      <c r="F413" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G413" t="inlineStr">
@@ -24630,7 +24618,7 @@
           <t>11BG159</t>
         </is>
       </c>
-      <c r="F414" s="2" t="n">
+      <c r="F414" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G414" t="inlineStr">
@@ -24680,7 +24668,7 @@
           <t>A76103</t>
         </is>
       </c>
-      <c r="F415" s="2" t="n">
+      <c r="F415" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G415" t="inlineStr">
@@ -24730,7 +24718,7 @@
       <c r="E416" t="n">
         <v>5844</v>
       </c>
-      <c r="F416" s="2" t="n">
+      <c r="F416" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G416" t="inlineStr">
@@ -24780,7 +24768,7 @@
           <t>S00456</t>
         </is>
       </c>
-      <c r="F417" s="2" t="n">
+      <c r="F417" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G417" t="inlineStr">
@@ -24830,7 +24818,7 @@
           <t>S00167XL</t>
         </is>
       </c>
-      <c r="F418" s="2" t="n">
+      <c r="F418" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G418" t="inlineStr">
@@ -24880,7 +24868,7 @@
           <t>S00006XL2</t>
         </is>
       </c>
-      <c r="F419" s="2" t="n">
+      <c r="F419" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G419" t="inlineStr">
@@ -24930,7 +24918,7 @@
       <c r="E420" t="n">
         <v>580</v>
       </c>
-      <c r="F420" s="2" t="n">
+      <c r="F420" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G420" t="inlineStr">
@@ -24980,7 +24968,7 @@
           <t>T97125Q</t>
         </is>
       </c>
-      <c r="F421" s="2" t="n">
+      <c r="F421" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G421" t="inlineStr">
@@ -25030,7 +25018,7 @@
           <t>T1011900</t>
         </is>
       </c>
-      <c r="F422" s="2" t="n">
+      <c r="F422" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G422" t="inlineStr">
@@ -25080,7 +25068,7 @@
           <t>T91786Q</t>
         </is>
       </c>
-      <c r="F423" s="2" t="n">
+      <c r="F423" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G423" t="inlineStr">
@@ -25130,7 +25118,7 @@
           <t>00D10</t>
         </is>
       </c>
-      <c r="F424" s="2" t="n">
+      <c r="F424" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G424" t="inlineStr">
@@ -25180,7 +25168,7 @@
           <t>00D175</t>
         </is>
       </c>
-      <c r="F425" s="2" t="n">
+      <c r="F425" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G425" t="inlineStr">
@@ -25232,7 +25220,7 @@
           <t>E05-11026</t>
         </is>
       </c>
-      <c r="F426" s="2" t="n">
+      <c r="F426" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G426" t="inlineStr">
@@ -25282,7 +25270,7 @@
       <c r="E427" t="n">
         <v>6309</v>
       </c>
-      <c r="F427" s="2" t="n">
+      <c r="F427" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G427" t="inlineStr">
@@ -25332,7 +25320,7 @@
       <c r="E428" t="n">
         <v>504011190625165</v>
       </c>
-      <c r="F428" s="2" t="n">
+      <c r="F428" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G428" t="inlineStr">
@@ -25382,7 +25370,7 @@
       <c r="E429" t="n">
         <v>504011190625185</v>
       </c>
-      <c r="F429" s="2" t="n">
+      <c r="F429" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G429" t="inlineStr">
@@ -25432,7 +25420,7 @@
           <t>1116740R</t>
         </is>
       </c>
-      <c r="F430" s="2" t="n">
+      <c r="F430" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G430" t="inlineStr">
@@ -25482,7 +25470,7 @@
           <t>1992457/AC</t>
         </is>
       </c>
-      <c r="F431" s="2" t="n">
+      <c r="F431" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G431" t="inlineStr">
@@ -25532,7 +25520,7 @@
           <t>1715715AC</t>
         </is>
       </c>
-      <c r="F432" s="2" t="n">
+      <c r="F432" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G432" t="inlineStr">
@@ -25582,7 +25570,7 @@
           <t>L442</t>
         </is>
       </c>
-      <c r="F433" s="2" t="n">
+      <c r="F433" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G433" t="inlineStr">
@@ -25630,7 +25618,7 @@
       <c r="E434" t="n">
         <v>328</v>
       </c>
-      <c r="F434" s="2" t="n">
+      <c r="F434" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G434" t="inlineStr">
@@ -25678,7 +25666,7 @@
       <c r="E435" t="n">
         <v>277</v>
       </c>
-      <c r="F435" s="2" t="n">
+      <c r="F435" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G435" t="inlineStr">
@@ -25726,7 +25714,7 @@
       <c r="E436" t="n">
         <v>477</v>
       </c>
-      <c r="F436" s="2" t="n">
+      <c r="F436" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G436" t="inlineStr">
@@ -25774,7 +25762,7 @@
       <c r="E437" t="n">
         <v>11</v>
       </c>
-      <c r="F437" s="2" t="n">
+      <c r="F437" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G437" t="inlineStr">
@@ -25824,7 +25812,7 @@
           <t>196L</t>
         </is>
       </c>
-      <c r="F438" s="2" t="n">
+      <c r="F438" s="1" t="n">
         <v>46188</v>
       </c>
       <c r="G438" t="inlineStr">
@@ -25876,7 +25864,7 @@
           <t>15W013724</t>
         </is>
       </c>
-      <c r="F439" s="2" t="n">
+      <c r="F439" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="G439" t="inlineStr">
@@ -25928,7 +25916,7 @@
           <t>15W013930</t>
         </is>
       </c>
-      <c r="F440" s="2" t="n">
+      <c r="F440" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="G440" t="inlineStr">
@@ -25978,7 +25966,7 @@
       <c r="E441" t="n">
         <v>86815651</v>
       </c>
-      <c r="F441" s="2" t="n">
+      <c r="F441" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="G441" t="inlineStr">
@@ -26028,7 +26016,7 @@
       <c r="E442" t="n">
         <v>86817554</v>
       </c>
-      <c r="F442" s="2" t="n">
+      <c r="F442" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="G442" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: reparaveis (10/07/2026 20:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,82 +433,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>os</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>cff</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>data_inicio</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>unidade_solicitante</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tat_siloms</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>onde_se_encontra</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>recibo</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>condicao</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>data_retorno_prevista</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>sn_trocado_exchange</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>termo_recebimento</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>em_aberto</t>
         </is>
@@ -528,7 +540,7 @@
           <t>3859</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>45698</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -588,7 +600,7 @@
           <t>382750-016</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>45714</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -648,7 +660,7 @@
           <t>382750-023</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>45714</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -708,7 +720,7 @@
           <t>003342</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>45714</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -735,7 +747,7 @@
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" s="1" t="n">
+      <c r="M5" s="2" t="n">
         <v>45993</v>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -770,7 +782,7 @@
           <t>09450</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -797,7 +809,7 @@
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" s="1" t="n">
+      <c r="M6" s="2" t="n">
         <v>45889</v>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -832,7 +844,7 @@
           <t>1920</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -859,7 +871,7 @@
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" s="1" t="n">
+      <c r="M7" s="2" t="n">
         <v>45848</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -898,7 +910,7 @@
           <t>96967</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -948,7 +960,7 @@
           <t>2410</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -975,7 +987,7 @@
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" s="1" t="n">
+      <c r="M9" s="2" t="n">
         <v>46098</v>
       </c>
       <c r="N9" t="n">
@@ -1012,7 +1024,7 @@
           <t>P1916</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -1039,7 +1051,7 @@
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" s="1" t="n">
+      <c r="M10" s="2" t="n">
         <v>46114</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -1078,7 +1090,7 @@
           <t>2697</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -1105,7 +1117,7 @@
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" s="1" t="n">
+      <c r="M11" s="2" t="n">
         <v>45848</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -1144,7 +1156,7 @@
           <t>1569</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -1171,7 +1183,7 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" s="1" t="n">
+      <c r="M12" s="2" t="n">
         <v>45860</v>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -1206,7 +1218,7 @@
           <t>2706</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1264,7 +1276,7 @@
           <t>0215-217</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -1291,7 +1303,7 @@
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
-      <c r="M14" s="1" t="n">
+      <c r="M14" s="2" t="n">
         <v>45800</v>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -1326,7 +1338,7 @@
           <t>K010158</t>
         </is>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1386,7 +1398,7 @@
           <t>9911-257</t>
         </is>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1446,7 +1458,7 @@
           <t>791</t>
         </is>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1473,7 +1485,7 @@
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" s="1" t="n">
+      <c r="M17" s="2" t="n">
         <v>45897</v>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -1508,7 +1520,7 @@
           <t>7077</t>
         </is>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G18" t="inlineStr">
@@ -1535,7 +1547,7 @@
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" s="1" t="n">
+      <c r="M18" s="2" t="n">
         <v>45802</v>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -1570,7 +1582,7 @@
           <t>3890</t>
         </is>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G19" t="inlineStr">
@@ -1628,7 +1640,7 @@
           <t>KI256-25711</t>
         </is>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G20" t="inlineStr">
@@ -1655,7 +1667,7 @@
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" s="1" t="n">
+      <c r="M20" s="2" t="n">
         <v>46135</v>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -1690,7 +1702,7 @@
           <t>KI256-25707</t>
         </is>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="F21" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -1748,7 +1760,7 @@
           <t>3885</t>
         </is>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -1808,7 +1820,7 @@
           <t>3861</t>
         </is>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -1835,7 +1847,7 @@
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" s="1" t="n">
+      <c r="M23" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -1874,7 +1886,7 @@
           <t>17143</t>
         </is>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G24" t="inlineStr">
@@ -1932,7 +1944,7 @@
           <t>96782</t>
         </is>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G25" t="inlineStr">
@@ -1990,7 +2002,7 @@
           <t>KMD540-10071</t>
         </is>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -2017,7 +2029,7 @@
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" s="1" t="n">
+      <c r="M26" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="N26" t="inlineStr"/>
@@ -2056,7 +2068,7 @@
           <t>75123</t>
         </is>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G27" t="inlineStr">
@@ -2116,7 +2128,7 @@
           <t>00B205C</t>
         </is>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -2166,7 +2178,7 @@
           <t>277</t>
         </is>
       </c>
-      <c r="F29" s="1" t="n">
+      <c r="F29" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G29" t="inlineStr">
@@ -2224,7 +2236,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="F30" s="1" t="n">
+      <c r="F30" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G30" t="inlineStr">
@@ -2251,7 +2263,7 @@
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" s="1" t="n">
+      <c r="M30" s="2" t="n">
         <v>45945</v>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -2286,7 +2298,7 @@
           <t>7951</t>
         </is>
       </c>
-      <c r="F31" s="1" t="n">
+      <c r="F31" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G31" t="inlineStr">
@@ -2344,7 +2356,7 @@
           <t>5028A</t>
         </is>
       </c>
-      <c r="F32" s="1" t="n">
+      <c r="F32" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G32" t="inlineStr">
@@ -2404,7 +2416,7 @@
           <t>122</t>
         </is>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G33" t="inlineStr">
@@ -2462,7 +2474,7 @@
           <t>27</t>
         </is>
       </c>
-      <c r="F34" s="1" t="n">
+      <c r="F34" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G34" t="inlineStr">
@@ -2512,7 +2524,7 @@
           <t>02B</t>
         </is>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="F35" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G35" t="inlineStr">
@@ -2562,7 +2574,7 @@
           <t>291</t>
         </is>
       </c>
-      <c r="F36" s="1" t="n">
+      <c r="F36" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G36" t="inlineStr">
@@ -2620,7 +2632,7 @@
           <t>0011</t>
         </is>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="F37" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G37" t="inlineStr">
@@ -2678,7 +2690,7 @@
           <t>791</t>
         </is>
       </c>
-      <c r="F38" s="1" t="n">
+      <c r="F38" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G38" t="inlineStr">
@@ -2732,7 +2744,7 @@
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" s="1" t="n">
+      <c r="F39" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G39" t="inlineStr">
@@ -2788,7 +2800,7 @@
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
-      <c r="F40" s="1" t="n">
+      <c r="F40" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G40" t="inlineStr">
@@ -2848,7 +2860,7 @@
           <t>988</t>
         </is>
       </c>
-      <c r="F41" s="1" t="n">
+      <c r="F41" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G41" t="inlineStr">
@@ -2906,7 +2918,7 @@
           <t>994</t>
         </is>
       </c>
-      <c r="F42" s="1" t="n">
+      <c r="F42" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G42" t="inlineStr">
@@ -2964,7 +2976,7 @@
           <t>10603745</t>
         </is>
       </c>
-      <c r="F43" s="1" t="n">
+      <c r="F43" s="2" t="n">
         <v>45736</v>
       </c>
       <c r="G43" t="inlineStr">
@@ -3022,7 +3034,7 @@
           <t>LS0414</t>
         </is>
       </c>
-      <c r="F44" s="1" t="n">
+      <c r="F44" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G44" t="inlineStr">
@@ -3049,7 +3061,7 @@
         </is>
       </c>
       <c r="L44" t="inlineStr"/>
-      <c r="M44" s="1" t="n">
+      <c r="M44" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="N44" t="inlineStr"/>
@@ -3088,7 +3100,7 @@
           <t>86805596</t>
         </is>
       </c>
-      <c r="F45" s="1" t="n">
+      <c r="F45" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G45" t="inlineStr">
@@ -3115,7 +3127,7 @@
         </is>
       </c>
       <c r="L45" t="inlineStr"/>
-      <c r="M45" s="1" t="n">
+      <c r="M45" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="N45" t="n">
@@ -3152,7 +3164,7 @@
           <t>R50653</t>
         </is>
       </c>
-      <c r="F46" s="1" t="n">
+      <c r="F46" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G46" t="inlineStr">
@@ -3212,7 +3224,7 @@
           <t>53450</t>
         </is>
       </c>
-      <c r="F47" s="1" t="n">
+      <c r="F47" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G47" t="inlineStr">
@@ -3239,7 +3251,7 @@
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
-      <c r="M47" s="1" t="n">
+      <c r="M47" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="N47" t="inlineStr"/>
@@ -3278,7 +3290,7 @@
           <t>52537</t>
         </is>
       </c>
-      <c r="F48" s="1" t="n">
+      <c r="F48" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G48" t="inlineStr">
@@ -3338,7 +3350,7 @@
           <t>51767</t>
         </is>
       </c>
-      <c r="F49" s="1" t="n">
+      <c r="F49" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G49" t="inlineStr">
@@ -3388,7 +3400,7 @@
           <t>28411</t>
         </is>
       </c>
-      <c r="F50" s="1" t="n">
+      <c r="F50" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G50" t="inlineStr">
@@ -3448,7 +3460,7 @@
           <t>36025</t>
         </is>
       </c>
-      <c r="F51" s="1" t="n">
+      <c r="F51" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G51" t="inlineStr">
@@ -3506,7 +3518,7 @@
           <t>34257</t>
         </is>
       </c>
-      <c r="F52" s="1" t="n">
+      <c r="F52" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G52" t="inlineStr">
@@ -3566,7 +3578,7 @@
           <t>30865</t>
         </is>
       </c>
-      <c r="F53" s="1" t="n">
+      <c r="F53" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G53" t="inlineStr">
@@ -3626,7 +3638,7 @@
           <t>4355</t>
         </is>
       </c>
-      <c r="F54" s="1" t="n">
+      <c r="F54" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G54" t="inlineStr">
@@ -3686,7 +3698,7 @@
           <t>38197</t>
         </is>
       </c>
-      <c r="F55" s="1" t="n">
+      <c r="F55" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G55" t="inlineStr">
@@ -3736,7 +3748,7 @@
           <t>85131</t>
         </is>
       </c>
-      <c r="F56" s="1" t="n">
+      <c r="F56" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G56" t="inlineStr">
@@ -3794,7 +3806,7 @@
           <t>86012</t>
         </is>
       </c>
-      <c r="F57" s="1" t="n">
+      <c r="F57" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G57" t="inlineStr">
@@ -3854,7 +3866,7 @@
           <t>85068</t>
         </is>
       </c>
-      <c r="F58" s="1" t="n">
+      <c r="F58" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G58" t="inlineStr">
@@ -3904,7 +3916,7 @@
           <t>84459</t>
         </is>
       </c>
-      <c r="F59" s="1" t="n">
+      <c r="F59" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G59" t="inlineStr">
@@ -3962,7 +3974,7 @@
           <t>AAT5599</t>
         </is>
       </c>
-      <c r="F60" s="1" t="n">
+      <c r="F60" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G60" t="inlineStr">
@@ -4020,7 +4032,7 @@
           <t>AAE3882</t>
         </is>
       </c>
-      <c r="F61" s="1" t="n">
+      <c r="F61" s="2" t="n">
         <v>45769</v>
       </c>
       <c r="G61" t="inlineStr">
@@ -4074,7 +4086,7 @@
           <t>22005920</t>
         </is>
       </c>
-      <c r="F62" s="1" t="n">
+      <c r="F62" s="2" t="n">
         <v>45770</v>
       </c>
       <c r="G62" t="inlineStr">
@@ -4124,7 +4136,7 @@
           <t>1882C</t>
         </is>
       </c>
-      <c r="F63" s="1" t="n">
+      <c r="F63" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="G63" t="inlineStr">
@@ -4151,7 +4163,7 @@
         </is>
       </c>
       <c r="L63" t="inlineStr"/>
-      <c r="M63" s="1" t="n">
+      <c r="M63" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="N63" t="inlineStr"/>
@@ -4190,7 +4202,7 @@
           <t>02</t>
         </is>
       </c>
-      <c r="F64" s="1" t="n">
+      <c r="F64" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="G64" t="inlineStr">
@@ -4217,7 +4229,7 @@
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
-      <c r="M64" s="1" t="n">
+      <c r="M64" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="N64" t="inlineStr"/>
@@ -4252,7 +4264,7 @@
           <t>323</t>
         </is>
       </c>
-      <c r="F65" s="1" t="n">
+      <c r="F65" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="G65" t="inlineStr">
@@ -4310,7 +4322,7 @@
           <t>297</t>
         </is>
       </c>
-      <c r="F66" s="1" t="n">
+      <c r="F66" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="G66" t="inlineStr">
@@ -4368,7 +4380,7 @@
           <t>144</t>
         </is>
       </c>
-      <c r="F67" s="1" t="n">
+      <c r="F67" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="G67" t="inlineStr">
@@ -4426,7 +4438,7 @@
           <t>324</t>
         </is>
       </c>
-      <c r="F68" s="1" t="n">
+      <c r="F68" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="G68" t="inlineStr">
@@ -4484,7 +4496,7 @@
           <t>475</t>
         </is>
       </c>
-      <c r="F69" s="1" t="n">
+      <c r="F69" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G69" t="inlineStr">
@@ -4542,7 +4554,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="F70" s="1" t="n">
+      <c r="F70" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G70" t="inlineStr">
@@ -4602,7 +4614,7 @@
           <t>UNK01</t>
         </is>
       </c>
-      <c r="F71" s="1" t="n">
+      <c r="F71" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G71" t="inlineStr">
@@ -4658,7 +4670,7 @@
           <t>278</t>
         </is>
       </c>
-      <c r="F72" s="1" t="n">
+      <c r="F72" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G72" t="inlineStr">
@@ -4716,7 +4728,7 @@
           <t>967</t>
         </is>
       </c>
-      <c r="F73" s="1" t="n">
+      <c r="F73" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G73" t="inlineStr">
@@ -4776,7 +4788,7 @@
           <t>278</t>
         </is>
       </c>
-      <c r="F74" s="1" t="n">
+      <c r="F74" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G74" t="inlineStr">
@@ -4834,7 +4846,7 @@
           <t>772</t>
         </is>
       </c>
-      <c r="F75" s="1" t="n">
+      <c r="F75" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G75" t="inlineStr">
@@ -4894,7 +4906,7 @@
           <t>49</t>
         </is>
       </c>
-      <c r="F76" s="1" t="n">
+      <c r="F76" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G76" t="inlineStr">
@@ -4950,7 +4962,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="F77" s="1" t="n">
+      <c r="F77" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G77" t="inlineStr">
@@ -5008,7 +5020,7 @@
           <t>289</t>
         </is>
       </c>
-      <c r="F78" s="1" t="n">
+      <c r="F78" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G78" t="inlineStr">
@@ -5066,7 +5078,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="F79" s="1" t="n">
+      <c r="F79" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G79" t="inlineStr">
@@ -5122,7 +5134,7 @@
           <t>969</t>
         </is>
       </c>
-      <c r="F80" s="1" t="n">
+      <c r="F80" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="G80" t="inlineStr">
@@ -5182,7 +5194,7 @@
           <t>1311</t>
         </is>
       </c>
-      <c r="F81" s="1" t="n">
+      <c r="F81" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G81" t="inlineStr">
@@ -5240,7 +5252,7 @@
           <t>3945</t>
         </is>
       </c>
-      <c r="F82" s="1" t="n">
+      <c r="F82" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G82" t="inlineStr">
@@ -5300,7 +5312,7 @@
           <t>35378</t>
         </is>
       </c>
-      <c r="F83" s="1" t="n">
+      <c r="F83" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G83" t="inlineStr">
@@ -5358,7 +5370,7 @@
           <t>2469</t>
         </is>
       </c>
-      <c r="F84" s="1" t="n">
+      <c r="F84" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G84" t="inlineStr">
@@ -5385,7 +5397,7 @@
         </is>
       </c>
       <c r="L84" t="inlineStr"/>
-      <c r="M84" s="1" t="n">
+      <c r="M84" s="2" t="n">
         <v>45853</v>
       </c>
       <c r="N84" t="n">
@@ -5422,7 +5434,7 @@
           <t>292</t>
         </is>
       </c>
-      <c r="F85" s="1" t="n">
+      <c r="F85" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G85" t="inlineStr">
@@ -5482,7 +5494,7 @@
           <t>168394-05</t>
         </is>
       </c>
-      <c r="F86" s="1" t="n">
+      <c r="F86" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G86" t="inlineStr">
@@ -5542,7 +5554,7 @@
           <t>197</t>
         </is>
       </c>
-      <c r="F87" s="1" t="n">
+      <c r="F87" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G87" t="inlineStr">
@@ -5569,7 +5581,7 @@
         </is>
       </c>
       <c r="L87" t="inlineStr"/>
-      <c r="M87" s="1" t="n">
+      <c r="M87" s="2" t="n">
         <v>45797</v>
       </c>
       <c r="N87" t="inlineStr">
@@ -5608,7 +5620,7 @@
           <t>10603744</t>
         </is>
       </c>
-      <c r="F88" s="1" t="n">
+      <c r="F88" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G88" t="inlineStr">
@@ -5666,7 +5678,7 @@
           <t>11200477</t>
         </is>
       </c>
-      <c r="F89" s="1" t="n">
+      <c r="F89" s="2" t="n">
         <v>45813</v>
       </c>
       <c r="G89" t="inlineStr">
@@ -5724,7 +5736,7 @@
           <t>5385</t>
         </is>
       </c>
-      <c r="F90" s="1" t="n">
+      <c r="F90" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G90" t="inlineStr">
@@ -5788,7 +5800,7 @@
           <t>001</t>
         </is>
       </c>
-      <c r="F91" s="1" t="n">
+      <c r="F91" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G91" t="inlineStr">
@@ -5844,7 +5856,7 @@
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
-      <c r="F92" s="1" t="n">
+      <c r="F92" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G92" t="inlineStr">
@@ -5894,7 +5906,7 @@
           <t>CE-11200</t>
         </is>
       </c>
-      <c r="F93" s="1" t="n">
+      <c r="F93" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G93" t="inlineStr">
@@ -5954,7 +5966,7 @@
           <t>CE-09234</t>
         </is>
       </c>
-      <c r="F94" s="1" t="n">
+      <c r="F94" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G94" t="inlineStr">
@@ -6014,7 +6026,7 @@
           <t>CE-08838</t>
         </is>
       </c>
-      <c r="F95" s="1" t="n">
+      <c r="F95" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G95" t="inlineStr">
@@ -6074,7 +6086,7 @@
           <t>908</t>
         </is>
       </c>
-      <c r="F96" s="1" t="n">
+      <c r="F96" s="2" t="n">
         <v>45831</v>
       </c>
       <c r="G96" t="inlineStr">
@@ -6101,7 +6113,7 @@
         </is>
       </c>
       <c r="L96" t="inlineStr"/>
-      <c r="M96" s="1" t="n">
+      <c r="M96" s="2" t="n">
         <v>45848</v>
       </c>
       <c r="N96" t="inlineStr">
@@ -6140,7 +6152,7 @@
           <t>203103</t>
         </is>
       </c>
-      <c r="F97" s="1" t="n">
+      <c r="F97" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G97" t="inlineStr">
@@ -6204,7 +6216,7 @@
           <t>56422</t>
         </is>
       </c>
-      <c r="F98" s="1" t="n">
+      <c r="F98" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G98" t="inlineStr">
@@ -6264,7 +6276,7 @@
           <t>07915</t>
         </is>
       </c>
-      <c r="F99" s="1" t="n">
+      <c r="F99" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G99" t="inlineStr">
@@ -6314,7 +6326,7 @@
           <t>X-330970</t>
         </is>
       </c>
-      <c r="F100" s="1" t="n">
+      <c r="F100" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G100" t="inlineStr">
@@ -6374,7 +6386,7 @@
           <t>X-412785</t>
         </is>
       </c>
-      <c r="F101" s="1" t="n">
+      <c r="F101" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G101" t="inlineStr">
@@ -6424,7 +6436,7 @@
           <t>B10811721</t>
         </is>
       </c>
-      <c r="F102" s="1" t="n">
+      <c r="F102" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G102" t="inlineStr">
@@ -6474,7 +6486,7 @@
           <t>X330978</t>
         </is>
       </c>
-      <c r="F103" s="1" t="n">
+      <c r="F103" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G103" t="inlineStr">
@@ -6524,7 +6536,7 @@
           <t>X-467664</t>
         </is>
       </c>
-      <c r="F104" s="1" t="n">
+      <c r="F104" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G104" t="inlineStr">
@@ -6584,7 +6596,7 @@
           <t>D00397798</t>
         </is>
       </c>
-      <c r="F105" s="1" t="n">
+      <c r="F105" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G105" t="inlineStr">
@@ -6644,7 +6656,7 @@
           <t>6132</t>
         </is>
       </c>
-      <c r="F106" s="1" t="n">
+      <c r="F106" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G106" t="inlineStr">
@@ -6671,7 +6683,7 @@
         </is>
       </c>
       <c r="L106" t="inlineStr"/>
-      <c r="M106" s="1" t="n">
+      <c r="M106" s="2" t="n">
         <v>45889</v>
       </c>
       <c r="N106" t="inlineStr"/>
@@ -6706,7 +6718,7 @@
           <t>030998</t>
         </is>
       </c>
-      <c r="F107" s="1" t="n">
+      <c r="F107" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G107" t="inlineStr">
@@ -6733,7 +6745,7 @@
         </is>
       </c>
       <c r="L107" t="inlineStr"/>
-      <c r="M107" s="1" t="n">
+      <c r="M107" s="2" t="n">
         <v>45876</v>
       </c>
       <c r="N107" t="inlineStr"/>
@@ -6768,7 +6780,7 @@
           <t>5AL</t>
         </is>
       </c>
-      <c r="F108" s="1" t="n">
+      <c r="F108" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G108" t="inlineStr">
@@ -6828,7 +6840,7 @@
           <t>7AC</t>
         </is>
       </c>
-      <c r="F109" s="1" t="n">
+      <c r="F109" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G109" t="inlineStr">
@@ -6888,7 +6900,7 @@
           <t>2668-5</t>
         </is>
       </c>
-      <c r="F110" s="1" t="n">
+      <c r="F110" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G110" t="inlineStr">
@@ -6946,7 +6958,7 @@
           <t>3155-5</t>
         </is>
       </c>
-      <c r="F111" s="1" t="n">
+      <c r="F111" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G111" t="inlineStr">
@@ -7004,7 +7016,7 @@
           <t>3124-5</t>
         </is>
       </c>
-      <c r="F112" s="1" t="n">
+      <c r="F112" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G112" t="inlineStr">
@@ -7054,7 +7066,7 @@
           <t>3275-5</t>
         </is>
       </c>
-      <c r="F113" s="1" t="n">
+      <c r="F113" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G113" t="inlineStr">
@@ -7112,7 +7124,7 @@
           <t>9902509</t>
         </is>
       </c>
-      <c r="F114" s="1" t="n">
+      <c r="F114" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G114" t="inlineStr">
@@ -7170,7 +7182,7 @@
           <t>369783-021</t>
         </is>
       </c>
-      <c r="F115" s="1" t="n">
+      <c r="F115" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G115" t="inlineStr">
@@ -7230,7 +7242,7 @@
           <t>363749-030</t>
         </is>
       </c>
-      <c r="F116" s="1" t="n">
+      <c r="F116" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G116" t="inlineStr">
@@ -7290,7 +7302,7 @@
           <t>376422-005</t>
         </is>
       </c>
-      <c r="F117" s="1" t="n">
+      <c r="F117" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G117" t="inlineStr">
@@ -7350,7 +7362,7 @@
           <t>376415-037</t>
         </is>
       </c>
-      <c r="F118" s="1" t="n">
+      <c r="F118" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G118" t="inlineStr">
@@ -7410,7 +7422,7 @@
           <t>363761-060</t>
         </is>
       </c>
-      <c r="F119" s="1" t="n">
+      <c r="F119" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G119" t="inlineStr">
@@ -7470,7 +7482,7 @@
           <t>363749-085</t>
         </is>
       </c>
-      <c r="F120" s="1" t="n">
+      <c r="F120" s="2" t="n">
         <v>45840</v>
       </c>
       <c r="G120" t="inlineStr">
@@ -7530,7 +7542,7 @@
           <t>86800893</t>
         </is>
       </c>
-      <c r="F121" s="1" t="n">
+      <c r="F121" s="2" t="n">
         <v>45849</v>
       </c>
       <c r="G121" t="inlineStr">
@@ -7557,7 +7569,7 @@
         </is>
       </c>
       <c r="L121" t="inlineStr"/>
-      <c r="M121" s="1" t="n">
+      <c r="M121" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="N121" t="n">
@@ -7594,7 +7606,7 @@
           <t>003614</t>
         </is>
       </c>
-      <c r="F122" s="1" t="n">
+      <c r="F122" s="2" t="n">
         <v>45849</v>
       </c>
       <c r="G122" t="inlineStr">
@@ -7654,7 +7666,7 @@
           <t>15100008</t>
         </is>
       </c>
-      <c r="F123" s="1" t="n">
+      <c r="F123" s="2" t="n">
         <v>45849</v>
       </c>
       <c r="G123" t="inlineStr">
@@ -7704,7 +7716,7 @@
           <t>0235</t>
         </is>
       </c>
-      <c r="F124" s="1" t="n">
+      <c r="F124" s="2" t="n">
         <v>45853</v>
       </c>
       <c r="G124" t="inlineStr">
@@ -7764,7 +7776,7 @@
           <t>5236</t>
         </is>
       </c>
-      <c r="F125" s="1" t="n">
+      <c r="F125" s="2" t="n">
         <v>45855</v>
       </c>
       <c r="G125" t="inlineStr">
@@ -7824,7 +7836,7 @@
           <t>ART2000-13237</t>
         </is>
       </c>
-      <c r="F126" s="1" t="n">
+      <c r="F126" s="2" t="n">
         <v>45855</v>
       </c>
       <c r="G126" t="inlineStr">
@@ -7882,7 +7894,7 @@
           <t>T23740</t>
         </is>
       </c>
-      <c r="F127" s="1" t="n">
+      <c r="F127" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="G127" t="inlineStr">
@@ -7932,7 +7944,7 @@
           <t>5K660</t>
         </is>
       </c>
-      <c r="F128" s="1" t="n">
+      <c r="F128" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="G128" t="inlineStr">
@@ -7992,7 +8004,7 @@
           <t>71306307</t>
         </is>
       </c>
-      <c r="F129" s="1" t="n">
+      <c r="F129" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="G129" t="inlineStr">
@@ -8052,7 +8064,7 @@
           <t>47204432</t>
         </is>
       </c>
-      <c r="F130" s="1" t="n">
+      <c r="F130" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="G130" t="inlineStr">
@@ -8079,7 +8091,7 @@
         </is>
       </c>
       <c r="L130" t="inlineStr"/>
-      <c r="M130" s="1" t="n">
+      <c r="M130" s="2" t="n">
         <v>45916</v>
       </c>
       <c r="N130" t="n">
@@ -8116,7 +8128,7 @@
           <t>409496</t>
         </is>
       </c>
-      <c r="F131" s="1" t="n">
+      <c r="F131" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="G131" t="inlineStr">
@@ -8174,7 +8186,7 @@
           <t>71308676</t>
         </is>
       </c>
-      <c r="F132" s="1" t="n">
+      <c r="F132" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="G132" t="inlineStr">
@@ -8201,7 +8213,7 @@
         </is>
       </c>
       <c r="L132" t="inlineStr"/>
-      <c r="M132" s="1" t="n">
+      <c r="M132" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="N132" t="n">
@@ -8238,7 +8250,7 @@
           <t>86819178</t>
         </is>
       </c>
-      <c r="F133" s="1" t="n">
+      <c r="F133" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="G133" t="inlineStr">
@@ -8288,7 +8300,7 @@
           <t>8259</t>
         </is>
       </c>
-      <c r="F134" s="1" t="n">
+      <c r="F134" s="2" t="n">
         <v>45882</v>
       </c>
       <c r="G134" t="inlineStr">
@@ -8348,7 +8360,7 @@
           <t>22A805</t>
         </is>
       </c>
-      <c r="F135" s="1" t="n">
+      <c r="F135" s="2" t="n">
         <v>45882</v>
       </c>
       <c r="G135" t="inlineStr">
@@ -8398,7 +8410,7 @@
           <t>T22974</t>
         </is>
       </c>
-      <c r="F136" s="1" t="n">
+      <c r="F136" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G136" t="inlineStr">
@@ -8448,7 +8460,7 @@
           <t>15508160</t>
         </is>
       </c>
-      <c r="F137" s="1" t="n">
+      <c r="F137" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G137" t="inlineStr">
@@ -8498,7 +8510,7 @@
           <t>12056029</t>
         </is>
       </c>
-      <c r="F138" s="1" t="n">
+      <c r="F138" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G138" t="inlineStr">
@@ -8558,7 +8570,7 @@
           <t>T20503</t>
         </is>
       </c>
-      <c r="F139" s="1" t="n">
+      <c r="F139" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G139" t="inlineStr">
@@ -8608,7 +8620,7 @@
           <t>T25426</t>
         </is>
       </c>
-      <c r="F140" s="1" t="n">
+      <c r="F140" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G140" t="inlineStr">
@@ -8666,7 +8678,7 @@
           <t>03</t>
         </is>
       </c>
-      <c r="F141" s="1" t="n">
+      <c r="F141" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G141" t="inlineStr">
@@ -8716,7 +8728,7 @@
           <t>778</t>
         </is>
       </c>
-      <c r="F142" s="1" t="n">
+      <c r="F142" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G142" t="inlineStr">
@@ -8766,7 +8778,7 @@
           <t>356</t>
         </is>
       </c>
-      <c r="F143" s="1" t="n">
+      <c r="F143" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G143" t="inlineStr">
@@ -8816,7 +8828,7 @@
           <t>28</t>
         </is>
       </c>
-      <c r="F144" s="1" t="n">
+      <c r="F144" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G144" t="inlineStr">
@@ -8866,7 +8878,7 @@
           <t>048F</t>
         </is>
       </c>
-      <c r="F145" s="1" t="n">
+      <c r="F145" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G145" t="inlineStr">
@@ -8924,7 +8936,7 @@
           <t>3270</t>
         </is>
       </c>
-      <c r="F146" s="1" t="n">
+      <c r="F146" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G146" t="inlineStr">
@@ -8974,7 +8986,7 @@
           <t>LSEAM3250</t>
         </is>
       </c>
-      <c r="F147" s="1" t="n">
+      <c r="F147" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G147" t="inlineStr">
@@ -9032,7 +9044,7 @@
           <t>A4H-106-02</t>
         </is>
       </c>
-      <c r="F148" s="1" t="n">
+      <c r="F148" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G148" t="inlineStr">
@@ -9092,7 +9104,7 @@
           <t>K517</t>
         </is>
       </c>
-      <c r="F149" s="1" t="n">
+      <c r="F149" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G149" t="inlineStr">
@@ -9148,7 +9160,7 @@
           <t>016B</t>
         </is>
       </c>
-      <c r="F150" s="1" t="n">
+      <c r="F150" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G150" t="inlineStr">
@@ -9175,7 +9187,7 @@
         </is>
       </c>
       <c r="L150" t="inlineStr"/>
-      <c r="M150" s="1" t="n">
+      <c r="M150" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="N150" t="inlineStr"/>
@@ -9214,7 +9226,7 @@
           <t>935</t>
         </is>
       </c>
-      <c r="F151" s="1" t="n">
+      <c r="F151" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G151" t="inlineStr">
@@ -9272,7 +9284,7 @@
           <t>03</t>
         </is>
       </c>
-      <c r="F152" s="1" t="n">
+      <c r="F152" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G152" t="inlineStr">
@@ -9299,7 +9311,7 @@
         </is>
       </c>
       <c r="L152" t="inlineStr"/>
-      <c r="M152" s="1" t="n">
+      <c r="M152" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="N152" t="inlineStr"/>
@@ -9334,7 +9346,7 @@
           <t>B4H-018</t>
         </is>
       </c>
-      <c r="F153" s="1" t="n">
+      <c r="F153" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G153" t="inlineStr">
@@ -9394,7 +9406,7 @@
           <t>108</t>
         </is>
       </c>
-      <c r="F154" s="1" t="n">
+      <c r="F154" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G154" t="inlineStr">
@@ -9452,7 +9464,7 @@
           <t>66306636</t>
         </is>
       </c>
-      <c r="F155" s="1" t="n">
+      <c r="F155" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G155" t="inlineStr">
@@ -9508,7 +9520,7 @@
           <t>66305791</t>
         </is>
       </c>
-      <c r="F156" s="1" t="n">
+      <c r="F156" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G156" t="inlineStr">
@@ -9568,7 +9580,7 @@
           <t>47203806</t>
         </is>
       </c>
-      <c r="F157" s="1" t="n">
+      <c r="F157" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="G157" t="inlineStr">
@@ -9628,7 +9640,7 @@
           <t>28A403</t>
         </is>
       </c>
-      <c r="F158" s="1" t="n">
+      <c r="F158" s="2" t="n">
         <v>45894</v>
       </c>
       <c r="G158" t="inlineStr">
@@ -9655,7 +9667,7 @@
         </is>
       </c>
       <c r="L158" t="inlineStr"/>
-      <c r="M158" s="1" t="n">
+      <c r="M158" s="2" t="n">
         <v>45946</v>
       </c>
       <c r="N158" t="inlineStr"/>
@@ -9690,7 +9702,7 @@
           <t>479</t>
         </is>
       </c>
-      <c r="F159" s="1" t="n">
+      <c r="F159" s="2" t="n">
         <v>45894</v>
       </c>
       <c r="G159" t="inlineStr">
@@ -9750,7 +9762,7 @@
           <t>15W008701</t>
         </is>
       </c>
-      <c r="F160" s="1" t="n">
+      <c r="F160" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="G160" t="inlineStr">
@@ -9810,7 +9822,7 @@
           <t>15W006615</t>
         </is>
       </c>
-      <c r="F161" s="1" t="n">
+      <c r="F161" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="G161" t="inlineStr">
@@ -9837,7 +9849,7 @@
         </is>
       </c>
       <c r="L161" t="inlineStr"/>
-      <c r="M161" s="1" t="n">
+      <c r="M161" s="2" t="n">
         <v>45953</v>
       </c>
       <c r="N161" t="inlineStr">
@@ -9876,7 +9888,7 @@
           <t>2953</t>
         </is>
       </c>
-      <c r="F162" s="1" t="n">
+      <c r="F162" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="G162" t="inlineStr">
@@ -9903,7 +9915,7 @@
         </is>
       </c>
       <c r="L162" t="inlineStr"/>
-      <c r="M162" s="1" t="n">
+      <c r="M162" s="2" t="n">
         <v>45940</v>
       </c>
       <c r="N162" t="inlineStr"/>
@@ -9938,7 +9950,7 @@
           <t>2982</t>
         </is>
       </c>
-      <c r="F163" s="1" t="n">
+      <c r="F163" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="G163" t="inlineStr">
@@ -9965,7 +9977,7 @@
         </is>
       </c>
       <c r="L163" t="inlineStr"/>
-      <c r="M163" s="1" t="n">
+      <c r="M163" s="2" t="n">
         <v>45940</v>
       </c>
       <c r="N163" t="inlineStr"/>
@@ -10000,7 +10012,7 @@
           <t>37F</t>
         </is>
       </c>
-      <c r="F164" s="1" t="n">
+      <c r="F164" s="2" t="n">
         <v>45910</v>
       </c>
       <c r="G164" t="inlineStr">
@@ -10056,7 +10068,7 @@
           <t>02LS</t>
         </is>
       </c>
-      <c r="F165" s="1" t="n">
+      <c r="F165" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G165" t="inlineStr">
@@ -10116,7 +10128,7 @@
           <t>B10133</t>
         </is>
       </c>
-      <c r="F166" s="1" t="n">
+      <c r="F166" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G166" t="inlineStr">
@@ -10174,7 +10186,7 @@
           <t>T20874</t>
         </is>
       </c>
-      <c r="F167" s="1" t="n">
+      <c r="F167" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G167" t="inlineStr">
@@ -10224,7 +10236,7 @@
           <t>T20976</t>
         </is>
       </c>
-      <c r="F168" s="1" t="n">
+      <c r="F168" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G168" t="inlineStr">
@@ -10288,7 +10300,7 @@
           <t>C25361</t>
         </is>
       </c>
-      <c r="F169" s="1" t="n">
+      <c r="F169" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G169" t="inlineStr">
@@ -10315,7 +10327,7 @@
         </is>
       </c>
       <c r="L169" t="inlineStr"/>
-      <c r="M169" s="1" t="n">
+      <c r="M169" s="2" t="n">
         <v>45973</v>
       </c>
       <c r="N169" t="inlineStr"/>
@@ -10350,7 +10362,7 @@
           <t>C25208</t>
         </is>
       </c>
-      <c r="F170" s="1" t="n">
+      <c r="F170" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G170" t="inlineStr">
@@ -10408,7 +10420,7 @@
           <t>571</t>
         </is>
       </c>
-      <c r="F171" s="1" t="n">
+      <c r="F171" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G171" t="inlineStr">
@@ -10468,7 +10480,7 @@
           <t>776</t>
         </is>
       </c>
-      <c r="F172" s="1" t="n">
+      <c r="F172" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G172" t="inlineStr">
@@ -10526,7 +10538,7 @@
           <t>LSEAM3239</t>
         </is>
       </c>
-      <c r="F173" s="1" t="n">
+      <c r="F173" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G173" t="inlineStr">
@@ -10584,7 +10596,7 @@
           <t>10603742</t>
         </is>
       </c>
-      <c r="F174" s="1" t="n">
+      <c r="F174" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G174" t="inlineStr">
@@ -10642,7 +10654,7 @@
           <t>015A</t>
         </is>
       </c>
-      <c r="F175" s="1" t="n">
+      <c r="F175" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G175" t="inlineStr">
@@ -10669,7 +10681,7 @@
         </is>
       </c>
       <c r="L175" t="inlineStr"/>
-      <c r="M175" s="1" t="n">
+      <c r="M175" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="N175" t="inlineStr"/>
@@ -10708,7 +10720,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="F176" s="1" t="n">
+      <c r="F176" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G176" t="inlineStr">
@@ -10768,7 +10780,7 @@
           <t>327</t>
         </is>
       </c>
-      <c r="F177" s="1" t="n">
+      <c r="F177" s="2" t="n">
         <v>45917</v>
       </c>
       <c r="G177" t="inlineStr">
@@ -10795,7 +10807,7 @@
         </is>
       </c>
       <c r="L177" t="inlineStr"/>
-      <c r="M177" s="1" t="n">
+      <c r="M177" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="N177" t="inlineStr"/>
@@ -10834,7 +10846,7 @@
           <t>16389901</t>
         </is>
       </c>
-      <c r="F178" s="1" t="n">
+      <c r="F178" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="G178" t="inlineStr">
@@ -10894,7 +10906,7 @@
           <t>18384912</t>
         </is>
       </c>
-      <c r="F179" s="1" t="n">
+      <c r="F179" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="G179" t="inlineStr">
@@ -10944,7 +10956,7 @@
           <t>12253839V</t>
         </is>
       </c>
-      <c r="F180" s="1" t="n">
+      <c r="F180" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="G180" t="inlineStr">
@@ -11004,7 +11016,7 @@
           <t>12245097V</t>
         </is>
       </c>
-      <c r="F181" s="1" t="n">
+      <c r="F181" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="G181" t="inlineStr">
@@ -11062,7 +11074,7 @@
           <t>16940865</t>
         </is>
       </c>
-      <c r="F182" s="1" t="n">
+      <c r="F182" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="G182" t="inlineStr">
@@ -11112,7 +11124,7 @@
           <t>66307595</t>
         </is>
       </c>
-      <c r="F183" s="1" t="n">
+      <c r="F183" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="G183" t="inlineStr">
@@ -11168,7 +11180,7 @@
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
-      <c r="F184" s="1" t="n">
+      <c r="F184" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="G184" t="inlineStr">
@@ -11224,7 +11236,7 @@
           <t>66307562</t>
         </is>
       </c>
-      <c r="F185" s="1" t="n">
+      <c r="F185" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="G185" t="inlineStr">
@@ -11284,7 +11296,7 @@
           <t>66306759</t>
         </is>
       </c>
-      <c r="F186" s="1" t="n">
+      <c r="F186" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="G186" t="inlineStr">
@@ -11344,7 +11356,7 @@
           <t>66307058</t>
         </is>
       </c>
-      <c r="F187" s="1" t="n">
+      <c r="F187" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="G187" t="inlineStr">
@@ -11371,7 +11383,7 @@
         </is>
       </c>
       <c r="L187" t="inlineStr"/>
-      <c r="M187" s="1" t="n">
+      <c r="M187" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="N187" t="n">
@@ -11408,7 +11420,7 @@
           <t>21107</t>
         </is>
       </c>
-      <c r="F188" s="1" t="n">
+      <c r="F188" s="2" t="n">
         <v>45946</v>
       </c>
       <c r="G188" t="inlineStr">
@@ -11435,7 +11447,7 @@
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
-      <c r="M188" s="1" t="n">
+      <c r="M188" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="N188" t="inlineStr"/>
@@ -11474,7 +11486,7 @@
           <t>1318</t>
         </is>
       </c>
-      <c r="F189" s="1" t="n">
+      <c r="F189" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="G189" t="inlineStr">
@@ -11501,7 +11513,7 @@
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
-      <c r="M189" s="1" t="n">
+      <c r="M189" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="N189" t="inlineStr"/>
@@ -11536,7 +11548,7 @@
           <t>1608</t>
         </is>
       </c>
-      <c r="F190" s="1" t="n">
+      <c r="F190" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="G190" t="inlineStr">
@@ -11596,7 +11608,7 @@
           <t>17869</t>
         </is>
       </c>
-      <c r="F191" s="1" t="n">
+      <c r="F191" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="G191" t="inlineStr">
@@ -11623,7 +11635,7 @@
         </is>
       </c>
       <c r="L191" t="inlineStr"/>
-      <c r="M191" s="1" t="n">
+      <c r="M191" s="2" t="n">
         <v>45972</v>
       </c>
       <c r="N191" t="inlineStr"/>
@@ -11658,7 +11670,7 @@
           <t>T97147Q</t>
         </is>
       </c>
-      <c r="F192" s="1" t="n">
+      <c r="F192" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="G192" t="inlineStr">
@@ -11718,7 +11730,7 @@
           <t>07</t>
         </is>
       </c>
-      <c r="F193" s="1" t="n">
+      <c r="F193" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="G193" t="inlineStr">
@@ -11778,7 +11790,7 @@
           <t>6891</t>
         </is>
       </c>
-      <c r="F194" s="1" t="n">
+      <c r="F194" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="G194" t="inlineStr">
@@ -11828,7 +11840,7 @@
           <t>D12-10002</t>
         </is>
       </c>
-      <c r="F195" s="1" t="n">
+      <c r="F195" s="2" t="n">
         <v>45971</v>
       </c>
       <c r="G195" t="inlineStr">
@@ -11888,7 +11900,7 @@
           <t>0709LS</t>
         </is>
       </c>
-      <c r="F196" s="1" t="n">
+      <c r="F196" s="2" t="n">
         <v>45978</v>
       </c>
       <c r="G196" t="inlineStr">
@@ -11938,7 +11950,7 @@
           <t>H9533</t>
         </is>
       </c>
-      <c r="F197" s="1" t="n">
+      <c r="F197" s="2" t="n">
         <v>45978</v>
       </c>
       <c r="G197" t="inlineStr">
@@ -11988,7 +12000,7 @@
           <t>1902269</t>
         </is>
       </c>
-      <c r="F198" s="1" t="n">
+      <c r="F198" s="2" t="n">
         <v>45978</v>
       </c>
       <c r="G198" t="inlineStr">
@@ -12038,7 +12050,7 @@
           <t>1439</t>
         </is>
       </c>
-      <c r="F199" s="1" t="n">
+      <c r="F199" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="G199" t="inlineStr">
@@ -12065,7 +12077,7 @@
         </is>
       </c>
       <c r="L199" t="inlineStr"/>
-      <c r="M199" s="1" t="n">
+      <c r="M199" s="2" t="n">
         <v>46049</v>
       </c>
       <c r="N199" t="inlineStr"/>
@@ -12100,7 +12112,7 @@
           <t>182</t>
         </is>
       </c>
-      <c r="F200" s="1" t="n">
+      <c r="F200" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G200" t="inlineStr">
@@ -12160,7 +12172,7 @@
           <t>0707LS</t>
         </is>
       </c>
-      <c r="F201" s="1" t="n">
+      <c r="F201" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G201" t="inlineStr">
@@ -12220,7 +12232,7 @@
           <t>0801LS</t>
         </is>
       </c>
-      <c r="F202" s="1" t="n">
+      <c r="F202" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G202" t="inlineStr">
@@ -12280,7 +12292,7 @@
           <t>H9817</t>
         </is>
       </c>
-      <c r="F203" s="1" t="n">
+      <c r="F203" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G203" t="inlineStr">
@@ -12340,7 +12352,7 @@
           <t>37940</t>
         </is>
       </c>
-      <c r="F204" s="1" t="n">
+      <c r="F204" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G204" t="inlineStr">
@@ -12400,7 +12412,7 @@
           <t>39816</t>
         </is>
       </c>
-      <c r="F205" s="1" t="n">
+      <c r="F205" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G205" t="inlineStr">
@@ -12460,7 +12472,7 @@
           <t>89292</t>
         </is>
       </c>
-      <c r="F206" s="1" t="n">
+      <c r="F206" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G206" t="inlineStr">
@@ -12518,7 +12530,7 @@
           <t>96293</t>
         </is>
       </c>
-      <c r="F207" s="1" t="n">
+      <c r="F207" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G207" t="inlineStr">
@@ -12545,7 +12557,7 @@
         </is>
       </c>
       <c r="L207" t="inlineStr"/>
-      <c r="M207" s="1" t="n">
+      <c r="M207" s="2" t="n">
         <v>46153</v>
       </c>
       <c r="N207" t="inlineStr"/>
@@ -12580,7 +12592,7 @@
           <t>89287</t>
         </is>
       </c>
-      <c r="F208" s="1" t="n">
+      <c r="F208" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="G208" t="inlineStr">
@@ -12607,7 +12619,7 @@
         </is>
       </c>
       <c r="L208" t="inlineStr"/>
-      <c r="M208" s="1" t="n">
+      <c r="M208" s="2" t="n">
         <v>46031</v>
       </c>
       <c r="N208" t="inlineStr"/>
@@ -12642,7 +12654,7 @@
           <t>86805429</t>
         </is>
       </c>
-      <c r="F209" s="1" t="n">
+      <c r="F209" s="2" t="n">
         <v>46000</v>
       </c>
       <c r="G209" t="inlineStr">
@@ -12669,7 +12681,7 @@
         </is>
       </c>
       <c r="L209" t="inlineStr"/>
-      <c r="M209" s="1" t="n">
+      <c r="M209" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="N209" t="inlineStr"/>
@@ -12704,7 +12716,7 @@
           <t>073200G02170010AE</t>
         </is>
       </c>
-      <c r="F210" s="1" t="n">
+      <c r="F210" s="2" t="n">
         <v>46000</v>
       </c>
       <c r="G210" t="inlineStr">
@@ -12764,7 +12776,7 @@
           <t>073200G71030137AE</t>
         </is>
       </c>
-      <c r="F211" s="1" t="n">
+      <c r="F211" s="2" t="n">
         <v>46000</v>
       </c>
       <c r="G211" t="inlineStr">
@@ -12822,7 +12834,7 @@
           <t>073200G71360003AE</t>
         </is>
       </c>
-      <c r="F212" s="1" t="n">
+      <c r="F212" s="2" t="n">
         <v>46000</v>
       </c>
       <c r="G212" t="inlineStr">
@@ -12880,7 +12892,7 @@
           <t>01381310971</t>
         </is>
       </c>
-      <c r="F213" s="1" t="n">
+      <c r="F213" s="2" t="n">
         <v>46007</v>
       </c>
       <c r="G213" t="inlineStr">
@@ -12940,7 +12952,7 @@
           <t>KC225-3029</t>
         </is>
       </c>
-      <c r="F214" s="1" t="n">
+      <c r="F214" s="2" t="n">
         <v>46007</v>
       </c>
       <c r="G214" t="inlineStr">
@@ -12967,7 +12979,7 @@
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
-      <c r="M214" s="1" t="n">
+      <c r="M214" s="2" t="n">
         <v>46021</v>
       </c>
       <c r="N214" t="n">
@@ -13004,7 +13016,7 @@
           <t>1141111980</t>
         </is>
       </c>
-      <c r="F215" s="1" t="n">
+      <c r="F215" s="2" t="n">
         <v>46007</v>
       </c>
       <c r="G215" t="inlineStr">
@@ -13064,7 +13076,7 @@
           <t>A-184434</t>
         </is>
       </c>
-      <c r="F216" s="1" t="n">
+      <c r="F216" s="2" t="n">
         <v>46010</v>
       </c>
       <c r="G216" t="inlineStr">
@@ -13114,7 +13126,7 @@
           <t>3201</t>
         </is>
       </c>
-      <c r="F217" s="1" t="n">
+      <c r="F217" s="2" t="n">
         <v>46010</v>
       </c>
       <c r="G217" t="inlineStr">
@@ -13141,7 +13153,7 @@
         </is>
       </c>
       <c r="L217" t="inlineStr"/>
-      <c r="M217" s="1" t="n">
+      <c r="M217" s="2" t="n">
         <v>46052</v>
       </c>
       <c r="N217" t="inlineStr"/>
@@ -13176,7 +13188,7 @@
           <t>A-183643</t>
         </is>
       </c>
-      <c r="F218" s="1" t="n">
+      <c r="F218" s="2" t="n">
         <v>46010</v>
       </c>
       <c r="G218" t="inlineStr">
@@ -13236,7 +13248,7 @@
           <t>A-180560</t>
         </is>
       </c>
-      <c r="F219" s="1" t="n">
+      <c r="F219" s="2" t="n">
         <v>46010</v>
       </c>
       <c r="G219" t="inlineStr">
@@ -13296,7 +13308,7 @@
           <t>A-134709</t>
         </is>
       </c>
-      <c r="F220" s="1" t="n">
+      <c r="F220" s="2" t="n">
         <v>46010</v>
       </c>
       <c r="G220" t="inlineStr">
@@ -13356,7 +13368,7 @@
           <t>822</t>
         </is>
       </c>
-      <c r="F221" s="1" t="n">
+      <c r="F221" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G221" t="inlineStr">
@@ -13414,7 +13426,7 @@
           <t>795</t>
         </is>
       </c>
-      <c r="F222" s="1" t="n">
+      <c r="F222" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G222" t="inlineStr">
@@ -13474,7 +13486,7 @@
           <t>784</t>
         </is>
       </c>
-      <c r="F223" s="1" t="n">
+      <c r="F223" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G223" t="inlineStr">
@@ -13534,7 +13546,7 @@
           <t>482</t>
         </is>
       </c>
-      <c r="F224" s="1" t="n">
+      <c r="F224" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G224" t="inlineStr">
@@ -13594,7 +13606,7 @@
           <t>LSEAM3218</t>
         </is>
       </c>
-      <c r="F225" s="1" t="n">
+      <c r="F225" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G225" t="inlineStr">
@@ -13654,7 +13666,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="F226" s="1" t="n">
+      <c r="F226" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G226" t="inlineStr">
@@ -13714,7 +13726,7 @@
           <t>LSEAM3167</t>
         </is>
       </c>
-      <c r="F227" s="1" t="n">
+      <c r="F227" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G227" t="inlineStr">
@@ -13774,7 +13786,7 @@
           <t>01B</t>
         </is>
       </c>
-      <c r="F228" s="1" t="n">
+      <c r="F228" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G228" t="inlineStr">
@@ -13834,7 +13846,7 @@
           <t>392-000003</t>
         </is>
       </c>
-      <c r="F229" s="1" t="n">
+      <c r="F229" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G229" t="inlineStr">
@@ -13892,7 +13904,7 @@
           <t>073200G90080062AE</t>
         </is>
       </c>
-      <c r="F230" s="1" t="n">
+      <c r="F230" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G230" t="inlineStr">
@@ -13952,7 +13964,7 @@
           <t>073200G02170087AE</t>
         </is>
       </c>
-      <c r="F231" s="1" t="n">
+      <c r="F231" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G231" t="inlineStr">
@@ -13979,7 +13991,7 @@
         </is>
       </c>
       <c r="L231" t="inlineStr"/>
-      <c r="M231" s="1" t="n">
+      <c r="M231" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="N231" t="inlineStr"/>
@@ -14014,7 +14026,7 @@
           <t>073200G02170089AE</t>
         </is>
       </c>
-      <c r="F232" s="1" t="n">
+      <c r="F232" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G232" t="inlineStr">
@@ -14072,7 +14084,7 @@
           <t>073200G63200008AE</t>
         </is>
       </c>
-      <c r="F233" s="1" t="n">
+      <c r="F233" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G233" t="inlineStr">
@@ -14130,7 +14142,7 @@
           <t>073200G02170034AE</t>
         </is>
       </c>
-      <c r="F234" s="1" t="n">
+      <c r="F234" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G234" t="inlineStr">
@@ -14157,7 +14169,7 @@
         </is>
       </c>
       <c r="L234" t="inlineStr"/>
-      <c r="M234" s="1" t="n">
+      <c r="M234" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="N234" t="inlineStr"/>
@@ -14196,7 +14208,7 @@
           <t>073200G90080045AE</t>
         </is>
       </c>
-      <c r="F235" s="1" t="n">
+      <c r="F235" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G235" t="inlineStr">
@@ -14223,7 +14235,7 @@
         </is>
       </c>
       <c r="L235" t="inlineStr"/>
-      <c r="M235" s="1" t="n">
+      <c r="M235" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="N235" t="inlineStr"/>
@@ -14262,7 +14274,7 @@
           <t>2165</t>
         </is>
       </c>
-      <c r="F236" s="1" t="n">
+      <c r="F236" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G236" t="inlineStr">
@@ -14289,7 +14301,7 @@
         </is>
       </c>
       <c r="L236" t="inlineStr"/>
-      <c r="M236" s="1" t="n">
+      <c r="M236" s="2" t="n">
         <v>46114</v>
       </c>
       <c r="N236" t="inlineStr"/>
@@ -14324,7 +14336,7 @@
           <t>1270</t>
         </is>
       </c>
-      <c r="F237" s="1" t="n">
+      <c r="F237" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G237" t="inlineStr">
@@ -14384,7 +14396,7 @@
           <t>B10274</t>
         </is>
       </c>
-      <c r="F238" s="1" t="n">
+      <c r="F238" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="G238" t="inlineStr">
@@ -14434,7 +14446,7 @@
           <t>F66933</t>
         </is>
       </c>
-      <c r="F239" s="1" t="n">
+      <c r="F239" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="G239" t="inlineStr">
@@ -14461,7 +14473,7 @@
         </is>
       </c>
       <c r="L239" t="inlineStr"/>
-      <c r="M239" s="1" t="n">
+      <c r="M239" s="2" t="n">
         <v>46052</v>
       </c>
       <c r="N239" t="inlineStr"/>
@@ -14496,7 +14508,7 @@
           <t>C66477</t>
         </is>
       </c>
-      <c r="F240" s="1" t="n">
+      <c r="F240" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="G240" t="inlineStr">
@@ -14554,7 +14566,7 @@
           <t>A76103</t>
         </is>
       </c>
-      <c r="F241" s="1" t="n">
+      <c r="F241" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="G241" t="inlineStr">
@@ -14612,7 +14624,7 @@
           <t>B10380</t>
         </is>
       </c>
-      <c r="F242" s="1" t="n">
+      <c r="F242" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="G242" t="inlineStr">
@@ -14672,7 +14684,7 @@
           <t>6949</t>
         </is>
       </c>
-      <c r="F243" s="1" t="n">
+      <c r="F243" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="G243" t="inlineStr">
@@ -14726,7 +14738,7 @@
           <t>24277</t>
         </is>
       </c>
-      <c r="F244" s="1" t="n">
+      <c r="F244" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="G244" t="inlineStr">
@@ -14786,7 +14798,7 @@
           <t>22102</t>
         </is>
       </c>
-      <c r="F245" s="1" t="n">
+      <c r="F245" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="G245" t="inlineStr">
@@ -14846,7 +14858,7 @@
           <t>002798</t>
         </is>
       </c>
-      <c r="F246" s="1" t="n">
+      <c r="F246" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="G246" t="inlineStr">
@@ -14873,7 +14885,7 @@
         </is>
       </c>
       <c r="L246" t="inlineStr"/>
-      <c r="M246" s="1" t="n">
+      <c r="M246" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="N246" t="inlineStr"/>
@@ -14908,7 +14920,7 @@
           <t>004106</t>
         </is>
       </c>
-      <c r="F247" s="1" t="n">
+      <c r="F247" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="G247" t="inlineStr">
@@ -14958,7 +14970,7 @@
           <t>968</t>
         </is>
       </c>
-      <c r="F248" s="1" t="n">
+      <c r="F248" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="G248" t="inlineStr">
@@ -15008,7 +15020,7 @@
           <t>2L094</t>
         </is>
       </c>
-      <c r="F249" s="1" t="n">
+      <c r="F249" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="G249" t="inlineStr">
@@ -15068,7 +15080,7 @@
           <t>003665</t>
         </is>
       </c>
-      <c r="F250" s="1" t="n">
+      <c r="F250" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G250" t="inlineStr">
@@ -15128,7 +15140,7 @@
           <t>004201</t>
         </is>
       </c>
-      <c r="F251" s="1" t="n">
+      <c r="F251" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G251" t="inlineStr">
@@ -15186,7 +15198,7 @@
           <t>004207</t>
         </is>
       </c>
-      <c r="F252" s="1" t="n">
+      <c r="F252" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G252" t="inlineStr">
@@ -15244,7 +15256,7 @@
           <t>1656</t>
         </is>
       </c>
-      <c r="F253" s="1" t="n">
+      <c r="F253" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G253" t="inlineStr">
@@ -15304,7 +15316,7 @@
           <t>T49314</t>
         </is>
       </c>
-      <c r="F254" s="1" t="n">
+      <c r="F254" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G254" t="inlineStr">
@@ -15364,7 +15376,7 @@
           <t>T49816</t>
         </is>
       </c>
-      <c r="F255" s="1" t="n">
+      <c r="F255" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G255" t="inlineStr">
@@ -15424,7 +15436,7 @@
           <t>46710866</t>
         </is>
       </c>
-      <c r="F256" s="1" t="n">
+      <c r="F256" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G256" t="inlineStr">
@@ -15486,7 +15498,7 @@
           <t>20624851</t>
         </is>
       </c>
-      <c r="F257" s="1" t="n">
+      <c r="F257" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G257" t="inlineStr">
@@ -15536,7 +15548,7 @@
           <t>20625310</t>
         </is>
       </c>
-      <c r="F258" s="1" t="n">
+      <c r="F258" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G258" t="inlineStr">
@@ -15586,7 +15598,7 @@
           <t>2926</t>
         </is>
       </c>
-      <c r="F259" s="1" t="n">
+      <c r="F259" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G259" t="inlineStr">
@@ -15646,7 +15658,7 @@
           <t>12023</t>
         </is>
       </c>
-      <c r="F260" s="1" t="n">
+      <c r="F260" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G260" t="inlineStr">
@@ -15706,7 +15718,7 @@
           <t>KAS297B-A23223</t>
         </is>
       </c>
-      <c r="F261" s="1" t="n">
+      <c r="F261" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G261" t="inlineStr">
@@ -15766,7 +15778,7 @@
           <t>42966</t>
         </is>
       </c>
-      <c r="F262" s="1" t="n">
+      <c r="F262" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G262" t="inlineStr">
@@ -15793,7 +15805,7 @@
         </is>
       </c>
       <c r="L262" t="inlineStr"/>
-      <c r="M262" s="1" t="n">
+      <c r="M262" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="N262" t="inlineStr"/>
@@ -15832,7 +15844,7 @@
           <t>48741</t>
         </is>
       </c>
-      <c r="F263" s="1" t="n">
+      <c r="F263" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G263" t="inlineStr">
@@ -15890,7 +15902,7 @@
           <t>21940</t>
         </is>
       </c>
-      <c r="F264" s="1" t="n">
+      <c r="F264" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G264" t="inlineStr">
@@ -15950,7 +15962,7 @@
           <t>22950</t>
         </is>
       </c>
-      <c r="F265" s="1" t="n">
+      <c r="F265" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G265" t="inlineStr">
@@ -16010,7 +16022,7 @@
           <t>7310</t>
         </is>
       </c>
-      <c r="F266" s="1" t="n">
+      <c r="F266" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G266" t="inlineStr">
@@ -16070,7 +16082,7 @@
           <t>11154</t>
         </is>
       </c>
-      <c r="F267" s="1" t="n">
+      <c r="F267" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G267" t="inlineStr">
@@ -16130,7 +16142,7 @@
           <t>17714</t>
         </is>
       </c>
-      <c r="F268" s="1" t="n">
+      <c r="F268" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G268" t="inlineStr">
@@ -16186,7 +16198,7 @@
         </is>
       </c>
       <c r="E269" t="inlineStr"/>
-      <c r="F269" s="1" t="n">
+      <c r="F269" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G269" t="inlineStr">
@@ -16246,7 +16258,7 @@
           <t>KTA77B-A87365</t>
         </is>
       </c>
-      <c r="F270" s="1" t="n">
+      <c r="F270" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G270" t="inlineStr">
@@ -16306,7 +16318,7 @@
           <t>8306</t>
         </is>
       </c>
-      <c r="F271" s="1" t="n">
+      <c r="F271" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G271" t="inlineStr">
@@ -16366,7 +16378,7 @@
           <t>5BE34</t>
         </is>
       </c>
-      <c r="F272" s="1" t="n">
+      <c r="F272" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G272" t="inlineStr">
@@ -16393,7 +16405,7 @@
         </is>
       </c>
       <c r="L272" t="inlineStr"/>
-      <c r="M272" s="1" t="n">
+      <c r="M272" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="N272" t="inlineStr">
@@ -16432,7 +16444,7 @@
           <t>S4H004</t>
         </is>
       </c>
-      <c r="F273" s="1" t="n">
+      <c r="F273" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G273" t="inlineStr">
@@ -16490,7 +16502,7 @@
           <t>0919</t>
         </is>
       </c>
-      <c r="F274" s="1" t="n">
+      <c r="F274" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G274" t="inlineStr">
@@ -16550,7 +16562,7 @@
           <t>B4H-015</t>
         </is>
       </c>
-      <c r="F275" s="1" t="n">
+      <c r="F275" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G275" t="inlineStr">
@@ -16608,7 +16620,7 @@
           <t>B4H-011</t>
         </is>
       </c>
-      <c r="F276" s="1" t="n">
+      <c r="F276" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G276" t="inlineStr">
@@ -16668,7 +16680,7 @@
           <t>20675473</t>
         </is>
       </c>
-      <c r="F277" s="1" t="n">
+      <c r="F277" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="G277" t="inlineStr">
@@ -16728,7 +16740,7 @@
           <t>470055</t>
         </is>
       </c>
-      <c r="F278" s="1" t="n">
+      <c r="F278" s="2" t="n">
         <v>46077</v>
       </c>
       <c r="G278" t="inlineStr">
@@ -16788,7 +16800,7 @@
           <t>471591</t>
         </is>
       </c>
-      <c r="F279" s="1" t="n">
+      <c r="F279" s="2" t="n">
         <v>46077</v>
       </c>
       <c r="G279" t="inlineStr">
@@ -16852,7 +16864,7 @@
           <t>8868</t>
         </is>
       </c>
-      <c r="F280" s="1" t="n">
+      <c r="F280" s="2" t="n">
         <v>46085</v>
       </c>
       <c r="G280" t="inlineStr">
@@ -16912,7 +16924,7 @@
           <t>4965</t>
         </is>
       </c>
-      <c r="F281" s="1" t="n">
+      <c r="F281" s="2" t="n">
         <v>46085</v>
       </c>
       <c r="G281" t="inlineStr">
@@ -16972,7 +16984,7 @@
           <t>000745</t>
         </is>
       </c>
-      <c r="F282" s="1" t="n">
+      <c r="F282" s="2" t="n">
         <v>46090</v>
       </c>
       <c r="G282" t="inlineStr">
@@ -17030,7 +17042,7 @@
           <t>8459XL2</t>
         </is>
       </c>
-      <c r="F283" s="1" t="n">
+      <c r="F283" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="G283" t="inlineStr">
@@ -17086,7 +17098,7 @@
           <t>S00062XL</t>
         </is>
       </c>
-      <c r="F284" s="1" t="n">
+      <c r="F284" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="G284" t="inlineStr">
@@ -17142,7 +17154,7 @@
           <t>073200G02170082AE</t>
         </is>
       </c>
-      <c r="F285" s="1" t="n">
+      <c r="F285" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="G285" t="inlineStr">
@@ -17198,7 +17210,7 @@
           <t>073200G91260061AE</t>
         </is>
       </c>
-      <c r="F286" s="1" t="n">
+      <c r="F286" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="G286" t="inlineStr">
@@ -17252,7 +17264,7 @@
       <c r="E287" t="n">
         <v>35971</v>
       </c>
-      <c r="F287" s="1" t="n">
+      <c r="F287" s="2" t="n">
         <v>46107</v>
       </c>
       <c r="G287" t="inlineStr">
@@ -17298,7 +17310,7 @@
       <c r="E288" t="n">
         <v>107178</v>
       </c>
-      <c r="F288" s="1" t="n">
+      <c r="F288" s="2" t="n">
         <v>46107</v>
       </c>
       <c r="G288" t="inlineStr">
@@ -17354,7 +17366,7 @@
       <c r="E289" t="n">
         <v>108773</v>
       </c>
-      <c r="F289" s="1" t="n">
+      <c r="F289" s="2" t="n">
         <v>46107</v>
       </c>
       <c r="G289" t="inlineStr">
@@ -17402,7 +17414,7 @@
       <c r="E290" t="n">
         <v>7086</v>
       </c>
-      <c r="F290" s="1" t="n">
+      <c r="F290" s="2" t="n">
         <v>46107</v>
       </c>
       <c r="G290" t="inlineStr">
@@ -17425,7 +17437,7 @@
       </c>
       <c r="K290" t="inlineStr"/>
       <c r="L290" t="inlineStr"/>
-      <c r="M290" s="1" t="n">
+      <c r="M290" s="2" t="n">
         <v>46127</v>
       </c>
       <c r="N290" t="inlineStr"/>
@@ -17456,7 +17468,7 @@
       <c r="E291" t="n">
         <v>99743</v>
       </c>
-      <c r="F291" s="1" t="n">
+      <c r="F291" s="2" t="n">
         <v>46107</v>
       </c>
       <c r="G291" t="inlineStr">
@@ -17514,7 +17526,7 @@
           <t>KS272A-49392</t>
         </is>
       </c>
-      <c r="F292" s="1" t="n">
+      <c r="F292" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="G292" t="inlineStr">
@@ -17572,7 +17584,7 @@
           <t>B-10811222</t>
         </is>
       </c>
-      <c r="F293" s="1" t="n">
+      <c r="F293" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G293" t="inlineStr">
@@ -17630,7 +17642,7 @@
           <t>B10811221</t>
         </is>
       </c>
-      <c r="F294" s="1" t="n">
+      <c r="F294" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G294" t="inlineStr">
@@ -17684,7 +17696,7 @@
           <t>B10811220</t>
         </is>
       </c>
-      <c r="F295" s="1" t="n">
+      <c r="F295" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G295" t="inlineStr">
@@ -17738,7 +17750,7 @@
           <t>B10811724</t>
         </is>
       </c>
-      <c r="F296" s="1" t="n">
+      <c r="F296" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G296" t="inlineStr">
@@ -17792,7 +17804,7 @@
       <c r="E297" t="n">
         <v>47203152</v>
       </c>
-      <c r="F297" s="1" t="n">
+      <c r="F297" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G297" t="inlineStr">
@@ -17850,7 +17862,7 @@
       <c r="E298" t="n">
         <v>47202512</v>
       </c>
-      <c r="F298" s="1" t="n">
+      <c r="F298" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G298" t="inlineStr">
@@ -17908,7 +17920,7 @@
       <c r="E299" t="n">
         <v>22005580</v>
       </c>
-      <c r="F299" s="1" t="n">
+      <c r="F299" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G299" t="inlineStr">
@@ -17966,7 +17978,7 @@
       <c r="E300" t="n">
         <v>22005955</v>
       </c>
-      <c r="F300" s="1" t="n">
+      <c r="F300" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G300" t="inlineStr">
@@ -18024,7 +18036,7 @@
       <c r="E301" t="n">
         <v>22005661</v>
       </c>
-      <c r="F301" s="1" t="n">
+      <c r="F301" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G301" t="inlineStr">
@@ -18080,7 +18092,7 @@
       <c r="E302" t="n">
         <v>32207</v>
       </c>
-      <c r="F302" s="1" t="n">
+      <c r="F302" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G302" t="inlineStr">
@@ -18136,7 +18148,7 @@
       <c r="E303" t="n">
         <v>18156</v>
       </c>
-      <c r="F303" s="1" t="n">
+      <c r="F303" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G303" t="inlineStr">
@@ -18192,7 +18204,7 @@
       <c r="E304" t="n">
         <v>37971</v>
       </c>
-      <c r="F304" s="1" t="n">
+      <c r="F304" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G304" t="inlineStr">
@@ -18248,7 +18260,7 @@
       <c r="E305" t="n">
         <v>84317</v>
       </c>
-      <c r="F305" s="1" t="n">
+      <c r="F305" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G305" t="inlineStr">
@@ -18275,7 +18287,7 @@
         </is>
       </c>
       <c r="L305" t="inlineStr"/>
-      <c r="M305" s="1" t="n">
+      <c r="M305" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="N305" t="inlineStr"/>
@@ -18306,7 +18318,7 @@
       <c r="E306" t="n">
         <v>83773</v>
       </c>
-      <c r="F306" s="1" t="n">
+      <c r="F306" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G306" t="inlineStr">
@@ -18333,7 +18345,7 @@
         </is>
       </c>
       <c r="L306" t="inlineStr"/>
-      <c r="M306" s="1" t="n">
+      <c r="M306" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="N306" t="inlineStr"/>
@@ -18364,7 +18376,7 @@
       <c r="E307" t="n">
         <v>83740</v>
       </c>
-      <c r="F307" s="1" t="n">
+      <c r="F307" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G307" t="inlineStr">
@@ -18420,7 +18432,7 @@
       <c r="E308" t="n">
         <v>84326</v>
       </c>
-      <c r="F308" s="1" t="n">
+      <c r="F308" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G308" t="inlineStr">
@@ -18476,7 +18488,7 @@
       <c r="E309" t="n">
         <v>6708</v>
       </c>
-      <c r="F309" s="1" t="n">
+      <c r="F309" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G309" t="inlineStr">
@@ -18534,7 +18546,7 @@
           <t>LSEAM3269</t>
         </is>
       </c>
-      <c r="F310" s="1" t="n">
+      <c r="F310" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G310" t="inlineStr">
@@ -18590,7 +18602,7 @@
       <c r="E311" t="n">
         <v>9727</v>
       </c>
-      <c r="F311" s="1" t="n">
+      <c r="F311" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G311" t="inlineStr">
@@ -18648,7 +18660,7 @@
           <t>LSEAM3168</t>
         </is>
       </c>
-      <c r="F312" s="1" t="n">
+      <c r="F312" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G312" t="inlineStr">
@@ -18704,7 +18716,7 @@
       <c r="E313" t="n">
         <v>31</v>
       </c>
-      <c r="F313" s="1" t="n">
+      <c r="F313" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G313" t="inlineStr">
@@ -18758,7 +18770,7 @@
       <c r="E314" t="n">
         <v>965</v>
       </c>
-      <c r="F314" s="1" t="n">
+      <c r="F314" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G314" t="inlineStr">
@@ -18814,7 +18826,7 @@
       <c r="E315" t="n">
         <v>2007</v>
       </c>
-      <c r="F315" s="1" t="n">
+      <c r="F315" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G315" t="inlineStr">
@@ -18870,7 +18882,7 @@
       <c r="E316" t="n">
         <v>688</v>
       </c>
-      <c r="F316" s="1" t="n">
+      <c r="F316" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G316" t="inlineStr">
@@ -18928,7 +18940,7 @@
           <t>B4H-038</t>
         </is>
       </c>
-      <c r="F317" s="1" t="n">
+      <c r="F317" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G317" t="inlineStr">
@@ -18986,7 +18998,7 @@
           <t>1938-XL</t>
         </is>
       </c>
-      <c r="F318" s="1" t="n">
+      <c r="F318" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G318" t="inlineStr">
@@ -19034,7 +19046,7 @@
           <t>3711XL</t>
         </is>
       </c>
-      <c r="F319" s="1" t="n">
+      <c r="F319" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G319" t="inlineStr">
@@ -19059,7 +19071,7 @@
         </is>
       </c>
       <c r="L319" t="inlineStr"/>
-      <c r="M319" s="1" t="n">
+      <c r="M319" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="N319" t="inlineStr"/>
@@ -19090,7 +19102,7 @@
       <c r="E320" t="n">
         <v>1391</v>
       </c>
-      <c r="F320" s="1" t="n">
+      <c r="F320" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G320" t="inlineStr">
@@ -19148,7 +19160,7 @@
       <c r="E321" t="n">
         <v>120315</v>
       </c>
-      <c r="F321" s="1" t="n">
+      <c r="F321" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G321" t="inlineStr">
@@ -19208,7 +19220,7 @@
           <t>1588-5</t>
         </is>
       </c>
-      <c r="F322" s="1" t="n">
+      <c r="F322" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G322" t="inlineStr">
@@ -19235,7 +19247,7 @@
         </is>
       </c>
       <c r="L322" t="inlineStr"/>
-      <c r="M322" s="1" t="n">
+      <c r="M322" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="N322" t="inlineStr"/>
@@ -19268,7 +19280,7 @@
       <c r="E323" t="n">
         <v>535933</v>
       </c>
-      <c r="F323" s="1" t="n">
+      <c r="F323" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G323" t="inlineStr">
@@ -19326,7 +19338,7 @@
       <c r="E324" t="n">
         <v>289029</v>
       </c>
-      <c r="F324" s="1" t="n">
+      <c r="F324" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G324" t="inlineStr">
@@ -19384,7 +19396,7 @@
       <c r="E325" t="n">
         <v>3454</v>
       </c>
-      <c r="F325" s="1" t="n">
+      <c r="F325" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G325" t="inlineStr">
@@ -19411,7 +19423,7 @@
         </is>
       </c>
       <c r="L325" t="inlineStr"/>
-      <c r="M325" s="1" t="n">
+      <c r="M325" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="N325" t="inlineStr"/>
@@ -19444,7 +19456,7 @@
       <c r="E326" t="n">
         <v>3493</v>
       </c>
-      <c r="F326" s="1" t="n">
+      <c r="F326" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G326" t="inlineStr">
@@ -19504,7 +19516,7 @@
           <t>1588-5</t>
         </is>
       </c>
-      <c r="F327" s="1" t="n">
+      <c r="F327" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G327" t="inlineStr">
@@ -19531,7 +19543,7 @@
         </is>
       </c>
       <c r="L327" t="inlineStr"/>
-      <c r="M327" s="1" t="n">
+      <c r="M327" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="N327" t="inlineStr"/>
@@ -19564,7 +19576,7 @@
       <c r="E328" t="n">
         <v>3235</v>
       </c>
-      <c r="F328" s="1" t="n">
+      <c r="F328" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G328" t="inlineStr">
@@ -19591,7 +19603,7 @@
         </is>
       </c>
       <c r="L328" t="inlineStr"/>
-      <c r="M328" s="1" t="n">
+      <c r="M328" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="N328" t="inlineStr"/>
@@ -19624,7 +19636,7 @@
       <c r="E329" t="n">
         <v>625052</v>
       </c>
-      <c r="F329" s="1" t="n">
+      <c r="F329" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G329" t="inlineStr">
@@ -19651,7 +19663,7 @@
         </is>
       </c>
       <c r="L329" t="inlineStr"/>
-      <c r="M329" s="1" t="n">
+      <c r="M329" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="N329" t="inlineStr"/>
@@ -19684,7 +19696,7 @@
       <c r="E330" t="n">
         <v>614095</v>
       </c>
-      <c r="F330" s="1" t="n">
+      <c r="F330" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G330" t="inlineStr">
@@ -19711,7 +19723,7 @@
         </is>
       </c>
       <c r="L330" t="inlineStr"/>
-      <c r="M330" s="1" t="n">
+      <c r="M330" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="N330" t="inlineStr"/>
@@ -19744,7 +19756,7 @@
           <t>B10274</t>
         </is>
       </c>
-      <c r="F331" s="1" t="n">
+      <c r="F331" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G331" t="inlineStr">
@@ -19802,7 +19814,7 @@
           <t>9715-096</t>
         </is>
       </c>
-      <c r="F332" s="1" t="n">
+      <c r="F332" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G332" t="inlineStr">
@@ -19858,7 +19870,7 @@
       <c r="E333" t="n">
         <v>197</v>
       </c>
-      <c r="F333" s="1" t="n">
+      <c r="F333" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G333" t="inlineStr">
@@ -19914,7 +19926,7 @@
       <c r="E334" t="n">
         <v>1378</v>
       </c>
-      <c r="F334" s="1" t="n">
+      <c r="F334" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="G334" t="inlineStr">
@@ -19974,7 +19986,7 @@
           <t>ATE2717</t>
         </is>
       </c>
-      <c r="F335" s="1" t="n">
+      <c r="F335" s="2" t="n">
         <v>46127</v>
       </c>
       <c r="G335" t="inlineStr">
@@ -19999,7 +20011,7 @@
         </is>
       </c>
       <c r="L335" t="inlineStr"/>
-      <c r="M335" s="1" t="n">
+      <c r="M335" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="N335" t="inlineStr"/>
@@ -20034,7 +20046,7 @@
           <t>LS005</t>
         </is>
       </c>
-      <c r="F336" s="1" t="n">
+      <c r="F336" s="2" t="n">
         <v>46127</v>
       </c>
       <c r="G336" t="inlineStr">
@@ -20094,7 +20106,7 @@
           <t>ATE2714</t>
         </is>
       </c>
-      <c r="F337" s="1" t="n">
+      <c r="F337" s="2" t="n">
         <v>46127</v>
       </c>
       <c r="G337" t="inlineStr">
@@ -20119,7 +20131,7 @@
         </is>
       </c>
       <c r="L337" t="inlineStr"/>
-      <c r="M337" s="1" t="n">
+      <c r="M337" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="N337" t="inlineStr"/>
@@ -20154,7 +20166,7 @@
           <t>ATE2730</t>
         </is>
       </c>
-      <c r="F338" s="1" t="n">
+      <c r="F338" s="2" t="n">
         <v>46127</v>
       </c>
       <c r="G338" t="inlineStr">
@@ -20210,7 +20222,7 @@
       <c r="E339" t="n">
         <v>6291</v>
       </c>
-      <c r="F339" s="1" t="n">
+      <c r="F339" s="2" t="n">
         <v>46129</v>
       </c>
       <c r="G339" t="inlineStr">
@@ -20260,7 +20272,7 @@
           <t>1062</t>
         </is>
       </c>
-      <c r="F340" s="1" t="n">
+      <c r="F340" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G340" t="inlineStr">
@@ -20320,7 +20332,7 @@
           <t>8619</t>
         </is>
       </c>
-      <c r="F341" s="1" t="n">
+      <c r="F341" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G341" t="inlineStr">
@@ -20380,7 +20392,7 @@
           <t>4136</t>
         </is>
       </c>
-      <c r="F342" s="1" t="n">
+      <c r="F342" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G342" t="inlineStr">
@@ -20440,7 +20452,7 @@
           <t>T35158</t>
         </is>
       </c>
-      <c r="F343" s="1" t="n">
+      <c r="F343" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G343" t="inlineStr">
@@ -20500,7 +20512,7 @@
           <t>T35507</t>
         </is>
       </c>
-      <c r="F344" s="1" t="n">
+      <c r="F344" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G344" t="inlineStr">
@@ -20560,7 +20572,7 @@
           <t>20238</t>
         </is>
       </c>
-      <c r="F345" s="1" t="n">
+      <c r="F345" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G345" t="inlineStr">
@@ -20620,7 +20632,7 @@
           <t>102549</t>
         </is>
       </c>
-      <c r="F346" s="1" t="n">
+      <c r="F346" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G346" t="inlineStr">
@@ -20680,7 +20692,7 @@
           <t>16784</t>
         </is>
       </c>
-      <c r="F347" s="1" t="n">
+      <c r="F347" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G347" t="inlineStr">
@@ -20707,7 +20719,7 @@
         </is>
       </c>
       <c r="L347" t="inlineStr"/>
-      <c r="M347" s="1" t="n">
+      <c r="M347" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="N347" t="inlineStr"/>
@@ -20742,7 +20754,7 @@
           <t>16810</t>
         </is>
       </c>
-      <c r="F348" s="1" t="n">
+      <c r="F348" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G348" t="inlineStr">
@@ -20769,7 +20781,7 @@
         </is>
       </c>
       <c r="L348" t="inlineStr"/>
-      <c r="M348" s="1" t="n">
+      <c r="M348" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="N348" t="inlineStr"/>
@@ -20804,7 +20816,7 @@
           <t>108207</t>
         </is>
       </c>
-      <c r="F349" s="1" t="n">
+      <c r="F349" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G349" t="inlineStr">
@@ -20864,7 +20876,7 @@
           <t>4152</t>
         </is>
       </c>
-      <c r="F350" s="1" t="n">
+      <c r="F350" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G350" t="inlineStr">
@@ -20920,7 +20932,7 @@
           <t>96123</t>
         </is>
       </c>
-      <c r="F351" s="1" t="n">
+      <c r="F351" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G351" t="inlineStr">
@@ -20980,7 +20992,7 @@
           <t>4100932</t>
         </is>
       </c>
-      <c r="F352" s="1" t="n">
+      <c r="F352" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G352" t="inlineStr">
@@ -21040,7 +21052,7 @@
           <t>T36593</t>
         </is>
       </c>
-      <c r="F353" s="1" t="n">
+      <c r="F353" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G353" t="inlineStr">
@@ -21100,7 +21112,7 @@
           <t>30316</t>
         </is>
       </c>
-      <c r="F354" s="1" t="n">
+      <c r="F354" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G354" t="inlineStr">
@@ -21160,7 +21172,7 @@
           <t>4155</t>
         </is>
       </c>
-      <c r="F355" s="1" t="n">
+      <c r="F355" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G355" t="inlineStr">
@@ -21187,7 +21199,7 @@
         </is>
       </c>
       <c r="L355" t="inlineStr"/>
-      <c r="M355" s="1" t="n">
+      <c r="M355" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="N355" t="inlineStr"/>
@@ -21222,7 +21234,7 @@
           <t>18685</t>
         </is>
       </c>
-      <c r="F356" s="1" t="n">
+      <c r="F356" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G356" t="inlineStr">
@@ -21247,7 +21259,7 @@
         </is>
       </c>
       <c r="L356" t="inlineStr"/>
-      <c r="M356" s="1" t="n">
+      <c r="M356" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="N356" t="inlineStr"/>
@@ -21282,7 +21294,7 @@
           <t>86815595</t>
         </is>
       </c>
-      <c r="F357" s="1" t="n">
+      <c r="F357" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G357" t="inlineStr">
@@ -21342,7 +21354,7 @@
           <t>86816588</t>
         </is>
       </c>
-      <c r="F358" s="1" t="n">
+      <c r="F358" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G358" t="inlineStr">
@@ -21402,7 +21414,7 @@
           <t>86815646</t>
         </is>
       </c>
-      <c r="F359" s="1" t="n">
+      <c r="F359" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G359" t="inlineStr">
@@ -21462,7 +21474,7 @@
           <t>T23740</t>
         </is>
       </c>
-      <c r="F360" s="1" t="n">
+      <c r="F360" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G360" t="inlineStr">
@@ -21522,7 +21534,7 @@
           <t>T20503</t>
         </is>
       </c>
-      <c r="F361" s="1" t="n">
+      <c r="F361" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G361" t="inlineStr">
@@ -21582,7 +21594,7 @@
           <t>T23036</t>
         </is>
       </c>
-      <c r="F362" s="1" t="n">
+      <c r="F362" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G362" t="inlineStr">
@@ -21642,7 +21654,7 @@
           <t>T25488</t>
         </is>
       </c>
-      <c r="F363" s="1" t="n">
+      <c r="F363" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G363" t="inlineStr">
@@ -21702,7 +21714,7 @@
           <t>T22974</t>
         </is>
       </c>
-      <c r="F364" s="1" t="n">
+      <c r="F364" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G364" t="inlineStr">
@@ -21762,7 +21774,7 @@
           <t>4112112</t>
         </is>
       </c>
-      <c r="F365" s="1" t="n">
+      <c r="F365" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="G365" t="inlineStr">
@@ -21822,7 +21834,7 @@
           <t>30559</t>
         </is>
       </c>
-      <c r="F366" s="1" t="n">
+      <c r="F366" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G366" t="inlineStr">
@@ -21882,7 +21894,7 @@
           <t>34851</t>
         </is>
       </c>
-      <c r="F367" s="1" t="n">
+      <c r="F367" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G367" t="inlineStr">
@@ -21942,7 +21954,7 @@
           <t>3958</t>
         </is>
       </c>
-      <c r="F368" s="1" t="n">
+      <c r="F368" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G368" t="inlineStr">
@@ -22002,7 +22014,7 @@
           <t>4157</t>
         </is>
       </c>
-      <c r="F369" s="1" t="n">
+      <c r="F369" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G369" t="inlineStr">
@@ -22062,7 +22074,7 @@
           <t>2913</t>
         </is>
       </c>
-      <c r="F370" s="1" t="n">
+      <c r="F370" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G370" t="inlineStr">
@@ -22122,7 +22134,7 @@
           <t>4129</t>
         </is>
       </c>
-      <c r="F371" s="1" t="n">
+      <c r="F371" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G371" t="inlineStr">
@@ -22149,7 +22161,7 @@
         </is>
       </c>
       <c r="L371" t="inlineStr"/>
-      <c r="M371" s="1" t="n">
+      <c r="M371" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="N371" t="inlineStr"/>
@@ -22184,7 +22196,7 @@
           <t>KI525A-B100660</t>
         </is>
       </c>
-      <c r="F372" s="1" t="n">
+      <c r="F372" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="G372" t="inlineStr">
@@ -22211,7 +22223,7 @@
         </is>
       </c>
       <c r="L372" t="inlineStr"/>
-      <c r="M372" s="1" t="n">
+      <c r="M372" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="N372" t="inlineStr"/>
@@ -22250,7 +22262,7 @@
           <t>C66508</t>
         </is>
       </c>
-      <c r="F373" s="1" t="n">
+      <c r="F373" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="G373" t="inlineStr">
@@ -22310,7 +22322,7 @@
           <t>C66698</t>
         </is>
       </c>
-      <c r="F374" s="1" t="n">
+      <c r="F374" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="G374" t="inlineStr">
@@ -22370,7 +22382,7 @@
           <t>35511</t>
         </is>
       </c>
-      <c r="F375" s="1" t="n">
+      <c r="F375" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G375" t="inlineStr">
@@ -22430,7 +22442,7 @@
           <t>85023</t>
         </is>
       </c>
-      <c r="F376" s="1" t="n">
+      <c r="F376" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G376" t="inlineStr">
@@ -22490,7 +22502,7 @@
           <t>64318</t>
         </is>
       </c>
-      <c r="F377" s="1" t="n">
+      <c r="F377" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G377" t="inlineStr">
@@ -22554,7 +22566,7 @@
           <t>83287</t>
         </is>
       </c>
-      <c r="F378" s="1" t="n">
+      <c r="F378" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G378" t="inlineStr">
@@ -22614,7 +22626,7 @@
           <t>25424</t>
         </is>
       </c>
-      <c r="F379" s="1" t="n">
+      <c r="F379" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G379" t="inlineStr">
@@ -22641,7 +22653,7 @@
         </is>
       </c>
       <c r="L379" t="inlineStr"/>
-      <c r="M379" s="1" t="n">
+      <c r="M379" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="N379" t="inlineStr"/>
@@ -22676,7 +22688,7 @@
           <t>24970</t>
         </is>
       </c>
-      <c r="F380" s="1" t="n">
+      <c r="F380" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G380" t="inlineStr">
@@ -22736,7 +22748,7 @@
           <t>21156</t>
         </is>
       </c>
-      <c r="F381" s="1" t="n">
+      <c r="F381" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G381" t="inlineStr">
@@ -22796,7 +22808,7 @@
           <t>1652</t>
         </is>
       </c>
-      <c r="F382" s="1" t="n">
+      <c r="F382" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G382" t="inlineStr">
@@ -22856,7 +22868,7 @@
           <t>1713</t>
         </is>
       </c>
-      <c r="F383" s="1" t="n">
+      <c r="F383" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="G383" t="inlineStr">
@@ -22916,7 +22928,7 @@
           <t>1328-5</t>
         </is>
       </c>
-      <c r="F384" s="1" t="n">
+      <c r="F384" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="G384" t="inlineStr">
@@ -22976,7 +22988,7 @@
           <t>2309-5</t>
         </is>
       </c>
-      <c r="F385" s="1" t="n">
+      <c r="F385" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="G385" t="inlineStr">
@@ -23036,7 +23048,7 @@
           <t>4154</t>
         </is>
       </c>
-      <c r="F386" s="1" t="n">
+      <c r="F386" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G386" t="inlineStr">
@@ -23096,7 +23108,7 @@
           <t>4164</t>
         </is>
       </c>
-      <c r="F387" s="1" t="n">
+      <c r="F387" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G387" t="inlineStr">
@@ -23156,7 +23168,7 @@
           <t>17143</t>
         </is>
       </c>
-      <c r="F388" s="1" t="n">
+      <c r="F388" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G388" t="inlineStr">
@@ -23216,7 +23228,7 @@
           <t>3391XL</t>
         </is>
       </c>
-      <c r="F389" s="1" t="n">
+      <c r="F389" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G389" t="inlineStr">
@@ -23276,7 +23288,7 @@
           <t>S00007XL</t>
         </is>
       </c>
-      <c r="F390" s="1" t="n">
+      <c r="F390" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G390" t="inlineStr">
@@ -23303,7 +23315,7 @@
         </is>
       </c>
       <c r="L390" t="inlineStr"/>
-      <c r="M390" s="1" t="n">
+      <c r="M390" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="N390" t="inlineStr"/>
@@ -23338,7 +23350,7 @@
           <t>C66691</t>
         </is>
       </c>
-      <c r="F391" s="1" t="n">
+      <c r="F391" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G391" t="inlineStr">
@@ -23402,7 +23414,7 @@
           <t>9933-49</t>
         </is>
       </c>
-      <c r="F392" s="1" t="n">
+      <c r="F392" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G392" t="inlineStr">
@@ -23427,7 +23439,7 @@
         </is>
       </c>
       <c r="L392" t="inlineStr"/>
-      <c r="M392" s="1" t="n">
+      <c r="M392" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="N392" t="inlineStr"/>
@@ -23462,7 +23474,7 @@
           <t>0612</t>
         </is>
       </c>
-      <c r="F393" s="1" t="n">
+      <c r="F393" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G393" t="inlineStr">
@@ -23522,7 +23534,7 @@
           <t>070407910680166AE</t>
         </is>
       </c>
-      <c r="F394" s="1" t="n">
+      <c r="F394" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G394" t="inlineStr">
@@ -23582,7 +23594,7 @@
           <t>070407983320094AE</t>
         </is>
       </c>
-      <c r="F395" s="1" t="n">
+      <c r="F395" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G395" t="inlineStr">
@@ -23642,7 +23654,7 @@
           <t>070407983320096AE</t>
         </is>
       </c>
-      <c r="F396" s="1" t="n">
+      <c r="F396" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G396" t="inlineStr">
@@ -23702,7 +23714,7 @@
           <t>070407983320111AE</t>
         </is>
       </c>
-      <c r="F397" s="1" t="n">
+      <c r="F397" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G397" t="inlineStr">
@@ -23762,7 +23774,7 @@
           <t>070407983320130AE</t>
         </is>
       </c>
-      <c r="F398" s="1" t="n">
+      <c r="F398" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G398" t="inlineStr">
@@ -23822,7 +23834,7 @@
           <t>B10133</t>
         </is>
       </c>
-      <c r="F399" s="1" t="n">
+      <c r="F399" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="G399" t="inlineStr">
@@ -23847,7 +23859,7 @@
         </is>
       </c>
       <c r="L399" t="inlineStr"/>
-      <c r="M399" s="1" t="n">
+      <c r="M399" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="N399" t="inlineStr"/>
@@ -23882,7 +23894,7 @@
           <t>89177</t>
         </is>
       </c>
-      <c r="F400" s="1" t="n">
+      <c r="F400" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G400" t="inlineStr">
@@ -23942,7 +23954,7 @@
           <t>25304</t>
         </is>
       </c>
-      <c r="F401" s="1" t="n">
+      <c r="F401" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G401" t="inlineStr">
@@ -24002,7 +24014,7 @@
           <t>94934</t>
         </is>
       </c>
-      <c r="F402" s="1" t="n">
+      <c r="F402" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G402" t="inlineStr">
@@ -24062,7 +24074,7 @@
           <t>5155</t>
         </is>
       </c>
-      <c r="F403" s="1" t="n">
+      <c r="F403" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G403" t="inlineStr">
@@ -24118,7 +24130,7 @@
           <t>2333</t>
         </is>
       </c>
-      <c r="F404" s="1" t="n">
+      <c r="F404" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="G404" t="inlineStr">
@@ -24170,7 +24182,7 @@
       <c r="E405" t="n">
         <v>9599</v>
       </c>
-      <c r="F405" s="1" t="n">
+      <c r="F405" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="G405" t="inlineStr">
@@ -24218,7 +24230,7 @@
       <c r="E406" t="n">
         <v>14251</v>
       </c>
-      <c r="F406" s="1" t="n">
+      <c r="F406" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="G406" t="inlineStr">
@@ -24266,7 +24278,7 @@
       <c r="E407" t="n">
         <v>19945</v>
       </c>
-      <c r="F407" s="1" t="n">
+      <c r="F407" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="G407" t="inlineStr">
@@ -24314,7 +24326,7 @@
       <c r="E408" t="n">
         <v>14396</v>
       </c>
-      <c r="F408" s="1" t="n">
+      <c r="F408" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="G408" t="inlineStr">
@@ -24362,7 +24374,7 @@
       <c r="E409" t="n">
         <v>9920</v>
       </c>
-      <c r="F409" s="1" t="n">
+      <c r="F409" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="G409" t="inlineStr">
@@ -24410,7 +24422,7 @@
       <c r="E410" t="n">
         <v>20528</v>
       </c>
-      <c r="F410" s="1" t="n">
+      <c r="F410" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="G410" t="inlineStr">
@@ -24462,7 +24474,7 @@
           <t>3BF23</t>
         </is>
       </c>
-      <c r="F411" s="1" t="n">
+      <c r="F411" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G411" t="inlineStr">
@@ -24514,7 +24526,7 @@
           <t>10BE80</t>
         </is>
       </c>
-      <c r="F412" s="1" t="n">
+      <c r="F412" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G412" t="inlineStr">
@@ -24566,7 +24578,7 @@
           <t>2BC10</t>
         </is>
       </c>
-      <c r="F413" s="1" t="n">
+      <c r="F413" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G413" t="inlineStr">
@@ -24618,7 +24630,7 @@
           <t>11BG159</t>
         </is>
       </c>
-      <c r="F414" s="1" t="n">
+      <c r="F414" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G414" t="inlineStr">
@@ -24668,7 +24680,7 @@
           <t>A76103</t>
         </is>
       </c>
-      <c r="F415" s="1" t="n">
+      <c r="F415" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G415" t="inlineStr">
@@ -24718,7 +24730,7 @@
       <c r="E416" t="n">
         <v>5844</v>
       </c>
-      <c r="F416" s="1" t="n">
+      <c r="F416" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G416" t="inlineStr">
@@ -24768,7 +24780,7 @@
           <t>S00456</t>
         </is>
       </c>
-      <c r="F417" s="1" t="n">
+      <c r="F417" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G417" t="inlineStr">
@@ -24818,7 +24830,7 @@
           <t>S00167XL</t>
         </is>
       </c>
-      <c r="F418" s="1" t="n">
+      <c r="F418" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G418" t="inlineStr">
@@ -24868,7 +24880,7 @@
           <t>S00006XL2</t>
         </is>
       </c>
-      <c r="F419" s="1" t="n">
+      <c r="F419" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G419" t="inlineStr">
@@ -24918,7 +24930,7 @@
       <c r="E420" t="n">
         <v>580</v>
       </c>
-      <c r="F420" s="1" t="n">
+      <c r="F420" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G420" t="inlineStr">
@@ -24968,7 +24980,7 @@
           <t>T97125Q</t>
         </is>
       </c>
-      <c r="F421" s="1" t="n">
+      <c r="F421" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G421" t="inlineStr">
@@ -25018,7 +25030,7 @@
           <t>T1011900</t>
         </is>
       </c>
-      <c r="F422" s="1" t="n">
+      <c r="F422" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G422" t="inlineStr">
@@ -25068,7 +25080,7 @@
           <t>T91786Q</t>
         </is>
       </c>
-      <c r="F423" s="1" t="n">
+      <c r="F423" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G423" t="inlineStr">
@@ -25118,7 +25130,7 @@
           <t>00D10</t>
         </is>
       </c>
-      <c r="F424" s="1" t="n">
+      <c r="F424" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G424" t="inlineStr">
@@ -25168,7 +25180,7 @@
           <t>00D175</t>
         </is>
       </c>
-      <c r="F425" s="1" t="n">
+      <c r="F425" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G425" t="inlineStr">
@@ -25220,7 +25232,7 @@
           <t>E05-11026</t>
         </is>
       </c>
-      <c r="F426" s="1" t="n">
+      <c r="F426" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G426" t="inlineStr">
@@ -25270,7 +25282,7 @@
       <c r="E427" t="n">
         <v>6309</v>
       </c>
-      <c r="F427" s="1" t="n">
+      <c r="F427" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G427" t="inlineStr">
@@ -25320,7 +25332,7 @@
       <c r="E428" t="n">
         <v>504011190625165</v>
       </c>
-      <c r="F428" s="1" t="n">
+      <c r="F428" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G428" t="inlineStr">
@@ -25370,7 +25382,7 @@
       <c r="E429" t="n">
         <v>504011190625185</v>
       </c>
-      <c r="F429" s="1" t="n">
+      <c r="F429" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G429" t="inlineStr">
@@ -25420,7 +25432,7 @@
           <t>1116740R</t>
         </is>
       </c>
-      <c r="F430" s="1" t="n">
+      <c r="F430" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G430" t="inlineStr">
@@ -25470,7 +25482,7 @@
           <t>1992457/AC</t>
         </is>
       </c>
-      <c r="F431" s="1" t="n">
+      <c r="F431" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G431" t="inlineStr">
@@ -25520,7 +25532,7 @@
           <t>1715715AC</t>
         </is>
       </c>
-      <c r="F432" s="1" t="n">
+      <c r="F432" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G432" t="inlineStr">
@@ -25570,7 +25582,7 @@
           <t>L442</t>
         </is>
       </c>
-      <c r="F433" s="1" t="n">
+      <c r="F433" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G433" t="inlineStr">
@@ -25618,7 +25630,7 @@
       <c r="E434" t="n">
         <v>328</v>
       </c>
-      <c r="F434" s="1" t="n">
+      <c r="F434" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G434" t="inlineStr">
@@ -25666,7 +25678,7 @@
       <c r="E435" t="n">
         <v>277</v>
       </c>
-      <c r="F435" s="1" t="n">
+      <c r="F435" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G435" t="inlineStr">
@@ -25714,7 +25726,7 @@
       <c r="E436" t="n">
         <v>477</v>
       </c>
-      <c r="F436" s="1" t="n">
+      <c r="F436" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G436" t="inlineStr">
@@ -25762,7 +25774,7 @@
       <c r="E437" t="n">
         <v>11</v>
       </c>
-      <c r="F437" s="1" t="n">
+      <c r="F437" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G437" t="inlineStr">
@@ -25812,7 +25824,7 @@
           <t>196L</t>
         </is>
       </c>
-      <c r="F438" s="1" t="n">
+      <c r="F438" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="G438" t="inlineStr">
@@ -25864,7 +25876,7 @@
           <t>15W013724</t>
         </is>
       </c>
-      <c r="F439" s="1" t="n">
+      <c r="F439" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="G439" t="inlineStr">
@@ -25916,7 +25928,7 @@
           <t>15W013930</t>
         </is>
       </c>
-      <c r="F440" s="1" t="n">
+      <c r="F440" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="G440" t="inlineStr">
@@ -25966,7 +25978,7 @@
       <c r="E441" t="n">
         <v>86815651</v>
       </c>
-      <c r="F441" s="1" t="n">
+      <c r="F441" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="G441" t="inlineStr">
@@ -26016,7 +26028,7 @@
       <c r="E442" t="n">
         <v>86817554</v>
       </c>
-      <c r="F442" s="1" t="n">
+      <c r="F442" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="G442" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: reparaveis (14/07/2026 06:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1522,7 +1522,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2238,7 +2238,7 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -3102,7 +3102,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -3166,7 +3166,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -3226,7 +3226,7 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -3292,7 +3292,7 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -3520,7 +3520,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3580,7 +3580,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -4204,7 +4204,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -4556,7 +4556,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -4730,7 +4730,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -4908,7 +4908,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -5136,7 +5136,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -5496,7 +5496,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -5556,7 +5556,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -5738,7 +5738,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -5802,7 +5802,7 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -5968,7 +5968,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -6218,7 +6218,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="I104" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
@@ -6658,7 +6658,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -6720,7 +6720,7 @@
         </is>
       </c>
       <c r="I107" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J107" t="inlineStr">
         <is>
@@ -6782,7 +6782,7 @@
         </is>
       </c>
       <c r="I108" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
         </is>
       </c>
       <c r="I109" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -7184,7 +7184,7 @@
         </is>
       </c>
       <c r="I115" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -7244,7 +7244,7 @@
         </is>
       </c>
       <c r="I116" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J116" t="inlineStr">
         <is>
@@ -7304,7 +7304,7 @@
         </is>
       </c>
       <c r="I117" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J117" t="inlineStr">
         <is>
@@ -7364,7 +7364,7 @@
         </is>
       </c>
       <c r="I118" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="I119" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
@@ -7484,7 +7484,7 @@
         </is>
       </c>
       <c r="I120" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -7544,7 +7544,7 @@
         </is>
       </c>
       <c r="I121" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -7608,7 +7608,7 @@
         </is>
       </c>
       <c r="I122" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -7718,7 +7718,7 @@
         </is>
       </c>
       <c r="I124" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -7778,7 +7778,7 @@
         </is>
       </c>
       <c r="I125" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -7946,7 +7946,7 @@
         </is>
       </c>
       <c r="I128" t="n">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -8006,7 +8006,7 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -8066,7 +8066,7 @@
         </is>
       </c>
       <c r="I130" t="n">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -8188,7 +8188,7 @@
         </is>
       </c>
       <c r="I132" t="n">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J132" t="inlineStr">
         <is>
@@ -8302,7 +8302,7 @@
         </is>
       </c>
       <c r="I134" t="n">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J134" t="inlineStr">
         <is>
@@ -8512,7 +8512,7 @@
         </is>
       </c>
       <c r="I138" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J138" t="inlineStr">
         <is>
@@ -9046,7 +9046,7 @@
         </is>
       </c>
       <c r="I148" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
@@ -9106,7 +9106,7 @@
         </is>
       </c>
       <c r="I149" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J149" t="inlineStr">
         <is>
@@ -9162,7 +9162,7 @@
         </is>
       </c>
       <c r="I150" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -9286,7 +9286,7 @@
         </is>
       </c>
       <c r="I152" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J152" t="inlineStr">
         <is>
@@ -9348,7 +9348,7 @@
         </is>
       </c>
       <c r="I153" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
         </is>
       </c>
       <c r="I155" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J155" t="inlineStr">
         <is>
@@ -9522,7 +9522,7 @@
         </is>
       </c>
       <c r="I156" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J156" t="inlineStr">
         <is>
@@ -9582,7 +9582,7 @@
         </is>
       </c>
       <c r="I157" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J157" t="inlineStr">
         <is>
@@ -9642,7 +9642,7 @@
         </is>
       </c>
       <c r="I158" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J158" t="inlineStr">
         <is>
@@ -9704,7 +9704,7 @@
         </is>
       </c>
       <c r="I159" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J159" t="inlineStr">
         <is>
@@ -9764,7 +9764,7 @@
         </is>
       </c>
       <c r="I160" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J160" t="inlineStr">
         <is>
@@ -9824,7 +9824,7 @@
         </is>
       </c>
       <c r="I161" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J161" t="inlineStr">
         <is>
@@ -9890,7 +9890,7 @@
         </is>
       </c>
       <c r="I162" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J162" t="inlineStr">
         <is>
@@ -9952,7 +9952,7 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J163" t="inlineStr">
         <is>
@@ -10014,7 +10014,7 @@
         </is>
       </c>
       <c r="I164" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J164" t="inlineStr">
         <is>
@@ -10070,7 +10070,7 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J165" t="inlineStr">
         <is>
@@ -10238,7 +10238,7 @@
         </is>
       </c>
       <c r="I168" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J168" t="inlineStr">
         <is>
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="I169" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="I171" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J171" t="inlineStr">
         <is>
@@ -10656,7 +10656,7 @@
         </is>
       </c>
       <c r="I175" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
@@ -10722,7 +10722,7 @@
         </is>
       </c>
       <c r="I176" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J176" t="inlineStr">
         <is>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="I177" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
@@ -10848,7 +10848,7 @@
         </is>
       </c>
       <c r="I178" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
         </is>
       </c>
       <c r="I180" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="I183" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -11182,7 +11182,7 @@
         </is>
       </c>
       <c r="I184" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
@@ -11238,7 +11238,7 @@
         </is>
       </c>
       <c r="I185" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
@@ -11298,7 +11298,7 @@
         </is>
       </c>
       <c r="I186" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
@@ -11358,7 +11358,7 @@
         </is>
       </c>
       <c r="I187" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
@@ -11422,7 +11422,7 @@
         </is>
       </c>
       <c r="I188" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -11488,7 +11488,7 @@
         </is>
       </c>
       <c r="I189" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
@@ -11550,7 +11550,7 @@
         </is>
       </c>
       <c r="I190" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
@@ -11610,7 +11610,7 @@
         </is>
       </c>
       <c r="I191" t="n">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
@@ -11672,7 +11672,7 @@
         </is>
       </c>
       <c r="I192" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
@@ -11732,7 +11732,7 @@
         </is>
       </c>
       <c r="I193" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
@@ -11842,7 +11842,7 @@
         </is>
       </c>
       <c r="I195" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
@@ -12052,7 +12052,7 @@
         </is>
       </c>
       <c r="I199" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
@@ -12114,7 +12114,7 @@
         </is>
       </c>
       <c r="I200" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J200" t="inlineStr">
         <is>
@@ -12174,7 +12174,7 @@
         </is>
       </c>
       <c r="I201" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J201" t="inlineStr">
         <is>
@@ -12234,7 +12234,7 @@
         </is>
       </c>
       <c r="I202" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J202" t="inlineStr">
         <is>
@@ -12294,7 +12294,7 @@
         </is>
       </c>
       <c r="I203" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J203" t="inlineStr">
         <is>
@@ -12354,7 +12354,7 @@
         </is>
       </c>
       <c r="I204" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J204" t="inlineStr">
         <is>
@@ -12414,7 +12414,7 @@
         </is>
       </c>
       <c r="I205" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J205" t="inlineStr">
         <is>
@@ -12532,7 +12532,7 @@
         </is>
       </c>
       <c r="I207" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J207" t="inlineStr">
         <is>
@@ -12594,7 +12594,7 @@
         </is>
       </c>
       <c r="I208" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J208" t="inlineStr">
         <is>
@@ -12656,7 +12656,7 @@
         </is>
       </c>
       <c r="I209" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J209" t="inlineStr">
         <is>
@@ -12718,7 +12718,7 @@
         </is>
       </c>
       <c r="I210" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J210" t="inlineStr">
         <is>
@@ -12894,7 +12894,7 @@
         </is>
       </c>
       <c r="I213" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J213" t="inlineStr">
         <is>
@@ -12954,7 +12954,7 @@
         </is>
       </c>
       <c r="I214" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J214" t="inlineStr">
         <is>
@@ -13018,7 +13018,7 @@
         </is>
       </c>
       <c r="I215" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J215" t="inlineStr">
         <is>
@@ -13128,7 +13128,7 @@
         </is>
       </c>
       <c r="I217" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J217" t="inlineStr">
         <is>
@@ -13190,7 +13190,7 @@
         </is>
       </c>
       <c r="I218" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J218" t="inlineStr">
         <is>
@@ -13250,7 +13250,7 @@
         </is>
       </c>
       <c r="I219" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J219" t="inlineStr">
         <is>
@@ -13310,7 +13310,7 @@
         </is>
       </c>
       <c r="I220" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J220" t="inlineStr">
         <is>
@@ -13428,7 +13428,7 @@
         </is>
       </c>
       <c r="I222" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J222" t="inlineStr">
         <is>
@@ -13488,7 +13488,7 @@
         </is>
       </c>
       <c r="I223" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J223" t="inlineStr">
         <is>
@@ -13548,7 +13548,7 @@
         </is>
       </c>
       <c r="I224" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J224" t="inlineStr">
         <is>
@@ -13608,7 +13608,7 @@
         </is>
       </c>
       <c r="I225" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J225" t="inlineStr">
         <is>
@@ -13668,7 +13668,7 @@
         </is>
       </c>
       <c r="I226" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J226" t="inlineStr">
         <is>
@@ -13728,7 +13728,7 @@
         </is>
       </c>
       <c r="I227" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J227" t="inlineStr">
         <is>
@@ -13788,7 +13788,7 @@
         </is>
       </c>
       <c r="I228" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
@@ -13906,7 +13906,7 @@
         </is>
       </c>
       <c r="I230" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J230" t="inlineStr">
         <is>
@@ -13966,7 +13966,7 @@
         </is>
       </c>
       <c r="I231" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J231" t="inlineStr">
         <is>
@@ -14144,7 +14144,7 @@
         </is>
       </c>
       <c r="I234" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
@@ -14210,7 +14210,7 @@
         </is>
       </c>
       <c r="I235" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J235" t="inlineStr">
         <is>
@@ -14276,7 +14276,7 @@
         </is>
       </c>
       <c r="I236" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J236" t="inlineStr">
         <is>
@@ -14338,7 +14338,7 @@
         </is>
       </c>
       <c r="I237" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
@@ -14448,7 +14448,7 @@
         </is>
       </c>
       <c r="I239" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J239" t="inlineStr">
         <is>
@@ -14626,7 +14626,7 @@
         </is>
       </c>
       <c r="I242" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J242" t="inlineStr">
         <is>
@@ -14740,7 +14740,7 @@
         </is>
       </c>
       <c r="I244" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J244" t="inlineStr">
         <is>
@@ -14800,7 +14800,7 @@
         </is>
       </c>
       <c r="I245" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J245" t="inlineStr">
         <is>
@@ -14860,7 +14860,7 @@
         </is>
       </c>
       <c r="I246" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -15022,7 +15022,7 @@
         </is>
       </c>
       <c r="I249" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J249" t="inlineStr">
         <is>
@@ -15082,7 +15082,7 @@
         </is>
       </c>
       <c r="I250" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J250" t="inlineStr">
         <is>
@@ -15258,7 +15258,7 @@
         </is>
       </c>
       <c r="I253" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J253" t="inlineStr">
         <is>
@@ -15318,7 +15318,7 @@
         </is>
       </c>
       <c r="I254" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J254" t="inlineStr">
         <is>
@@ -15378,7 +15378,7 @@
         </is>
       </c>
       <c r="I255" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J255" t="inlineStr">
         <is>
@@ -15438,7 +15438,7 @@
         </is>
       </c>
       <c r="I256" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J256" t="inlineStr">
         <is>
@@ -15600,7 +15600,7 @@
         </is>
       </c>
       <c r="I259" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J259" t="inlineStr">
         <is>
@@ -15660,7 +15660,7 @@
         </is>
       </c>
       <c r="I260" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J260" t="inlineStr">
         <is>
@@ -15720,7 +15720,7 @@
         </is>
       </c>
       <c r="I261" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J261" t="inlineStr">
         <is>
@@ -15780,7 +15780,7 @@
         </is>
       </c>
       <c r="I262" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J262" t="inlineStr">
         <is>
@@ -15904,7 +15904,7 @@
         </is>
       </c>
       <c r="I264" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J264" t="inlineStr">
         <is>
@@ -15964,7 +15964,7 @@
         </is>
       </c>
       <c r="I265" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J265" t="inlineStr">
         <is>
@@ -16024,7 +16024,7 @@
         </is>
       </c>
       <c r="I266" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J266" t="inlineStr">
         <is>
@@ -16084,7 +16084,7 @@
         </is>
       </c>
       <c r="I267" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J267" t="inlineStr">
         <is>
@@ -16144,7 +16144,7 @@
         </is>
       </c>
       <c r="I268" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J268" t="inlineStr">
         <is>
@@ -16200,7 +16200,7 @@
         </is>
       </c>
       <c r="I269" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J269" t="inlineStr">
         <is>
@@ -16260,7 +16260,7 @@
         </is>
       </c>
       <c r="I270" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J270" t="inlineStr">
         <is>
@@ -16320,7 +16320,7 @@
         </is>
       </c>
       <c r="I271" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J271" t="inlineStr">
         <is>
@@ -16380,7 +16380,7 @@
         </is>
       </c>
       <c r="I272" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J272" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         </is>
       </c>
       <c r="I274" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J274" t="inlineStr">
         <is>
@@ -16622,7 +16622,7 @@
         </is>
       </c>
       <c r="I276" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J276" t="inlineStr">
         <is>
@@ -16682,7 +16682,7 @@
         </is>
       </c>
       <c r="I277" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J277" t="inlineStr">
         <is>
@@ -16742,7 +16742,7 @@
         </is>
       </c>
       <c r="I278" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J278" t="inlineStr">
         <is>
@@ -16802,7 +16802,7 @@
         </is>
       </c>
       <c r="I279" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J279" t="inlineStr">
         <is>
@@ -16866,7 +16866,7 @@
         </is>
       </c>
       <c r="I280" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J280" t="inlineStr">
         <is>
@@ -16926,7 +16926,7 @@
         </is>
       </c>
       <c r="I281" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J281" t="inlineStr">
         <is>
@@ -16986,7 +16986,7 @@
         </is>
       </c>
       <c r="I282" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J282" t="inlineStr">
         <is>
@@ -17312,7 +17312,7 @@
         </is>
       </c>
       <c r="I288" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J288" t="inlineStr">
         <is>
@@ -17416,7 +17416,7 @@
         </is>
       </c>
       <c r="I290" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J290" t="inlineStr">
         <is>
@@ -17470,7 +17470,7 @@
         </is>
       </c>
       <c r="I291" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J291" t="inlineStr">
         <is>
@@ -17528,7 +17528,7 @@
         </is>
       </c>
       <c r="I292" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J292" t="inlineStr">
         <is>
@@ -17586,7 +17586,7 @@
         </is>
       </c>
       <c r="I293" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J293" t="inlineStr">
         <is>
@@ -17644,7 +17644,7 @@
         </is>
       </c>
       <c r="I294" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J294" t="inlineStr">
         <is>
@@ -17698,7 +17698,7 @@
         </is>
       </c>
       <c r="I295" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J295" t="inlineStr">
         <is>
@@ -17752,7 +17752,7 @@
         </is>
       </c>
       <c r="I296" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J296" t="inlineStr">
         <is>
@@ -17862,7 +17862,7 @@
         </is>
       </c>
       <c r="I298" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J298" t="inlineStr">
         <is>
@@ -17920,7 +17920,7 @@
         </is>
       </c>
       <c r="I299" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J299" t="inlineStr">
         <is>
@@ -17978,7 +17978,7 @@
         </is>
       </c>
       <c r="I300" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J300" t="inlineStr">
         <is>
@@ -18036,7 +18036,7 @@
         </is>
       </c>
       <c r="I301" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J301" t="inlineStr">
         <is>
@@ -18092,7 +18092,7 @@
         </is>
       </c>
       <c r="I302" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J302" t="inlineStr">
         <is>
@@ -18148,7 +18148,7 @@
         </is>
       </c>
       <c r="I303" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J303" t="inlineStr">
         <is>
@@ -18204,7 +18204,7 @@
         </is>
       </c>
       <c r="I304" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J304" t="inlineStr">
         <is>
@@ -18260,7 +18260,7 @@
         </is>
       </c>
       <c r="I305" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J305" t="inlineStr">
         <is>
@@ -18318,7 +18318,7 @@
         </is>
       </c>
       <c r="I306" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J306" t="inlineStr">
         <is>
@@ -18376,7 +18376,7 @@
         </is>
       </c>
       <c r="I307" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J307" t="inlineStr">
         <is>
@@ -18432,7 +18432,7 @@
         </is>
       </c>
       <c r="I308" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J308" t="inlineStr">
         <is>
@@ -18488,7 +18488,7 @@
         </is>
       </c>
       <c r="I309" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J309" t="inlineStr">
         <is>
@@ -18546,7 +18546,7 @@
         </is>
       </c>
       <c r="I310" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J310" t="inlineStr">
         <is>
@@ -18602,7 +18602,7 @@
         </is>
       </c>
       <c r="I311" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J311" t="inlineStr">
         <is>
@@ -18660,7 +18660,7 @@
         </is>
       </c>
       <c r="I312" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J312" t="inlineStr">
         <is>
@@ -18770,7 +18770,7 @@
         </is>
       </c>
       <c r="I314" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J314" t="inlineStr">
         <is>
@@ -18826,7 +18826,7 @@
         </is>
       </c>
       <c r="I315" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J315" t="inlineStr">
         <is>
@@ -18882,7 +18882,7 @@
         </is>
       </c>
       <c r="I316" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J316" t="inlineStr">
         <is>
@@ -18940,7 +18940,7 @@
         </is>
       </c>
       <c r="I317" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J317" t="inlineStr">
         <is>
@@ -19102,7 +19102,7 @@
         </is>
       </c>
       <c r="I320" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J320" t="inlineStr">
         <is>
@@ -19160,7 +19160,7 @@
         </is>
       </c>
       <c r="I321" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J321" t="inlineStr">
         <is>
@@ -19220,7 +19220,7 @@
         </is>
       </c>
       <c r="I322" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J322" t="inlineStr">
         <is>
@@ -19280,7 +19280,7 @@
         </is>
       </c>
       <c r="I323" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J323" t="inlineStr">
         <is>
@@ -19338,7 +19338,7 @@
         </is>
       </c>
       <c r="I324" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J324" t="inlineStr">
         <is>
@@ -19396,7 +19396,7 @@
         </is>
       </c>
       <c r="I325" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J325" t="inlineStr">
         <is>
@@ -19456,7 +19456,7 @@
         </is>
       </c>
       <c r="I326" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J326" t="inlineStr">
         <is>
@@ -19516,7 +19516,7 @@
         </is>
       </c>
       <c r="I327" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J327" t="inlineStr">
         <is>
@@ -19576,7 +19576,7 @@
         </is>
       </c>
       <c r="I328" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J328" t="inlineStr">
         <is>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="I329" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J329" t="inlineStr">
         <is>
@@ -19696,7 +19696,7 @@
         </is>
       </c>
       <c r="I330" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J330" t="inlineStr">
         <is>
@@ -19756,7 +19756,7 @@
         </is>
       </c>
       <c r="I331" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J331" t="inlineStr">
         <is>
@@ -19814,7 +19814,7 @@
         </is>
       </c>
       <c r="I332" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J332" t="inlineStr">
         <is>
@@ -19870,7 +19870,7 @@
         </is>
       </c>
       <c r="I333" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J333" t="inlineStr">
         <is>
@@ -19926,7 +19926,7 @@
         </is>
       </c>
       <c r="I334" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J334" t="inlineStr">
         <is>
@@ -20046,7 +20046,7 @@
         </is>
       </c>
       <c r="I336" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J336" t="inlineStr">
         <is>
@@ -20166,7 +20166,7 @@
         </is>
       </c>
       <c r="I338" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J338" t="inlineStr">
         <is>
@@ -20272,7 +20272,7 @@
         </is>
       </c>
       <c r="I340" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J340" t="inlineStr">
         <is>
@@ -20332,7 +20332,7 @@
         </is>
       </c>
       <c r="I341" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J341" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
         </is>
       </c>
       <c r="I342" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J342" t="inlineStr">
         <is>
@@ -20452,7 +20452,7 @@
         </is>
       </c>
       <c r="I343" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J343" t="inlineStr">
         <is>
@@ -20512,7 +20512,7 @@
         </is>
       </c>
       <c r="I344" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J344" t="inlineStr">
         <is>
@@ -20572,7 +20572,7 @@
         </is>
       </c>
       <c r="I345" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J345" t="inlineStr">
         <is>
@@ -20632,7 +20632,7 @@
         </is>
       </c>
       <c r="I346" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J346" t="inlineStr">
         <is>
@@ -20692,7 +20692,7 @@
         </is>
       </c>
       <c r="I347" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J347" t="inlineStr">
         <is>
@@ -20754,7 +20754,7 @@
         </is>
       </c>
       <c r="I348" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J348" t="inlineStr">
         <is>
@@ -20816,7 +20816,7 @@
         </is>
       </c>
       <c r="I349" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J349" t="inlineStr">
         <is>
@@ -20876,7 +20876,7 @@
         </is>
       </c>
       <c r="I350" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J350" t="inlineStr">
         <is>
@@ -20932,7 +20932,7 @@
         </is>
       </c>
       <c r="I351" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J351" t="inlineStr">
         <is>
@@ -20992,7 +20992,7 @@
         </is>
       </c>
       <c r="I352" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J352" t="inlineStr">
         <is>
@@ -21052,7 +21052,7 @@
         </is>
       </c>
       <c r="I353" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J353" t="inlineStr">
         <is>
@@ -21112,7 +21112,7 @@
         </is>
       </c>
       <c r="I354" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J354" t="inlineStr">
         <is>
@@ -21172,7 +21172,7 @@
         </is>
       </c>
       <c r="I355" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J355" t="inlineStr">
         <is>
@@ -21294,7 +21294,7 @@
         </is>
       </c>
       <c r="I357" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J357" t="inlineStr">
         <is>
@@ -21354,7 +21354,7 @@
         </is>
       </c>
       <c r="I358" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J358" t="inlineStr">
         <is>
@@ -21414,7 +21414,7 @@
         </is>
       </c>
       <c r="I359" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J359" t="inlineStr">
         <is>
@@ -21474,7 +21474,7 @@
         </is>
       </c>
       <c r="I360" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J360" t="inlineStr">
         <is>
@@ -21534,7 +21534,7 @@
         </is>
       </c>
       <c r="I361" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J361" t="inlineStr">
         <is>
@@ -21594,7 +21594,7 @@
         </is>
       </c>
       <c r="I362" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J362" t="inlineStr">
         <is>
@@ -21654,7 +21654,7 @@
         </is>
       </c>
       <c r="I363" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J363" t="inlineStr">
         <is>
@@ -21714,7 +21714,7 @@
         </is>
       </c>
       <c r="I364" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J364" t="inlineStr">
         <is>
@@ -21774,7 +21774,7 @@
         </is>
       </c>
       <c r="I365" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J365" t="inlineStr">
         <is>
@@ -21834,7 +21834,7 @@
         </is>
       </c>
       <c r="I366" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J366" t="inlineStr">
         <is>
@@ -21894,7 +21894,7 @@
         </is>
       </c>
       <c r="I367" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J367" t="inlineStr">
         <is>
@@ -21954,7 +21954,7 @@
         </is>
       </c>
       <c r="I368" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J368" t="inlineStr">
         <is>
@@ -22014,7 +22014,7 @@
         </is>
       </c>
       <c r="I369" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J369" t="inlineStr">
         <is>
@@ -22074,7 +22074,7 @@
         </is>
       </c>
       <c r="I370" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J370" t="inlineStr">
         <is>
@@ -22134,7 +22134,7 @@
         </is>
       </c>
       <c r="I371" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J371" t="inlineStr">
         <is>
@@ -22196,7 +22196,7 @@
         </is>
       </c>
       <c r="I372" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J372" t="inlineStr">
         <is>
@@ -22262,7 +22262,7 @@
         </is>
       </c>
       <c r="I373" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J373" t="inlineStr">
         <is>
@@ -22322,7 +22322,7 @@
         </is>
       </c>
       <c r="I374" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J374" t="inlineStr">
         <is>
@@ -22382,7 +22382,7 @@
         </is>
       </c>
       <c r="I375" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J375" t="inlineStr">
         <is>
@@ -22442,7 +22442,7 @@
         </is>
       </c>
       <c r="I376" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J376" t="inlineStr">
         <is>
@@ -22564,7 +22564,7 @@
         </is>
       </c>
       <c r="I378" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J378" t="inlineStr">
         <is>
@@ -22624,7 +22624,7 @@
         </is>
       </c>
       <c r="I379" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J379" t="inlineStr">
         <is>
@@ -22686,7 +22686,7 @@
         </is>
       </c>
       <c r="I380" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J380" t="inlineStr">
         <is>
@@ -22746,7 +22746,7 @@
         </is>
       </c>
       <c r="I381" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J381" t="inlineStr">
         <is>
@@ -22806,7 +22806,7 @@
         </is>
       </c>
       <c r="I382" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J382" t="inlineStr">
         <is>
@@ -22866,7 +22866,7 @@
         </is>
       </c>
       <c r="I383" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J383" t="inlineStr">
         <is>
@@ -22926,7 +22926,7 @@
         </is>
       </c>
       <c r="I384" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J384" t="inlineStr">
         <is>
@@ -22986,7 +22986,7 @@
         </is>
       </c>
       <c r="I385" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J385" t="inlineStr">
         <is>
@@ -23046,7 +23046,7 @@
         </is>
       </c>
       <c r="I386" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J386" t="inlineStr">
         <is>
@@ -23106,7 +23106,7 @@
         </is>
       </c>
       <c r="I387" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J387" t="inlineStr">
         <is>
@@ -23166,7 +23166,7 @@
         </is>
       </c>
       <c r="I388" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J388" t="inlineStr">
         <is>
@@ -23226,7 +23226,7 @@
         </is>
       </c>
       <c r="I389" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J389" t="inlineStr">
         <is>
@@ -23286,7 +23286,7 @@
         </is>
       </c>
       <c r="I390" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J390" t="inlineStr">
         <is>
@@ -23470,7 +23470,7 @@
         </is>
       </c>
       <c r="I393" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J393" t="inlineStr">
         <is>
@@ -23530,7 +23530,7 @@
         </is>
       </c>
       <c r="I394" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J394" t="inlineStr">
         <is>
@@ -23590,7 +23590,7 @@
         </is>
       </c>
       <c r="I395" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J395" t="inlineStr">
         <is>
@@ -23650,7 +23650,7 @@
         </is>
       </c>
       <c r="I396" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J396" t="inlineStr">
         <is>
@@ -23710,7 +23710,7 @@
         </is>
       </c>
       <c r="I397" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J397" t="inlineStr">
         <is>
@@ -23770,7 +23770,7 @@
         </is>
       </c>
       <c r="I398" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J398" t="inlineStr">
         <is>
@@ -23890,7 +23890,7 @@
         </is>
       </c>
       <c r="I400" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J400" t="inlineStr">
         <is>
@@ -23950,7 +23950,7 @@
         </is>
       </c>
       <c r="I401" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J401" t="inlineStr">
         <is>
@@ -24010,7 +24010,7 @@
         </is>
       </c>
       <c r="I402" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J402" t="inlineStr">
         <is>
@@ -24070,7 +24070,7 @@
         </is>
       </c>
       <c r="I403" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J403" t="inlineStr">
         <is>
@@ -24126,7 +24126,7 @@
         </is>
       </c>
       <c r="I404" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J404" t="inlineStr">
         <is>
@@ -24224,7 +24224,7 @@
         </is>
       </c>
       <c r="I406" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J406" t="inlineStr"/>
       <c r="K406" t="inlineStr"/>
@@ -24272,7 +24272,7 @@
         </is>
       </c>
       <c r="I407" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J407" t="inlineStr"/>
       <c r="K407" t="inlineStr"/>
@@ -24320,7 +24320,7 @@
         </is>
       </c>
       <c r="I408" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J408" t="inlineStr"/>
       <c r="K408" t="inlineStr"/>
@@ -24368,7 +24368,7 @@
         </is>
       </c>
       <c r="I409" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J409" t="inlineStr"/>
       <c r="K409" t="inlineStr"/>
@@ -24416,7 +24416,7 @@
         </is>
       </c>
       <c r="I410" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J410" t="inlineStr"/>
       <c r="K410" t="inlineStr"/>
@@ -24468,7 +24468,7 @@
         </is>
       </c>
       <c r="I411" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J411" t="inlineStr"/>
       <c r="K411" t="inlineStr"/>
@@ -24520,7 +24520,7 @@
         </is>
       </c>
       <c r="I412" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J412" t="inlineStr"/>
       <c r="K412" t="inlineStr"/>
@@ -24572,7 +24572,7 @@
         </is>
       </c>
       <c r="I413" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J413" t="inlineStr"/>
       <c r="K413" t="inlineStr"/>
@@ -24624,7 +24624,7 @@
         </is>
       </c>
       <c r="I414" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J414" t="inlineStr"/>
       <c r="K414" t="inlineStr"/>
@@ -24674,7 +24674,7 @@
         </is>
       </c>
       <c r="I415" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J415" t="inlineStr"/>
       <c r="K415" t="inlineStr"/>
@@ -24724,7 +24724,7 @@
         </is>
       </c>
       <c r="I416" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J416" t="inlineStr"/>
       <c r="K416" t="inlineStr"/>
@@ -24774,7 +24774,7 @@
         </is>
       </c>
       <c r="I417" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J417" t="inlineStr"/>
       <c r="K417" t="inlineStr"/>
@@ -24824,7 +24824,7 @@
         </is>
       </c>
       <c r="I418" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J418" t="inlineStr"/>
       <c r="K418" t="inlineStr"/>
@@ -24874,7 +24874,7 @@
         </is>
       </c>
       <c r="I419" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J419" t="inlineStr"/>
       <c r="K419" t="inlineStr"/>
@@ -24924,7 +24924,7 @@
         </is>
       </c>
       <c r="I420" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J420" t="inlineStr"/>
       <c r="K420" t="inlineStr"/>
@@ -24974,7 +24974,7 @@
         </is>
       </c>
       <c r="I421" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J421" t="inlineStr"/>
       <c r="K421" t="inlineStr"/>
@@ -25024,7 +25024,7 @@
         </is>
       </c>
       <c r="I422" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J422" t="inlineStr"/>
       <c r="K422" t="inlineStr"/>
@@ -25074,7 +25074,7 @@
         </is>
       </c>
       <c r="I423" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J423" t="inlineStr"/>
       <c r="K423" t="inlineStr"/>
@@ -25124,7 +25124,7 @@
         </is>
       </c>
       <c r="I424" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J424" t="inlineStr"/>
       <c r="K424" t="inlineStr"/>
@@ -25174,7 +25174,7 @@
         </is>
       </c>
       <c r="I425" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J425" t="inlineStr"/>
       <c r="K425" t="inlineStr"/>
@@ -25226,7 +25226,7 @@
         </is>
       </c>
       <c r="I426" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J426" t="inlineStr"/>
       <c r="K426" t="inlineStr"/>
@@ -25276,7 +25276,7 @@
         </is>
       </c>
       <c r="I427" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J427" t="inlineStr"/>
       <c r="K427" t="inlineStr"/>
@@ -25326,7 +25326,7 @@
         </is>
       </c>
       <c r="I428" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J428" t="inlineStr"/>
       <c r="K428" t="inlineStr"/>
@@ -25376,7 +25376,7 @@
         </is>
       </c>
       <c r="I429" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J429" t="inlineStr"/>
       <c r="K429" t="inlineStr"/>
@@ -25426,7 +25426,7 @@
         </is>
       </c>
       <c r="I430" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J430" t="inlineStr"/>
       <c r="K430" t="inlineStr"/>
@@ -25476,7 +25476,7 @@
         </is>
       </c>
       <c r="I431" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J431" t="inlineStr"/>
       <c r="K431" t="inlineStr"/>
@@ -25526,7 +25526,7 @@
         </is>
       </c>
       <c r="I432" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J432" t="inlineStr"/>
       <c r="K432" t="inlineStr"/>
@@ -25576,7 +25576,7 @@
         </is>
       </c>
       <c r="I433" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J433" t="inlineStr"/>
       <c r="K433" t="inlineStr"/>
@@ -25624,7 +25624,7 @@
         </is>
       </c>
       <c r="I434" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J434" t="inlineStr"/>
       <c r="K434" t="inlineStr"/>
@@ -25672,7 +25672,7 @@
         </is>
       </c>
       <c r="I435" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J435" t="inlineStr"/>
       <c r="K435" t="inlineStr"/>
@@ -25720,7 +25720,7 @@
         </is>
       </c>
       <c r="I436" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J436" t="inlineStr"/>
       <c r="K436" t="inlineStr"/>
@@ -25768,7 +25768,7 @@
         </is>
       </c>
       <c r="I437" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J437" t="inlineStr"/>
       <c r="K437" t="inlineStr"/>
@@ -25818,7 +25818,7 @@
         </is>
       </c>
       <c r="I438" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J438" t="inlineStr"/>
       <c r="K438" t="inlineStr"/>
@@ -25870,7 +25870,7 @@
         </is>
       </c>
       <c r="I439" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J439" t="inlineStr"/>
       <c r="K439" t="inlineStr"/>
@@ -25922,7 +25922,7 @@
         </is>
       </c>
       <c r="I440" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J440" t="inlineStr"/>
       <c r="K440" t="inlineStr"/>
@@ -25972,7 +25972,7 @@
         </is>
       </c>
       <c r="I441" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J441" t="inlineStr"/>
       <c r="K441" t="inlineStr"/>
@@ -26022,7 +26022,7 @@
         </is>
       </c>
       <c r="I442" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J442" t="inlineStr"/>
       <c r="K442" t="inlineStr"/>
@@ -26072,7 +26072,7 @@
         </is>
       </c>
       <c r="I443" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J443" t="inlineStr"/>
       <c r="K443" t="inlineStr"/>
@@ -26122,7 +26122,7 @@
         </is>
       </c>
       <c r="I444" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J444" t="inlineStr"/>
       <c r="K444" t="inlineStr"/>
@@ -26170,7 +26170,7 @@
         </is>
       </c>
       <c r="I445" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J445" t="inlineStr"/>
       <c r="K445" t="inlineStr"/>
@@ -26220,7 +26220,7 @@
         </is>
       </c>
       <c r="I446" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J446" t="inlineStr"/>
       <c r="K446" t="inlineStr"/>
@@ -26270,7 +26270,7 @@
         </is>
       </c>
       <c r="I447" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J447" t="inlineStr"/>
       <c r="K447" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (15/07/2026 16:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3744" uniqueCount="1271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3746" uniqueCount="1273">
   <si>
     <t>os</t>
   </si>
@@ -3808,6 +3808,9 @@
     <t>027/2025</t>
   </si>
   <si>
+    <t>080/2026</t>
+  </si>
+  <si>
     <t>062/2026</t>
   </si>
   <si>
@@ -3824,6 +3827,9 @@
   </si>
   <si>
     <t>006/2026</t>
+  </si>
+  <si>
+    <t>078/2026</t>
   </si>
   <si>
     <t>024/2026</t>
@@ -4241,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4279,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4317,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4355,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4396,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4437,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4510,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4554,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4598,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4642,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4718,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4759,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4797,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4835,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4876,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4952,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5028,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5066,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5180,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5224,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5326,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5402,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5635,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5670,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5813,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5857,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5901,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5939,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5983,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6050,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6123,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6161,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6199,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6301,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6499,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6543,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6759,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6797,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6867,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6940,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6978,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7083,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7118,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7191,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7264,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7308,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7346,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7384,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7498,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7539,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7603,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7641,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7679,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7717,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7761,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7802,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7869,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -7994,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8032,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8070,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8111,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8152,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8190,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8397,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8435,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8473,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8511,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8549,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8587,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8625,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8669,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8736,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8774,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8876,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8914,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8952,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9031,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9104,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9229,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9546,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9584,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9619,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9698,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9739,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9812,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9847,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9885,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9923,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9964,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10002,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10040,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10084,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10125,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10166,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10201,13 +10207,16 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
       </c>
       <c r="L165" t="s">
         <v>1242</v>
+      </c>
+      <c r="O165" t="s">
+        <v>1264</v>
       </c>
       <c r="P165" t="b">
         <v>1</v>
@@ -10303,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10344,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10420,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10563,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10575,7 +10584,7 @@
         <v>46122</v>
       </c>
       <c r="O175" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="P175" t="b">
         <v>1</v>
@@ -10607,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10645,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10657,7 +10666,7 @@
         <v>45961</v>
       </c>
       <c r="O177" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="P177" t="b">
         <v>1</v>
@@ -10689,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10756,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10858,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10893,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10928,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10966,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11004,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11048,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11060,7 +11069,7 @@
         <v>45986</v>
       </c>
       <c r="O188" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="P188" t="b">
         <v>1</v>
@@ -11092,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11133,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11171,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11212,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11250,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11317,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11442,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11483,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11521,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11559,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11597,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11635,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11673,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11746,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11787,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11828,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11869,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11977,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12015,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12059,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12126,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12167,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12205,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12243,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12316,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12354,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12392,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12430,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12468,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12506,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12544,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12617,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12655,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12766,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12778,7 +12787,7 @@
         <v>46063</v>
       </c>
       <c r="O234" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="P234" t="b">
         <v>1</v>
@@ -12810,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12822,7 +12831,7 @@
         <v>46063</v>
       </c>
       <c r="O235" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="P235" t="b">
         <v>1</v>
@@ -12854,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12895,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12962,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13073,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13143,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13181,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13219,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13318,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13356,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13464,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13502,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13540,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13578,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13677,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13715,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13753,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13791,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13803,7 +13812,7 @@
         <v>46113</v>
       </c>
       <c r="O262" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="P262" t="b">
         <v>1</v>
@@ -13870,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13908,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13946,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13984,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14022,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14057,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14095,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14133,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14171,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14250,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14323,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14361,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14399,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14437,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14446,7 +14455,7 @@
         <v>1242</v>
       </c>
       <c r="O279" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="P279" t="b">
         <v>1</v>
@@ -14478,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14516,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14554,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14761,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14828,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14866,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14904,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14942,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14980,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15015,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15050,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15120,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15158,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15196,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15234,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15272,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15310,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15348,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15386,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15427,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15468,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15506,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15544,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15582,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15620,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15658,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15731,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15769,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15807,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15845,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15950,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15988,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16026,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16067,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16105,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16143,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16184,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16222,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16263,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16304,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16345,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16386,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16424,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16462,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16500,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16576,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16652,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16719,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16757,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16795,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16833,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16871,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16909,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16947,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16985,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17026,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17067,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17105,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17140,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17178,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17216,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17254,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17292,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17371,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17409,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17447,13 +17456,16 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
       </c>
       <c r="L359" t="s">
         <v>1240</v>
+      </c>
+      <c r="O359" t="s">
+        <v>1271</v>
       </c>
       <c r="P359" t="b">
         <v>1</v>
@@ -17485,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17523,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17561,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17599,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17637,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17675,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17713,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17751,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17789,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17827,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17865,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17903,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17944,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -17956,7 +17968,7 @@
         <v>46113</v>
       </c>
       <c r="O372" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="P372" t="b">
         <v>1</v>
@@ -17988,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18026,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18064,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18102,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18146,7 +18158,7 @@
         <v>1244</v>
       </c>
       <c r="O377" t="s">
-        <v>1270</v>
+        <v>1272</v>
       </c>
       <c r="P377" t="b">
         <v>0</v>
@@ -18178,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18216,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18257,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18295,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18333,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18371,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18409,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18447,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18485,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18523,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18561,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18599,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18637,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18684,7 +18696,7 @@
         <v>1240</v>
       </c>
       <c r="O391" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="P391" t="b">
         <v>0</v>
@@ -18754,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18792,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18830,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18868,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18906,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18944,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19020,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19058,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19096,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19134,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19169,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19233,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19265,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19297,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19329,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19361,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19393,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19425,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19457,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19489,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19521,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19553,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19585,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19617,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19649,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19681,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19713,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19745,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19777,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19809,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19841,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19873,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19905,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19937,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19969,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20001,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20033,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20065,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20097,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20129,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20161,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20193,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20225,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20257,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20289,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20321,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20353,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20385,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20417,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20449,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20481,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20513,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20545,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (16/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (17/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (20/07/2026 16:20)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (21/07/2026 16:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (22/07/2026 16:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -3842,16 +3842,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3867,7 +3859,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -3875,30 +3867,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4198,52 +4172,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4263,7 +4237,7 @@
       <c r="E2" t="s">
         <v>737</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>45698</v>
       </c>
       <c r="G2" t="s">
@@ -4301,7 +4275,7 @@
       <c r="E3" t="s">
         <v>738</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>45714</v>
       </c>
       <c r="G3" t="s">
@@ -4339,7 +4313,7 @@
       <c r="E4" t="s">
         <v>739</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>45714</v>
       </c>
       <c r="G4" t="s">
@@ -4377,7 +4351,7 @@
       <c r="E5" t="s">
         <v>740</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>45714</v>
       </c>
       <c r="G5" t="s">
@@ -4395,7 +4369,7 @@
       <c r="K5" t="s">
         <v>1151</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="1">
         <v>45993</v>
       </c>
       <c r="P5" t="b">
@@ -4418,7 +4392,7 @@
       <c r="E6" t="s">
         <v>741</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>45736</v>
       </c>
       <c r="G6" t="s">
@@ -4436,7 +4410,7 @@
       <c r="K6" t="s">
         <v>1152</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="1">
         <v>45889</v>
       </c>
       <c r="P6" t="b">
@@ -4459,7 +4433,7 @@
       <c r="E7" t="s">
         <v>742</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>45736</v>
       </c>
       <c r="G7" t="s">
@@ -4477,7 +4451,7 @@
       <c r="K7" t="s">
         <v>1153</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="1">
         <v>45848</v>
       </c>
       <c r="N7" t="s">
@@ -4503,7 +4477,7 @@
       <c r="E8" t="s">
         <v>743</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>45736</v>
       </c>
       <c r="G8" t="s">
@@ -4532,7 +4506,7 @@
       <c r="E9" t="s">
         <v>744</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>45736</v>
       </c>
       <c r="G9" t="s">
@@ -4550,7 +4524,7 @@
       <c r="K9" t="s">
         <v>1154</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="1">
         <v>46098</v>
       </c>
       <c r="N9">
@@ -4576,7 +4550,7 @@
       <c r="E10" t="s">
         <v>745</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>45736</v>
       </c>
       <c r="G10" t="s">
@@ -4594,7 +4568,7 @@
       <c r="K10" t="s">
         <v>1155</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46114</v>
       </c>
       <c r="N10" t="s">
@@ -4620,7 +4594,7 @@
       <c r="E11" t="s">
         <v>746</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>45736</v>
       </c>
       <c r="G11" t="s">
@@ -4638,7 +4612,7 @@
       <c r="K11" t="s">
         <v>1153</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>45848</v>
       </c>
       <c r="N11" t="s">
@@ -4664,7 +4638,7 @@
       <c r="E12" t="s">
         <v>747</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="1">
         <v>45736</v>
       </c>
       <c r="G12" t="s">
@@ -4682,7 +4656,7 @@
       <c r="K12" t="s">
         <v>1156</v>
       </c>
-      <c r="M12" s="2">
+      <c r="M12" s="1">
         <v>45860</v>
       </c>
       <c r="P12" t="b">
@@ -4705,7 +4679,7 @@
       <c r="E13" t="s">
         <v>748</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="1">
         <v>45736</v>
       </c>
       <c r="G13" t="s">
@@ -4740,7 +4714,7 @@
       <c r="E14" t="s">
         <v>749</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="1">
         <v>45736</v>
       </c>
       <c r="G14" t="s">
@@ -4758,7 +4732,7 @@
       <c r="K14" t="s">
         <v>1157</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="1">
         <v>45800</v>
       </c>
       <c r="P14" t="b">
@@ -4781,7 +4755,7 @@
       <c r="E15" t="s">
         <v>750</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="1">
         <v>45736</v>
       </c>
       <c r="G15" t="s">
@@ -4819,7 +4793,7 @@
       <c r="E16" t="s">
         <v>751</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>45736</v>
       </c>
       <c r="G16" t="s">
@@ -4857,7 +4831,7 @@
       <c r="E17" t="s">
         <v>752</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>45736</v>
       </c>
       <c r="G17" t="s">
@@ -4875,7 +4849,7 @@
       <c r="K17" t="s">
         <v>1152</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>45897</v>
       </c>
       <c r="P17" t="b">
@@ -4898,7 +4872,7 @@
       <c r="E18" t="s">
         <v>753</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="1">
         <v>45736</v>
       </c>
       <c r="G18" t="s">
@@ -4916,7 +4890,7 @@
       <c r="K18" t="s">
         <v>1157</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>45802</v>
       </c>
       <c r="P18" t="b">
@@ -4939,7 +4913,7 @@
       <c r="E19" t="s">
         <v>754</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="1">
         <v>45736</v>
       </c>
       <c r="G19" t="s">
@@ -4974,7 +4948,7 @@
       <c r="E20" t="s">
         <v>755</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="1">
         <v>45736</v>
       </c>
       <c r="G20" t="s">
@@ -4992,7 +4966,7 @@
       <c r="K20" t="s">
         <v>1159</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46135</v>
       </c>
       <c r="P20" t="b">
@@ -5015,7 +4989,7 @@
       <c r="E21" t="s">
         <v>756</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="1">
         <v>45736</v>
       </c>
       <c r="G21" t="s">
@@ -5050,7 +5024,7 @@
       <c r="E22" t="s">
         <v>757</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="1">
         <v>45736</v>
       </c>
       <c r="G22" t="s">
@@ -5088,7 +5062,7 @@
       <c r="E23" t="s">
         <v>758</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="1">
         <v>45736</v>
       </c>
       <c r="G23" t="s">
@@ -5106,7 +5080,7 @@
       <c r="K23" t="s">
         <v>1161</v>
       </c>
-      <c r="M23" s="2">
+      <c r="M23" s="1">
         <v>45965</v>
       </c>
       <c r="O23" t="s">
@@ -5132,7 +5106,7 @@
       <c r="E24" t="s">
         <v>759</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="1">
         <v>45736</v>
       </c>
       <c r="G24" t="s">
@@ -5167,7 +5141,7 @@
       <c r="E25" t="s">
         <v>760</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="1">
         <v>45736</v>
       </c>
       <c r="G25" t="s">
@@ -5202,7 +5176,7 @@
       <c r="E26" t="s">
         <v>761</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="1">
         <v>45736</v>
       </c>
       <c r="G26" t="s">
@@ -5220,7 +5194,7 @@
       <c r="K26" t="s">
         <v>1164</v>
       </c>
-      <c r="M26" s="2">
+      <c r="M26" s="1">
         <v>45891</v>
       </c>
       <c r="O26" t="s">
@@ -5246,7 +5220,7 @@
       <c r="E27" t="s">
         <v>762</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>45736</v>
       </c>
       <c r="G27" t="s">
@@ -5284,7 +5258,7 @@
       <c r="E28" t="s">
         <v>763</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="1">
         <v>45736</v>
       </c>
       <c r="G28" t="s">
@@ -5313,7 +5287,7 @@
       <c r="E29" t="s">
         <v>764</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="1">
         <v>45736</v>
       </c>
       <c r="G29" t="s">
@@ -5348,7 +5322,7 @@
       <c r="E30" t="s">
         <v>765</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="1">
         <v>45736</v>
       </c>
       <c r="G30" t="s">
@@ -5366,7 +5340,7 @@
       <c r="K30" t="s">
         <v>1165</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>45945</v>
       </c>
       <c r="P30" t="b">
@@ -5389,7 +5363,7 @@
       <c r="E31" t="s">
         <v>766</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="1">
         <v>45736</v>
       </c>
       <c r="G31" t="s">
@@ -5424,7 +5398,7 @@
       <c r="E32" t="s">
         <v>767</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="1">
         <v>45736</v>
       </c>
       <c r="G32" t="s">
@@ -5462,7 +5436,7 @@
       <c r="E33" t="s">
         <v>768</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="1">
         <v>45736</v>
       </c>
       <c r="G33" t="s">
@@ -5497,7 +5471,7 @@
       <c r="E34" t="s">
         <v>769</v>
       </c>
-      <c r="F34" s="2">
+      <c r="F34" s="1">
         <v>45736</v>
       </c>
       <c r="G34" t="s">
@@ -5526,7 +5500,7 @@
       <c r="E35" t="s">
         <v>770</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="1">
         <v>45736</v>
       </c>
       <c r="G35" t="s">
@@ -5555,7 +5529,7 @@
       <c r="E36" t="s">
         <v>771</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="1">
         <v>45736</v>
       </c>
       <c r="G36" t="s">
@@ -5590,7 +5564,7 @@
       <c r="E37" t="s">
         <v>772</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="1">
         <v>45736</v>
       </c>
       <c r="G37" t="s">
@@ -5625,7 +5599,7 @@
       <c r="E38" t="s">
         <v>752</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="1">
         <v>45736</v>
       </c>
       <c r="G38" t="s">
@@ -5657,7 +5631,7 @@
       <c r="D39" t="s">
         <v>644</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="1">
         <v>45736</v>
       </c>
       <c r="G39" t="s">
@@ -5692,7 +5666,7 @@
       <c r="D40" t="s">
         <v>644</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="1">
         <v>45736</v>
       </c>
       <c r="G40" t="s">
@@ -5730,7 +5704,7 @@
       <c r="E41" t="s">
         <v>773</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="1">
         <v>45736</v>
       </c>
       <c r="G41" t="s">
@@ -5765,7 +5739,7 @@
       <c r="E42" t="s">
         <v>774</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="1">
         <v>45736</v>
       </c>
       <c r="G42" t="s">
@@ -5800,7 +5774,7 @@
       <c r="E43" t="s">
         <v>775</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>45736</v>
       </c>
       <c r="G43" t="s">
@@ -5835,7 +5809,7 @@
       <c r="E44" t="s">
         <v>776</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="1">
         <v>45769</v>
       </c>
       <c r="G44" t="s">
@@ -5853,7 +5827,7 @@
       <c r="K44" t="s">
         <v>1168</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>45856</v>
       </c>
       <c r="O44" t="s">
@@ -5879,7 +5853,7 @@
       <c r="E45" t="s">
         <v>777</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="1">
         <v>45769</v>
       </c>
       <c r="G45" t="s">
@@ -5897,7 +5871,7 @@
       <c r="K45" t="s">
         <v>1169</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46100</v>
       </c>
       <c r="N45">
@@ -5923,7 +5897,7 @@
       <c r="E46" t="s">
         <v>778</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="1">
         <v>45769</v>
       </c>
       <c r="G46" t="s">
@@ -5961,7 +5935,7 @@
       <c r="E47" t="s">
         <v>779</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="1">
         <v>45769</v>
       </c>
       <c r="G47" t="s">
@@ -5979,7 +5953,7 @@
       <c r="K47" t="s">
         <v>1170</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46113</v>
       </c>
       <c r="O47" t="s">
@@ -6005,7 +5979,7 @@
       <c r="E48" t="s">
         <v>780</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="1">
         <v>45769</v>
       </c>
       <c r="G48" t="s">
@@ -6043,7 +6017,7 @@
       <c r="E49" t="s">
         <v>781</v>
       </c>
-      <c r="F49" s="2">
+      <c r="F49" s="1">
         <v>45769</v>
       </c>
       <c r="G49" t="s">
@@ -6072,7 +6046,7 @@
       <c r="E50" t="s">
         <v>782</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="1">
         <v>45769</v>
       </c>
       <c r="G50" t="s">
@@ -6110,7 +6084,7 @@
       <c r="E51" t="s">
         <v>783</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="1">
         <v>45769</v>
       </c>
       <c r="G51" t="s">
@@ -6145,7 +6119,7 @@
       <c r="E52" t="s">
         <v>784</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="1">
         <v>45769</v>
       </c>
       <c r="G52" t="s">
@@ -6183,7 +6157,7 @@
       <c r="E53" t="s">
         <v>785</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="1">
         <v>45769</v>
       </c>
       <c r="G53" t="s">
@@ -6221,7 +6195,7 @@
       <c r="E54" t="s">
         <v>786</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="1">
         <v>45769</v>
       </c>
       <c r="G54" t="s">
@@ -6259,7 +6233,7 @@
       <c r="E55" t="s">
         <v>787</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="1">
         <v>45769</v>
       </c>
       <c r="G55" t="s">
@@ -6288,7 +6262,7 @@
       <c r="E56" t="s">
         <v>788</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="1">
         <v>45769</v>
       </c>
       <c r="G56" t="s">
@@ -6323,7 +6297,7 @@
       <c r="E57" t="s">
         <v>789</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="1">
         <v>45769</v>
       </c>
       <c r="G57" t="s">
@@ -6361,7 +6335,7 @@
       <c r="E58" t="s">
         <v>790</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="1">
         <v>45769</v>
       </c>
       <c r="G58" t="s">
@@ -6390,7 +6364,7 @@
       <c r="E59" t="s">
         <v>791</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="1">
         <v>45769</v>
       </c>
       <c r="G59" t="s">
@@ -6425,7 +6399,7 @@
       <c r="E60" t="s">
         <v>792</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <v>45769</v>
       </c>
       <c r="G60" t="s">
@@ -6460,7 +6434,7 @@
       <c r="E61" t="s">
         <v>793</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="1">
         <v>45769</v>
       </c>
       <c r="G61" t="s">
@@ -6492,7 +6466,7 @@
       <c r="E62" t="s">
         <v>794</v>
       </c>
-      <c r="F62" s="2">
+      <c r="F62" s="1">
         <v>45770</v>
       </c>
       <c r="G62" t="s">
@@ -6521,7 +6495,7 @@
       <c r="E63" t="s">
         <v>795</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="1">
         <v>45799</v>
       </c>
       <c r="G63" t="s">
@@ -6539,7 +6513,7 @@
       <c r="K63" t="s">
         <v>1173</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46092</v>
       </c>
       <c r="O63" t="s">
@@ -6565,7 +6539,7 @@
       <c r="E64" t="s">
         <v>796</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="1">
         <v>45799</v>
       </c>
       <c r="G64" t="s">
@@ -6583,7 +6557,7 @@
       <c r="K64" t="s">
         <v>1174</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46119</v>
       </c>
       <c r="P64" t="b">
@@ -6606,7 +6580,7 @@
       <c r="E65" t="s">
         <v>797</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="1">
         <v>45799</v>
       </c>
       <c r="G65" t="s">
@@ -6641,7 +6615,7 @@
       <c r="E66" t="s">
         <v>798</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="1">
         <v>45799</v>
       </c>
       <c r="G66" t="s">
@@ -6676,7 +6650,7 @@
       <c r="E67" t="s">
         <v>799</v>
       </c>
-      <c r="F67" s="2">
+      <c r="F67" s="1">
         <v>45799</v>
       </c>
       <c r="G67" t="s">
@@ -6711,7 +6685,7 @@
       <c r="E68" t="s">
         <v>800</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="1">
         <v>45799</v>
       </c>
       <c r="G68" t="s">
@@ -6746,7 +6720,7 @@
       <c r="E69" t="s">
         <v>801</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>45803</v>
       </c>
       <c r="G69" t="s">
@@ -6781,7 +6755,7 @@
       <c r="E70" t="s">
         <v>802</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="1">
         <v>45803</v>
       </c>
       <c r="G70" t="s">
@@ -6819,7 +6793,7 @@
       <c r="E71" t="s">
         <v>803</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="1">
         <v>45803</v>
       </c>
       <c r="G71" t="s">
@@ -6854,7 +6828,7 @@
       <c r="E72" t="s">
         <v>804</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>45803</v>
       </c>
       <c r="G72" t="s">
@@ -6889,7 +6863,7 @@
       <c r="E73" t="s">
         <v>805</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="1">
         <v>45803</v>
       </c>
       <c r="G73" t="s">
@@ -6927,7 +6901,7 @@
       <c r="E74" t="s">
         <v>804</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="1">
         <v>45803</v>
       </c>
       <c r="G74" t="s">
@@ -6962,7 +6936,7 @@
       <c r="E75" t="s">
         <v>806</v>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="1">
         <v>45803</v>
       </c>
       <c r="G75" t="s">
@@ -7000,7 +6974,7 @@
       <c r="E76" t="s">
         <v>807</v>
       </c>
-      <c r="F76" s="2">
+      <c r="F76" s="1">
         <v>45803</v>
       </c>
       <c r="G76" t="s">
@@ -7035,7 +7009,7 @@
       <c r="E77" t="s">
         <v>808</v>
       </c>
-      <c r="F77" s="2">
+      <c r="F77" s="1">
         <v>45803</v>
       </c>
       <c r="G77" t="s">
@@ -7070,7 +7044,7 @@
       <c r="E78" t="s">
         <v>809</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="1">
         <v>45803</v>
       </c>
       <c r="G78" t="s">
@@ -7105,7 +7079,7 @@
       <c r="E79" t="s">
         <v>810</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="1">
         <v>45803</v>
       </c>
       <c r="G79" t="s">
@@ -7140,7 +7114,7 @@
       <c r="E80" t="s">
         <v>811</v>
       </c>
-      <c r="F80" s="2">
+      <c r="F80" s="1">
         <v>45803</v>
       </c>
       <c r="G80" t="s">
@@ -7178,7 +7152,7 @@
       <c r="E81" t="s">
         <v>812</v>
       </c>
-      <c r="F81" s="2">
+      <c r="F81" s="1">
         <v>45813</v>
       </c>
       <c r="G81" t="s">
@@ -7213,7 +7187,7 @@
       <c r="E82" t="s">
         <v>813</v>
       </c>
-      <c r="F82" s="2">
+      <c r="F82" s="1">
         <v>45813</v>
       </c>
       <c r="G82" t="s">
@@ -7251,7 +7225,7 @@
       <c r="E83" t="s">
         <v>814</v>
       </c>
-      <c r="F83" s="2">
+      <c r="F83" s="1">
         <v>45813</v>
       </c>
       <c r="G83" t="s">
@@ -7286,7 +7260,7 @@
       <c r="E84" t="s">
         <v>815</v>
       </c>
-      <c r="F84" s="2">
+      <c r="F84" s="1">
         <v>45813</v>
       </c>
       <c r="G84" t="s">
@@ -7304,7 +7278,7 @@
       <c r="K84" t="s">
         <v>1178</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>45853</v>
       </c>
       <c r="N84">
@@ -7330,7 +7304,7 @@
       <c r="E85" t="s">
         <v>816</v>
       </c>
-      <c r="F85" s="2">
+      <c r="F85" s="1">
         <v>45813</v>
       </c>
       <c r="G85" t="s">
@@ -7368,7 +7342,7 @@
       <c r="E86" t="s">
         <v>817</v>
       </c>
-      <c r="F86" s="2">
+      <c r="F86" s="1">
         <v>45813</v>
       </c>
       <c r="G86" t="s">
@@ -7406,7 +7380,7 @@
       <c r="E87" t="s">
         <v>818</v>
       </c>
-      <c r="F87" s="2">
+      <c r="F87" s="1">
         <v>45813</v>
       </c>
       <c r="G87" t="s">
@@ -7424,7 +7398,7 @@
       <c r="K87" t="s">
         <v>1179</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>45797</v>
       </c>
       <c r="N87" t="s">
@@ -7450,7 +7424,7 @@
       <c r="E88" t="s">
         <v>819</v>
       </c>
-      <c r="F88" s="2">
+      <c r="F88" s="1">
         <v>45813</v>
       </c>
       <c r="G88" t="s">
@@ -7485,7 +7459,7 @@
       <c r="E89" t="s">
         <v>820</v>
       </c>
-      <c r="F89" s="2">
+      <c r="F89" s="1">
         <v>45813</v>
       </c>
       <c r="G89" t="s">
@@ -7520,7 +7494,7 @@
       <c r="E90" t="s">
         <v>821</v>
       </c>
-      <c r="F90" s="2">
+      <c r="F90" s="1">
         <v>45831</v>
       </c>
       <c r="G90" t="s">
@@ -7561,7 +7535,7 @@
       <c r="E91" t="s">
         <v>822</v>
       </c>
-      <c r="F91" s="2">
+      <c r="F91" s="1">
         <v>45831</v>
       </c>
       <c r="G91" t="s">
@@ -7596,7 +7570,7 @@
       <c r="D92" t="s">
         <v>661</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="1">
         <v>45831</v>
       </c>
       <c r="G92" t="s">
@@ -7625,7 +7599,7 @@
       <c r="E93" t="s">
         <v>823</v>
       </c>
-      <c r="F93" s="2">
+      <c r="F93" s="1">
         <v>45831</v>
       </c>
       <c r="G93" t="s">
@@ -7663,7 +7637,7 @@
       <c r="E94" t="s">
         <v>824</v>
       </c>
-      <c r="F94" s="2">
+      <c r="F94" s="1">
         <v>45831</v>
       </c>
       <c r="G94" t="s">
@@ -7701,7 +7675,7 @@
       <c r="E95" t="s">
         <v>825</v>
       </c>
-      <c r="F95" s="2">
+      <c r="F95" s="1">
         <v>45831</v>
       </c>
       <c r="G95" t="s">
@@ -7739,7 +7713,7 @@
       <c r="E96" t="s">
         <v>826</v>
       </c>
-      <c r="F96" s="2">
+      <c r="F96" s="1">
         <v>45831</v>
       </c>
       <c r="G96" t="s">
@@ -7757,7 +7731,7 @@
       <c r="K96" t="s">
         <v>1153</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>45848</v>
       </c>
       <c r="N96" t="s">
@@ -7783,7 +7757,7 @@
       <c r="E97" t="s">
         <v>827</v>
       </c>
-      <c r="F97" s="2">
+      <c r="F97" s="1">
         <v>45840</v>
       </c>
       <c r="G97" t="s">
@@ -7824,7 +7798,7 @@
       <c r="E98" t="s">
         <v>828</v>
       </c>
-      <c r="F98" s="2">
+      <c r="F98" s="1">
         <v>45840</v>
       </c>
       <c r="G98" t="s">
@@ -7862,7 +7836,7 @@
       <c r="E99" t="s">
         <v>829</v>
       </c>
-      <c r="F99" s="2">
+      <c r="F99" s="1">
         <v>45840</v>
       </c>
       <c r="G99" t="s">
@@ -7891,7 +7865,7 @@
       <c r="E100" t="s">
         <v>830</v>
       </c>
-      <c r="F100" s="2">
+      <c r="F100" s="1">
         <v>45840</v>
       </c>
       <c r="G100" t="s">
@@ -7929,7 +7903,7 @@
       <c r="E101" t="s">
         <v>831</v>
       </c>
-      <c r="F101" s="2">
+      <c r="F101" s="1">
         <v>45840</v>
       </c>
       <c r="G101" t="s">
@@ -7958,7 +7932,7 @@
       <c r="E102" t="s">
         <v>832</v>
       </c>
-      <c r="F102" s="2">
+      <c r="F102" s="1">
         <v>45840</v>
       </c>
       <c r="G102" t="s">
@@ -7987,7 +7961,7 @@
       <c r="E103" t="s">
         <v>833</v>
       </c>
-      <c r="F103" s="2">
+      <c r="F103" s="1">
         <v>45840</v>
       </c>
       <c r="G103" t="s">
@@ -8016,7 +7990,7 @@
       <c r="E104" t="s">
         <v>834</v>
       </c>
-      <c r="F104" s="2">
+      <c r="F104" s="1">
         <v>45840</v>
       </c>
       <c r="G104" t="s">
@@ -8054,7 +8028,7 @@
       <c r="E105" t="s">
         <v>835</v>
       </c>
-      <c r="F105" s="2">
+      <c r="F105" s="1">
         <v>45840</v>
       </c>
       <c r="G105" t="s">
@@ -8092,7 +8066,7 @@
       <c r="E106" t="s">
         <v>836</v>
       </c>
-      <c r="F106" s="2">
+      <c r="F106" s="1">
         <v>45840</v>
       </c>
       <c r="G106" t="s">
@@ -8110,7 +8084,7 @@
       <c r="K106" t="s">
         <v>1182</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>45889</v>
       </c>
       <c r="P106" t="b">
@@ -8133,7 +8107,7 @@
       <c r="E107" t="s">
         <v>837</v>
       </c>
-      <c r="F107" s="2">
+      <c r="F107" s="1">
         <v>45840</v>
       </c>
       <c r="G107" t="s">
@@ -8151,7 +8125,7 @@
       <c r="K107" t="s">
         <v>1183</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>45876</v>
       </c>
       <c r="P107" t="b">
@@ -8174,7 +8148,7 @@
       <c r="E108" t="s">
         <v>838</v>
       </c>
-      <c r="F108" s="2">
+      <c r="F108" s="1">
         <v>45840</v>
       </c>
       <c r="G108" t="s">
@@ -8212,7 +8186,7 @@
       <c r="E109" t="s">
         <v>839</v>
       </c>
-      <c r="F109" s="2">
+      <c r="F109" s="1">
         <v>45840</v>
       </c>
       <c r="G109" t="s">
@@ -8250,7 +8224,7 @@
       <c r="E110" t="s">
         <v>840</v>
       </c>
-      <c r="F110" s="2">
+      <c r="F110" s="1">
         <v>45840</v>
       </c>
       <c r="G110" t="s">
@@ -8285,7 +8259,7 @@
       <c r="E111" t="s">
         <v>841</v>
       </c>
-      <c r="F111" s="2">
+      <c r="F111" s="1">
         <v>45840</v>
       </c>
       <c r="G111" t="s">
@@ -8320,7 +8294,7 @@
       <c r="E112" t="s">
         <v>842</v>
       </c>
-      <c r="F112" s="2">
+      <c r="F112" s="1">
         <v>45840</v>
       </c>
       <c r="G112" t="s">
@@ -8349,7 +8323,7 @@
       <c r="E113" t="s">
         <v>843</v>
       </c>
-      <c r="F113" s="2">
+      <c r="F113" s="1">
         <v>45840</v>
       </c>
       <c r="G113" t="s">
@@ -8384,7 +8358,7 @@
       <c r="E114" t="s">
         <v>844</v>
       </c>
-      <c r="F114" s="2">
+      <c r="F114" s="1">
         <v>45840</v>
       </c>
       <c r="G114" t="s">
@@ -8419,7 +8393,7 @@
       <c r="E115" t="s">
         <v>845</v>
       </c>
-      <c r="F115" s="2">
+      <c r="F115" s="1">
         <v>45840</v>
       </c>
       <c r="G115" t="s">
@@ -8457,7 +8431,7 @@
       <c r="E116" t="s">
         <v>846</v>
       </c>
-      <c r="F116" s="2">
+      <c r="F116" s="1">
         <v>45840</v>
       </c>
       <c r="G116" t="s">
@@ -8495,7 +8469,7 @@
       <c r="E117" t="s">
         <v>847</v>
       </c>
-      <c r="F117" s="2">
+      <c r="F117" s="1">
         <v>45840</v>
       </c>
       <c r="G117" t="s">
@@ -8533,7 +8507,7 @@
       <c r="E118" t="s">
         <v>848</v>
       </c>
-      <c r="F118" s="2">
+      <c r="F118" s="1">
         <v>45840</v>
       </c>
       <c r="G118" t="s">
@@ -8571,7 +8545,7 @@
       <c r="E119" t="s">
         <v>849</v>
       </c>
-      <c r="F119" s="2">
+      <c r="F119" s="1">
         <v>45840</v>
       </c>
       <c r="G119" t="s">
@@ -8609,7 +8583,7 @@
       <c r="E120" t="s">
         <v>850</v>
       </c>
-      <c r="F120" s="2">
+      <c r="F120" s="1">
         <v>45840</v>
       </c>
       <c r="G120" t="s">
@@ -8647,7 +8621,7 @@
       <c r="E121" t="s">
         <v>851</v>
       </c>
-      <c r="F121" s="2">
+      <c r="F121" s="1">
         <v>45849</v>
       </c>
       <c r="G121" t="s">
@@ -8665,7 +8639,7 @@
       <c r="K121" t="s">
         <v>1169</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46100</v>
       </c>
       <c r="N121">
@@ -8691,7 +8665,7 @@
       <c r="E122" t="s">
         <v>852</v>
       </c>
-      <c r="F122" s="2">
+      <c r="F122" s="1">
         <v>45849</v>
       </c>
       <c r="G122" t="s">
@@ -8729,7 +8703,7 @@
       <c r="E123" t="s">
         <v>853</v>
       </c>
-      <c r="F123" s="2">
+      <c r="F123" s="1">
         <v>45849</v>
       </c>
       <c r="G123" t="s">
@@ -8758,7 +8732,7 @@
       <c r="E124" t="s">
         <v>854</v>
       </c>
-      <c r="F124" s="2">
+      <c r="F124" s="1">
         <v>45853</v>
       </c>
       <c r="G124" t="s">
@@ -8796,7 +8770,7 @@
       <c r="E125" t="s">
         <v>855</v>
       </c>
-      <c r="F125" s="2">
+      <c r="F125" s="1">
         <v>45855</v>
       </c>
       <c r="G125" t="s">
@@ -8834,7 +8808,7 @@
       <c r="E126" t="s">
         <v>856</v>
       </c>
-      <c r="F126" s="2">
+      <c r="F126" s="1">
         <v>45855</v>
       </c>
       <c r="G126" t="s">
@@ -8869,7 +8843,7 @@
       <c r="E127" t="s">
         <v>857</v>
       </c>
-      <c r="F127" s="2">
+      <c r="F127" s="1">
         <v>45856</v>
       </c>
       <c r="G127" t="s">
@@ -8898,7 +8872,7 @@
       <c r="E128" t="s">
         <v>858</v>
       </c>
-      <c r="F128" s="2">
+      <c r="F128" s="1">
         <v>45869</v>
       </c>
       <c r="G128" t="s">
@@ -8936,7 +8910,7 @@
       <c r="E129" t="s">
         <v>859</v>
       </c>
-      <c r="F129" s="2">
+      <c r="F129" s="1">
         <v>45869</v>
       </c>
       <c r="G129" t="s">
@@ -8974,7 +8948,7 @@
       <c r="E130" t="s">
         <v>860</v>
       </c>
-      <c r="F130" s="2">
+      <c r="F130" s="1">
         <v>45869</v>
       </c>
       <c r="G130" t="s">
@@ -8992,7 +8966,7 @@
       <c r="K130" t="s">
         <v>1187</v>
       </c>
-      <c r="M130" s="2">
+      <c r="M130" s="1">
         <v>45916</v>
       </c>
       <c r="N130">
@@ -9018,7 +8992,7 @@
       <c r="E131" t="s">
         <v>861</v>
       </c>
-      <c r="F131" s="2">
+      <c r="F131" s="1">
         <v>45869</v>
       </c>
       <c r="G131" t="s">
@@ -9053,7 +9027,7 @@
       <c r="E132" t="s">
         <v>862</v>
       </c>
-      <c r="F132" s="2">
+      <c r="F132" s="1">
         <v>45869</v>
       </c>
       <c r="G132" t="s">
@@ -9071,7 +9045,7 @@
       <c r="K132" t="s">
         <v>1189</v>
       </c>
-      <c r="M132" s="2">
+      <c r="M132" s="1">
         <v>46014</v>
       </c>
       <c r="N132">
@@ -9097,7 +9071,7 @@
       <c r="E133" t="s">
         <v>863</v>
       </c>
-      <c r="F133" s="2">
+      <c r="F133" s="1">
         <v>45869</v>
       </c>
       <c r="G133" t="s">
@@ -9126,7 +9100,7 @@
       <c r="E134" t="s">
         <v>864</v>
       </c>
-      <c r="F134" s="2">
+      <c r="F134" s="1">
         <v>45882</v>
       </c>
       <c r="G134" t="s">
@@ -9164,7 +9138,7 @@
       <c r="E135" t="s">
         <v>865</v>
       </c>
-      <c r="F135" s="2">
+      <c r="F135" s="1">
         <v>45882</v>
       </c>
       <c r="G135" t="s">
@@ -9193,7 +9167,7 @@
       <c r="E136" t="s">
         <v>866</v>
       </c>
-      <c r="F136" s="2">
+      <c r="F136" s="1">
         <v>45891</v>
       </c>
       <c r="G136" t="s">
@@ -9222,7 +9196,7 @@
       <c r="E137" t="s">
         <v>867</v>
       </c>
-      <c r="F137" s="2">
+      <c r="F137" s="1">
         <v>45891</v>
       </c>
       <c r="G137" t="s">
@@ -9251,7 +9225,7 @@
       <c r="E138" t="s">
         <v>868</v>
       </c>
-      <c r="F138" s="2">
+      <c r="F138" s="1">
         <v>45891</v>
       </c>
       <c r="G138" t="s">
@@ -9289,7 +9263,7 @@
       <c r="E139" t="s">
         <v>869</v>
       </c>
-      <c r="F139" s="2">
+      <c r="F139" s="1">
         <v>45891</v>
       </c>
       <c r="G139" t="s">
@@ -9318,7 +9292,7 @@
       <c r="E140" t="s">
         <v>870</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140" s="1">
         <v>45891</v>
       </c>
       <c r="G140" t="s">
@@ -9353,7 +9327,7 @@
       <c r="E141" t="s">
         <v>871</v>
       </c>
-      <c r="F141" s="2">
+      <c r="F141" s="1">
         <v>45891</v>
       </c>
       <c r="G141" t="s">
@@ -9382,7 +9356,7 @@
       <c r="E142" t="s">
         <v>872</v>
       </c>
-      <c r="F142" s="2">
+      <c r="F142" s="1">
         <v>45891</v>
       </c>
       <c r="G142" t="s">
@@ -9411,7 +9385,7 @@
       <c r="E143" t="s">
         <v>873</v>
       </c>
-      <c r="F143" s="2">
+      <c r="F143" s="1">
         <v>45891</v>
       </c>
       <c r="G143" t="s">
@@ -9440,7 +9414,7 @@
       <c r="E144" t="s">
         <v>874</v>
       </c>
-      <c r="F144" s="2">
+      <c r="F144" s="1">
         <v>45891</v>
       </c>
       <c r="G144" t="s">
@@ -9469,7 +9443,7 @@
       <c r="E145" t="s">
         <v>875</v>
       </c>
-      <c r="F145" s="2">
+      <c r="F145" s="1">
         <v>45891</v>
       </c>
       <c r="G145" t="s">
@@ -9504,7 +9478,7 @@
       <c r="E146" t="s">
         <v>876</v>
       </c>
-      <c r="F146" s="2">
+      <c r="F146" s="1">
         <v>45891</v>
       </c>
       <c r="G146" t="s">
@@ -9533,7 +9507,7 @@
       <c r="E147" t="s">
         <v>877</v>
       </c>
-      <c r="F147" s="2">
+      <c r="F147" s="1">
         <v>45891</v>
       </c>
       <c r="G147" t="s">
@@ -9568,7 +9542,7 @@
       <c r="E148" t="s">
         <v>878</v>
       </c>
-      <c r="F148" s="2">
+      <c r="F148" s="1">
         <v>45891</v>
       </c>
       <c r="G148" t="s">
@@ -9606,7 +9580,7 @@
       <c r="E149" t="s">
         <v>879</v>
       </c>
-      <c r="F149" s="2">
+      <c r="F149" s="1">
         <v>45891</v>
       </c>
       <c r="G149" t="s">
@@ -9641,7 +9615,7 @@
       <c r="E150" t="s">
         <v>880</v>
       </c>
-      <c r="F150" s="2">
+      <c r="F150" s="1">
         <v>45891</v>
       </c>
       <c r="G150" t="s">
@@ -9659,7 +9633,7 @@
       <c r="K150" t="s">
         <v>1173</v>
       </c>
-      <c r="M150" s="2">
+      <c r="M150" s="1">
         <v>46092</v>
       </c>
       <c r="O150" t="s">
@@ -9685,7 +9659,7 @@
       <c r="E151" t="s">
         <v>881</v>
       </c>
-      <c r="F151" s="2">
+      <c r="F151" s="1">
         <v>45891</v>
       </c>
       <c r="G151" t="s">
@@ -9720,7 +9694,7 @@
       <c r="E152" t="s">
         <v>871</v>
       </c>
-      <c r="F152" s="2">
+      <c r="F152" s="1">
         <v>45891</v>
       </c>
       <c r="G152" t="s">
@@ -9738,7 +9712,7 @@
       <c r="K152" t="s">
         <v>1174</v>
       </c>
-      <c r="M152" s="2">
+      <c r="M152" s="1">
         <v>46119</v>
       </c>
       <c r="P152" t="b">
@@ -9761,7 +9735,7 @@
       <c r="E153" t="s">
         <v>882</v>
       </c>
-      <c r="F153" s="2">
+      <c r="F153" s="1">
         <v>45891</v>
       </c>
       <c r="G153" t="s">
@@ -9799,7 +9773,7 @@
       <c r="E154" t="s">
         <v>883</v>
       </c>
-      <c r="F154" s="2">
+      <c r="F154" s="1">
         <v>45891</v>
       </c>
       <c r="G154" t="s">
@@ -9834,7 +9808,7 @@
       <c r="E155" t="s">
         <v>884</v>
       </c>
-      <c r="F155" s="2">
+      <c r="F155" s="1">
         <v>45891</v>
       </c>
       <c r="G155" t="s">
@@ -9869,7 +9843,7 @@
       <c r="E156" t="s">
         <v>885</v>
       </c>
-      <c r="F156" s="2">
+      <c r="F156" s="1">
         <v>45891</v>
       </c>
       <c r="G156" t="s">
@@ -9907,7 +9881,7 @@
       <c r="E157" t="s">
         <v>886</v>
       </c>
-      <c r="F157" s="2">
+      <c r="F157" s="1">
         <v>45891</v>
       </c>
       <c r="G157" t="s">
@@ -9945,7 +9919,7 @@
       <c r="E158" t="s">
         <v>887</v>
       </c>
-      <c r="F158" s="2">
+      <c r="F158" s="1">
         <v>45894</v>
       </c>
       <c r="G158" t="s">
@@ -9963,7 +9937,7 @@
       <c r="K158" t="s">
         <v>1192</v>
       </c>
-      <c r="M158" s="2">
+      <c r="M158" s="1">
         <v>45946</v>
       </c>
       <c r="P158" t="b">
@@ -9986,7 +9960,7 @@
       <c r="E159" t="s">
         <v>888</v>
       </c>
-      <c r="F159" s="2">
+      <c r="F159" s="1">
         <v>45894</v>
       </c>
       <c r="G159" t="s">
@@ -10024,7 +9998,7 @@
       <c r="E160" t="s">
         <v>889</v>
       </c>
-      <c r="F160" s="2">
+      <c r="F160" s="1">
         <v>45898</v>
       </c>
       <c r="G160" t="s">
@@ -10062,7 +10036,7 @@
       <c r="E161" t="s">
         <v>890</v>
       </c>
-      <c r="F161" s="2">
+      <c r="F161" s="1">
         <v>45898</v>
       </c>
       <c r="G161" t="s">
@@ -10080,7 +10054,7 @@
       <c r="K161" t="s">
         <v>1193</v>
       </c>
-      <c r="M161" s="2">
+      <c r="M161" s="1">
         <v>45953</v>
       </c>
       <c r="N161" t="s">
@@ -10106,7 +10080,7 @@
       <c r="E162" t="s">
         <v>891</v>
       </c>
-      <c r="F162" s="2">
+      <c r="F162" s="1">
         <v>45898</v>
       </c>
       <c r="G162" t="s">
@@ -10124,7 +10098,7 @@
       <c r="K162" t="s">
         <v>1194</v>
       </c>
-      <c r="M162" s="2">
+      <c r="M162" s="1">
         <v>45940</v>
       </c>
       <c r="P162" t="b">
@@ -10147,7 +10121,7 @@
       <c r="E163" t="s">
         <v>892</v>
       </c>
-      <c r="F163" s="2">
+      <c r="F163" s="1">
         <v>45898</v>
       </c>
       <c r="G163" t="s">
@@ -10165,7 +10139,7 @@
       <c r="K163" t="s">
         <v>1194</v>
       </c>
-      <c r="M163" s="2">
+      <c r="M163" s="1">
         <v>45940</v>
       </c>
       <c r="P163" t="b">
@@ -10188,7 +10162,7 @@
       <c r="E164" t="s">
         <v>893</v>
       </c>
-      <c r="F164" s="2">
+      <c r="F164" s="1">
         <v>45910</v>
       </c>
       <c r="G164" t="s">
@@ -10223,7 +10197,7 @@
       <c r="E165" t="s">
         <v>894</v>
       </c>
-      <c r="F165" s="2">
+      <c r="F165" s="1">
         <v>45917</v>
       </c>
       <c r="G165" t="s">
@@ -10264,7 +10238,7 @@
       <c r="E166" t="s">
         <v>895</v>
       </c>
-      <c r="F166" s="2">
+      <c r="F166" s="1">
         <v>45917</v>
       </c>
       <c r="G166" t="s">
@@ -10299,7 +10273,7 @@
       <c r="E167" t="s">
         <v>896</v>
       </c>
-      <c r="F167" s="2">
+      <c r="F167" s="1">
         <v>45917</v>
       </c>
       <c r="G167" t="s">
@@ -10328,7 +10302,7 @@
       <c r="E168" t="s">
         <v>897</v>
       </c>
-      <c r="F168" s="2">
+      <c r="F168" s="1">
         <v>45917</v>
       </c>
       <c r="G168" t="s">
@@ -10369,7 +10343,7 @@
       <c r="E169" t="s">
         <v>898</v>
       </c>
-      <c r="F169" s="2">
+      <c r="F169" s="1">
         <v>45917</v>
       </c>
       <c r="G169" t="s">
@@ -10387,7 +10361,7 @@
       <c r="K169" t="s">
         <v>1197</v>
       </c>
-      <c r="M169" s="2">
+      <c r="M169" s="1">
         <v>45973</v>
       </c>
       <c r="P169" t="b">
@@ -10410,7 +10384,7 @@
       <c r="E170" t="s">
         <v>899</v>
       </c>
-      <c r="F170" s="2">
+      <c r="F170" s="1">
         <v>45917</v>
       </c>
       <c r="G170" t="s">
@@ -10445,7 +10419,7 @@
       <c r="E171" t="s">
         <v>900</v>
       </c>
-      <c r="F171" s="2">
+      <c r="F171" s="1">
         <v>45917</v>
       </c>
       <c r="G171" t="s">
@@ -10483,7 +10457,7 @@
       <c r="E172" t="s">
         <v>901</v>
       </c>
-      <c r="F172" s="2">
+      <c r="F172" s="1">
         <v>45917</v>
       </c>
       <c r="G172" t="s">
@@ -10518,7 +10492,7 @@
       <c r="E173" t="s">
         <v>902</v>
       </c>
-      <c r="F173" s="2">
+      <c r="F173" s="1">
         <v>45917</v>
       </c>
       <c r="G173" t="s">
@@ -10553,7 +10527,7 @@
       <c r="E174" t="s">
         <v>903</v>
       </c>
-      <c r="F174" s="2">
+      <c r="F174" s="1">
         <v>45917</v>
       </c>
       <c r="G174" t="s">
@@ -10588,7 +10562,7 @@
       <c r="E175" t="s">
         <v>904</v>
       </c>
-      <c r="F175" s="2">
+      <c r="F175" s="1">
         <v>45917</v>
       </c>
       <c r="G175" t="s">
@@ -10606,7 +10580,7 @@
       <c r="K175" t="s">
         <v>1198</v>
       </c>
-      <c r="M175" s="2">
+      <c r="M175" s="1">
         <v>46122</v>
       </c>
       <c r="O175" t="s">
@@ -10632,7 +10606,7 @@
       <c r="E176" t="s">
         <v>808</v>
       </c>
-      <c r="F176" s="2">
+      <c r="F176" s="1">
         <v>45917</v>
       </c>
       <c r="G176" t="s">
@@ -10670,7 +10644,7 @@
       <c r="E177" t="s">
         <v>905</v>
       </c>
-      <c r="F177" s="2">
+      <c r="F177" s="1">
         <v>45917</v>
       </c>
       <c r="G177" t="s">
@@ -10688,7 +10662,7 @@
       <c r="K177" t="s">
         <v>1199</v>
       </c>
-      <c r="M177" s="2">
+      <c r="M177" s="1">
         <v>45961</v>
       </c>
       <c r="O177" t="s">
@@ -10714,7 +10688,7 @@
       <c r="E178" t="s">
         <v>906</v>
       </c>
-      <c r="F178" s="2">
+      <c r="F178" s="1">
         <v>45937</v>
       </c>
       <c r="G178" t="s">
@@ -10752,7 +10726,7 @@
       <c r="E179" t="s">
         <v>907</v>
       </c>
-      <c r="F179" s="2">
+      <c r="F179" s="1">
         <v>45937</v>
       </c>
       <c r="G179" t="s">
@@ -10781,7 +10755,7 @@
       <c r="E180" t="s">
         <v>908</v>
       </c>
-      <c r="F180" s="2">
+      <c r="F180" s="1">
         <v>45937</v>
       </c>
       <c r="G180" t="s">
@@ -10819,7 +10793,7 @@
       <c r="E181" t="s">
         <v>909</v>
       </c>
-      <c r="F181" s="2">
+      <c r="F181" s="1">
         <v>45937</v>
       </c>
       <c r="G181" t="s">
@@ -10854,7 +10828,7 @@
       <c r="E182" t="s">
         <v>910</v>
       </c>
-      <c r="F182" s="2">
+      <c r="F182" s="1">
         <v>45937</v>
       </c>
       <c r="G182" t="s">
@@ -10883,7 +10857,7 @@
       <c r="E183" t="s">
         <v>911</v>
       </c>
-      <c r="F183" s="2">
+      <c r="F183" s="1">
         <v>45937</v>
       </c>
       <c r="G183" t="s">
@@ -10918,7 +10892,7 @@
       <c r="D184" t="s">
         <v>687</v>
       </c>
-      <c r="F184" s="2">
+      <c r="F184" s="1">
         <v>45939</v>
       </c>
       <c r="G184" t="s">
@@ -10953,7 +10927,7 @@
       <c r="E185" t="s">
         <v>912</v>
       </c>
-      <c r="F185" s="2">
+      <c r="F185" s="1">
         <v>45939</v>
       </c>
       <c r="G185" t="s">
@@ -10991,7 +10965,7 @@
       <c r="E186" t="s">
         <v>913</v>
       </c>
-      <c r="F186" s="2">
+      <c r="F186" s="1">
         <v>45939</v>
       </c>
       <c r="G186" t="s">
@@ -11029,7 +11003,7 @@
       <c r="E187" t="s">
         <v>914</v>
       </c>
-      <c r="F187" s="2">
+      <c r="F187" s="1">
         <v>45939</v>
       </c>
       <c r="G187" t="s">
@@ -11047,7 +11021,7 @@
       <c r="K187" t="s">
         <v>1201</v>
       </c>
-      <c r="M187" s="2">
+      <c r="M187" s="1">
         <v>46014</v>
       </c>
       <c r="N187">
@@ -11073,7 +11047,7 @@
       <c r="E188" t="s">
         <v>915</v>
       </c>
-      <c r="F188" s="2">
+      <c r="F188" s="1">
         <v>45946</v>
       </c>
       <c r="G188" t="s">
@@ -11091,7 +11065,7 @@
       <c r="K188" t="s">
         <v>1202</v>
       </c>
-      <c r="M188" s="2">
+      <c r="M188" s="1">
         <v>45986</v>
       </c>
       <c r="O188" t="s">
@@ -11117,7 +11091,7 @@
       <c r="E189" t="s">
         <v>916</v>
       </c>
-      <c r="F189" s="2">
+      <c r="F189" s="1">
         <v>45965</v>
       </c>
       <c r="G189" t="s">
@@ -11135,7 +11109,7 @@
       <c r="K189" t="s">
         <v>1203</v>
       </c>
-      <c r="M189" s="2">
+      <c r="M189" s="1">
         <v>46120</v>
       </c>
       <c r="P189" t="b">
@@ -11158,7 +11132,7 @@
       <c r="E190" t="s">
         <v>917</v>
       </c>
-      <c r="F190" s="2">
+      <c r="F190" s="1">
         <v>45965</v>
       </c>
       <c r="G190" t="s">
@@ -11196,7 +11170,7 @@
       <c r="E191" t="s">
         <v>918</v>
       </c>
-      <c r="F191" s="2">
+      <c r="F191" s="1">
         <v>45967</v>
       </c>
       <c r="G191" t="s">
@@ -11214,7 +11188,7 @@
       <c r="K191" t="s">
         <v>1204</v>
       </c>
-      <c r="M191" s="2">
+      <c r="M191" s="1">
         <v>45972</v>
       </c>
       <c r="P191" t="b">
@@ -11237,7 +11211,7 @@
       <c r="E192" t="s">
         <v>919</v>
       </c>
-      <c r="F192" s="2">
+      <c r="F192" s="1">
         <v>45968</v>
       </c>
       <c r="G192" t="s">
@@ -11275,7 +11249,7 @@
       <c r="E193" t="s">
         <v>920</v>
       </c>
-      <c r="F193" s="2">
+      <c r="F193" s="1">
         <v>45968</v>
       </c>
       <c r="G193" t="s">
@@ -11313,7 +11287,7 @@
       <c r="E194" t="s">
         <v>921</v>
       </c>
-      <c r="F194" s="2">
+      <c r="F194" s="1">
         <v>45968</v>
       </c>
       <c r="G194" t="s">
@@ -11342,7 +11316,7 @@
       <c r="E195" t="s">
         <v>922</v>
       </c>
-      <c r="F195" s="2">
+      <c r="F195" s="1">
         <v>45971</v>
       </c>
       <c r="G195" t="s">
@@ -11380,7 +11354,7 @@
       <c r="E196" t="s">
         <v>923</v>
       </c>
-      <c r="F196" s="2">
+      <c r="F196" s="1">
         <v>45978</v>
       </c>
       <c r="G196" t="s">
@@ -11409,7 +11383,7 @@
       <c r="E197" t="s">
         <v>924</v>
       </c>
-      <c r="F197" s="2">
+      <c r="F197" s="1">
         <v>45978</v>
       </c>
       <c r="G197" t="s">
@@ -11438,7 +11412,7 @@
       <c r="E198" t="s">
         <v>925</v>
       </c>
-      <c r="F198" s="2">
+      <c r="F198" s="1">
         <v>45978</v>
       </c>
       <c r="G198" t="s">
@@ -11467,7 +11441,7 @@
       <c r="E199" t="s">
         <v>926</v>
       </c>
-      <c r="F199" s="2">
+      <c r="F199" s="1">
         <v>45979</v>
       </c>
       <c r="G199" t="s">
@@ -11485,7 +11459,7 @@
       <c r="K199" t="s">
         <v>1205</v>
       </c>
-      <c r="M199" s="2">
+      <c r="M199" s="1">
         <v>46049</v>
       </c>
       <c r="P199" t="b">
@@ -11508,7 +11482,7 @@
       <c r="E200" t="s">
         <v>927</v>
       </c>
-      <c r="F200" s="2">
+      <c r="F200" s="1">
         <v>45986</v>
       </c>
       <c r="G200" t="s">
@@ -11546,7 +11520,7 @@
       <c r="E201" t="s">
         <v>928</v>
       </c>
-      <c r="F201" s="2">
+      <c r="F201" s="1">
         <v>45986</v>
       </c>
       <c r="G201" t="s">
@@ -11584,7 +11558,7 @@
       <c r="E202" t="s">
         <v>929</v>
       </c>
-      <c r="F202" s="2">
+      <c r="F202" s="1">
         <v>45986</v>
       </c>
       <c r="G202" t="s">
@@ -11622,7 +11596,7 @@
       <c r="E203" t="s">
         <v>930</v>
       </c>
-      <c r="F203" s="2">
+      <c r="F203" s="1">
         <v>45986</v>
       </c>
       <c r="G203" t="s">
@@ -11660,7 +11634,7 @@
       <c r="E204" t="s">
         <v>931</v>
       </c>
-      <c r="F204" s="2">
+      <c r="F204" s="1">
         <v>45986</v>
       </c>
       <c r="G204" t="s">
@@ -11698,7 +11672,7 @@
       <c r="E205" t="s">
         <v>932</v>
       </c>
-      <c r="F205" s="2">
+      <c r="F205" s="1">
         <v>45986</v>
       </c>
       <c r="G205" t="s">
@@ -11736,7 +11710,7 @@
       <c r="E206" t="s">
         <v>933</v>
       </c>
-      <c r="F206" s="2">
+      <c r="F206" s="1">
         <v>45986</v>
       </c>
       <c r="G206" t="s">
@@ -11771,7 +11745,7 @@
       <c r="E207" t="s">
         <v>934</v>
       </c>
-      <c r="F207" s="2">
+      <c r="F207" s="1">
         <v>45986</v>
       </c>
       <c r="G207" t="s">
@@ -11789,7 +11763,7 @@
       <c r="K207" t="s">
         <v>1207</v>
       </c>
-      <c r="M207" s="2">
+      <c r="M207" s="1">
         <v>46153</v>
       </c>
       <c r="P207" t="b">
@@ -11812,7 +11786,7 @@
       <c r="E208" t="s">
         <v>935</v>
       </c>
-      <c r="F208" s="2">
+      <c r="F208" s="1">
         <v>45986</v>
       </c>
       <c r="G208" t="s">
@@ -11830,7 +11804,7 @@
       <c r="K208" t="s">
         <v>1208</v>
       </c>
-      <c r="M208" s="2">
+      <c r="M208" s="1">
         <v>46031</v>
       </c>
       <c r="P208" t="b">
@@ -11853,7 +11827,7 @@
       <c r="E209" t="s">
         <v>936</v>
       </c>
-      <c r="F209" s="2">
+      <c r="F209" s="1">
         <v>46000</v>
       </c>
       <c r="G209" t="s">
@@ -11871,7 +11845,7 @@
       <c r="K209" t="s">
         <v>1209</v>
       </c>
-      <c r="M209" s="2">
+      <c r="M209" s="1">
         <v>46191</v>
       </c>
       <c r="P209" t="b">
@@ -11894,7 +11868,7 @@
       <c r="E210" t="s">
         <v>937</v>
       </c>
-      <c r="F210" s="2">
+      <c r="F210" s="1">
         <v>46000</v>
       </c>
       <c r="G210" t="s">
@@ -11932,7 +11906,7 @@
       <c r="E211" t="s">
         <v>938</v>
       </c>
-      <c r="F211" s="2">
+      <c r="F211" s="1">
         <v>46000</v>
       </c>
       <c r="G211" t="s">
@@ -11967,7 +11941,7 @@
       <c r="E212" t="s">
         <v>939</v>
       </c>
-      <c r="F212" s="2">
+      <c r="F212" s="1">
         <v>46000</v>
       </c>
       <c r="G212" t="s">
@@ -12002,7 +11976,7 @@
       <c r="E213" t="s">
         <v>940</v>
       </c>
-      <c r="F213" s="2">
+      <c r="F213" s="1">
         <v>46007</v>
       </c>
       <c r="G213" t="s">
@@ -12040,7 +12014,7 @@
       <c r="E214" t="s">
         <v>941</v>
       </c>
-      <c r="F214" s="2">
+      <c r="F214" s="1">
         <v>46007</v>
       </c>
       <c r="G214" t="s">
@@ -12058,7 +12032,7 @@
       <c r="K214" t="s">
         <v>1212</v>
       </c>
-      <c r="M214" s="2">
+      <c r="M214" s="1">
         <v>46021</v>
       </c>
       <c r="N214">
@@ -12084,7 +12058,7 @@
       <c r="E215" t="s">
         <v>942</v>
       </c>
-      <c r="F215" s="2">
+      <c r="F215" s="1">
         <v>46007</v>
       </c>
       <c r="G215" t="s">
@@ -12122,7 +12096,7 @@
       <c r="E216" t="s">
         <v>943</v>
       </c>
-      <c r="F216" s="2">
+      <c r="F216" s="1">
         <v>46010</v>
       </c>
       <c r="G216" t="s">
@@ -12151,7 +12125,7 @@
       <c r="E217" t="s">
         <v>944</v>
       </c>
-      <c r="F217" s="2">
+      <c r="F217" s="1">
         <v>46010</v>
       </c>
       <c r="G217" t="s">
@@ -12169,7 +12143,7 @@
       <c r="K217" t="s">
         <v>1213</v>
       </c>
-      <c r="M217" s="2">
+      <c r="M217" s="1">
         <v>46052</v>
       </c>
       <c r="P217" t="b">
@@ -12192,7 +12166,7 @@
       <c r="E218" t="s">
         <v>945</v>
       </c>
-      <c r="F218" s="2">
+      <c r="F218" s="1">
         <v>46010</v>
       </c>
       <c r="G218" t="s">
@@ -12230,7 +12204,7 @@
       <c r="E219" t="s">
         <v>946</v>
       </c>
-      <c r="F219" s="2">
+      <c r="F219" s="1">
         <v>46010</v>
       </c>
       <c r="G219" t="s">
@@ -12268,7 +12242,7 @@
       <c r="E220" t="s">
         <v>947</v>
       </c>
-      <c r="F220" s="2">
+      <c r="F220" s="1">
         <v>46010</v>
       </c>
       <c r="G220" t="s">
@@ -12306,7 +12280,7 @@
       <c r="E221" t="s">
         <v>948</v>
       </c>
-      <c r="F221" s="2">
+      <c r="F221" s="1">
         <v>46028</v>
       </c>
       <c r="G221" t="s">
@@ -12341,7 +12315,7 @@
       <c r="E222" t="s">
         <v>949</v>
       </c>
-      <c r="F222" s="2">
+      <c r="F222" s="1">
         <v>46028</v>
       </c>
       <c r="G222" t="s">
@@ -12379,7 +12353,7 @@
       <c r="E223" t="s">
         <v>950</v>
       </c>
-      <c r="F223" s="2">
+      <c r="F223" s="1">
         <v>46028</v>
       </c>
       <c r="G223" t="s">
@@ -12417,7 +12391,7 @@
       <c r="E224" t="s">
         <v>951</v>
       </c>
-      <c r="F224" s="2">
+      <c r="F224" s="1">
         <v>46028</v>
       </c>
       <c r="G224" t="s">
@@ -12455,7 +12429,7 @@
       <c r="E225" t="s">
         <v>952</v>
       </c>
-      <c r="F225" s="2">
+      <c r="F225" s="1">
         <v>46028</v>
       </c>
       <c r="G225" t="s">
@@ -12493,7 +12467,7 @@
       <c r="E226" t="s">
         <v>953</v>
       </c>
-      <c r="F226" s="2">
+      <c r="F226" s="1">
         <v>46028</v>
       </c>
       <c r="G226" t="s">
@@ -12531,7 +12505,7 @@
       <c r="E227" t="s">
         <v>954</v>
       </c>
-      <c r="F227" s="2">
+      <c r="F227" s="1">
         <v>46028</v>
       </c>
       <c r="G227" t="s">
@@ -12569,7 +12543,7 @@
       <c r="E228" t="s">
         <v>955</v>
       </c>
-      <c r="F228" s="2">
+      <c r="F228" s="1">
         <v>46028</v>
       </c>
       <c r="G228" t="s">
@@ -12607,7 +12581,7 @@
       <c r="E229" t="s">
         <v>956</v>
       </c>
-      <c r="F229" s="2">
+      <c r="F229" s="1">
         <v>46028</v>
       </c>
       <c r="G229" t="s">
@@ -12642,7 +12616,7 @@
       <c r="E230" t="s">
         <v>957</v>
       </c>
-      <c r="F230" s="2">
+      <c r="F230" s="1">
         <v>46028</v>
       </c>
       <c r="G230" t="s">
@@ -12680,7 +12654,7 @@
       <c r="E231" t="s">
         <v>958</v>
       </c>
-      <c r="F231" s="2">
+      <c r="F231" s="1">
         <v>46028</v>
       </c>
       <c r="G231" t="s">
@@ -12698,7 +12672,7 @@
       <c r="K231" t="s">
         <v>1214</v>
       </c>
-      <c r="M231" s="2">
+      <c r="M231" s="1">
         <v>46063</v>
       </c>
       <c r="P231" t="b">
@@ -12721,7 +12695,7 @@
       <c r="E232" t="s">
         <v>959</v>
       </c>
-      <c r="F232" s="2">
+      <c r="F232" s="1">
         <v>46028</v>
       </c>
       <c r="G232" t="s">
@@ -12756,7 +12730,7 @@
       <c r="E233" t="s">
         <v>960</v>
       </c>
-      <c r="F233" s="2">
+      <c r="F233" s="1">
         <v>46028</v>
       </c>
       <c r="G233" t="s">
@@ -12791,7 +12765,7 @@
       <c r="E234" t="s">
         <v>961</v>
       </c>
-      <c r="F234" s="2">
+      <c r="F234" s="1">
         <v>46028</v>
       </c>
       <c r="G234" t="s">
@@ -12809,7 +12783,7 @@
       <c r="K234" t="s">
         <v>1214</v>
       </c>
-      <c r="M234" s="2">
+      <c r="M234" s="1">
         <v>46063</v>
       </c>
       <c r="O234" t="s">
@@ -12835,7 +12809,7 @@
       <c r="E235" t="s">
         <v>962</v>
       </c>
-      <c r="F235" s="2">
+      <c r="F235" s="1">
         <v>46028</v>
       </c>
       <c r="G235" t="s">
@@ -12853,7 +12827,7 @@
       <c r="K235" t="s">
         <v>1214</v>
       </c>
-      <c r="M235" s="2">
+      <c r="M235" s="1">
         <v>46063</v>
       </c>
       <c r="O235" t="s">
@@ -12879,7 +12853,7 @@
       <c r="E236" t="s">
         <v>963</v>
       </c>
-      <c r="F236" s="2">
+      <c r="F236" s="1">
         <v>46028</v>
       </c>
       <c r="G236" t="s">
@@ -12897,7 +12871,7 @@
       <c r="K236" t="s">
         <v>1216</v>
       </c>
-      <c r="M236" s="2">
+      <c r="M236" s="1">
         <v>46114</v>
       </c>
       <c r="P236" t="b">
@@ -12920,7 +12894,7 @@
       <c r="E237" t="s">
         <v>964</v>
       </c>
-      <c r="F237" s="2">
+      <c r="F237" s="1">
         <v>46028</v>
       </c>
       <c r="G237" t="s">
@@ -12958,7 +12932,7 @@
       <c r="E238" t="s">
         <v>965</v>
       </c>
-      <c r="F238" s="2">
+      <c r="F238" s="1">
         <v>46028</v>
       </c>
       <c r="G238" t="s">
@@ -12987,7 +12961,7 @@
       <c r="E239" t="s">
         <v>966</v>
       </c>
-      <c r="F239" s="2">
+      <c r="F239" s="1">
         <v>46036</v>
       </c>
       <c r="G239" t="s">
@@ -13005,7 +12979,7 @@
       <c r="K239" t="s">
         <v>1217</v>
       </c>
-      <c r="M239" s="2">
+      <c r="M239" s="1">
         <v>46052</v>
       </c>
       <c r="P239" t="b">
@@ -13028,7 +13002,7 @@
       <c r="E240" t="s">
         <v>967</v>
       </c>
-      <c r="F240" s="2">
+      <c r="F240" s="1">
         <v>46036</v>
       </c>
       <c r="G240" t="s">
@@ -13063,7 +13037,7 @@
       <c r="E241" t="s">
         <v>968</v>
       </c>
-      <c r="F241" s="2">
+      <c r="F241" s="1">
         <v>46036</v>
       </c>
       <c r="G241" t="s">
@@ -13098,7 +13072,7 @@
       <c r="E242" t="s">
         <v>969</v>
       </c>
-      <c r="F242" s="2">
+      <c r="F242" s="1">
         <v>46036</v>
       </c>
       <c r="G242" t="s">
@@ -13136,7 +13110,7 @@
       <c r="E243" t="s">
         <v>970</v>
       </c>
-      <c r="F243" s="2">
+      <c r="F243" s="1">
         <v>46048</v>
       </c>
       <c r="G243" t="s">
@@ -13168,7 +13142,7 @@
       <c r="E244" t="s">
         <v>971</v>
       </c>
-      <c r="F244" s="2">
+      <c r="F244" s="1">
         <v>46048</v>
       </c>
       <c r="G244" t="s">
@@ -13206,7 +13180,7 @@
       <c r="E245" t="s">
         <v>972</v>
       </c>
-      <c r="F245" s="2">
+      <c r="F245" s="1">
         <v>46048</v>
       </c>
       <c r="G245" t="s">
@@ -13244,7 +13218,7 @@
       <c r="E246" t="s">
         <v>973</v>
       </c>
-      <c r="F246" s="2">
+      <c r="F246" s="1">
         <v>46050</v>
       </c>
       <c r="G246" t="s">
@@ -13262,7 +13236,7 @@
       <c r="K246" t="s">
         <v>1220</v>
       </c>
-      <c r="M246" s="2">
+      <c r="M246" s="1">
         <v>46191</v>
       </c>
       <c r="P246" t="b">
@@ -13285,7 +13259,7 @@
       <c r="E247" t="s">
         <v>974</v>
       </c>
-      <c r="F247" s="2">
+      <c r="F247" s="1">
         <v>46050</v>
       </c>
       <c r="G247" t="s">
@@ -13314,7 +13288,7 @@
       <c r="E248" t="s">
         <v>975</v>
       </c>
-      <c r="F248" s="2">
+      <c r="F248" s="1">
         <v>46050</v>
       </c>
       <c r="G248" t="s">
@@ -13343,7 +13317,7 @@
       <c r="E249" t="s">
         <v>976</v>
       </c>
-      <c r="F249" s="2">
+      <c r="F249" s="1">
         <v>46050</v>
       </c>
       <c r="G249" t="s">
@@ -13381,7 +13355,7 @@
       <c r="E250" t="s">
         <v>977</v>
       </c>
-      <c r="F250" s="2">
+      <c r="F250" s="1">
         <v>46063</v>
       </c>
       <c r="G250" t="s">
@@ -13419,7 +13393,7 @@
       <c r="E251" t="s">
         <v>978</v>
       </c>
-      <c r="F251" s="2">
+      <c r="F251" s="1">
         <v>46063</v>
       </c>
       <c r="G251" t="s">
@@ -13454,7 +13428,7 @@
       <c r="E252" t="s">
         <v>979</v>
       </c>
-      <c r="F252" s="2">
+      <c r="F252" s="1">
         <v>46063</v>
       </c>
       <c r="G252" t="s">
@@ -13489,7 +13463,7 @@
       <c r="E253" t="s">
         <v>980</v>
       </c>
-      <c r="F253" s="2">
+      <c r="F253" s="1">
         <v>46063</v>
       </c>
       <c r="G253" t="s">
@@ -13527,7 +13501,7 @@
       <c r="E254" t="s">
         <v>981</v>
       </c>
-      <c r="F254" s="2">
+      <c r="F254" s="1">
         <v>46063</v>
       </c>
       <c r="G254" t="s">
@@ -13565,7 +13539,7 @@
       <c r="E255" t="s">
         <v>982</v>
       </c>
-      <c r="F255" s="2">
+      <c r="F255" s="1">
         <v>46063</v>
       </c>
       <c r="G255" t="s">
@@ -13603,7 +13577,7 @@
       <c r="E256" t="s">
         <v>983</v>
       </c>
-      <c r="F256" s="2">
+      <c r="F256" s="1">
         <v>46063</v>
       </c>
       <c r="G256" t="s">
@@ -13644,7 +13618,7 @@
       <c r="E257" t="s">
         <v>984</v>
       </c>
-      <c r="F257" s="2">
+      <c r="F257" s="1">
         <v>46063</v>
       </c>
       <c r="G257" t="s">
@@ -13673,7 +13647,7 @@
       <c r="E258" t="s">
         <v>985</v>
       </c>
-      <c r="F258" s="2">
+      <c r="F258" s="1">
         <v>46063</v>
       </c>
       <c r="G258" t="s">
@@ -13702,7 +13676,7 @@
       <c r="E259" t="s">
         <v>986</v>
       </c>
-      <c r="F259" s="2">
+      <c r="F259" s="1">
         <v>46063</v>
       </c>
       <c r="G259" t="s">
@@ -13740,7 +13714,7 @@
       <c r="E260" t="s">
         <v>987</v>
       </c>
-      <c r="F260" s="2">
+      <c r="F260" s="1">
         <v>46063</v>
       </c>
       <c r="G260" t="s">
@@ -13778,7 +13752,7 @@
       <c r="E261" t="s">
         <v>988</v>
       </c>
-      <c r="F261" s="2">
+      <c r="F261" s="1">
         <v>46063</v>
       </c>
       <c r="G261" t="s">
@@ -13816,7 +13790,7 @@
       <c r="E262" t="s">
         <v>989</v>
       </c>
-      <c r="F262" s="2">
+      <c r="F262" s="1">
         <v>46063</v>
       </c>
       <c r="G262" t="s">
@@ -13834,7 +13808,7 @@
       <c r="K262" t="s">
         <v>1223</v>
       </c>
-      <c r="M262" s="2">
+      <c r="M262" s="1">
         <v>46113</v>
       </c>
       <c r="O262" t="s">
@@ -13860,7 +13834,7 @@
       <c r="E263" t="s">
         <v>990</v>
       </c>
-      <c r="F263" s="2">
+      <c r="F263" s="1">
         <v>46063</v>
       </c>
       <c r="G263" t="s">
@@ -13895,7 +13869,7 @@
       <c r="E264" t="s">
         <v>991</v>
       </c>
-      <c r="F264" s="2">
+      <c r="F264" s="1">
         <v>46063</v>
       </c>
       <c r="G264" t="s">
@@ -13933,7 +13907,7 @@
       <c r="E265" t="s">
         <v>992</v>
       </c>
-      <c r="F265" s="2">
+      <c r="F265" s="1">
         <v>46063</v>
       </c>
       <c r="G265" t="s">
@@ -13971,7 +13945,7 @@
       <c r="E266" t="s">
         <v>993</v>
       </c>
-      <c r="F266" s="2">
+      <c r="F266" s="1">
         <v>46063</v>
       </c>
       <c r="G266" t="s">
@@ -14009,7 +13983,7 @@
       <c r="E267" t="s">
         <v>994</v>
       </c>
-      <c r="F267" s="2">
+      <c r="F267" s="1">
         <v>46063</v>
       </c>
       <c r="G267" t="s">
@@ -14047,7 +14021,7 @@
       <c r="E268" t="s">
         <v>995</v>
       </c>
-      <c r="F268" s="2">
+      <c r="F268" s="1">
         <v>46063</v>
       </c>
       <c r="G268" t="s">
@@ -14082,7 +14056,7 @@
       <c r="D269" t="s">
         <v>711</v>
       </c>
-      <c r="F269" s="2">
+      <c r="F269" s="1">
         <v>46063</v>
       </c>
       <c r="G269" t="s">
@@ -14120,7 +14094,7 @@
       <c r="E270" t="s">
         <v>996</v>
       </c>
-      <c r="F270" s="2">
+      <c r="F270" s="1">
         <v>46063</v>
       </c>
       <c r="G270" t="s">
@@ -14158,7 +14132,7 @@
       <c r="E271" t="s">
         <v>997</v>
       </c>
-      <c r="F271" s="2">
+      <c r="F271" s="1">
         <v>46063</v>
       </c>
       <c r="G271" t="s">
@@ -14196,7 +14170,7 @@
       <c r="E272" t="s">
         <v>998</v>
       </c>
-      <c r="F272" s="2">
+      <c r="F272" s="1">
         <v>46063</v>
       </c>
       <c r="G272" t="s">
@@ -14214,7 +14188,7 @@
       <c r="K272" t="s">
         <v>1225</v>
       </c>
-      <c r="M272" s="2">
+      <c r="M272" s="1">
         <v>46185</v>
       </c>
       <c r="N272" t="s">
@@ -14240,7 +14214,7 @@
       <c r="E273" t="s">
         <v>999</v>
       </c>
-      <c r="F273" s="2">
+      <c r="F273" s="1">
         <v>46063</v>
       </c>
       <c r="G273" t="s">
@@ -14275,7 +14249,7 @@
       <c r="E274" t="s">
         <v>1000</v>
       </c>
-      <c r="F274" s="2">
+      <c r="F274" s="1">
         <v>46063</v>
       </c>
       <c r="G274" t="s">
@@ -14313,7 +14287,7 @@
       <c r="E275" t="s">
         <v>1001</v>
       </c>
-      <c r="F275" s="2">
+      <c r="F275" s="1">
         <v>46063</v>
       </c>
       <c r="G275" t="s">
@@ -14348,7 +14322,7 @@
       <c r="E276" t="s">
         <v>1002</v>
       </c>
-      <c r="F276" s="2">
+      <c r="F276" s="1">
         <v>46063</v>
       </c>
       <c r="G276" t="s">
@@ -14386,7 +14360,7 @@
       <c r="E277" t="s">
         <v>1003</v>
       </c>
-      <c r="F277" s="2">
+      <c r="F277" s="1">
         <v>46063</v>
       </c>
       <c r="G277" t="s">
@@ -14424,7 +14398,7 @@
       <c r="E278" t="s">
         <v>1004</v>
       </c>
-      <c r="F278" s="2">
+      <c r="F278" s="1">
         <v>46077</v>
       </c>
       <c r="G278" t="s">
@@ -14462,7 +14436,7 @@
       <c r="E279" t="s">
         <v>1005</v>
       </c>
-      <c r="F279" s="2">
+      <c r="F279" s="1">
         <v>46077</v>
       </c>
       <c r="G279" t="s">
@@ -14503,7 +14477,7 @@
       <c r="E280" t="s">
         <v>1006</v>
       </c>
-      <c r="F280" s="2">
+      <c r="F280" s="1">
         <v>46085</v>
       </c>
       <c r="G280" t="s">
@@ -14541,7 +14515,7 @@
       <c r="E281" t="s">
         <v>1007</v>
       </c>
-      <c r="F281" s="2">
+      <c r="F281" s="1">
         <v>46085</v>
       </c>
       <c r="G281" t="s">
@@ -14579,7 +14553,7 @@
       <c r="E282" t="s">
         <v>1008</v>
       </c>
-      <c r="F282" s="2">
+      <c r="F282" s="1">
         <v>46090</v>
       </c>
       <c r="G282" t="s">
@@ -14617,7 +14591,7 @@
       <c r="E283" t="s">
         <v>1009</v>
       </c>
-      <c r="F283" s="2">
+      <c r="F283" s="1">
         <v>46100</v>
       </c>
       <c r="G283" t="s">
@@ -14652,7 +14626,7 @@
       <c r="E284" t="s">
         <v>1010</v>
       </c>
-      <c r="F284" s="2">
+      <c r="F284" s="1">
         <v>46100</v>
       </c>
       <c r="G284" t="s">
@@ -14687,7 +14661,7 @@
       <c r="E285" t="s">
         <v>1011</v>
       </c>
-      <c r="F285" s="2">
+      <c r="F285" s="1">
         <v>46100</v>
       </c>
       <c r="G285" t="s">
@@ -14722,7 +14696,7 @@
       <c r="E286" t="s">
         <v>1012</v>
       </c>
-      <c r="F286" s="2">
+      <c r="F286" s="1">
         <v>46100</v>
       </c>
       <c r="G286" t="s">
@@ -14757,7 +14731,7 @@
       <c r="E287">
         <v>35971</v>
       </c>
-      <c r="F287" s="2">
+      <c r="F287" s="1">
         <v>46107</v>
       </c>
       <c r="G287" t="s">
@@ -14786,7 +14760,7 @@
       <c r="E288">
         <v>107178</v>
       </c>
-      <c r="F288" s="2">
+      <c r="F288" s="1">
         <v>46107</v>
       </c>
       <c r="G288" t="s">
@@ -14824,7 +14798,7 @@
       <c r="E289">
         <v>108773</v>
       </c>
-      <c r="F289" s="2">
+      <c r="F289" s="1">
         <v>46107</v>
       </c>
       <c r="G289" t="s">
@@ -14853,7 +14827,7 @@
       <c r="E290">
         <v>7086</v>
       </c>
-      <c r="F290" s="2">
+      <c r="F290" s="1">
         <v>46107</v>
       </c>
       <c r="G290" t="s">
@@ -14868,7 +14842,7 @@
       <c r="J290" t="s">
         <v>1145</v>
       </c>
-      <c r="M290" s="2">
+      <c r="M290" s="1">
         <v>46127</v>
       </c>
       <c r="P290" t="b">
@@ -14891,7 +14865,7 @@
       <c r="E291">
         <v>99743</v>
       </c>
-      <c r="F291" s="2">
+      <c r="F291" s="1">
         <v>46107</v>
       </c>
       <c r="G291" t="s">
@@ -14929,7 +14903,7 @@
       <c r="E292" t="s">
         <v>1013</v>
       </c>
-      <c r="F292" s="2">
+      <c r="F292" s="1">
         <v>46112</v>
       </c>
       <c r="G292" t="s">
@@ -14967,7 +14941,7 @@
       <c r="E293" t="s">
         <v>1014</v>
       </c>
-      <c r="F293" s="2">
+      <c r="F293" s="1">
         <v>46125</v>
       </c>
       <c r="G293" t="s">
@@ -15005,7 +14979,7 @@
       <c r="E294" t="s">
         <v>1015</v>
       </c>
-      <c r="F294" s="2">
+      <c r="F294" s="1">
         <v>46125</v>
       </c>
       <c r="G294" t="s">
@@ -15040,7 +15014,7 @@
       <c r="E295" t="s">
         <v>1016</v>
       </c>
-      <c r="F295" s="2">
+      <c r="F295" s="1">
         <v>46125</v>
       </c>
       <c r="G295" t="s">
@@ -15075,7 +15049,7 @@
       <c r="E296" t="s">
         <v>1017</v>
       </c>
-      <c r="F296" s="2">
+      <c r="F296" s="1">
         <v>46125</v>
       </c>
       <c r="G296" t="s">
@@ -15110,7 +15084,7 @@
       <c r="E297">
         <v>47203152</v>
       </c>
-      <c r="F297" s="2">
+      <c r="F297" s="1">
         <v>46125</v>
       </c>
       <c r="G297" t="s">
@@ -15145,7 +15119,7 @@
       <c r="E298">
         <v>47202512</v>
       </c>
-      <c r="F298" s="2">
+      <c r="F298" s="1">
         <v>46125</v>
       </c>
       <c r="G298" t="s">
@@ -15183,7 +15157,7 @@
       <c r="E299">
         <v>22005580</v>
       </c>
-      <c r="F299" s="2">
+      <c r="F299" s="1">
         <v>46125</v>
       </c>
       <c r="G299" t="s">
@@ -15221,7 +15195,7 @@
       <c r="E300">
         <v>22005955</v>
       </c>
-      <c r="F300" s="2">
+      <c r="F300" s="1">
         <v>46125</v>
       </c>
       <c r="G300" t="s">
@@ -15259,7 +15233,7 @@
       <c r="E301">
         <v>22005661</v>
       </c>
-      <c r="F301" s="2">
+      <c r="F301" s="1">
         <v>46125</v>
       </c>
       <c r="G301" t="s">
@@ -15297,7 +15271,7 @@
       <c r="E302">
         <v>32207</v>
       </c>
-      <c r="F302" s="2">
+      <c r="F302" s="1">
         <v>46125</v>
       </c>
       <c r="G302" t="s">
@@ -15335,7 +15309,7 @@
       <c r="E303">
         <v>18156</v>
       </c>
-      <c r="F303" s="2">
+      <c r="F303" s="1">
         <v>46125</v>
       </c>
       <c r="G303" t="s">
@@ -15373,7 +15347,7 @@
       <c r="E304">
         <v>37971</v>
       </c>
-      <c r="F304" s="2">
+      <c r="F304" s="1">
         <v>46125</v>
       </c>
       <c r="G304" t="s">
@@ -15411,7 +15385,7 @@
       <c r="E305">
         <v>84317</v>
       </c>
-      <c r="F305" s="2">
+      <c r="F305" s="1">
         <v>46125</v>
       </c>
       <c r="G305" t="s">
@@ -15429,7 +15403,7 @@
       <c r="K305" t="s">
         <v>1230</v>
       </c>
-      <c r="M305" s="2">
+      <c r="M305" s="1">
         <v>46160</v>
       </c>
       <c r="P305" t="b">
@@ -15452,7 +15426,7 @@
       <c r="E306">
         <v>83773</v>
       </c>
-      <c r="F306" s="2">
+      <c r="F306" s="1">
         <v>46125</v>
       </c>
       <c r="G306" t="s">
@@ -15470,7 +15444,7 @@
       <c r="K306" t="s">
         <v>1231</v>
       </c>
-      <c r="M306" s="2">
+      <c r="M306" s="1">
         <v>46156</v>
       </c>
       <c r="P306" t="b">
@@ -15493,7 +15467,7 @@
       <c r="E307">
         <v>83740</v>
       </c>
-      <c r="F307" s="2">
+      <c r="F307" s="1">
         <v>46125</v>
       </c>
       <c r="G307" t="s">
@@ -15531,7 +15505,7 @@
       <c r="E308">
         <v>84326</v>
       </c>
-      <c r="F308" s="2">
+      <c r="F308" s="1">
         <v>46125</v>
       </c>
       <c r="G308" t="s">
@@ -15569,7 +15543,7 @@
       <c r="E309">
         <v>6708</v>
       </c>
-      <c r="F309" s="2">
+      <c r="F309" s="1">
         <v>46125</v>
       </c>
       <c r="G309" t="s">
@@ -15607,7 +15581,7 @@
       <c r="E310" t="s">
         <v>1018</v>
       </c>
-      <c r="F310" s="2">
+      <c r="F310" s="1">
         <v>46125</v>
       </c>
       <c r="G310" t="s">
@@ -15645,7 +15619,7 @@
       <c r="E311">
         <v>9727</v>
       </c>
-      <c r="F311" s="2">
+      <c r="F311" s="1">
         <v>46125</v>
       </c>
       <c r="G311" t="s">
@@ -15683,7 +15657,7 @@
       <c r="E312" t="s">
         <v>1019</v>
       </c>
-      <c r="F312" s="2">
+      <c r="F312" s="1">
         <v>46125</v>
       </c>
       <c r="G312" t="s">
@@ -15721,7 +15695,7 @@
       <c r="E313">
         <v>31</v>
       </c>
-      <c r="F313" s="2">
+      <c r="F313" s="1">
         <v>46125</v>
       </c>
       <c r="G313" t="s">
@@ -15756,7 +15730,7 @@
       <c r="E314">
         <v>965</v>
       </c>
-      <c r="F314" s="2">
+      <c r="F314" s="1">
         <v>46125</v>
       </c>
       <c r="G314" t="s">
@@ -15794,7 +15768,7 @@
       <c r="E315">
         <v>2007</v>
       </c>
-      <c r="F315" s="2">
+      <c r="F315" s="1">
         <v>46125</v>
       </c>
       <c r="G315" t="s">
@@ -15832,7 +15806,7 @@
       <c r="E316">
         <v>688</v>
       </c>
-      <c r="F316" s="2">
+      <c r="F316" s="1">
         <v>46125</v>
       </c>
       <c r="G316" t="s">
@@ -15870,7 +15844,7 @@
       <c r="E317" t="s">
         <v>1020</v>
       </c>
-      <c r="F317" s="2">
+      <c r="F317" s="1">
         <v>46125</v>
       </c>
       <c r="G317" t="s">
@@ -15908,7 +15882,7 @@
       <c r="E318" t="s">
         <v>1021</v>
       </c>
-      <c r="F318" s="2">
+      <c r="F318" s="1">
         <v>46125</v>
       </c>
       <c r="G318" t="s">
@@ -15937,7 +15911,7 @@
       <c r="E319" t="s">
         <v>1022</v>
       </c>
-      <c r="F319" s="2">
+      <c r="F319" s="1">
         <v>46125</v>
       </c>
       <c r="G319" t="s">
@@ -15952,7 +15926,7 @@
       <c r="K319" t="s">
         <v>1232</v>
       </c>
-      <c r="M319" s="2">
+      <c r="M319" s="1">
         <v>46175</v>
       </c>
       <c r="P319" t="b">
@@ -15975,7 +15949,7 @@
       <c r="E320">
         <v>1391</v>
       </c>
-      <c r="F320" s="2">
+      <c r="F320" s="1">
         <v>46125</v>
       </c>
       <c r="G320" t="s">
@@ -16013,7 +15987,7 @@
       <c r="E321">
         <v>120315</v>
       </c>
-      <c r="F321" s="2">
+      <c r="F321" s="1">
         <v>46125</v>
       </c>
       <c r="G321" t="s">
@@ -16051,7 +16025,7 @@
       <c r="E322" t="s">
         <v>1023</v>
       </c>
-      <c r="F322" s="2">
+      <c r="F322" s="1">
         <v>46125</v>
       </c>
       <c r="G322" t="s">
@@ -16069,7 +16043,7 @@
       <c r="K322" t="s">
         <v>1233</v>
       </c>
-      <c r="M322" s="2">
+      <c r="M322" s="1">
         <v>46182</v>
       </c>
       <c r="P322" t="b">
@@ -16092,7 +16066,7 @@
       <c r="E323">
         <v>535933</v>
       </c>
-      <c r="F323" s="2">
+      <c r="F323" s="1">
         <v>46125</v>
       </c>
       <c r="G323" t="s">
@@ -16130,7 +16104,7 @@
       <c r="E324">
         <v>289029</v>
       </c>
-      <c r="F324" s="2">
+      <c r="F324" s="1">
         <v>46125</v>
       </c>
       <c r="G324" t="s">
@@ -16168,7 +16142,7 @@
       <c r="E325">
         <v>3454</v>
       </c>
-      <c r="F325" s="2">
+      <c r="F325" s="1">
         <v>46125</v>
       </c>
       <c r="G325" t="s">
@@ -16186,7 +16160,7 @@
       <c r="K325" t="s">
         <v>1233</v>
       </c>
-      <c r="M325" s="2">
+      <c r="M325" s="1">
         <v>46182</v>
       </c>
       <c r="P325" t="b">
@@ -16209,7 +16183,7 @@
       <c r="E326">
         <v>3493</v>
       </c>
-      <c r="F326" s="2">
+      <c r="F326" s="1">
         <v>46125</v>
       </c>
       <c r="G326" t="s">
@@ -16247,7 +16221,7 @@
       <c r="E327" t="s">
         <v>1023</v>
       </c>
-      <c r="F327" s="2">
+      <c r="F327" s="1">
         <v>46125</v>
       </c>
       <c r="G327" t="s">
@@ -16265,7 +16239,7 @@
       <c r="K327" t="s">
         <v>1233</v>
       </c>
-      <c r="M327" s="2">
+      <c r="M327" s="1">
         <v>46182</v>
       </c>
       <c r="P327" t="b">
@@ -16288,7 +16262,7 @@
       <c r="E328">
         <v>3235</v>
       </c>
-      <c r="F328" s="2">
+      <c r="F328" s="1">
         <v>46125</v>
       </c>
       <c r="G328" t="s">
@@ -16306,7 +16280,7 @@
       <c r="K328" t="s">
         <v>1233</v>
       </c>
-      <c r="M328" s="2">
+      <c r="M328" s="1">
         <v>46182</v>
       </c>
       <c r="P328" t="b">
@@ -16329,7 +16303,7 @@
       <c r="E329">
         <v>625052</v>
       </c>
-      <c r="F329" s="2">
+      <c r="F329" s="1">
         <v>46125</v>
       </c>
       <c r="G329" t="s">
@@ -16347,7 +16321,7 @@
       <c r="K329" t="s">
         <v>1233</v>
       </c>
-      <c r="M329" s="2">
+      <c r="M329" s="1">
         <v>46182</v>
       </c>
       <c r="P329" t="b">
@@ -16370,7 +16344,7 @@
       <c r="E330">
         <v>614095</v>
       </c>
-      <c r="F330" s="2">
+      <c r="F330" s="1">
         <v>46125</v>
       </c>
       <c r="G330" t="s">
@@ -16388,7 +16362,7 @@
       <c r="K330" t="s">
         <v>1233</v>
       </c>
-      <c r="M330" s="2">
+      <c r="M330" s="1">
         <v>46182</v>
       </c>
       <c r="P330" t="b">
@@ -16411,7 +16385,7 @@
       <c r="E331" t="s">
         <v>965</v>
       </c>
-      <c r="F331" s="2">
+      <c r="F331" s="1">
         <v>46125</v>
       </c>
       <c r="G331" t="s">
@@ -16449,7 +16423,7 @@
       <c r="E332" t="s">
         <v>1024</v>
       </c>
-      <c r="F332" s="2">
+      <c r="F332" s="1">
         <v>46125</v>
       </c>
       <c r="G332" t="s">
@@ -16487,7 +16461,7 @@
       <c r="E333">
         <v>197</v>
       </c>
-      <c r="F333" s="2">
+      <c r="F333" s="1">
         <v>46125</v>
       </c>
       <c r="G333" t="s">
@@ -16525,7 +16499,7 @@
       <c r="E334">
         <v>1378</v>
       </c>
-      <c r="F334" s="2">
+      <c r="F334" s="1">
         <v>46125</v>
       </c>
       <c r="G334" t="s">
@@ -16563,7 +16537,7 @@
       <c r="E335" t="s">
         <v>1025</v>
       </c>
-      <c r="F335" s="2">
+      <c r="F335" s="1">
         <v>46127</v>
       </c>
       <c r="G335" t="s">
@@ -16578,7 +16552,7 @@
       <c r="K335" t="s">
         <v>1232</v>
       </c>
-      <c r="M335" s="2">
+      <c r="M335" s="1">
         <v>46175</v>
       </c>
       <c r="P335" t="b">
@@ -16601,7 +16575,7 @@
       <c r="E336" t="s">
         <v>1026</v>
       </c>
-      <c r="F336" s="2">
+      <c r="F336" s="1">
         <v>46127</v>
       </c>
       <c r="G336" t="s">
@@ -16639,7 +16613,7 @@
       <c r="E337" t="s">
         <v>1027</v>
       </c>
-      <c r="F337" s="2">
+      <c r="F337" s="1">
         <v>46127</v>
       </c>
       <c r="G337" t="s">
@@ -16654,7 +16628,7 @@
       <c r="K337" t="s">
         <v>1232</v>
       </c>
-      <c r="M337" s="2">
+      <c r="M337" s="1">
         <v>46175</v>
       </c>
       <c r="P337" t="b">
@@ -16677,7 +16651,7 @@
       <c r="E338" t="s">
         <v>1028</v>
       </c>
-      <c r="F338" s="2">
+      <c r="F338" s="1">
         <v>46127</v>
       </c>
       <c r="G338" t="s">
@@ -16715,7 +16689,7 @@
       <c r="E339">
         <v>6291</v>
       </c>
-      <c r="F339" s="2">
+      <c r="F339" s="1">
         <v>46129</v>
       </c>
       <c r="G339" t="s">
@@ -16744,7 +16718,7 @@
       <c r="E340" t="s">
         <v>1029</v>
       </c>
-      <c r="F340" s="2">
+      <c r="F340" s="1">
         <v>46142</v>
       </c>
       <c r="G340" t="s">
@@ -16782,7 +16756,7 @@
       <c r="E341" t="s">
         <v>1030</v>
       </c>
-      <c r="F341" s="2">
+      <c r="F341" s="1">
         <v>46142</v>
       </c>
       <c r="G341" t="s">
@@ -16820,7 +16794,7 @@
       <c r="E342" t="s">
         <v>1031</v>
       </c>
-      <c r="F342" s="2">
+      <c r="F342" s="1">
         <v>46142</v>
       </c>
       <c r="G342" t="s">
@@ -16858,7 +16832,7 @@
       <c r="E343" t="s">
         <v>1032</v>
       </c>
-      <c r="F343" s="2">
+      <c r="F343" s="1">
         <v>46142</v>
       </c>
       <c r="G343" t="s">
@@ -16896,7 +16870,7 @@
       <c r="E344" t="s">
         <v>1033</v>
       </c>
-      <c r="F344" s="2">
+      <c r="F344" s="1">
         <v>46142</v>
       </c>
       <c r="G344" t="s">
@@ -16934,7 +16908,7 @@
       <c r="E345" t="s">
         <v>1034</v>
       </c>
-      <c r="F345" s="2">
+      <c r="F345" s="1">
         <v>46142</v>
       </c>
       <c r="G345" t="s">
@@ -16972,7 +16946,7 @@
       <c r="E346" t="s">
         <v>1035</v>
       </c>
-      <c r="F346" s="2">
+      <c r="F346" s="1">
         <v>46142</v>
       </c>
       <c r="G346" t="s">
@@ -17010,7 +16984,7 @@
       <c r="E347" t="s">
         <v>1036</v>
       </c>
-      <c r="F347" s="2">
+      <c r="F347" s="1">
         <v>46142</v>
       </c>
       <c r="G347" t="s">
@@ -17028,7 +17002,7 @@
       <c r="K347" t="s">
         <v>1230</v>
       </c>
-      <c r="M347" s="2">
+      <c r="M347" s="1">
         <v>46160</v>
       </c>
       <c r="P347" t="b">
@@ -17051,7 +17025,7 @@
       <c r="E348" t="s">
         <v>1037</v>
       </c>
-      <c r="F348" s="2">
+      <c r="F348" s="1">
         <v>46142</v>
       </c>
       <c r="G348" t="s">
@@ -17069,7 +17043,7 @@
       <c r="K348" t="s">
         <v>1231</v>
       </c>
-      <c r="M348" s="2">
+      <c r="M348" s="1">
         <v>46156</v>
       </c>
       <c r="P348" t="b">
@@ -17092,7 +17066,7 @@
       <c r="E349" t="s">
         <v>1038</v>
       </c>
-      <c r="F349" s="2">
+      <c r="F349" s="1">
         <v>46142</v>
       </c>
       <c r="G349" t="s">
@@ -17130,7 +17104,7 @@
       <c r="E350" t="s">
         <v>1039</v>
       </c>
-      <c r="F350" s="2">
+      <c r="F350" s="1">
         <v>46142</v>
       </c>
       <c r="G350" t="s">
@@ -17165,7 +17139,7 @@
       <c r="E351" t="s">
         <v>1040</v>
       </c>
-      <c r="F351" s="2">
+      <c r="F351" s="1">
         <v>46142</v>
       </c>
       <c r="G351" t="s">
@@ -17203,7 +17177,7 @@
       <c r="E352" t="s">
         <v>1041</v>
       </c>
-      <c r="F352" s="2">
+      <c r="F352" s="1">
         <v>46142</v>
       </c>
       <c r="G352" t="s">
@@ -17241,7 +17215,7 @@
       <c r="E353" t="s">
         <v>1042</v>
       </c>
-      <c r="F353" s="2">
+      <c r="F353" s="1">
         <v>46142</v>
       </c>
       <c r="G353" t="s">
@@ -17279,7 +17253,7 @@
       <c r="E354" t="s">
         <v>1043</v>
       </c>
-      <c r="F354" s="2">
+      <c r="F354" s="1">
         <v>46142</v>
       </c>
       <c r="G354" t="s">
@@ -17317,7 +17291,7 @@
       <c r="E355" t="s">
         <v>1044</v>
       </c>
-      <c r="F355" s="2">
+      <c r="F355" s="1">
         <v>46142</v>
       </c>
       <c r="G355" t="s">
@@ -17335,7 +17309,7 @@
       <c r="K355" t="s">
         <v>1234</v>
       </c>
-      <c r="M355" s="2">
+      <c r="M355" s="1">
         <v>46150</v>
       </c>
       <c r="P355" t="b">
@@ -17358,7 +17332,7 @@
       <c r="E356" t="s">
         <v>1045</v>
       </c>
-      <c r="F356" s="2">
+      <c r="F356" s="1">
         <v>46142</v>
       </c>
       <c r="G356" t="s">
@@ -17373,7 +17347,7 @@
       <c r="K356" t="s">
         <v>1235</v>
       </c>
-      <c r="M356" s="2">
+      <c r="M356" s="1">
         <v>46176</v>
       </c>
       <c r="P356" t="b">
@@ -17396,7 +17370,7 @@
       <c r="E357" t="s">
         <v>1046</v>
       </c>
-      <c r="F357" s="2">
+      <c r="F357" s="1">
         <v>46142</v>
       </c>
       <c r="G357" t="s">
@@ -17434,7 +17408,7 @@
       <c r="E358" t="s">
         <v>1047</v>
       </c>
-      <c r="F358" s="2">
+      <c r="F358" s="1">
         <v>46142</v>
       </c>
       <c r="G358" t="s">
@@ -17472,7 +17446,7 @@
       <c r="E359" t="s">
         <v>1048</v>
       </c>
-      <c r="F359" s="2">
+      <c r="F359" s="1">
         <v>46142</v>
       </c>
       <c r="G359" t="s">
@@ -17513,7 +17487,7 @@
       <c r="E360" t="s">
         <v>857</v>
       </c>
-      <c r="F360" s="2">
+      <c r="F360" s="1">
         <v>46142</v>
       </c>
       <c r="G360" t="s">
@@ -17551,7 +17525,7 @@
       <c r="E361" t="s">
         <v>869</v>
       </c>
-      <c r="F361" s="2">
+      <c r="F361" s="1">
         <v>46142</v>
       </c>
       <c r="G361" t="s">
@@ -17589,7 +17563,7 @@
       <c r="E362" t="s">
         <v>1049</v>
       </c>
-      <c r="F362" s="2">
+      <c r="F362" s="1">
         <v>46142</v>
       </c>
       <c r="G362" t="s">
@@ -17627,7 +17601,7 @@
       <c r="E363" t="s">
         <v>1050</v>
       </c>
-      <c r="F363" s="2">
+      <c r="F363" s="1">
         <v>46142</v>
       </c>
       <c r="G363" t="s">
@@ -17665,7 +17639,7 @@
       <c r="E364" t="s">
         <v>866</v>
       </c>
-      <c r="F364" s="2">
+      <c r="F364" s="1">
         <v>46142</v>
       </c>
       <c r="G364" t="s">
@@ -17703,7 +17677,7 @@
       <c r="E365" t="s">
         <v>1051</v>
       </c>
-      <c r="F365" s="2">
+      <c r="F365" s="1">
         <v>46142</v>
       </c>
       <c r="G365" t="s">
@@ -17741,7 +17715,7 @@
       <c r="E366" t="s">
         <v>1052</v>
       </c>
-      <c r="F366" s="2">
+      <c r="F366" s="1">
         <v>46148</v>
       </c>
       <c r="G366" t="s">
@@ -17779,7 +17753,7 @@
       <c r="E367" t="s">
         <v>1053</v>
       </c>
-      <c r="F367" s="2">
+      <c r="F367" s="1">
         <v>46148</v>
       </c>
       <c r="G367" t="s">
@@ -17817,7 +17791,7 @@
       <c r="E368" t="s">
         <v>1054</v>
       </c>
-      <c r="F368" s="2">
+      <c r="F368" s="1">
         <v>46148</v>
       </c>
       <c r="G368" t="s">
@@ -17855,7 +17829,7 @@
       <c r="E369" t="s">
         <v>1055</v>
       </c>
-      <c r="F369" s="2">
+      <c r="F369" s="1">
         <v>46148</v>
       </c>
       <c r="G369" t="s">
@@ -17893,7 +17867,7 @@
       <c r="E370" t="s">
         <v>1056</v>
       </c>
-      <c r="F370" s="2">
+      <c r="F370" s="1">
         <v>46148</v>
       </c>
       <c r="G370" t="s">
@@ -17931,7 +17905,7 @@
       <c r="E371" t="s">
         <v>1057</v>
       </c>
-      <c r="F371" s="2">
+      <c r="F371" s="1">
         <v>46148</v>
       </c>
       <c r="G371" t="s">
@@ -17949,7 +17923,7 @@
       <c r="K371" t="s">
         <v>1236</v>
       </c>
-      <c r="M371" s="2">
+      <c r="M371" s="1">
         <v>46164</v>
       </c>
       <c r="P371" t="b">
@@ -17972,7 +17946,7 @@
       <c r="E372" t="s">
         <v>1058</v>
       </c>
-      <c r="F372" s="2">
+      <c r="F372" s="1">
         <v>46148</v>
       </c>
       <c r="G372" t="s">
@@ -17990,7 +17964,7 @@
       <c r="K372" t="s">
         <v>1223</v>
       </c>
-      <c r="M372" s="2">
+      <c r="M372" s="1">
         <v>46113</v>
       </c>
       <c r="O372" t="s">
@@ -18016,7 +17990,7 @@
       <c r="E373" t="s">
         <v>1059</v>
       </c>
-      <c r="F373" s="2">
+      <c r="F373" s="1">
         <v>46149</v>
       </c>
       <c r="G373" t="s">
@@ -18054,7 +18028,7 @@
       <c r="E374" t="s">
         <v>1060</v>
       </c>
-      <c r="F374" s="2">
+      <c r="F374" s="1">
         <v>46149</v>
       </c>
       <c r="G374" t="s">
@@ -18092,7 +18066,7 @@
       <c r="E375" t="s">
         <v>1061</v>
       </c>
-      <c r="F375" s="2">
+      <c r="F375" s="1">
         <v>46154</v>
       </c>
       <c r="G375" t="s">
@@ -18130,7 +18104,7 @@
       <c r="E376" t="s">
         <v>1062</v>
       </c>
-      <c r="F376" s="2">
+      <c r="F376" s="1">
         <v>46154</v>
       </c>
       <c r="G376" t="s">
@@ -18168,7 +18142,7 @@
       <c r="E377" t="s">
         <v>1063</v>
       </c>
-      <c r="F377" s="2">
+      <c r="F377" s="1">
         <v>46154</v>
       </c>
       <c r="G377" t="s">
@@ -18206,7 +18180,7 @@
       <c r="E378" t="s">
         <v>1064</v>
       </c>
-      <c r="F378" s="2">
+      <c r="F378" s="1">
         <v>46154</v>
       </c>
       <c r="G378" t="s">
@@ -18244,7 +18218,7 @@
       <c r="E379" t="s">
         <v>1065</v>
       </c>
-      <c r="F379" s="2">
+      <c r="F379" s="1">
         <v>46154</v>
       </c>
       <c r="G379" t="s">
@@ -18262,7 +18236,7 @@
       <c r="K379" t="s">
         <v>1237</v>
       </c>
-      <c r="M379" s="2">
+      <c r="M379" s="1">
         <v>46174</v>
       </c>
       <c r="P379" t="b">
@@ -18285,7 +18259,7 @@
       <c r="E380" t="s">
         <v>1066</v>
       </c>
-      <c r="F380" s="2">
+      <c r="F380" s="1">
         <v>46154</v>
       </c>
       <c r="G380" t="s">
@@ -18323,7 +18297,7 @@
       <c r="E381" t="s">
         <v>1067</v>
       </c>
-      <c r="F381" s="2">
+      <c r="F381" s="1">
         <v>46154</v>
       </c>
       <c r="G381" t="s">
@@ -18361,7 +18335,7 @@
       <c r="E382" t="s">
         <v>1068</v>
       </c>
-      <c r="F382" s="2">
+      <c r="F382" s="1">
         <v>46154</v>
       </c>
       <c r="G382" t="s">
@@ -18399,7 +18373,7 @@
       <c r="E383" t="s">
         <v>1069</v>
       </c>
-      <c r="F383" s="2">
+      <c r="F383" s="1">
         <v>46154</v>
       </c>
       <c r="G383" t="s">
@@ -18437,7 +18411,7 @@
       <c r="E384" t="s">
         <v>1070</v>
       </c>
-      <c r="F384" s="2">
+      <c r="F384" s="1">
         <v>46164</v>
       </c>
       <c r="G384" t="s">
@@ -18475,7 +18449,7 @@
       <c r="E385" t="s">
         <v>1071</v>
       </c>
-      <c r="F385" s="2">
+      <c r="F385" s="1">
         <v>46164</v>
       </c>
       <c r="G385" t="s">
@@ -18513,7 +18487,7 @@
       <c r="E386" t="s">
         <v>1072</v>
       </c>
-      <c r="F386" s="2">
+      <c r="F386" s="1">
         <v>46171</v>
       </c>
       <c r="G386" t="s">
@@ -18551,7 +18525,7 @@
       <c r="E387" t="s">
         <v>1073</v>
       </c>
-      <c r="F387" s="2">
+      <c r="F387" s="1">
         <v>46171</v>
       </c>
       <c r="G387" t="s">
@@ -18589,7 +18563,7 @@
       <c r="E388" t="s">
         <v>759</v>
       </c>
-      <c r="F388" s="2">
+      <c r="F388" s="1">
         <v>46171</v>
       </c>
       <c r="G388" t="s">
@@ -18627,7 +18601,7 @@
       <c r="E389" t="s">
         <v>1074</v>
       </c>
-      <c r="F389" s="2">
+      <c r="F389" s="1">
         <v>46171</v>
       </c>
       <c r="G389" t="s">
@@ -18665,7 +18639,7 @@
       <c r="E390" t="s">
         <v>1075</v>
       </c>
-      <c r="F390" s="2">
+      <c r="F390" s="1">
         <v>46171</v>
       </c>
       <c r="G390" t="s">
@@ -18683,7 +18657,7 @@
       <c r="K390" t="s">
         <v>1238</v>
       </c>
-      <c r="M390" s="2">
+      <c r="M390" s="1">
         <v>46191</v>
       </c>
       <c r="P390" t="b">
@@ -18706,7 +18680,7 @@
       <c r="E391" t="s">
         <v>1076</v>
       </c>
-      <c r="F391" s="2">
+      <c r="F391" s="1">
         <v>46171</v>
       </c>
       <c r="G391" t="s">
@@ -18744,7 +18718,7 @@
       <c r="E392" t="s">
         <v>1077</v>
       </c>
-      <c r="F392" s="2">
+      <c r="F392" s="1">
         <v>46171</v>
       </c>
       <c r="G392" t="s">
@@ -18759,7 +18733,7 @@
       <c r="K392" t="s">
         <v>1235</v>
       </c>
-      <c r="M392" s="2">
+      <c r="M392" s="1">
         <v>46176</v>
       </c>
       <c r="P392" t="b">
@@ -18782,7 +18756,7 @@
       <c r="E393" t="s">
         <v>1078</v>
       </c>
-      <c r="F393" s="2">
+      <c r="F393" s="1">
         <v>46171</v>
       </c>
       <c r="G393" t="s">
@@ -18820,7 +18794,7 @@
       <c r="E394" t="s">
         <v>1079</v>
       </c>
-      <c r="F394" s="2">
+      <c r="F394" s="1">
         <v>46171</v>
       </c>
       <c r="G394" t="s">
@@ -18858,7 +18832,7 @@
       <c r="E395" t="s">
         <v>1080</v>
       </c>
-      <c r="F395" s="2">
+      <c r="F395" s="1">
         <v>46171</v>
       </c>
       <c r="G395" t="s">
@@ -18896,7 +18870,7 @@
       <c r="E396" t="s">
         <v>1081</v>
       </c>
-      <c r="F396" s="2">
+      <c r="F396" s="1">
         <v>46171</v>
       </c>
       <c r="G396" t="s">
@@ -18934,7 +18908,7 @@
       <c r="E397" t="s">
         <v>1082</v>
       </c>
-      <c r="F397" s="2">
+      <c r="F397" s="1">
         <v>46171</v>
       </c>
       <c r="G397" t="s">
@@ -18972,7 +18946,7 @@
       <c r="E398" t="s">
         <v>1083</v>
       </c>
-      <c r="F398" s="2">
+      <c r="F398" s="1">
         <v>46171</v>
       </c>
       <c r="G398" t="s">
@@ -19010,7 +18984,7 @@
       <c r="E399" t="s">
         <v>895</v>
       </c>
-      <c r="F399" s="2">
+      <c r="F399" s="1">
         <v>46163</v>
       </c>
       <c r="G399" t="s">
@@ -19025,7 +18999,7 @@
       <c r="K399" t="s">
         <v>1239</v>
       </c>
-      <c r="M399" s="2">
+      <c r="M399" s="1">
         <v>46171</v>
       </c>
       <c r="P399" t="b">
@@ -19048,7 +19022,7 @@
       <c r="E400" t="s">
         <v>1084</v>
       </c>
-      <c r="F400" s="2">
+      <c r="F400" s="1">
         <v>46171</v>
       </c>
       <c r="G400" t="s">
@@ -19086,7 +19060,7 @@
       <c r="E401" t="s">
         <v>1085</v>
       </c>
-      <c r="F401" s="2">
+      <c r="F401" s="1">
         <v>46171</v>
       </c>
       <c r="G401" t="s">
@@ -19124,7 +19098,7 @@
       <c r="E402" t="s">
         <v>1086</v>
       </c>
-      <c r="F402" s="2">
+      <c r="F402" s="1">
         <v>46171</v>
       </c>
       <c r="G402" t="s">
@@ -19162,7 +19136,7 @@
       <c r="E403" t="s">
         <v>1087</v>
       </c>
-      <c r="F403" s="2">
+      <c r="F403" s="1">
         <v>46171</v>
       </c>
       <c r="G403" t="s">
@@ -19197,7 +19171,7 @@
       <c r="E404" t="s">
         <v>1088</v>
       </c>
-      <c r="F404" s="2">
+      <c r="F404" s="1">
         <v>46171</v>
       </c>
       <c r="G404" t="s">
@@ -19232,7 +19206,7 @@
       <c r="E405">
         <v>9599</v>
       </c>
-      <c r="F405" s="2">
+      <c r="F405" s="1">
         <v>46183</v>
       </c>
       <c r="G405" t="s">
@@ -19261,7 +19235,7 @@
       <c r="E406">
         <v>14251</v>
       </c>
-      <c r="F406" s="2">
+      <c r="F406" s="1">
         <v>46183</v>
       </c>
       <c r="G406" t="s">
@@ -19293,7 +19267,7 @@
       <c r="E407">
         <v>19945</v>
       </c>
-      <c r="F407" s="2">
+      <c r="F407" s="1">
         <v>46183</v>
       </c>
       <c r="G407" t="s">
@@ -19325,7 +19299,7 @@
       <c r="E408">
         <v>14396</v>
       </c>
-      <c r="F408" s="2">
+      <c r="F408" s="1">
         <v>46183</v>
       </c>
       <c r="G408" t="s">
@@ -19357,7 +19331,7 @@
       <c r="E409">
         <v>9920</v>
       </c>
-      <c r="F409" s="2">
+      <c r="F409" s="1">
         <v>46183</v>
       </c>
       <c r="G409" t="s">
@@ -19389,7 +19363,7 @@
       <c r="E410">
         <v>20528</v>
       </c>
-      <c r="F410" s="2">
+      <c r="F410" s="1">
         <v>46183</v>
       </c>
       <c r="G410" t="s">
@@ -19421,7 +19395,7 @@
       <c r="E411" t="s">
         <v>1089</v>
       </c>
-      <c r="F411" s="2">
+      <c r="F411" s="1">
         <v>46188</v>
       </c>
       <c r="G411" t="s">
@@ -19453,7 +19427,7 @@
       <c r="E412" t="s">
         <v>1090</v>
       </c>
-      <c r="F412" s="2">
+      <c r="F412" s="1">
         <v>46188</v>
       </c>
       <c r="G412" t="s">
@@ -19485,7 +19459,7 @@
       <c r="E413" t="s">
         <v>1091</v>
       </c>
-      <c r="F413" s="2">
+      <c r="F413" s="1">
         <v>46188</v>
       </c>
       <c r="G413" t="s">
@@ -19517,7 +19491,7 @@
       <c r="E414" t="s">
         <v>1092</v>
       </c>
-      <c r="F414" s="2">
+      <c r="F414" s="1">
         <v>46188</v>
       </c>
       <c r="G414" t="s">
@@ -19549,7 +19523,7 @@
       <c r="E415" t="s">
         <v>968</v>
       </c>
-      <c r="F415" s="2">
+      <c r="F415" s="1">
         <v>46188</v>
       </c>
       <c r="G415" t="s">
@@ -19581,7 +19555,7 @@
       <c r="E416">
         <v>5844</v>
       </c>
-      <c r="F416" s="2">
+      <c r="F416" s="1">
         <v>46188</v>
       </c>
       <c r="G416" t="s">
@@ -19613,7 +19587,7 @@
       <c r="E417" t="s">
         <v>1093</v>
       </c>
-      <c r="F417" s="2">
+      <c r="F417" s="1">
         <v>46188</v>
       </c>
       <c r="G417" t="s">
@@ -19645,7 +19619,7 @@
       <c r="E418" t="s">
         <v>1094</v>
       </c>
-      <c r="F418" s="2">
+      <c r="F418" s="1">
         <v>46188</v>
       </c>
       <c r="G418" t="s">
@@ -19677,7 +19651,7 @@
       <c r="E419" t="s">
         <v>1095</v>
       </c>
-      <c r="F419" s="2">
+      <c r="F419" s="1">
         <v>46188</v>
       </c>
       <c r="G419" t="s">
@@ -19709,7 +19683,7 @@
       <c r="E420">
         <v>580</v>
       </c>
-      <c r="F420" s="2">
+      <c r="F420" s="1">
         <v>46188</v>
       </c>
       <c r="G420" t="s">
@@ -19741,7 +19715,7 @@
       <c r="E421" t="s">
         <v>1096</v>
       </c>
-      <c r="F421" s="2">
+      <c r="F421" s="1">
         <v>46188</v>
       </c>
       <c r="G421" t="s">
@@ -19773,7 +19747,7 @@
       <c r="E422" t="s">
         <v>1097</v>
       </c>
-      <c r="F422" s="2">
+      <c r="F422" s="1">
         <v>46188</v>
       </c>
       <c r="G422" t="s">
@@ -19805,7 +19779,7 @@
       <c r="E423" t="s">
         <v>1098</v>
       </c>
-      <c r="F423" s="2">
+      <c r="F423" s="1">
         <v>46188</v>
       </c>
       <c r="G423" t="s">
@@ -19837,7 +19811,7 @@
       <c r="E424" t="s">
         <v>1099</v>
       </c>
-      <c r="F424" s="2">
+      <c r="F424" s="1">
         <v>46188</v>
       </c>
       <c r="G424" t="s">
@@ -19869,7 +19843,7 @@
       <c r="E425" t="s">
         <v>1100</v>
       </c>
-      <c r="F425" s="2">
+      <c r="F425" s="1">
         <v>46188</v>
       </c>
       <c r="G425" t="s">
@@ -19901,7 +19875,7 @@
       <c r="E426" t="s">
         <v>1101</v>
       </c>
-      <c r="F426" s="2">
+      <c r="F426" s="1">
         <v>46188</v>
       </c>
       <c r="G426" t="s">
@@ -19933,7 +19907,7 @@
       <c r="E427">
         <v>6309</v>
       </c>
-      <c r="F427" s="2">
+      <c r="F427" s="1">
         <v>46188</v>
       </c>
       <c r="G427" t="s">
@@ -19965,7 +19939,7 @@
       <c r="E428">
         <v>504011190625165</v>
       </c>
-      <c r="F428" s="2">
+      <c r="F428" s="1">
         <v>46188</v>
       </c>
       <c r="G428" t="s">
@@ -19997,7 +19971,7 @@
       <c r="E429">
         <v>504011190625185</v>
       </c>
-      <c r="F429" s="2">
+      <c r="F429" s="1">
         <v>46188</v>
       </c>
       <c r="G429" t="s">
@@ -20029,7 +20003,7 @@
       <c r="E430" t="s">
         <v>1102</v>
       </c>
-      <c r="F430" s="2">
+      <c r="F430" s="1">
         <v>46188</v>
       </c>
       <c r="G430" t="s">
@@ -20061,7 +20035,7 @@
       <c r="E431" t="s">
         <v>1103</v>
       </c>
-      <c r="F431" s="2">
+      <c r="F431" s="1">
         <v>46188</v>
       </c>
       <c r="G431" t="s">
@@ -20093,7 +20067,7 @@
       <c r="E432" t="s">
         <v>1104</v>
       </c>
-      <c r="F432" s="2">
+      <c r="F432" s="1">
         <v>46188</v>
       </c>
       <c r="G432" t="s">
@@ -20125,7 +20099,7 @@
       <c r="E433" t="s">
         <v>1105</v>
       </c>
-      <c r="F433" s="2">
+      <c r="F433" s="1">
         <v>46188</v>
       </c>
       <c r="G433" t="s">
@@ -20157,7 +20131,7 @@
       <c r="E434">
         <v>328</v>
       </c>
-      <c r="F434" s="2">
+      <c r="F434" s="1">
         <v>46188</v>
       </c>
       <c r="G434" t="s">
@@ -20189,7 +20163,7 @@
       <c r="E435">
         <v>277</v>
       </c>
-      <c r="F435" s="2">
+      <c r="F435" s="1">
         <v>46188</v>
       </c>
       <c r="G435" t="s">
@@ -20221,7 +20195,7 @@
       <c r="E436">
         <v>477</v>
       </c>
-      <c r="F436" s="2">
+      <c r="F436" s="1">
         <v>46188</v>
       </c>
       <c r="G436" t="s">
@@ -20253,7 +20227,7 @@
       <c r="E437">
         <v>11</v>
       </c>
-      <c r="F437" s="2">
+      <c r="F437" s="1">
         <v>46188</v>
       </c>
       <c r="G437" t="s">
@@ -20285,7 +20259,7 @@
       <c r="E438" t="s">
         <v>1106</v>
       </c>
-      <c r="F438" s="2">
+      <c r="F438" s="1">
         <v>46188</v>
       </c>
       <c r="G438" t="s">
@@ -20317,7 +20291,7 @@
       <c r="E439" t="s">
         <v>1107</v>
       </c>
-      <c r="F439" s="2">
+      <c r="F439" s="1">
         <v>46196</v>
       </c>
       <c r="G439" t="s">
@@ -20349,7 +20323,7 @@
       <c r="E440" t="s">
         <v>1108</v>
       </c>
-      <c r="F440" s="2">
+      <c r="F440" s="1">
         <v>46196</v>
       </c>
       <c r="G440" t="s">
@@ -20381,7 +20355,7 @@
       <c r="E441">
         <v>86815651</v>
       </c>
-      <c r="F441" s="2">
+      <c r="F441" s="1">
         <v>46203</v>
       </c>
       <c r="G441" t="s">
@@ -20413,7 +20387,7 @@
       <c r="E442">
         <v>86817554</v>
       </c>
-      <c r="F442" s="2">
+      <c r="F442" s="1">
         <v>46203</v>
       </c>
       <c r="G442" t="s">
@@ -20445,7 +20419,7 @@
       <c r="E443" t="s">
         <v>1109</v>
       </c>
-      <c r="F443" s="2">
+      <c r="F443" s="1">
         <v>46205</v>
       </c>
       <c r="G443" t="s">
@@ -20477,7 +20451,7 @@
       <c r="E444" t="s">
         <v>1110</v>
       </c>
-      <c r="F444" s="2">
+      <c r="F444" s="1">
         <v>46205</v>
       </c>
       <c r="G444" t="s">
@@ -20509,7 +20483,7 @@
       <c r="E445">
         <v>4134</v>
       </c>
-      <c r="F445" s="2">
+      <c r="F445" s="1">
         <v>46205</v>
       </c>
       <c r="G445" t="s">
@@ -20541,7 +20515,7 @@
       <c r="E446">
         <v>22006508</v>
       </c>
-      <c r="F446" s="2">
+      <c r="F446" s="1">
         <v>46211</v>
       </c>
       <c r="G446" t="s">
@@ -20573,7 +20547,7 @@
       <c r="E447">
         <v>22005733</v>
       </c>
-      <c r="F447" s="2">
+      <c r="F447" s="1">
         <v>46211</v>
       </c>
       <c r="G447" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis (23/07/2026 06:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (23/07/2026 11:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -3842,8 +3842,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3859,7 +3867,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -3867,12 +3875,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4172,52 +4198,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4237,7 +4263,7 @@
       <c r="E2" t="s">
         <v>737</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <v>45698</v>
       </c>
       <c r="G2" t="s">
@@ -4275,7 +4301,7 @@
       <c r="E3" t="s">
         <v>738</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>45714</v>
       </c>
       <c r="G3" t="s">
@@ -4313,7 +4339,7 @@
       <c r="E4" t="s">
         <v>739</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="2">
         <v>45714</v>
       </c>
       <c r="G4" t="s">
@@ -4351,7 +4377,7 @@
       <c r="E5" t="s">
         <v>740</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="2">
         <v>45714</v>
       </c>
       <c r="G5" t="s">
@@ -4369,7 +4395,7 @@
       <c r="K5" t="s">
         <v>1151</v>
       </c>
-      <c r="M5" s="1">
+      <c r="M5" s="2">
         <v>45993</v>
       </c>
       <c r="P5" t="b">
@@ -4392,7 +4418,7 @@
       <c r="E6" t="s">
         <v>741</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="2">
         <v>45736</v>
       </c>
       <c r="G6" t="s">
@@ -4410,7 +4436,7 @@
       <c r="K6" t="s">
         <v>1152</v>
       </c>
-      <c r="M6" s="1">
+      <c r="M6" s="2">
         <v>45889</v>
       </c>
       <c r="P6" t="b">
@@ -4433,7 +4459,7 @@
       <c r="E7" t="s">
         <v>742</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="2">
         <v>45736</v>
       </c>
       <c r="G7" t="s">
@@ -4451,7 +4477,7 @@
       <c r="K7" t="s">
         <v>1153</v>
       </c>
-      <c r="M7" s="1">
+      <c r="M7" s="2">
         <v>45848</v>
       </c>
       <c r="N7" t="s">
@@ -4477,7 +4503,7 @@
       <c r="E8" t="s">
         <v>743</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="2">
         <v>45736</v>
       </c>
       <c r="G8" t="s">
@@ -4506,7 +4532,7 @@
       <c r="E9" t="s">
         <v>744</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="2">
         <v>45736</v>
       </c>
       <c r="G9" t="s">
@@ -4524,7 +4550,7 @@
       <c r="K9" t="s">
         <v>1154</v>
       </c>
-      <c r="M9" s="1">
+      <c r="M9" s="2">
         <v>46098</v>
       </c>
       <c r="N9">
@@ -4550,7 +4576,7 @@
       <c r="E10" t="s">
         <v>745</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="2">
         <v>45736</v>
       </c>
       <c r="G10" t="s">
@@ -4568,7 +4594,7 @@
       <c r="K10" t="s">
         <v>1155</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46114</v>
       </c>
       <c r="N10" t="s">
@@ -4594,7 +4620,7 @@
       <c r="E11" t="s">
         <v>746</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="2">
         <v>45736</v>
       </c>
       <c r="G11" t="s">
@@ -4612,7 +4638,7 @@
       <c r="K11" t="s">
         <v>1153</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>45848</v>
       </c>
       <c r="N11" t="s">
@@ -4638,7 +4664,7 @@
       <c r="E12" t="s">
         <v>747</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="2">
         <v>45736</v>
       </c>
       <c r="G12" t="s">
@@ -4656,7 +4682,7 @@
       <c r="K12" t="s">
         <v>1156</v>
       </c>
-      <c r="M12" s="1">
+      <c r="M12" s="2">
         <v>45860</v>
       </c>
       <c r="P12" t="b">
@@ -4679,7 +4705,7 @@
       <c r="E13" t="s">
         <v>748</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="2">
         <v>45736</v>
       </c>
       <c r="G13" t="s">
@@ -4714,7 +4740,7 @@
       <c r="E14" t="s">
         <v>749</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="2">
         <v>45736</v>
       </c>
       <c r="G14" t="s">
@@ -4732,7 +4758,7 @@
       <c r="K14" t="s">
         <v>1157</v>
       </c>
-      <c r="M14" s="1">
+      <c r="M14" s="2">
         <v>45800</v>
       </c>
       <c r="P14" t="b">
@@ -4755,7 +4781,7 @@
       <c r="E15" t="s">
         <v>750</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15" s="2">
         <v>45736</v>
       </c>
       <c r="G15" t="s">
@@ -4793,7 +4819,7 @@
       <c r="E16" t="s">
         <v>751</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="2">
         <v>45736</v>
       </c>
       <c r="G16" t="s">
@@ -4831,7 +4857,7 @@
       <c r="E17" t="s">
         <v>752</v>
       </c>
-      <c r="F17" s="1">
+      <c r="F17" s="2">
         <v>45736</v>
       </c>
       <c r="G17" t="s">
@@ -4849,7 +4875,7 @@
       <c r="K17" t="s">
         <v>1152</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>45897</v>
       </c>
       <c r="P17" t="b">
@@ -4872,7 +4898,7 @@
       <c r="E18" t="s">
         <v>753</v>
       </c>
-      <c r="F18" s="1">
+      <c r="F18" s="2">
         <v>45736</v>
       </c>
       <c r="G18" t="s">
@@ -4890,7 +4916,7 @@
       <c r="K18" t="s">
         <v>1157</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>45802</v>
       </c>
       <c r="P18" t="b">
@@ -4913,7 +4939,7 @@
       <c r="E19" t="s">
         <v>754</v>
       </c>
-      <c r="F19" s="1">
+      <c r="F19" s="2">
         <v>45736</v>
       </c>
       <c r="G19" t="s">
@@ -4948,7 +4974,7 @@
       <c r="E20" t="s">
         <v>755</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20" s="2">
         <v>45736</v>
       </c>
       <c r="G20" t="s">
@@ -4966,7 +4992,7 @@
       <c r="K20" t="s">
         <v>1159</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46135</v>
       </c>
       <c r="P20" t="b">
@@ -4989,7 +5015,7 @@
       <c r="E21" t="s">
         <v>756</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21" s="2">
         <v>45736</v>
       </c>
       <c r="G21" t="s">
@@ -5024,7 +5050,7 @@
       <c r="E22" t="s">
         <v>757</v>
       </c>
-      <c r="F22" s="1">
+      <c r="F22" s="2">
         <v>45736</v>
       </c>
       <c r="G22" t="s">
@@ -5062,7 +5088,7 @@
       <c r="E23" t="s">
         <v>758</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F23" s="2">
         <v>45736</v>
       </c>
       <c r="G23" t="s">
@@ -5080,7 +5106,7 @@
       <c r="K23" t="s">
         <v>1161</v>
       </c>
-      <c r="M23" s="1">
+      <c r="M23" s="2">
         <v>45965</v>
       </c>
       <c r="O23" t="s">
@@ -5106,7 +5132,7 @@
       <c r="E24" t="s">
         <v>759</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F24" s="2">
         <v>45736</v>
       </c>
       <c r="G24" t="s">
@@ -5141,7 +5167,7 @@
       <c r="E25" t="s">
         <v>760</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25" s="2">
         <v>45736</v>
       </c>
       <c r="G25" t="s">
@@ -5176,7 +5202,7 @@
       <c r="E26" t="s">
         <v>761</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="2">
         <v>45736</v>
       </c>
       <c r="G26" t="s">
@@ -5194,7 +5220,7 @@
       <c r="K26" t="s">
         <v>1164</v>
       </c>
-      <c r="M26" s="1">
+      <c r="M26" s="2">
         <v>45891</v>
       </c>
       <c r="O26" t="s">
@@ -5220,7 +5246,7 @@
       <c r="E27" t="s">
         <v>762</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27" s="2">
         <v>45736</v>
       </c>
       <c r="G27" t="s">
@@ -5258,7 +5284,7 @@
       <c r="E28" t="s">
         <v>763</v>
       </c>
-      <c r="F28" s="1">
+      <c r="F28" s="2">
         <v>45736</v>
       </c>
       <c r="G28" t="s">
@@ -5287,7 +5313,7 @@
       <c r="E29" t="s">
         <v>764</v>
       </c>
-      <c r="F29" s="1">
+      <c r="F29" s="2">
         <v>45736</v>
       </c>
       <c r="G29" t="s">
@@ -5322,7 +5348,7 @@
       <c r="E30" t="s">
         <v>765</v>
       </c>
-      <c r="F30" s="1">
+      <c r="F30" s="2">
         <v>45736</v>
       </c>
       <c r="G30" t="s">
@@ -5340,7 +5366,7 @@
       <c r="K30" t="s">
         <v>1165</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>45945</v>
       </c>
       <c r="P30" t="b">
@@ -5363,7 +5389,7 @@
       <c r="E31" t="s">
         <v>766</v>
       </c>
-      <c r="F31" s="1">
+      <c r="F31" s="2">
         <v>45736</v>
       </c>
       <c r="G31" t="s">
@@ -5398,7 +5424,7 @@
       <c r="E32" t="s">
         <v>767</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F32" s="2">
         <v>45736</v>
       </c>
       <c r="G32" t="s">
@@ -5436,7 +5462,7 @@
       <c r="E33" t="s">
         <v>768</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33" s="2">
         <v>45736</v>
       </c>
       <c r="G33" t="s">
@@ -5471,7 +5497,7 @@
       <c r="E34" t="s">
         <v>769</v>
       </c>
-      <c r="F34" s="1">
+      <c r="F34" s="2">
         <v>45736</v>
       </c>
       <c r="G34" t="s">
@@ -5500,7 +5526,7 @@
       <c r="E35" t="s">
         <v>770</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35" s="2">
         <v>45736</v>
       </c>
       <c r="G35" t="s">
@@ -5529,7 +5555,7 @@
       <c r="E36" t="s">
         <v>771</v>
       </c>
-      <c r="F36" s="1">
+      <c r="F36" s="2">
         <v>45736</v>
       </c>
       <c r="G36" t="s">
@@ -5564,7 +5590,7 @@
       <c r="E37" t="s">
         <v>772</v>
       </c>
-      <c r="F37" s="1">
+      <c r="F37" s="2">
         <v>45736</v>
       </c>
       <c r="G37" t="s">
@@ -5599,7 +5625,7 @@
       <c r="E38" t="s">
         <v>752</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F38" s="2">
         <v>45736</v>
       </c>
       <c r="G38" t="s">
@@ -5631,7 +5657,7 @@
       <c r="D39" t="s">
         <v>644</v>
       </c>
-      <c r="F39" s="1">
+      <c r="F39" s="2">
         <v>45736</v>
       </c>
       <c r="G39" t="s">
@@ -5666,7 +5692,7 @@
       <c r="D40" t="s">
         <v>644</v>
       </c>
-      <c r="F40" s="1">
+      <c r="F40" s="2">
         <v>45736</v>
       </c>
       <c r="G40" t="s">
@@ -5704,7 +5730,7 @@
       <c r="E41" t="s">
         <v>773</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F41" s="2">
         <v>45736</v>
       </c>
       <c r="G41" t="s">
@@ -5739,7 +5765,7 @@
       <c r="E42" t="s">
         <v>774</v>
       </c>
-      <c r="F42" s="1">
+      <c r="F42" s="2">
         <v>45736</v>
       </c>
       <c r="G42" t="s">
@@ -5774,7 +5800,7 @@
       <c r="E43" t="s">
         <v>775</v>
       </c>
-      <c r="F43" s="1">
+      <c r="F43" s="2">
         <v>45736</v>
       </c>
       <c r="G43" t="s">
@@ -5809,7 +5835,7 @@
       <c r="E44" t="s">
         <v>776</v>
       </c>
-      <c r="F44" s="1">
+      <c r="F44" s="2">
         <v>45769</v>
       </c>
       <c r="G44" t="s">
@@ -5827,7 +5853,7 @@
       <c r="K44" t="s">
         <v>1168</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>45856</v>
       </c>
       <c r="O44" t="s">
@@ -5853,7 +5879,7 @@
       <c r="E45" t="s">
         <v>777</v>
       </c>
-      <c r="F45" s="1">
+      <c r="F45" s="2">
         <v>45769</v>
       </c>
       <c r="G45" t="s">
@@ -5871,7 +5897,7 @@
       <c r="K45" t="s">
         <v>1169</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46100</v>
       </c>
       <c r="N45">
@@ -5897,7 +5923,7 @@
       <c r="E46" t="s">
         <v>778</v>
       </c>
-      <c r="F46" s="1">
+      <c r="F46" s="2">
         <v>45769</v>
       </c>
       <c r="G46" t="s">
@@ -5935,7 +5961,7 @@
       <c r="E47" t="s">
         <v>779</v>
       </c>
-      <c r="F47" s="1">
+      <c r="F47" s="2">
         <v>45769</v>
       </c>
       <c r="G47" t="s">
@@ -5953,7 +5979,7 @@
       <c r="K47" t="s">
         <v>1170</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46113</v>
       </c>
       <c r="O47" t="s">
@@ -5979,7 +6005,7 @@
       <c r="E48" t="s">
         <v>780</v>
       </c>
-      <c r="F48" s="1">
+      <c r="F48" s="2">
         <v>45769</v>
       </c>
       <c r="G48" t="s">
@@ -6017,7 +6043,7 @@
       <c r="E49" t="s">
         <v>781</v>
       </c>
-      <c r="F49" s="1">
+      <c r="F49" s="2">
         <v>45769</v>
       </c>
       <c r="G49" t="s">
@@ -6046,7 +6072,7 @@
       <c r="E50" t="s">
         <v>782</v>
       </c>
-      <c r="F50" s="1">
+      <c r="F50" s="2">
         <v>45769</v>
       </c>
       <c r="G50" t="s">
@@ -6084,7 +6110,7 @@
       <c r="E51" t="s">
         <v>783</v>
       </c>
-      <c r="F51" s="1">
+      <c r="F51" s="2">
         <v>45769</v>
       </c>
       <c r="G51" t="s">
@@ -6119,7 +6145,7 @@
       <c r="E52" t="s">
         <v>784</v>
       </c>
-      <c r="F52" s="1">
+      <c r="F52" s="2">
         <v>45769</v>
       </c>
       <c r="G52" t="s">
@@ -6157,7 +6183,7 @@
       <c r="E53" t="s">
         <v>785</v>
       </c>
-      <c r="F53" s="1">
+      <c r="F53" s="2">
         <v>45769</v>
       </c>
       <c r="G53" t="s">
@@ -6195,7 +6221,7 @@
       <c r="E54" t="s">
         <v>786</v>
       </c>
-      <c r="F54" s="1">
+      <c r="F54" s="2">
         <v>45769</v>
       </c>
       <c r="G54" t="s">
@@ -6233,7 +6259,7 @@
       <c r="E55" t="s">
         <v>787</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55" s="2">
         <v>45769</v>
       </c>
       <c r="G55" t="s">
@@ -6262,7 +6288,7 @@
       <c r="E56" t="s">
         <v>788</v>
       </c>
-      <c r="F56" s="1">
+      <c r="F56" s="2">
         <v>45769</v>
       </c>
       <c r="G56" t="s">
@@ -6297,7 +6323,7 @@
       <c r="E57" t="s">
         <v>789</v>
       </c>
-      <c r="F57" s="1">
+      <c r="F57" s="2">
         <v>45769</v>
       </c>
       <c r="G57" t="s">
@@ -6335,7 +6361,7 @@
       <c r="E58" t="s">
         <v>790</v>
       </c>
-      <c r="F58" s="1">
+      <c r="F58" s="2">
         <v>45769</v>
       </c>
       <c r="G58" t="s">
@@ -6364,7 +6390,7 @@
       <c r="E59" t="s">
         <v>791</v>
       </c>
-      <c r="F59" s="1">
+      <c r="F59" s="2">
         <v>45769</v>
       </c>
       <c r="G59" t="s">
@@ -6399,7 +6425,7 @@
       <c r="E60" t="s">
         <v>792</v>
       </c>
-      <c r="F60" s="1">
+      <c r="F60" s="2">
         <v>45769</v>
       </c>
       <c r="G60" t="s">
@@ -6434,7 +6460,7 @@
       <c r="E61" t="s">
         <v>793</v>
       </c>
-      <c r="F61" s="1">
+      <c r="F61" s="2">
         <v>45769</v>
       </c>
       <c r="G61" t="s">
@@ -6466,7 +6492,7 @@
       <c r="E62" t="s">
         <v>794</v>
       </c>
-      <c r="F62" s="1">
+      <c r="F62" s="2">
         <v>45770</v>
       </c>
       <c r="G62" t="s">
@@ -6495,7 +6521,7 @@
       <c r="E63" t="s">
         <v>795</v>
       </c>
-      <c r="F63" s="1">
+      <c r="F63" s="2">
         <v>45799</v>
       </c>
       <c r="G63" t="s">
@@ -6513,7 +6539,7 @@
       <c r="K63" t="s">
         <v>1173</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46092</v>
       </c>
       <c r="O63" t="s">
@@ -6539,7 +6565,7 @@
       <c r="E64" t="s">
         <v>796</v>
       </c>
-      <c r="F64" s="1">
+      <c r="F64" s="2">
         <v>45799</v>
       </c>
       <c r="G64" t="s">
@@ -6557,7 +6583,7 @@
       <c r="K64" t="s">
         <v>1174</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46119</v>
       </c>
       <c r="P64" t="b">
@@ -6580,7 +6606,7 @@
       <c r="E65" t="s">
         <v>797</v>
       </c>
-      <c r="F65" s="1">
+      <c r="F65" s="2">
         <v>45799</v>
       </c>
       <c r="G65" t="s">
@@ -6615,7 +6641,7 @@
       <c r="E66" t="s">
         <v>798</v>
       </c>
-      <c r="F66" s="1">
+      <c r="F66" s="2">
         <v>45799</v>
       </c>
       <c r="G66" t="s">
@@ -6650,7 +6676,7 @@
       <c r="E67" t="s">
         <v>799</v>
       </c>
-      <c r="F67" s="1">
+      <c r="F67" s="2">
         <v>45799</v>
       </c>
       <c r="G67" t="s">
@@ -6685,7 +6711,7 @@
       <c r="E68" t="s">
         <v>800</v>
       </c>
-      <c r="F68" s="1">
+      <c r="F68" s="2">
         <v>45799</v>
       </c>
       <c r="G68" t="s">
@@ -6720,7 +6746,7 @@
       <c r="E69" t="s">
         <v>801</v>
       </c>
-      <c r="F69" s="1">
+      <c r="F69" s="2">
         <v>45803</v>
       </c>
       <c r="G69" t="s">
@@ -6755,7 +6781,7 @@
       <c r="E70" t="s">
         <v>802</v>
       </c>
-      <c r="F70" s="1">
+      <c r="F70" s="2">
         <v>45803</v>
       </c>
       <c r="G70" t="s">
@@ -6793,7 +6819,7 @@
       <c r="E71" t="s">
         <v>803</v>
       </c>
-      <c r="F71" s="1">
+      <c r="F71" s="2">
         <v>45803</v>
       </c>
       <c r="G71" t="s">
@@ -6828,7 +6854,7 @@
       <c r="E72" t="s">
         <v>804</v>
       </c>
-      <c r="F72" s="1">
+      <c r="F72" s="2">
         <v>45803</v>
       </c>
       <c r="G72" t="s">
@@ -6863,7 +6889,7 @@
       <c r="E73" t="s">
         <v>805</v>
       </c>
-      <c r="F73" s="1">
+      <c r="F73" s="2">
         <v>45803</v>
       </c>
       <c r="G73" t="s">
@@ -6901,7 +6927,7 @@
       <c r="E74" t="s">
         <v>804</v>
       </c>
-      <c r="F74" s="1">
+      <c r="F74" s="2">
         <v>45803</v>
       </c>
       <c r="G74" t="s">
@@ -6936,7 +6962,7 @@
       <c r="E75" t="s">
         <v>806</v>
       </c>
-      <c r="F75" s="1">
+      <c r="F75" s="2">
         <v>45803</v>
       </c>
       <c r="G75" t="s">
@@ -6974,7 +7000,7 @@
       <c r="E76" t="s">
         <v>807</v>
       </c>
-      <c r="F76" s="1">
+      <c r="F76" s="2">
         <v>45803</v>
       </c>
       <c r="G76" t="s">
@@ -7009,7 +7035,7 @@
       <c r="E77" t="s">
         <v>808</v>
       </c>
-      <c r="F77" s="1">
+      <c r="F77" s="2">
         <v>45803</v>
       </c>
       <c r="G77" t="s">
@@ -7044,7 +7070,7 @@
       <c r="E78" t="s">
         <v>809</v>
       </c>
-      <c r="F78" s="1">
+      <c r="F78" s="2">
         <v>45803</v>
       </c>
       <c r="G78" t="s">
@@ -7079,7 +7105,7 @@
       <c r="E79" t="s">
         <v>810</v>
       </c>
-      <c r="F79" s="1">
+      <c r="F79" s="2">
         <v>45803</v>
       </c>
       <c r="G79" t="s">
@@ -7114,7 +7140,7 @@
       <c r="E80" t="s">
         <v>811</v>
       </c>
-      <c r="F80" s="1">
+      <c r="F80" s="2">
         <v>45803</v>
       </c>
       <c r="G80" t="s">
@@ -7152,7 +7178,7 @@
       <c r="E81" t="s">
         <v>812</v>
       </c>
-      <c r="F81" s="1">
+      <c r="F81" s="2">
         <v>45813</v>
       </c>
       <c r="G81" t="s">
@@ -7187,7 +7213,7 @@
       <c r="E82" t="s">
         <v>813</v>
       </c>
-      <c r="F82" s="1">
+      <c r="F82" s="2">
         <v>45813</v>
       </c>
       <c r="G82" t="s">
@@ -7225,7 +7251,7 @@
       <c r="E83" t="s">
         <v>814</v>
       </c>
-      <c r="F83" s="1">
+      <c r="F83" s="2">
         <v>45813</v>
       </c>
       <c r="G83" t="s">
@@ -7260,7 +7286,7 @@
       <c r="E84" t="s">
         <v>815</v>
       </c>
-      <c r="F84" s="1">
+      <c r="F84" s="2">
         <v>45813</v>
       </c>
       <c r="G84" t="s">
@@ -7278,7 +7304,7 @@
       <c r="K84" t="s">
         <v>1178</v>
       </c>
-      <c r="M84" s="1">
+      <c r="M84" s="2">
         <v>45853</v>
       </c>
       <c r="N84">
@@ -7304,7 +7330,7 @@
       <c r="E85" t="s">
         <v>816</v>
       </c>
-      <c r="F85" s="1">
+      <c r="F85" s="2">
         <v>45813</v>
       </c>
       <c r="G85" t="s">
@@ -7342,7 +7368,7 @@
       <c r="E86" t="s">
         <v>817</v>
       </c>
-      <c r="F86" s="1">
+      <c r="F86" s="2">
         <v>45813</v>
       </c>
       <c r="G86" t="s">
@@ -7380,7 +7406,7 @@
       <c r="E87" t="s">
         <v>818</v>
       </c>
-      <c r="F87" s="1">
+      <c r="F87" s="2">
         <v>45813</v>
       </c>
       <c r="G87" t="s">
@@ -7398,7 +7424,7 @@
       <c r="K87" t="s">
         <v>1179</v>
       </c>
-      <c r="M87" s="1">
+      <c r="M87" s="2">
         <v>45797</v>
       </c>
       <c r="N87" t="s">
@@ -7424,7 +7450,7 @@
       <c r="E88" t="s">
         <v>819</v>
       </c>
-      <c r="F88" s="1">
+      <c r="F88" s="2">
         <v>45813</v>
       </c>
       <c r="G88" t="s">
@@ -7459,7 +7485,7 @@
       <c r="E89" t="s">
         <v>820</v>
       </c>
-      <c r="F89" s="1">
+      <c r="F89" s="2">
         <v>45813</v>
       </c>
       <c r="G89" t="s">
@@ -7494,7 +7520,7 @@
       <c r="E90" t="s">
         <v>821</v>
       </c>
-      <c r="F90" s="1">
+      <c r="F90" s="2">
         <v>45831</v>
       </c>
       <c r="G90" t="s">
@@ -7535,7 +7561,7 @@
       <c r="E91" t="s">
         <v>822</v>
       </c>
-      <c r="F91" s="1">
+      <c r="F91" s="2">
         <v>45831</v>
       </c>
       <c r="G91" t="s">
@@ -7570,7 +7596,7 @@
       <c r="D92" t="s">
         <v>661</v>
       </c>
-      <c r="F92" s="1">
+      <c r="F92" s="2">
         <v>45831</v>
       </c>
       <c r="G92" t="s">
@@ -7599,7 +7625,7 @@
       <c r="E93" t="s">
         <v>823</v>
       </c>
-      <c r="F93" s="1">
+      <c r="F93" s="2">
         <v>45831</v>
       </c>
       <c r="G93" t="s">
@@ -7637,7 +7663,7 @@
       <c r="E94" t="s">
         <v>824</v>
       </c>
-      <c r="F94" s="1">
+      <c r="F94" s="2">
         <v>45831</v>
       </c>
       <c r="G94" t="s">
@@ -7675,7 +7701,7 @@
       <c r="E95" t="s">
         <v>825</v>
       </c>
-      <c r="F95" s="1">
+      <c r="F95" s="2">
         <v>45831</v>
       </c>
       <c r="G95" t="s">
@@ -7713,7 +7739,7 @@
       <c r="E96" t="s">
         <v>826</v>
       </c>
-      <c r="F96" s="1">
+      <c r="F96" s="2">
         <v>45831</v>
       </c>
       <c r="G96" t="s">
@@ -7731,7 +7757,7 @@
       <c r="K96" t="s">
         <v>1153</v>
       </c>
-      <c r="M96" s="1">
+      <c r="M96" s="2">
         <v>45848</v>
       </c>
       <c r="N96" t="s">
@@ -7757,7 +7783,7 @@
       <c r="E97" t="s">
         <v>827</v>
       </c>
-      <c r="F97" s="1">
+      <c r="F97" s="2">
         <v>45840</v>
       </c>
       <c r="G97" t="s">
@@ -7798,7 +7824,7 @@
       <c r="E98" t="s">
         <v>828</v>
       </c>
-      <c r="F98" s="1">
+      <c r="F98" s="2">
         <v>45840</v>
       </c>
       <c r="G98" t="s">
@@ -7836,7 +7862,7 @@
       <c r="E99" t="s">
         <v>829</v>
       </c>
-      <c r="F99" s="1">
+      <c r="F99" s="2">
         <v>45840</v>
       </c>
       <c r="G99" t="s">
@@ -7865,7 +7891,7 @@
       <c r="E100" t="s">
         <v>830</v>
       </c>
-      <c r="F100" s="1">
+      <c r="F100" s="2">
         <v>45840</v>
       </c>
       <c r="G100" t="s">
@@ -7903,7 +7929,7 @@
       <c r="E101" t="s">
         <v>831</v>
       </c>
-      <c r="F101" s="1">
+      <c r="F101" s="2">
         <v>45840</v>
       </c>
       <c r="G101" t="s">
@@ -7932,7 +7958,7 @@
       <c r="E102" t="s">
         <v>832</v>
       </c>
-      <c r="F102" s="1">
+      <c r="F102" s="2">
         <v>45840</v>
       </c>
       <c r="G102" t="s">
@@ -7961,7 +7987,7 @@
       <c r="E103" t="s">
         <v>833</v>
       </c>
-      <c r="F103" s="1">
+      <c r="F103" s="2">
         <v>45840</v>
       </c>
       <c r="G103" t="s">
@@ -7990,7 +8016,7 @@
       <c r="E104" t="s">
         <v>834</v>
       </c>
-      <c r="F104" s="1">
+      <c r="F104" s="2">
         <v>45840</v>
       </c>
       <c r="G104" t="s">
@@ -8028,7 +8054,7 @@
       <c r="E105" t="s">
         <v>835</v>
       </c>
-      <c r="F105" s="1">
+      <c r="F105" s="2">
         <v>45840</v>
       </c>
       <c r="G105" t="s">
@@ -8066,7 +8092,7 @@
       <c r="E106" t="s">
         <v>836</v>
       </c>
-      <c r="F106" s="1">
+      <c r="F106" s="2">
         <v>45840</v>
       </c>
       <c r="G106" t="s">
@@ -8084,7 +8110,7 @@
       <c r="K106" t="s">
         <v>1182</v>
       </c>
-      <c r="M106" s="1">
+      <c r="M106" s="2">
         <v>45889</v>
       </c>
       <c r="P106" t="b">
@@ -8107,7 +8133,7 @@
       <c r="E107" t="s">
         <v>837</v>
       </c>
-      <c r="F107" s="1">
+      <c r="F107" s="2">
         <v>45840</v>
       </c>
       <c r="G107" t="s">
@@ -8125,7 +8151,7 @@
       <c r="K107" t="s">
         <v>1183</v>
       </c>
-      <c r="M107" s="1">
+      <c r="M107" s="2">
         <v>45876</v>
       </c>
       <c r="P107" t="b">
@@ -8148,7 +8174,7 @@
       <c r="E108" t="s">
         <v>838</v>
       </c>
-      <c r="F108" s="1">
+      <c r="F108" s="2">
         <v>45840</v>
       </c>
       <c r="G108" t="s">
@@ -8186,7 +8212,7 @@
       <c r="E109" t="s">
         <v>839</v>
       </c>
-      <c r="F109" s="1">
+      <c r="F109" s="2">
         <v>45840</v>
       </c>
       <c r="G109" t="s">
@@ -8224,7 +8250,7 @@
       <c r="E110" t="s">
         <v>840</v>
       </c>
-      <c r="F110" s="1">
+      <c r="F110" s="2">
         <v>45840</v>
       </c>
       <c r="G110" t="s">
@@ -8259,7 +8285,7 @@
       <c r="E111" t="s">
         <v>841</v>
       </c>
-      <c r="F111" s="1">
+      <c r="F111" s="2">
         <v>45840</v>
       </c>
       <c r="G111" t="s">
@@ -8294,7 +8320,7 @@
       <c r="E112" t="s">
         <v>842</v>
       </c>
-      <c r="F112" s="1">
+      <c r="F112" s="2">
         <v>45840</v>
       </c>
       <c r="G112" t="s">
@@ -8323,7 +8349,7 @@
       <c r="E113" t="s">
         <v>843</v>
       </c>
-      <c r="F113" s="1">
+      <c r="F113" s="2">
         <v>45840</v>
       </c>
       <c r="G113" t="s">
@@ -8358,7 +8384,7 @@
       <c r="E114" t="s">
         <v>844</v>
       </c>
-      <c r="F114" s="1">
+      <c r="F114" s="2">
         <v>45840</v>
       </c>
       <c r="G114" t="s">
@@ -8393,7 +8419,7 @@
       <c r="E115" t="s">
         <v>845</v>
       </c>
-      <c r="F115" s="1">
+      <c r="F115" s="2">
         <v>45840</v>
       </c>
       <c r="G115" t="s">
@@ -8431,7 +8457,7 @@
       <c r="E116" t="s">
         <v>846</v>
       </c>
-      <c r="F116" s="1">
+      <c r="F116" s="2">
         <v>45840</v>
       </c>
       <c r="G116" t="s">
@@ -8469,7 +8495,7 @@
       <c r="E117" t="s">
         <v>847</v>
       </c>
-      <c r="F117" s="1">
+      <c r="F117" s="2">
         <v>45840</v>
       </c>
       <c r="G117" t="s">
@@ -8507,7 +8533,7 @@
       <c r="E118" t="s">
         <v>848</v>
       </c>
-      <c r="F118" s="1">
+      <c r="F118" s="2">
         <v>45840</v>
       </c>
       <c r="G118" t="s">
@@ -8545,7 +8571,7 @@
       <c r="E119" t="s">
         <v>849</v>
       </c>
-      <c r="F119" s="1">
+      <c r="F119" s="2">
         <v>45840</v>
       </c>
       <c r="G119" t="s">
@@ -8583,7 +8609,7 @@
       <c r="E120" t="s">
         <v>850</v>
       </c>
-      <c r="F120" s="1">
+      <c r="F120" s="2">
         <v>45840</v>
       </c>
       <c r="G120" t="s">
@@ -8621,7 +8647,7 @@
       <c r="E121" t="s">
         <v>851</v>
       </c>
-      <c r="F121" s="1">
+      <c r="F121" s="2">
         <v>45849</v>
       </c>
       <c r="G121" t="s">
@@ -8639,7 +8665,7 @@
       <c r="K121" t="s">
         <v>1169</v>
       </c>
-      <c r="M121" s="1">
+      <c r="M121" s="2">
         <v>46100</v>
       </c>
       <c r="N121">
@@ -8665,7 +8691,7 @@
       <c r="E122" t="s">
         <v>852</v>
       </c>
-      <c r="F122" s="1">
+      <c r="F122" s="2">
         <v>45849</v>
       </c>
       <c r="G122" t="s">
@@ -8703,7 +8729,7 @@
       <c r="E123" t="s">
         <v>853</v>
       </c>
-      <c r="F123" s="1">
+      <c r="F123" s="2">
         <v>45849</v>
       </c>
       <c r="G123" t="s">
@@ -8732,7 +8758,7 @@
       <c r="E124" t="s">
         <v>854</v>
       </c>
-      <c r="F124" s="1">
+      <c r="F124" s="2">
         <v>45853</v>
       </c>
       <c r="G124" t="s">
@@ -8770,7 +8796,7 @@
       <c r="E125" t="s">
         <v>855</v>
       </c>
-      <c r="F125" s="1">
+      <c r="F125" s="2">
         <v>45855</v>
       </c>
       <c r="G125" t="s">
@@ -8808,7 +8834,7 @@
       <c r="E126" t="s">
         <v>856</v>
       </c>
-      <c r="F126" s="1">
+      <c r="F126" s="2">
         <v>45855</v>
       </c>
       <c r="G126" t="s">
@@ -8843,7 +8869,7 @@
       <c r="E127" t="s">
         <v>857</v>
       </c>
-      <c r="F127" s="1">
+      <c r="F127" s="2">
         <v>45856</v>
       </c>
       <c r="G127" t="s">
@@ -8872,7 +8898,7 @@
       <c r="E128" t="s">
         <v>858</v>
       </c>
-      <c r="F128" s="1">
+      <c r="F128" s="2">
         <v>45869</v>
       </c>
       <c r="G128" t="s">
@@ -8910,7 +8936,7 @@
       <c r="E129" t="s">
         <v>859</v>
       </c>
-      <c r="F129" s="1">
+      <c r="F129" s="2">
         <v>45869</v>
       </c>
       <c r="G129" t="s">
@@ -8948,7 +8974,7 @@
       <c r="E130" t="s">
         <v>860</v>
       </c>
-      <c r="F130" s="1">
+      <c r="F130" s="2">
         <v>45869</v>
       </c>
       <c r="G130" t="s">
@@ -8966,7 +8992,7 @@
       <c r="K130" t="s">
         <v>1187</v>
       </c>
-      <c r="M130" s="1">
+      <c r="M130" s="2">
         <v>45916</v>
       </c>
       <c r="N130">
@@ -8992,7 +9018,7 @@
       <c r="E131" t="s">
         <v>861</v>
       </c>
-      <c r="F131" s="1">
+      <c r="F131" s="2">
         <v>45869</v>
       </c>
       <c r="G131" t="s">
@@ -9027,7 +9053,7 @@
       <c r="E132" t="s">
         <v>862</v>
       </c>
-      <c r="F132" s="1">
+      <c r="F132" s="2">
         <v>45869</v>
       </c>
       <c r="G132" t="s">
@@ -9045,7 +9071,7 @@
       <c r="K132" t="s">
         <v>1189</v>
       </c>
-      <c r="M132" s="1">
+      <c r="M132" s="2">
         <v>46014</v>
       </c>
       <c r="N132">
@@ -9071,7 +9097,7 @@
       <c r="E133" t="s">
         <v>863</v>
       </c>
-      <c r="F133" s="1">
+      <c r="F133" s="2">
         <v>45869</v>
       </c>
       <c r="G133" t="s">
@@ -9100,7 +9126,7 @@
       <c r="E134" t="s">
         <v>864</v>
       </c>
-      <c r="F134" s="1">
+      <c r="F134" s="2">
         <v>45882</v>
       </c>
       <c r="G134" t="s">
@@ -9138,7 +9164,7 @@
       <c r="E135" t="s">
         <v>865</v>
       </c>
-      <c r="F135" s="1">
+      <c r="F135" s="2">
         <v>45882</v>
       </c>
       <c r="G135" t="s">
@@ -9167,7 +9193,7 @@
       <c r="E136" t="s">
         <v>866</v>
       </c>
-      <c r="F136" s="1">
+      <c r="F136" s="2">
         <v>45891</v>
       </c>
       <c r="G136" t="s">
@@ -9196,7 +9222,7 @@
       <c r="E137" t="s">
         <v>867</v>
       </c>
-      <c r="F137" s="1">
+      <c r="F137" s="2">
         <v>45891</v>
       </c>
       <c r="G137" t="s">
@@ -9225,7 +9251,7 @@
       <c r="E138" t="s">
         <v>868</v>
       </c>
-      <c r="F138" s="1">
+      <c r="F138" s="2">
         <v>45891</v>
       </c>
       <c r="G138" t="s">
@@ -9263,7 +9289,7 @@
       <c r="E139" t="s">
         <v>869</v>
       </c>
-      <c r="F139" s="1">
+      <c r="F139" s="2">
         <v>45891</v>
       </c>
       <c r="G139" t="s">
@@ -9292,7 +9318,7 @@
       <c r="E140" t="s">
         <v>870</v>
       </c>
-      <c r="F140" s="1">
+      <c r="F140" s="2">
         <v>45891</v>
       </c>
       <c r="G140" t="s">
@@ -9327,7 +9353,7 @@
       <c r="E141" t="s">
         <v>871</v>
       </c>
-      <c r="F141" s="1">
+      <c r="F141" s="2">
         <v>45891</v>
       </c>
       <c r="G141" t="s">
@@ -9356,7 +9382,7 @@
       <c r="E142" t="s">
         <v>872</v>
       </c>
-      <c r="F142" s="1">
+      <c r="F142" s="2">
         <v>45891</v>
       </c>
       <c r="G142" t="s">
@@ -9385,7 +9411,7 @@
       <c r="E143" t="s">
         <v>873</v>
       </c>
-      <c r="F143" s="1">
+      <c r="F143" s="2">
         <v>45891</v>
       </c>
       <c r="G143" t="s">
@@ -9414,7 +9440,7 @@
       <c r="E144" t="s">
         <v>874</v>
       </c>
-      <c r="F144" s="1">
+      <c r="F144" s="2">
         <v>45891</v>
       </c>
       <c r="G144" t="s">
@@ -9443,7 +9469,7 @@
       <c r="E145" t="s">
         <v>875</v>
       </c>
-      <c r="F145" s="1">
+      <c r="F145" s="2">
         <v>45891</v>
       </c>
       <c r="G145" t="s">
@@ -9478,7 +9504,7 @@
       <c r="E146" t="s">
         <v>876</v>
       </c>
-      <c r="F146" s="1">
+      <c r="F146" s="2">
         <v>45891</v>
       </c>
       <c r="G146" t="s">
@@ -9507,7 +9533,7 @@
       <c r="E147" t="s">
         <v>877</v>
       </c>
-      <c r="F147" s="1">
+      <c r="F147" s="2">
         <v>45891</v>
       </c>
       <c r="G147" t="s">
@@ -9542,7 +9568,7 @@
       <c r="E148" t="s">
         <v>878</v>
       </c>
-      <c r="F148" s="1">
+      <c r="F148" s="2">
         <v>45891</v>
       </c>
       <c r="G148" t="s">
@@ -9580,7 +9606,7 @@
       <c r="E149" t="s">
         <v>879</v>
       </c>
-      <c r="F149" s="1">
+      <c r="F149" s="2">
         <v>45891</v>
       </c>
       <c r="G149" t="s">
@@ -9615,7 +9641,7 @@
       <c r="E150" t="s">
         <v>880</v>
       </c>
-      <c r="F150" s="1">
+      <c r="F150" s="2">
         <v>45891</v>
       </c>
       <c r="G150" t="s">
@@ -9633,7 +9659,7 @@
       <c r="K150" t="s">
         <v>1173</v>
       </c>
-      <c r="M150" s="1">
+      <c r="M150" s="2">
         <v>46092</v>
       </c>
       <c r="O150" t="s">
@@ -9659,7 +9685,7 @@
       <c r="E151" t="s">
         <v>881</v>
       </c>
-      <c r="F151" s="1">
+      <c r="F151" s="2">
         <v>45891</v>
       </c>
       <c r="G151" t="s">
@@ -9694,7 +9720,7 @@
       <c r="E152" t="s">
         <v>871</v>
       </c>
-      <c r="F152" s="1">
+      <c r="F152" s="2">
         <v>45891</v>
       </c>
       <c r="G152" t="s">
@@ -9712,7 +9738,7 @@
       <c r="K152" t="s">
         <v>1174</v>
       </c>
-      <c r="M152" s="1">
+      <c r="M152" s="2">
         <v>46119</v>
       </c>
       <c r="P152" t="b">
@@ -9735,7 +9761,7 @@
       <c r="E153" t="s">
         <v>882</v>
       </c>
-      <c r="F153" s="1">
+      <c r="F153" s="2">
         <v>45891</v>
       </c>
       <c r="G153" t="s">
@@ -9773,7 +9799,7 @@
       <c r="E154" t="s">
         <v>883</v>
       </c>
-      <c r="F154" s="1">
+      <c r="F154" s="2">
         <v>45891</v>
       </c>
       <c r="G154" t="s">
@@ -9808,7 +9834,7 @@
       <c r="E155" t="s">
         <v>884</v>
       </c>
-      <c r="F155" s="1">
+      <c r="F155" s="2">
         <v>45891</v>
       </c>
       <c r="G155" t="s">
@@ -9843,7 +9869,7 @@
       <c r="E156" t="s">
         <v>885</v>
       </c>
-      <c r="F156" s="1">
+      <c r="F156" s="2">
         <v>45891</v>
       </c>
       <c r="G156" t="s">
@@ -9881,7 +9907,7 @@
       <c r="E157" t="s">
         <v>886</v>
       </c>
-      <c r="F157" s="1">
+      <c r="F157" s="2">
         <v>45891</v>
       </c>
       <c r="G157" t="s">
@@ -9919,7 +9945,7 @@
       <c r="E158" t="s">
         <v>887</v>
       </c>
-      <c r="F158" s="1">
+      <c r="F158" s="2">
         <v>45894</v>
       </c>
       <c r="G158" t="s">
@@ -9937,7 +9963,7 @@
       <c r="K158" t="s">
         <v>1192</v>
       </c>
-      <c r="M158" s="1">
+      <c r="M158" s="2">
         <v>45946</v>
       </c>
       <c r="P158" t="b">
@@ -9960,7 +9986,7 @@
       <c r="E159" t="s">
         <v>888</v>
       </c>
-      <c r="F159" s="1">
+      <c r="F159" s="2">
         <v>45894</v>
       </c>
       <c r="G159" t="s">
@@ -9998,7 +10024,7 @@
       <c r="E160" t="s">
         <v>889</v>
       </c>
-      <c r="F160" s="1">
+      <c r="F160" s="2">
         <v>45898</v>
       </c>
       <c r="G160" t="s">
@@ -10036,7 +10062,7 @@
       <c r="E161" t="s">
         <v>890</v>
       </c>
-      <c r="F161" s="1">
+      <c r="F161" s="2">
         <v>45898</v>
       </c>
       <c r="G161" t="s">
@@ -10054,7 +10080,7 @@
       <c r="K161" t="s">
         <v>1193</v>
       </c>
-      <c r="M161" s="1">
+      <c r="M161" s="2">
         <v>45953</v>
       </c>
       <c r="N161" t="s">
@@ -10080,7 +10106,7 @@
       <c r="E162" t="s">
         <v>891</v>
       </c>
-      <c r="F162" s="1">
+      <c r="F162" s="2">
         <v>45898</v>
       </c>
       <c r="G162" t="s">
@@ -10098,7 +10124,7 @@
       <c r="K162" t="s">
         <v>1194</v>
       </c>
-      <c r="M162" s="1">
+      <c r="M162" s="2">
         <v>45940</v>
       </c>
       <c r="P162" t="b">
@@ -10121,7 +10147,7 @@
       <c r="E163" t="s">
         <v>892</v>
       </c>
-      <c r="F163" s="1">
+      <c r="F163" s="2">
         <v>45898</v>
       </c>
       <c r="G163" t="s">
@@ -10139,7 +10165,7 @@
       <c r="K163" t="s">
         <v>1194</v>
       </c>
-      <c r="M163" s="1">
+      <c r="M163" s="2">
         <v>45940</v>
       </c>
       <c r="P163" t="b">
@@ -10162,7 +10188,7 @@
       <c r="E164" t="s">
         <v>893</v>
       </c>
-      <c r="F164" s="1">
+      <c r="F164" s="2">
         <v>45910</v>
       </c>
       <c r="G164" t="s">
@@ -10197,7 +10223,7 @@
       <c r="E165" t="s">
         <v>894</v>
       </c>
-      <c r="F165" s="1">
+      <c r="F165" s="2">
         <v>45917</v>
       </c>
       <c r="G165" t="s">
@@ -10238,7 +10264,7 @@
       <c r="E166" t="s">
         <v>895</v>
       </c>
-      <c r="F166" s="1">
+      <c r="F166" s="2">
         <v>45917</v>
       </c>
       <c r="G166" t="s">
@@ -10273,7 +10299,7 @@
       <c r="E167" t="s">
         <v>896</v>
       </c>
-      <c r="F167" s="1">
+      <c r="F167" s="2">
         <v>45917</v>
       </c>
       <c r="G167" t="s">
@@ -10302,7 +10328,7 @@
       <c r="E168" t="s">
         <v>897</v>
       </c>
-      <c r="F168" s="1">
+      <c r="F168" s="2">
         <v>45917</v>
       </c>
       <c r="G168" t="s">
@@ -10343,7 +10369,7 @@
       <c r="E169" t="s">
         <v>898</v>
       </c>
-      <c r="F169" s="1">
+      <c r="F169" s="2">
         <v>45917</v>
       </c>
       <c r="G169" t="s">
@@ -10361,7 +10387,7 @@
       <c r="K169" t="s">
         <v>1197</v>
       </c>
-      <c r="M169" s="1">
+      <c r="M169" s="2">
         <v>45973</v>
       </c>
       <c r="P169" t="b">
@@ -10384,7 +10410,7 @@
       <c r="E170" t="s">
         <v>899</v>
       </c>
-      <c r="F170" s="1">
+      <c r="F170" s="2">
         <v>45917</v>
       </c>
       <c r="G170" t="s">
@@ -10419,7 +10445,7 @@
       <c r="E171" t="s">
         <v>900</v>
       </c>
-      <c r="F171" s="1">
+      <c r="F171" s="2">
         <v>45917</v>
       </c>
       <c r="G171" t="s">
@@ -10457,7 +10483,7 @@
       <c r="E172" t="s">
         <v>901</v>
       </c>
-      <c r="F172" s="1">
+      <c r="F172" s="2">
         <v>45917</v>
       </c>
       <c r="G172" t="s">
@@ -10492,7 +10518,7 @@
       <c r="E173" t="s">
         <v>902</v>
       </c>
-      <c r="F173" s="1">
+      <c r="F173" s="2">
         <v>45917</v>
       </c>
       <c r="G173" t="s">
@@ -10527,7 +10553,7 @@
       <c r="E174" t="s">
         <v>903</v>
       </c>
-      <c r="F174" s="1">
+      <c r="F174" s="2">
         <v>45917</v>
       </c>
       <c r="G174" t="s">
@@ -10562,7 +10588,7 @@
       <c r="E175" t="s">
         <v>904</v>
       </c>
-      <c r="F175" s="1">
+      <c r="F175" s="2">
         <v>45917</v>
       </c>
       <c r="G175" t="s">
@@ -10580,7 +10606,7 @@
       <c r="K175" t="s">
         <v>1198</v>
       </c>
-      <c r="M175" s="1">
+      <c r="M175" s="2">
         <v>46122</v>
       </c>
       <c r="O175" t="s">
@@ -10606,7 +10632,7 @@
       <c r="E176" t="s">
         <v>808</v>
       </c>
-      <c r="F176" s="1">
+      <c r="F176" s="2">
         <v>45917</v>
       </c>
       <c r="G176" t="s">
@@ -10644,7 +10670,7 @@
       <c r="E177" t="s">
         <v>905</v>
       </c>
-      <c r="F177" s="1">
+      <c r="F177" s="2">
         <v>45917</v>
       </c>
       <c r="G177" t="s">
@@ -10662,7 +10688,7 @@
       <c r="K177" t="s">
         <v>1199</v>
       </c>
-      <c r="M177" s="1">
+      <c r="M177" s="2">
         <v>45961</v>
       </c>
       <c r="O177" t="s">
@@ -10688,7 +10714,7 @@
       <c r="E178" t="s">
         <v>906</v>
       </c>
-      <c r="F178" s="1">
+      <c r="F178" s="2">
         <v>45937</v>
       </c>
       <c r="G178" t="s">
@@ -10726,7 +10752,7 @@
       <c r="E179" t="s">
         <v>907</v>
       </c>
-      <c r="F179" s="1">
+      <c r="F179" s="2">
         <v>45937</v>
       </c>
       <c r="G179" t="s">
@@ -10755,7 +10781,7 @@
       <c r="E180" t="s">
         <v>908</v>
       </c>
-      <c r="F180" s="1">
+      <c r="F180" s="2">
         <v>45937</v>
       </c>
       <c r="G180" t="s">
@@ -10793,7 +10819,7 @@
       <c r="E181" t="s">
         <v>909</v>
       </c>
-      <c r="F181" s="1">
+      <c r="F181" s="2">
         <v>45937</v>
       </c>
       <c r="G181" t="s">
@@ -10828,7 +10854,7 @@
       <c r="E182" t="s">
         <v>910</v>
       </c>
-      <c r="F182" s="1">
+      <c r="F182" s="2">
         <v>45937</v>
       </c>
       <c r="G182" t="s">
@@ -10857,7 +10883,7 @@
       <c r="E183" t="s">
         <v>911</v>
       </c>
-      <c r="F183" s="1">
+      <c r="F183" s="2">
         <v>45937</v>
       </c>
       <c r="G183" t="s">
@@ -10892,7 +10918,7 @@
       <c r="D184" t="s">
         <v>687</v>
       </c>
-      <c r="F184" s="1">
+      <c r="F184" s="2">
         <v>45939</v>
       </c>
       <c r="G184" t="s">
@@ -10927,7 +10953,7 @@
       <c r="E185" t="s">
         <v>912</v>
       </c>
-      <c r="F185" s="1">
+      <c r="F185" s="2">
         <v>45939</v>
       </c>
       <c r="G185" t="s">
@@ -10965,7 +10991,7 @@
       <c r="E186" t="s">
         <v>913</v>
       </c>
-      <c r="F186" s="1">
+      <c r="F186" s="2">
         <v>45939</v>
       </c>
       <c r="G186" t="s">
@@ -11003,7 +11029,7 @@
       <c r="E187" t="s">
         <v>914</v>
       </c>
-      <c r="F187" s="1">
+      <c r="F187" s="2">
         <v>45939</v>
       </c>
       <c r="G187" t="s">
@@ -11021,7 +11047,7 @@
       <c r="K187" t="s">
         <v>1201</v>
       </c>
-      <c r="M187" s="1">
+      <c r="M187" s="2">
         <v>46014</v>
       </c>
       <c r="N187">
@@ -11047,7 +11073,7 @@
       <c r="E188" t="s">
         <v>915</v>
       </c>
-      <c r="F188" s="1">
+      <c r="F188" s="2">
         <v>45946</v>
       </c>
       <c r="G188" t="s">
@@ -11065,7 +11091,7 @@
       <c r="K188" t="s">
         <v>1202</v>
       </c>
-      <c r="M188" s="1">
+      <c r="M188" s="2">
         <v>45986</v>
       </c>
       <c r="O188" t="s">
@@ -11091,7 +11117,7 @@
       <c r="E189" t="s">
         <v>916</v>
       </c>
-      <c r="F189" s="1">
+      <c r="F189" s="2">
         <v>45965</v>
       </c>
       <c r="G189" t="s">
@@ -11109,7 +11135,7 @@
       <c r="K189" t="s">
         <v>1203</v>
       </c>
-      <c r="M189" s="1">
+      <c r="M189" s="2">
         <v>46120</v>
       </c>
       <c r="P189" t="b">
@@ -11132,7 +11158,7 @@
       <c r="E190" t="s">
         <v>917</v>
       </c>
-      <c r="F190" s="1">
+      <c r="F190" s="2">
         <v>45965</v>
       </c>
       <c r="G190" t="s">
@@ -11170,7 +11196,7 @@
       <c r="E191" t="s">
         <v>918</v>
       </c>
-      <c r="F191" s="1">
+      <c r="F191" s="2">
         <v>45967</v>
       </c>
       <c r="G191" t="s">
@@ -11188,7 +11214,7 @@
       <c r="K191" t="s">
         <v>1204</v>
       </c>
-      <c r="M191" s="1">
+      <c r="M191" s="2">
         <v>45972</v>
       </c>
       <c r="P191" t="b">
@@ -11211,7 +11237,7 @@
       <c r="E192" t="s">
         <v>919</v>
       </c>
-      <c r="F192" s="1">
+      <c r="F192" s="2">
         <v>45968</v>
       </c>
       <c r="G192" t="s">
@@ -11249,7 +11275,7 @@
       <c r="E193" t="s">
         <v>920</v>
       </c>
-      <c r="F193" s="1">
+      <c r="F193" s="2">
         <v>45968</v>
       </c>
       <c r="G193" t="s">
@@ -11287,7 +11313,7 @@
       <c r="E194" t="s">
         <v>921</v>
       </c>
-      <c r="F194" s="1">
+      <c r="F194" s="2">
         <v>45968</v>
       </c>
       <c r="G194" t="s">
@@ -11316,7 +11342,7 @@
       <c r="E195" t="s">
         <v>922</v>
       </c>
-      <c r="F195" s="1">
+      <c r="F195" s="2">
         <v>45971</v>
       </c>
       <c r="G195" t="s">
@@ -11354,7 +11380,7 @@
       <c r="E196" t="s">
         <v>923</v>
       </c>
-      <c r="F196" s="1">
+      <c r="F196" s="2">
         <v>45978</v>
       </c>
       <c r="G196" t="s">
@@ -11383,7 +11409,7 @@
       <c r="E197" t="s">
         <v>924</v>
       </c>
-      <c r="F197" s="1">
+      <c r="F197" s="2">
         <v>45978</v>
       </c>
       <c r="G197" t="s">
@@ -11412,7 +11438,7 @@
       <c r="E198" t="s">
         <v>925</v>
       </c>
-      <c r="F198" s="1">
+      <c r="F198" s="2">
         <v>45978</v>
       </c>
       <c r="G198" t="s">
@@ -11441,7 +11467,7 @@
       <c r="E199" t="s">
         <v>926</v>
       </c>
-      <c r="F199" s="1">
+      <c r="F199" s="2">
         <v>45979</v>
       </c>
       <c r="G199" t="s">
@@ -11459,7 +11485,7 @@
       <c r="K199" t="s">
         <v>1205</v>
       </c>
-      <c r="M199" s="1">
+      <c r="M199" s="2">
         <v>46049</v>
       </c>
       <c r="P199" t="b">
@@ -11482,7 +11508,7 @@
       <c r="E200" t="s">
         <v>927</v>
       </c>
-      <c r="F200" s="1">
+      <c r="F200" s="2">
         <v>45986</v>
       </c>
       <c r="G200" t="s">
@@ -11520,7 +11546,7 @@
       <c r="E201" t="s">
         <v>928</v>
       </c>
-      <c r="F201" s="1">
+      <c r="F201" s="2">
         <v>45986</v>
       </c>
       <c r="G201" t="s">
@@ -11558,7 +11584,7 @@
       <c r="E202" t="s">
         <v>929</v>
       </c>
-      <c r="F202" s="1">
+      <c r="F202" s="2">
         <v>45986</v>
       </c>
       <c r="G202" t="s">
@@ -11596,7 +11622,7 @@
       <c r="E203" t="s">
         <v>930</v>
       </c>
-      <c r="F203" s="1">
+      <c r="F203" s="2">
         <v>45986</v>
       </c>
       <c r="G203" t="s">
@@ -11634,7 +11660,7 @@
       <c r="E204" t="s">
         <v>931</v>
       </c>
-      <c r="F204" s="1">
+      <c r="F204" s="2">
         <v>45986</v>
       </c>
       <c r="G204" t="s">
@@ -11672,7 +11698,7 @@
       <c r="E205" t="s">
         <v>932</v>
       </c>
-      <c r="F205" s="1">
+      <c r="F205" s="2">
         <v>45986</v>
       </c>
       <c r="G205" t="s">
@@ -11710,7 +11736,7 @@
       <c r="E206" t="s">
         <v>933</v>
       </c>
-      <c r="F206" s="1">
+      <c r="F206" s="2">
         <v>45986</v>
       </c>
       <c r="G206" t="s">
@@ -11745,7 +11771,7 @@
       <c r="E207" t="s">
         <v>934</v>
       </c>
-      <c r="F207" s="1">
+      <c r="F207" s="2">
         <v>45986</v>
       </c>
       <c r="G207" t="s">
@@ -11763,7 +11789,7 @@
       <c r="K207" t="s">
         <v>1207</v>
       </c>
-      <c r="M207" s="1">
+      <c r="M207" s="2">
         <v>46153</v>
       </c>
       <c r="P207" t="b">
@@ -11786,7 +11812,7 @@
       <c r="E208" t="s">
         <v>935</v>
       </c>
-      <c r="F208" s="1">
+      <c r="F208" s="2">
         <v>45986</v>
       </c>
       <c r="G208" t="s">
@@ -11804,7 +11830,7 @@
       <c r="K208" t="s">
         <v>1208</v>
       </c>
-      <c r="M208" s="1">
+      <c r="M208" s="2">
         <v>46031</v>
       </c>
       <c r="P208" t="b">
@@ -11827,7 +11853,7 @@
       <c r="E209" t="s">
         <v>936</v>
       </c>
-      <c r="F209" s="1">
+      <c r="F209" s="2">
         <v>46000</v>
       </c>
       <c r="G209" t="s">
@@ -11845,7 +11871,7 @@
       <c r="K209" t="s">
         <v>1209</v>
       </c>
-      <c r="M209" s="1">
+      <c r="M209" s="2">
         <v>46191</v>
       </c>
       <c r="P209" t="b">
@@ -11868,7 +11894,7 @@
       <c r="E210" t="s">
         <v>937</v>
       </c>
-      <c r="F210" s="1">
+      <c r="F210" s="2">
         <v>46000</v>
       </c>
       <c r="G210" t="s">
@@ -11906,7 +11932,7 @@
       <c r="E211" t="s">
         <v>938</v>
       </c>
-      <c r="F211" s="1">
+      <c r="F211" s="2">
         <v>46000</v>
       </c>
       <c r="G211" t="s">
@@ -11941,7 +11967,7 @@
       <c r="E212" t="s">
         <v>939</v>
       </c>
-      <c r="F212" s="1">
+      <c r="F212" s="2">
         <v>46000</v>
       </c>
       <c r="G212" t="s">
@@ -11976,7 +12002,7 @@
       <c r="E213" t="s">
         <v>940</v>
       </c>
-      <c r="F213" s="1">
+      <c r="F213" s="2">
         <v>46007</v>
       </c>
       <c r="G213" t="s">
@@ -12014,7 +12040,7 @@
       <c r="E214" t="s">
         <v>941</v>
       </c>
-      <c r="F214" s="1">
+      <c r="F214" s="2">
         <v>46007</v>
       </c>
       <c r="G214" t="s">
@@ -12032,7 +12058,7 @@
       <c r="K214" t="s">
         <v>1212</v>
       </c>
-      <c r="M214" s="1">
+      <c r="M214" s="2">
         <v>46021</v>
       </c>
       <c r="N214">
@@ -12058,7 +12084,7 @@
       <c r="E215" t="s">
         <v>942</v>
       </c>
-      <c r="F215" s="1">
+      <c r="F215" s="2">
         <v>46007</v>
       </c>
       <c r="G215" t="s">
@@ -12096,7 +12122,7 @@
       <c r="E216" t="s">
         <v>943</v>
       </c>
-      <c r="F216" s="1">
+      <c r="F216" s="2">
         <v>46010</v>
       </c>
       <c r="G216" t="s">
@@ -12125,7 +12151,7 @@
       <c r="E217" t="s">
         <v>944</v>
       </c>
-      <c r="F217" s="1">
+      <c r="F217" s="2">
         <v>46010</v>
       </c>
       <c r="G217" t="s">
@@ -12143,7 +12169,7 @@
       <c r="K217" t="s">
         <v>1213</v>
       </c>
-      <c r="M217" s="1">
+      <c r="M217" s="2">
         <v>46052</v>
       </c>
       <c r="P217" t="b">
@@ -12166,7 +12192,7 @@
       <c r="E218" t="s">
         <v>945</v>
       </c>
-      <c r="F218" s="1">
+      <c r="F218" s="2">
         <v>46010</v>
       </c>
       <c r="G218" t="s">
@@ -12204,7 +12230,7 @@
       <c r="E219" t="s">
         <v>946</v>
       </c>
-      <c r="F219" s="1">
+      <c r="F219" s="2">
         <v>46010</v>
       </c>
       <c r="G219" t="s">
@@ -12242,7 +12268,7 @@
       <c r="E220" t="s">
         <v>947</v>
       </c>
-      <c r="F220" s="1">
+      <c r="F220" s="2">
         <v>46010</v>
       </c>
       <c r="G220" t="s">
@@ -12280,7 +12306,7 @@
       <c r="E221" t="s">
         <v>948</v>
       </c>
-      <c r="F221" s="1">
+      <c r="F221" s="2">
         <v>46028</v>
       </c>
       <c r="G221" t="s">
@@ -12315,7 +12341,7 @@
       <c r="E222" t="s">
         <v>949</v>
       </c>
-      <c r="F222" s="1">
+      <c r="F222" s="2">
         <v>46028</v>
       </c>
       <c r="G222" t="s">
@@ -12353,7 +12379,7 @@
       <c r="E223" t="s">
         <v>950</v>
       </c>
-      <c r="F223" s="1">
+      <c r="F223" s="2">
         <v>46028</v>
       </c>
       <c r="G223" t="s">
@@ -12391,7 +12417,7 @@
       <c r="E224" t="s">
         <v>951</v>
       </c>
-      <c r="F224" s="1">
+      <c r="F224" s="2">
         <v>46028</v>
       </c>
       <c r="G224" t="s">
@@ -12429,7 +12455,7 @@
       <c r="E225" t="s">
         <v>952</v>
       </c>
-      <c r="F225" s="1">
+      <c r="F225" s="2">
         <v>46028</v>
       </c>
       <c r="G225" t="s">
@@ -12467,7 +12493,7 @@
       <c r="E226" t="s">
         <v>953</v>
       </c>
-      <c r="F226" s="1">
+      <c r="F226" s="2">
         <v>46028</v>
       </c>
       <c r="G226" t="s">
@@ -12505,7 +12531,7 @@
       <c r="E227" t="s">
         <v>954</v>
       </c>
-      <c r="F227" s="1">
+      <c r="F227" s="2">
         <v>46028</v>
       </c>
       <c r="G227" t="s">
@@ -12543,7 +12569,7 @@
       <c r="E228" t="s">
         <v>955</v>
       </c>
-      <c r="F228" s="1">
+      <c r="F228" s="2">
         <v>46028</v>
       </c>
       <c r="G228" t="s">
@@ -12581,7 +12607,7 @@
       <c r="E229" t="s">
         <v>956</v>
       </c>
-      <c r="F229" s="1">
+      <c r="F229" s="2">
         <v>46028</v>
       </c>
       <c r="G229" t="s">
@@ -12616,7 +12642,7 @@
       <c r="E230" t="s">
         <v>957</v>
       </c>
-      <c r="F230" s="1">
+      <c r="F230" s="2">
         <v>46028</v>
       </c>
       <c r="G230" t="s">
@@ -12654,7 +12680,7 @@
       <c r="E231" t="s">
         <v>958</v>
       </c>
-      <c r="F231" s="1">
+      <c r="F231" s="2">
         <v>46028</v>
       </c>
       <c r="G231" t="s">
@@ -12672,7 +12698,7 @@
       <c r="K231" t="s">
         <v>1214</v>
       </c>
-      <c r="M231" s="1">
+      <c r="M231" s="2">
         <v>46063</v>
       </c>
       <c r="P231" t="b">
@@ -12695,7 +12721,7 @@
       <c r="E232" t="s">
         <v>959</v>
       </c>
-      <c r="F232" s="1">
+      <c r="F232" s="2">
         <v>46028</v>
       </c>
       <c r="G232" t="s">
@@ -12730,7 +12756,7 @@
       <c r="E233" t="s">
         <v>960</v>
       </c>
-      <c r="F233" s="1">
+      <c r="F233" s="2">
         <v>46028</v>
       </c>
       <c r="G233" t="s">
@@ -12765,7 +12791,7 @@
       <c r="E234" t="s">
         <v>961</v>
       </c>
-      <c r="F234" s="1">
+      <c r="F234" s="2">
         <v>46028</v>
       </c>
       <c r="G234" t="s">
@@ -12783,7 +12809,7 @@
       <c r="K234" t="s">
         <v>1214</v>
       </c>
-      <c r="M234" s="1">
+      <c r="M234" s="2">
         <v>46063</v>
       </c>
       <c r="O234" t="s">
@@ -12809,7 +12835,7 @@
       <c r="E235" t="s">
         <v>962</v>
       </c>
-      <c r="F235" s="1">
+      <c r="F235" s="2">
         <v>46028</v>
       </c>
       <c r="G235" t="s">
@@ -12827,7 +12853,7 @@
       <c r="K235" t="s">
         <v>1214</v>
       </c>
-      <c r="M235" s="1">
+      <c r="M235" s="2">
         <v>46063</v>
       </c>
       <c r="O235" t="s">
@@ -12853,7 +12879,7 @@
       <c r="E236" t="s">
         <v>963</v>
       </c>
-      <c r="F236" s="1">
+      <c r="F236" s="2">
         <v>46028</v>
       </c>
       <c r="G236" t="s">
@@ -12871,7 +12897,7 @@
       <c r="K236" t="s">
         <v>1216</v>
       </c>
-      <c r="M236" s="1">
+      <c r="M236" s="2">
         <v>46114</v>
       </c>
       <c r="P236" t="b">
@@ -12894,7 +12920,7 @@
       <c r="E237" t="s">
         <v>964</v>
       </c>
-      <c r="F237" s="1">
+      <c r="F237" s="2">
         <v>46028</v>
       </c>
       <c r="G237" t="s">
@@ -12932,7 +12958,7 @@
       <c r="E238" t="s">
         <v>965</v>
       </c>
-      <c r="F238" s="1">
+      <c r="F238" s="2">
         <v>46028</v>
       </c>
       <c r="G238" t="s">
@@ -12961,7 +12987,7 @@
       <c r="E239" t="s">
         <v>966</v>
       </c>
-      <c r="F239" s="1">
+      <c r="F239" s="2">
         <v>46036</v>
       </c>
       <c r="G239" t="s">
@@ -12979,7 +13005,7 @@
       <c r="K239" t="s">
         <v>1217</v>
       </c>
-      <c r="M239" s="1">
+      <c r="M239" s="2">
         <v>46052</v>
       </c>
       <c r="P239" t="b">
@@ -13002,7 +13028,7 @@
       <c r="E240" t="s">
         <v>967</v>
       </c>
-      <c r="F240" s="1">
+      <c r="F240" s="2">
         <v>46036</v>
       </c>
       <c r="G240" t="s">
@@ -13037,7 +13063,7 @@
       <c r="E241" t="s">
         <v>968</v>
       </c>
-      <c r="F241" s="1">
+      <c r="F241" s="2">
         <v>46036</v>
       </c>
       <c r="G241" t="s">
@@ -13072,7 +13098,7 @@
       <c r="E242" t="s">
         <v>969</v>
       </c>
-      <c r="F242" s="1">
+      <c r="F242" s="2">
         <v>46036</v>
       </c>
       <c r="G242" t="s">
@@ -13110,7 +13136,7 @@
       <c r="E243" t="s">
         <v>970</v>
       </c>
-      <c r="F243" s="1">
+      <c r="F243" s="2">
         <v>46048</v>
       </c>
       <c r="G243" t="s">
@@ -13142,7 +13168,7 @@
       <c r="E244" t="s">
         <v>971</v>
       </c>
-      <c r="F244" s="1">
+      <c r="F244" s="2">
         <v>46048</v>
       </c>
       <c r="G244" t="s">
@@ -13180,7 +13206,7 @@
       <c r="E245" t="s">
         <v>972</v>
       </c>
-      <c r="F245" s="1">
+      <c r="F245" s="2">
         <v>46048</v>
       </c>
       <c r="G245" t="s">
@@ -13218,7 +13244,7 @@
       <c r="E246" t="s">
         <v>973</v>
       </c>
-      <c r="F246" s="1">
+      <c r="F246" s="2">
         <v>46050</v>
       </c>
       <c r="G246" t="s">
@@ -13236,7 +13262,7 @@
       <c r="K246" t="s">
         <v>1220</v>
       </c>
-      <c r="M246" s="1">
+      <c r="M246" s="2">
         <v>46191</v>
       </c>
       <c r="P246" t="b">
@@ -13259,7 +13285,7 @@
       <c r="E247" t="s">
         <v>974</v>
       </c>
-      <c r="F247" s="1">
+      <c r="F247" s="2">
         <v>46050</v>
       </c>
       <c r="G247" t="s">
@@ -13288,7 +13314,7 @@
       <c r="E248" t="s">
         <v>975</v>
       </c>
-      <c r="F248" s="1">
+      <c r="F248" s="2">
         <v>46050</v>
       </c>
       <c r="G248" t="s">
@@ -13317,7 +13343,7 @@
       <c r="E249" t="s">
         <v>976</v>
       </c>
-      <c r="F249" s="1">
+      <c r="F249" s="2">
         <v>46050</v>
       </c>
       <c r="G249" t="s">
@@ -13355,7 +13381,7 @@
       <c r="E250" t="s">
         <v>977</v>
       </c>
-      <c r="F250" s="1">
+      <c r="F250" s="2">
         <v>46063</v>
       </c>
       <c r="G250" t="s">
@@ -13393,7 +13419,7 @@
       <c r="E251" t="s">
         <v>978</v>
       </c>
-      <c r="F251" s="1">
+      <c r="F251" s="2">
         <v>46063</v>
       </c>
       <c r="G251" t="s">
@@ -13428,7 +13454,7 @@
       <c r="E252" t="s">
         <v>979</v>
       </c>
-      <c r="F252" s="1">
+      <c r="F252" s="2">
         <v>46063</v>
       </c>
       <c r="G252" t="s">
@@ -13463,7 +13489,7 @@
       <c r="E253" t="s">
         <v>980</v>
       </c>
-      <c r="F253" s="1">
+      <c r="F253" s="2">
         <v>46063</v>
       </c>
       <c r="G253" t="s">
@@ -13501,7 +13527,7 @@
       <c r="E254" t="s">
         <v>981</v>
       </c>
-      <c r="F254" s="1">
+      <c r="F254" s="2">
         <v>46063</v>
       </c>
       <c r="G254" t="s">
@@ -13539,7 +13565,7 @@
       <c r="E255" t="s">
         <v>982</v>
       </c>
-      <c r="F255" s="1">
+      <c r="F255" s="2">
         <v>46063</v>
       </c>
       <c r="G255" t="s">
@@ -13577,7 +13603,7 @@
       <c r="E256" t="s">
         <v>983</v>
       </c>
-      <c r="F256" s="1">
+      <c r="F256" s="2">
         <v>46063</v>
       </c>
       <c r="G256" t="s">
@@ -13618,7 +13644,7 @@
       <c r="E257" t="s">
         <v>984</v>
       </c>
-      <c r="F257" s="1">
+      <c r="F257" s="2">
         <v>46063</v>
       </c>
       <c r="G257" t="s">
@@ -13647,7 +13673,7 @@
       <c r="E258" t="s">
         <v>985</v>
       </c>
-      <c r="F258" s="1">
+      <c r="F258" s="2">
         <v>46063</v>
       </c>
       <c r="G258" t="s">
@@ -13676,7 +13702,7 @@
       <c r="E259" t="s">
         <v>986</v>
       </c>
-      <c r="F259" s="1">
+      <c r="F259" s="2">
         <v>46063</v>
       </c>
       <c r="G259" t="s">
@@ -13714,7 +13740,7 @@
       <c r="E260" t="s">
         <v>987</v>
       </c>
-      <c r="F260" s="1">
+      <c r="F260" s="2">
         <v>46063</v>
       </c>
       <c r="G260" t="s">
@@ -13752,7 +13778,7 @@
       <c r="E261" t="s">
         <v>988</v>
       </c>
-      <c r="F261" s="1">
+      <c r="F261" s="2">
         <v>46063</v>
       </c>
       <c r="G261" t="s">
@@ -13790,7 +13816,7 @@
       <c r="E262" t="s">
         <v>989</v>
       </c>
-      <c r="F262" s="1">
+      <c r="F262" s="2">
         <v>46063</v>
       </c>
       <c r="G262" t="s">
@@ -13808,7 +13834,7 @@
       <c r="K262" t="s">
         <v>1223</v>
       </c>
-      <c r="M262" s="1">
+      <c r="M262" s="2">
         <v>46113</v>
       </c>
       <c r="O262" t="s">
@@ -13834,7 +13860,7 @@
       <c r="E263" t="s">
         <v>990</v>
       </c>
-      <c r="F263" s="1">
+      <c r="F263" s="2">
         <v>46063</v>
       </c>
       <c r="G263" t="s">
@@ -13869,7 +13895,7 @@
       <c r="E264" t="s">
         <v>991</v>
       </c>
-      <c r="F264" s="1">
+      <c r="F264" s="2">
         <v>46063</v>
       </c>
       <c r="G264" t="s">
@@ -13907,7 +13933,7 @@
       <c r="E265" t="s">
         <v>992</v>
       </c>
-      <c r="F265" s="1">
+      <c r="F265" s="2">
         <v>46063</v>
       </c>
       <c r="G265" t="s">
@@ -13945,7 +13971,7 @@
       <c r="E266" t="s">
         <v>993</v>
       </c>
-      <c r="F266" s="1">
+      <c r="F266" s="2">
         <v>46063</v>
       </c>
       <c r="G266" t="s">
@@ -13983,7 +14009,7 @@
       <c r="E267" t="s">
         <v>994</v>
       </c>
-      <c r="F267" s="1">
+      <c r="F267" s="2">
         <v>46063</v>
       </c>
       <c r="G267" t="s">
@@ -14021,7 +14047,7 @@
       <c r="E268" t="s">
         <v>995</v>
       </c>
-      <c r="F268" s="1">
+      <c r="F268" s="2">
         <v>46063</v>
       </c>
       <c r="G268" t="s">
@@ -14056,7 +14082,7 @@
       <c r="D269" t="s">
         <v>711</v>
       </c>
-      <c r="F269" s="1">
+      <c r="F269" s="2">
         <v>46063</v>
       </c>
       <c r="G269" t="s">
@@ -14094,7 +14120,7 @@
       <c r="E270" t="s">
         <v>996</v>
       </c>
-      <c r="F270" s="1">
+      <c r="F270" s="2">
         <v>46063</v>
       </c>
       <c r="G270" t="s">
@@ -14132,7 +14158,7 @@
       <c r="E271" t="s">
         <v>997</v>
       </c>
-      <c r="F271" s="1">
+      <c r="F271" s="2">
         <v>46063</v>
       </c>
       <c r="G271" t="s">
@@ -14170,7 +14196,7 @@
       <c r="E272" t="s">
         <v>998</v>
       </c>
-      <c r="F272" s="1">
+      <c r="F272" s="2">
         <v>46063</v>
       </c>
       <c r="G272" t="s">
@@ -14188,7 +14214,7 @@
       <c r="K272" t="s">
         <v>1225</v>
       </c>
-      <c r="M272" s="1">
+      <c r="M272" s="2">
         <v>46185</v>
       </c>
       <c r="N272" t="s">
@@ -14214,7 +14240,7 @@
       <c r="E273" t="s">
         <v>999</v>
       </c>
-      <c r="F273" s="1">
+      <c r="F273" s="2">
         <v>46063</v>
       </c>
       <c r="G273" t="s">
@@ -14249,7 +14275,7 @@
       <c r="E274" t="s">
         <v>1000</v>
       </c>
-      <c r="F274" s="1">
+      <c r="F274" s="2">
         <v>46063</v>
       </c>
       <c r="G274" t="s">
@@ -14287,7 +14313,7 @@
       <c r="E275" t="s">
         <v>1001</v>
       </c>
-      <c r="F275" s="1">
+      <c r="F275" s="2">
         <v>46063</v>
       </c>
       <c r="G275" t="s">
@@ -14322,7 +14348,7 @@
       <c r="E276" t="s">
         <v>1002</v>
       </c>
-      <c r="F276" s="1">
+      <c r="F276" s="2">
         <v>46063</v>
       </c>
       <c r="G276" t="s">
@@ -14360,7 +14386,7 @@
       <c r="E277" t="s">
         <v>1003</v>
       </c>
-      <c r="F277" s="1">
+      <c r="F277" s="2">
         <v>46063</v>
       </c>
       <c r="G277" t="s">
@@ -14398,7 +14424,7 @@
       <c r="E278" t="s">
         <v>1004</v>
       </c>
-      <c r="F278" s="1">
+      <c r="F278" s="2">
         <v>46077</v>
       </c>
       <c r="G278" t="s">
@@ -14436,7 +14462,7 @@
       <c r="E279" t="s">
         <v>1005</v>
       </c>
-      <c r="F279" s="1">
+      <c r="F279" s="2">
         <v>46077</v>
       </c>
       <c r="G279" t="s">
@@ -14477,7 +14503,7 @@
       <c r="E280" t="s">
         <v>1006</v>
       </c>
-      <c r="F280" s="1">
+      <c r="F280" s="2">
         <v>46085</v>
       </c>
       <c r="G280" t="s">
@@ -14515,7 +14541,7 @@
       <c r="E281" t="s">
         <v>1007</v>
       </c>
-      <c r="F281" s="1">
+      <c r="F281" s="2">
         <v>46085</v>
       </c>
       <c r="G281" t="s">
@@ -14553,7 +14579,7 @@
       <c r="E282" t="s">
         <v>1008</v>
       </c>
-      <c r="F282" s="1">
+      <c r="F282" s="2">
         <v>46090</v>
       </c>
       <c r="G282" t="s">
@@ -14591,7 +14617,7 @@
       <c r="E283" t="s">
         <v>1009</v>
       </c>
-      <c r="F283" s="1">
+      <c r="F283" s="2">
         <v>46100</v>
       </c>
       <c r="G283" t="s">
@@ -14626,7 +14652,7 @@
       <c r="E284" t="s">
         <v>1010</v>
       </c>
-      <c r="F284" s="1">
+      <c r="F284" s="2">
         <v>46100</v>
       </c>
       <c r="G284" t="s">
@@ -14661,7 +14687,7 @@
       <c r="E285" t="s">
         <v>1011</v>
       </c>
-      <c r="F285" s="1">
+      <c r="F285" s="2">
         <v>46100</v>
       </c>
       <c r="G285" t="s">
@@ -14696,7 +14722,7 @@
       <c r="E286" t="s">
         <v>1012</v>
       </c>
-      <c r="F286" s="1">
+      <c r="F286" s="2">
         <v>46100</v>
       </c>
       <c r="G286" t="s">
@@ -14731,7 +14757,7 @@
       <c r="E287">
         <v>35971</v>
       </c>
-      <c r="F287" s="1">
+      <c r="F287" s="2">
         <v>46107</v>
       </c>
       <c r="G287" t="s">
@@ -14760,7 +14786,7 @@
       <c r="E288">
         <v>107178</v>
       </c>
-      <c r="F288" s="1">
+      <c r="F288" s="2">
         <v>46107</v>
       </c>
       <c r="G288" t="s">
@@ -14798,7 +14824,7 @@
       <c r="E289">
         <v>108773</v>
       </c>
-      <c r="F289" s="1">
+      <c r="F289" s="2">
         <v>46107</v>
       </c>
       <c r="G289" t="s">
@@ -14827,7 +14853,7 @@
       <c r="E290">
         <v>7086</v>
       </c>
-      <c r="F290" s="1">
+      <c r="F290" s="2">
         <v>46107</v>
       </c>
       <c r="G290" t="s">
@@ -14842,7 +14868,7 @@
       <c r="J290" t="s">
         <v>1145</v>
       </c>
-      <c r="M290" s="1">
+      <c r="M290" s="2">
         <v>46127</v>
       </c>
       <c r="P290" t="b">
@@ -14865,7 +14891,7 @@
       <c r="E291">
         <v>99743</v>
       </c>
-      <c r="F291" s="1">
+      <c r="F291" s="2">
         <v>46107</v>
       </c>
       <c r="G291" t="s">
@@ -14903,7 +14929,7 @@
       <c r="E292" t="s">
         <v>1013</v>
       </c>
-      <c r="F292" s="1">
+      <c r="F292" s="2">
         <v>46112</v>
       </c>
       <c r="G292" t="s">
@@ -14941,7 +14967,7 @@
       <c r="E293" t="s">
         <v>1014</v>
       </c>
-      <c r="F293" s="1">
+      <c r="F293" s="2">
         <v>46125</v>
       </c>
       <c r="G293" t="s">
@@ -14979,7 +15005,7 @@
       <c r="E294" t="s">
         <v>1015</v>
       </c>
-      <c r="F294" s="1">
+      <c r="F294" s="2">
         <v>46125</v>
       </c>
       <c r="G294" t="s">
@@ -15014,7 +15040,7 @@
       <c r="E295" t="s">
         <v>1016</v>
       </c>
-      <c r="F295" s="1">
+      <c r="F295" s="2">
         <v>46125</v>
       </c>
       <c r="G295" t="s">
@@ -15049,7 +15075,7 @@
       <c r="E296" t="s">
         <v>1017</v>
       </c>
-      <c r="F296" s="1">
+      <c r="F296" s="2">
         <v>46125</v>
       </c>
       <c r="G296" t="s">
@@ -15084,7 +15110,7 @@
       <c r="E297">
         <v>47203152</v>
       </c>
-      <c r="F297" s="1">
+      <c r="F297" s="2">
         <v>46125</v>
       </c>
       <c r="G297" t="s">
@@ -15119,7 +15145,7 @@
       <c r="E298">
         <v>47202512</v>
       </c>
-      <c r="F298" s="1">
+      <c r="F298" s="2">
         <v>46125</v>
       </c>
       <c r="G298" t="s">
@@ -15157,7 +15183,7 @@
       <c r="E299">
         <v>22005580</v>
       </c>
-      <c r="F299" s="1">
+      <c r="F299" s="2">
         <v>46125</v>
       </c>
       <c r="G299" t="s">
@@ -15195,7 +15221,7 @@
       <c r="E300">
         <v>22005955</v>
       </c>
-      <c r="F300" s="1">
+      <c r="F300" s="2">
         <v>46125</v>
       </c>
       <c r="G300" t="s">
@@ -15233,7 +15259,7 @@
       <c r="E301">
         <v>22005661</v>
       </c>
-      <c r="F301" s="1">
+      <c r="F301" s="2">
         <v>46125</v>
       </c>
       <c r="G301" t="s">
@@ -15271,7 +15297,7 @@
       <c r="E302">
         <v>32207</v>
       </c>
-      <c r="F302" s="1">
+      <c r="F302" s="2">
         <v>46125</v>
       </c>
       <c r="G302" t="s">
@@ -15309,7 +15335,7 @@
       <c r="E303">
         <v>18156</v>
       </c>
-      <c r="F303" s="1">
+      <c r="F303" s="2">
         <v>46125</v>
       </c>
       <c r="G303" t="s">
@@ -15347,7 +15373,7 @@
       <c r="E304">
         <v>37971</v>
       </c>
-      <c r="F304" s="1">
+      <c r="F304" s="2">
         <v>46125</v>
       </c>
       <c r="G304" t="s">
@@ -15385,7 +15411,7 @@
       <c r="E305">
         <v>84317</v>
       </c>
-      <c r="F305" s="1">
+      <c r="F305" s="2">
         <v>46125</v>
       </c>
       <c r="G305" t="s">
@@ -15403,7 +15429,7 @@
       <c r="K305" t="s">
         <v>1230</v>
       </c>
-      <c r="M305" s="1">
+      <c r="M305" s="2">
         <v>46160</v>
       </c>
       <c r="P305" t="b">
@@ -15426,7 +15452,7 @@
       <c r="E306">
         <v>83773</v>
       </c>
-      <c r="F306" s="1">
+      <c r="F306" s="2">
         <v>46125</v>
       </c>
       <c r="G306" t="s">
@@ -15444,7 +15470,7 @@
       <c r="K306" t="s">
         <v>1231</v>
       </c>
-      <c r="M306" s="1">
+      <c r="M306" s="2">
         <v>46156</v>
       </c>
       <c r="P306" t="b">
@@ -15467,7 +15493,7 @@
       <c r="E307">
         <v>83740</v>
       </c>
-      <c r="F307" s="1">
+      <c r="F307" s="2">
         <v>46125</v>
       </c>
       <c r="G307" t="s">
@@ -15505,7 +15531,7 @@
       <c r="E308">
         <v>84326</v>
       </c>
-      <c r="F308" s="1">
+      <c r="F308" s="2">
         <v>46125</v>
       </c>
       <c r="G308" t="s">
@@ -15543,7 +15569,7 @@
       <c r="E309">
         <v>6708</v>
       </c>
-      <c r="F309" s="1">
+      <c r="F309" s="2">
         <v>46125</v>
       </c>
       <c r="G309" t="s">
@@ -15581,7 +15607,7 @@
       <c r="E310" t="s">
         <v>1018</v>
       </c>
-      <c r="F310" s="1">
+      <c r="F310" s="2">
         <v>46125</v>
       </c>
       <c r="G310" t="s">
@@ -15619,7 +15645,7 @@
       <c r="E311">
         <v>9727</v>
       </c>
-      <c r="F311" s="1">
+      <c r="F311" s="2">
         <v>46125</v>
       </c>
       <c r="G311" t="s">
@@ -15657,7 +15683,7 @@
       <c r="E312" t="s">
         <v>1019</v>
       </c>
-      <c r="F312" s="1">
+      <c r="F312" s="2">
         <v>46125</v>
       </c>
       <c r="G312" t="s">
@@ -15695,7 +15721,7 @@
       <c r="E313">
         <v>31</v>
       </c>
-      <c r="F313" s="1">
+      <c r="F313" s="2">
         <v>46125</v>
       </c>
       <c r="G313" t="s">
@@ -15730,7 +15756,7 @@
       <c r="E314">
         <v>965</v>
       </c>
-      <c r="F314" s="1">
+      <c r="F314" s="2">
         <v>46125</v>
       </c>
       <c r="G314" t="s">
@@ -15768,7 +15794,7 @@
       <c r="E315">
         <v>2007</v>
       </c>
-      <c r="F315" s="1">
+      <c r="F315" s="2">
         <v>46125</v>
       </c>
       <c r="G315" t="s">
@@ -15806,7 +15832,7 @@
       <c r="E316">
         <v>688</v>
       </c>
-      <c r="F316" s="1">
+      <c r="F316" s="2">
         <v>46125</v>
       </c>
       <c r="G316" t="s">
@@ -15844,7 +15870,7 @@
       <c r="E317" t="s">
         <v>1020</v>
       </c>
-      <c r="F317" s="1">
+      <c r="F317" s="2">
         <v>46125</v>
       </c>
       <c r="G317" t="s">
@@ -15882,7 +15908,7 @@
       <c r="E318" t="s">
         <v>1021</v>
       </c>
-      <c r="F318" s="1">
+      <c r="F318" s="2">
         <v>46125</v>
       </c>
       <c r="G318" t="s">
@@ -15911,7 +15937,7 @@
       <c r="E319" t="s">
         <v>1022</v>
       </c>
-      <c r="F319" s="1">
+      <c r="F319" s="2">
         <v>46125</v>
       </c>
       <c r="G319" t="s">
@@ -15926,7 +15952,7 @@
       <c r="K319" t="s">
         <v>1232</v>
       </c>
-      <c r="M319" s="1">
+      <c r="M319" s="2">
         <v>46175</v>
       </c>
       <c r="P319" t="b">
@@ -15949,7 +15975,7 @@
       <c r="E320">
         <v>1391</v>
       </c>
-      <c r="F320" s="1">
+      <c r="F320" s="2">
         <v>46125</v>
       </c>
       <c r="G320" t="s">
@@ -15987,7 +16013,7 @@
       <c r="E321">
         <v>120315</v>
       </c>
-      <c r="F321" s="1">
+      <c r="F321" s="2">
         <v>46125</v>
       </c>
       <c r="G321" t="s">
@@ -16025,7 +16051,7 @@
       <c r="E322" t="s">
         <v>1023</v>
       </c>
-      <c r="F322" s="1">
+      <c r="F322" s="2">
         <v>46125</v>
       </c>
       <c r="G322" t="s">
@@ -16043,7 +16069,7 @@
       <c r="K322" t="s">
         <v>1233</v>
       </c>
-      <c r="M322" s="1">
+      <c r="M322" s="2">
         <v>46182</v>
       </c>
       <c r="P322" t="b">
@@ -16066,7 +16092,7 @@
       <c r="E323">
         <v>535933</v>
       </c>
-      <c r="F323" s="1">
+      <c r="F323" s="2">
         <v>46125</v>
       </c>
       <c r="G323" t="s">
@@ -16104,7 +16130,7 @@
       <c r="E324">
         <v>289029</v>
       </c>
-      <c r="F324" s="1">
+      <c r="F324" s="2">
         <v>46125</v>
       </c>
       <c r="G324" t="s">
@@ -16142,7 +16168,7 @@
       <c r="E325">
         <v>3454</v>
       </c>
-      <c r="F325" s="1">
+      <c r="F325" s="2">
         <v>46125</v>
       </c>
       <c r="G325" t="s">
@@ -16160,7 +16186,7 @@
       <c r="K325" t="s">
         <v>1233</v>
       </c>
-      <c r="M325" s="1">
+      <c r="M325" s="2">
         <v>46182</v>
       </c>
       <c r="P325" t="b">
@@ -16183,7 +16209,7 @@
       <c r="E326">
         <v>3493</v>
       </c>
-      <c r="F326" s="1">
+      <c r="F326" s="2">
         <v>46125</v>
       </c>
       <c r="G326" t="s">
@@ -16221,7 +16247,7 @@
       <c r="E327" t="s">
         <v>1023</v>
       </c>
-      <c r="F327" s="1">
+      <c r="F327" s="2">
         <v>46125</v>
       </c>
       <c r="G327" t="s">
@@ -16239,7 +16265,7 @@
       <c r="K327" t="s">
         <v>1233</v>
       </c>
-      <c r="M327" s="1">
+      <c r="M327" s="2">
         <v>46182</v>
       </c>
       <c r="P327" t="b">
@@ -16262,7 +16288,7 @@
       <c r="E328">
         <v>3235</v>
       </c>
-      <c r="F328" s="1">
+      <c r="F328" s="2">
         <v>46125</v>
       </c>
       <c r="G328" t="s">
@@ -16280,7 +16306,7 @@
       <c r="K328" t="s">
         <v>1233</v>
       </c>
-      <c r="M328" s="1">
+      <c r="M328" s="2">
         <v>46182</v>
       </c>
       <c r="P328" t="b">
@@ -16303,7 +16329,7 @@
       <c r="E329">
         <v>625052</v>
       </c>
-      <c r="F329" s="1">
+      <c r="F329" s="2">
         <v>46125</v>
       </c>
       <c r="G329" t="s">
@@ -16321,7 +16347,7 @@
       <c r="K329" t="s">
         <v>1233</v>
       </c>
-      <c r="M329" s="1">
+      <c r="M329" s="2">
         <v>46182</v>
       </c>
       <c r="P329" t="b">
@@ -16344,7 +16370,7 @@
       <c r="E330">
         <v>614095</v>
       </c>
-      <c r="F330" s="1">
+      <c r="F330" s="2">
         <v>46125</v>
       </c>
       <c r="G330" t="s">
@@ -16362,7 +16388,7 @@
       <c r="K330" t="s">
         <v>1233</v>
       </c>
-      <c r="M330" s="1">
+      <c r="M330" s="2">
         <v>46182</v>
       </c>
       <c r="P330" t="b">
@@ -16385,7 +16411,7 @@
       <c r="E331" t="s">
         <v>965</v>
       </c>
-      <c r="F331" s="1">
+      <c r="F331" s="2">
         <v>46125</v>
       </c>
       <c r="G331" t="s">
@@ -16423,7 +16449,7 @@
       <c r="E332" t="s">
         <v>1024</v>
       </c>
-      <c r="F332" s="1">
+      <c r="F332" s="2">
         <v>46125</v>
       </c>
       <c r="G332" t="s">
@@ -16461,7 +16487,7 @@
       <c r="E333">
         <v>197</v>
       </c>
-      <c r="F333" s="1">
+      <c r="F333" s="2">
         <v>46125</v>
       </c>
       <c r="G333" t="s">
@@ -16499,7 +16525,7 @@
       <c r="E334">
         <v>1378</v>
       </c>
-      <c r="F334" s="1">
+      <c r="F334" s="2">
         <v>46125</v>
       </c>
       <c r="G334" t="s">
@@ -16537,7 +16563,7 @@
       <c r="E335" t="s">
         <v>1025</v>
       </c>
-      <c r="F335" s="1">
+      <c r="F335" s="2">
         <v>46127</v>
       </c>
       <c r="G335" t="s">
@@ -16552,7 +16578,7 @@
       <c r="K335" t="s">
         <v>1232</v>
       </c>
-      <c r="M335" s="1">
+      <c r="M335" s="2">
         <v>46175</v>
       </c>
       <c r="P335" t="b">
@@ -16575,7 +16601,7 @@
       <c r="E336" t="s">
         <v>1026</v>
       </c>
-      <c r="F336" s="1">
+      <c r="F336" s="2">
         <v>46127</v>
       </c>
       <c r="G336" t="s">
@@ -16613,7 +16639,7 @@
       <c r="E337" t="s">
         <v>1027</v>
       </c>
-      <c r="F337" s="1">
+      <c r="F337" s="2">
         <v>46127</v>
       </c>
       <c r="G337" t="s">
@@ -16628,7 +16654,7 @@
       <c r="K337" t="s">
         <v>1232</v>
       </c>
-      <c r="M337" s="1">
+      <c r="M337" s="2">
         <v>46175</v>
       </c>
       <c r="P337" t="b">
@@ -16651,7 +16677,7 @@
       <c r="E338" t="s">
         <v>1028</v>
       </c>
-      <c r="F338" s="1">
+      <c r="F338" s="2">
         <v>46127</v>
       </c>
       <c r="G338" t="s">
@@ -16689,7 +16715,7 @@
       <c r="E339">
         <v>6291</v>
       </c>
-      <c r="F339" s="1">
+      <c r="F339" s="2">
         <v>46129</v>
       </c>
       <c r="G339" t="s">
@@ -16718,7 +16744,7 @@
       <c r="E340" t="s">
         <v>1029</v>
       </c>
-      <c r="F340" s="1">
+      <c r="F340" s="2">
         <v>46142</v>
       </c>
       <c r="G340" t="s">
@@ -16756,7 +16782,7 @@
       <c r="E341" t="s">
         <v>1030</v>
       </c>
-      <c r="F341" s="1">
+      <c r="F341" s="2">
         <v>46142</v>
       </c>
       <c r="G341" t="s">
@@ -16794,7 +16820,7 @@
       <c r="E342" t="s">
         <v>1031</v>
       </c>
-      <c r="F342" s="1">
+      <c r="F342" s="2">
         <v>46142</v>
       </c>
       <c r="G342" t="s">
@@ -16832,7 +16858,7 @@
       <c r="E343" t="s">
         <v>1032</v>
       </c>
-      <c r="F343" s="1">
+      <c r="F343" s="2">
         <v>46142</v>
       </c>
       <c r="G343" t="s">
@@ -16870,7 +16896,7 @@
       <c r="E344" t="s">
         <v>1033</v>
       </c>
-      <c r="F344" s="1">
+      <c r="F344" s="2">
         <v>46142</v>
       </c>
       <c r="G344" t="s">
@@ -16908,7 +16934,7 @@
       <c r="E345" t="s">
         <v>1034</v>
       </c>
-      <c r="F345" s="1">
+      <c r="F345" s="2">
         <v>46142</v>
       </c>
       <c r="G345" t="s">
@@ -16946,7 +16972,7 @@
       <c r="E346" t="s">
         <v>1035</v>
       </c>
-      <c r="F346" s="1">
+      <c r="F346" s="2">
         <v>46142</v>
       </c>
       <c r="G346" t="s">
@@ -16984,7 +17010,7 @@
       <c r="E347" t="s">
         <v>1036</v>
       </c>
-      <c r="F347" s="1">
+      <c r="F347" s="2">
         <v>46142</v>
       </c>
       <c r="G347" t="s">
@@ -17002,7 +17028,7 @@
       <c r="K347" t="s">
         <v>1230</v>
       </c>
-      <c r="M347" s="1">
+      <c r="M347" s="2">
         <v>46160</v>
       </c>
       <c r="P347" t="b">
@@ -17025,7 +17051,7 @@
       <c r="E348" t="s">
         <v>1037</v>
       </c>
-      <c r="F348" s="1">
+      <c r="F348" s="2">
         <v>46142</v>
       </c>
       <c r="G348" t="s">
@@ -17043,7 +17069,7 @@
       <c r="K348" t="s">
         <v>1231</v>
       </c>
-      <c r="M348" s="1">
+      <c r="M348" s="2">
         <v>46156</v>
       </c>
       <c r="P348" t="b">
@@ -17066,7 +17092,7 @@
       <c r="E349" t="s">
         <v>1038</v>
       </c>
-      <c r="F349" s="1">
+      <c r="F349" s="2">
         <v>46142</v>
       </c>
       <c r="G349" t="s">
@@ -17104,7 +17130,7 @@
       <c r="E350" t="s">
         <v>1039</v>
       </c>
-      <c r="F350" s="1">
+      <c r="F350" s="2">
         <v>46142</v>
       </c>
       <c r="G350" t="s">
@@ -17139,7 +17165,7 @@
       <c r="E351" t="s">
         <v>1040</v>
       </c>
-      <c r="F351" s="1">
+      <c r="F351" s="2">
         <v>46142</v>
       </c>
       <c r="G351" t="s">
@@ -17177,7 +17203,7 @@
       <c r="E352" t="s">
         <v>1041</v>
       </c>
-      <c r="F352" s="1">
+      <c r="F352" s="2">
         <v>46142</v>
       </c>
       <c r="G352" t="s">
@@ -17215,7 +17241,7 @@
       <c r="E353" t="s">
         <v>1042</v>
       </c>
-      <c r="F353" s="1">
+      <c r="F353" s="2">
         <v>46142</v>
       </c>
       <c r="G353" t="s">
@@ -17253,7 +17279,7 @@
       <c r="E354" t="s">
         <v>1043</v>
       </c>
-      <c r="F354" s="1">
+      <c r="F354" s="2">
         <v>46142</v>
       </c>
       <c r="G354" t="s">
@@ -17291,7 +17317,7 @@
       <c r="E355" t="s">
         <v>1044</v>
       </c>
-      <c r="F355" s="1">
+      <c r="F355" s="2">
         <v>46142</v>
       </c>
       <c r="G355" t="s">
@@ -17309,7 +17335,7 @@
       <c r="K355" t="s">
         <v>1234</v>
       </c>
-      <c r="M355" s="1">
+      <c r="M355" s="2">
         <v>46150</v>
       </c>
       <c r="P355" t="b">
@@ -17332,7 +17358,7 @@
       <c r="E356" t="s">
         <v>1045</v>
       </c>
-      <c r="F356" s="1">
+      <c r="F356" s="2">
         <v>46142</v>
       </c>
       <c r="G356" t="s">
@@ -17347,7 +17373,7 @@
       <c r="K356" t="s">
         <v>1235</v>
       </c>
-      <c r="M356" s="1">
+      <c r="M356" s="2">
         <v>46176</v>
       </c>
       <c r="P356" t="b">
@@ -17370,7 +17396,7 @@
       <c r="E357" t="s">
         <v>1046</v>
       </c>
-      <c r="F357" s="1">
+      <c r="F357" s="2">
         <v>46142</v>
       </c>
       <c r="G357" t="s">
@@ -17408,7 +17434,7 @@
       <c r="E358" t="s">
         <v>1047</v>
       </c>
-      <c r="F358" s="1">
+      <c r="F358" s="2">
         <v>46142</v>
       </c>
       <c r="G358" t="s">
@@ -17446,7 +17472,7 @@
       <c r="E359" t="s">
         <v>1048</v>
       </c>
-      <c r="F359" s="1">
+      <c r="F359" s="2">
         <v>46142</v>
       </c>
       <c r="G359" t="s">
@@ -17487,7 +17513,7 @@
       <c r="E360" t="s">
         <v>857</v>
       </c>
-      <c r="F360" s="1">
+      <c r="F360" s="2">
         <v>46142</v>
       </c>
       <c r="G360" t="s">
@@ -17525,7 +17551,7 @@
       <c r="E361" t="s">
         <v>869</v>
       </c>
-      <c r="F361" s="1">
+      <c r="F361" s="2">
         <v>46142</v>
       </c>
       <c r="G361" t="s">
@@ -17563,7 +17589,7 @@
       <c r="E362" t="s">
         <v>1049</v>
       </c>
-      <c r="F362" s="1">
+      <c r="F362" s="2">
         <v>46142</v>
       </c>
       <c r="G362" t="s">
@@ -17601,7 +17627,7 @@
       <c r="E363" t="s">
         <v>1050</v>
       </c>
-      <c r="F363" s="1">
+      <c r="F363" s="2">
         <v>46142</v>
       </c>
       <c r="G363" t="s">
@@ -17639,7 +17665,7 @@
       <c r="E364" t="s">
         <v>866</v>
       </c>
-      <c r="F364" s="1">
+      <c r="F364" s="2">
         <v>46142</v>
       </c>
       <c r="G364" t="s">
@@ -17677,7 +17703,7 @@
       <c r="E365" t="s">
         <v>1051</v>
       </c>
-      <c r="F365" s="1">
+      <c r="F365" s="2">
         <v>46142</v>
       </c>
       <c r="G365" t="s">
@@ -17715,7 +17741,7 @@
       <c r="E366" t="s">
         <v>1052</v>
       </c>
-      <c r="F366" s="1">
+      <c r="F366" s="2">
         <v>46148</v>
       </c>
       <c r="G366" t="s">
@@ -17753,7 +17779,7 @@
       <c r="E367" t="s">
         <v>1053</v>
       </c>
-      <c r="F367" s="1">
+      <c r="F367" s="2">
         <v>46148</v>
       </c>
       <c r="G367" t="s">
@@ -17791,7 +17817,7 @@
       <c r="E368" t="s">
         <v>1054</v>
       </c>
-      <c r="F368" s="1">
+      <c r="F368" s="2">
         <v>46148</v>
       </c>
       <c r="G368" t="s">
@@ -17829,7 +17855,7 @@
       <c r="E369" t="s">
         <v>1055</v>
       </c>
-      <c r="F369" s="1">
+      <c r="F369" s="2">
         <v>46148</v>
       </c>
       <c r="G369" t="s">
@@ -17867,7 +17893,7 @@
       <c r="E370" t="s">
         <v>1056</v>
       </c>
-      <c r="F370" s="1">
+      <c r="F370" s="2">
         <v>46148</v>
       </c>
       <c r="G370" t="s">
@@ -17905,7 +17931,7 @@
       <c r="E371" t="s">
         <v>1057</v>
       </c>
-      <c r="F371" s="1">
+      <c r="F371" s="2">
         <v>46148</v>
       </c>
       <c r="G371" t="s">
@@ -17923,7 +17949,7 @@
       <c r="K371" t="s">
         <v>1236</v>
       </c>
-      <c r="M371" s="1">
+      <c r="M371" s="2">
         <v>46164</v>
       </c>
       <c r="P371" t="b">
@@ -17946,7 +17972,7 @@
       <c r="E372" t="s">
         <v>1058</v>
       </c>
-      <c r="F372" s="1">
+      <c r="F372" s="2">
         <v>46148</v>
       </c>
       <c r="G372" t="s">
@@ -17964,7 +17990,7 @@
       <c r="K372" t="s">
         <v>1223</v>
       </c>
-      <c r="M372" s="1">
+      <c r="M372" s="2">
         <v>46113</v>
       </c>
       <c r="O372" t="s">
@@ -17990,7 +18016,7 @@
       <c r="E373" t="s">
         <v>1059</v>
       </c>
-      <c r="F373" s="1">
+      <c r="F373" s="2">
         <v>46149</v>
       </c>
       <c r="G373" t="s">
@@ -18028,7 +18054,7 @@
       <c r="E374" t="s">
         <v>1060</v>
       </c>
-      <c r="F374" s="1">
+      <c r="F374" s="2">
         <v>46149</v>
       </c>
       <c r="G374" t="s">
@@ -18066,7 +18092,7 @@
       <c r="E375" t="s">
         <v>1061</v>
       </c>
-      <c r="F375" s="1">
+      <c r="F375" s="2">
         <v>46154</v>
       </c>
       <c r="G375" t="s">
@@ -18104,7 +18130,7 @@
       <c r="E376" t="s">
         <v>1062</v>
       </c>
-      <c r="F376" s="1">
+      <c r="F376" s="2">
         <v>46154</v>
       </c>
       <c r="G376" t="s">
@@ -18142,7 +18168,7 @@
       <c r="E377" t="s">
         <v>1063</v>
       </c>
-      <c r="F377" s="1">
+      <c r="F377" s="2">
         <v>46154</v>
       </c>
       <c r="G377" t="s">
@@ -18180,7 +18206,7 @@
       <c r="E378" t="s">
         <v>1064</v>
       </c>
-      <c r="F378" s="1">
+      <c r="F378" s="2">
         <v>46154</v>
       </c>
       <c r="G378" t="s">
@@ -18218,7 +18244,7 @@
       <c r="E379" t="s">
         <v>1065</v>
       </c>
-      <c r="F379" s="1">
+      <c r="F379" s="2">
         <v>46154</v>
       </c>
       <c r="G379" t="s">
@@ -18236,7 +18262,7 @@
       <c r="K379" t="s">
         <v>1237</v>
       </c>
-      <c r="M379" s="1">
+      <c r="M379" s="2">
         <v>46174</v>
       </c>
       <c r="P379" t="b">
@@ -18259,7 +18285,7 @@
       <c r="E380" t="s">
         <v>1066</v>
       </c>
-      <c r="F380" s="1">
+      <c r="F380" s="2">
         <v>46154</v>
       </c>
       <c r="G380" t="s">
@@ -18297,7 +18323,7 @@
       <c r="E381" t="s">
         <v>1067</v>
       </c>
-      <c r="F381" s="1">
+      <c r="F381" s="2">
         <v>46154</v>
       </c>
       <c r="G381" t="s">
@@ -18335,7 +18361,7 @@
       <c r="E382" t="s">
         <v>1068</v>
       </c>
-      <c r="F382" s="1">
+      <c r="F382" s="2">
         <v>46154</v>
       </c>
       <c r="G382" t="s">
@@ -18373,7 +18399,7 @@
       <c r="E383" t="s">
         <v>1069</v>
       </c>
-      <c r="F383" s="1">
+      <c r="F383" s="2">
         <v>46154</v>
       </c>
       <c r="G383" t="s">
@@ -18411,7 +18437,7 @@
       <c r="E384" t="s">
         <v>1070</v>
       </c>
-      <c r="F384" s="1">
+      <c r="F384" s="2">
         <v>46164</v>
       </c>
       <c r="G384" t="s">
@@ -18449,7 +18475,7 @@
       <c r="E385" t="s">
         <v>1071</v>
       </c>
-      <c r="F385" s="1">
+      <c r="F385" s="2">
         <v>46164</v>
       </c>
       <c r="G385" t="s">
@@ -18487,7 +18513,7 @@
       <c r="E386" t="s">
         <v>1072</v>
       </c>
-      <c r="F386" s="1">
+      <c r="F386" s="2">
         <v>46171</v>
       </c>
       <c r="G386" t="s">
@@ -18525,7 +18551,7 @@
       <c r="E387" t="s">
         <v>1073</v>
       </c>
-      <c r="F387" s="1">
+      <c r="F387" s="2">
         <v>46171</v>
       </c>
       <c r="G387" t="s">
@@ -18563,7 +18589,7 @@
       <c r="E388" t="s">
         <v>759</v>
       </c>
-      <c r="F388" s="1">
+      <c r="F388" s="2">
         <v>46171</v>
       </c>
       <c r="G388" t="s">
@@ -18601,7 +18627,7 @@
       <c r="E389" t="s">
         <v>1074</v>
       </c>
-      <c r="F389" s="1">
+      <c r="F389" s="2">
         <v>46171</v>
       </c>
       <c r="G389" t="s">
@@ -18639,7 +18665,7 @@
       <c r="E390" t="s">
         <v>1075</v>
       </c>
-      <c r="F390" s="1">
+      <c r="F390" s="2">
         <v>46171</v>
       </c>
       <c r="G390" t="s">
@@ -18657,7 +18683,7 @@
       <c r="K390" t="s">
         <v>1238</v>
       </c>
-      <c r="M390" s="1">
+      <c r="M390" s="2">
         <v>46191</v>
       </c>
       <c r="P390" t="b">
@@ -18680,7 +18706,7 @@
       <c r="E391" t="s">
         <v>1076</v>
       </c>
-      <c r="F391" s="1">
+      <c r="F391" s="2">
         <v>46171</v>
       </c>
       <c r="G391" t="s">
@@ -18718,7 +18744,7 @@
       <c r="E392" t="s">
         <v>1077</v>
       </c>
-      <c r="F392" s="1">
+      <c r="F392" s="2">
         <v>46171</v>
       </c>
       <c r="G392" t="s">
@@ -18733,7 +18759,7 @@
       <c r="K392" t="s">
         <v>1235</v>
       </c>
-      <c r="M392" s="1">
+      <c r="M392" s="2">
         <v>46176</v>
       </c>
       <c r="P392" t="b">
@@ -18756,7 +18782,7 @@
       <c r="E393" t="s">
         <v>1078</v>
       </c>
-      <c r="F393" s="1">
+      <c r="F393" s="2">
         <v>46171</v>
       </c>
       <c r="G393" t="s">
@@ -18794,7 +18820,7 @@
       <c r="E394" t="s">
         <v>1079</v>
       </c>
-      <c r="F394" s="1">
+      <c r="F394" s="2">
         <v>46171</v>
       </c>
       <c r="G394" t="s">
@@ -18832,7 +18858,7 @@
       <c r="E395" t="s">
         <v>1080</v>
       </c>
-      <c r="F395" s="1">
+      <c r="F395" s="2">
         <v>46171</v>
       </c>
       <c r="G395" t="s">
@@ -18870,7 +18896,7 @@
       <c r="E396" t="s">
         <v>1081</v>
       </c>
-      <c r="F396" s="1">
+      <c r="F396" s="2">
         <v>46171</v>
       </c>
       <c r="G396" t="s">
@@ -18908,7 +18934,7 @@
       <c r="E397" t="s">
         <v>1082</v>
       </c>
-      <c r="F397" s="1">
+      <c r="F397" s="2">
         <v>46171</v>
       </c>
       <c r="G397" t="s">
@@ -18946,7 +18972,7 @@
       <c r="E398" t="s">
         <v>1083</v>
       </c>
-      <c r="F398" s="1">
+      <c r="F398" s="2">
         <v>46171</v>
       </c>
       <c r="G398" t="s">
@@ -18984,7 +19010,7 @@
       <c r="E399" t="s">
         <v>895</v>
       </c>
-      <c r="F399" s="1">
+      <c r="F399" s="2">
         <v>46163</v>
       </c>
       <c r="G399" t="s">
@@ -18999,7 +19025,7 @@
       <c r="K399" t="s">
         <v>1239</v>
       </c>
-      <c r="M399" s="1">
+      <c r="M399" s="2">
         <v>46171</v>
       </c>
       <c r="P399" t="b">
@@ -19022,7 +19048,7 @@
       <c r="E400" t="s">
         <v>1084</v>
       </c>
-      <c r="F400" s="1">
+      <c r="F400" s="2">
         <v>46171</v>
       </c>
       <c r="G400" t="s">
@@ -19060,7 +19086,7 @@
       <c r="E401" t="s">
         <v>1085</v>
       </c>
-      <c r="F401" s="1">
+      <c r="F401" s="2">
         <v>46171</v>
       </c>
       <c r="G401" t="s">
@@ -19098,7 +19124,7 @@
       <c r="E402" t="s">
         <v>1086</v>
       </c>
-      <c r="F402" s="1">
+      <c r="F402" s="2">
         <v>46171</v>
       </c>
       <c r="G402" t="s">
@@ -19136,7 +19162,7 @@
       <c r="E403" t="s">
         <v>1087</v>
       </c>
-      <c r="F403" s="1">
+      <c r="F403" s="2">
         <v>46171</v>
       </c>
       <c r="G403" t="s">
@@ -19171,7 +19197,7 @@
       <c r="E404" t="s">
         <v>1088</v>
       </c>
-      <c r="F404" s="1">
+      <c r="F404" s="2">
         <v>46171</v>
       </c>
       <c r="G404" t="s">
@@ -19206,7 +19232,7 @@
       <c r="E405">
         <v>9599</v>
       </c>
-      <c r="F405" s="1">
+      <c r="F405" s="2">
         <v>46183</v>
       </c>
       <c r="G405" t="s">
@@ -19235,7 +19261,7 @@
       <c r="E406">
         <v>14251</v>
       </c>
-      <c r="F406" s="1">
+      <c r="F406" s="2">
         <v>46183</v>
       </c>
       <c r="G406" t="s">
@@ -19267,7 +19293,7 @@
       <c r="E407">
         <v>19945</v>
       </c>
-      <c r="F407" s="1">
+      <c r="F407" s="2">
         <v>46183</v>
       </c>
       <c r="G407" t="s">
@@ -19299,7 +19325,7 @@
       <c r="E408">
         <v>14396</v>
       </c>
-      <c r="F408" s="1">
+      <c r="F408" s="2">
         <v>46183</v>
       </c>
       <c r="G408" t="s">
@@ -19331,7 +19357,7 @@
       <c r="E409">
         <v>9920</v>
       </c>
-      <c r="F409" s="1">
+      <c r="F409" s="2">
         <v>46183</v>
       </c>
       <c r="G409" t="s">
@@ -19363,7 +19389,7 @@
       <c r="E410">
         <v>20528</v>
       </c>
-      <c r="F410" s="1">
+      <c r="F410" s="2">
         <v>46183</v>
       </c>
       <c r="G410" t="s">
@@ -19395,7 +19421,7 @@
       <c r="E411" t="s">
         <v>1089</v>
       </c>
-      <c r="F411" s="1">
+      <c r="F411" s="2">
         <v>46188</v>
       </c>
       <c r="G411" t="s">
@@ -19427,7 +19453,7 @@
       <c r="E412" t="s">
         <v>1090</v>
       </c>
-      <c r="F412" s="1">
+      <c r="F412" s="2">
         <v>46188</v>
       </c>
       <c r="G412" t="s">
@@ -19459,7 +19485,7 @@
       <c r="E413" t="s">
         <v>1091</v>
       </c>
-      <c r="F413" s="1">
+      <c r="F413" s="2">
         <v>46188</v>
       </c>
       <c r="G413" t="s">
@@ -19491,7 +19517,7 @@
       <c r="E414" t="s">
         <v>1092</v>
       </c>
-      <c r="F414" s="1">
+      <c r="F414" s="2">
         <v>46188</v>
       </c>
       <c r="G414" t="s">
@@ -19523,7 +19549,7 @@
       <c r="E415" t="s">
         <v>968</v>
       </c>
-      <c r="F415" s="1">
+      <c r="F415" s="2">
         <v>46188</v>
       </c>
       <c r="G415" t="s">
@@ -19555,7 +19581,7 @@
       <c r="E416">
         <v>5844</v>
       </c>
-      <c r="F416" s="1">
+      <c r="F416" s="2">
         <v>46188</v>
       </c>
       <c r="G416" t="s">
@@ -19587,7 +19613,7 @@
       <c r="E417" t="s">
         <v>1093</v>
       </c>
-      <c r="F417" s="1">
+      <c r="F417" s="2">
         <v>46188</v>
       </c>
       <c r="G417" t="s">
@@ -19619,7 +19645,7 @@
       <c r="E418" t="s">
         <v>1094</v>
       </c>
-      <c r="F418" s="1">
+      <c r="F418" s="2">
         <v>46188</v>
       </c>
       <c r="G418" t="s">
@@ -19651,7 +19677,7 @@
       <c r="E419" t="s">
         <v>1095</v>
       </c>
-      <c r="F419" s="1">
+      <c r="F419" s="2">
         <v>46188</v>
       </c>
       <c r="G419" t="s">
@@ -19683,7 +19709,7 @@
       <c r="E420">
         <v>580</v>
       </c>
-      <c r="F420" s="1">
+      <c r="F420" s="2">
         <v>46188</v>
       </c>
       <c r="G420" t="s">
@@ -19715,7 +19741,7 @@
       <c r="E421" t="s">
         <v>1096</v>
       </c>
-      <c r="F421" s="1">
+      <c r="F421" s="2">
         <v>46188</v>
       </c>
       <c r="G421" t="s">
@@ -19747,7 +19773,7 @@
       <c r="E422" t="s">
         <v>1097</v>
       </c>
-      <c r="F422" s="1">
+      <c r="F422" s="2">
         <v>46188</v>
       </c>
       <c r="G422" t="s">
@@ -19779,7 +19805,7 @@
       <c r="E423" t="s">
         <v>1098</v>
       </c>
-      <c r="F423" s="1">
+      <c r="F423" s="2">
         <v>46188</v>
       </c>
       <c r="G423" t="s">
@@ -19811,7 +19837,7 @@
       <c r="E424" t="s">
         <v>1099</v>
       </c>
-      <c r="F424" s="1">
+      <c r="F424" s="2">
         <v>46188</v>
       </c>
       <c r="G424" t="s">
@@ -19843,7 +19869,7 @@
       <c r="E425" t="s">
         <v>1100</v>
       </c>
-      <c r="F425" s="1">
+      <c r="F425" s="2">
         <v>46188</v>
       </c>
       <c r="G425" t="s">
@@ -19875,7 +19901,7 @@
       <c r="E426" t="s">
         <v>1101</v>
       </c>
-      <c r="F426" s="1">
+      <c r="F426" s="2">
         <v>46188</v>
       </c>
       <c r="G426" t="s">
@@ -19907,7 +19933,7 @@
       <c r="E427">
         <v>6309</v>
       </c>
-      <c r="F427" s="1">
+      <c r="F427" s="2">
         <v>46188</v>
       </c>
       <c r="G427" t="s">
@@ -19939,7 +19965,7 @@
       <c r="E428">
         <v>504011190625165</v>
       </c>
-      <c r="F428" s="1">
+      <c r="F428" s="2">
         <v>46188</v>
       </c>
       <c r="G428" t="s">
@@ -19971,7 +19997,7 @@
       <c r="E429">
         <v>504011190625185</v>
       </c>
-      <c r="F429" s="1">
+      <c r="F429" s="2">
         <v>46188</v>
       </c>
       <c r="G429" t="s">
@@ -20003,7 +20029,7 @@
       <c r="E430" t="s">
         <v>1102</v>
       </c>
-      <c r="F430" s="1">
+      <c r="F430" s="2">
         <v>46188</v>
       </c>
       <c r="G430" t="s">
@@ -20035,7 +20061,7 @@
       <c r="E431" t="s">
         <v>1103</v>
       </c>
-      <c r="F431" s="1">
+      <c r="F431" s="2">
         <v>46188</v>
       </c>
       <c r="G431" t="s">
@@ -20067,7 +20093,7 @@
       <c r="E432" t="s">
         <v>1104</v>
       </c>
-      <c r="F432" s="1">
+      <c r="F432" s="2">
         <v>46188</v>
       </c>
       <c r="G432" t="s">
@@ -20099,7 +20125,7 @@
       <c r="E433" t="s">
         <v>1105</v>
       </c>
-      <c r="F433" s="1">
+      <c r="F433" s="2">
         <v>46188</v>
       </c>
       <c r="G433" t="s">
@@ -20131,7 +20157,7 @@
       <c r="E434">
         <v>328</v>
       </c>
-      <c r="F434" s="1">
+      <c r="F434" s="2">
         <v>46188</v>
       </c>
       <c r="G434" t="s">
@@ -20163,7 +20189,7 @@
       <c r="E435">
         <v>277</v>
       </c>
-      <c r="F435" s="1">
+      <c r="F435" s="2">
         <v>46188</v>
       </c>
       <c r="G435" t="s">
@@ -20195,7 +20221,7 @@
       <c r="E436">
         <v>477</v>
       </c>
-      <c r="F436" s="1">
+      <c r="F436" s="2">
         <v>46188</v>
       </c>
       <c r="G436" t="s">
@@ -20227,7 +20253,7 @@
       <c r="E437">
         <v>11</v>
       </c>
-      <c r="F437" s="1">
+      <c r="F437" s="2">
         <v>46188</v>
       </c>
       <c r="G437" t="s">
@@ -20259,7 +20285,7 @@
       <c r="E438" t="s">
         <v>1106</v>
       </c>
-      <c r="F438" s="1">
+      <c r="F438" s="2">
         <v>46188</v>
       </c>
       <c r="G438" t="s">
@@ -20291,7 +20317,7 @@
       <c r="E439" t="s">
         <v>1107</v>
       </c>
-      <c r="F439" s="1">
+      <c r="F439" s="2">
         <v>46196</v>
       </c>
       <c r="G439" t="s">
@@ -20323,7 +20349,7 @@
       <c r="E440" t="s">
         <v>1108</v>
       </c>
-      <c r="F440" s="1">
+      <c r="F440" s="2">
         <v>46196</v>
       </c>
       <c r="G440" t="s">
@@ -20355,7 +20381,7 @@
       <c r="E441">
         <v>86815651</v>
       </c>
-      <c r="F441" s="1">
+      <c r="F441" s="2">
         <v>46203</v>
       </c>
       <c r="G441" t="s">
@@ -20387,7 +20413,7 @@
       <c r="E442">
         <v>86817554</v>
       </c>
-      <c r="F442" s="1">
+      <c r="F442" s="2">
         <v>46203</v>
       </c>
       <c r="G442" t="s">
@@ -20419,7 +20445,7 @@
       <c r="E443" t="s">
         <v>1109</v>
       </c>
-      <c r="F443" s="1">
+      <c r="F443" s="2">
         <v>46205</v>
       </c>
       <c r="G443" t="s">
@@ -20451,7 +20477,7 @@
       <c r="E444" t="s">
         <v>1110</v>
       </c>
-      <c r="F444" s="1">
+      <c r="F444" s="2">
         <v>46205</v>
       </c>
       <c r="G444" t="s">
@@ -20483,7 +20509,7 @@
       <c r="E445">
         <v>4134</v>
       </c>
-      <c r="F445" s="1">
+      <c r="F445" s="2">
         <v>46205</v>
       </c>
       <c r="G445" t="s">
@@ -20515,7 +20541,7 @@
       <c r="E446">
         <v>22006508</v>
       </c>
-      <c r="F446" s="1">
+      <c r="F446" s="2">
         <v>46211</v>
       </c>
       <c r="G446" t="s">
@@ -20547,7 +20573,7 @@
       <c r="E447">
         <v>22005733</v>
       </c>
-      <c r="F447" s="1">
+      <c r="F447" s="2">
         <v>46211</v>
       </c>
       <c r="G447" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis (23/07/2026 16:18)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -3842,16 +3842,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3867,7 +3859,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -3875,30 +3867,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4198,52 +4172,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4263,7 +4237,7 @@
       <c r="E2" t="s">
         <v>737</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>45698</v>
       </c>
       <c r="G2" t="s">
@@ -4301,7 +4275,7 @@
       <c r="E3" t="s">
         <v>738</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>45714</v>
       </c>
       <c r="G3" t="s">
@@ -4339,7 +4313,7 @@
       <c r="E4" t="s">
         <v>739</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>45714</v>
       </c>
       <c r="G4" t="s">
@@ -4377,7 +4351,7 @@
       <c r="E5" t="s">
         <v>740</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>45714</v>
       </c>
       <c r="G5" t="s">
@@ -4395,7 +4369,7 @@
       <c r="K5" t="s">
         <v>1151</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="1">
         <v>45993</v>
       </c>
       <c r="P5" t="b">
@@ -4418,7 +4392,7 @@
       <c r="E6" t="s">
         <v>741</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>45736</v>
       </c>
       <c r="G6" t="s">
@@ -4436,7 +4410,7 @@
       <c r="K6" t="s">
         <v>1152</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="1">
         <v>45889</v>
       </c>
       <c r="P6" t="b">
@@ -4459,7 +4433,7 @@
       <c r="E7" t="s">
         <v>742</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>45736</v>
       </c>
       <c r="G7" t="s">
@@ -4477,7 +4451,7 @@
       <c r="K7" t="s">
         <v>1153</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="1">
         <v>45848</v>
       </c>
       <c r="N7" t="s">
@@ -4503,7 +4477,7 @@
       <c r="E8" t="s">
         <v>743</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>45736</v>
       </c>
       <c r="G8" t="s">
@@ -4532,7 +4506,7 @@
       <c r="E9" t="s">
         <v>744</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>45736</v>
       </c>
       <c r="G9" t="s">
@@ -4550,7 +4524,7 @@
       <c r="K9" t="s">
         <v>1154</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="1">
         <v>46098</v>
       </c>
       <c r="N9">
@@ -4576,7 +4550,7 @@
       <c r="E10" t="s">
         <v>745</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>45736</v>
       </c>
       <c r="G10" t="s">
@@ -4594,7 +4568,7 @@
       <c r="K10" t="s">
         <v>1155</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46114</v>
       </c>
       <c r="N10" t="s">
@@ -4620,7 +4594,7 @@
       <c r="E11" t="s">
         <v>746</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>45736</v>
       </c>
       <c r="G11" t="s">
@@ -4638,7 +4612,7 @@
       <c r="K11" t="s">
         <v>1153</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>45848</v>
       </c>
       <c r="N11" t="s">
@@ -4664,7 +4638,7 @@
       <c r="E12" t="s">
         <v>747</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="1">
         <v>45736</v>
       </c>
       <c r="G12" t="s">
@@ -4682,7 +4656,7 @@
       <c r="K12" t="s">
         <v>1156</v>
       </c>
-      <c r="M12" s="2">
+      <c r="M12" s="1">
         <v>45860</v>
       </c>
       <c r="P12" t="b">
@@ -4705,7 +4679,7 @@
       <c r="E13" t="s">
         <v>748</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="1">
         <v>45736</v>
       </c>
       <c r="G13" t="s">
@@ -4740,7 +4714,7 @@
       <c r="E14" t="s">
         <v>749</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="1">
         <v>45736</v>
       </c>
       <c r="G14" t="s">
@@ -4758,7 +4732,7 @@
       <c r="K14" t="s">
         <v>1157</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="1">
         <v>45800</v>
       </c>
       <c r="P14" t="b">
@@ -4781,7 +4755,7 @@
       <c r="E15" t="s">
         <v>750</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="1">
         <v>45736</v>
       </c>
       <c r="G15" t="s">
@@ -4819,7 +4793,7 @@
       <c r="E16" t="s">
         <v>751</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>45736</v>
       </c>
       <c r="G16" t="s">
@@ -4857,7 +4831,7 @@
       <c r="E17" t="s">
         <v>752</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>45736</v>
       </c>
       <c r="G17" t="s">
@@ -4875,7 +4849,7 @@
       <c r="K17" t="s">
         <v>1152</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>45897</v>
       </c>
       <c r="P17" t="b">
@@ -4898,7 +4872,7 @@
       <c r="E18" t="s">
         <v>753</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="1">
         <v>45736</v>
       </c>
       <c r="G18" t="s">
@@ -4916,7 +4890,7 @@
       <c r="K18" t="s">
         <v>1157</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>45802</v>
       </c>
       <c r="P18" t="b">
@@ -4939,7 +4913,7 @@
       <c r="E19" t="s">
         <v>754</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="1">
         <v>45736</v>
       </c>
       <c r="G19" t="s">
@@ -4974,7 +4948,7 @@
       <c r="E20" t="s">
         <v>755</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="1">
         <v>45736</v>
       </c>
       <c r="G20" t="s">
@@ -4992,7 +4966,7 @@
       <c r="K20" t="s">
         <v>1159</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46135</v>
       </c>
       <c r="P20" t="b">
@@ -5015,7 +4989,7 @@
       <c r="E21" t="s">
         <v>756</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="1">
         <v>45736</v>
       </c>
       <c r="G21" t="s">
@@ -5050,7 +5024,7 @@
       <c r="E22" t="s">
         <v>757</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="1">
         <v>45736</v>
       </c>
       <c r="G22" t="s">
@@ -5088,7 +5062,7 @@
       <c r="E23" t="s">
         <v>758</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="1">
         <v>45736</v>
       </c>
       <c r="G23" t="s">
@@ -5106,7 +5080,7 @@
       <c r="K23" t="s">
         <v>1161</v>
       </c>
-      <c r="M23" s="2">
+      <c r="M23" s="1">
         <v>45965</v>
       </c>
       <c r="O23" t="s">
@@ -5132,7 +5106,7 @@
       <c r="E24" t="s">
         <v>759</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="1">
         <v>45736</v>
       </c>
       <c r="G24" t="s">
@@ -5167,7 +5141,7 @@
       <c r="E25" t="s">
         <v>760</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="1">
         <v>45736</v>
       </c>
       <c r="G25" t="s">
@@ -5202,7 +5176,7 @@
       <c r="E26" t="s">
         <v>761</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="1">
         <v>45736</v>
       </c>
       <c r="G26" t="s">
@@ -5220,7 +5194,7 @@
       <c r="K26" t="s">
         <v>1164</v>
       </c>
-      <c r="M26" s="2">
+      <c r="M26" s="1">
         <v>45891</v>
       </c>
       <c r="O26" t="s">
@@ -5246,7 +5220,7 @@
       <c r="E27" t="s">
         <v>762</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>45736</v>
       </c>
       <c r="G27" t="s">
@@ -5284,7 +5258,7 @@
       <c r="E28" t="s">
         <v>763</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="1">
         <v>45736</v>
       </c>
       <c r="G28" t="s">
@@ -5313,7 +5287,7 @@
       <c r="E29" t="s">
         <v>764</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="1">
         <v>45736</v>
       </c>
       <c r="G29" t="s">
@@ -5348,7 +5322,7 @@
       <c r="E30" t="s">
         <v>765</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="1">
         <v>45736</v>
       </c>
       <c r="G30" t="s">
@@ -5366,7 +5340,7 @@
       <c r="K30" t="s">
         <v>1165</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>45945</v>
       </c>
       <c r="P30" t="b">
@@ -5389,7 +5363,7 @@
       <c r="E31" t="s">
         <v>766</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="1">
         <v>45736</v>
       </c>
       <c r="G31" t="s">
@@ -5424,7 +5398,7 @@
       <c r="E32" t="s">
         <v>767</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="1">
         <v>45736</v>
       </c>
       <c r="G32" t="s">
@@ -5462,7 +5436,7 @@
       <c r="E33" t="s">
         <v>768</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="1">
         <v>45736</v>
       </c>
       <c r="G33" t="s">
@@ -5497,7 +5471,7 @@
       <c r="E34" t="s">
         <v>769</v>
       </c>
-      <c r="F34" s="2">
+      <c r="F34" s="1">
         <v>45736</v>
       </c>
       <c r="G34" t="s">
@@ -5526,7 +5500,7 @@
       <c r="E35" t="s">
         <v>770</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="1">
         <v>45736</v>
       </c>
       <c r="G35" t="s">
@@ -5555,7 +5529,7 @@
       <c r="E36" t="s">
         <v>771</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="1">
         <v>45736</v>
       </c>
       <c r="G36" t="s">
@@ -5590,7 +5564,7 @@
       <c r="E37" t="s">
         <v>772</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="1">
         <v>45736</v>
       </c>
       <c r="G37" t="s">
@@ -5625,7 +5599,7 @@
       <c r="E38" t="s">
         <v>752</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="1">
         <v>45736</v>
       </c>
       <c r="G38" t="s">
@@ -5657,7 +5631,7 @@
       <c r="D39" t="s">
         <v>644</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="1">
         <v>45736</v>
       </c>
       <c r="G39" t="s">
@@ -5692,7 +5666,7 @@
       <c r="D40" t="s">
         <v>644</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="1">
         <v>45736</v>
       </c>
       <c r="G40" t="s">
@@ -5730,7 +5704,7 @@
       <c r="E41" t="s">
         <v>773</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="1">
         <v>45736</v>
       </c>
       <c r="G41" t="s">
@@ -5765,7 +5739,7 @@
       <c r="E42" t="s">
         <v>774</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="1">
         <v>45736</v>
       </c>
       <c r="G42" t="s">
@@ -5800,7 +5774,7 @@
       <c r="E43" t="s">
         <v>775</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>45736</v>
       </c>
       <c r="G43" t="s">
@@ -5835,7 +5809,7 @@
       <c r="E44" t="s">
         <v>776</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="1">
         <v>45769</v>
       </c>
       <c r="G44" t="s">
@@ -5853,7 +5827,7 @@
       <c r="K44" t="s">
         <v>1168</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>45856</v>
       </c>
       <c r="O44" t="s">
@@ -5879,7 +5853,7 @@
       <c r="E45" t="s">
         <v>777</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="1">
         <v>45769</v>
       </c>
       <c r="G45" t="s">
@@ -5897,7 +5871,7 @@
       <c r="K45" t="s">
         <v>1169</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46100</v>
       </c>
       <c r="N45">
@@ -5923,7 +5897,7 @@
       <c r="E46" t="s">
         <v>778</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="1">
         <v>45769</v>
       </c>
       <c r="G46" t="s">
@@ -5961,7 +5935,7 @@
       <c r="E47" t="s">
         <v>779</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="1">
         <v>45769</v>
       </c>
       <c r="G47" t="s">
@@ -5979,7 +5953,7 @@
       <c r="K47" t="s">
         <v>1170</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46113</v>
       </c>
       <c r="O47" t="s">
@@ -6005,7 +5979,7 @@
       <c r="E48" t="s">
         <v>780</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="1">
         <v>45769</v>
       </c>
       <c r="G48" t="s">
@@ -6043,7 +6017,7 @@
       <c r="E49" t="s">
         <v>781</v>
       </c>
-      <c r="F49" s="2">
+      <c r="F49" s="1">
         <v>45769</v>
       </c>
       <c r="G49" t="s">
@@ -6072,7 +6046,7 @@
       <c r="E50" t="s">
         <v>782</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="1">
         <v>45769</v>
       </c>
       <c r="G50" t="s">
@@ -6110,7 +6084,7 @@
       <c r="E51" t="s">
         <v>783</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="1">
         <v>45769</v>
       </c>
       <c r="G51" t="s">
@@ -6145,7 +6119,7 @@
       <c r="E52" t="s">
         <v>784</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="1">
         <v>45769</v>
       </c>
       <c r="G52" t="s">
@@ -6183,7 +6157,7 @@
       <c r="E53" t="s">
         <v>785</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="1">
         <v>45769</v>
       </c>
       <c r="G53" t="s">
@@ -6221,7 +6195,7 @@
       <c r="E54" t="s">
         <v>786</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="1">
         <v>45769</v>
       </c>
       <c r="G54" t="s">
@@ -6259,7 +6233,7 @@
       <c r="E55" t="s">
         <v>787</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="1">
         <v>45769</v>
       </c>
       <c r="G55" t="s">
@@ -6288,7 +6262,7 @@
       <c r="E56" t="s">
         <v>788</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="1">
         <v>45769</v>
       </c>
       <c r="G56" t="s">
@@ -6323,7 +6297,7 @@
       <c r="E57" t="s">
         <v>789</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="1">
         <v>45769</v>
       </c>
       <c r="G57" t="s">
@@ -6361,7 +6335,7 @@
       <c r="E58" t="s">
         <v>790</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="1">
         <v>45769</v>
       </c>
       <c r="G58" t="s">
@@ -6390,7 +6364,7 @@
       <c r="E59" t="s">
         <v>791</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="1">
         <v>45769</v>
       </c>
       <c r="G59" t="s">
@@ -6425,7 +6399,7 @@
       <c r="E60" t="s">
         <v>792</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <v>45769</v>
       </c>
       <c r="G60" t="s">
@@ -6460,7 +6434,7 @@
       <c r="E61" t="s">
         <v>793</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="1">
         <v>45769</v>
       </c>
       <c r="G61" t="s">
@@ -6492,7 +6466,7 @@
       <c r="E62" t="s">
         <v>794</v>
       </c>
-      <c r="F62" s="2">
+      <c r="F62" s="1">
         <v>45770</v>
       </c>
       <c r="G62" t="s">
@@ -6521,7 +6495,7 @@
       <c r="E63" t="s">
         <v>795</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="1">
         <v>45799</v>
       </c>
       <c r="G63" t="s">
@@ -6539,7 +6513,7 @@
       <c r="K63" t="s">
         <v>1173</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46092</v>
       </c>
       <c r="O63" t="s">
@@ -6565,7 +6539,7 @@
       <c r="E64" t="s">
         <v>796</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="1">
         <v>45799</v>
       </c>
       <c r="G64" t="s">
@@ -6583,7 +6557,7 @@
       <c r="K64" t="s">
         <v>1174</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46119</v>
       </c>
       <c r="P64" t="b">
@@ -6606,7 +6580,7 @@
       <c r="E65" t="s">
         <v>797</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="1">
         <v>45799</v>
       </c>
       <c r="G65" t="s">
@@ -6641,7 +6615,7 @@
       <c r="E66" t="s">
         <v>798</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="1">
         <v>45799</v>
       </c>
       <c r="G66" t="s">
@@ -6676,7 +6650,7 @@
       <c r="E67" t="s">
         <v>799</v>
       </c>
-      <c r="F67" s="2">
+      <c r="F67" s="1">
         <v>45799</v>
       </c>
       <c r="G67" t="s">
@@ -6711,7 +6685,7 @@
       <c r="E68" t="s">
         <v>800</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="1">
         <v>45799</v>
       </c>
       <c r="G68" t="s">
@@ -6746,7 +6720,7 @@
       <c r="E69" t="s">
         <v>801</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>45803</v>
       </c>
       <c r="G69" t="s">
@@ -6781,7 +6755,7 @@
       <c r="E70" t="s">
         <v>802</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="1">
         <v>45803</v>
       </c>
       <c r="G70" t="s">
@@ -6819,7 +6793,7 @@
       <c r="E71" t="s">
         <v>803</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="1">
         <v>45803</v>
       </c>
       <c r="G71" t="s">
@@ -6854,7 +6828,7 @@
       <c r="E72" t="s">
         <v>804</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>45803</v>
       </c>
       <c r="G72" t="s">
@@ -6889,7 +6863,7 @@
       <c r="E73" t="s">
         <v>805</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="1">
         <v>45803</v>
       </c>
       <c r="G73" t="s">
@@ -6927,7 +6901,7 @@
       <c r="E74" t="s">
         <v>804</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="1">
         <v>45803</v>
       </c>
       <c r="G74" t="s">
@@ -6962,7 +6936,7 @@
       <c r="E75" t="s">
         <v>806</v>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="1">
         <v>45803</v>
       </c>
       <c r="G75" t="s">
@@ -7000,7 +6974,7 @@
       <c r="E76" t="s">
         <v>807</v>
       </c>
-      <c r="F76" s="2">
+      <c r="F76" s="1">
         <v>45803</v>
       </c>
       <c r="G76" t="s">
@@ -7035,7 +7009,7 @@
       <c r="E77" t="s">
         <v>808</v>
       </c>
-      <c r="F77" s="2">
+      <c r="F77" s="1">
         <v>45803</v>
       </c>
       <c r="G77" t="s">
@@ -7070,7 +7044,7 @@
       <c r="E78" t="s">
         <v>809</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="1">
         <v>45803</v>
       </c>
       <c r="G78" t="s">
@@ -7105,7 +7079,7 @@
       <c r="E79" t="s">
         <v>810</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="1">
         <v>45803</v>
       </c>
       <c r="G79" t="s">
@@ -7140,7 +7114,7 @@
       <c r="E80" t="s">
         <v>811</v>
       </c>
-      <c r="F80" s="2">
+      <c r="F80" s="1">
         <v>45803</v>
       </c>
       <c r="G80" t="s">
@@ -7178,7 +7152,7 @@
       <c r="E81" t="s">
         <v>812</v>
       </c>
-      <c r="F81" s="2">
+      <c r="F81" s="1">
         <v>45813</v>
       </c>
       <c r="G81" t="s">
@@ -7213,7 +7187,7 @@
       <c r="E82" t="s">
         <v>813</v>
       </c>
-      <c r="F82" s="2">
+      <c r="F82" s="1">
         <v>45813</v>
       </c>
       <c r="G82" t="s">
@@ -7251,7 +7225,7 @@
       <c r="E83" t="s">
         <v>814</v>
       </c>
-      <c r="F83" s="2">
+      <c r="F83" s="1">
         <v>45813</v>
       </c>
       <c r="G83" t="s">
@@ -7286,7 +7260,7 @@
       <c r="E84" t="s">
         <v>815</v>
       </c>
-      <c r="F84" s="2">
+      <c r="F84" s="1">
         <v>45813</v>
       </c>
       <c r="G84" t="s">
@@ -7304,7 +7278,7 @@
       <c r="K84" t="s">
         <v>1178</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>45853</v>
       </c>
       <c r="N84">
@@ -7330,7 +7304,7 @@
       <c r="E85" t="s">
         <v>816</v>
       </c>
-      <c r="F85" s="2">
+      <c r="F85" s="1">
         <v>45813</v>
       </c>
       <c r="G85" t="s">
@@ -7368,7 +7342,7 @@
       <c r="E86" t="s">
         <v>817</v>
       </c>
-      <c r="F86" s="2">
+      <c r="F86" s="1">
         <v>45813</v>
       </c>
       <c r="G86" t="s">
@@ -7406,7 +7380,7 @@
       <c r="E87" t="s">
         <v>818</v>
       </c>
-      <c r="F87" s="2">
+      <c r="F87" s="1">
         <v>45813</v>
       </c>
       <c r="G87" t="s">
@@ -7424,7 +7398,7 @@
       <c r="K87" t="s">
         <v>1179</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>45797</v>
       </c>
       <c r="N87" t="s">
@@ -7450,7 +7424,7 @@
       <c r="E88" t="s">
         <v>819</v>
       </c>
-      <c r="F88" s="2">
+      <c r="F88" s="1">
         <v>45813</v>
       </c>
       <c r="G88" t="s">
@@ -7485,7 +7459,7 @@
       <c r="E89" t="s">
         <v>820</v>
       </c>
-      <c r="F89" s="2">
+      <c r="F89" s="1">
         <v>45813</v>
       </c>
       <c r="G89" t="s">
@@ -7520,7 +7494,7 @@
       <c r="E90" t="s">
         <v>821</v>
       </c>
-      <c r="F90" s="2">
+      <c r="F90" s="1">
         <v>45831</v>
       </c>
       <c r="G90" t="s">
@@ -7561,7 +7535,7 @@
       <c r="E91" t="s">
         <v>822</v>
       </c>
-      <c r="F91" s="2">
+      <c r="F91" s="1">
         <v>45831</v>
       </c>
       <c r="G91" t="s">
@@ -7596,7 +7570,7 @@
       <c r="D92" t="s">
         <v>661</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="1">
         <v>45831</v>
       </c>
       <c r="G92" t="s">
@@ -7625,7 +7599,7 @@
       <c r="E93" t="s">
         <v>823</v>
       </c>
-      <c r="F93" s="2">
+      <c r="F93" s="1">
         <v>45831</v>
       </c>
       <c r="G93" t="s">
@@ -7663,7 +7637,7 @@
       <c r="E94" t="s">
         <v>824</v>
       </c>
-      <c r="F94" s="2">
+      <c r="F94" s="1">
         <v>45831</v>
       </c>
       <c r="G94" t="s">
@@ -7701,7 +7675,7 @@
       <c r="E95" t="s">
         <v>825</v>
       </c>
-      <c r="F95" s="2">
+      <c r="F95" s="1">
         <v>45831</v>
       </c>
       <c r="G95" t="s">
@@ -7739,7 +7713,7 @@
       <c r="E96" t="s">
         <v>826</v>
       </c>
-      <c r="F96" s="2">
+      <c r="F96" s="1">
         <v>45831</v>
       </c>
       <c r="G96" t="s">
@@ -7757,7 +7731,7 @@
       <c r="K96" t="s">
         <v>1153</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>45848</v>
       </c>
       <c r="N96" t="s">
@@ -7783,7 +7757,7 @@
       <c r="E97" t="s">
         <v>827</v>
       </c>
-      <c r="F97" s="2">
+      <c r="F97" s="1">
         <v>45840</v>
       </c>
       <c r="G97" t="s">
@@ -7824,7 +7798,7 @@
       <c r="E98" t="s">
         <v>828</v>
       </c>
-      <c r="F98" s="2">
+      <c r="F98" s="1">
         <v>45840</v>
       </c>
       <c r="G98" t="s">
@@ -7862,7 +7836,7 @@
       <c r="E99" t="s">
         <v>829</v>
       </c>
-      <c r="F99" s="2">
+      <c r="F99" s="1">
         <v>45840</v>
       </c>
       <c r="G99" t="s">
@@ -7891,7 +7865,7 @@
       <c r="E100" t="s">
         <v>830</v>
       </c>
-      <c r="F100" s="2">
+      <c r="F100" s="1">
         <v>45840</v>
       </c>
       <c r="G100" t="s">
@@ -7929,7 +7903,7 @@
       <c r="E101" t="s">
         <v>831</v>
       </c>
-      <c r="F101" s="2">
+      <c r="F101" s="1">
         <v>45840</v>
       </c>
       <c r="G101" t="s">
@@ -7958,7 +7932,7 @@
       <c r="E102" t="s">
         <v>832</v>
       </c>
-      <c r="F102" s="2">
+      <c r="F102" s="1">
         <v>45840</v>
       </c>
       <c r="G102" t="s">
@@ -7987,7 +7961,7 @@
       <c r="E103" t="s">
         <v>833</v>
       </c>
-      <c r="F103" s="2">
+      <c r="F103" s="1">
         <v>45840</v>
       </c>
       <c r="G103" t="s">
@@ -8016,7 +7990,7 @@
       <c r="E104" t="s">
         <v>834</v>
       </c>
-      <c r="F104" s="2">
+      <c r="F104" s="1">
         <v>45840</v>
       </c>
       <c r="G104" t="s">
@@ -8054,7 +8028,7 @@
       <c r="E105" t="s">
         <v>835</v>
       </c>
-      <c r="F105" s="2">
+      <c r="F105" s="1">
         <v>45840</v>
       </c>
       <c r="G105" t="s">
@@ -8092,7 +8066,7 @@
       <c r="E106" t="s">
         <v>836</v>
       </c>
-      <c r="F106" s="2">
+      <c r="F106" s="1">
         <v>45840</v>
       </c>
       <c r="G106" t="s">
@@ -8110,7 +8084,7 @@
       <c r="K106" t="s">
         <v>1182</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>45889</v>
       </c>
       <c r="P106" t="b">
@@ -8133,7 +8107,7 @@
       <c r="E107" t="s">
         <v>837</v>
       </c>
-      <c r="F107" s="2">
+      <c r="F107" s="1">
         <v>45840</v>
       </c>
       <c r="G107" t="s">
@@ -8151,7 +8125,7 @@
       <c r="K107" t="s">
         <v>1183</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>45876</v>
       </c>
       <c r="P107" t="b">
@@ -8174,7 +8148,7 @@
       <c r="E108" t="s">
         <v>838</v>
       </c>
-      <c r="F108" s="2">
+      <c r="F108" s="1">
         <v>45840</v>
       </c>
       <c r="G108" t="s">
@@ -8212,7 +8186,7 @@
       <c r="E109" t="s">
         <v>839</v>
       </c>
-      <c r="F109" s="2">
+      <c r="F109" s="1">
         <v>45840</v>
       </c>
       <c r="G109" t="s">
@@ -8250,7 +8224,7 @@
       <c r="E110" t="s">
         <v>840</v>
       </c>
-      <c r="F110" s="2">
+      <c r="F110" s="1">
         <v>45840</v>
       </c>
       <c r="G110" t="s">
@@ -8285,7 +8259,7 @@
       <c r="E111" t="s">
         <v>841</v>
       </c>
-      <c r="F111" s="2">
+      <c r="F111" s="1">
         <v>45840</v>
       </c>
       <c r="G111" t="s">
@@ -8320,7 +8294,7 @@
       <c r="E112" t="s">
         <v>842</v>
       </c>
-      <c r="F112" s="2">
+      <c r="F112" s="1">
         <v>45840</v>
       </c>
       <c r="G112" t="s">
@@ -8349,7 +8323,7 @@
       <c r="E113" t="s">
         <v>843</v>
       </c>
-      <c r="F113" s="2">
+      <c r="F113" s="1">
         <v>45840</v>
       </c>
       <c r="G113" t="s">
@@ -8384,7 +8358,7 @@
       <c r="E114" t="s">
         <v>844</v>
       </c>
-      <c r="F114" s="2">
+      <c r="F114" s="1">
         <v>45840</v>
       </c>
       <c r="G114" t="s">
@@ -8419,7 +8393,7 @@
       <c r="E115" t="s">
         <v>845</v>
       </c>
-      <c r="F115" s="2">
+      <c r="F115" s="1">
         <v>45840</v>
       </c>
       <c r="G115" t="s">
@@ -8457,7 +8431,7 @@
       <c r="E116" t="s">
         <v>846</v>
       </c>
-      <c r="F116" s="2">
+      <c r="F116" s="1">
         <v>45840</v>
       </c>
       <c r="G116" t="s">
@@ -8495,7 +8469,7 @@
       <c r="E117" t="s">
         <v>847</v>
       </c>
-      <c r="F117" s="2">
+      <c r="F117" s="1">
         <v>45840</v>
       </c>
       <c r="G117" t="s">
@@ -8533,7 +8507,7 @@
       <c r="E118" t="s">
         <v>848</v>
       </c>
-      <c r="F118" s="2">
+      <c r="F118" s="1">
         <v>45840</v>
       </c>
       <c r="G118" t="s">
@@ -8571,7 +8545,7 @@
       <c r="E119" t="s">
         <v>849</v>
       </c>
-      <c r="F119" s="2">
+      <c r="F119" s="1">
         <v>45840</v>
       </c>
       <c r="G119" t="s">
@@ -8609,7 +8583,7 @@
       <c r="E120" t="s">
         <v>850</v>
       </c>
-      <c r="F120" s="2">
+      <c r="F120" s="1">
         <v>45840</v>
       </c>
       <c r="G120" t="s">
@@ -8647,7 +8621,7 @@
       <c r="E121" t="s">
         <v>851</v>
       </c>
-      <c r="F121" s="2">
+      <c r="F121" s="1">
         <v>45849</v>
       </c>
       <c r="G121" t="s">
@@ -8665,7 +8639,7 @@
       <c r="K121" t="s">
         <v>1169</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46100</v>
       </c>
       <c r="N121">
@@ -8691,7 +8665,7 @@
       <c r="E122" t="s">
         <v>852</v>
       </c>
-      <c r="F122" s="2">
+      <c r="F122" s="1">
         <v>45849</v>
       </c>
       <c r="G122" t="s">
@@ -8729,7 +8703,7 @@
       <c r="E123" t="s">
         <v>853</v>
       </c>
-      <c r="F123" s="2">
+      <c r="F123" s="1">
         <v>45849</v>
       </c>
       <c r="G123" t="s">
@@ -8758,7 +8732,7 @@
       <c r="E124" t="s">
         <v>854</v>
       </c>
-      <c r="F124" s="2">
+      <c r="F124" s="1">
         <v>45853</v>
       </c>
       <c r="G124" t="s">
@@ -8796,7 +8770,7 @@
       <c r="E125" t="s">
         <v>855</v>
       </c>
-      <c r="F125" s="2">
+      <c r="F125" s="1">
         <v>45855</v>
       </c>
       <c r="G125" t="s">
@@ -8834,7 +8808,7 @@
       <c r="E126" t="s">
         <v>856</v>
       </c>
-      <c r="F126" s="2">
+      <c r="F126" s="1">
         <v>45855</v>
       </c>
       <c r="G126" t="s">
@@ -8869,7 +8843,7 @@
       <c r="E127" t="s">
         <v>857</v>
       </c>
-      <c r="F127" s="2">
+      <c r="F127" s="1">
         <v>45856</v>
       </c>
       <c r="G127" t="s">
@@ -8898,7 +8872,7 @@
       <c r="E128" t="s">
         <v>858</v>
       </c>
-      <c r="F128" s="2">
+      <c r="F128" s="1">
         <v>45869</v>
       </c>
       <c r="G128" t="s">
@@ -8936,7 +8910,7 @@
       <c r="E129" t="s">
         <v>859</v>
       </c>
-      <c r="F129" s="2">
+      <c r="F129" s="1">
         <v>45869</v>
       </c>
       <c r="G129" t="s">
@@ -8974,7 +8948,7 @@
       <c r="E130" t="s">
         <v>860</v>
       </c>
-      <c r="F130" s="2">
+      <c r="F130" s="1">
         <v>45869</v>
       </c>
       <c r="G130" t="s">
@@ -8992,7 +8966,7 @@
       <c r="K130" t="s">
         <v>1187</v>
       </c>
-      <c r="M130" s="2">
+      <c r="M130" s="1">
         <v>45916</v>
       </c>
       <c r="N130">
@@ -9018,7 +8992,7 @@
       <c r="E131" t="s">
         <v>861</v>
       </c>
-      <c r="F131" s="2">
+      <c r="F131" s="1">
         <v>45869</v>
       </c>
       <c r="G131" t="s">
@@ -9053,7 +9027,7 @@
       <c r="E132" t="s">
         <v>862</v>
       </c>
-      <c r="F132" s="2">
+      <c r="F132" s="1">
         <v>45869</v>
       </c>
       <c r="G132" t="s">
@@ -9071,7 +9045,7 @@
       <c r="K132" t="s">
         <v>1189</v>
       </c>
-      <c r="M132" s="2">
+      <c r="M132" s="1">
         <v>46014</v>
       </c>
       <c r="N132">
@@ -9097,7 +9071,7 @@
       <c r="E133" t="s">
         <v>863</v>
       </c>
-      <c r="F133" s="2">
+      <c r="F133" s="1">
         <v>45869</v>
       </c>
       <c r="G133" t="s">
@@ -9126,7 +9100,7 @@
       <c r="E134" t="s">
         <v>864</v>
       </c>
-      <c r="F134" s="2">
+      <c r="F134" s="1">
         <v>45882</v>
       </c>
       <c r="G134" t="s">
@@ -9164,7 +9138,7 @@
       <c r="E135" t="s">
         <v>865</v>
       </c>
-      <c r="F135" s="2">
+      <c r="F135" s="1">
         <v>45882</v>
       </c>
       <c r="G135" t="s">
@@ -9193,7 +9167,7 @@
       <c r="E136" t="s">
         <v>866</v>
       </c>
-      <c r="F136" s="2">
+      <c r="F136" s="1">
         <v>45891</v>
       </c>
       <c r="G136" t="s">
@@ -9222,7 +9196,7 @@
       <c r="E137" t="s">
         <v>867</v>
       </c>
-      <c r="F137" s="2">
+      <c r="F137" s="1">
         <v>45891</v>
       </c>
       <c r="G137" t="s">
@@ -9251,7 +9225,7 @@
       <c r="E138" t="s">
         <v>868</v>
       </c>
-      <c r="F138" s="2">
+      <c r="F138" s="1">
         <v>45891</v>
       </c>
       <c r="G138" t="s">
@@ -9289,7 +9263,7 @@
       <c r="E139" t="s">
         <v>869</v>
       </c>
-      <c r="F139" s="2">
+      <c r="F139" s="1">
         <v>45891</v>
       </c>
       <c r="G139" t="s">
@@ -9318,7 +9292,7 @@
       <c r="E140" t="s">
         <v>870</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140" s="1">
         <v>45891</v>
       </c>
       <c r="G140" t="s">
@@ -9353,7 +9327,7 @@
       <c r="E141" t="s">
         <v>871</v>
       </c>
-      <c r="F141" s="2">
+      <c r="F141" s="1">
         <v>45891</v>
       </c>
       <c r="G141" t="s">
@@ -9382,7 +9356,7 @@
       <c r="E142" t="s">
         <v>872</v>
       </c>
-      <c r="F142" s="2">
+      <c r="F142" s="1">
         <v>45891</v>
       </c>
       <c r="G142" t="s">
@@ -9411,7 +9385,7 @@
       <c r="E143" t="s">
         <v>873</v>
       </c>
-      <c r="F143" s="2">
+      <c r="F143" s="1">
         <v>45891</v>
       </c>
       <c r="G143" t="s">
@@ -9440,7 +9414,7 @@
       <c r="E144" t="s">
         <v>874</v>
       </c>
-      <c r="F144" s="2">
+      <c r="F144" s="1">
         <v>45891</v>
       </c>
       <c r="G144" t="s">
@@ -9469,7 +9443,7 @@
       <c r="E145" t="s">
         <v>875</v>
       </c>
-      <c r="F145" s="2">
+      <c r="F145" s="1">
         <v>45891</v>
       </c>
       <c r="G145" t="s">
@@ -9504,7 +9478,7 @@
       <c r="E146" t="s">
         <v>876</v>
       </c>
-      <c r="F146" s="2">
+      <c r="F146" s="1">
         <v>45891</v>
       </c>
       <c r="G146" t="s">
@@ -9533,7 +9507,7 @@
       <c r="E147" t="s">
         <v>877</v>
       </c>
-      <c r="F147" s="2">
+      <c r="F147" s="1">
         <v>45891</v>
       </c>
       <c r="G147" t="s">
@@ -9568,7 +9542,7 @@
       <c r="E148" t="s">
         <v>878</v>
       </c>
-      <c r="F148" s="2">
+      <c r="F148" s="1">
         <v>45891</v>
       </c>
       <c r="G148" t="s">
@@ -9606,7 +9580,7 @@
       <c r="E149" t="s">
         <v>879</v>
       </c>
-      <c r="F149" s="2">
+      <c r="F149" s="1">
         <v>45891</v>
       </c>
       <c r="G149" t="s">
@@ -9641,7 +9615,7 @@
       <c r="E150" t="s">
         <v>880</v>
       </c>
-      <c r="F150" s="2">
+      <c r="F150" s="1">
         <v>45891</v>
       </c>
       <c r="G150" t="s">
@@ -9659,7 +9633,7 @@
       <c r="K150" t="s">
         <v>1173</v>
       </c>
-      <c r="M150" s="2">
+      <c r="M150" s="1">
         <v>46092</v>
       </c>
       <c r="O150" t="s">
@@ -9685,7 +9659,7 @@
       <c r="E151" t="s">
         <v>881</v>
       </c>
-      <c r="F151" s="2">
+      <c r="F151" s="1">
         <v>45891</v>
       </c>
       <c r="G151" t="s">
@@ -9720,7 +9694,7 @@
       <c r="E152" t="s">
         <v>871</v>
       </c>
-      <c r="F152" s="2">
+      <c r="F152" s="1">
         <v>45891</v>
       </c>
       <c r="G152" t="s">
@@ -9738,7 +9712,7 @@
       <c r="K152" t="s">
         <v>1174</v>
       </c>
-      <c r="M152" s="2">
+      <c r="M152" s="1">
         <v>46119</v>
       </c>
       <c r="P152" t="b">
@@ -9761,7 +9735,7 @@
       <c r="E153" t="s">
         <v>882</v>
       </c>
-      <c r="F153" s="2">
+      <c r="F153" s="1">
         <v>45891</v>
       </c>
       <c r="G153" t="s">
@@ -9799,7 +9773,7 @@
       <c r="E154" t="s">
         <v>883</v>
       </c>
-      <c r="F154" s="2">
+      <c r="F154" s="1">
         <v>45891</v>
       </c>
       <c r="G154" t="s">
@@ -9834,7 +9808,7 @@
       <c r="E155" t="s">
         <v>884</v>
       </c>
-      <c r="F155" s="2">
+      <c r="F155" s="1">
         <v>45891</v>
       </c>
       <c r="G155" t="s">
@@ -9869,7 +9843,7 @@
       <c r="E156" t="s">
         <v>885</v>
       </c>
-      <c r="F156" s="2">
+      <c r="F156" s="1">
         <v>45891</v>
       </c>
       <c r="G156" t="s">
@@ -9907,7 +9881,7 @@
       <c r="E157" t="s">
         <v>886</v>
       </c>
-      <c r="F157" s="2">
+      <c r="F157" s="1">
         <v>45891</v>
       </c>
       <c r="G157" t="s">
@@ -9945,7 +9919,7 @@
       <c r="E158" t="s">
         <v>887</v>
       </c>
-      <c r="F158" s="2">
+      <c r="F158" s="1">
         <v>45894</v>
       </c>
       <c r="G158" t="s">
@@ -9963,7 +9937,7 @@
       <c r="K158" t="s">
         <v>1192</v>
       </c>
-      <c r="M158" s="2">
+      <c r="M158" s="1">
         <v>45946</v>
       </c>
       <c r="P158" t="b">
@@ -9986,7 +9960,7 @@
       <c r="E159" t="s">
         <v>888</v>
       </c>
-      <c r="F159" s="2">
+      <c r="F159" s="1">
         <v>45894</v>
       </c>
       <c r="G159" t="s">
@@ -10024,7 +9998,7 @@
       <c r="E160" t="s">
         <v>889</v>
       </c>
-      <c r="F160" s="2">
+      <c r="F160" s="1">
         <v>45898</v>
       </c>
       <c r="G160" t="s">
@@ -10062,7 +10036,7 @@
       <c r="E161" t="s">
         <v>890</v>
       </c>
-      <c r="F161" s="2">
+      <c r="F161" s="1">
         <v>45898</v>
       </c>
       <c r="G161" t="s">
@@ -10080,7 +10054,7 @@
       <c r="K161" t="s">
         <v>1193</v>
       </c>
-      <c r="M161" s="2">
+      <c r="M161" s="1">
         <v>45953</v>
       </c>
       <c r="N161" t="s">
@@ -10106,7 +10080,7 @@
       <c r="E162" t="s">
         <v>891</v>
       </c>
-      <c r="F162" s="2">
+      <c r="F162" s="1">
         <v>45898</v>
       </c>
       <c r="G162" t="s">
@@ -10124,7 +10098,7 @@
       <c r="K162" t="s">
         <v>1194</v>
       </c>
-      <c r="M162" s="2">
+      <c r="M162" s="1">
         <v>45940</v>
       </c>
       <c r="P162" t="b">
@@ -10147,7 +10121,7 @@
       <c r="E163" t="s">
         <v>892</v>
       </c>
-      <c r="F163" s="2">
+      <c r="F163" s="1">
         <v>45898</v>
       </c>
       <c r="G163" t="s">
@@ -10165,7 +10139,7 @@
       <c r="K163" t="s">
         <v>1194</v>
       </c>
-      <c r="M163" s="2">
+      <c r="M163" s="1">
         <v>45940</v>
       </c>
       <c r="P163" t="b">
@@ -10188,7 +10162,7 @@
       <c r="E164" t="s">
         <v>893</v>
       </c>
-      <c r="F164" s="2">
+      <c r="F164" s="1">
         <v>45910</v>
       </c>
       <c r="G164" t="s">
@@ -10223,7 +10197,7 @@
       <c r="E165" t="s">
         <v>894</v>
       </c>
-      <c r="F165" s="2">
+      <c r="F165" s="1">
         <v>45917</v>
       </c>
       <c r="G165" t="s">
@@ -10264,7 +10238,7 @@
       <c r="E166" t="s">
         <v>895</v>
       </c>
-      <c r="F166" s="2">
+      <c r="F166" s="1">
         <v>45917</v>
       </c>
       <c r="G166" t="s">
@@ -10299,7 +10273,7 @@
       <c r="E167" t="s">
         <v>896</v>
       </c>
-      <c r="F167" s="2">
+      <c r="F167" s="1">
         <v>45917</v>
       </c>
       <c r="G167" t="s">
@@ -10328,7 +10302,7 @@
       <c r="E168" t="s">
         <v>897</v>
       </c>
-      <c r="F168" s="2">
+      <c r="F168" s="1">
         <v>45917</v>
       </c>
       <c r="G168" t="s">
@@ -10369,7 +10343,7 @@
       <c r="E169" t="s">
         <v>898</v>
       </c>
-      <c r="F169" s="2">
+      <c r="F169" s="1">
         <v>45917</v>
       </c>
       <c r="G169" t="s">
@@ -10387,7 +10361,7 @@
       <c r="K169" t="s">
         <v>1197</v>
       </c>
-      <c r="M169" s="2">
+      <c r="M169" s="1">
         <v>45973</v>
       </c>
       <c r="P169" t="b">
@@ -10410,7 +10384,7 @@
       <c r="E170" t="s">
         <v>899</v>
       </c>
-      <c r="F170" s="2">
+      <c r="F170" s="1">
         <v>45917</v>
       </c>
       <c r="G170" t="s">
@@ -10445,7 +10419,7 @@
       <c r="E171" t="s">
         <v>900</v>
       </c>
-      <c r="F171" s="2">
+      <c r="F171" s="1">
         <v>45917</v>
       </c>
       <c r="G171" t="s">
@@ -10483,7 +10457,7 @@
       <c r="E172" t="s">
         <v>901</v>
       </c>
-      <c r="F172" s="2">
+      <c r="F172" s="1">
         <v>45917</v>
       </c>
       <c r="G172" t="s">
@@ -10518,7 +10492,7 @@
       <c r="E173" t="s">
         <v>902</v>
       </c>
-      <c r="F173" s="2">
+      <c r="F173" s="1">
         <v>45917</v>
       </c>
       <c r="G173" t="s">
@@ -10553,7 +10527,7 @@
       <c r="E174" t="s">
         <v>903</v>
       </c>
-      <c r="F174" s="2">
+      <c r="F174" s="1">
         <v>45917</v>
       </c>
       <c r="G174" t="s">
@@ -10588,7 +10562,7 @@
       <c r="E175" t="s">
         <v>904</v>
       </c>
-      <c r="F175" s="2">
+      <c r="F175" s="1">
         <v>45917</v>
       </c>
       <c r="G175" t="s">
@@ -10606,7 +10580,7 @@
       <c r="K175" t="s">
         <v>1198</v>
       </c>
-      <c r="M175" s="2">
+      <c r="M175" s="1">
         <v>46122</v>
       </c>
       <c r="O175" t="s">
@@ -10632,7 +10606,7 @@
       <c r="E176" t="s">
         <v>808</v>
       </c>
-      <c r="F176" s="2">
+      <c r="F176" s="1">
         <v>45917</v>
       </c>
       <c r="G176" t="s">
@@ -10670,7 +10644,7 @@
       <c r="E177" t="s">
         <v>905</v>
       </c>
-      <c r="F177" s="2">
+      <c r="F177" s="1">
         <v>45917</v>
       </c>
       <c r="G177" t="s">
@@ -10688,7 +10662,7 @@
       <c r="K177" t="s">
         <v>1199</v>
       </c>
-      <c r="M177" s="2">
+      <c r="M177" s="1">
         <v>45961</v>
       </c>
       <c r="O177" t="s">
@@ -10714,7 +10688,7 @@
       <c r="E178" t="s">
         <v>906</v>
       </c>
-      <c r="F178" s="2">
+      <c r="F178" s="1">
         <v>45937</v>
       </c>
       <c r="G178" t="s">
@@ -10752,7 +10726,7 @@
       <c r="E179" t="s">
         <v>907</v>
       </c>
-      <c r="F179" s="2">
+      <c r="F179" s="1">
         <v>45937</v>
       </c>
       <c r="G179" t="s">
@@ -10781,7 +10755,7 @@
       <c r="E180" t="s">
         <v>908</v>
       </c>
-      <c r="F180" s="2">
+      <c r="F180" s="1">
         <v>45937</v>
       </c>
       <c r="G180" t="s">
@@ -10819,7 +10793,7 @@
       <c r="E181" t="s">
         <v>909</v>
       </c>
-      <c r="F181" s="2">
+      <c r="F181" s="1">
         <v>45937</v>
       </c>
       <c r="G181" t="s">
@@ -10854,7 +10828,7 @@
       <c r="E182" t="s">
         <v>910</v>
       </c>
-      <c r="F182" s="2">
+      <c r="F182" s="1">
         <v>45937</v>
       </c>
       <c r="G182" t="s">
@@ -10883,7 +10857,7 @@
       <c r="E183" t="s">
         <v>911</v>
       </c>
-      <c r="F183" s="2">
+      <c r="F183" s="1">
         <v>45937</v>
       </c>
       <c r="G183" t="s">
@@ -10918,7 +10892,7 @@
       <c r="D184" t="s">
         <v>687</v>
       </c>
-      <c r="F184" s="2">
+      <c r="F184" s="1">
         <v>45939</v>
       </c>
       <c r="G184" t="s">
@@ -10953,7 +10927,7 @@
       <c r="E185" t="s">
         <v>912</v>
       </c>
-      <c r="F185" s="2">
+      <c r="F185" s="1">
         <v>45939</v>
       </c>
       <c r="G185" t="s">
@@ -10991,7 +10965,7 @@
       <c r="E186" t="s">
         <v>913</v>
       </c>
-      <c r="F186" s="2">
+      <c r="F186" s="1">
         <v>45939</v>
       </c>
       <c r="G186" t="s">
@@ -11029,7 +11003,7 @@
       <c r="E187" t="s">
         <v>914</v>
       </c>
-      <c r="F187" s="2">
+      <c r="F187" s="1">
         <v>45939</v>
       </c>
       <c r="G187" t="s">
@@ -11047,7 +11021,7 @@
       <c r="K187" t="s">
         <v>1201</v>
       </c>
-      <c r="M187" s="2">
+      <c r="M187" s="1">
         <v>46014</v>
       </c>
       <c r="N187">
@@ -11073,7 +11047,7 @@
       <c r="E188" t="s">
         <v>915</v>
       </c>
-      <c r="F188" s="2">
+      <c r="F188" s="1">
         <v>45946</v>
       </c>
       <c r="G188" t="s">
@@ -11091,7 +11065,7 @@
       <c r="K188" t="s">
         <v>1202</v>
       </c>
-      <c r="M188" s="2">
+      <c r="M188" s="1">
         <v>45986</v>
       </c>
       <c r="O188" t="s">
@@ -11117,7 +11091,7 @@
       <c r="E189" t="s">
         <v>916</v>
       </c>
-      <c r="F189" s="2">
+      <c r="F189" s="1">
         <v>45965</v>
       </c>
       <c r="G189" t="s">
@@ -11135,7 +11109,7 @@
       <c r="K189" t="s">
         <v>1203</v>
       </c>
-      <c r="M189" s="2">
+      <c r="M189" s="1">
         <v>46120</v>
       </c>
       <c r="P189" t="b">
@@ -11158,7 +11132,7 @@
       <c r="E190" t="s">
         <v>917</v>
       </c>
-      <c r="F190" s="2">
+      <c r="F190" s="1">
         <v>45965</v>
       </c>
       <c r="G190" t="s">
@@ -11196,7 +11170,7 @@
       <c r="E191" t="s">
         <v>918</v>
       </c>
-      <c r="F191" s="2">
+      <c r="F191" s="1">
         <v>45967</v>
       </c>
       <c r="G191" t="s">
@@ -11214,7 +11188,7 @@
       <c r="K191" t="s">
         <v>1204</v>
       </c>
-      <c r="M191" s="2">
+      <c r="M191" s="1">
         <v>45972</v>
       </c>
       <c r="P191" t="b">
@@ -11237,7 +11211,7 @@
       <c r="E192" t="s">
         <v>919</v>
       </c>
-      <c r="F192" s="2">
+      <c r="F192" s="1">
         <v>45968</v>
       </c>
       <c r="G192" t="s">
@@ -11275,7 +11249,7 @@
       <c r="E193" t="s">
         <v>920</v>
       </c>
-      <c r="F193" s="2">
+      <c r="F193" s="1">
         <v>45968</v>
       </c>
       <c r="G193" t="s">
@@ -11313,7 +11287,7 @@
       <c r="E194" t="s">
         <v>921</v>
       </c>
-      <c r="F194" s="2">
+      <c r="F194" s="1">
         <v>45968</v>
       </c>
       <c r="G194" t="s">
@@ -11342,7 +11316,7 @@
       <c r="E195" t="s">
         <v>922</v>
       </c>
-      <c r="F195" s="2">
+      <c r="F195" s="1">
         <v>45971</v>
       </c>
       <c r="G195" t="s">
@@ -11380,7 +11354,7 @@
       <c r="E196" t="s">
         <v>923</v>
       </c>
-      <c r="F196" s="2">
+      <c r="F196" s="1">
         <v>45978</v>
       </c>
       <c r="G196" t="s">
@@ -11409,7 +11383,7 @@
       <c r="E197" t="s">
         <v>924</v>
       </c>
-      <c r="F197" s="2">
+      <c r="F197" s="1">
         <v>45978</v>
       </c>
       <c r="G197" t="s">
@@ -11438,7 +11412,7 @@
       <c r="E198" t="s">
         <v>925</v>
       </c>
-      <c r="F198" s="2">
+      <c r="F198" s="1">
         <v>45978</v>
       </c>
       <c r="G198" t="s">
@@ -11467,7 +11441,7 @@
       <c r="E199" t="s">
         <v>926</v>
       </c>
-      <c r="F199" s="2">
+      <c r="F199" s="1">
         <v>45979</v>
       </c>
       <c r="G199" t="s">
@@ -11485,7 +11459,7 @@
       <c r="K199" t="s">
         <v>1205</v>
       </c>
-      <c r="M199" s="2">
+      <c r="M199" s="1">
         <v>46049</v>
       </c>
       <c r="P199" t="b">
@@ -11508,7 +11482,7 @@
       <c r="E200" t="s">
         <v>927</v>
       </c>
-      <c r="F200" s="2">
+      <c r="F200" s="1">
         <v>45986</v>
       </c>
       <c r="G200" t="s">
@@ -11546,7 +11520,7 @@
       <c r="E201" t="s">
         <v>928</v>
       </c>
-      <c r="F201" s="2">
+      <c r="F201" s="1">
         <v>45986</v>
       </c>
       <c r="G201" t="s">
@@ -11584,7 +11558,7 @@
       <c r="E202" t="s">
         <v>929</v>
       </c>
-      <c r="F202" s="2">
+      <c r="F202" s="1">
         <v>45986</v>
       </c>
       <c r="G202" t="s">
@@ -11622,7 +11596,7 @@
       <c r="E203" t="s">
         <v>930</v>
       </c>
-      <c r="F203" s="2">
+      <c r="F203" s="1">
         <v>45986</v>
       </c>
       <c r="G203" t="s">
@@ -11660,7 +11634,7 @@
       <c r="E204" t="s">
         <v>931</v>
       </c>
-      <c r="F204" s="2">
+      <c r="F204" s="1">
         <v>45986</v>
       </c>
       <c r="G204" t="s">
@@ -11698,7 +11672,7 @@
       <c r="E205" t="s">
         <v>932</v>
       </c>
-      <c r="F205" s="2">
+      <c r="F205" s="1">
         <v>45986</v>
       </c>
       <c r="G205" t="s">
@@ -11736,7 +11710,7 @@
       <c r="E206" t="s">
         <v>933</v>
       </c>
-      <c r="F206" s="2">
+      <c r="F206" s="1">
         <v>45986</v>
       </c>
       <c r="G206" t="s">
@@ -11771,7 +11745,7 @@
       <c r="E207" t="s">
         <v>934</v>
       </c>
-      <c r="F207" s="2">
+      <c r="F207" s="1">
         <v>45986</v>
       </c>
       <c r="G207" t="s">
@@ -11789,7 +11763,7 @@
       <c r="K207" t="s">
         <v>1207</v>
       </c>
-      <c r="M207" s="2">
+      <c r="M207" s="1">
         <v>46153</v>
       </c>
       <c r="P207" t="b">
@@ -11812,7 +11786,7 @@
       <c r="E208" t="s">
         <v>935</v>
       </c>
-      <c r="F208" s="2">
+      <c r="F208" s="1">
         <v>45986</v>
       </c>
       <c r="G208" t="s">
@@ -11830,7 +11804,7 @@
       <c r="K208" t="s">
         <v>1208</v>
       </c>
-      <c r="M208" s="2">
+      <c r="M208" s="1">
         <v>46031</v>
       </c>
       <c r="P208" t="b">
@@ -11853,7 +11827,7 @@
       <c r="E209" t="s">
         <v>936</v>
       </c>
-      <c r="F209" s="2">
+      <c r="F209" s="1">
         <v>46000</v>
       </c>
       <c r="G209" t="s">
@@ -11871,7 +11845,7 @@
       <c r="K209" t="s">
         <v>1209</v>
       </c>
-      <c r="M209" s="2">
+      <c r="M209" s="1">
         <v>46191</v>
       </c>
       <c r="P209" t="b">
@@ -11894,7 +11868,7 @@
       <c r="E210" t="s">
         <v>937</v>
       </c>
-      <c r="F210" s="2">
+      <c r="F210" s="1">
         <v>46000</v>
       </c>
       <c r="G210" t="s">
@@ -11932,7 +11906,7 @@
       <c r="E211" t="s">
         <v>938</v>
       </c>
-      <c r="F211" s="2">
+      <c r="F211" s="1">
         <v>46000</v>
       </c>
       <c r="G211" t="s">
@@ -11967,7 +11941,7 @@
       <c r="E212" t="s">
         <v>939</v>
       </c>
-      <c r="F212" s="2">
+      <c r="F212" s="1">
         <v>46000</v>
       </c>
       <c r="G212" t="s">
@@ -12002,7 +11976,7 @@
       <c r="E213" t="s">
         <v>940</v>
       </c>
-      <c r="F213" s="2">
+      <c r="F213" s="1">
         <v>46007</v>
       </c>
       <c r="G213" t="s">
@@ -12040,7 +12014,7 @@
       <c r="E214" t="s">
         <v>941</v>
       </c>
-      <c r="F214" s="2">
+      <c r="F214" s="1">
         <v>46007</v>
       </c>
       <c r="G214" t="s">
@@ -12058,7 +12032,7 @@
       <c r="K214" t="s">
         <v>1212</v>
       </c>
-      <c r="M214" s="2">
+      <c r="M214" s="1">
         <v>46021</v>
       </c>
       <c r="N214">
@@ -12084,7 +12058,7 @@
       <c r="E215" t="s">
         <v>942</v>
       </c>
-      <c r="F215" s="2">
+      <c r="F215" s="1">
         <v>46007</v>
       </c>
       <c r="G215" t="s">
@@ -12122,7 +12096,7 @@
       <c r="E216" t="s">
         <v>943</v>
       </c>
-      <c r="F216" s="2">
+      <c r="F216" s="1">
         <v>46010</v>
       </c>
       <c r="G216" t="s">
@@ -12151,7 +12125,7 @@
       <c r="E217" t="s">
         <v>944</v>
       </c>
-      <c r="F217" s="2">
+      <c r="F217" s="1">
         <v>46010</v>
       </c>
       <c r="G217" t="s">
@@ -12169,7 +12143,7 @@
       <c r="K217" t="s">
         <v>1213</v>
       </c>
-      <c r="M217" s="2">
+      <c r="M217" s="1">
         <v>46052</v>
       </c>
       <c r="P217" t="b">
@@ -12192,7 +12166,7 @@
       <c r="E218" t="s">
         <v>945</v>
       </c>
-      <c r="F218" s="2">
+      <c r="F218" s="1">
         <v>46010</v>
       </c>
       <c r="G218" t="s">
@@ -12230,7 +12204,7 @@
       <c r="E219" t="s">
         <v>946</v>
       </c>
-      <c r="F219" s="2">
+      <c r="F219" s="1">
         <v>46010</v>
       </c>
       <c r="G219" t="s">
@@ -12268,7 +12242,7 @@
       <c r="E220" t="s">
         <v>947</v>
       </c>
-      <c r="F220" s="2">
+      <c r="F220" s="1">
         <v>46010</v>
       </c>
       <c r="G220" t="s">
@@ -12306,7 +12280,7 @@
       <c r="E221" t="s">
         <v>948</v>
       </c>
-      <c r="F221" s="2">
+      <c r="F221" s="1">
         <v>46028</v>
       </c>
       <c r="G221" t="s">
@@ -12341,7 +12315,7 @@
       <c r="E222" t="s">
         <v>949</v>
       </c>
-      <c r="F222" s="2">
+      <c r="F222" s="1">
         <v>46028</v>
       </c>
       <c r="G222" t="s">
@@ -12379,7 +12353,7 @@
       <c r="E223" t="s">
         <v>950</v>
       </c>
-      <c r="F223" s="2">
+      <c r="F223" s="1">
         <v>46028</v>
       </c>
       <c r="G223" t="s">
@@ -12417,7 +12391,7 @@
       <c r="E224" t="s">
         <v>951</v>
       </c>
-      <c r="F224" s="2">
+      <c r="F224" s="1">
         <v>46028</v>
       </c>
       <c r="G224" t="s">
@@ -12455,7 +12429,7 @@
       <c r="E225" t="s">
         <v>952</v>
       </c>
-      <c r="F225" s="2">
+      <c r="F225" s="1">
         <v>46028</v>
       </c>
       <c r="G225" t="s">
@@ -12493,7 +12467,7 @@
       <c r="E226" t="s">
         <v>953</v>
       </c>
-      <c r="F226" s="2">
+      <c r="F226" s="1">
         <v>46028</v>
       </c>
       <c r="G226" t="s">
@@ -12531,7 +12505,7 @@
       <c r="E227" t="s">
         <v>954</v>
       </c>
-      <c r="F227" s="2">
+      <c r="F227" s="1">
         <v>46028</v>
       </c>
       <c r="G227" t="s">
@@ -12569,7 +12543,7 @@
       <c r="E228" t="s">
         <v>955</v>
       </c>
-      <c r="F228" s="2">
+      <c r="F228" s="1">
         <v>46028</v>
       </c>
       <c r="G228" t="s">
@@ -12607,7 +12581,7 @@
       <c r="E229" t="s">
         <v>956</v>
       </c>
-      <c r="F229" s="2">
+      <c r="F229" s="1">
         <v>46028</v>
       </c>
       <c r="G229" t="s">
@@ -12642,7 +12616,7 @@
       <c r="E230" t="s">
         <v>957</v>
       </c>
-      <c r="F230" s="2">
+      <c r="F230" s="1">
         <v>46028</v>
       </c>
       <c r="G230" t="s">
@@ -12680,7 +12654,7 @@
       <c r="E231" t="s">
         <v>958</v>
       </c>
-      <c r="F231" s="2">
+      <c r="F231" s="1">
         <v>46028</v>
       </c>
       <c r="G231" t="s">
@@ -12698,7 +12672,7 @@
       <c r="K231" t="s">
         <v>1214</v>
       </c>
-      <c r="M231" s="2">
+      <c r="M231" s="1">
         <v>46063</v>
       </c>
       <c r="P231" t="b">
@@ -12721,7 +12695,7 @@
       <c r="E232" t="s">
         <v>959</v>
       </c>
-      <c r="F232" s="2">
+      <c r="F232" s="1">
         <v>46028</v>
       </c>
       <c r="G232" t="s">
@@ -12756,7 +12730,7 @@
       <c r="E233" t="s">
         <v>960</v>
       </c>
-      <c r="F233" s="2">
+      <c r="F233" s="1">
         <v>46028</v>
       </c>
       <c r="G233" t="s">
@@ -12791,7 +12765,7 @@
       <c r="E234" t="s">
         <v>961</v>
       </c>
-      <c r="F234" s="2">
+      <c r="F234" s="1">
         <v>46028</v>
       </c>
       <c r="G234" t="s">
@@ -12809,7 +12783,7 @@
       <c r="K234" t="s">
         <v>1214</v>
       </c>
-      <c r="M234" s="2">
+      <c r="M234" s="1">
         <v>46063</v>
       </c>
       <c r="O234" t="s">
@@ -12835,7 +12809,7 @@
       <c r="E235" t="s">
         <v>962</v>
       </c>
-      <c r="F235" s="2">
+      <c r="F235" s="1">
         <v>46028</v>
       </c>
       <c r="G235" t="s">
@@ -12853,7 +12827,7 @@
       <c r="K235" t="s">
         <v>1214</v>
       </c>
-      <c r="M235" s="2">
+      <c r="M235" s="1">
         <v>46063</v>
       </c>
       <c r="O235" t="s">
@@ -12879,7 +12853,7 @@
       <c r="E236" t="s">
         <v>963</v>
       </c>
-      <c r="F236" s="2">
+      <c r="F236" s="1">
         <v>46028</v>
       </c>
       <c r="G236" t="s">
@@ -12897,7 +12871,7 @@
       <c r="K236" t="s">
         <v>1216</v>
       </c>
-      <c r="M236" s="2">
+      <c r="M236" s="1">
         <v>46114</v>
       </c>
       <c r="P236" t="b">
@@ -12920,7 +12894,7 @@
       <c r="E237" t="s">
         <v>964</v>
       </c>
-      <c r="F237" s="2">
+      <c r="F237" s="1">
         <v>46028</v>
       </c>
       <c r="G237" t="s">
@@ -12958,7 +12932,7 @@
       <c r="E238" t="s">
         <v>965</v>
       </c>
-      <c r="F238" s="2">
+      <c r="F238" s="1">
         <v>46028</v>
       </c>
       <c r="G238" t="s">
@@ -12987,7 +12961,7 @@
       <c r="E239" t="s">
         <v>966</v>
       </c>
-      <c r="F239" s="2">
+      <c r="F239" s="1">
         <v>46036</v>
       </c>
       <c r="G239" t="s">
@@ -13005,7 +12979,7 @@
       <c r="K239" t="s">
         <v>1217</v>
       </c>
-      <c r="M239" s="2">
+      <c r="M239" s="1">
         <v>46052</v>
       </c>
       <c r="P239" t="b">
@@ -13028,7 +13002,7 @@
       <c r="E240" t="s">
         <v>967</v>
       </c>
-      <c r="F240" s="2">
+      <c r="F240" s="1">
         <v>46036</v>
       </c>
       <c r="G240" t="s">
@@ -13063,7 +13037,7 @@
       <c r="E241" t="s">
         <v>968</v>
       </c>
-      <c r="F241" s="2">
+      <c r="F241" s="1">
         <v>46036</v>
       </c>
       <c r="G241" t="s">
@@ -13098,7 +13072,7 @@
       <c r="E242" t="s">
         <v>969</v>
       </c>
-      <c r="F242" s="2">
+      <c r="F242" s="1">
         <v>46036</v>
       </c>
       <c r="G242" t="s">
@@ -13136,7 +13110,7 @@
       <c r="E243" t="s">
         <v>970</v>
       </c>
-      <c r="F243" s="2">
+      <c r="F243" s="1">
         <v>46048</v>
       </c>
       <c r="G243" t="s">
@@ -13168,7 +13142,7 @@
       <c r="E244" t="s">
         <v>971</v>
       </c>
-      <c r="F244" s="2">
+      <c r="F244" s="1">
         <v>46048</v>
       </c>
       <c r="G244" t="s">
@@ -13206,7 +13180,7 @@
       <c r="E245" t="s">
         <v>972</v>
       </c>
-      <c r="F245" s="2">
+      <c r="F245" s="1">
         <v>46048</v>
       </c>
       <c r="G245" t="s">
@@ -13244,7 +13218,7 @@
       <c r="E246" t="s">
         <v>973</v>
       </c>
-      <c r="F246" s="2">
+      <c r="F246" s="1">
         <v>46050</v>
       </c>
       <c r="G246" t="s">
@@ -13262,7 +13236,7 @@
       <c r="K246" t="s">
         <v>1220</v>
       </c>
-      <c r="M246" s="2">
+      <c r="M246" s="1">
         <v>46191</v>
       </c>
       <c r="P246" t="b">
@@ -13285,7 +13259,7 @@
       <c r="E247" t="s">
         <v>974</v>
       </c>
-      <c r="F247" s="2">
+      <c r="F247" s="1">
         <v>46050</v>
       </c>
       <c r="G247" t="s">
@@ -13314,7 +13288,7 @@
       <c r="E248" t="s">
         <v>975</v>
       </c>
-      <c r="F248" s="2">
+      <c r="F248" s="1">
         <v>46050</v>
       </c>
       <c r="G248" t="s">
@@ -13343,7 +13317,7 @@
       <c r="E249" t="s">
         <v>976</v>
       </c>
-      <c r="F249" s="2">
+      <c r="F249" s="1">
         <v>46050</v>
       </c>
       <c r="G249" t="s">
@@ -13381,7 +13355,7 @@
       <c r="E250" t="s">
         <v>977</v>
       </c>
-      <c r="F250" s="2">
+      <c r="F250" s="1">
         <v>46063</v>
       </c>
       <c r="G250" t="s">
@@ -13419,7 +13393,7 @@
       <c r="E251" t="s">
         <v>978</v>
       </c>
-      <c r="F251" s="2">
+      <c r="F251" s="1">
         <v>46063</v>
       </c>
       <c r="G251" t="s">
@@ -13454,7 +13428,7 @@
       <c r="E252" t="s">
         <v>979</v>
       </c>
-      <c r="F252" s="2">
+      <c r="F252" s="1">
         <v>46063</v>
       </c>
       <c r="G252" t="s">
@@ -13489,7 +13463,7 @@
       <c r="E253" t="s">
         <v>980</v>
       </c>
-      <c r="F253" s="2">
+      <c r="F253" s="1">
         <v>46063</v>
       </c>
       <c r="G253" t="s">
@@ -13527,7 +13501,7 @@
       <c r="E254" t="s">
         <v>981</v>
       </c>
-      <c r="F254" s="2">
+      <c r="F254" s="1">
         <v>46063</v>
       </c>
       <c r="G254" t="s">
@@ -13565,7 +13539,7 @@
       <c r="E255" t="s">
         <v>982</v>
       </c>
-      <c r="F255" s="2">
+      <c r="F255" s="1">
         <v>46063</v>
       </c>
       <c r="G255" t="s">
@@ -13603,7 +13577,7 @@
       <c r="E256" t="s">
         <v>983</v>
       </c>
-      <c r="F256" s="2">
+      <c r="F256" s="1">
         <v>46063</v>
       </c>
       <c r="G256" t="s">
@@ -13644,7 +13618,7 @@
       <c r="E257" t="s">
         <v>984</v>
       </c>
-      <c r="F257" s="2">
+      <c r="F257" s="1">
         <v>46063</v>
       </c>
       <c r="G257" t="s">
@@ -13673,7 +13647,7 @@
       <c r="E258" t="s">
         <v>985</v>
       </c>
-      <c r="F258" s="2">
+      <c r="F258" s="1">
         <v>46063</v>
       </c>
       <c r="G258" t="s">
@@ -13702,7 +13676,7 @@
       <c r="E259" t="s">
         <v>986</v>
       </c>
-      <c r="F259" s="2">
+      <c r="F259" s="1">
         <v>46063</v>
       </c>
       <c r="G259" t="s">
@@ -13740,7 +13714,7 @@
       <c r="E260" t="s">
         <v>987</v>
       </c>
-      <c r="F260" s="2">
+      <c r="F260" s="1">
         <v>46063</v>
       </c>
       <c r="G260" t="s">
@@ -13778,7 +13752,7 @@
       <c r="E261" t="s">
         <v>988</v>
       </c>
-      <c r="F261" s="2">
+      <c r="F261" s="1">
         <v>46063</v>
       </c>
       <c r="G261" t="s">
@@ -13816,7 +13790,7 @@
       <c r="E262" t="s">
         <v>989</v>
       </c>
-      <c r="F262" s="2">
+      <c r="F262" s="1">
         <v>46063</v>
       </c>
       <c r="G262" t="s">
@@ -13834,7 +13808,7 @@
       <c r="K262" t="s">
         <v>1223</v>
       </c>
-      <c r="M262" s="2">
+      <c r="M262" s="1">
         <v>46113</v>
       </c>
       <c r="O262" t="s">
@@ -13860,7 +13834,7 @@
       <c r="E263" t="s">
         <v>990</v>
       </c>
-      <c r="F263" s="2">
+      <c r="F263" s="1">
         <v>46063</v>
       </c>
       <c r="G263" t="s">
@@ -13895,7 +13869,7 @@
       <c r="E264" t="s">
         <v>991</v>
       </c>
-      <c r="F264" s="2">
+      <c r="F264" s="1">
         <v>46063</v>
       </c>
       <c r="G264" t="s">
@@ -13933,7 +13907,7 @@
       <c r="E265" t="s">
         <v>992</v>
       </c>
-      <c r="F265" s="2">
+      <c r="F265" s="1">
         <v>46063</v>
       </c>
       <c r="G265" t="s">
@@ -13971,7 +13945,7 @@
       <c r="E266" t="s">
         <v>993</v>
       </c>
-      <c r="F266" s="2">
+      <c r="F266" s="1">
         <v>46063</v>
       </c>
       <c r="G266" t="s">
@@ -14009,7 +13983,7 @@
       <c r="E267" t="s">
         <v>994</v>
       </c>
-      <c r="F267" s="2">
+      <c r="F267" s="1">
         <v>46063</v>
       </c>
       <c r="G267" t="s">
@@ -14047,7 +14021,7 @@
       <c r="E268" t="s">
         <v>995</v>
       </c>
-      <c r="F268" s="2">
+      <c r="F268" s="1">
         <v>46063</v>
       </c>
       <c r="G268" t="s">
@@ -14082,7 +14056,7 @@
       <c r="D269" t="s">
         <v>711</v>
       </c>
-      <c r="F269" s="2">
+      <c r="F269" s="1">
         <v>46063</v>
       </c>
       <c r="G269" t="s">
@@ -14120,7 +14094,7 @@
       <c r="E270" t="s">
         <v>996</v>
       </c>
-      <c r="F270" s="2">
+      <c r="F270" s="1">
         <v>46063</v>
       </c>
       <c r="G270" t="s">
@@ -14158,7 +14132,7 @@
       <c r="E271" t="s">
         <v>997</v>
       </c>
-      <c r="F271" s="2">
+      <c r="F271" s="1">
         <v>46063</v>
       </c>
       <c r="G271" t="s">
@@ -14196,7 +14170,7 @@
       <c r="E272" t="s">
         <v>998</v>
       </c>
-      <c r="F272" s="2">
+      <c r="F272" s="1">
         <v>46063</v>
       </c>
       <c r="G272" t="s">
@@ -14214,7 +14188,7 @@
       <c r="K272" t="s">
         <v>1225</v>
       </c>
-      <c r="M272" s="2">
+      <c r="M272" s="1">
         <v>46185</v>
       </c>
       <c r="N272" t="s">
@@ -14240,7 +14214,7 @@
       <c r="E273" t="s">
         <v>999</v>
       </c>
-      <c r="F273" s="2">
+      <c r="F273" s="1">
         <v>46063</v>
       </c>
       <c r="G273" t="s">
@@ -14275,7 +14249,7 @@
       <c r="E274" t="s">
         <v>1000</v>
       </c>
-      <c r="F274" s="2">
+      <c r="F274" s="1">
         <v>46063</v>
       </c>
       <c r="G274" t="s">
@@ -14313,7 +14287,7 @@
       <c r="E275" t="s">
         <v>1001</v>
       </c>
-      <c r="F275" s="2">
+      <c r="F275" s="1">
         <v>46063</v>
       </c>
       <c r="G275" t="s">
@@ -14348,7 +14322,7 @@
       <c r="E276" t="s">
         <v>1002</v>
       </c>
-      <c r="F276" s="2">
+      <c r="F276" s="1">
         <v>46063</v>
       </c>
       <c r="G276" t="s">
@@ -14386,7 +14360,7 @@
       <c r="E277" t="s">
         <v>1003</v>
       </c>
-      <c r="F277" s="2">
+      <c r="F277" s="1">
         <v>46063</v>
       </c>
       <c r="G277" t="s">
@@ -14424,7 +14398,7 @@
       <c r="E278" t="s">
         <v>1004</v>
       </c>
-      <c r="F278" s="2">
+      <c r="F278" s="1">
         <v>46077</v>
       </c>
       <c r="G278" t="s">
@@ -14462,7 +14436,7 @@
       <c r="E279" t="s">
         <v>1005</v>
       </c>
-      <c r="F279" s="2">
+      <c r="F279" s="1">
         <v>46077</v>
       </c>
       <c r="G279" t="s">
@@ -14503,7 +14477,7 @@
       <c r="E280" t="s">
         <v>1006</v>
       </c>
-      <c r="F280" s="2">
+      <c r="F280" s="1">
         <v>46085</v>
       </c>
       <c r="G280" t="s">
@@ -14541,7 +14515,7 @@
       <c r="E281" t="s">
         <v>1007</v>
       </c>
-      <c r="F281" s="2">
+      <c r="F281" s="1">
         <v>46085</v>
       </c>
       <c r="G281" t="s">
@@ -14579,7 +14553,7 @@
       <c r="E282" t="s">
         <v>1008</v>
       </c>
-      <c r="F282" s="2">
+      <c r="F282" s="1">
         <v>46090</v>
       </c>
       <c r="G282" t="s">
@@ -14617,7 +14591,7 @@
       <c r="E283" t="s">
         <v>1009</v>
       </c>
-      <c r="F283" s="2">
+      <c r="F283" s="1">
         <v>46100</v>
       </c>
       <c r="G283" t="s">
@@ -14652,7 +14626,7 @@
       <c r="E284" t="s">
         <v>1010</v>
       </c>
-      <c r="F284" s="2">
+      <c r="F284" s="1">
         <v>46100</v>
       </c>
       <c r="G284" t="s">
@@ -14687,7 +14661,7 @@
       <c r="E285" t="s">
         <v>1011</v>
       </c>
-      <c r="F285" s="2">
+      <c r="F285" s="1">
         <v>46100</v>
       </c>
       <c r="G285" t="s">
@@ -14722,7 +14696,7 @@
       <c r="E286" t="s">
         <v>1012</v>
       </c>
-      <c r="F286" s="2">
+      <c r="F286" s="1">
         <v>46100</v>
       </c>
       <c r="G286" t="s">
@@ -14757,7 +14731,7 @@
       <c r="E287">
         <v>35971</v>
       </c>
-      <c r="F287" s="2">
+      <c r="F287" s="1">
         <v>46107</v>
       </c>
       <c r="G287" t="s">
@@ -14786,7 +14760,7 @@
       <c r="E288">
         <v>107178</v>
       </c>
-      <c r="F288" s="2">
+      <c r="F288" s="1">
         <v>46107</v>
       </c>
       <c r="G288" t="s">
@@ -14824,7 +14798,7 @@
       <c r="E289">
         <v>108773</v>
       </c>
-      <c r="F289" s="2">
+      <c r="F289" s="1">
         <v>46107</v>
       </c>
       <c r="G289" t="s">
@@ -14853,7 +14827,7 @@
       <c r="E290">
         <v>7086</v>
       </c>
-      <c r="F290" s="2">
+      <c r="F290" s="1">
         <v>46107</v>
       </c>
       <c r="G290" t="s">
@@ -14868,7 +14842,7 @@
       <c r="J290" t="s">
         <v>1145</v>
       </c>
-      <c r="M290" s="2">
+      <c r="M290" s="1">
         <v>46127</v>
       </c>
       <c r="P290" t="b">
@@ -14891,7 +14865,7 @@
       <c r="E291">
         <v>99743</v>
       </c>
-      <c r="F291" s="2">
+      <c r="F291" s="1">
         <v>46107</v>
       </c>
       <c r="G291" t="s">
@@ -14929,7 +14903,7 @@
       <c r="E292" t="s">
         <v>1013</v>
       </c>
-      <c r="F292" s="2">
+      <c r="F292" s="1">
         <v>46112</v>
       </c>
       <c r="G292" t="s">
@@ -14967,7 +14941,7 @@
       <c r="E293" t="s">
         <v>1014</v>
       </c>
-      <c r="F293" s="2">
+      <c r="F293" s="1">
         <v>46125</v>
       </c>
       <c r="G293" t="s">
@@ -15005,7 +14979,7 @@
       <c r="E294" t="s">
         <v>1015</v>
       </c>
-      <c r="F294" s="2">
+      <c r="F294" s="1">
         <v>46125</v>
       </c>
       <c r="G294" t="s">
@@ -15040,7 +15014,7 @@
       <c r="E295" t="s">
         <v>1016</v>
       </c>
-      <c r="F295" s="2">
+      <c r="F295" s="1">
         <v>46125</v>
       </c>
       <c r="G295" t="s">
@@ -15075,7 +15049,7 @@
       <c r="E296" t="s">
         <v>1017</v>
       </c>
-      <c r="F296" s="2">
+      <c r="F296" s="1">
         <v>46125</v>
       </c>
       <c r="G296" t="s">
@@ -15110,7 +15084,7 @@
       <c r="E297">
         <v>47203152</v>
       </c>
-      <c r="F297" s="2">
+      <c r="F297" s="1">
         <v>46125</v>
       </c>
       <c r="G297" t="s">
@@ -15145,7 +15119,7 @@
       <c r="E298">
         <v>47202512</v>
       </c>
-      <c r="F298" s="2">
+      <c r="F298" s="1">
         <v>46125</v>
       </c>
       <c r="G298" t="s">
@@ -15183,7 +15157,7 @@
       <c r="E299">
         <v>22005580</v>
       </c>
-      <c r="F299" s="2">
+      <c r="F299" s="1">
         <v>46125</v>
       </c>
       <c r="G299" t="s">
@@ -15221,7 +15195,7 @@
       <c r="E300">
         <v>22005955</v>
       </c>
-      <c r="F300" s="2">
+      <c r="F300" s="1">
         <v>46125</v>
       </c>
       <c r="G300" t="s">
@@ -15259,7 +15233,7 @@
       <c r="E301">
         <v>22005661</v>
       </c>
-      <c r="F301" s="2">
+      <c r="F301" s="1">
         <v>46125</v>
       </c>
       <c r="G301" t="s">
@@ -15297,7 +15271,7 @@
       <c r="E302">
         <v>32207</v>
       </c>
-      <c r="F302" s="2">
+      <c r="F302" s="1">
         <v>46125</v>
       </c>
       <c r="G302" t="s">
@@ -15335,7 +15309,7 @@
       <c r="E303">
         <v>18156</v>
       </c>
-      <c r="F303" s="2">
+      <c r="F303" s="1">
         <v>46125</v>
       </c>
       <c r="G303" t="s">
@@ -15373,7 +15347,7 @@
       <c r="E304">
         <v>37971</v>
       </c>
-      <c r="F304" s="2">
+      <c r="F304" s="1">
         <v>46125</v>
       </c>
       <c r="G304" t="s">
@@ -15411,7 +15385,7 @@
       <c r="E305">
         <v>84317</v>
       </c>
-      <c r="F305" s="2">
+      <c r="F305" s="1">
         <v>46125</v>
       </c>
       <c r="G305" t="s">
@@ -15429,7 +15403,7 @@
       <c r="K305" t="s">
         <v>1230</v>
       </c>
-      <c r="M305" s="2">
+      <c r="M305" s="1">
         <v>46160</v>
       </c>
       <c r="P305" t="b">
@@ -15452,7 +15426,7 @@
       <c r="E306">
         <v>83773</v>
       </c>
-      <c r="F306" s="2">
+      <c r="F306" s="1">
         <v>46125</v>
       </c>
       <c r="G306" t="s">
@@ -15470,7 +15444,7 @@
       <c r="K306" t="s">
         <v>1231</v>
       </c>
-      <c r="M306" s="2">
+      <c r="M306" s="1">
         <v>46156</v>
       </c>
       <c r="P306" t="b">
@@ -15493,7 +15467,7 @@
       <c r="E307">
         <v>83740</v>
       </c>
-      <c r="F307" s="2">
+      <c r="F307" s="1">
         <v>46125</v>
       </c>
       <c r="G307" t="s">
@@ -15531,7 +15505,7 @@
       <c r="E308">
         <v>84326</v>
       </c>
-      <c r="F308" s="2">
+      <c r="F308" s="1">
         <v>46125</v>
       </c>
       <c r="G308" t="s">
@@ -15569,7 +15543,7 @@
       <c r="E309">
         <v>6708</v>
       </c>
-      <c r="F309" s="2">
+      <c r="F309" s="1">
         <v>46125</v>
       </c>
       <c r="G309" t="s">
@@ -15607,7 +15581,7 @@
       <c r="E310" t="s">
         <v>1018</v>
       </c>
-      <c r="F310" s="2">
+      <c r="F310" s="1">
         <v>46125</v>
       </c>
       <c r="G310" t="s">
@@ -15645,7 +15619,7 @@
       <c r="E311">
         <v>9727</v>
       </c>
-      <c r="F311" s="2">
+      <c r="F311" s="1">
         <v>46125</v>
       </c>
       <c r="G311" t="s">
@@ -15683,7 +15657,7 @@
       <c r="E312" t="s">
         <v>1019</v>
       </c>
-      <c r="F312" s="2">
+      <c r="F312" s="1">
         <v>46125</v>
       </c>
       <c r="G312" t="s">
@@ -15721,7 +15695,7 @@
       <c r="E313">
         <v>31</v>
       </c>
-      <c r="F313" s="2">
+      <c r="F313" s="1">
         <v>46125</v>
       </c>
       <c r="G313" t="s">
@@ -15756,7 +15730,7 @@
       <c r="E314">
         <v>965</v>
       </c>
-      <c r="F314" s="2">
+      <c r="F314" s="1">
         <v>46125</v>
       </c>
       <c r="G314" t="s">
@@ -15794,7 +15768,7 @@
       <c r="E315">
         <v>2007</v>
       </c>
-      <c r="F315" s="2">
+      <c r="F315" s="1">
         <v>46125</v>
       </c>
       <c r="G315" t="s">
@@ -15832,7 +15806,7 @@
       <c r="E316">
         <v>688</v>
       </c>
-      <c r="F316" s="2">
+      <c r="F316" s="1">
         <v>46125</v>
       </c>
       <c r="G316" t="s">
@@ -15870,7 +15844,7 @@
       <c r="E317" t="s">
         <v>1020</v>
       </c>
-      <c r="F317" s="2">
+      <c r="F317" s="1">
         <v>46125</v>
       </c>
       <c r="G317" t="s">
@@ -15908,7 +15882,7 @@
       <c r="E318" t="s">
         <v>1021</v>
       </c>
-      <c r="F318" s="2">
+      <c r="F318" s="1">
         <v>46125</v>
       </c>
       <c r="G318" t="s">
@@ -15937,7 +15911,7 @@
       <c r="E319" t="s">
         <v>1022</v>
       </c>
-      <c r="F319" s="2">
+      <c r="F319" s="1">
         <v>46125</v>
       </c>
       <c r="G319" t="s">
@@ -15952,7 +15926,7 @@
       <c r="K319" t="s">
         <v>1232</v>
       </c>
-      <c r="M319" s="2">
+      <c r="M319" s="1">
         <v>46175</v>
       </c>
       <c r="P319" t="b">
@@ -15975,7 +15949,7 @@
       <c r="E320">
         <v>1391</v>
       </c>
-      <c r="F320" s="2">
+      <c r="F320" s="1">
         <v>46125</v>
       </c>
       <c r="G320" t="s">
@@ -16013,7 +15987,7 @@
       <c r="E321">
         <v>120315</v>
       </c>
-      <c r="F321" s="2">
+      <c r="F321" s="1">
         <v>46125</v>
       </c>
       <c r="G321" t="s">
@@ -16051,7 +16025,7 @@
       <c r="E322" t="s">
         <v>1023</v>
       </c>
-      <c r="F322" s="2">
+      <c r="F322" s="1">
         <v>46125</v>
       </c>
       <c r="G322" t="s">
@@ -16069,7 +16043,7 @@
       <c r="K322" t="s">
         <v>1233</v>
       </c>
-      <c r="M322" s="2">
+      <c r="M322" s="1">
         <v>46182</v>
       </c>
       <c r="P322" t="b">
@@ -16092,7 +16066,7 @@
       <c r="E323">
         <v>535933</v>
       </c>
-      <c r="F323" s="2">
+      <c r="F323" s="1">
         <v>46125</v>
       </c>
       <c r="G323" t="s">
@@ -16130,7 +16104,7 @@
       <c r="E324">
         <v>289029</v>
       </c>
-      <c r="F324" s="2">
+      <c r="F324" s="1">
         <v>46125</v>
       </c>
       <c r="G324" t="s">
@@ -16168,7 +16142,7 @@
       <c r="E325">
         <v>3454</v>
       </c>
-      <c r="F325" s="2">
+      <c r="F325" s="1">
         <v>46125</v>
       </c>
       <c r="G325" t="s">
@@ -16186,7 +16160,7 @@
       <c r="K325" t="s">
         <v>1233</v>
       </c>
-      <c r="M325" s="2">
+      <c r="M325" s="1">
         <v>46182</v>
       </c>
       <c r="P325" t="b">
@@ -16209,7 +16183,7 @@
       <c r="E326">
         <v>3493</v>
       </c>
-      <c r="F326" s="2">
+      <c r="F326" s="1">
         <v>46125</v>
       </c>
       <c r="G326" t="s">
@@ -16247,7 +16221,7 @@
       <c r="E327" t="s">
         <v>1023</v>
       </c>
-      <c r="F327" s="2">
+      <c r="F327" s="1">
         <v>46125</v>
       </c>
       <c r="G327" t="s">
@@ -16265,7 +16239,7 @@
       <c r="K327" t="s">
         <v>1233</v>
       </c>
-      <c r="M327" s="2">
+      <c r="M327" s="1">
         <v>46182</v>
       </c>
       <c r="P327" t="b">
@@ -16288,7 +16262,7 @@
       <c r="E328">
         <v>3235</v>
       </c>
-      <c r="F328" s="2">
+      <c r="F328" s="1">
         <v>46125</v>
       </c>
       <c r="G328" t="s">
@@ -16306,7 +16280,7 @@
       <c r="K328" t="s">
         <v>1233</v>
       </c>
-      <c r="M328" s="2">
+      <c r="M328" s="1">
         <v>46182</v>
       </c>
       <c r="P328" t="b">
@@ -16329,7 +16303,7 @@
       <c r="E329">
         <v>625052</v>
       </c>
-      <c r="F329" s="2">
+      <c r="F329" s="1">
         <v>46125</v>
       </c>
       <c r="G329" t="s">
@@ -16347,7 +16321,7 @@
       <c r="K329" t="s">
         <v>1233</v>
       </c>
-      <c r="M329" s="2">
+      <c r="M329" s="1">
         <v>46182</v>
       </c>
       <c r="P329" t="b">
@@ -16370,7 +16344,7 @@
       <c r="E330">
         <v>614095</v>
       </c>
-      <c r="F330" s="2">
+      <c r="F330" s="1">
         <v>46125</v>
       </c>
       <c r="G330" t="s">
@@ -16388,7 +16362,7 @@
       <c r="K330" t="s">
         <v>1233</v>
       </c>
-      <c r="M330" s="2">
+      <c r="M330" s="1">
         <v>46182</v>
       </c>
       <c r="P330" t="b">
@@ -16411,7 +16385,7 @@
       <c r="E331" t="s">
         <v>965</v>
       </c>
-      <c r="F331" s="2">
+      <c r="F331" s="1">
         <v>46125</v>
       </c>
       <c r="G331" t="s">
@@ -16449,7 +16423,7 @@
       <c r="E332" t="s">
         <v>1024</v>
       </c>
-      <c r="F332" s="2">
+      <c r="F332" s="1">
         <v>46125</v>
       </c>
       <c r="G332" t="s">
@@ -16487,7 +16461,7 @@
       <c r="E333">
         <v>197</v>
       </c>
-      <c r="F333" s="2">
+      <c r="F333" s="1">
         <v>46125</v>
       </c>
       <c r="G333" t="s">
@@ -16525,7 +16499,7 @@
       <c r="E334">
         <v>1378</v>
       </c>
-      <c r="F334" s="2">
+      <c r="F334" s="1">
         <v>46125</v>
       </c>
       <c r="G334" t="s">
@@ -16563,7 +16537,7 @@
       <c r="E335" t="s">
         <v>1025</v>
       </c>
-      <c r="F335" s="2">
+      <c r="F335" s="1">
         <v>46127</v>
       </c>
       <c r="G335" t="s">
@@ -16578,7 +16552,7 @@
       <c r="K335" t="s">
         <v>1232</v>
       </c>
-      <c r="M335" s="2">
+      <c r="M335" s="1">
         <v>46175</v>
       </c>
       <c r="P335" t="b">
@@ -16601,7 +16575,7 @@
       <c r="E336" t="s">
         <v>1026</v>
       </c>
-      <c r="F336" s="2">
+      <c r="F336" s="1">
         <v>46127</v>
       </c>
       <c r="G336" t="s">
@@ -16639,7 +16613,7 @@
       <c r="E337" t="s">
         <v>1027</v>
       </c>
-      <c r="F337" s="2">
+      <c r="F337" s="1">
         <v>46127</v>
       </c>
       <c r="G337" t="s">
@@ -16654,7 +16628,7 @@
       <c r="K337" t="s">
         <v>1232</v>
       </c>
-      <c r="M337" s="2">
+      <c r="M337" s="1">
         <v>46175</v>
       </c>
       <c r="P337" t="b">
@@ -16677,7 +16651,7 @@
       <c r="E338" t="s">
         <v>1028</v>
       </c>
-      <c r="F338" s="2">
+      <c r="F338" s="1">
         <v>46127</v>
       </c>
       <c r="G338" t="s">
@@ -16715,7 +16689,7 @@
       <c r="E339">
         <v>6291</v>
       </c>
-      <c r="F339" s="2">
+      <c r="F339" s="1">
         <v>46129</v>
       </c>
       <c r="G339" t="s">
@@ -16744,7 +16718,7 @@
       <c r="E340" t="s">
         <v>1029</v>
       </c>
-      <c r="F340" s="2">
+      <c r="F340" s="1">
         <v>46142</v>
       </c>
       <c r="G340" t="s">
@@ -16782,7 +16756,7 @@
       <c r="E341" t="s">
         <v>1030</v>
       </c>
-      <c r="F341" s="2">
+      <c r="F341" s="1">
         <v>46142</v>
       </c>
       <c r="G341" t="s">
@@ -16820,7 +16794,7 @@
       <c r="E342" t="s">
         <v>1031</v>
       </c>
-      <c r="F342" s="2">
+      <c r="F342" s="1">
         <v>46142</v>
       </c>
       <c r="G342" t="s">
@@ -16858,7 +16832,7 @@
       <c r="E343" t="s">
         <v>1032</v>
       </c>
-      <c r="F343" s="2">
+      <c r="F343" s="1">
         <v>46142</v>
       </c>
       <c r="G343" t="s">
@@ -16896,7 +16870,7 @@
       <c r="E344" t="s">
         <v>1033</v>
       </c>
-      <c r="F344" s="2">
+      <c r="F344" s="1">
         <v>46142</v>
       </c>
       <c r="G344" t="s">
@@ -16934,7 +16908,7 @@
       <c r="E345" t="s">
         <v>1034</v>
       </c>
-      <c r="F345" s="2">
+      <c r="F345" s="1">
         <v>46142</v>
       </c>
       <c r="G345" t="s">
@@ -16972,7 +16946,7 @@
       <c r="E346" t="s">
         <v>1035</v>
       </c>
-      <c r="F346" s="2">
+      <c r="F346" s="1">
         <v>46142</v>
       </c>
       <c r="G346" t="s">
@@ -17010,7 +16984,7 @@
       <c r="E347" t="s">
         <v>1036</v>
       </c>
-      <c r="F347" s="2">
+      <c r="F347" s="1">
         <v>46142</v>
       </c>
       <c r="G347" t="s">
@@ -17028,7 +17002,7 @@
       <c r="K347" t="s">
         <v>1230</v>
       </c>
-      <c r="M347" s="2">
+      <c r="M347" s="1">
         <v>46160</v>
       </c>
       <c r="P347" t="b">
@@ -17051,7 +17025,7 @@
       <c r="E348" t="s">
         <v>1037</v>
       </c>
-      <c r="F348" s="2">
+      <c r="F348" s="1">
         <v>46142</v>
       </c>
       <c r="G348" t="s">
@@ -17069,7 +17043,7 @@
       <c r="K348" t="s">
         <v>1231</v>
       </c>
-      <c r="M348" s="2">
+      <c r="M348" s="1">
         <v>46156</v>
       </c>
       <c r="P348" t="b">
@@ -17092,7 +17066,7 @@
       <c r="E349" t="s">
         <v>1038</v>
       </c>
-      <c r="F349" s="2">
+      <c r="F349" s="1">
         <v>46142</v>
       </c>
       <c r="G349" t="s">
@@ -17130,7 +17104,7 @@
       <c r="E350" t="s">
         <v>1039</v>
       </c>
-      <c r="F350" s="2">
+      <c r="F350" s="1">
         <v>46142</v>
       </c>
       <c r="G350" t="s">
@@ -17165,7 +17139,7 @@
       <c r="E351" t="s">
         <v>1040</v>
       </c>
-      <c r="F351" s="2">
+      <c r="F351" s="1">
         <v>46142</v>
       </c>
       <c r="G351" t="s">
@@ -17203,7 +17177,7 @@
       <c r="E352" t="s">
         <v>1041</v>
       </c>
-      <c r="F352" s="2">
+      <c r="F352" s="1">
         <v>46142</v>
       </c>
       <c r="G352" t="s">
@@ -17241,7 +17215,7 @@
       <c r="E353" t="s">
         <v>1042</v>
       </c>
-      <c r="F353" s="2">
+      <c r="F353" s="1">
         <v>46142</v>
       </c>
       <c r="G353" t="s">
@@ -17279,7 +17253,7 @@
       <c r="E354" t="s">
         <v>1043</v>
       </c>
-      <c r="F354" s="2">
+      <c r="F354" s="1">
         <v>46142</v>
       </c>
       <c r="G354" t="s">
@@ -17317,7 +17291,7 @@
       <c r="E355" t="s">
         <v>1044</v>
       </c>
-      <c r="F355" s="2">
+      <c r="F355" s="1">
         <v>46142</v>
       </c>
       <c r="G355" t="s">
@@ -17335,7 +17309,7 @@
       <c r="K355" t="s">
         <v>1234</v>
       </c>
-      <c r="M355" s="2">
+      <c r="M355" s="1">
         <v>46150</v>
       </c>
       <c r="P355" t="b">
@@ -17358,7 +17332,7 @@
       <c r="E356" t="s">
         <v>1045</v>
       </c>
-      <c r="F356" s="2">
+      <c r="F356" s="1">
         <v>46142</v>
       </c>
       <c r="G356" t="s">
@@ -17373,7 +17347,7 @@
       <c r="K356" t="s">
         <v>1235</v>
       </c>
-      <c r="M356" s="2">
+      <c r="M356" s="1">
         <v>46176</v>
       </c>
       <c r="P356" t="b">
@@ -17396,7 +17370,7 @@
       <c r="E357" t="s">
         <v>1046</v>
       </c>
-      <c r="F357" s="2">
+      <c r="F357" s="1">
         <v>46142</v>
       </c>
       <c r="G357" t="s">
@@ -17434,7 +17408,7 @@
       <c r="E358" t="s">
         <v>1047</v>
       </c>
-      <c r="F358" s="2">
+      <c r="F358" s="1">
         <v>46142</v>
       </c>
       <c r="G358" t="s">
@@ -17472,7 +17446,7 @@
       <c r="E359" t="s">
         <v>1048</v>
       </c>
-      <c r="F359" s="2">
+      <c r="F359" s="1">
         <v>46142</v>
       </c>
       <c r="G359" t="s">
@@ -17513,7 +17487,7 @@
       <c r="E360" t="s">
         <v>857</v>
       </c>
-      <c r="F360" s="2">
+      <c r="F360" s="1">
         <v>46142</v>
       </c>
       <c r="G360" t="s">
@@ -17551,7 +17525,7 @@
       <c r="E361" t="s">
         <v>869</v>
       </c>
-      <c r="F361" s="2">
+      <c r="F361" s="1">
         <v>46142</v>
       </c>
       <c r="G361" t="s">
@@ -17589,7 +17563,7 @@
       <c r="E362" t="s">
         <v>1049</v>
       </c>
-      <c r="F362" s="2">
+      <c r="F362" s="1">
         <v>46142</v>
       </c>
       <c r="G362" t="s">
@@ -17627,7 +17601,7 @@
       <c r="E363" t="s">
         <v>1050</v>
       </c>
-      <c r="F363" s="2">
+      <c r="F363" s="1">
         <v>46142</v>
       </c>
       <c r="G363" t="s">
@@ -17665,7 +17639,7 @@
       <c r="E364" t="s">
         <v>866</v>
       </c>
-      <c r="F364" s="2">
+      <c r="F364" s="1">
         <v>46142</v>
       </c>
       <c r="G364" t="s">
@@ -17703,7 +17677,7 @@
       <c r="E365" t="s">
         <v>1051</v>
       </c>
-      <c r="F365" s="2">
+      <c r="F365" s="1">
         <v>46142</v>
       </c>
       <c r="G365" t="s">
@@ -17741,7 +17715,7 @@
       <c r="E366" t="s">
         <v>1052</v>
       </c>
-      <c r="F366" s="2">
+      <c r="F366" s="1">
         <v>46148</v>
       </c>
       <c r="G366" t="s">
@@ -17779,7 +17753,7 @@
       <c r="E367" t="s">
         <v>1053</v>
       </c>
-      <c r="F367" s="2">
+      <c r="F367" s="1">
         <v>46148</v>
       </c>
       <c r="G367" t="s">
@@ -17817,7 +17791,7 @@
       <c r="E368" t="s">
         <v>1054</v>
       </c>
-      <c r="F368" s="2">
+      <c r="F368" s="1">
         <v>46148</v>
       </c>
       <c r="G368" t="s">
@@ -17855,7 +17829,7 @@
       <c r="E369" t="s">
         <v>1055</v>
       </c>
-      <c r="F369" s="2">
+      <c r="F369" s="1">
         <v>46148</v>
       </c>
       <c r="G369" t="s">
@@ -17893,7 +17867,7 @@
       <c r="E370" t="s">
         <v>1056</v>
       </c>
-      <c r="F370" s="2">
+      <c r="F370" s="1">
         <v>46148</v>
       </c>
       <c r="G370" t="s">
@@ -17931,7 +17905,7 @@
       <c r="E371" t="s">
         <v>1057</v>
       </c>
-      <c r="F371" s="2">
+      <c r="F371" s="1">
         <v>46148</v>
       </c>
       <c r="G371" t="s">
@@ -17949,7 +17923,7 @@
       <c r="K371" t="s">
         <v>1236</v>
       </c>
-      <c r="M371" s="2">
+      <c r="M371" s="1">
         <v>46164</v>
       </c>
       <c r="P371" t="b">
@@ -17972,7 +17946,7 @@
       <c r="E372" t="s">
         <v>1058</v>
       </c>
-      <c r="F372" s="2">
+      <c r="F372" s="1">
         <v>46148</v>
       </c>
       <c r="G372" t="s">
@@ -17990,7 +17964,7 @@
       <c r="K372" t="s">
         <v>1223</v>
       </c>
-      <c r="M372" s="2">
+      <c r="M372" s="1">
         <v>46113</v>
       </c>
       <c r="O372" t="s">
@@ -18016,7 +17990,7 @@
       <c r="E373" t="s">
         <v>1059</v>
       </c>
-      <c r="F373" s="2">
+      <c r="F373" s="1">
         <v>46149</v>
       </c>
       <c r="G373" t="s">
@@ -18054,7 +18028,7 @@
       <c r="E374" t="s">
         <v>1060</v>
       </c>
-      <c r="F374" s="2">
+      <c r="F374" s="1">
         <v>46149</v>
       </c>
       <c r="G374" t="s">
@@ -18092,7 +18066,7 @@
       <c r="E375" t="s">
         <v>1061</v>
       </c>
-      <c r="F375" s="2">
+      <c r="F375" s="1">
         <v>46154</v>
       </c>
       <c r="G375" t="s">
@@ -18130,7 +18104,7 @@
       <c r="E376" t="s">
         <v>1062</v>
       </c>
-      <c r="F376" s="2">
+      <c r="F376" s="1">
         <v>46154</v>
       </c>
       <c r="G376" t="s">
@@ -18168,7 +18142,7 @@
       <c r="E377" t="s">
         <v>1063</v>
       </c>
-      <c r="F377" s="2">
+      <c r="F377" s="1">
         <v>46154</v>
       </c>
       <c r="G377" t="s">
@@ -18206,7 +18180,7 @@
       <c r="E378" t="s">
         <v>1064</v>
       </c>
-      <c r="F378" s="2">
+      <c r="F378" s="1">
         <v>46154</v>
       </c>
       <c r="G378" t="s">
@@ -18244,7 +18218,7 @@
       <c r="E379" t="s">
         <v>1065</v>
       </c>
-      <c r="F379" s="2">
+      <c r="F379" s="1">
         <v>46154</v>
       </c>
       <c r="G379" t="s">
@@ -18262,7 +18236,7 @@
       <c r="K379" t="s">
         <v>1237</v>
       </c>
-      <c r="M379" s="2">
+      <c r="M379" s="1">
         <v>46174</v>
       </c>
       <c r="P379" t="b">
@@ -18285,7 +18259,7 @@
       <c r="E380" t="s">
         <v>1066</v>
       </c>
-      <c r="F380" s="2">
+      <c r="F380" s="1">
         <v>46154</v>
       </c>
       <c r="G380" t="s">
@@ -18323,7 +18297,7 @@
       <c r="E381" t="s">
         <v>1067</v>
       </c>
-      <c r="F381" s="2">
+      <c r="F381" s="1">
         <v>46154</v>
       </c>
       <c r="G381" t="s">
@@ -18361,7 +18335,7 @@
       <c r="E382" t="s">
         <v>1068</v>
       </c>
-      <c r="F382" s="2">
+      <c r="F382" s="1">
         <v>46154</v>
       </c>
       <c r="G382" t="s">
@@ -18399,7 +18373,7 @@
       <c r="E383" t="s">
         <v>1069</v>
       </c>
-      <c r="F383" s="2">
+      <c r="F383" s="1">
         <v>46154</v>
       </c>
       <c r="G383" t="s">
@@ -18437,7 +18411,7 @@
       <c r="E384" t="s">
         <v>1070</v>
       </c>
-      <c r="F384" s="2">
+      <c r="F384" s="1">
         <v>46164</v>
       </c>
       <c r="G384" t="s">
@@ -18475,7 +18449,7 @@
       <c r="E385" t="s">
         <v>1071</v>
       </c>
-      <c r="F385" s="2">
+      <c r="F385" s="1">
         <v>46164</v>
       </c>
       <c r="G385" t="s">
@@ -18513,7 +18487,7 @@
       <c r="E386" t="s">
         <v>1072</v>
       </c>
-      <c r="F386" s="2">
+      <c r="F386" s="1">
         <v>46171</v>
       </c>
       <c r="G386" t="s">
@@ -18551,7 +18525,7 @@
       <c r="E387" t="s">
         <v>1073</v>
       </c>
-      <c r="F387" s="2">
+      <c r="F387" s="1">
         <v>46171</v>
       </c>
       <c r="G387" t="s">
@@ -18589,7 +18563,7 @@
       <c r="E388" t="s">
         <v>759</v>
       </c>
-      <c r="F388" s="2">
+      <c r="F388" s="1">
         <v>46171</v>
       </c>
       <c r="G388" t="s">
@@ -18627,7 +18601,7 @@
       <c r="E389" t="s">
         <v>1074</v>
       </c>
-      <c r="F389" s="2">
+      <c r="F389" s="1">
         <v>46171</v>
       </c>
       <c r="G389" t="s">
@@ -18665,7 +18639,7 @@
       <c r="E390" t="s">
         <v>1075</v>
       </c>
-      <c r="F390" s="2">
+      <c r="F390" s="1">
         <v>46171</v>
       </c>
       <c r="G390" t="s">
@@ -18683,7 +18657,7 @@
       <c r="K390" t="s">
         <v>1238</v>
       </c>
-      <c r="M390" s="2">
+      <c r="M390" s="1">
         <v>46191</v>
       </c>
       <c r="P390" t="b">
@@ -18706,7 +18680,7 @@
       <c r="E391" t="s">
         <v>1076</v>
       </c>
-      <c r="F391" s="2">
+      <c r="F391" s="1">
         <v>46171</v>
       </c>
       <c r="G391" t="s">
@@ -18744,7 +18718,7 @@
       <c r="E392" t="s">
         <v>1077</v>
       </c>
-      <c r="F392" s="2">
+      <c r="F392" s="1">
         <v>46171</v>
       </c>
       <c r="G392" t="s">
@@ -18759,7 +18733,7 @@
       <c r="K392" t="s">
         <v>1235</v>
       </c>
-      <c r="M392" s="2">
+      <c r="M392" s="1">
         <v>46176</v>
       </c>
       <c r="P392" t="b">
@@ -18782,7 +18756,7 @@
       <c r="E393" t="s">
         <v>1078</v>
       </c>
-      <c r="F393" s="2">
+      <c r="F393" s="1">
         <v>46171</v>
       </c>
       <c r="G393" t="s">
@@ -18820,7 +18794,7 @@
       <c r="E394" t="s">
         <v>1079</v>
       </c>
-      <c r="F394" s="2">
+      <c r="F394" s="1">
         <v>46171</v>
       </c>
       <c r="G394" t="s">
@@ -18858,7 +18832,7 @@
       <c r="E395" t="s">
         <v>1080</v>
       </c>
-      <c r="F395" s="2">
+      <c r="F395" s="1">
         <v>46171</v>
       </c>
       <c r="G395" t="s">
@@ -18896,7 +18870,7 @@
       <c r="E396" t="s">
         <v>1081</v>
       </c>
-      <c r="F396" s="2">
+      <c r="F396" s="1">
         <v>46171</v>
       </c>
       <c r="G396" t="s">
@@ -18934,7 +18908,7 @@
       <c r="E397" t="s">
         <v>1082</v>
       </c>
-      <c r="F397" s="2">
+      <c r="F397" s="1">
         <v>46171</v>
       </c>
       <c r="G397" t="s">
@@ -18972,7 +18946,7 @@
       <c r="E398" t="s">
         <v>1083</v>
       </c>
-      <c r="F398" s="2">
+      <c r="F398" s="1">
         <v>46171</v>
       </c>
       <c r="G398" t="s">
@@ -19010,7 +18984,7 @@
       <c r="E399" t="s">
         <v>895</v>
       </c>
-      <c r="F399" s="2">
+      <c r="F399" s="1">
         <v>46163</v>
       </c>
       <c r="G399" t="s">
@@ -19025,7 +18999,7 @@
       <c r="K399" t="s">
         <v>1239</v>
       </c>
-      <c r="M399" s="2">
+      <c r="M399" s="1">
         <v>46171</v>
       </c>
       <c r="P399" t="b">
@@ -19048,7 +19022,7 @@
       <c r="E400" t="s">
         <v>1084</v>
       </c>
-      <c r="F400" s="2">
+      <c r="F400" s="1">
         <v>46171</v>
       </c>
       <c r="G400" t="s">
@@ -19086,7 +19060,7 @@
       <c r="E401" t="s">
         <v>1085</v>
       </c>
-      <c r="F401" s="2">
+      <c r="F401" s="1">
         <v>46171</v>
       </c>
       <c r="G401" t="s">
@@ -19124,7 +19098,7 @@
       <c r="E402" t="s">
         <v>1086</v>
       </c>
-      <c r="F402" s="2">
+      <c r="F402" s="1">
         <v>46171</v>
       </c>
       <c r="G402" t="s">
@@ -19162,7 +19136,7 @@
       <c r="E403" t="s">
         <v>1087</v>
       </c>
-      <c r="F403" s="2">
+      <c r="F403" s="1">
         <v>46171</v>
       </c>
       <c r="G403" t="s">
@@ -19197,7 +19171,7 @@
       <c r="E404" t="s">
         <v>1088</v>
       </c>
-      <c r="F404" s="2">
+      <c r="F404" s="1">
         <v>46171</v>
       </c>
       <c r="G404" t="s">
@@ -19232,7 +19206,7 @@
       <c r="E405">
         <v>9599</v>
       </c>
-      <c r="F405" s="2">
+      <c r="F405" s="1">
         <v>46183</v>
       </c>
       <c r="G405" t="s">
@@ -19261,7 +19235,7 @@
       <c r="E406">
         <v>14251</v>
       </c>
-      <c r="F406" s="2">
+      <c r="F406" s="1">
         <v>46183</v>
       </c>
       <c r="G406" t="s">
@@ -19293,7 +19267,7 @@
       <c r="E407">
         <v>19945</v>
       </c>
-      <c r="F407" s="2">
+      <c r="F407" s="1">
         <v>46183</v>
       </c>
       <c r="G407" t="s">
@@ -19325,7 +19299,7 @@
       <c r="E408">
         <v>14396</v>
       </c>
-      <c r="F408" s="2">
+      <c r="F408" s="1">
         <v>46183</v>
       </c>
       <c r="G408" t="s">
@@ -19357,7 +19331,7 @@
       <c r="E409">
         <v>9920</v>
       </c>
-      <c r="F409" s="2">
+      <c r="F409" s="1">
         <v>46183</v>
       </c>
       <c r="G409" t="s">
@@ -19389,7 +19363,7 @@
       <c r="E410">
         <v>20528</v>
       </c>
-      <c r="F410" s="2">
+      <c r="F410" s="1">
         <v>46183</v>
       </c>
       <c r="G410" t="s">
@@ -19421,7 +19395,7 @@
       <c r="E411" t="s">
         <v>1089</v>
       </c>
-      <c r="F411" s="2">
+      <c r="F411" s="1">
         <v>46188</v>
       </c>
       <c r="G411" t="s">
@@ -19453,7 +19427,7 @@
       <c r="E412" t="s">
         <v>1090</v>
       </c>
-      <c r="F412" s="2">
+      <c r="F412" s="1">
         <v>46188</v>
       </c>
       <c r="G412" t="s">
@@ -19485,7 +19459,7 @@
       <c r="E413" t="s">
         <v>1091</v>
       </c>
-      <c r="F413" s="2">
+      <c r="F413" s="1">
         <v>46188</v>
       </c>
       <c r="G413" t="s">
@@ -19517,7 +19491,7 @@
       <c r="E414" t="s">
         <v>1092</v>
       </c>
-      <c r="F414" s="2">
+      <c r="F414" s="1">
         <v>46188</v>
       </c>
       <c r="G414" t="s">
@@ -19549,7 +19523,7 @@
       <c r="E415" t="s">
         <v>968</v>
       </c>
-      <c r="F415" s="2">
+      <c r="F415" s="1">
         <v>46188</v>
       </c>
       <c r="G415" t="s">
@@ -19581,7 +19555,7 @@
       <c r="E416">
         <v>5844</v>
       </c>
-      <c r="F416" s="2">
+      <c r="F416" s="1">
         <v>46188</v>
       </c>
       <c r="G416" t="s">
@@ -19613,7 +19587,7 @@
       <c r="E417" t="s">
         <v>1093</v>
       </c>
-      <c r="F417" s="2">
+      <c r="F417" s="1">
         <v>46188</v>
       </c>
       <c r="G417" t="s">
@@ -19645,7 +19619,7 @@
       <c r="E418" t="s">
         <v>1094</v>
       </c>
-      <c r="F418" s="2">
+      <c r="F418" s="1">
         <v>46188</v>
       </c>
       <c r="G418" t="s">
@@ -19677,7 +19651,7 @@
       <c r="E419" t="s">
         <v>1095</v>
       </c>
-      <c r="F419" s="2">
+      <c r="F419" s="1">
         <v>46188</v>
       </c>
       <c r="G419" t="s">
@@ -19709,7 +19683,7 @@
       <c r="E420">
         <v>580</v>
       </c>
-      <c r="F420" s="2">
+      <c r="F420" s="1">
         <v>46188</v>
       </c>
       <c r="G420" t="s">
@@ -19741,7 +19715,7 @@
       <c r="E421" t="s">
         <v>1096</v>
       </c>
-      <c r="F421" s="2">
+      <c r="F421" s="1">
         <v>46188</v>
       </c>
       <c r="G421" t="s">
@@ -19773,7 +19747,7 @@
       <c r="E422" t="s">
         <v>1097</v>
       </c>
-      <c r="F422" s="2">
+      <c r="F422" s="1">
         <v>46188</v>
       </c>
       <c r="G422" t="s">
@@ -19805,7 +19779,7 @@
       <c r="E423" t="s">
         <v>1098</v>
       </c>
-      <c r="F423" s="2">
+      <c r="F423" s="1">
         <v>46188</v>
       </c>
       <c r="G423" t="s">
@@ -19837,7 +19811,7 @@
       <c r="E424" t="s">
         <v>1099</v>
       </c>
-      <c r="F424" s="2">
+      <c r="F424" s="1">
         <v>46188</v>
       </c>
       <c r="G424" t="s">
@@ -19869,7 +19843,7 @@
       <c r="E425" t="s">
         <v>1100</v>
       </c>
-      <c r="F425" s="2">
+      <c r="F425" s="1">
         <v>46188</v>
       </c>
       <c r="G425" t="s">
@@ -19901,7 +19875,7 @@
       <c r="E426" t="s">
         <v>1101</v>
       </c>
-      <c r="F426" s="2">
+      <c r="F426" s="1">
         <v>46188</v>
       </c>
       <c r="G426" t="s">
@@ -19933,7 +19907,7 @@
       <c r="E427">
         <v>6309</v>
       </c>
-      <c r="F427" s="2">
+      <c r="F427" s="1">
         <v>46188</v>
       </c>
       <c r="G427" t="s">
@@ -19965,7 +19939,7 @@
       <c r="E428">
         <v>504011190625165</v>
       </c>
-      <c r="F428" s="2">
+      <c r="F428" s="1">
         <v>46188</v>
       </c>
       <c r="G428" t="s">
@@ -19997,7 +19971,7 @@
       <c r="E429">
         <v>504011190625185</v>
       </c>
-      <c r="F429" s="2">
+      <c r="F429" s="1">
         <v>46188</v>
       </c>
       <c r="G429" t="s">
@@ -20029,7 +20003,7 @@
       <c r="E430" t="s">
         <v>1102</v>
       </c>
-      <c r="F430" s="2">
+      <c r="F430" s="1">
         <v>46188</v>
       </c>
       <c r="G430" t="s">
@@ -20061,7 +20035,7 @@
       <c r="E431" t="s">
         <v>1103</v>
       </c>
-      <c r="F431" s="2">
+      <c r="F431" s="1">
         <v>46188</v>
       </c>
       <c r="G431" t="s">
@@ -20093,7 +20067,7 @@
       <c r="E432" t="s">
         <v>1104</v>
       </c>
-      <c r="F432" s="2">
+      <c r="F432" s="1">
         <v>46188</v>
       </c>
       <c r="G432" t="s">
@@ -20125,7 +20099,7 @@
       <c r="E433" t="s">
         <v>1105</v>
       </c>
-      <c r="F433" s="2">
+      <c r="F433" s="1">
         <v>46188</v>
       </c>
       <c r="G433" t="s">
@@ -20157,7 +20131,7 @@
       <c r="E434">
         <v>328</v>
       </c>
-      <c r="F434" s="2">
+      <c r="F434" s="1">
         <v>46188</v>
       </c>
       <c r="G434" t="s">
@@ -20189,7 +20163,7 @@
       <c r="E435">
         <v>277</v>
       </c>
-      <c r="F435" s="2">
+      <c r="F435" s="1">
         <v>46188</v>
       </c>
       <c r="G435" t="s">
@@ -20221,7 +20195,7 @@
       <c r="E436">
         <v>477</v>
       </c>
-      <c r="F436" s="2">
+      <c r="F436" s="1">
         <v>46188</v>
       </c>
       <c r="G436" t="s">
@@ -20253,7 +20227,7 @@
       <c r="E437">
         <v>11</v>
       </c>
-      <c r="F437" s="2">
+      <c r="F437" s="1">
         <v>46188</v>
       </c>
       <c r="G437" t="s">
@@ -20285,7 +20259,7 @@
       <c r="E438" t="s">
         <v>1106</v>
       </c>
-      <c r="F438" s="2">
+      <c r="F438" s="1">
         <v>46188</v>
       </c>
       <c r="G438" t="s">
@@ -20317,7 +20291,7 @@
       <c r="E439" t="s">
         <v>1107</v>
       </c>
-      <c r="F439" s="2">
+      <c r="F439" s="1">
         <v>46196</v>
       </c>
       <c r="G439" t="s">
@@ -20349,7 +20323,7 @@
       <c r="E440" t="s">
         <v>1108</v>
       </c>
-      <c r="F440" s="2">
+      <c r="F440" s="1">
         <v>46196</v>
       </c>
       <c r="G440" t="s">
@@ -20381,7 +20355,7 @@
       <c r="E441">
         <v>86815651</v>
       </c>
-      <c r="F441" s="2">
+      <c r="F441" s="1">
         <v>46203</v>
       </c>
       <c r="G441" t="s">
@@ -20413,7 +20387,7 @@
       <c r="E442">
         <v>86817554</v>
       </c>
-      <c r="F442" s="2">
+      <c r="F442" s="1">
         <v>46203</v>
       </c>
       <c r="G442" t="s">
@@ -20445,7 +20419,7 @@
       <c r="E443" t="s">
         <v>1109</v>
       </c>
-      <c r="F443" s="2">
+      <c r="F443" s="1">
         <v>46205</v>
       </c>
       <c r="G443" t="s">
@@ -20477,7 +20451,7 @@
       <c r="E444" t="s">
         <v>1110</v>
       </c>
-      <c r="F444" s="2">
+      <c r="F444" s="1">
         <v>46205</v>
       </c>
       <c r="G444" t="s">
@@ -20509,7 +20483,7 @@
       <c r="E445">
         <v>4134</v>
       </c>
-      <c r="F445" s="2">
+      <c r="F445" s="1">
         <v>46205</v>
       </c>
       <c r="G445" t="s">
@@ -20541,7 +20515,7 @@
       <c r="E446">
         <v>22006508</v>
       </c>
-      <c r="F446" s="2">
+      <c r="F446" s="1">
         <v>46211</v>
       </c>
       <c r="G446" t="s">
@@ -20573,7 +20547,7 @@
       <c r="E447">
         <v>22005733</v>
       </c>
-      <c r="F447" s="2">
+      <c r="F447" s="1">
         <v>46211</v>
       </c>
       <c r="G447" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis (24/07/2026 17:54)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (25/07/2026 03:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4247,7 +4247,7 @@
         <v>1139</v>
       </c>
       <c r="I2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J2" t="s">
         <v>1142</v>
@@ -4285,7 +4285,7 @@
         <v>1139</v>
       </c>
       <c r="I3">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="J3" t="s">
         <v>1143</v>
@@ -4323,7 +4323,7 @@
         <v>1139</v>
       </c>
       <c r="I4">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="J4" t="s">
         <v>1143</v>
@@ -4361,7 +4361,7 @@
         <v>1139</v>
       </c>
       <c r="I5">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="J5" t="s">
         <v>1116</v>
@@ -4402,7 +4402,7 @@
         <v>1139</v>
       </c>
       <c r="I6">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J6" t="s">
         <v>1144</v>
@@ -4443,7 +4443,7 @@
         <v>1139</v>
       </c>
       <c r="I7">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J7" t="s">
         <v>1116</v>
@@ -4516,7 +4516,7 @@
         <v>1139</v>
       </c>
       <c r="I9">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J9" t="s">
         <v>1112</v>
@@ -4560,7 +4560,7 @@
         <v>1139</v>
       </c>
       <c r="I10">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J10" t="s">
         <v>1112</v>
@@ -4604,7 +4604,7 @@
         <v>1139</v>
       </c>
       <c r="I11">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J11" t="s">
         <v>1116</v>
@@ -4648,7 +4648,7 @@
         <v>1139</v>
       </c>
       <c r="I12">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J12" t="s">
         <v>1113</v>
@@ -4724,7 +4724,7 @@
         <v>1139</v>
       </c>
       <c r="I14">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J14" t="s">
         <v>1144</v>
@@ -4765,7 +4765,7 @@
         <v>1139</v>
       </c>
       <c r="I15">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J15" t="s">
         <v>1145</v>
@@ -4803,7 +4803,7 @@
         <v>1139</v>
       </c>
       <c r="I16">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J16" t="s">
         <v>1142</v>
@@ -4841,7 +4841,7 @@
         <v>1139</v>
       </c>
       <c r="I17">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J17" t="s">
         <v>1144</v>
@@ -4882,7 +4882,7 @@
         <v>1139</v>
       </c>
       <c r="I18">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J18" t="s">
         <v>1144</v>
@@ -4958,7 +4958,7 @@
         <v>1139</v>
       </c>
       <c r="I20">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J20" t="s">
         <v>1116</v>
@@ -5034,7 +5034,7 @@
         <v>1139</v>
       </c>
       <c r="I22">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J22" t="s">
         <v>1146</v>
@@ -5072,7 +5072,7 @@
         <v>1139</v>
       </c>
       <c r="I23">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J23" t="s">
         <v>1112</v>
@@ -5186,7 +5186,7 @@
         <v>1139</v>
       </c>
       <c r="I26">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J26" t="s">
         <v>1116</v>
@@ -5230,7 +5230,7 @@
         <v>1139</v>
       </c>
       <c r="I27">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J27" t="s">
         <v>1146</v>
@@ -5332,7 +5332,7 @@
         <v>1139</v>
       </c>
       <c r="I30">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J30" t="s">
         <v>1115</v>
@@ -5408,7 +5408,7 @@
         <v>1139</v>
       </c>
       <c r="I32">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J32" t="s">
         <v>1142</v>
@@ -5641,7 +5641,7 @@
         <v>1139</v>
       </c>
       <c r="I39">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J39" t="s">
         <v>1147</v>
@@ -5676,7 +5676,7 @@
         <v>1139</v>
       </c>
       <c r="I40">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J40" t="s">
         <v>1145</v>
@@ -5819,7 +5819,7 @@
         <v>1139</v>
       </c>
       <c r="I44">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J44" t="s">
         <v>1112</v>
@@ -5863,7 +5863,7 @@
         <v>1139</v>
       </c>
       <c r="I45">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J45" t="s">
         <v>1113</v>
@@ -5907,7 +5907,7 @@
         <v>1139</v>
       </c>
       <c r="I46">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J46" t="s">
         <v>1146</v>
@@ -5945,7 +5945,7 @@
         <v>1139</v>
       </c>
       <c r="I47">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J47" t="s">
         <v>1124</v>
@@ -5989,7 +5989,7 @@
         <v>1139</v>
       </c>
       <c r="I48">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J48" t="s">
         <v>1146</v>
@@ -6056,7 +6056,7 @@
         <v>1139</v>
       </c>
       <c r="I50">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J50" t="s">
         <v>1146</v>
@@ -6129,7 +6129,7 @@
         <v>1139</v>
       </c>
       <c r="I52">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J52" t="s">
         <v>1142</v>
@@ -6167,7 +6167,7 @@
         <v>1139</v>
       </c>
       <c r="I53">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J53" t="s">
         <v>1143</v>
@@ -6205,7 +6205,7 @@
         <v>1139</v>
       </c>
       <c r="I54">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J54" t="s">
         <v>1143</v>
@@ -6307,7 +6307,7 @@
         <v>1139</v>
       </c>
       <c r="I57">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J57" t="s">
         <v>1146</v>
@@ -6505,7 +6505,7 @@
         <v>1139</v>
       </c>
       <c r="I63">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J63" t="s">
         <v>1113</v>
@@ -6549,7 +6549,7 @@
         <v>1139</v>
       </c>
       <c r="I64">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J64" t="s">
         <v>1144</v>
@@ -6765,7 +6765,7 @@
         <v>1139</v>
       </c>
       <c r="I70">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J70" t="s">
         <v>1143</v>
@@ -6803,7 +6803,7 @@
         <v>1139</v>
       </c>
       <c r="I71">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J71" t="s">
         <v>1149</v>
@@ -6873,7 +6873,7 @@
         <v>1139</v>
       </c>
       <c r="I73">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J73" t="s">
         <v>1142</v>
@@ -6946,7 +6946,7 @@
         <v>1139</v>
       </c>
       <c r="I75">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J75" t="s">
         <v>1143</v>
@@ -6984,7 +6984,7 @@
         <v>1139</v>
       </c>
       <c r="I76">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J76" t="s">
         <v>1149</v>
@@ -7089,7 +7089,7 @@
         <v>1139</v>
       </c>
       <c r="I79">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J79" t="s">
         <v>1149</v>
@@ -7124,7 +7124,7 @@
         <v>1139</v>
       </c>
       <c r="I80">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J80" t="s">
         <v>1143</v>
@@ -7197,7 +7197,7 @@
         <v>1139</v>
       </c>
       <c r="I82">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J82" t="s">
         <v>1146</v>
@@ -7270,7 +7270,7 @@
         <v>1139</v>
       </c>
       <c r="I84">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J84" t="s">
         <v>1116</v>
@@ -7314,7 +7314,7 @@
         <v>1139</v>
       </c>
       <c r="I85">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J85" t="s">
         <v>1143</v>
@@ -7352,7 +7352,7 @@
         <v>1139</v>
       </c>
       <c r="I86">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J86" t="s">
         <v>1143</v>
@@ -7390,7 +7390,7 @@
         <v>1139</v>
       </c>
       <c r="I87">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J87" t="s">
         <v>1116</v>
@@ -7504,7 +7504,7 @@
         <v>1139</v>
       </c>
       <c r="I90">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J90" t="s">
         <v>1116</v>
@@ -7545,7 +7545,7 @@
         <v>1139</v>
       </c>
       <c r="I91">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J91" t="s">
         <v>1145</v>
@@ -7609,7 +7609,7 @@
         <v>1139</v>
       </c>
       <c r="I93">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J93" t="s">
         <v>1145</v>
@@ -7647,7 +7647,7 @@
         <v>1139</v>
       </c>
       <c r="I94">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J94" t="s">
         <v>1146</v>
@@ -7685,7 +7685,7 @@
         <v>1139</v>
       </c>
       <c r="I95">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J95" t="s">
         <v>1145</v>
@@ -7723,7 +7723,7 @@
         <v>1139</v>
       </c>
       <c r="I96">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J96" t="s">
         <v>1116</v>
@@ -7767,7 +7767,7 @@
         <v>1139</v>
       </c>
       <c r="I97">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J97" t="s">
         <v>1116</v>
@@ -7808,7 +7808,7 @@
         <v>1139</v>
       </c>
       <c r="I98">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J98" t="s">
         <v>1146</v>
@@ -7875,7 +7875,7 @@
         <v>1139</v>
       </c>
       <c r="I100">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J100" t="s">
         <v>1145</v>
@@ -8000,7 +8000,7 @@
         <v>1139</v>
       </c>
       <c r="I104">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J104" t="s">
         <v>1145</v>
@@ -8038,7 +8038,7 @@
         <v>1139</v>
       </c>
       <c r="I105">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J105" t="s">
         <v>1145</v>
@@ -8076,7 +8076,7 @@
         <v>1139</v>
       </c>
       <c r="I106">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J106" t="s">
         <v>1144</v>
@@ -8117,7 +8117,7 @@
         <v>1139</v>
       </c>
       <c r="I107">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J107" t="s">
         <v>1144</v>
@@ -8158,7 +8158,7 @@
         <v>1139</v>
       </c>
       <c r="I108">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J108" t="s">
         <v>1143</v>
@@ -8196,7 +8196,7 @@
         <v>1139</v>
       </c>
       <c r="I109">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J109" t="s">
         <v>1143</v>
@@ -8403,7 +8403,7 @@
         <v>1139</v>
       </c>
       <c r="I115">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J115" t="s">
         <v>1143</v>
@@ -8441,7 +8441,7 @@
         <v>1139</v>
       </c>
       <c r="I116">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J116" t="s">
         <v>1143</v>
@@ -8479,7 +8479,7 @@
         <v>1139</v>
       </c>
       <c r="I117">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J117" t="s">
         <v>1143</v>
@@ -8517,7 +8517,7 @@
         <v>1139</v>
       </c>
       <c r="I118">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J118" t="s">
         <v>1143</v>
@@ -8555,7 +8555,7 @@
         <v>1139</v>
       </c>
       <c r="I119">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J119" t="s">
         <v>1143</v>
@@ -8593,7 +8593,7 @@
         <v>1139</v>
       </c>
       <c r="I120">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J120" t="s">
         <v>1143</v>
@@ -8631,7 +8631,7 @@
         <v>1139</v>
       </c>
       <c r="I121">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J121" t="s">
         <v>1113</v>
@@ -8675,7 +8675,7 @@
         <v>1139</v>
       </c>
       <c r="I122">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J122" t="s">
         <v>1143</v>
@@ -8742,7 +8742,7 @@
         <v>1139</v>
       </c>
       <c r="I124">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J124" t="s">
         <v>1143</v>
@@ -8780,7 +8780,7 @@
         <v>1139</v>
       </c>
       <c r="I125">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J125" t="s">
         <v>1149</v>
@@ -8882,7 +8882,7 @@
         <v>1139</v>
       </c>
       <c r="I128">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J128" t="s">
         <v>1143</v>
@@ -8920,7 +8920,7 @@
         <v>1139</v>
       </c>
       <c r="I129">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J129" t="s">
         <v>1142</v>
@@ -8958,7 +8958,7 @@
         <v>1139</v>
       </c>
       <c r="I130">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J130" t="s">
         <v>1113</v>
@@ -9037,7 +9037,7 @@
         <v>1139</v>
       </c>
       <c r="I132">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J132" t="s">
         <v>1114</v>
@@ -9110,7 +9110,7 @@
         <v>1139</v>
       </c>
       <c r="I134">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J134" t="s">
         <v>1142</v>
@@ -9235,7 +9235,7 @@
         <v>1139</v>
       </c>
       <c r="I138">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J138" t="s">
         <v>1143</v>
@@ -9552,7 +9552,7 @@
         <v>1139</v>
       </c>
       <c r="I148">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J148" t="s">
         <v>1143</v>
@@ -9590,7 +9590,7 @@
         <v>1139</v>
       </c>
       <c r="I149">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J149" t="s">
         <v>1149</v>
@@ -9625,7 +9625,7 @@
         <v>1139</v>
       </c>
       <c r="I150">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J150" t="s">
         <v>1113</v>
@@ -9704,7 +9704,7 @@
         <v>1139</v>
       </c>
       <c r="I152">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J152" t="s">
         <v>1144</v>
@@ -9745,7 +9745,7 @@
         <v>1139</v>
       </c>
       <c r="I153">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J153" t="s">
         <v>1143</v>
@@ -9818,7 +9818,7 @@
         <v>1139</v>
       </c>
       <c r="I155">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J155" t="s">
         <v>1149</v>
@@ -9853,7 +9853,7 @@
         <v>1139</v>
       </c>
       <c r="I156">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J156" t="s">
         <v>1143</v>
@@ -9891,7 +9891,7 @@
         <v>1139</v>
       </c>
       <c r="I157">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J157" t="s">
         <v>1145</v>
@@ -9929,7 +9929,7 @@
         <v>1139</v>
       </c>
       <c r="I158">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J158" t="s">
         <v>1116</v>
@@ -9970,7 +9970,7 @@
         <v>1139</v>
       </c>
       <c r="I159">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J159" t="s">
         <v>1143</v>
@@ -10008,7 +10008,7 @@
         <v>1139</v>
       </c>
       <c r="I160">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J160" t="s">
         <v>1143</v>
@@ -10046,7 +10046,7 @@
         <v>1139</v>
       </c>
       <c r="I161">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J161" t="s">
         <v>1113</v>
@@ -10090,7 +10090,7 @@
         <v>1139</v>
       </c>
       <c r="I162">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J162" t="s">
         <v>1116</v>
@@ -10131,7 +10131,7 @@
         <v>1139</v>
       </c>
       <c r="I163">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J163" t="s">
         <v>1116</v>
@@ -10172,7 +10172,7 @@
         <v>1141</v>
       </c>
       <c r="I164">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J164" t="s">
         <v>1150</v>
@@ -10207,7 +10207,7 @@
         <v>1139</v>
       </c>
       <c r="I165">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J165" t="s">
         <v>1143</v>
@@ -10312,7 +10312,7 @@
         <v>1139</v>
       </c>
       <c r="I168">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J168" t="s">
         <v>1146</v>
@@ -10353,7 +10353,7 @@
         <v>1139</v>
       </c>
       <c r="I169">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J169" t="s">
         <v>1116</v>
@@ -10429,7 +10429,7 @@
         <v>1139</v>
       </c>
       <c r="I171">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J171" t="s">
         <v>1143</v>
@@ -10572,7 +10572,7 @@
         <v>1139</v>
       </c>
       <c r="I175">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J175" t="s">
         <v>1113</v>
@@ -10616,7 +10616,7 @@
         <v>1139</v>
       </c>
       <c r="I176">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J176" t="s">
         <v>1143</v>
@@ -10654,7 +10654,7 @@
         <v>1139</v>
       </c>
       <c r="I177">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J177" t="s">
         <v>1113</v>
@@ -10698,7 +10698,7 @@
         <v>1139</v>
       </c>
       <c r="I178">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J178" t="s">
         <v>1142</v>
@@ -10765,7 +10765,7 @@
         <v>1139</v>
       </c>
       <c r="I180">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J180" t="s">
         <v>1142</v>
@@ -10867,7 +10867,7 @@
         <v>1139</v>
       </c>
       <c r="I183">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J183" t="s">
         <v>1143</v>
@@ -10902,7 +10902,7 @@
         <v>1139</v>
       </c>
       <c r="I184">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J184" t="s">
         <v>1149</v>
@@ -10937,7 +10937,7 @@
         <v>1139</v>
       </c>
       <c r="I185">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J185" t="s">
         <v>1143</v>
@@ -10975,7 +10975,7 @@
         <v>1139</v>
       </c>
       <c r="I186">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J186" t="s">
         <v>1143</v>
@@ -11013,7 +11013,7 @@
         <v>1139</v>
       </c>
       <c r="I187">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J187" t="s">
         <v>1114</v>
@@ -11057,7 +11057,7 @@
         <v>1139</v>
       </c>
       <c r="I188">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J188" t="s">
         <v>1116</v>
@@ -11101,7 +11101,7 @@
         <v>1139</v>
       </c>
       <c r="I189">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J189" t="s">
         <v>1116</v>
@@ -11142,7 +11142,7 @@
         <v>1139</v>
       </c>
       <c r="I190">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J190" t="s">
         <v>1145</v>
@@ -11180,7 +11180,7 @@
         <v>1139</v>
       </c>
       <c r="I191">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J191" t="s">
         <v>1118</v>
@@ -11221,7 +11221,7 @@
         <v>1139</v>
       </c>
       <c r="I192">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J192" t="s">
         <v>1143</v>
@@ -11259,7 +11259,7 @@
         <v>1139</v>
       </c>
       <c r="I193">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J193" t="s">
         <v>1148</v>
@@ -11326,7 +11326,7 @@
         <v>1139</v>
       </c>
       <c r="I195">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J195" t="s">
         <v>1145</v>
@@ -11451,7 +11451,7 @@
         <v>1139</v>
       </c>
       <c r="I199">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J199" t="s">
         <v>1114</v>
@@ -11492,7 +11492,7 @@
         <v>1139</v>
       </c>
       <c r="I200">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J200" t="s">
         <v>1145</v>
@@ -11530,7 +11530,7 @@
         <v>1139</v>
       </c>
       <c r="I201">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J201" t="s">
         <v>1143</v>
@@ -11568,7 +11568,7 @@
         <v>1139</v>
       </c>
       <c r="I202">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J202" t="s">
         <v>1143</v>
@@ -11606,7 +11606,7 @@
         <v>1139</v>
       </c>
       <c r="I203">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J203" t="s">
         <v>1143</v>
@@ -11644,7 +11644,7 @@
         <v>1139</v>
       </c>
       <c r="I204">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J204" t="s">
         <v>1142</v>
@@ -11682,7 +11682,7 @@
         <v>1139</v>
       </c>
       <c r="I205">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J205" t="s">
         <v>1142</v>
@@ -11755,7 +11755,7 @@
         <v>1139</v>
       </c>
       <c r="I207">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J207" t="s">
         <v>1116</v>
@@ -11796,7 +11796,7 @@
         <v>1139</v>
       </c>
       <c r="I208">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J208" t="s">
         <v>1144</v>
@@ -11837,7 +11837,7 @@
         <v>1139</v>
       </c>
       <c r="I209">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J209" t="s">
         <v>1113</v>
@@ -11878,7 +11878,7 @@
         <v>1139</v>
       </c>
       <c r="I210">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J210" t="s">
         <v>1146</v>
@@ -11986,7 +11986,7 @@
         <v>1139</v>
       </c>
       <c r="I213">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J213" t="s">
         <v>1143</v>
@@ -12024,7 +12024,7 @@
         <v>1139</v>
       </c>
       <c r="I214">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J214" t="s">
         <v>1116</v>
@@ -12068,7 +12068,7 @@
         <v>1139</v>
       </c>
       <c r="I215">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J215" t="s">
         <v>1143</v>
@@ -12135,7 +12135,7 @@
         <v>1139</v>
       </c>
       <c r="I217">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J217" t="s">
         <v>1115</v>
@@ -12176,7 +12176,7 @@
         <v>1139</v>
       </c>
       <c r="I218">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J218" t="s">
         <v>1145</v>
@@ -12214,7 +12214,7 @@
         <v>1139</v>
       </c>
       <c r="I219">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J219" t="s">
         <v>1145</v>
@@ -12252,7 +12252,7 @@
         <v>1139</v>
       </c>
       <c r="I220">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J220" t="s">
         <v>1145</v>
@@ -12325,7 +12325,7 @@
         <v>1139</v>
       </c>
       <c r="I222">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J222" t="s">
         <v>1143</v>
@@ -12363,7 +12363,7 @@
         <v>1139</v>
       </c>
       <c r="I223">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J223" t="s">
         <v>1143</v>
@@ -12401,7 +12401,7 @@
         <v>1139</v>
       </c>
       <c r="I224">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J224" t="s">
         <v>1143</v>
@@ -12439,7 +12439,7 @@
         <v>1139</v>
       </c>
       <c r="I225">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J225" t="s">
         <v>1143</v>
@@ -12477,7 +12477,7 @@
         <v>1139</v>
       </c>
       <c r="I226">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J226" t="s">
         <v>1143</v>
@@ -12515,7 +12515,7 @@
         <v>1139</v>
       </c>
       <c r="I227">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J227" t="s">
         <v>1143</v>
@@ -12553,7 +12553,7 @@
         <v>1139</v>
       </c>
       <c r="I228">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J228" t="s">
         <v>1143</v>
@@ -12626,7 +12626,7 @@
         <v>1139</v>
       </c>
       <c r="I230">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J230" t="s">
         <v>1146</v>
@@ -12664,7 +12664,7 @@
         <v>1139</v>
       </c>
       <c r="I231">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J231" t="s">
         <v>1124</v>
@@ -12775,7 +12775,7 @@
         <v>1139</v>
       </c>
       <c r="I234">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J234" t="s">
         <v>1124</v>
@@ -12819,7 +12819,7 @@
         <v>1139</v>
       </c>
       <c r="I235">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J235" t="s">
         <v>1124</v>
@@ -12863,7 +12863,7 @@
         <v>1139</v>
       </c>
       <c r="I236">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J236" t="s">
         <v>1113</v>
@@ -12904,7 +12904,7 @@
         <v>1139</v>
       </c>
       <c r="I237">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J237" t="s">
         <v>1143</v>
@@ -12971,7 +12971,7 @@
         <v>1139</v>
       </c>
       <c r="I239">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J239" t="s">
         <v>1116</v>
@@ -13082,7 +13082,7 @@
         <v>1139</v>
       </c>
       <c r="I242">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J242" t="s">
         <v>1142</v>
@@ -13152,7 +13152,7 @@
         <v>1139</v>
       </c>
       <c r="I244">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J244" t="s">
         <v>1145</v>
@@ -13190,7 +13190,7 @@
         <v>1139</v>
       </c>
       <c r="I245">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J245" t="s">
         <v>1145</v>
@@ -13228,7 +13228,7 @@
         <v>1139</v>
       </c>
       <c r="I246">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J246" t="s">
         <v>1112</v>
@@ -13327,7 +13327,7 @@
         <v>1139</v>
       </c>
       <c r="I249">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J249" t="s">
         <v>1143</v>
@@ -13365,7 +13365,7 @@
         <v>1139</v>
       </c>
       <c r="I250">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J250" t="s">
         <v>1145</v>
@@ -13473,7 +13473,7 @@
         <v>1139</v>
       </c>
       <c r="I253">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J253" t="s">
         <v>1146</v>
@@ -13511,7 +13511,7 @@
         <v>1139</v>
       </c>
       <c r="I254">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J254" t="s">
         <v>1146</v>
@@ -13549,7 +13549,7 @@
         <v>1139</v>
       </c>
       <c r="I255">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J255" t="s">
         <v>1145</v>
@@ -13587,7 +13587,7 @@
         <v>1139</v>
       </c>
       <c r="I256">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J256" t="s">
         <v>1143</v>
@@ -13686,7 +13686,7 @@
         <v>1139</v>
       </c>
       <c r="I259">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J259" t="s">
         <v>1145</v>
@@ -13724,7 +13724,7 @@
         <v>1139</v>
       </c>
       <c r="I260">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J260" t="s">
         <v>1145</v>
@@ -13762,7 +13762,7 @@
         <v>1139</v>
       </c>
       <c r="I261">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J261" t="s">
         <v>1146</v>
@@ -13800,7 +13800,7 @@
         <v>1139</v>
       </c>
       <c r="I262">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J262" t="s">
         <v>1112</v>
@@ -13879,7 +13879,7 @@
         <v>1139</v>
       </c>
       <c r="I264">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J264" t="s">
         <v>1146</v>
@@ -13917,7 +13917,7 @@
         <v>1139</v>
       </c>
       <c r="I265">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J265" t="s">
         <v>1146</v>
@@ -13955,7 +13955,7 @@
         <v>1139</v>
       </c>
       <c r="I266">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J266" t="s">
         <v>1145</v>
@@ -13993,7 +13993,7 @@
         <v>1139</v>
       </c>
       <c r="I267">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J267" t="s">
         <v>1146</v>
@@ -14031,7 +14031,7 @@
         <v>1139</v>
       </c>
       <c r="I268">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J268" t="s">
         <v>1143</v>
@@ -14066,7 +14066,7 @@
         <v>1139</v>
       </c>
       <c r="I269">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J269" t="s">
         <v>1143</v>
@@ -14104,7 +14104,7 @@
         <v>1139</v>
       </c>
       <c r="I270">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J270" t="s">
         <v>1146</v>
@@ -14142,7 +14142,7 @@
         <v>1139</v>
       </c>
       <c r="I271">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J271" t="s">
         <v>1146</v>
@@ -14180,7 +14180,7 @@
         <v>1139</v>
       </c>
       <c r="I272">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J272" t="s">
         <v>1113</v>
@@ -14259,7 +14259,7 @@
         <v>1139</v>
       </c>
       <c r="I274">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J274" t="s">
         <v>1143</v>
@@ -14332,7 +14332,7 @@
         <v>1139</v>
       </c>
       <c r="I276">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J276" t="s">
         <v>1147</v>
@@ -14370,7 +14370,7 @@
         <v>1139</v>
       </c>
       <c r="I277">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J277" t="s">
         <v>1143</v>
@@ -14408,7 +14408,7 @@
         <v>1139</v>
       </c>
       <c r="I278">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J278" t="s">
         <v>1146</v>
@@ -14446,7 +14446,7 @@
         <v>1139</v>
       </c>
       <c r="I279">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J279" t="s">
         <v>1145</v>
@@ -14487,7 +14487,7 @@
         <v>1139</v>
       </c>
       <c r="I280">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J280" t="s">
         <v>1143</v>
@@ -14525,7 +14525,7 @@
         <v>1139</v>
       </c>
       <c r="I281">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J281" t="s">
         <v>1143</v>
@@ -14563,7 +14563,7 @@
         <v>1139</v>
       </c>
       <c r="I282">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J282" t="s">
         <v>1143</v>
@@ -14770,7 +14770,7 @@
         <v>1139</v>
       </c>
       <c r="I288">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J288" t="s">
         <v>1146</v>
@@ -14837,7 +14837,7 @@
         <v>1139</v>
       </c>
       <c r="I290">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J290" t="s">
         <v>1145</v>
@@ -14875,7 +14875,7 @@
         <v>1139</v>
       </c>
       <c r="I291">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J291" t="s">
         <v>1145</v>
@@ -14913,7 +14913,7 @@
         <v>1139</v>
       </c>
       <c r="I292">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J292" t="s">
         <v>1146</v>
@@ -14951,7 +14951,7 @@
         <v>1139</v>
       </c>
       <c r="I293">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J293" t="s">
         <v>1147</v>
@@ -14989,7 +14989,7 @@
         <v>1139</v>
       </c>
       <c r="I294">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J294" t="s">
         <v>1149</v>
@@ -15024,7 +15024,7 @@
         <v>1139</v>
       </c>
       <c r="I295">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J295" t="s">
         <v>1149</v>
@@ -15059,7 +15059,7 @@
         <v>1139</v>
       </c>
       <c r="I296">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J296" t="s">
         <v>1149</v>
@@ -15129,7 +15129,7 @@
         <v>1139</v>
       </c>
       <c r="I298">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J298" t="s">
         <v>1143</v>
@@ -15167,7 +15167,7 @@
         <v>1139</v>
       </c>
       <c r="I299">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J299" t="s">
         <v>1146</v>
@@ -15205,7 +15205,7 @@
         <v>1139</v>
       </c>
       <c r="I300">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J300" t="s">
         <v>1146</v>
@@ -15243,7 +15243,7 @@
         <v>1139</v>
       </c>
       <c r="I301">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J301" t="s">
         <v>1146</v>
@@ -15281,7 +15281,7 @@
         <v>1139</v>
       </c>
       <c r="I302">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J302" t="s">
         <v>1146</v>
@@ -15319,7 +15319,7 @@
         <v>1139</v>
       </c>
       <c r="I303">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J303" t="s">
         <v>1143</v>
@@ -15357,7 +15357,7 @@
         <v>1139</v>
       </c>
       <c r="I304">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J304" t="s">
         <v>1146</v>
@@ -15395,7 +15395,7 @@
         <v>1139</v>
       </c>
       <c r="I305">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J305" t="s">
         <v>1116</v>
@@ -15436,7 +15436,7 @@
         <v>1139</v>
       </c>
       <c r="I306">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J306" t="s">
         <v>1116</v>
@@ -15477,7 +15477,7 @@
         <v>1139</v>
       </c>
       <c r="I307">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J307" t="s">
         <v>1142</v>
@@ -15515,7 +15515,7 @@
         <v>1139</v>
       </c>
       <c r="I308">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J308" t="s">
         <v>1142</v>
@@ -15553,7 +15553,7 @@
         <v>1139</v>
       </c>
       <c r="I309">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J309" t="s">
         <v>1142</v>
@@ -15591,7 +15591,7 @@
         <v>1139</v>
       </c>
       <c r="I310">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J310" t="s">
         <v>1143</v>
@@ -15629,7 +15629,7 @@
         <v>1139</v>
       </c>
       <c r="I311">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J311" t="s">
         <v>1142</v>
@@ -15667,7 +15667,7 @@
         <v>1139</v>
       </c>
       <c r="I312">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J312" t="s">
         <v>1143</v>
@@ -15740,7 +15740,7 @@
         <v>1139</v>
       </c>
       <c r="I314">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J314" t="s">
         <v>1143</v>
@@ -15778,7 +15778,7 @@
         <v>1139</v>
       </c>
       <c r="I315">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J315" t="s">
         <v>1143</v>
@@ -15816,7 +15816,7 @@
         <v>1139</v>
       </c>
       <c r="I316">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J316" t="s">
         <v>1143</v>
@@ -15854,7 +15854,7 @@
         <v>1139</v>
       </c>
       <c r="I317">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J317" t="s">
         <v>1143</v>
@@ -15959,7 +15959,7 @@
         <v>1139</v>
       </c>
       <c r="I320">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J320" t="s">
         <v>1147</v>
@@ -15997,7 +15997,7 @@
         <v>1139</v>
       </c>
       <c r="I321">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J321" t="s">
         <v>1143</v>
@@ -16035,7 +16035,7 @@
         <v>1139</v>
       </c>
       <c r="I322">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J322" t="s">
         <v>1116</v>
@@ -16076,7 +16076,7 @@
         <v>1139</v>
       </c>
       <c r="I323">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J323" t="s">
         <v>1143</v>
@@ -16114,7 +16114,7 @@
         <v>1139</v>
       </c>
       <c r="I324">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J324" t="s">
         <v>1143</v>
@@ -16152,7 +16152,7 @@
         <v>1139</v>
       </c>
       <c r="I325">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J325" t="s">
         <v>1116</v>
@@ -16193,7 +16193,7 @@
         <v>1139</v>
       </c>
       <c r="I326">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J326" t="s">
         <v>1143</v>
@@ -16231,7 +16231,7 @@
         <v>1139</v>
       </c>
       <c r="I327">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J327" t="s">
         <v>1116</v>
@@ -16272,7 +16272,7 @@
         <v>1139</v>
       </c>
       <c r="I328">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J328" t="s">
         <v>1116</v>
@@ -16313,7 +16313,7 @@
         <v>1139</v>
       </c>
       <c r="I329">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J329" t="s">
         <v>1116</v>
@@ -16354,7 +16354,7 @@
         <v>1139</v>
       </c>
       <c r="I330">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J330" t="s">
         <v>1116</v>
@@ -16395,7 +16395,7 @@
         <v>1139</v>
       </c>
       <c r="I331">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J331" t="s">
         <v>1142</v>
@@ -16433,7 +16433,7 @@
         <v>1139</v>
       </c>
       <c r="I332">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J332" t="s">
         <v>1143</v>
@@ -16471,7 +16471,7 @@
         <v>1139</v>
       </c>
       <c r="I333">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J333" t="s">
         <v>1146</v>
@@ -16509,7 +16509,7 @@
         <v>1139</v>
       </c>
       <c r="I334">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J334" t="s">
         <v>1143</v>
@@ -16585,7 +16585,7 @@
         <v>1139</v>
       </c>
       <c r="I336">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J336" t="s">
         <v>1145</v>
@@ -16661,7 +16661,7 @@
         <v>1139</v>
       </c>
       <c r="I338">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J338" t="s">
         <v>1145</v>
@@ -16728,7 +16728,7 @@
         <v>1139</v>
       </c>
       <c r="I340">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J340" t="s">
         <v>1142</v>
@@ -16766,7 +16766,7 @@
         <v>1139</v>
       </c>
       <c r="I341">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J341" t="s">
         <v>1142</v>
@@ -16804,7 +16804,7 @@
         <v>1139</v>
       </c>
       <c r="I342">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J342" t="s">
         <v>1142</v>
@@ -16842,7 +16842,7 @@
         <v>1139</v>
       </c>
       <c r="I343">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J343" t="s">
         <v>1143</v>
@@ -16880,7 +16880,7 @@
         <v>1139</v>
       </c>
       <c r="I344">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J344" t="s">
         <v>1143</v>
@@ -16918,7 +16918,7 @@
         <v>1139</v>
       </c>
       <c r="I345">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J345" t="s">
         <v>1142</v>
@@ -16956,7 +16956,7 @@
         <v>1139</v>
       </c>
       <c r="I346">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J346" t="s">
         <v>1143</v>
@@ -16994,7 +16994,7 @@
         <v>1139</v>
       </c>
       <c r="I347">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J347" t="s">
         <v>1116</v>
@@ -17035,7 +17035,7 @@
         <v>1139</v>
       </c>
       <c r="I348">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J348" t="s">
         <v>1116</v>
@@ -17076,7 +17076,7 @@
         <v>1139</v>
       </c>
       <c r="I349">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J349" t="s">
         <v>1147</v>
@@ -17114,7 +17114,7 @@
         <v>1139</v>
       </c>
       <c r="I350">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J350" t="s">
         <v>1149</v>
@@ -17149,7 +17149,7 @@
         <v>1139</v>
       </c>
       <c r="I351">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J351" t="s">
         <v>1147</v>
@@ -17187,7 +17187,7 @@
         <v>1139</v>
       </c>
       <c r="I352">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J352" t="s">
         <v>1147</v>
@@ -17225,7 +17225,7 @@
         <v>1139</v>
       </c>
       <c r="I353">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J353" t="s">
         <v>1146</v>
@@ -17263,7 +17263,7 @@
         <v>1139</v>
       </c>
       <c r="I354">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J354" t="s">
         <v>1146</v>
@@ -17301,7 +17301,7 @@
         <v>1139</v>
       </c>
       <c r="I355">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J355" t="s">
         <v>1116</v>
@@ -17380,7 +17380,7 @@
         <v>1139</v>
       </c>
       <c r="I357">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J357" t="s">
         <v>1146</v>
@@ -17418,7 +17418,7 @@
         <v>1139</v>
       </c>
       <c r="I358">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J358" t="s">
         <v>1146</v>
@@ -17456,7 +17456,7 @@
         <v>1139</v>
       </c>
       <c r="I359">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J359" t="s">
         <v>1146</v>
@@ -17497,7 +17497,7 @@
         <v>1139</v>
       </c>
       <c r="I360">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J360" t="s">
         <v>1146</v>
@@ -17535,7 +17535,7 @@
         <v>1139</v>
       </c>
       <c r="I361">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J361" t="s">
         <v>1146</v>
@@ -17573,7 +17573,7 @@
         <v>1139</v>
       </c>
       <c r="I362">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J362" t="s">
         <v>1146</v>
@@ -17611,7 +17611,7 @@
         <v>1139</v>
       </c>
       <c r="I363">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J363" t="s">
         <v>1146</v>
@@ -17649,7 +17649,7 @@
         <v>1139</v>
       </c>
       <c r="I364">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J364" t="s">
         <v>1146</v>
@@ -17687,7 +17687,7 @@
         <v>1139</v>
       </c>
       <c r="I365">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J365" t="s">
         <v>1145</v>
@@ -17725,7 +17725,7 @@
         <v>1139</v>
       </c>
       <c r="I366">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J366" t="s">
         <v>1146</v>
@@ -17763,7 +17763,7 @@
         <v>1139</v>
       </c>
       <c r="I367">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J367" t="s">
         <v>1146</v>
@@ -17801,7 +17801,7 @@
         <v>1139</v>
       </c>
       <c r="I368">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J368" t="s">
         <v>1146</v>
@@ -17839,7 +17839,7 @@
         <v>1139</v>
       </c>
       <c r="I369">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J369" t="s">
         <v>1146</v>
@@ -17877,7 +17877,7 @@
         <v>1139</v>
       </c>
       <c r="I370">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J370" t="s">
         <v>1146</v>
@@ -17915,7 +17915,7 @@
         <v>1139</v>
       </c>
       <c r="I371">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J371" t="s">
         <v>1116</v>
@@ -17956,7 +17956,7 @@
         <v>1139</v>
       </c>
       <c r="I372">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J372" t="s">
         <v>1112</v>
@@ -18000,7 +18000,7 @@
         <v>1139</v>
       </c>
       <c r="I373">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J373" t="s">
         <v>1142</v>
@@ -18038,7 +18038,7 @@
         <v>1139</v>
       </c>
       <c r="I374">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J374" t="s">
         <v>1142</v>
@@ -18076,7 +18076,7 @@
         <v>1139</v>
       </c>
       <c r="I375">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J375" t="s">
         <v>1146</v>
@@ -18114,7 +18114,7 @@
         <v>1139</v>
       </c>
       <c r="I376">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J376" t="s">
         <v>1146</v>
@@ -18190,7 +18190,7 @@
         <v>1139</v>
       </c>
       <c r="I378">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J378" t="s">
         <v>1146</v>
@@ -18228,7 +18228,7 @@
         <v>1139</v>
       </c>
       <c r="I379">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J379" t="s">
         <v>1112</v>
@@ -18269,7 +18269,7 @@
         <v>1139</v>
       </c>
       <c r="I380">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J380" t="s">
         <v>1146</v>
@@ -18307,7 +18307,7 @@
         <v>1139</v>
       </c>
       <c r="I381">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J381" t="s">
         <v>1146</v>
@@ -18345,7 +18345,7 @@
         <v>1139</v>
       </c>
       <c r="I382">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J382" t="s">
         <v>1146</v>
@@ -18383,7 +18383,7 @@
         <v>1139</v>
       </c>
       <c r="I383">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J383" t="s">
         <v>1146</v>
@@ -18421,7 +18421,7 @@
         <v>1139</v>
       </c>
       <c r="I384">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J384" t="s">
         <v>1142</v>
@@ -18459,7 +18459,7 @@
         <v>1139</v>
       </c>
       <c r="I385">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J385" t="s">
         <v>1142</v>
@@ -18497,7 +18497,7 @@
         <v>1139</v>
       </c>
       <c r="I386">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J386" t="s">
         <v>1146</v>
@@ -18535,7 +18535,7 @@
         <v>1139</v>
       </c>
       <c r="I387">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J387" t="s">
         <v>1146</v>
@@ -18573,7 +18573,7 @@
         <v>1139</v>
       </c>
       <c r="I388">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J388" t="s">
         <v>1146</v>
@@ -18611,7 +18611,7 @@
         <v>1139</v>
       </c>
       <c r="I389">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J389" t="s">
         <v>1147</v>
@@ -18649,7 +18649,7 @@
         <v>1139</v>
       </c>
       <c r="I390">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J390" t="s">
         <v>1124</v>
@@ -18766,7 +18766,7 @@
         <v>1139</v>
       </c>
       <c r="I393">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J393" t="s">
         <v>1146</v>
@@ -18804,7 +18804,7 @@
         <v>1139</v>
       </c>
       <c r="I394">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J394" t="s">
         <v>1146</v>
@@ -18842,7 +18842,7 @@
         <v>1139</v>
       </c>
       <c r="I395">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J395" t="s">
         <v>1146</v>
@@ -18880,7 +18880,7 @@
         <v>1139</v>
       </c>
       <c r="I396">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J396" t="s">
         <v>1146</v>
@@ -18918,7 +18918,7 @@
         <v>1139</v>
       </c>
       <c r="I397">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J397" t="s">
         <v>1146</v>
@@ -18956,7 +18956,7 @@
         <v>1139</v>
       </c>
       <c r="I398">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J398" t="s">
         <v>1146</v>
@@ -19032,7 +19032,7 @@
         <v>1139</v>
       </c>
       <c r="I400">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J400" t="s">
         <v>1146</v>
@@ -19070,7 +19070,7 @@
         <v>1139</v>
       </c>
       <c r="I401">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J401" t="s">
         <v>1146</v>
@@ -19108,7 +19108,7 @@
         <v>1139</v>
       </c>
       <c r="I402">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J402" t="s">
         <v>1146</v>
@@ -19146,7 +19146,7 @@
         <v>1139</v>
       </c>
       <c r="I403">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J403" t="s">
         <v>1149</v>
@@ -19181,7 +19181,7 @@
         <v>1139</v>
       </c>
       <c r="I404">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J404" t="s">
         <v>1149</v>
@@ -19245,7 +19245,7 @@
         <v>1139</v>
       </c>
       <c r="I406">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P406" t="b">
         <v>1</v>
@@ -19277,7 +19277,7 @@
         <v>1139</v>
       </c>
       <c r="I407">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P407" t="b">
         <v>1</v>
@@ -19309,7 +19309,7 @@
         <v>1139</v>
       </c>
       <c r="I408">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P408" t="b">
         <v>1</v>
@@ -19341,7 +19341,7 @@
         <v>1139</v>
       </c>
       <c r="I409">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P409" t="b">
         <v>1</v>
@@ -19373,7 +19373,7 @@
         <v>1139</v>
       </c>
       <c r="I410">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P410" t="b">
         <v>1</v>
@@ -19405,7 +19405,7 @@
         <v>1139</v>
       </c>
       <c r="I411">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P411" t="b">
         <v>1</v>
@@ -19437,7 +19437,7 @@
         <v>1139</v>
       </c>
       <c r="I412">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P412" t="b">
         <v>1</v>
@@ -19469,7 +19469,7 @@
         <v>1139</v>
       </c>
       <c r="I413">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P413" t="b">
         <v>1</v>
@@ -19501,7 +19501,7 @@
         <v>1139</v>
       </c>
       <c r="I414">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P414" t="b">
         <v>1</v>
@@ -19533,7 +19533,7 @@
         <v>1139</v>
       </c>
       <c r="I415">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P415" t="b">
         <v>1</v>
@@ -19565,7 +19565,7 @@
         <v>1139</v>
       </c>
       <c r="I416">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P416" t="b">
         <v>1</v>
@@ -19597,7 +19597,7 @@
         <v>1139</v>
       </c>
       <c r="I417">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P417" t="b">
         <v>1</v>
@@ -19629,7 +19629,7 @@
         <v>1139</v>
       </c>
       <c r="I418">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P418" t="b">
         <v>1</v>
@@ -19661,7 +19661,7 @@
         <v>1139</v>
       </c>
       <c r="I419">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P419" t="b">
         <v>1</v>
@@ -19693,7 +19693,7 @@
         <v>1139</v>
       </c>
       <c r="I420">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P420" t="b">
         <v>1</v>
@@ -19725,7 +19725,7 @@
         <v>1139</v>
       </c>
       <c r="I421">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P421" t="b">
         <v>1</v>
@@ -19757,7 +19757,7 @@
         <v>1139</v>
       </c>
       <c r="I422">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P422" t="b">
         <v>1</v>
@@ -19789,7 +19789,7 @@
         <v>1139</v>
       </c>
       <c r="I423">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P423" t="b">
         <v>1</v>
@@ -19821,7 +19821,7 @@
         <v>1139</v>
       </c>
       <c r="I424">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P424" t="b">
         <v>1</v>
@@ -19853,7 +19853,7 @@
         <v>1139</v>
       </c>
       <c r="I425">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P425" t="b">
         <v>1</v>
@@ -19885,7 +19885,7 @@
         <v>1139</v>
       </c>
       <c r="I426">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P426" t="b">
         <v>1</v>
@@ -19917,7 +19917,7 @@
         <v>1139</v>
       </c>
       <c r="I427">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P427" t="b">
         <v>1</v>
@@ -19949,7 +19949,7 @@
         <v>1139</v>
       </c>
       <c r="I428">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P428" t="b">
         <v>1</v>
@@ -19981,7 +19981,7 @@
         <v>1139</v>
       </c>
       <c r="I429">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P429" t="b">
         <v>1</v>
@@ -20013,7 +20013,7 @@
         <v>1139</v>
       </c>
       <c r="I430">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P430" t="b">
         <v>1</v>
@@ -20045,7 +20045,7 @@
         <v>1139</v>
       </c>
       <c r="I431">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P431" t="b">
         <v>1</v>
@@ -20077,7 +20077,7 @@
         <v>1139</v>
       </c>
       <c r="I432">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P432" t="b">
         <v>1</v>
@@ -20109,7 +20109,7 @@
         <v>1139</v>
       </c>
       <c r="I433">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P433" t="b">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>1139</v>
       </c>
       <c r="I434">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P434" t="b">
         <v>1</v>
@@ -20173,7 +20173,7 @@
         <v>1139</v>
       </c>
       <c r="I435">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P435" t="b">
         <v>1</v>
@@ -20205,7 +20205,7 @@
         <v>1139</v>
       </c>
       <c r="I436">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P436" t="b">
         <v>1</v>
@@ -20237,7 +20237,7 @@
         <v>1141</v>
       </c>
       <c r="I437">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P437" t="b">
         <v>1</v>
@@ -20269,7 +20269,7 @@
         <v>1141</v>
       </c>
       <c r="I438">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P438" t="b">
         <v>1</v>
@@ -20301,7 +20301,7 @@
         <v>1139</v>
       </c>
       <c r="I439">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P439" t="b">
         <v>1</v>
@@ -20333,7 +20333,7 @@
         <v>1139</v>
       </c>
       <c r="I440">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P440" t="b">
         <v>1</v>
@@ -20365,7 +20365,7 @@
         <v>1139</v>
       </c>
       <c r="I441">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P441" t="b">
         <v>1</v>
@@ -20397,7 +20397,7 @@
         <v>1139</v>
       </c>
       <c r="I442">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P442" t="b">
         <v>1</v>
@@ -20429,7 +20429,7 @@
         <v>1139</v>
       </c>
       <c r="I443">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P443" t="b">
         <v>1</v>
@@ -20461,7 +20461,7 @@
         <v>1139</v>
       </c>
       <c r="I444">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P444" t="b">
         <v>1</v>
@@ -20493,7 +20493,7 @@
         <v>1139</v>
       </c>
       <c r="I445">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P445" t="b">
         <v>1</v>
@@ -20525,7 +20525,7 @@
         <v>1139</v>
       </c>
       <c r="I446">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P446" t="b">
         <v>1</v>
@@ -20557,7 +20557,7 @@
         <v>1139</v>
       </c>
       <c r="I447">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (27/07/2026 14:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -3845,16 +3845,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3870,7 +3862,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -3878,30 +3870,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4201,55 +4175,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -4269,7 +4243,7 @@
       <c r="E2" t="s">
         <v>738</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>45698</v>
       </c>
       <c r="G2" t="s">
@@ -4307,7 +4281,7 @@
       <c r="E3" t="s">
         <v>739</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>45714</v>
       </c>
       <c r="G3" t="s">
@@ -4345,7 +4319,7 @@
       <c r="E4" t="s">
         <v>740</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>45714</v>
       </c>
       <c r="G4" t="s">
@@ -4383,7 +4357,7 @@
       <c r="E5" t="s">
         <v>741</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>45714</v>
       </c>
       <c r="G5" t="s">
@@ -4404,7 +4378,7 @@
       <c r="L5" t="s">
         <v>1152</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>45993</v>
       </c>
       <c r="Q5" t="b">
@@ -4427,7 +4401,7 @@
       <c r="E6" t="s">
         <v>742</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>45736</v>
       </c>
       <c r="G6" t="s">
@@ -4448,7 +4422,7 @@
       <c r="L6" t="s">
         <v>1153</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>45889</v>
       </c>
       <c r="Q6" t="b">
@@ -4471,7 +4445,7 @@
       <c r="E7" t="s">
         <v>743</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>45736</v>
       </c>
       <c r="G7" t="s">
@@ -4492,7 +4466,7 @@
       <c r="L7" t="s">
         <v>1154</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>45848</v>
       </c>
       <c r="O7" t="s">
@@ -4518,7 +4492,7 @@
       <c r="E8" t="s">
         <v>744</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>45736</v>
       </c>
       <c r="G8" t="s">
@@ -4547,7 +4521,7 @@
       <c r="E9" t="s">
         <v>745</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>45736</v>
       </c>
       <c r="G9" t="s">
@@ -4568,7 +4542,7 @@
       <c r="L9" t="s">
         <v>1155</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46098</v>
       </c>
       <c r="O9">
@@ -4594,7 +4568,7 @@
       <c r="E10" t="s">
         <v>746</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>45736</v>
       </c>
       <c r="G10" t="s">
@@ -4615,7 +4589,7 @@
       <c r="L10" t="s">
         <v>1156</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46114</v>
       </c>
       <c r="O10" t="s">
@@ -4641,7 +4615,7 @@
       <c r="E11" t="s">
         <v>747</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>45736</v>
       </c>
       <c r="G11" t="s">
@@ -4662,7 +4636,7 @@
       <c r="L11" t="s">
         <v>1154</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>45848</v>
       </c>
       <c r="O11" t="s">
@@ -4688,7 +4662,7 @@
       <c r="E12" t="s">
         <v>748</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="1">
         <v>45736</v>
       </c>
       <c r="G12" t="s">
@@ -4709,7 +4683,7 @@
       <c r="L12" t="s">
         <v>1157</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>45860</v>
       </c>
       <c r="Q12" t="b">
@@ -4732,7 +4706,7 @@
       <c r="E13" t="s">
         <v>749</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="1">
         <v>45736</v>
       </c>
       <c r="G13" t="s">
@@ -4767,7 +4741,7 @@
       <c r="E14" t="s">
         <v>750</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="1">
         <v>45736</v>
       </c>
       <c r="G14" t="s">
@@ -4788,7 +4762,7 @@
       <c r="L14" t="s">
         <v>1158</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>45800</v>
       </c>
       <c r="Q14" t="b">
@@ -4811,7 +4785,7 @@
       <c r="E15" t="s">
         <v>751</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="1">
         <v>45736</v>
       </c>
       <c r="G15" t="s">
@@ -4849,7 +4823,7 @@
       <c r="E16" t="s">
         <v>752</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>45736</v>
       </c>
       <c r="G16" t="s">
@@ -4887,7 +4861,7 @@
       <c r="E17" t="s">
         <v>753</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>45736</v>
       </c>
       <c r="G17" t="s">
@@ -4908,7 +4882,7 @@
       <c r="L17" t="s">
         <v>1153</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>45897</v>
       </c>
       <c r="Q17" t="b">
@@ -4931,7 +4905,7 @@
       <c r="E18" t="s">
         <v>754</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="1">
         <v>45736</v>
       </c>
       <c r="G18" t="s">
@@ -4952,7 +4926,7 @@
       <c r="L18" t="s">
         <v>1158</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>45802</v>
       </c>
       <c r="Q18" t="b">
@@ -4975,7 +4949,7 @@
       <c r="E19" t="s">
         <v>755</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="1">
         <v>45736</v>
       </c>
       <c r="G19" t="s">
@@ -5010,7 +4984,7 @@
       <c r="E20" t="s">
         <v>756</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="1">
         <v>45736</v>
       </c>
       <c r="G20" t="s">
@@ -5031,7 +5005,7 @@
       <c r="L20" t="s">
         <v>1160</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46135</v>
       </c>
       <c r="Q20" t="b">
@@ -5054,7 +5028,7 @@
       <c r="E21" t="s">
         <v>757</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="1">
         <v>45736</v>
       </c>
       <c r="G21" t="s">
@@ -5089,7 +5063,7 @@
       <c r="E22" t="s">
         <v>758</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="1">
         <v>45736</v>
       </c>
       <c r="G22" t="s">
@@ -5127,7 +5101,7 @@
       <c r="E23" t="s">
         <v>759</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="1">
         <v>45736</v>
       </c>
       <c r="G23" t="s">
@@ -5148,7 +5122,7 @@
       <c r="L23" t="s">
         <v>1162</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23" s="1">
         <v>45965</v>
       </c>
       <c r="P23" t="s">
@@ -5174,7 +5148,7 @@
       <c r="E24" t="s">
         <v>760</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="1">
         <v>45736</v>
       </c>
       <c r="G24" t="s">
@@ -5212,7 +5186,7 @@
       <c r="E25" t="s">
         <v>761</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="1">
         <v>45736</v>
       </c>
       <c r="G25" t="s">
@@ -5250,7 +5224,7 @@
       <c r="E26" t="s">
         <v>762</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="1">
         <v>45736</v>
       </c>
       <c r="G26" t="s">
@@ -5271,7 +5245,7 @@
       <c r="L26" t="s">
         <v>1165</v>
       </c>
-      <c r="N26" s="2">
+      <c r="N26" s="1">
         <v>45891</v>
       </c>
       <c r="P26" t="s">
@@ -5297,7 +5271,7 @@
       <c r="E27" t="s">
         <v>763</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>45736</v>
       </c>
       <c r="G27" t="s">
@@ -5335,7 +5309,7 @@
       <c r="E28" t="s">
         <v>764</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="1">
         <v>45736</v>
       </c>
       <c r="G28" t="s">
@@ -5364,7 +5338,7 @@
       <c r="E29" t="s">
         <v>765</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="1">
         <v>45736</v>
       </c>
       <c r="G29" t="s">
@@ -5402,7 +5376,7 @@
       <c r="E30" t="s">
         <v>766</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="1">
         <v>45736</v>
       </c>
       <c r="G30" t="s">
@@ -5423,7 +5397,7 @@
       <c r="L30" t="s">
         <v>1166</v>
       </c>
-      <c r="N30" s="2">
+      <c r="N30" s="1">
         <v>45945</v>
       </c>
       <c r="Q30" t="b">
@@ -5446,7 +5420,7 @@
       <c r="E31" t="s">
         <v>767</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="1">
         <v>45736</v>
       </c>
       <c r="G31" t="s">
@@ -5484,7 +5458,7 @@
       <c r="E32" t="s">
         <v>768</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="1">
         <v>45736</v>
       </c>
       <c r="G32" t="s">
@@ -5522,7 +5496,7 @@
       <c r="E33" t="s">
         <v>769</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="1">
         <v>45736</v>
       </c>
       <c r="G33" t="s">
@@ -5557,7 +5531,7 @@
       <c r="E34" t="s">
         <v>770</v>
       </c>
-      <c r="F34" s="2">
+      <c r="F34" s="1">
         <v>45736</v>
       </c>
       <c r="G34" t="s">
@@ -5586,7 +5560,7 @@
       <c r="E35" t="s">
         <v>771</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="1">
         <v>45736</v>
       </c>
       <c r="G35" t="s">
@@ -5615,7 +5589,7 @@
       <c r="E36" t="s">
         <v>772</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="1">
         <v>45736</v>
       </c>
       <c r="G36" t="s">
@@ -5653,7 +5627,7 @@
       <c r="E37" t="s">
         <v>773</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="1">
         <v>45736</v>
       </c>
       <c r="G37" t="s">
@@ -5691,7 +5665,7 @@
       <c r="E38" t="s">
         <v>753</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="1">
         <v>45736</v>
       </c>
       <c r="G38" t="s">
@@ -5726,7 +5700,7 @@
       <c r="D39" t="s">
         <v>645</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="1">
         <v>45736</v>
       </c>
       <c r="G39" t="s">
@@ -5761,7 +5735,7 @@
       <c r="D40" t="s">
         <v>645</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="1">
         <v>45736</v>
       </c>
       <c r="G40" t="s">
@@ -5799,7 +5773,7 @@
       <c r="E41" t="s">
         <v>774</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="1">
         <v>45736</v>
       </c>
       <c r="G41" t="s">
@@ -5837,7 +5811,7 @@
       <c r="E42" t="s">
         <v>775</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="1">
         <v>45736</v>
       </c>
       <c r="G42" t="s">
@@ -5875,7 +5849,7 @@
       <c r="E43" t="s">
         <v>776</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>45736</v>
       </c>
       <c r="G43" t="s">
@@ -5910,7 +5884,7 @@
       <c r="E44" t="s">
         <v>777</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="1">
         <v>45769</v>
       </c>
       <c r="G44" t="s">
@@ -5931,7 +5905,7 @@
       <c r="L44" t="s">
         <v>1169</v>
       </c>
-      <c r="N44" s="2">
+      <c r="N44" s="1">
         <v>45856</v>
       </c>
       <c r="P44" t="s">
@@ -5957,7 +5931,7 @@
       <c r="E45" t="s">
         <v>778</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="1">
         <v>45769</v>
       </c>
       <c r="G45" t="s">
@@ -5978,7 +5952,7 @@
       <c r="L45" t="s">
         <v>1170</v>
       </c>
-      <c r="N45" s="2">
+      <c r="N45" s="1">
         <v>46100</v>
       </c>
       <c r="O45">
@@ -6004,7 +5978,7 @@
       <c r="E46" t="s">
         <v>779</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="1">
         <v>45769</v>
       </c>
       <c r="G46" t="s">
@@ -6042,7 +6016,7 @@
       <c r="E47" t="s">
         <v>780</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="1">
         <v>45769</v>
       </c>
       <c r="G47" t="s">
@@ -6063,7 +6037,7 @@
       <c r="L47" t="s">
         <v>1171</v>
       </c>
-      <c r="N47" s="2">
+      <c r="N47" s="1">
         <v>46113</v>
       </c>
       <c r="P47" t="s">
@@ -6089,7 +6063,7 @@
       <c r="E48" t="s">
         <v>781</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="1">
         <v>45769</v>
       </c>
       <c r="G48" t="s">
@@ -6127,7 +6101,7 @@
       <c r="E49" t="s">
         <v>782</v>
       </c>
-      <c r="F49" s="2">
+      <c r="F49" s="1">
         <v>45769</v>
       </c>
       <c r="G49" t="s">
@@ -6159,7 +6133,7 @@
       <c r="E50" t="s">
         <v>783</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="1">
         <v>45769</v>
       </c>
       <c r="G50" t="s">
@@ -6197,7 +6171,7 @@
       <c r="E51" t="s">
         <v>784</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="1">
         <v>45769</v>
       </c>
       <c r="G51" t="s">
@@ -6235,7 +6209,7 @@
       <c r="E52" t="s">
         <v>785</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="1">
         <v>45769</v>
       </c>
       <c r="G52" t="s">
@@ -6273,7 +6247,7 @@
       <c r="E53" t="s">
         <v>786</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="1">
         <v>45769</v>
       </c>
       <c r="G53" t="s">
@@ -6311,7 +6285,7 @@
       <c r="E54" t="s">
         <v>787</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="1">
         <v>45769</v>
       </c>
       <c r="G54" t="s">
@@ -6349,7 +6323,7 @@
       <c r="E55" t="s">
         <v>788</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="1">
         <v>45769</v>
       </c>
       <c r="G55" t="s">
@@ -6381,7 +6355,7 @@
       <c r="E56" t="s">
         <v>789</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="1">
         <v>45769</v>
       </c>
       <c r="G56" t="s">
@@ -6419,7 +6393,7 @@
       <c r="E57" t="s">
         <v>790</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="1">
         <v>45769</v>
       </c>
       <c r="G57" t="s">
@@ -6457,7 +6431,7 @@
       <c r="E58" t="s">
         <v>791</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="1">
         <v>45769</v>
       </c>
       <c r="G58" t="s">
@@ -6489,7 +6463,7 @@
       <c r="E59" t="s">
         <v>792</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="1">
         <v>45769</v>
       </c>
       <c r="G59" t="s">
@@ -6524,7 +6498,7 @@
       <c r="E60" t="s">
         <v>793</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <v>45769</v>
       </c>
       <c r="G60" t="s">
@@ -6559,7 +6533,7 @@
       <c r="E61" t="s">
         <v>794</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="1">
         <v>45769</v>
       </c>
       <c r="G61" t="s">
@@ -6591,7 +6565,7 @@
       <c r="E62" t="s">
         <v>795</v>
       </c>
-      <c r="F62" s="2">
+      <c r="F62" s="1">
         <v>45770</v>
       </c>
       <c r="G62" t="s">
@@ -6623,7 +6597,7 @@
       <c r="E63" t="s">
         <v>796</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="1">
         <v>45799</v>
       </c>
       <c r="G63" t="s">
@@ -6644,7 +6618,7 @@
       <c r="L63" t="s">
         <v>1174</v>
       </c>
-      <c r="N63" s="2">
+      <c r="N63" s="1">
         <v>46092</v>
       </c>
       <c r="P63" t="s">
@@ -6670,7 +6644,7 @@
       <c r="E64" t="s">
         <v>797</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="1">
         <v>45799</v>
       </c>
       <c r="G64" t="s">
@@ -6691,7 +6665,7 @@
       <c r="L64" t="s">
         <v>1175</v>
       </c>
-      <c r="N64" s="2">
+      <c r="N64" s="1">
         <v>46119</v>
       </c>
       <c r="Q64" t="b">
@@ -6714,7 +6688,7 @@
       <c r="E65" t="s">
         <v>798</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="1">
         <v>45799</v>
       </c>
       <c r="G65" t="s">
@@ -6752,7 +6726,7 @@
       <c r="E66" t="s">
         <v>799</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="1">
         <v>45799</v>
       </c>
       <c r="G66" t="s">
@@ -6790,7 +6764,7 @@
       <c r="E67" t="s">
         <v>800</v>
       </c>
-      <c r="F67" s="2">
+      <c r="F67" s="1">
         <v>45799</v>
       </c>
       <c r="G67" t="s">
@@ -6825,7 +6799,7 @@
       <c r="E68" t="s">
         <v>801</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="1">
         <v>45799</v>
       </c>
       <c r="G68" t="s">
@@ -6863,7 +6837,7 @@
       <c r="E69" t="s">
         <v>802</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>45803</v>
       </c>
       <c r="G69" t="s">
@@ -6901,7 +6875,7 @@
       <c r="E70" t="s">
         <v>803</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="1">
         <v>45803</v>
       </c>
       <c r="G70" t="s">
@@ -6939,7 +6913,7 @@
       <c r="E71" t="s">
         <v>804</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="1">
         <v>45803</v>
       </c>
       <c r="G71" t="s">
@@ -6974,7 +6948,7 @@
       <c r="E72" t="s">
         <v>805</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>45803</v>
       </c>
       <c r="G72" t="s">
@@ -7009,7 +6983,7 @@
       <c r="E73" t="s">
         <v>806</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="1">
         <v>45803</v>
       </c>
       <c r="G73" t="s">
@@ -7047,7 +7021,7 @@
       <c r="E74" t="s">
         <v>805</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="1">
         <v>45803</v>
       </c>
       <c r="G74" t="s">
@@ -7085,7 +7059,7 @@
       <c r="E75" t="s">
         <v>807</v>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="1">
         <v>45803</v>
       </c>
       <c r="G75" t="s">
@@ -7123,7 +7097,7 @@
       <c r="E76" t="s">
         <v>808</v>
       </c>
-      <c r="F76" s="2">
+      <c r="F76" s="1">
         <v>45803</v>
       </c>
       <c r="G76" t="s">
@@ -7158,7 +7132,7 @@
       <c r="E77" t="s">
         <v>809</v>
       </c>
-      <c r="F77" s="2">
+      <c r="F77" s="1">
         <v>45803</v>
       </c>
       <c r="G77" t="s">
@@ -7193,7 +7167,7 @@
       <c r="E78" t="s">
         <v>810</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="1">
         <v>45803</v>
       </c>
       <c r="G78" t="s">
@@ -7231,7 +7205,7 @@
       <c r="E79" t="s">
         <v>811</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="1">
         <v>45803</v>
       </c>
       <c r="G79" t="s">
@@ -7266,7 +7240,7 @@
       <c r="E80" t="s">
         <v>812</v>
       </c>
-      <c r="F80" s="2">
+      <c r="F80" s="1">
         <v>45803</v>
       </c>
       <c r="G80" t="s">
@@ -7304,7 +7278,7 @@
       <c r="E81" t="s">
         <v>813</v>
       </c>
-      <c r="F81" s="2">
+      <c r="F81" s="1">
         <v>45813</v>
       </c>
       <c r="G81" t="s">
@@ -7342,7 +7316,7 @@
       <c r="E82" t="s">
         <v>814</v>
       </c>
-      <c r="F82" s="2">
+      <c r="F82" s="1">
         <v>45813</v>
       </c>
       <c r="G82" t="s">
@@ -7380,7 +7354,7 @@
       <c r="E83" t="s">
         <v>815</v>
       </c>
-      <c r="F83" s="2">
+      <c r="F83" s="1">
         <v>45813</v>
       </c>
       <c r="G83" t="s">
@@ -7415,7 +7389,7 @@
       <c r="E84" t="s">
         <v>816</v>
       </c>
-      <c r="F84" s="2">
+      <c r="F84" s="1">
         <v>45813</v>
       </c>
       <c r="G84" t="s">
@@ -7436,7 +7410,7 @@
       <c r="L84" t="s">
         <v>1179</v>
       </c>
-      <c r="N84" s="2">
+      <c r="N84" s="1">
         <v>45853</v>
       </c>
       <c r="O84">
@@ -7462,7 +7436,7 @@
       <c r="E85" t="s">
         <v>817</v>
       </c>
-      <c r="F85" s="2">
+      <c r="F85" s="1">
         <v>45813</v>
       </c>
       <c r="G85" t="s">
@@ -7500,7 +7474,7 @@
       <c r="E86" t="s">
         <v>818</v>
       </c>
-      <c r="F86" s="2">
+      <c r="F86" s="1">
         <v>45813</v>
       </c>
       <c r="G86" t="s">
@@ -7538,7 +7512,7 @@
       <c r="E87" t="s">
         <v>819</v>
       </c>
-      <c r="F87" s="2">
+      <c r="F87" s="1">
         <v>45813</v>
       </c>
       <c r="G87" t="s">
@@ -7559,7 +7533,7 @@
       <c r="L87" t="s">
         <v>1180</v>
       </c>
-      <c r="N87" s="2">
+      <c r="N87" s="1">
         <v>45797</v>
       </c>
       <c r="O87" t="s">
@@ -7585,7 +7559,7 @@
       <c r="E88" t="s">
         <v>820</v>
       </c>
-      <c r="F88" s="2">
+      <c r="F88" s="1">
         <v>45813</v>
       </c>
       <c r="G88" t="s">
@@ -7620,7 +7594,7 @@
       <c r="E89" t="s">
         <v>821</v>
       </c>
-      <c r="F89" s="2">
+      <c r="F89" s="1">
         <v>45813</v>
       </c>
       <c r="G89" t="s">
@@ -7655,7 +7629,7 @@
       <c r="E90" t="s">
         <v>822</v>
       </c>
-      <c r="F90" s="2">
+      <c r="F90" s="1">
         <v>45831</v>
       </c>
       <c r="G90" t="s">
@@ -7696,7 +7670,7 @@
       <c r="E91" t="s">
         <v>823</v>
       </c>
-      <c r="F91" s="2">
+      <c r="F91" s="1">
         <v>45831</v>
       </c>
       <c r="G91" t="s">
@@ -7731,7 +7705,7 @@
       <c r="D92" t="s">
         <v>662</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="1">
         <v>45831</v>
       </c>
       <c r="G92" t="s">
@@ -7763,7 +7737,7 @@
       <c r="E93" t="s">
         <v>824</v>
       </c>
-      <c r="F93" s="2">
+      <c r="F93" s="1">
         <v>45831</v>
       </c>
       <c r="G93" t="s">
@@ -7801,7 +7775,7 @@
       <c r="E94" t="s">
         <v>825</v>
       </c>
-      <c r="F94" s="2">
+      <c r="F94" s="1">
         <v>45831</v>
       </c>
       <c r="G94" t="s">
@@ -7839,7 +7813,7 @@
       <c r="E95" t="s">
         <v>826</v>
       </c>
-      <c r="F95" s="2">
+      <c r="F95" s="1">
         <v>45831</v>
       </c>
       <c r="G95" t="s">
@@ -7877,7 +7851,7 @@
       <c r="E96" t="s">
         <v>827</v>
       </c>
-      <c r="F96" s="2">
+      <c r="F96" s="1">
         <v>45831</v>
       </c>
       <c r="G96" t="s">
@@ -7898,7 +7872,7 @@
       <c r="L96" t="s">
         <v>1154</v>
       </c>
-      <c r="N96" s="2">
+      <c r="N96" s="1">
         <v>45848</v>
       </c>
       <c r="O96" t="s">
@@ -7924,7 +7898,7 @@
       <c r="E97" t="s">
         <v>828</v>
       </c>
-      <c r="F97" s="2">
+      <c r="F97" s="1">
         <v>45840</v>
       </c>
       <c r="G97" t="s">
@@ -7965,7 +7939,7 @@
       <c r="E98" t="s">
         <v>829</v>
       </c>
-      <c r="F98" s="2">
+      <c r="F98" s="1">
         <v>45840</v>
       </c>
       <c r="G98" t="s">
@@ -8003,7 +7977,7 @@
       <c r="E99" t="s">
         <v>830</v>
       </c>
-      <c r="F99" s="2">
+      <c r="F99" s="1">
         <v>45840</v>
       </c>
       <c r="G99" t="s">
@@ -8032,7 +8006,7 @@
       <c r="E100" t="s">
         <v>831</v>
       </c>
-      <c r="F100" s="2">
+      <c r="F100" s="1">
         <v>45840</v>
       </c>
       <c r="G100" t="s">
@@ -8070,7 +8044,7 @@
       <c r="E101" t="s">
         <v>832</v>
       </c>
-      <c r="F101" s="2">
+      <c r="F101" s="1">
         <v>45840</v>
       </c>
       <c r="G101" t="s">
@@ -8102,7 +8076,7 @@
       <c r="E102" t="s">
         <v>833</v>
       </c>
-      <c r="F102" s="2">
+      <c r="F102" s="1">
         <v>45840</v>
       </c>
       <c r="G102" t="s">
@@ -8131,7 +8105,7 @@
       <c r="E103" t="s">
         <v>834</v>
       </c>
-      <c r="F103" s="2">
+      <c r="F103" s="1">
         <v>45840</v>
       </c>
       <c r="G103" t="s">
@@ -8160,7 +8134,7 @@
       <c r="E104" t="s">
         <v>835</v>
       </c>
-      <c r="F104" s="2">
+      <c r="F104" s="1">
         <v>45840</v>
       </c>
       <c r="G104" t="s">
@@ -8198,7 +8172,7 @@
       <c r="E105" t="s">
         <v>836</v>
       </c>
-      <c r="F105" s="2">
+      <c r="F105" s="1">
         <v>45840</v>
       </c>
       <c r="G105" t="s">
@@ -8236,7 +8210,7 @@
       <c r="E106" t="s">
         <v>837</v>
       </c>
-      <c r="F106" s="2">
+      <c r="F106" s="1">
         <v>45840</v>
       </c>
       <c r="G106" t="s">
@@ -8257,7 +8231,7 @@
       <c r="L106" t="s">
         <v>1183</v>
       </c>
-      <c r="N106" s="2">
+      <c r="N106" s="1">
         <v>45889</v>
       </c>
       <c r="Q106" t="b">
@@ -8280,7 +8254,7 @@
       <c r="E107" t="s">
         <v>838</v>
       </c>
-      <c r="F107" s="2">
+      <c r="F107" s="1">
         <v>45840</v>
       </c>
       <c r="G107" t="s">
@@ -8301,7 +8275,7 @@
       <c r="L107" t="s">
         <v>1184</v>
       </c>
-      <c r="N107" s="2">
+      <c r="N107" s="1">
         <v>45876</v>
       </c>
       <c r="Q107" t="b">
@@ -8324,7 +8298,7 @@
       <c r="E108" t="s">
         <v>839</v>
       </c>
-      <c r="F108" s="2">
+      <c r="F108" s="1">
         <v>45840</v>
       </c>
       <c r="G108" t="s">
@@ -8362,7 +8336,7 @@
       <c r="E109" t="s">
         <v>840</v>
       </c>
-      <c r="F109" s="2">
+      <c r="F109" s="1">
         <v>45840</v>
       </c>
       <c r="G109" t="s">
@@ -8400,7 +8374,7 @@
       <c r="E110" t="s">
         <v>841</v>
       </c>
-      <c r="F110" s="2">
+      <c r="F110" s="1">
         <v>45840</v>
       </c>
       <c r="G110" t="s">
@@ -8435,7 +8409,7 @@
       <c r="E111" t="s">
         <v>842</v>
       </c>
-      <c r="F111" s="2">
+      <c r="F111" s="1">
         <v>45840</v>
       </c>
       <c r="G111" t="s">
@@ -8473,7 +8447,7 @@
       <c r="E112" t="s">
         <v>843</v>
       </c>
-      <c r="F112" s="2">
+      <c r="F112" s="1">
         <v>45840</v>
       </c>
       <c r="G112" t="s">
@@ -8505,7 +8479,7 @@
       <c r="E113" t="s">
         <v>844</v>
       </c>
-      <c r="F113" s="2">
+      <c r="F113" s="1">
         <v>45840</v>
       </c>
       <c r="G113" t="s">
@@ -8543,7 +8517,7 @@
       <c r="E114" t="s">
         <v>845</v>
       </c>
-      <c r="F114" s="2">
+      <c r="F114" s="1">
         <v>45840</v>
       </c>
       <c r="G114" t="s">
@@ -8578,7 +8552,7 @@
       <c r="E115" t="s">
         <v>846</v>
       </c>
-      <c r="F115" s="2">
+      <c r="F115" s="1">
         <v>45840</v>
       </c>
       <c r="G115" t="s">
@@ -8616,7 +8590,7 @@
       <c r="E116" t="s">
         <v>847</v>
       </c>
-      <c r="F116" s="2">
+      <c r="F116" s="1">
         <v>45840</v>
       </c>
       <c r="G116" t="s">
@@ -8654,7 +8628,7 @@
       <c r="E117" t="s">
         <v>848</v>
       </c>
-      <c r="F117" s="2">
+      <c r="F117" s="1">
         <v>45840</v>
       </c>
       <c r="G117" t="s">
@@ -8692,7 +8666,7 @@
       <c r="E118" t="s">
         <v>849</v>
       </c>
-      <c r="F118" s="2">
+      <c r="F118" s="1">
         <v>45840</v>
       </c>
       <c r="G118" t="s">
@@ -8730,7 +8704,7 @@
       <c r="E119" t="s">
         <v>850</v>
       </c>
-      <c r="F119" s="2">
+      <c r="F119" s="1">
         <v>45840</v>
       </c>
       <c r="G119" t="s">
@@ -8768,7 +8742,7 @@
       <c r="E120" t="s">
         <v>851</v>
       </c>
-      <c r="F120" s="2">
+      <c r="F120" s="1">
         <v>45840</v>
       </c>
       <c r="G120" t="s">
@@ -8806,7 +8780,7 @@
       <c r="E121" t="s">
         <v>852</v>
       </c>
-      <c r="F121" s="2">
+      <c r="F121" s="1">
         <v>45849</v>
       </c>
       <c r="G121" t="s">
@@ -8827,7 +8801,7 @@
       <c r="L121" t="s">
         <v>1170</v>
       </c>
-      <c r="N121" s="2">
+      <c r="N121" s="1">
         <v>46100</v>
       </c>
       <c r="O121">
@@ -8853,7 +8827,7 @@
       <c r="E122" t="s">
         <v>853</v>
       </c>
-      <c r="F122" s="2">
+      <c r="F122" s="1">
         <v>45849</v>
       </c>
       <c r="G122" t="s">
@@ -8891,7 +8865,7 @@
       <c r="E123" t="s">
         <v>854</v>
       </c>
-      <c r="F123" s="2">
+      <c r="F123" s="1">
         <v>45849</v>
       </c>
       <c r="G123" t="s">
@@ -8920,7 +8894,7 @@
       <c r="E124" t="s">
         <v>855</v>
       </c>
-      <c r="F124" s="2">
+      <c r="F124" s="1">
         <v>45853</v>
       </c>
       <c r="G124" t="s">
@@ -8958,7 +8932,7 @@
       <c r="E125" t="s">
         <v>856</v>
       </c>
-      <c r="F125" s="2">
+      <c r="F125" s="1">
         <v>45855</v>
       </c>
       <c r="G125" t="s">
@@ -8996,7 +8970,7 @@
       <c r="E126" t="s">
         <v>857</v>
       </c>
-      <c r="F126" s="2">
+      <c r="F126" s="1">
         <v>45855</v>
       </c>
       <c r="G126" t="s">
@@ -9034,7 +9008,7 @@
       <c r="E127" t="s">
         <v>858</v>
       </c>
-      <c r="F127" s="2">
+      <c r="F127" s="1">
         <v>45856</v>
       </c>
       <c r="G127" t="s">
@@ -9063,7 +9037,7 @@
       <c r="E128" t="s">
         <v>859</v>
       </c>
-      <c r="F128" s="2">
+      <c r="F128" s="1">
         <v>45869</v>
       </c>
       <c r="G128" t="s">
@@ -9101,7 +9075,7 @@
       <c r="E129" t="s">
         <v>860</v>
       </c>
-      <c r="F129" s="2">
+      <c r="F129" s="1">
         <v>45869</v>
       </c>
       <c r="G129" t="s">
@@ -9139,7 +9113,7 @@
       <c r="E130" t="s">
         <v>861</v>
       </c>
-      <c r="F130" s="2">
+      <c r="F130" s="1">
         <v>45869</v>
       </c>
       <c r="G130" t="s">
@@ -9160,7 +9134,7 @@
       <c r="L130" t="s">
         <v>1188</v>
       </c>
-      <c r="N130" s="2">
+      <c r="N130" s="1">
         <v>45916</v>
       </c>
       <c r="O130">
@@ -9186,7 +9160,7 @@
       <c r="E131" t="s">
         <v>862</v>
       </c>
-      <c r="F131" s="2">
+      <c r="F131" s="1">
         <v>45869</v>
       </c>
       <c r="G131" t="s">
@@ -9221,7 +9195,7 @@
       <c r="E132" t="s">
         <v>863</v>
       </c>
-      <c r="F132" s="2">
+      <c r="F132" s="1">
         <v>45869</v>
       </c>
       <c r="G132" t="s">
@@ -9242,7 +9216,7 @@
       <c r="L132" t="s">
         <v>1190</v>
       </c>
-      <c r="N132" s="2">
+      <c r="N132" s="1">
         <v>46014</v>
       </c>
       <c r="O132">
@@ -9268,7 +9242,7 @@
       <c r="E133" t="s">
         <v>864</v>
       </c>
-      <c r="F133" s="2">
+      <c r="F133" s="1">
         <v>45869</v>
       </c>
       <c r="G133" t="s">
@@ -9297,7 +9271,7 @@
       <c r="E134" t="s">
         <v>865</v>
       </c>
-      <c r="F134" s="2">
+      <c r="F134" s="1">
         <v>45882</v>
       </c>
       <c r="G134" t="s">
@@ -9335,7 +9309,7 @@
       <c r="E135" t="s">
         <v>866</v>
       </c>
-      <c r="F135" s="2">
+      <c r="F135" s="1">
         <v>45882</v>
       </c>
       <c r="G135" t="s">
@@ -9367,7 +9341,7 @@
       <c r="E136" t="s">
         <v>867</v>
       </c>
-      <c r="F136" s="2">
+      <c r="F136" s="1">
         <v>45891</v>
       </c>
       <c r="G136" t="s">
@@ -9396,7 +9370,7 @@
       <c r="E137" t="s">
         <v>868</v>
       </c>
-      <c r="F137" s="2">
+      <c r="F137" s="1">
         <v>45891</v>
       </c>
       <c r="G137" t="s">
@@ -9428,7 +9402,7 @@
       <c r="E138" t="s">
         <v>869</v>
       </c>
-      <c r="F138" s="2">
+      <c r="F138" s="1">
         <v>45891</v>
       </c>
       <c r="G138" t="s">
@@ -9466,7 +9440,7 @@
       <c r="E139" t="s">
         <v>870</v>
       </c>
-      <c r="F139" s="2">
+      <c r="F139" s="1">
         <v>45891</v>
       </c>
       <c r="G139" t="s">
@@ -9495,7 +9469,7 @@
       <c r="E140" t="s">
         <v>871</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140" s="1">
         <v>45891</v>
       </c>
       <c r="G140" t="s">
@@ -9530,7 +9504,7 @@
       <c r="E141" t="s">
         <v>872</v>
       </c>
-      <c r="F141" s="2">
+      <c r="F141" s="1">
         <v>45891</v>
       </c>
       <c r="G141" t="s">
@@ -9562,7 +9536,7 @@
       <c r="E142" t="s">
         <v>873</v>
       </c>
-      <c r="F142" s="2">
+      <c r="F142" s="1">
         <v>45891</v>
       </c>
       <c r="G142" t="s">
@@ -9594,7 +9568,7 @@
       <c r="E143" t="s">
         <v>874</v>
       </c>
-      <c r="F143" s="2">
+      <c r="F143" s="1">
         <v>45891</v>
       </c>
       <c r="G143" t="s">
@@ -9623,7 +9597,7 @@
       <c r="E144" t="s">
         <v>875</v>
       </c>
-      <c r="F144" s="2">
+      <c r="F144" s="1">
         <v>45891</v>
       </c>
       <c r="G144" t="s">
@@ -9655,7 +9629,7 @@
       <c r="E145" t="s">
         <v>876</v>
       </c>
-      <c r="F145" s="2">
+      <c r="F145" s="1">
         <v>45891</v>
       </c>
       <c r="G145" t="s">
@@ -9693,7 +9667,7 @@
       <c r="E146" t="s">
         <v>877</v>
       </c>
-      <c r="F146" s="2">
+      <c r="F146" s="1">
         <v>45891</v>
       </c>
       <c r="G146" t="s">
@@ -9722,7 +9696,7 @@
       <c r="E147" t="s">
         <v>878</v>
       </c>
-      <c r="F147" s="2">
+      <c r="F147" s="1">
         <v>45891</v>
       </c>
       <c r="G147" t="s">
@@ -9757,7 +9731,7 @@
       <c r="E148" t="s">
         <v>879</v>
       </c>
-      <c r="F148" s="2">
+      <c r="F148" s="1">
         <v>45891</v>
       </c>
       <c r="G148" t="s">
@@ -9795,7 +9769,7 @@
       <c r="E149" t="s">
         <v>880</v>
       </c>
-      <c r="F149" s="2">
+      <c r="F149" s="1">
         <v>45891</v>
       </c>
       <c r="G149" t="s">
@@ -9830,7 +9804,7 @@
       <c r="E150" t="s">
         <v>881</v>
       </c>
-      <c r="F150" s="2">
+      <c r="F150" s="1">
         <v>45891</v>
       </c>
       <c r="G150" t="s">
@@ -9851,7 +9825,7 @@
       <c r="L150" t="s">
         <v>1174</v>
       </c>
-      <c r="N150" s="2">
+      <c r="N150" s="1">
         <v>46092</v>
       </c>
       <c r="P150" t="s">
@@ -9877,7 +9851,7 @@
       <c r="E151" t="s">
         <v>882</v>
       </c>
-      <c r="F151" s="2">
+      <c r="F151" s="1">
         <v>45891</v>
       </c>
       <c r="G151" t="s">
@@ -9915,7 +9889,7 @@
       <c r="E152" t="s">
         <v>872</v>
       </c>
-      <c r="F152" s="2">
+      <c r="F152" s="1">
         <v>45891</v>
       </c>
       <c r="G152" t="s">
@@ -9936,7 +9910,7 @@
       <c r="L152" t="s">
         <v>1175</v>
       </c>
-      <c r="N152" s="2">
+      <c r="N152" s="1">
         <v>46119</v>
       </c>
       <c r="Q152" t="b">
@@ -9959,7 +9933,7 @@
       <c r="E153" t="s">
         <v>883</v>
       </c>
-      <c r="F153" s="2">
+      <c r="F153" s="1">
         <v>45891</v>
       </c>
       <c r="G153" t="s">
@@ -9997,7 +9971,7 @@
       <c r="E154" t="s">
         <v>884</v>
       </c>
-      <c r="F154" s="2">
+      <c r="F154" s="1">
         <v>45891</v>
       </c>
       <c r="G154" t="s">
@@ -10032,7 +10006,7 @@
       <c r="E155" t="s">
         <v>885</v>
       </c>
-      <c r="F155" s="2">
+      <c r="F155" s="1">
         <v>45891</v>
       </c>
       <c r="G155" t="s">
@@ -10067,7 +10041,7 @@
       <c r="E156" t="s">
         <v>886</v>
       </c>
-      <c r="F156" s="2">
+      <c r="F156" s="1">
         <v>45891</v>
       </c>
       <c r="G156" t="s">
@@ -10105,7 +10079,7 @@
       <c r="E157" t="s">
         <v>887</v>
       </c>
-      <c r="F157" s="2">
+      <c r="F157" s="1">
         <v>45891</v>
       </c>
       <c r="G157" t="s">
@@ -10143,7 +10117,7 @@
       <c r="E158" t="s">
         <v>888</v>
       </c>
-      <c r="F158" s="2">
+      <c r="F158" s="1">
         <v>45894</v>
       </c>
       <c r="G158" t="s">
@@ -10164,7 +10138,7 @@
       <c r="L158" t="s">
         <v>1193</v>
       </c>
-      <c r="N158" s="2">
+      <c r="N158" s="1">
         <v>45946</v>
       </c>
       <c r="Q158" t="b">
@@ -10187,7 +10161,7 @@
       <c r="E159" t="s">
         <v>889</v>
       </c>
-      <c r="F159" s="2">
+      <c r="F159" s="1">
         <v>45894</v>
       </c>
       <c r="G159" t="s">
@@ -10225,7 +10199,7 @@
       <c r="E160" t="s">
         <v>890</v>
       </c>
-      <c r="F160" s="2">
+      <c r="F160" s="1">
         <v>45898</v>
       </c>
       <c r="G160" t="s">
@@ -10263,7 +10237,7 @@
       <c r="E161" t="s">
         <v>891</v>
       </c>
-      <c r="F161" s="2">
+      <c r="F161" s="1">
         <v>45898</v>
       </c>
       <c r="G161" t="s">
@@ -10284,7 +10258,7 @@
       <c r="L161" t="s">
         <v>1194</v>
       </c>
-      <c r="N161" s="2">
+      <c r="N161" s="1">
         <v>45953</v>
       </c>
       <c r="O161" t="s">
@@ -10310,7 +10284,7 @@
       <c r="E162" t="s">
         <v>892</v>
       </c>
-      <c r="F162" s="2">
+      <c r="F162" s="1">
         <v>45898</v>
       </c>
       <c r="G162" t="s">
@@ -10331,7 +10305,7 @@
       <c r="L162" t="s">
         <v>1195</v>
       </c>
-      <c r="N162" s="2">
+      <c r="N162" s="1">
         <v>45940</v>
       </c>
       <c r="Q162" t="b">
@@ -10354,7 +10328,7 @@
       <c r="E163" t="s">
         <v>893</v>
       </c>
-      <c r="F163" s="2">
+      <c r="F163" s="1">
         <v>45898</v>
       </c>
       <c r="G163" t="s">
@@ -10375,7 +10349,7 @@
       <c r="L163" t="s">
         <v>1195</v>
       </c>
-      <c r="N163" s="2">
+      <c r="N163" s="1">
         <v>45940</v>
       </c>
       <c r="Q163" t="b">
@@ -10398,7 +10372,7 @@
       <c r="E164" t="s">
         <v>894</v>
       </c>
-      <c r="F164" s="2">
+      <c r="F164" s="1">
         <v>45910</v>
       </c>
       <c r="G164" t="s">
@@ -10433,7 +10407,7 @@
       <c r="E165" t="s">
         <v>895</v>
       </c>
-      <c r="F165" s="2">
+      <c r="F165" s="1">
         <v>45917</v>
       </c>
       <c r="G165" t="s">
@@ -10474,7 +10448,7 @@
       <c r="E166" t="s">
         <v>896</v>
       </c>
-      <c r="F166" s="2">
+      <c r="F166" s="1">
         <v>45917</v>
       </c>
       <c r="G166" t="s">
@@ -10509,7 +10483,7 @@
       <c r="E167" t="s">
         <v>897</v>
       </c>
-      <c r="F167" s="2">
+      <c r="F167" s="1">
         <v>45917</v>
       </c>
       <c r="G167" t="s">
@@ -10541,7 +10515,7 @@
       <c r="E168" t="s">
         <v>898</v>
       </c>
-      <c r="F168" s="2">
+      <c r="F168" s="1">
         <v>45917</v>
       </c>
       <c r="G168" t="s">
@@ -10582,7 +10556,7 @@
       <c r="E169" t="s">
         <v>899</v>
       </c>
-      <c r="F169" s="2">
+      <c r="F169" s="1">
         <v>45917</v>
       </c>
       <c r="G169" t="s">
@@ -10603,7 +10577,7 @@
       <c r="L169" t="s">
         <v>1198</v>
       </c>
-      <c r="N169" s="2">
+      <c r="N169" s="1">
         <v>45973</v>
       </c>
       <c r="Q169" t="b">
@@ -10626,7 +10600,7 @@
       <c r="E170" t="s">
         <v>900</v>
       </c>
-      <c r="F170" s="2">
+      <c r="F170" s="1">
         <v>45917</v>
       </c>
       <c r="G170" t="s">
@@ -10664,7 +10638,7 @@
       <c r="E171" t="s">
         <v>901</v>
       </c>
-      <c r="F171" s="2">
+      <c r="F171" s="1">
         <v>45917</v>
       </c>
       <c r="G171" t="s">
@@ -10702,7 +10676,7 @@
       <c r="E172" t="s">
         <v>902</v>
       </c>
-      <c r="F172" s="2">
+      <c r="F172" s="1">
         <v>45917</v>
       </c>
       <c r="G172" t="s">
@@ -10740,7 +10714,7 @@
       <c r="E173" t="s">
         <v>903</v>
       </c>
-      <c r="F173" s="2">
+      <c r="F173" s="1">
         <v>45917</v>
       </c>
       <c r="G173" t="s">
@@ -10775,7 +10749,7 @@
       <c r="E174" t="s">
         <v>904</v>
       </c>
-      <c r="F174" s="2">
+      <c r="F174" s="1">
         <v>45917</v>
       </c>
       <c r="G174" t="s">
@@ -10810,7 +10784,7 @@
       <c r="E175" t="s">
         <v>905</v>
       </c>
-      <c r="F175" s="2">
+      <c r="F175" s="1">
         <v>45917</v>
       </c>
       <c r="G175" t="s">
@@ -10831,7 +10805,7 @@
       <c r="L175" t="s">
         <v>1199</v>
       </c>
-      <c r="N175" s="2">
+      <c r="N175" s="1">
         <v>46122</v>
       </c>
       <c r="P175" t="s">
@@ -10857,7 +10831,7 @@
       <c r="E176" t="s">
         <v>809</v>
       </c>
-      <c r="F176" s="2">
+      <c r="F176" s="1">
         <v>45917</v>
       </c>
       <c r="G176" t="s">
@@ -10895,7 +10869,7 @@
       <c r="E177" t="s">
         <v>906</v>
       </c>
-      <c r="F177" s="2">
+      <c r="F177" s="1">
         <v>45917</v>
       </c>
       <c r="G177" t="s">
@@ -10916,7 +10890,7 @@
       <c r="L177" t="s">
         <v>1200</v>
       </c>
-      <c r="N177" s="2">
+      <c r="N177" s="1">
         <v>45961</v>
       </c>
       <c r="P177" t="s">
@@ -10942,7 +10916,7 @@
       <c r="E178" t="s">
         <v>907</v>
       </c>
-      <c r="F178" s="2">
+      <c r="F178" s="1">
         <v>45937</v>
       </c>
       <c r="G178" t="s">
@@ -10980,7 +10954,7 @@
       <c r="E179" t="s">
         <v>908</v>
       </c>
-      <c r="F179" s="2">
+      <c r="F179" s="1">
         <v>45937</v>
       </c>
       <c r="G179" t="s">
@@ -11009,7 +10983,7 @@
       <c r="E180" t="s">
         <v>909</v>
       </c>
-      <c r="F180" s="2">
+      <c r="F180" s="1">
         <v>45937</v>
       </c>
       <c r="G180" t="s">
@@ -11047,7 +11021,7 @@
       <c r="E181" t="s">
         <v>910</v>
       </c>
-      <c r="F181" s="2">
+      <c r="F181" s="1">
         <v>45937</v>
       </c>
       <c r="G181" t="s">
@@ -11085,7 +11059,7 @@
       <c r="E182" t="s">
         <v>911</v>
       </c>
-      <c r="F182" s="2">
+      <c r="F182" s="1">
         <v>45937</v>
       </c>
       <c r="G182" t="s">
@@ -11114,7 +11088,7 @@
       <c r="E183" t="s">
         <v>912</v>
       </c>
-      <c r="F183" s="2">
+      <c r="F183" s="1">
         <v>45937</v>
       </c>
       <c r="G183" t="s">
@@ -11149,7 +11123,7 @@
       <c r="D184" t="s">
         <v>688</v>
       </c>
-      <c r="F184" s="2">
+      <c r="F184" s="1">
         <v>45939</v>
       </c>
       <c r="G184" t="s">
@@ -11184,7 +11158,7 @@
       <c r="E185" t="s">
         <v>913</v>
       </c>
-      <c r="F185" s="2">
+      <c r="F185" s="1">
         <v>45939</v>
       </c>
       <c r="G185" t="s">
@@ -11222,7 +11196,7 @@
       <c r="E186" t="s">
         <v>914</v>
       </c>
-      <c r="F186" s="2">
+      <c r="F186" s="1">
         <v>45939</v>
       </c>
       <c r="G186" t="s">
@@ -11260,7 +11234,7 @@
       <c r="E187" t="s">
         <v>915</v>
       </c>
-      <c r="F187" s="2">
+      <c r="F187" s="1">
         <v>45939</v>
       </c>
       <c r="G187" t="s">
@@ -11281,7 +11255,7 @@
       <c r="L187" t="s">
         <v>1202</v>
       </c>
-      <c r="N187" s="2">
+      <c r="N187" s="1">
         <v>46014</v>
       </c>
       <c r="O187">
@@ -11307,7 +11281,7 @@
       <c r="E188" t="s">
         <v>916</v>
       </c>
-      <c r="F188" s="2">
+      <c r="F188" s="1">
         <v>45946</v>
       </c>
       <c r="G188" t="s">
@@ -11328,7 +11302,7 @@
       <c r="L188" t="s">
         <v>1203</v>
       </c>
-      <c r="N188" s="2">
+      <c r="N188" s="1">
         <v>45986</v>
       </c>
       <c r="P188" t="s">
@@ -11354,7 +11328,7 @@
       <c r="E189" t="s">
         <v>917</v>
       </c>
-      <c r="F189" s="2">
+      <c r="F189" s="1">
         <v>45965</v>
       </c>
       <c r="G189" t="s">
@@ -11375,7 +11349,7 @@
       <c r="L189" t="s">
         <v>1204</v>
       </c>
-      <c r="N189" s="2">
+      <c r="N189" s="1">
         <v>46120</v>
       </c>
       <c r="Q189" t="b">
@@ -11398,7 +11372,7 @@
       <c r="E190" t="s">
         <v>918</v>
       </c>
-      <c r="F190" s="2">
+      <c r="F190" s="1">
         <v>45965</v>
       </c>
       <c r="G190" t="s">
@@ -11436,7 +11410,7 @@
       <c r="E191" t="s">
         <v>919</v>
       </c>
-      <c r="F191" s="2">
+      <c r="F191" s="1">
         <v>45967</v>
       </c>
       <c r="G191" t="s">
@@ -11457,7 +11431,7 @@
       <c r="L191" t="s">
         <v>1205</v>
       </c>
-      <c r="N191" s="2">
+      <c r="N191" s="1">
         <v>45972</v>
       </c>
       <c r="Q191" t="b">
@@ -11480,7 +11454,7 @@
       <c r="E192" t="s">
         <v>920</v>
       </c>
-      <c r="F192" s="2">
+      <c r="F192" s="1">
         <v>45968</v>
       </c>
       <c r="G192" t="s">
@@ -11518,7 +11492,7 @@
       <c r="E193" t="s">
         <v>921</v>
       </c>
-      <c r="F193" s="2">
+      <c r="F193" s="1">
         <v>45968</v>
       </c>
       <c r="G193" t="s">
@@ -11556,7 +11530,7 @@
       <c r="E194" t="s">
         <v>922</v>
       </c>
-      <c r="F194" s="2">
+      <c r="F194" s="1">
         <v>45968</v>
       </c>
       <c r="G194" t="s">
@@ -11588,7 +11562,7 @@
       <c r="E195" t="s">
         <v>923</v>
       </c>
-      <c r="F195" s="2">
+      <c r="F195" s="1">
         <v>45971</v>
       </c>
       <c r="G195" t="s">
@@ -11626,7 +11600,7 @@
       <c r="E196" t="s">
         <v>924</v>
       </c>
-      <c r="F196" s="2">
+      <c r="F196" s="1">
         <v>45978</v>
       </c>
       <c r="G196" t="s">
@@ -11658,7 +11632,7 @@
       <c r="E197" t="s">
         <v>925</v>
       </c>
-      <c r="F197" s="2">
+      <c r="F197" s="1">
         <v>45978</v>
       </c>
       <c r="G197" t="s">
@@ -11690,7 +11664,7 @@
       <c r="E198" t="s">
         <v>926</v>
       </c>
-      <c r="F198" s="2">
+      <c r="F198" s="1">
         <v>45978</v>
       </c>
       <c r="G198" t="s">
@@ -11722,7 +11696,7 @@
       <c r="E199" t="s">
         <v>927</v>
       </c>
-      <c r="F199" s="2">
+      <c r="F199" s="1">
         <v>45979</v>
       </c>
       <c r="G199" t="s">
@@ -11743,7 +11717,7 @@
       <c r="L199" t="s">
         <v>1206</v>
       </c>
-      <c r="N199" s="2">
+      <c r="N199" s="1">
         <v>46049</v>
       </c>
       <c r="Q199" t="b">
@@ -11766,7 +11740,7 @@
       <c r="E200" t="s">
         <v>928</v>
       </c>
-      <c r="F200" s="2">
+      <c r="F200" s="1">
         <v>45986</v>
       </c>
       <c r="G200" t="s">
@@ -11804,7 +11778,7 @@
       <c r="E201" t="s">
         <v>929</v>
       </c>
-      <c r="F201" s="2">
+      <c r="F201" s="1">
         <v>45986</v>
       </c>
       <c r="G201" t="s">
@@ -11842,7 +11816,7 @@
       <c r="E202" t="s">
         <v>930</v>
       </c>
-      <c r="F202" s="2">
+      <c r="F202" s="1">
         <v>45986</v>
       </c>
       <c r="G202" t="s">
@@ -11880,7 +11854,7 @@
       <c r="E203" t="s">
         <v>931</v>
       </c>
-      <c r="F203" s="2">
+      <c r="F203" s="1">
         <v>45986</v>
       </c>
       <c r="G203" t="s">
@@ -11918,7 +11892,7 @@
       <c r="E204" t="s">
         <v>932</v>
       </c>
-      <c r="F204" s="2">
+      <c r="F204" s="1">
         <v>45986</v>
       </c>
       <c r="G204" t="s">
@@ -11956,7 +11930,7 @@
       <c r="E205" t="s">
         <v>933</v>
       </c>
-      <c r="F205" s="2">
+      <c r="F205" s="1">
         <v>45986</v>
       </c>
       <c r="G205" t="s">
@@ -11994,7 +11968,7 @@
       <c r="E206" t="s">
         <v>934</v>
       </c>
-      <c r="F206" s="2">
+      <c r="F206" s="1">
         <v>45986</v>
       </c>
       <c r="G206" t="s">
@@ -12029,7 +12003,7 @@
       <c r="E207" t="s">
         <v>935</v>
       </c>
-      <c r="F207" s="2">
+      <c r="F207" s="1">
         <v>45986</v>
       </c>
       <c r="G207" t="s">
@@ -12050,7 +12024,7 @@
       <c r="L207" t="s">
         <v>1208</v>
       </c>
-      <c r="N207" s="2">
+      <c r="N207" s="1">
         <v>46153</v>
       </c>
       <c r="Q207" t="b">
@@ -12073,7 +12047,7 @@
       <c r="E208" t="s">
         <v>936</v>
       </c>
-      <c r="F208" s="2">
+      <c r="F208" s="1">
         <v>45986</v>
       </c>
       <c r="G208" t="s">
@@ -12094,7 +12068,7 @@
       <c r="L208" t="s">
         <v>1209</v>
       </c>
-      <c r="N208" s="2">
+      <c r="N208" s="1">
         <v>46031</v>
       </c>
       <c r="Q208" t="b">
@@ -12117,7 +12091,7 @@
       <c r="E209" t="s">
         <v>937</v>
       </c>
-      <c r="F209" s="2">
+      <c r="F209" s="1">
         <v>46000</v>
       </c>
       <c r="G209" t="s">
@@ -12138,7 +12112,7 @@
       <c r="L209" t="s">
         <v>1210</v>
       </c>
-      <c r="N209" s="2">
+      <c r="N209" s="1">
         <v>46191</v>
       </c>
       <c r="Q209" t="b">
@@ -12161,7 +12135,7 @@
       <c r="E210" t="s">
         <v>938</v>
       </c>
-      <c r="F210" s="2">
+      <c r="F210" s="1">
         <v>46000</v>
       </c>
       <c r="G210" t="s">
@@ -12199,7 +12173,7 @@
       <c r="E211" t="s">
         <v>939</v>
       </c>
-      <c r="F211" s="2">
+      <c r="F211" s="1">
         <v>46000</v>
       </c>
       <c r="G211" t="s">
@@ -12234,7 +12208,7 @@
       <c r="E212" t="s">
         <v>940</v>
       </c>
-      <c r="F212" s="2">
+      <c r="F212" s="1">
         <v>46000</v>
       </c>
       <c r="G212" t="s">
@@ -12269,7 +12243,7 @@
       <c r="E213" t="s">
         <v>941</v>
       </c>
-      <c r="F213" s="2">
+      <c r="F213" s="1">
         <v>46007</v>
       </c>
       <c r="G213" t="s">
@@ -12307,7 +12281,7 @@
       <c r="E214" t="s">
         <v>942</v>
       </c>
-      <c r="F214" s="2">
+      <c r="F214" s="1">
         <v>46007</v>
       </c>
       <c r="G214" t="s">
@@ -12328,7 +12302,7 @@
       <c r="L214" t="s">
         <v>1213</v>
       </c>
-      <c r="N214" s="2">
+      <c r="N214" s="1">
         <v>46021</v>
       </c>
       <c r="O214">
@@ -12354,7 +12328,7 @@
       <c r="E215" t="s">
         <v>943</v>
       </c>
-      <c r="F215" s="2">
+      <c r="F215" s="1">
         <v>46007</v>
       </c>
       <c r="G215" t="s">
@@ -12392,7 +12366,7 @@
       <c r="E216" t="s">
         <v>944</v>
       </c>
-      <c r="F216" s="2">
+      <c r="F216" s="1">
         <v>46010</v>
       </c>
       <c r="G216" t="s">
@@ -12421,7 +12395,7 @@
       <c r="E217" t="s">
         <v>945</v>
       </c>
-      <c r="F217" s="2">
+      <c r="F217" s="1">
         <v>46010</v>
       </c>
       <c r="G217" t="s">
@@ -12442,7 +12416,7 @@
       <c r="L217" t="s">
         <v>1214</v>
       </c>
-      <c r="N217" s="2">
+      <c r="N217" s="1">
         <v>46052</v>
       </c>
       <c r="Q217" t="b">
@@ -12465,7 +12439,7 @@
       <c r="E218" t="s">
         <v>946</v>
       </c>
-      <c r="F218" s="2">
+      <c r="F218" s="1">
         <v>46010</v>
       </c>
       <c r="G218" t="s">
@@ -12503,7 +12477,7 @@
       <c r="E219" t="s">
         <v>947</v>
       </c>
-      <c r="F219" s="2">
+      <c r="F219" s="1">
         <v>46010</v>
       </c>
       <c r="G219" t="s">
@@ -12541,7 +12515,7 @@
       <c r="E220" t="s">
         <v>948</v>
       </c>
-      <c r="F220" s="2">
+      <c r="F220" s="1">
         <v>46010</v>
       </c>
       <c r="G220" t="s">
@@ -12579,7 +12553,7 @@
       <c r="E221" t="s">
         <v>949</v>
       </c>
-      <c r="F221" s="2">
+      <c r="F221" s="1">
         <v>46028</v>
       </c>
       <c r="G221" t="s">
@@ -12617,7 +12591,7 @@
       <c r="E222" t="s">
         <v>950</v>
       </c>
-      <c r="F222" s="2">
+      <c r="F222" s="1">
         <v>46028</v>
       </c>
       <c r="G222" t="s">
@@ -12655,7 +12629,7 @@
       <c r="E223" t="s">
         <v>951</v>
       </c>
-      <c r="F223" s="2">
+      <c r="F223" s="1">
         <v>46028</v>
       </c>
       <c r="G223" t="s">
@@ -12693,7 +12667,7 @@
       <c r="E224" t="s">
         <v>952</v>
       </c>
-      <c r="F224" s="2">
+      <c r="F224" s="1">
         <v>46028</v>
       </c>
       <c r="G224" t="s">
@@ -12731,7 +12705,7 @@
       <c r="E225" t="s">
         <v>953</v>
       </c>
-      <c r="F225" s="2">
+      <c r="F225" s="1">
         <v>46028</v>
       </c>
       <c r="G225" t="s">
@@ -12769,7 +12743,7 @@
       <c r="E226" t="s">
         <v>954</v>
       </c>
-      <c r="F226" s="2">
+      <c r="F226" s="1">
         <v>46028</v>
       </c>
       <c r="G226" t="s">
@@ -12807,7 +12781,7 @@
       <c r="E227" t="s">
         <v>955</v>
       </c>
-      <c r="F227" s="2">
+      <c r="F227" s="1">
         <v>46028</v>
       </c>
       <c r="G227" t="s">
@@ -12845,7 +12819,7 @@
       <c r="E228" t="s">
         <v>956</v>
       </c>
-      <c r="F228" s="2">
+      <c r="F228" s="1">
         <v>46028</v>
       </c>
       <c r="G228" t="s">
@@ -12883,7 +12857,7 @@
       <c r="E229" t="s">
         <v>957</v>
       </c>
-      <c r="F229" s="2">
+      <c r="F229" s="1">
         <v>46028</v>
       </c>
       <c r="G229" t="s">
@@ -12918,7 +12892,7 @@
       <c r="E230" t="s">
         <v>958</v>
       </c>
-      <c r="F230" s="2">
+      <c r="F230" s="1">
         <v>46028</v>
       </c>
       <c r="G230" t="s">
@@ -12956,7 +12930,7 @@
       <c r="E231" t="s">
         <v>959</v>
       </c>
-      <c r="F231" s="2">
+      <c r="F231" s="1">
         <v>46028</v>
       </c>
       <c r="G231" t="s">
@@ -12977,7 +12951,7 @@
       <c r="L231" t="s">
         <v>1215</v>
       </c>
-      <c r="N231" s="2">
+      <c r="N231" s="1">
         <v>46063</v>
       </c>
       <c r="Q231" t="b">
@@ -13000,7 +12974,7 @@
       <c r="E232" t="s">
         <v>960</v>
       </c>
-      <c r="F232" s="2">
+      <c r="F232" s="1">
         <v>46028</v>
       </c>
       <c r="G232" t="s">
@@ -13035,7 +13009,7 @@
       <c r="E233" t="s">
         <v>961</v>
       </c>
-      <c r="F233" s="2">
+      <c r="F233" s="1">
         <v>46028</v>
       </c>
       <c r="G233" t="s">
@@ -13070,7 +13044,7 @@
       <c r="E234" t="s">
         <v>962</v>
       </c>
-      <c r="F234" s="2">
+      <c r="F234" s="1">
         <v>46028</v>
       </c>
       <c r="G234" t="s">
@@ -13091,7 +13065,7 @@
       <c r="L234" t="s">
         <v>1215</v>
       </c>
-      <c r="N234" s="2">
+      <c r="N234" s="1">
         <v>46063</v>
       </c>
       <c r="P234" t="s">
@@ -13117,7 +13091,7 @@
       <c r="E235" t="s">
         <v>963</v>
       </c>
-      <c r="F235" s="2">
+      <c r="F235" s="1">
         <v>46028</v>
       </c>
       <c r="G235" t="s">
@@ -13138,7 +13112,7 @@
       <c r="L235" t="s">
         <v>1215</v>
       </c>
-      <c r="N235" s="2">
+      <c r="N235" s="1">
         <v>46063</v>
       </c>
       <c r="P235" t="s">
@@ -13164,7 +13138,7 @@
       <c r="E236" t="s">
         <v>964</v>
       </c>
-      <c r="F236" s="2">
+      <c r="F236" s="1">
         <v>46028</v>
       </c>
       <c r="G236" t="s">
@@ -13185,7 +13159,7 @@
       <c r="L236" t="s">
         <v>1217</v>
       </c>
-      <c r="N236" s="2">
+      <c r="N236" s="1">
         <v>46114</v>
       </c>
       <c r="Q236" t="b">
@@ -13208,7 +13182,7 @@
       <c r="E237" t="s">
         <v>965</v>
       </c>
-      <c r="F237" s="2">
+      <c r="F237" s="1">
         <v>46028</v>
       </c>
       <c r="G237" t="s">
@@ -13246,7 +13220,7 @@
       <c r="E238" t="s">
         <v>966</v>
       </c>
-      <c r="F238" s="2">
+      <c r="F238" s="1">
         <v>46028</v>
       </c>
       <c r="G238" t="s">
@@ -13275,7 +13249,7 @@
       <c r="E239" t="s">
         <v>967</v>
       </c>
-      <c r="F239" s="2">
+      <c r="F239" s="1">
         <v>46036</v>
       </c>
       <c r="G239" t="s">
@@ -13293,7 +13267,7 @@
       <c r="L239" t="s">
         <v>1218</v>
       </c>
-      <c r="N239" s="2">
+      <c r="N239" s="1">
         <v>46052</v>
       </c>
       <c r="Q239" t="b">
@@ -13316,7 +13290,7 @@
       <c r="E240" t="s">
         <v>968</v>
       </c>
-      <c r="F240" s="2">
+      <c r="F240" s="1">
         <v>46036</v>
       </c>
       <c r="G240" t="s">
@@ -13351,7 +13325,7 @@
       <c r="E241" t="s">
         <v>969</v>
       </c>
-      <c r="F241" s="2">
+      <c r="F241" s="1">
         <v>46036</v>
       </c>
       <c r="G241" t="s">
@@ -13386,7 +13360,7 @@
       <c r="E242" t="s">
         <v>970</v>
       </c>
-      <c r="F242" s="2">
+      <c r="F242" s="1">
         <v>46036</v>
       </c>
       <c r="G242" t="s">
@@ -13424,7 +13398,7 @@
       <c r="E243" t="s">
         <v>971</v>
       </c>
-      <c r="F243" s="2">
+      <c r="F243" s="1">
         <v>46048</v>
       </c>
       <c r="G243" t="s">
@@ -13456,7 +13430,7 @@
       <c r="E244" t="s">
         <v>972</v>
       </c>
-      <c r="F244" s="2">
+      <c r="F244" s="1">
         <v>46048</v>
       </c>
       <c r="G244" t="s">
@@ -13494,7 +13468,7 @@
       <c r="E245" t="s">
         <v>973</v>
       </c>
-      <c r="F245" s="2">
+      <c r="F245" s="1">
         <v>46048</v>
       </c>
       <c r="G245" t="s">
@@ -13532,7 +13506,7 @@
       <c r="E246" t="s">
         <v>974</v>
       </c>
-      <c r="F246" s="2">
+      <c r="F246" s="1">
         <v>46050</v>
       </c>
       <c r="G246" t="s">
@@ -13553,7 +13527,7 @@
       <c r="L246" t="s">
         <v>1221</v>
       </c>
-      <c r="N246" s="2">
+      <c r="N246" s="1">
         <v>46191</v>
       </c>
       <c r="Q246" t="b">
@@ -13576,7 +13550,7 @@
       <c r="E247" t="s">
         <v>975</v>
       </c>
-      <c r="F247" s="2">
+      <c r="F247" s="1">
         <v>46050</v>
       </c>
       <c r="G247" t="s">
@@ -13608,7 +13582,7 @@
       <c r="E248" t="s">
         <v>976</v>
       </c>
-      <c r="F248" s="2">
+      <c r="F248" s="1">
         <v>46050</v>
       </c>
       <c r="G248" t="s">
@@ -13637,7 +13611,7 @@
       <c r="E249" t="s">
         <v>977</v>
       </c>
-      <c r="F249" s="2">
+      <c r="F249" s="1">
         <v>46050</v>
       </c>
       <c r="G249" t="s">
@@ -13675,7 +13649,7 @@
       <c r="E250" t="s">
         <v>978</v>
       </c>
-      <c r="F250" s="2">
+      <c r="F250" s="1">
         <v>46063</v>
       </c>
       <c r="G250" t="s">
@@ -13713,7 +13687,7 @@
       <c r="E251" t="s">
         <v>979</v>
       </c>
-      <c r="F251" s="2">
+      <c r="F251" s="1">
         <v>46063</v>
       </c>
       <c r="G251" t="s">
@@ -13748,7 +13722,7 @@
       <c r="E252" t="s">
         <v>980</v>
       </c>
-      <c r="F252" s="2">
+      <c r="F252" s="1">
         <v>46063</v>
       </c>
       <c r="G252" t="s">
@@ -13783,7 +13757,7 @@
       <c r="E253" t="s">
         <v>981</v>
       </c>
-      <c r="F253" s="2">
+      <c r="F253" s="1">
         <v>46063</v>
       </c>
       <c r="G253" t="s">
@@ -13821,7 +13795,7 @@
       <c r="E254" t="s">
         <v>982</v>
       </c>
-      <c r="F254" s="2">
+      <c r="F254" s="1">
         <v>46063</v>
       </c>
       <c r="G254" t="s">
@@ -13859,7 +13833,7 @@
       <c r="E255" t="s">
         <v>983</v>
       </c>
-      <c r="F255" s="2">
+      <c r="F255" s="1">
         <v>46063</v>
       </c>
       <c r="G255" t="s">
@@ -13897,7 +13871,7 @@
       <c r="E256" t="s">
         <v>984</v>
       </c>
-      <c r="F256" s="2">
+      <c r="F256" s="1">
         <v>46063</v>
       </c>
       <c r="G256" t="s">
@@ -13938,7 +13912,7 @@
       <c r="E257" t="s">
         <v>985</v>
       </c>
-      <c r="F257" s="2">
+      <c r="F257" s="1">
         <v>46063</v>
       </c>
       <c r="G257" t="s">
@@ -13967,7 +13941,7 @@
       <c r="E258" t="s">
         <v>986</v>
       </c>
-      <c r="F258" s="2">
+      <c r="F258" s="1">
         <v>46063</v>
       </c>
       <c r="G258" t="s">
@@ -13996,7 +13970,7 @@
       <c r="E259" t="s">
         <v>987</v>
       </c>
-      <c r="F259" s="2">
+      <c r="F259" s="1">
         <v>46063</v>
       </c>
       <c r="G259" t="s">
@@ -14034,7 +14008,7 @@
       <c r="E260" t="s">
         <v>988</v>
       </c>
-      <c r="F260" s="2">
+      <c r="F260" s="1">
         <v>46063</v>
       </c>
       <c r="G260" t="s">
@@ -14072,7 +14046,7 @@
       <c r="E261" t="s">
         <v>989</v>
       </c>
-      <c r="F261" s="2">
+      <c r="F261" s="1">
         <v>46063</v>
       </c>
       <c r="G261" t="s">
@@ -14110,7 +14084,7 @@
       <c r="E262" t="s">
         <v>990</v>
       </c>
-      <c r="F262" s="2">
+      <c r="F262" s="1">
         <v>46063</v>
       </c>
       <c r="G262" t="s">
@@ -14131,7 +14105,7 @@
       <c r="L262" t="s">
         <v>1224</v>
       </c>
-      <c r="N262" s="2">
+      <c r="N262" s="1">
         <v>46113</v>
       </c>
       <c r="P262" t="s">
@@ -14157,7 +14131,7 @@
       <c r="E263" t="s">
         <v>991</v>
       </c>
-      <c r="F263" s="2">
+      <c r="F263" s="1">
         <v>46063</v>
       </c>
       <c r="G263" t="s">
@@ -14195,7 +14169,7 @@
       <c r="E264" t="s">
         <v>992</v>
       </c>
-      <c r="F264" s="2">
+      <c r="F264" s="1">
         <v>46063</v>
       </c>
       <c r="G264" t="s">
@@ -14233,7 +14207,7 @@
       <c r="E265" t="s">
         <v>993</v>
       </c>
-      <c r="F265" s="2">
+      <c r="F265" s="1">
         <v>46063</v>
       </c>
       <c r="G265" t="s">
@@ -14271,7 +14245,7 @@
       <c r="E266" t="s">
         <v>994</v>
       </c>
-      <c r="F266" s="2">
+      <c r="F266" s="1">
         <v>46063</v>
       </c>
       <c r="G266" t="s">
@@ -14309,7 +14283,7 @@
       <c r="E267" t="s">
         <v>995</v>
       </c>
-      <c r="F267" s="2">
+      <c r="F267" s="1">
         <v>46063</v>
       </c>
       <c r="G267" t="s">
@@ -14347,7 +14321,7 @@
       <c r="E268" t="s">
         <v>996</v>
       </c>
-      <c r="F268" s="2">
+      <c r="F268" s="1">
         <v>46063</v>
       </c>
       <c r="G268" t="s">
@@ -14382,7 +14356,7 @@
       <c r="D269" t="s">
         <v>712</v>
       </c>
-      <c r="F269" s="2">
+      <c r="F269" s="1">
         <v>46063</v>
       </c>
       <c r="G269" t="s">
@@ -14420,7 +14394,7 @@
       <c r="E270" t="s">
         <v>997</v>
       </c>
-      <c r="F270" s="2">
+      <c r="F270" s="1">
         <v>46063</v>
       </c>
       <c r="G270" t="s">
@@ -14458,7 +14432,7 @@
       <c r="E271" t="s">
         <v>998</v>
       </c>
-      <c r="F271" s="2">
+      <c r="F271" s="1">
         <v>46063</v>
       </c>
       <c r="G271" t="s">
@@ -14496,7 +14470,7 @@
       <c r="E272" t="s">
         <v>999</v>
       </c>
-      <c r="F272" s="2">
+      <c r="F272" s="1">
         <v>46063</v>
       </c>
       <c r="G272" t="s">
@@ -14517,7 +14491,7 @@
       <c r="L272" t="s">
         <v>1226</v>
       </c>
-      <c r="N272" s="2">
+      <c r="N272" s="1">
         <v>46185</v>
       </c>
       <c r="O272" t="s">
@@ -14543,7 +14517,7 @@
       <c r="E273" t="s">
         <v>1000</v>
       </c>
-      <c r="F273" s="2">
+      <c r="F273" s="1">
         <v>46063</v>
       </c>
       <c r="G273" t="s">
@@ -14578,7 +14552,7 @@
       <c r="E274" t="s">
         <v>1001</v>
       </c>
-      <c r="F274" s="2">
+      <c r="F274" s="1">
         <v>46063</v>
       </c>
       <c r="G274" t="s">
@@ -14616,7 +14590,7 @@
       <c r="E275" t="s">
         <v>1002</v>
       </c>
-      <c r="F275" s="2">
+      <c r="F275" s="1">
         <v>46063</v>
       </c>
       <c r="G275" t="s">
@@ -14651,7 +14625,7 @@
       <c r="E276" t="s">
         <v>1003</v>
       </c>
-      <c r="F276" s="2">
+      <c r="F276" s="1">
         <v>46063</v>
       </c>
       <c r="G276" t="s">
@@ -14689,7 +14663,7 @@
       <c r="E277" t="s">
         <v>1004</v>
       </c>
-      <c r="F277" s="2">
+      <c r="F277" s="1">
         <v>46063</v>
       </c>
       <c r="G277" t="s">
@@ -14727,7 +14701,7 @@
       <c r="E278" t="s">
         <v>1005</v>
       </c>
-      <c r="F278" s="2">
+      <c r="F278" s="1">
         <v>46077</v>
       </c>
       <c r="G278" t="s">
@@ -14765,7 +14739,7 @@
       <c r="E279" t="s">
         <v>1006</v>
       </c>
-      <c r="F279" s="2">
+      <c r="F279" s="1">
         <v>46077</v>
       </c>
       <c r="G279" t="s">
@@ -14806,7 +14780,7 @@
       <c r="E280" t="s">
         <v>1007</v>
       </c>
-      <c r="F280" s="2">
+      <c r="F280" s="1">
         <v>46085</v>
       </c>
       <c r="G280" t="s">
@@ -14844,7 +14818,7 @@
       <c r="E281" t="s">
         <v>1008</v>
       </c>
-      <c r="F281" s="2">
+      <c r="F281" s="1">
         <v>46085</v>
       </c>
       <c r="G281" t="s">
@@ -14882,7 +14856,7 @@
       <c r="E282" t="s">
         <v>1009</v>
       </c>
-      <c r="F282" s="2">
+      <c r="F282" s="1">
         <v>46090</v>
       </c>
       <c r="G282" t="s">
@@ -14920,7 +14894,7 @@
       <c r="E283" t="s">
         <v>1010</v>
       </c>
-      <c r="F283" s="2">
+      <c r="F283" s="1">
         <v>46100</v>
       </c>
       <c r="G283" t="s">
@@ -14955,7 +14929,7 @@
       <c r="E284" t="s">
         <v>1011</v>
       </c>
-      <c r="F284" s="2">
+      <c r="F284" s="1">
         <v>46100</v>
       </c>
       <c r="G284" t="s">
@@ -14990,7 +14964,7 @@
       <c r="E285" t="s">
         <v>1012</v>
       </c>
-      <c r="F285" s="2">
+      <c r="F285" s="1">
         <v>46100</v>
       </c>
       <c r="G285" t="s">
@@ -15025,7 +14999,7 @@
       <c r="E286" t="s">
         <v>1013</v>
       </c>
-      <c r="F286" s="2">
+      <c r="F286" s="1">
         <v>46100</v>
       </c>
       <c r="G286" t="s">
@@ -15060,7 +15034,7 @@
       <c r="E287">
         <v>35971</v>
       </c>
-      <c r="F287" s="2">
+      <c r="F287" s="1">
         <v>46107</v>
       </c>
       <c r="G287" t="s">
@@ -15089,7 +15063,7 @@
       <c r="E288">
         <v>107178</v>
       </c>
-      <c r="F288" s="2">
+      <c r="F288" s="1">
         <v>46107</v>
       </c>
       <c r="G288" t="s">
@@ -15127,7 +15101,7 @@
       <c r="E289">
         <v>108773</v>
       </c>
-      <c r="F289" s="2">
+      <c r="F289" s="1">
         <v>46107</v>
       </c>
       <c r="G289" t="s">
@@ -15156,7 +15130,7 @@
       <c r="E290">
         <v>7086</v>
       </c>
-      <c r="F290" s="2">
+      <c r="F290" s="1">
         <v>46107</v>
       </c>
       <c r="G290" t="s">
@@ -15174,7 +15148,7 @@
       <c r="K290" t="s">
         <v>1146</v>
       </c>
-      <c r="N290" s="2">
+      <c r="N290" s="1">
         <v>46127</v>
       </c>
       <c r="Q290" t="b">
@@ -15197,7 +15171,7 @@
       <c r="E291">
         <v>99743</v>
       </c>
-      <c r="F291" s="2">
+      <c r="F291" s="1">
         <v>46107</v>
       </c>
       <c r="G291" t="s">
@@ -15235,7 +15209,7 @@
       <c r="E292" t="s">
         <v>1014</v>
       </c>
-      <c r="F292" s="2">
+      <c r="F292" s="1">
         <v>46112</v>
       </c>
       <c r="G292" t="s">
@@ -15273,7 +15247,7 @@
       <c r="E293" t="s">
         <v>1015</v>
       </c>
-      <c r="F293" s="2">
+      <c r="F293" s="1">
         <v>46125</v>
       </c>
       <c r="G293" t="s">
@@ -15311,7 +15285,7 @@
       <c r="E294" t="s">
         <v>1016</v>
       </c>
-      <c r="F294" s="2">
+      <c r="F294" s="1">
         <v>46125</v>
       </c>
       <c r="G294" t="s">
@@ -15346,7 +15320,7 @@
       <c r="E295" t="s">
         <v>1017</v>
       </c>
-      <c r="F295" s="2">
+      <c r="F295" s="1">
         <v>46125</v>
       </c>
       <c r="G295" t="s">
@@ -15381,7 +15355,7 @@
       <c r="E296" t="s">
         <v>1018</v>
       </c>
-      <c r="F296" s="2">
+      <c r="F296" s="1">
         <v>46125</v>
       </c>
       <c r="G296" t="s">
@@ -15416,7 +15390,7 @@
       <c r="E297">
         <v>47203152</v>
       </c>
-      <c r="F297" s="2">
+      <c r="F297" s="1">
         <v>46125</v>
       </c>
       <c r="G297" t="s">
@@ -15451,7 +15425,7 @@
       <c r="E298">
         <v>47202512</v>
       </c>
-      <c r="F298" s="2">
+      <c r="F298" s="1">
         <v>46125</v>
       </c>
       <c r="G298" t="s">
@@ -15489,7 +15463,7 @@
       <c r="E299">
         <v>22005580</v>
       </c>
-      <c r="F299" s="2">
+      <c r="F299" s="1">
         <v>46125</v>
       </c>
       <c r="G299" t="s">
@@ -15527,7 +15501,7 @@
       <c r="E300">
         <v>22005955</v>
       </c>
-      <c r="F300" s="2">
+      <c r="F300" s="1">
         <v>46125</v>
       </c>
       <c r="G300" t="s">
@@ -15565,7 +15539,7 @@
       <c r="E301">
         <v>22005661</v>
       </c>
-      <c r="F301" s="2">
+      <c r="F301" s="1">
         <v>46125</v>
       </c>
       <c r="G301" t="s">
@@ -15603,7 +15577,7 @@
       <c r="E302">
         <v>32207</v>
       </c>
-      <c r="F302" s="2">
+      <c r="F302" s="1">
         <v>46125</v>
       </c>
       <c r="G302" t="s">
@@ -15641,7 +15615,7 @@
       <c r="E303">
         <v>18156</v>
       </c>
-      <c r="F303" s="2">
+      <c r="F303" s="1">
         <v>46125</v>
       </c>
       <c r="G303" t="s">
@@ -15679,7 +15653,7 @@
       <c r="E304">
         <v>37971</v>
       </c>
-      <c r="F304" s="2">
+      <c r="F304" s="1">
         <v>46125</v>
       </c>
       <c r="G304" t="s">
@@ -15717,7 +15691,7 @@
       <c r="E305">
         <v>84317</v>
       </c>
-      <c r="F305" s="2">
+      <c r="F305" s="1">
         <v>46125</v>
       </c>
       <c r="G305" t="s">
@@ -15738,7 +15712,7 @@
       <c r="L305" t="s">
         <v>1231</v>
       </c>
-      <c r="N305" s="2">
+      <c r="N305" s="1">
         <v>46160</v>
       </c>
       <c r="Q305" t="b">
@@ -15761,7 +15735,7 @@
       <c r="E306">
         <v>83773</v>
       </c>
-      <c r="F306" s="2">
+      <c r="F306" s="1">
         <v>46125</v>
       </c>
       <c r="G306" t="s">
@@ -15782,7 +15756,7 @@
       <c r="L306" t="s">
         <v>1232</v>
       </c>
-      <c r="N306" s="2">
+      <c r="N306" s="1">
         <v>46156</v>
       </c>
       <c r="Q306" t="b">
@@ -15805,7 +15779,7 @@
       <c r="E307">
         <v>83740</v>
       </c>
-      <c r="F307" s="2">
+      <c r="F307" s="1">
         <v>46125</v>
       </c>
       <c r="G307" t="s">
@@ -15843,7 +15817,7 @@
       <c r="E308">
         <v>84326</v>
       </c>
-      <c r="F308" s="2">
+      <c r="F308" s="1">
         <v>46125</v>
       </c>
       <c r="G308" t="s">
@@ -15881,7 +15855,7 @@
       <c r="E309">
         <v>6708</v>
       </c>
-      <c r="F309" s="2">
+      <c r="F309" s="1">
         <v>46125</v>
       </c>
       <c r="G309" t="s">
@@ -15919,7 +15893,7 @@
       <c r="E310" t="s">
         <v>1019</v>
       </c>
-      <c r="F310" s="2">
+      <c r="F310" s="1">
         <v>46125</v>
       </c>
       <c r="G310" t="s">
@@ -15957,7 +15931,7 @@
       <c r="E311">
         <v>9727</v>
       </c>
-      <c r="F311" s="2">
+      <c r="F311" s="1">
         <v>46125</v>
       </c>
       <c r="G311" t="s">
@@ -15995,7 +15969,7 @@
       <c r="E312" t="s">
         <v>1020</v>
       </c>
-      <c r="F312" s="2">
+      <c r="F312" s="1">
         <v>46125</v>
       </c>
       <c r="G312" t="s">
@@ -16033,7 +16007,7 @@
       <c r="E313">
         <v>31</v>
       </c>
-      <c r="F313" s="2">
+      <c r="F313" s="1">
         <v>46125</v>
       </c>
       <c r="G313" t="s">
@@ -16068,7 +16042,7 @@
       <c r="E314">
         <v>965</v>
       </c>
-      <c r="F314" s="2">
+      <c r="F314" s="1">
         <v>46125</v>
       </c>
       <c r="G314" t="s">
@@ -16106,7 +16080,7 @@
       <c r="E315">
         <v>2007</v>
       </c>
-      <c r="F315" s="2">
+      <c r="F315" s="1">
         <v>46125</v>
       </c>
       <c r="G315" t="s">
@@ -16144,7 +16118,7 @@
       <c r="E316">
         <v>688</v>
       </c>
-      <c r="F316" s="2">
+      <c r="F316" s="1">
         <v>46125</v>
       </c>
       <c r="G316" t="s">
@@ -16182,7 +16156,7 @@
       <c r="E317" t="s">
         <v>1021</v>
       </c>
-      <c r="F317" s="2">
+      <c r="F317" s="1">
         <v>46125</v>
       </c>
       <c r="G317" t="s">
@@ -16220,7 +16194,7 @@
       <c r="E318" t="s">
         <v>1022</v>
       </c>
-      <c r="F318" s="2">
+      <c r="F318" s="1">
         <v>46125</v>
       </c>
       <c r="G318" t="s">
@@ -16252,7 +16226,7 @@
       <c r="E319" t="s">
         <v>1023</v>
       </c>
-      <c r="F319" s="2">
+      <c r="F319" s="1">
         <v>46125</v>
       </c>
       <c r="G319" t="s">
@@ -16270,7 +16244,7 @@
       <c r="L319" t="s">
         <v>1233</v>
       </c>
-      <c r="N319" s="2">
+      <c r="N319" s="1">
         <v>46175</v>
       </c>
       <c r="Q319" t="b">
@@ -16293,7 +16267,7 @@
       <c r="E320">
         <v>1391</v>
       </c>
-      <c r="F320" s="2">
+      <c r="F320" s="1">
         <v>46125</v>
       </c>
       <c r="G320" t="s">
@@ -16331,7 +16305,7 @@
       <c r="E321">
         <v>120315</v>
       </c>
-      <c r="F321" s="2">
+      <c r="F321" s="1">
         <v>46125</v>
       </c>
       <c r="G321" t="s">
@@ -16369,7 +16343,7 @@
       <c r="E322" t="s">
         <v>1024</v>
       </c>
-      <c r="F322" s="2">
+      <c r="F322" s="1">
         <v>46125</v>
       </c>
       <c r="G322" t="s">
@@ -16390,7 +16364,7 @@
       <c r="L322" t="s">
         <v>1234</v>
       </c>
-      <c r="N322" s="2">
+      <c r="N322" s="1">
         <v>46182</v>
       </c>
       <c r="Q322" t="b">
@@ -16413,7 +16387,7 @@
       <c r="E323">
         <v>535933</v>
       </c>
-      <c r="F323" s="2">
+      <c r="F323" s="1">
         <v>46125</v>
       </c>
       <c r="G323" t="s">
@@ -16451,7 +16425,7 @@
       <c r="E324">
         <v>289029</v>
       </c>
-      <c r="F324" s="2">
+      <c r="F324" s="1">
         <v>46125</v>
       </c>
       <c r="G324" t="s">
@@ -16489,7 +16463,7 @@
       <c r="E325">
         <v>3454</v>
       </c>
-      <c r="F325" s="2">
+      <c r="F325" s="1">
         <v>46125</v>
       </c>
       <c r="G325" t="s">
@@ -16510,7 +16484,7 @@
       <c r="L325" t="s">
         <v>1234</v>
       </c>
-      <c r="N325" s="2">
+      <c r="N325" s="1">
         <v>46182</v>
       </c>
       <c r="Q325" t="b">
@@ -16533,7 +16507,7 @@
       <c r="E326">
         <v>3493</v>
       </c>
-      <c r="F326" s="2">
+      <c r="F326" s="1">
         <v>46125</v>
       </c>
       <c r="G326" t="s">
@@ -16571,7 +16545,7 @@
       <c r="E327" t="s">
         <v>1024</v>
       </c>
-      <c r="F327" s="2">
+      <c r="F327" s="1">
         <v>46125</v>
       </c>
       <c r="G327" t="s">
@@ -16592,7 +16566,7 @@
       <c r="L327" t="s">
         <v>1234</v>
       </c>
-      <c r="N327" s="2">
+      <c r="N327" s="1">
         <v>46182</v>
       </c>
       <c r="Q327" t="b">
@@ -16615,7 +16589,7 @@
       <c r="E328">
         <v>3235</v>
       </c>
-      <c r="F328" s="2">
+      <c r="F328" s="1">
         <v>46125</v>
       </c>
       <c r="G328" t="s">
@@ -16636,7 +16610,7 @@
       <c r="L328" t="s">
         <v>1234</v>
       </c>
-      <c r="N328" s="2">
+      <c r="N328" s="1">
         <v>46182</v>
       </c>
       <c r="Q328" t="b">
@@ -16659,7 +16633,7 @@
       <c r="E329">
         <v>625052</v>
       </c>
-      <c r="F329" s="2">
+      <c r="F329" s="1">
         <v>46125</v>
       </c>
       <c r="G329" t="s">
@@ -16680,7 +16654,7 @@
       <c r="L329" t="s">
         <v>1234</v>
       </c>
-      <c r="N329" s="2">
+      <c r="N329" s="1">
         <v>46182</v>
       </c>
       <c r="Q329" t="b">
@@ -16703,7 +16677,7 @@
       <c r="E330">
         <v>614095</v>
       </c>
-      <c r="F330" s="2">
+      <c r="F330" s="1">
         <v>46125</v>
       </c>
       <c r="G330" t="s">
@@ -16724,7 +16698,7 @@
       <c r="L330" t="s">
         <v>1234</v>
       </c>
-      <c r="N330" s="2">
+      <c r="N330" s="1">
         <v>46182</v>
       </c>
       <c r="Q330" t="b">
@@ -16747,7 +16721,7 @@
       <c r="E331" t="s">
         <v>966</v>
       </c>
-      <c r="F331" s="2">
+      <c r="F331" s="1">
         <v>46125</v>
       </c>
       <c r="G331" t="s">
@@ -16785,7 +16759,7 @@
       <c r="E332" t="s">
         <v>1025</v>
       </c>
-      <c r="F332" s="2">
+      <c r="F332" s="1">
         <v>46125</v>
       </c>
       <c r="G332" t="s">
@@ -16823,7 +16797,7 @@
       <c r="E333">
         <v>197</v>
       </c>
-      <c r="F333" s="2">
+      <c r="F333" s="1">
         <v>46125</v>
       </c>
       <c r="G333" t="s">
@@ -16861,7 +16835,7 @@
       <c r="E334">
         <v>1378</v>
       </c>
-      <c r="F334" s="2">
+      <c r="F334" s="1">
         <v>46125</v>
       </c>
       <c r="G334" t="s">
@@ -16899,7 +16873,7 @@
       <c r="E335" t="s">
         <v>1026</v>
       </c>
-      <c r="F335" s="2">
+      <c r="F335" s="1">
         <v>46127</v>
       </c>
       <c r="G335" t="s">
@@ -16917,7 +16891,7 @@
       <c r="L335" t="s">
         <v>1233</v>
       </c>
-      <c r="N335" s="2">
+      <c r="N335" s="1">
         <v>46175</v>
       </c>
       <c r="Q335" t="b">
@@ -16940,7 +16914,7 @@
       <c r="E336" t="s">
         <v>1027</v>
       </c>
-      <c r="F336" s="2">
+      <c r="F336" s="1">
         <v>46127</v>
       </c>
       <c r="G336" t="s">
@@ -16978,7 +16952,7 @@
       <c r="E337" t="s">
         <v>1028</v>
       </c>
-      <c r="F337" s="2">
+      <c r="F337" s="1">
         <v>46127</v>
       </c>
       <c r="G337" t="s">
@@ -16996,7 +16970,7 @@
       <c r="L337" t="s">
         <v>1233</v>
       </c>
-      <c r="N337" s="2">
+      <c r="N337" s="1">
         <v>46175</v>
       </c>
       <c r="Q337" t="b">
@@ -17019,7 +16993,7 @@
       <c r="E338" t="s">
         <v>1029</v>
       </c>
-      <c r="F338" s="2">
+      <c r="F338" s="1">
         <v>46127</v>
       </c>
       <c r="G338" t="s">
@@ -17057,7 +17031,7 @@
       <c r="E339">
         <v>6291</v>
       </c>
-      <c r="F339" s="2">
+      <c r="F339" s="1">
         <v>46129</v>
       </c>
       <c r="G339" t="s">
@@ -17086,7 +17060,7 @@
       <c r="E340" t="s">
         <v>1030</v>
       </c>
-      <c r="F340" s="2">
+      <c r="F340" s="1">
         <v>46142</v>
       </c>
       <c r="G340" t="s">
@@ -17124,7 +17098,7 @@
       <c r="E341" t="s">
         <v>1031</v>
       </c>
-      <c r="F341" s="2">
+      <c r="F341" s="1">
         <v>46142</v>
       </c>
       <c r="G341" t="s">
@@ -17162,7 +17136,7 @@
       <c r="E342" t="s">
         <v>1032</v>
       </c>
-      <c r="F342" s="2">
+      <c r="F342" s="1">
         <v>46142</v>
       </c>
       <c r="G342" t="s">
@@ -17200,7 +17174,7 @@
       <c r="E343" t="s">
         <v>1033</v>
       </c>
-      <c r="F343" s="2">
+      <c r="F343" s="1">
         <v>46142</v>
       </c>
       <c r="G343" t="s">
@@ -17238,7 +17212,7 @@
       <c r="E344" t="s">
         <v>1034</v>
       </c>
-      <c r="F344" s="2">
+      <c r="F344" s="1">
         <v>46142</v>
       </c>
       <c r="G344" t="s">
@@ -17276,7 +17250,7 @@
       <c r="E345" t="s">
         <v>1035</v>
       </c>
-      <c r="F345" s="2">
+      <c r="F345" s="1">
         <v>46142</v>
       </c>
       <c r="G345" t="s">
@@ -17314,7 +17288,7 @@
       <c r="E346" t="s">
         <v>1036</v>
       </c>
-      <c r="F346" s="2">
+      <c r="F346" s="1">
         <v>46142</v>
       </c>
       <c r="G346" t="s">
@@ -17352,7 +17326,7 @@
       <c r="E347" t="s">
         <v>1037</v>
       </c>
-      <c r="F347" s="2">
+      <c r="F347" s="1">
         <v>46142</v>
       </c>
       <c r="G347" t="s">
@@ -17373,7 +17347,7 @@
       <c r="L347" t="s">
         <v>1231</v>
       </c>
-      <c r="N347" s="2">
+      <c r="N347" s="1">
         <v>46160</v>
       </c>
       <c r="Q347" t="b">
@@ -17396,7 +17370,7 @@
       <c r="E348" t="s">
         <v>1038</v>
       </c>
-      <c r="F348" s="2">
+      <c r="F348" s="1">
         <v>46142</v>
       </c>
       <c r="G348" t="s">
@@ -17417,7 +17391,7 @@
       <c r="L348" t="s">
         <v>1232</v>
       </c>
-      <c r="N348" s="2">
+      <c r="N348" s="1">
         <v>46156</v>
       </c>
       <c r="Q348" t="b">
@@ -17440,7 +17414,7 @@
       <c r="E349" t="s">
         <v>1039</v>
       </c>
-      <c r="F349" s="2">
+      <c r="F349" s="1">
         <v>46142</v>
       </c>
       <c r="G349" t="s">
@@ -17478,7 +17452,7 @@
       <c r="E350" t="s">
         <v>1040</v>
       </c>
-      <c r="F350" s="2">
+      <c r="F350" s="1">
         <v>46142</v>
       </c>
       <c r="G350" t="s">
@@ -17513,7 +17487,7 @@
       <c r="E351" t="s">
         <v>1041</v>
       </c>
-      <c r="F351" s="2">
+      <c r="F351" s="1">
         <v>46142</v>
       </c>
       <c r="G351" t="s">
@@ -17551,7 +17525,7 @@
       <c r="E352" t="s">
         <v>1042</v>
       </c>
-      <c r="F352" s="2">
+      <c r="F352" s="1">
         <v>46142</v>
       </c>
       <c r="G352" t="s">
@@ -17589,7 +17563,7 @@
       <c r="E353" t="s">
         <v>1043</v>
       </c>
-      <c r="F353" s="2">
+      <c r="F353" s="1">
         <v>46142</v>
       </c>
       <c r="G353" t="s">
@@ -17627,7 +17601,7 @@
       <c r="E354" t="s">
         <v>1044</v>
       </c>
-      <c r="F354" s="2">
+      <c r="F354" s="1">
         <v>46142</v>
       </c>
       <c r="G354" t="s">
@@ -17665,7 +17639,7 @@
       <c r="E355" t="s">
         <v>1045</v>
       </c>
-      <c r="F355" s="2">
+      <c r="F355" s="1">
         <v>46142</v>
       </c>
       <c r="G355" t="s">
@@ -17686,7 +17660,7 @@
       <c r="L355" t="s">
         <v>1235</v>
       </c>
-      <c r="N355" s="2">
+      <c r="N355" s="1">
         <v>46150</v>
       </c>
       <c r="Q355" t="b">
@@ -17709,7 +17683,7 @@
       <c r="E356" t="s">
         <v>1046</v>
       </c>
-      <c r="F356" s="2">
+      <c r="F356" s="1">
         <v>46142</v>
       </c>
       <c r="G356" t="s">
@@ -17724,7 +17698,7 @@
       <c r="L356" t="s">
         <v>1236</v>
       </c>
-      <c r="N356" s="2">
+      <c r="N356" s="1">
         <v>46176</v>
       </c>
       <c r="Q356" t="b">
@@ -17747,7 +17721,7 @@
       <c r="E357" t="s">
         <v>1047</v>
       </c>
-      <c r="F357" s="2">
+      <c r="F357" s="1">
         <v>46142</v>
       </c>
       <c r="G357" t="s">
@@ -17785,7 +17759,7 @@
       <c r="E358" t="s">
         <v>1048</v>
       </c>
-      <c r="F358" s="2">
+      <c r="F358" s="1">
         <v>46142</v>
       </c>
       <c r="G358" t="s">
@@ -17823,7 +17797,7 @@
       <c r="E359" t="s">
         <v>1049</v>
       </c>
-      <c r="F359" s="2">
+      <c r="F359" s="1">
         <v>46142</v>
       </c>
       <c r="G359" t="s">
@@ -17864,7 +17838,7 @@
       <c r="E360" t="s">
         <v>858</v>
       </c>
-      <c r="F360" s="2">
+      <c r="F360" s="1">
         <v>46142</v>
       </c>
       <c r="G360" t="s">
@@ -17902,7 +17876,7 @@
       <c r="E361" t="s">
         <v>870</v>
       </c>
-      <c r="F361" s="2">
+      <c r="F361" s="1">
         <v>46142</v>
       </c>
       <c r="G361" t="s">
@@ -17940,7 +17914,7 @@
       <c r="E362" t="s">
         <v>1050</v>
       </c>
-      <c r="F362" s="2">
+      <c r="F362" s="1">
         <v>46142</v>
       </c>
       <c r="G362" t="s">
@@ -17978,7 +17952,7 @@
       <c r="E363" t="s">
         <v>1051</v>
       </c>
-      <c r="F363" s="2">
+      <c r="F363" s="1">
         <v>46142</v>
       </c>
       <c r="G363" t="s">
@@ -18016,7 +17990,7 @@
       <c r="E364" t="s">
         <v>867</v>
       </c>
-      <c r="F364" s="2">
+      <c r="F364" s="1">
         <v>46142</v>
       </c>
       <c r="G364" t="s">
@@ -18054,7 +18028,7 @@
       <c r="E365" t="s">
         <v>1052</v>
       </c>
-      <c r="F365" s="2">
+      <c r="F365" s="1">
         <v>46142</v>
       </c>
       <c r="G365" t="s">
@@ -18092,7 +18066,7 @@
       <c r="E366" t="s">
         <v>1053</v>
       </c>
-      <c r="F366" s="2">
+      <c r="F366" s="1">
         <v>46148</v>
       </c>
       <c r="G366" t="s">
@@ -18130,7 +18104,7 @@
       <c r="E367" t="s">
         <v>1054</v>
       </c>
-      <c r="F367" s="2">
+      <c r="F367" s="1">
         <v>46148</v>
       </c>
       <c r="G367" t="s">
@@ -18168,7 +18142,7 @@
       <c r="E368" t="s">
         <v>1055</v>
       </c>
-      <c r="F368" s="2">
+      <c r="F368" s="1">
         <v>46148</v>
       </c>
       <c r="G368" t="s">
@@ -18206,7 +18180,7 @@
       <c r="E369" t="s">
         <v>1056</v>
       </c>
-      <c r="F369" s="2">
+      <c r="F369" s="1">
         <v>46148</v>
       </c>
       <c r="G369" t="s">
@@ -18244,7 +18218,7 @@
       <c r="E370" t="s">
         <v>1057</v>
       </c>
-      <c r="F370" s="2">
+      <c r="F370" s="1">
         <v>46148</v>
       </c>
       <c r="G370" t="s">
@@ -18282,7 +18256,7 @@
       <c r="E371" t="s">
         <v>1058</v>
       </c>
-      <c r="F371" s="2">
+      <c r="F371" s="1">
         <v>46148</v>
       </c>
       <c r="G371" t="s">
@@ -18303,7 +18277,7 @@
       <c r="L371" t="s">
         <v>1237</v>
       </c>
-      <c r="N371" s="2">
+      <c r="N371" s="1">
         <v>46164</v>
       </c>
       <c r="Q371" t="b">
@@ -18326,7 +18300,7 @@
       <c r="E372" t="s">
         <v>1059</v>
       </c>
-      <c r="F372" s="2">
+      <c r="F372" s="1">
         <v>46148</v>
       </c>
       <c r="G372" t="s">
@@ -18347,7 +18321,7 @@
       <c r="L372" t="s">
         <v>1224</v>
       </c>
-      <c r="N372" s="2">
+      <c r="N372" s="1">
         <v>46113</v>
       </c>
       <c r="P372" t="s">
@@ -18373,7 +18347,7 @@
       <c r="E373" t="s">
         <v>1060</v>
       </c>
-      <c r="F373" s="2">
+      <c r="F373" s="1">
         <v>46149</v>
       </c>
       <c r="G373" t="s">
@@ -18411,7 +18385,7 @@
       <c r="E374" t="s">
         <v>1061</v>
       </c>
-      <c r="F374" s="2">
+      <c r="F374" s="1">
         <v>46149</v>
       </c>
       <c r="G374" t="s">
@@ -18449,7 +18423,7 @@
       <c r="E375" t="s">
         <v>1062</v>
       </c>
-      <c r="F375" s="2">
+      <c r="F375" s="1">
         <v>46154</v>
       </c>
       <c r="G375" t="s">
@@ -18487,7 +18461,7 @@
       <c r="E376" t="s">
         <v>1063</v>
       </c>
-      <c r="F376" s="2">
+      <c r="F376" s="1">
         <v>46154</v>
       </c>
       <c r="G376" t="s">
@@ -18525,7 +18499,7 @@
       <c r="E377" t="s">
         <v>1064</v>
       </c>
-      <c r="F377" s="2">
+      <c r="F377" s="1">
         <v>46154</v>
       </c>
       <c r="G377" t="s">
@@ -18563,7 +18537,7 @@
       <c r="E378" t="s">
         <v>1065</v>
       </c>
-      <c r="F378" s="2">
+      <c r="F378" s="1">
         <v>46154</v>
       </c>
       <c r="G378" t="s">
@@ -18601,7 +18575,7 @@
       <c r="E379" t="s">
         <v>1066</v>
       </c>
-      <c r="F379" s="2">
+      <c r="F379" s="1">
         <v>46154</v>
       </c>
       <c r="G379" t="s">
@@ -18622,7 +18596,7 @@
       <c r="L379" t="s">
         <v>1238</v>
       </c>
-      <c r="N379" s="2">
+      <c r="N379" s="1">
         <v>46174</v>
       </c>
       <c r="Q379" t="b">
@@ -18645,7 +18619,7 @@
       <c r="E380" t="s">
         <v>1067</v>
       </c>
-      <c r="F380" s="2">
+      <c r="F380" s="1">
         <v>46154</v>
       </c>
       <c r="G380" t="s">
@@ -18683,7 +18657,7 @@
       <c r="E381" t="s">
         <v>1068</v>
       </c>
-      <c r="F381" s="2">
+      <c r="F381" s="1">
         <v>46154</v>
       </c>
       <c r="G381" t="s">
@@ -18721,7 +18695,7 @@
       <c r="E382" t="s">
         <v>1069</v>
       </c>
-      <c r="F382" s="2">
+      <c r="F382" s="1">
         <v>46154</v>
       </c>
       <c r="G382" t="s">
@@ -18759,7 +18733,7 @@
       <c r="E383" t="s">
         <v>1070</v>
       </c>
-      <c r="F383" s="2">
+      <c r="F383" s="1">
         <v>46154</v>
       </c>
       <c r="G383" t="s">
@@ -18797,7 +18771,7 @@
       <c r="E384" t="s">
         <v>1071</v>
       </c>
-      <c r="F384" s="2">
+      <c r="F384" s="1">
         <v>46164</v>
       </c>
       <c r="G384" t="s">
@@ -18835,7 +18809,7 @@
       <c r="E385" t="s">
         <v>1072</v>
       </c>
-      <c r="F385" s="2">
+      <c r="F385" s="1">
         <v>46164</v>
       </c>
       <c r="G385" t="s">
@@ -18873,7 +18847,7 @@
       <c r="E386" t="s">
         <v>1073</v>
       </c>
-      <c r="F386" s="2">
+      <c r="F386" s="1">
         <v>46171</v>
       </c>
       <c r="G386" t="s">
@@ -18911,7 +18885,7 @@
       <c r="E387" t="s">
         <v>1074</v>
       </c>
-      <c r="F387" s="2">
+      <c r="F387" s="1">
         <v>46171</v>
       </c>
       <c r="G387" t="s">
@@ -18949,7 +18923,7 @@
       <c r="E388" t="s">
         <v>760</v>
       </c>
-      <c r="F388" s="2">
+      <c r="F388" s="1">
         <v>46171</v>
       </c>
       <c r="G388" t="s">
@@ -18987,7 +18961,7 @@
       <c r="E389" t="s">
         <v>1075</v>
       </c>
-      <c r="F389" s="2">
+      <c r="F389" s="1">
         <v>46171</v>
       </c>
       <c r="G389" t="s">
@@ -19025,7 +18999,7 @@
       <c r="E390" t="s">
         <v>1076</v>
       </c>
-      <c r="F390" s="2">
+      <c r="F390" s="1">
         <v>46171</v>
       </c>
       <c r="G390" t="s">
@@ -19046,7 +19020,7 @@
       <c r="L390" t="s">
         <v>1239</v>
       </c>
-      <c r="N390" s="2">
+      <c r="N390" s="1">
         <v>46191</v>
       </c>
       <c r="Q390" t="b">
@@ -19069,7 +19043,7 @@
       <c r="E391" t="s">
         <v>1077</v>
       </c>
-      <c r="F391" s="2">
+      <c r="F391" s="1">
         <v>46171</v>
       </c>
       <c r="G391" t="s">
@@ -19107,7 +19081,7 @@
       <c r="E392" t="s">
         <v>1078</v>
       </c>
-      <c r="F392" s="2">
+      <c r="F392" s="1">
         <v>46171</v>
       </c>
       <c r="G392" t="s">
@@ -19122,7 +19096,7 @@
       <c r="L392" t="s">
         <v>1236</v>
       </c>
-      <c r="N392" s="2">
+      <c r="N392" s="1">
         <v>46176</v>
       </c>
       <c r="Q392" t="b">
@@ -19145,7 +19119,7 @@
       <c r="E393" t="s">
         <v>1079</v>
       </c>
-      <c r="F393" s="2">
+      <c r="F393" s="1">
         <v>46171</v>
       </c>
       <c r="G393" t="s">
@@ -19183,7 +19157,7 @@
       <c r="E394" t="s">
         <v>1080</v>
       </c>
-      <c r="F394" s="2">
+      <c r="F394" s="1">
         <v>46171</v>
       </c>
       <c r="G394" t="s">
@@ -19221,7 +19195,7 @@
       <c r="E395" t="s">
         <v>1081</v>
       </c>
-      <c r="F395" s="2">
+      <c r="F395" s="1">
         <v>46171</v>
       </c>
       <c r="G395" t="s">
@@ -19259,7 +19233,7 @@
       <c r="E396" t="s">
         <v>1082</v>
       </c>
-      <c r="F396" s="2">
+      <c r="F396" s="1">
         <v>46171</v>
       </c>
       <c r="G396" t="s">
@@ -19297,7 +19271,7 @@
       <c r="E397" t="s">
         <v>1083</v>
       </c>
-      <c r="F397" s="2">
+      <c r="F397" s="1">
         <v>46171</v>
       </c>
       <c r="G397" t="s">
@@ -19335,7 +19309,7 @@
       <c r="E398" t="s">
         <v>1084</v>
       </c>
-      <c r="F398" s="2">
+      <c r="F398" s="1">
         <v>46171</v>
       </c>
       <c r="G398" t="s">
@@ -19373,7 +19347,7 @@
       <c r="E399" t="s">
         <v>896</v>
       </c>
-      <c r="F399" s="2">
+      <c r="F399" s="1">
         <v>46163</v>
       </c>
       <c r="G399" t="s">
@@ -19388,7 +19362,7 @@
       <c r="L399" t="s">
         <v>1240</v>
       </c>
-      <c r="N399" s="2">
+      <c r="N399" s="1">
         <v>46171</v>
       </c>
       <c r="Q399" t="b">
@@ -19411,7 +19385,7 @@
       <c r="E400" t="s">
         <v>1085</v>
       </c>
-      <c r="F400" s="2">
+      <c r="F400" s="1">
         <v>46171</v>
       </c>
       <c r="G400" t="s">
@@ -19449,7 +19423,7 @@
       <c r="E401" t="s">
         <v>1086</v>
       </c>
-      <c r="F401" s="2">
+      <c r="F401" s="1">
         <v>46171</v>
       </c>
       <c r="G401" t="s">
@@ -19487,7 +19461,7 @@
       <c r="E402" t="s">
         <v>1087</v>
       </c>
-      <c r="F402" s="2">
+      <c r="F402" s="1">
         <v>46171</v>
       </c>
       <c r="G402" t="s">
@@ -19525,7 +19499,7 @@
       <c r="E403" t="s">
         <v>1088</v>
       </c>
-      <c r="F403" s="2">
+      <c r="F403" s="1">
         <v>46171</v>
       </c>
       <c r="G403" t="s">
@@ -19560,7 +19534,7 @@
       <c r="E404" t="s">
         <v>1089</v>
       </c>
-      <c r="F404" s="2">
+      <c r="F404" s="1">
         <v>46171</v>
       </c>
       <c r="G404" t="s">
@@ -19595,7 +19569,7 @@
       <c r="E405">
         <v>9599</v>
       </c>
-      <c r="F405" s="2">
+      <c r="F405" s="1">
         <v>46183</v>
       </c>
       <c r="G405" t="s">
@@ -19624,7 +19598,7 @@
       <c r="E406">
         <v>14251</v>
       </c>
-      <c r="F406" s="2">
+      <c r="F406" s="1">
         <v>46183</v>
       </c>
       <c r="G406" t="s">
@@ -19656,7 +19630,7 @@
       <c r="E407">
         <v>19945</v>
       </c>
-      <c r="F407" s="2">
+      <c r="F407" s="1">
         <v>46183</v>
       </c>
       <c r="G407" t="s">
@@ -19688,7 +19662,7 @@
       <c r="E408">
         <v>14396</v>
       </c>
-      <c r="F408" s="2">
+      <c r="F408" s="1">
         <v>46183</v>
       </c>
       <c r="G408" t="s">
@@ -19720,7 +19694,7 @@
       <c r="E409">
         <v>9920</v>
       </c>
-      <c r="F409" s="2">
+      <c r="F409" s="1">
         <v>46183</v>
       </c>
       <c r="G409" t="s">
@@ -19752,7 +19726,7 @@
       <c r="E410">
         <v>20528</v>
       </c>
-      <c r="F410" s="2">
+      <c r="F410" s="1">
         <v>46183</v>
       </c>
       <c r="G410" t="s">
@@ -19784,7 +19758,7 @@
       <c r="E411" t="s">
         <v>1090</v>
       </c>
-      <c r="F411" s="2">
+      <c r="F411" s="1">
         <v>46188</v>
       </c>
       <c r="G411" t="s">
@@ -19816,7 +19790,7 @@
       <c r="E412" t="s">
         <v>1091</v>
       </c>
-      <c r="F412" s="2">
+      <c r="F412" s="1">
         <v>46188</v>
       </c>
       <c r="G412" t="s">
@@ -19848,7 +19822,7 @@
       <c r="E413" t="s">
         <v>1092</v>
       </c>
-      <c r="F413" s="2">
+      <c r="F413" s="1">
         <v>46188</v>
       </c>
       <c r="G413" t="s">
@@ -19880,7 +19854,7 @@
       <c r="E414" t="s">
         <v>1093</v>
       </c>
-      <c r="F414" s="2">
+      <c r="F414" s="1">
         <v>46188</v>
       </c>
       <c r="G414" t="s">
@@ -19912,7 +19886,7 @@
       <c r="E415" t="s">
         <v>969</v>
       </c>
-      <c r="F415" s="2">
+      <c r="F415" s="1">
         <v>46188</v>
       </c>
       <c r="G415" t="s">
@@ -19944,7 +19918,7 @@
       <c r="E416">
         <v>5844</v>
       </c>
-      <c r="F416" s="2">
+      <c r="F416" s="1">
         <v>46188</v>
       </c>
       <c r="G416" t="s">
@@ -19976,7 +19950,7 @@
       <c r="E417" t="s">
         <v>1094</v>
       </c>
-      <c r="F417" s="2">
+      <c r="F417" s="1">
         <v>46188</v>
       </c>
       <c r="G417" t="s">
@@ -20008,7 +19982,7 @@
       <c r="E418" t="s">
         <v>1095</v>
       </c>
-      <c r="F418" s="2">
+      <c r="F418" s="1">
         <v>46188</v>
       </c>
       <c r="G418" t="s">
@@ -20040,7 +20014,7 @@
       <c r="E419" t="s">
         <v>1096</v>
       </c>
-      <c r="F419" s="2">
+      <c r="F419" s="1">
         <v>46188</v>
       </c>
       <c r="G419" t="s">
@@ -20072,7 +20046,7 @@
       <c r="E420">
         <v>580</v>
       </c>
-      <c r="F420" s="2">
+      <c r="F420" s="1">
         <v>46188</v>
       </c>
       <c r="G420" t="s">
@@ -20104,7 +20078,7 @@
       <c r="E421" t="s">
         <v>1097</v>
       </c>
-      <c r="F421" s="2">
+      <c r="F421" s="1">
         <v>46188</v>
       </c>
       <c r="G421" t="s">
@@ -20136,7 +20110,7 @@
       <c r="E422" t="s">
         <v>1098</v>
       </c>
-      <c r="F422" s="2">
+      <c r="F422" s="1">
         <v>46188</v>
       </c>
       <c r="G422" t="s">
@@ -20168,7 +20142,7 @@
       <c r="E423" t="s">
         <v>1099</v>
       </c>
-      <c r="F423" s="2">
+      <c r="F423" s="1">
         <v>46188</v>
       </c>
       <c r="G423" t="s">
@@ -20200,7 +20174,7 @@
       <c r="E424" t="s">
         <v>1100</v>
       </c>
-      <c r="F424" s="2">
+      <c r="F424" s="1">
         <v>46188</v>
       </c>
       <c r="G424" t="s">
@@ -20232,7 +20206,7 @@
       <c r="E425" t="s">
         <v>1101</v>
       </c>
-      <c r="F425" s="2">
+      <c r="F425" s="1">
         <v>46188</v>
       </c>
       <c r="G425" t="s">
@@ -20264,7 +20238,7 @@
       <c r="E426" t="s">
         <v>1102</v>
       </c>
-      <c r="F426" s="2">
+      <c r="F426" s="1">
         <v>46188</v>
       </c>
       <c r="G426" t="s">
@@ -20296,7 +20270,7 @@
       <c r="E427">
         <v>6309</v>
       </c>
-      <c r="F427" s="2">
+      <c r="F427" s="1">
         <v>46188</v>
       </c>
       <c r="G427" t="s">
@@ -20328,7 +20302,7 @@
       <c r="E428">
         <v>504011190625165</v>
       </c>
-      <c r="F428" s="2">
+      <c r="F428" s="1">
         <v>46188</v>
       </c>
       <c r="G428" t="s">
@@ -20360,7 +20334,7 @@
       <c r="E429">
         <v>504011190625185</v>
       </c>
-      <c r="F429" s="2">
+      <c r="F429" s="1">
         <v>46188</v>
       </c>
       <c r="G429" t="s">
@@ -20392,7 +20366,7 @@
       <c r="E430" t="s">
         <v>1103</v>
       </c>
-      <c r="F430" s="2">
+      <c r="F430" s="1">
         <v>46188</v>
       </c>
       <c r="G430" t="s">
@@ -20424,7 +20398,7 @@
       <c r="E431" t="s">
         <v>1104</v>
       </c>
-      <c r="F431" s="2">
+      <c r="F431" s="1">
         <v>46188</v>
       </c>
       <c r="G431" t="s">
@@ -20456,7 +20430,7 @@
       <c r="E432" t="s">
         <v>1105</v>
       </c>
-      <c r="F432" s="2">
+      <c r="F432" s="1">
         <v>46188</v>
       </c>
       <c r="G432" t="s">
@@ -20488,7 +20462,7 @@
       <c r="E433" t="s">
         <v>1106</v>
       </c>
-      <c r="F433" s="2">
+      <c r="F433" s="1">
         <v>46188</v>
       </c>
       <c r="G433" t="s">
@@ -20520,7 +20494,7 @@
       <c r="E434">
         <v>328</v>
       </c>
-      <c r="F434" s="2">
+      <c r="F434" s="1">
         <v>46188</v>
       </c>
       <c r="G434" t="s">
@@ -20552,7 +20526,7 @@
       <c r="E435">
         <v>277</v>
       </c>
-      <c r="F435" s="2">
+      <c r="F435" s="1">
         <v>46188</v>
       </c>
       <c r="G435" t="s">
@@ -20584,7 +20558,7 @@
       <c r="E436">
         <v>477</v>
       </c>
-      <c r="F436" s="2">
+      <c r="F436" s="1">
         <v>46188</v>
       </c>
       <c r="G436" t="s">
@@ -20616,7 +20590,7 @@
       <c r="E437">
         <v>11</v>
       </c>
-      <c r="F437" s="2">
+      <c r="F437" s="1">
         <v>46188</v>
       </c>
       <c r="G437" t="s">
@@ -20648,7 +20622,7 @@
       <c r="E438" t="s">
         <v>1107</v>
       </c>
-      <c r="F438" s="2">
+      <c r="F438" s="1">
         <v>46188</v>
       </c>
       <c r="G438" t="s">
@@ -20680,7 +20654,7 @@
       <c r="E439" t="s">
         <v>1108</v>
       </c>
-      <c r="F439" s="2">
+      <c r="F439" s="1">
         <v>46196</v>
       </c>
       <c r="G439" t="s">
@@ -20712,7 +20686,7 @@
       <c r="E440" t="s">
         <v>1109</v>
       </c>
-      <c r="F440" s="2">
+      <c r="F440" s="1">
         <v>46196</v>
       </c>
       <c r="G440" t="s">
@@ -20744,7 +20718,7 @@
       <c r="E441">
         <v>86815651</v>
       </c>
-      <c r="F441" s="2">
+      <c r="F441" s="1">
         <v>46203</v>
       </c>
       <c r="G441" t="s">
@@ -20776,7 +20750,7 @@
       <c r="E442">
         <v>86817554</v>
       </c>
-      <c r="F442" s="2">
+      <c r="F442" s="1">
         <v>46203</v>
       </c>
       <c r="G442" t="s">
@@ -20808,7 +20782,7 @@
       <c r="E443" t="s">
         <v>1110</v>
       </c>
-      <c r="F443" s="2">
+      <c r="F443" s="1">
         <v>46205</v>
       </c>
       <c r="G443" t="s">
@@ -20840,7 +20814,7 @@
       <c r="E444" t="s">
         <v>1111</v>
       </c>
-      <c r="F444" s="2">
+      <c r="F444" s="1">
         <v>46205</v>
       </c>
       <c r="G444" t="s">
@@ -20872,7 +20846,7 @@
       <c r="E445">
         <v>4134</v>
       </c>
-      <c r="F445" s="2">
+      <c r="F445" s="1">
         <v>46205</v>
       </c>
       <c r="G445" t="s">
@@ -20904,7 +20878,7 @@
       <c r="E446">
         <v>22006508</v>
       </c>
-      <c r="F446" s="2">
+      <c r="F446" s="1">
         <v>46211</v>
       </c>
       <c r="G446" t="s">
@@ -20936,7 +20910,7 @@
       <c r="E447">
         <v>22005733</v>
       </c>
-      <c r="F447" s="2">
+      <c r="F447" s="1">
         <v>46211</v>
       </c>
       <c r="G447" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis (28/07/2026 05:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4253,7 +4253,7 @@
         <v>1140</v>
       </c>
       <c r="I2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="K2" t="s">
         <v>1143</v>
@@ -4291,7 +4291,7 @@
         <v>1140</v>
       </c>
       <c r="I3">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="K3" t="s">
         <v>1144</v>
@@ -4329,7 +4329,7 @@
         <v>1140</v>
       </c>
       <c r="I4">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="K4" t="s">
         <v>1144</v>
@@ -4367,7 +4367,7 @@
         <v>1140</v>
       </c>
       <c r="I5">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4411,7 +4411,7 @@
         <v>1140</v>
       </c>
       <c r="I6">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4455,7 +4455,7 @@
         <v>1140</v>
       </c>
       <c r="I7">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4531,7 +4531,7 @@
         <v>1140</v>
       </c>
       <c r="I9">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4578,7 +4578,7 @@
         <v>1140</v>
       </c>
       <c r="I10">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4625,7 +4625,7 @@
         <v>1140</v>
       </c>
       <c r="I11">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4672,7 +4672,7 @@
         <v>1140</v>
       </c>
       <c r="I12">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -4751,7 +4751,7 @@
         <v>1140</v>
       </c>
       <c r="I14">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -4795,7 +4795,7 @@
         <v>1140</v>
       </c>
       <c r="I15">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K15" t="s">
         <v>1146</v>
@@ -4833,7 +4833,7 @@
         <v>1140</v>
       </c>
       <c r="I16">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K16" t="s">
         <v>1143</v>
@@ -4871,7 +4871,7 @@
         <v>1140</v>
       </c>
       <c r="I17">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -4915,7 +4915,7 @@
         <v>1140</v>
       </c>
       <c r="I18">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -4994,7 +4994,7 @@
         <v>1140</v>
       </c>
       <c r="I20">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5073,7 +5073,7 @@
         <v>1140</v>
       </c>
       <c r="I22">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K22" t="s">
         <v>1147</v>
@@ -5111,7 +5111,7 @@
         <v>1140</v>
       </c>
       <c r="I23">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5234,7 +5234,7 @@
         <v>1140</v>
       </c>
       <c r="I26">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5281,7 +5281,7 @@
         <v>1140</v>
       </c>
       <c r="I27">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K27" t="s">
         <v>1147</v>
@@ -5386,7 +5386,7 @@
         <v>1140</v>
       </c>
       <c r="I30">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5468,7 +5468,7 @@
         <v>1140</v>
       </c>
       <c r="I32">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K32" t="s">
         <v>1143</v>
@@ -5710,7 +5710,7 @@
         <v>1140</v>
       </c>
       <c r="I39">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K39" t="s">
         <v>1148</v>
@@ -5745,7 +5745,7 @@
         <v>1140</v>
       </c>
       <c r="I40">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K40" t="s">
         <v>1146</v>
@@ -5894,7 +5894,7 @@
         <v>1140</v>
       </c>
       <c r="I44">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -5941,7 +5941,7 @@
         <v>1140</v>
       </c>
       <c r="I45">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -5988,7 +5988,7 @@
         <v>1140</v>
       </c>
       <c r="I46">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K46" t="s">
         <v>1147</v>
@@ -6026,7 +6026,7 @@
         <v>1140</v>
       </c>
       <c r="I47">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6073,7 +6073,7 @@
         <v>1140</v>
       </c>
       <c r="I48">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K48" t="s">
         <v>1147</v>
@@ -6143,7 +6143,7 @@
         <v>1140</v>
       </c>
       <c r="I50">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K50" t="s">
         <v>1147</v>
@@ -6219,7 +6219,7 @@
         <v>1140</v>
       </c>
       <c r="I52">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K52" t="s">
         <v>1143</v>
@@ -6257,7 +6257,7 @@
         <v>1140</v>
       </c>
       <c r="I53">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K53" t="s">
         <v>1144</v>
@@ -6295,7 +6295,7 @@
         <v>1140</v>
       </c>
       <c r="I54">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K54" t="s">
         <v>1144</v>
@@ -6403,7 +6403,7 @@
         <v>1140</v>
       </c>
       <c r="I57">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K57" t="s">
         <v>1147</v>
@@ -6607,7 +6607,7 @@
         <v>1140</v>
       </c>
       <c r="I63">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6654,7 +6654,7 @@
         <v>1140</v>
       </c>
       <c r="I64">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -6885,7 +6885,7 @@
         <v>1140</v>
       </c>
       <c r="I70">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K70" t="s">
         <v>1144</v>
@@ -6923,7 +6923,7 @@
         <v>1140</v>
       </c>
       <c r="I71">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K71" t="s">
         <v>1150</v>
@@ -6993,7 +6993,7 @@
         <v>1140</v>
       </c>
       <c r="I73">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K73" t="s">
         <v>1143</v>
@@ -7069,7 +7069,7 @@
         <v>1140</v>
       </c>
       <c r="I75">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K75" t="s">
         <v>1144</v>
@@ -7107,7 +7107,7 @@
         <v>1140</v>
       </c>
       <c r="I76">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K76" t="s">
         <v>1150</v>
@@ -7215,7 +7215,7 @@
         <v>1140</v>
       </c>
       <c r="I79">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K79" t="s">
         <v>1150</v>
@@ -7250,7 +7250,7 @@
         <v>1140</v>
       </c>
       <c r="I80">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K80" t="s">
         <v>1144</v>
@@ -7326,7 +7326,7 @@
         <v>1140</v>
       </c>
       <c r="I82">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K82" t="s">
         <v>1147</v>
@@ -7399,7 +7399,7 @@
         <v>1140</v>
       </c>
       <c r="I84">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7446,7 +7446,7 @@
         <v>1140</v>
       </c>
       <c r="I85">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K85" t="s">
         <v>1144</v>
@@ -7484,7 +7484,7 @@
         <v>1140</v>
       </c>
       <c r="I86">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K86" t="s">
         <v>1144</v>
@@ -7522,7 +7522,7 @@
         <v>1140</v>
       </c>
       <c r="I87">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7639,7 +7639,7 @@
         <v>1140</v>
       </c>
       <c r="I90">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K90" t="s">
         <v>1117</v>
@@ -7680,7 +7680,7 @@
         <v>1140</v>
       </c>
       <c r="I91">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K91" t="s">
         <v>1146</v>
@@ -7747,7 +7747,7 @@
         <v>1140</v>
       </c>
       <c r="I93">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K93" t="s">
         <v>1146</v>
@@ -7785,7 +7785,7 @@
         <v>1140</v>
       </c>
       <c r="I94">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K94" t="s">
         <v>1147</v>
@@ -7823,7 +7823,7 @@
         <v>1140</v>
       </c>
       <c r="I95">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K95" t="s">
         <v>1146</v>
@@ -7861,7 +7861,7 @@
         <v>1140</v>
       </c>
       <c r="I96">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -7908,7 +7908,7 @@
         <v>1140</v>
       </c>
       <c r="I97">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K97" t="s">
         <v>1117</v>
@@ -7949,7 +7949,7 @@
         <v>1140</v>
       </c>
       <c r="I98">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K98" t="s">
         <v>1147</v>
@@ -8016,7 +8016,7 @@
         <v>1140</v>
       </c>
       <c r="I100">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K100" t="s">
         <v>1146</v>
@@ -8144,7 +8144,7 @@
         <v>1140</v>
       </c>
       <c r="I104">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K104" t="s">
         <v>1146</v>
@@ -8182,7 +8182,7 @@
         <v>1140</v>
       </c>
       <c r="I105">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K105" t="s">
         <v>1146</v>
@@ -8220,7 +8220,7 @@
         <v>1140</v>
       </c>
       <c r="I106">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8264,7 +8264,7 @@
         <v>1140</v>
       </c>
       <c r="I107">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8308,7 +8308,7 @@
         <v>1140</v>
       </c>
       <c r="I108">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K108" t="s">
         <v>1144</v>
@@ -8346,7 +8346,7 @@
         <v>1140</v>
       </c>
       <c r="I109">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K109" t="s">
         <v>1144</v>
@@ -8562,7 +8562,7 @@
         <v>1140</v>
       </c>
       <c r="I115">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K115" t="s">
         <v>1144</v>
@@ -8600,7 +8600,7 @@
         <v>1140</v>
       </c>
       <c r="I116">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K116" t="s">
         <v>1144</v>
@@ -8638,7 +8638,7 @@
         <v>1140</v>
       </c>
       <c r="I117">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K117" t="s">
         <v>1144</v>
@@ -8676,7 +8676,7 @@
         <v>1140</v>
       </c>
       <c r="I118">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K118" t="s">
         <v>1144</v>
@@ -8714,7 +8714,7 @@
         <v>1140</v>
       </c>
       <c r="I119">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K119" t="s">
         <v>1144</v>
@@ -8752,7 +8752,7 @@
         <v>1140</v>
       </c>
       <c r="I120">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K120" t="s">
         <v>1144</v>
@@ -8790,7 +8790,7 @@
         <v>1140</v>
       </c>
       <c r="I121">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -8837,7 +8837,7 @@
         <v>1140</v>
       </c>
       <c r="I122">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="K122" t="s">
         <v>1144</v>
@@ -8904,7 +8904,7 @@
         <v>1140</v>
       </c>
       <c r="I124">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K124" t="s">
         <v>1144</v>
@@ -8942,7 +8942,7 @@
         <v>1140</v>
       </c>
       <c r="I125">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K125" t="s">
         <v>1150</v>
@@ -9047,7 +9047,7 @@
         <v>1140</v>
       </c>
       <c r="I128">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K128" t="s">
         <v>1144</v>
@@ -9085,7 +9085,7 @@
         <v>1140</v>
       </c>
       <c r="I129">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K129" t="s">
         <v>1143</v>
@@ -9123,7 +9123,7 @@
         <v>1140</v>
       </c>
       <c r="I130">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9205,7 +9205,7 @@
         <v>1140</v>
       </c>
       <c r="I132">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9281,7 +9281,7 @@
         <v>1140</v>
       </c>
       <c r="I134">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K134" t="s">
         <v>1143</v>
@@ -9412,7 +9412,7 @@
         <v>1140</v>
       </c>
       <c r="I138">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K138" t="s">
         <v>1144</v>
@@ -9741,7 +9741,7 @@
         <v>1140</v>
       </c>
       <c r="I148">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K148" t="s">
         <v>1144</v>
@@ -9779,7 +9779,7 @@
         <v>1140</v>
       </c>
       <c r="I149">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K149" t="s">
         <v>1150</v>
@@ -9814,7 +9814,7 @@
         <v>1140</v>
       </c>
       <c r="I150">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -9899,7 +9899,7 @@
         <v>1140</v>
       </c>
       <c r="I152">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -9943,7 +9943,7 @@
         <v>1140</v>
       </c>
       <c r="I153">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K153" t="s">
         <v>1144</v>
@@ -10016,7 +10016,7 @@
         <v>1140</v>
       </c>
       <c r="I155">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K155" t="s">
         <v>1150</v>
@@ -10051,7 +10051,7 @@
         <v>1140</v>
       </c>
       <c r="I156">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K156" t="s">
         <v>1144</v>
@@ -10089,7 +10089,7 @@
         <v>1140</v>
       </c>
       <c r="I157">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K157" t="s">
         <v>1146</v>
@@ -10127,7 +10127,7 @@
         <v>1140</v>
       </c>
       <c r="I158">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10171,7 +10171,7 @@
         <v>1140</v>
       </c>
       <c r="I159">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K159" t="s">
         <v>1144</v>
@@ -10209,7 +10209,7 @@
         <v>1140</v>
       </c>
       <c r="I160">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K160" t="s">
         <v>1144</v>
@@ -10247,7 +10247,7 @@
         <v>1140</v>
       </c>
       <c r="I161">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10294,7 +10294,7 @@
         <v>1140</v>
       </c>
       <c r="I162">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10338,7 +10338,7 @@
         <v>1140</v>
       </c>
       <c r="I163">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10382,7 +10382,7 @@
         <v>1142</v>
       </c>
       <c r="I164">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K164" t="s">
         <v>1151</v>
@@ -10417,7 +10417,7 @@
         <v>1140</v>
       </c>
       <c r="I165">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K165" t="s">
         <v>1144</v>
@@ -10525,7 +10525,7 @@
         <v>1140</v>
       </c>
       <c r="I168">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K168" t="s">
         <v>1147</v>
@@ -10566,7 +10566,7 @@
         <v>1140</v>
       </c>
       <c r="I169">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10648,7 +10648,7 @@
         <v>1140</v>
       </c>
       <c r="I171">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K171" t="s">
         <v>1144</v>
@@ -10794,7 +10794,7 @@
         <v>1140</v>
       </c>
       <c r="I175">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -10841,7 +10841,7 @@
         <v>1140</v>
       </c>
       <c r="I176">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K176" t="s">
         <v>1144</v>
@@ -10879,7 +10879,7 @@
         <v>1140</v>
       </c>
       <c r="I177">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -10926,7 +10926,7 @@
         <v>1140</v>
       </c>
       <c r="I178">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K178" t="s">
         <v>1143</v>
@@ -10993,7 +10993,7 @@
         <v>1140</v>
       </c>
       <c r="I180">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K180" t="s">
         <v>1143</v>
@@ -11098,7 +11098,7 @@
         <v>1140</v>
       </c>
       <c r="I183">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K183" t="s">
         <v>1144</v>
@@ -11133,7 +11133,7 @@
         <v>1140</v>
       </c>
       <c r="I184">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K184" t="s">
         <v>1150</v>
@@ -11168,7 +11168,7 @@
         <v>1140</v>
       </c>
       <c r="I185">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K185" t="s">
         <v>1144</v>
@@ -11206,7 +11206,7 @@
         <v>1140</v>
       </c>
       <c r="I186">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K186" t="s">
         <v>1144</v>
@@ -11244,7 +11244,7 @@
         <v>1140</v>
       </c>
       <c r="I187">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11291,7 +11291,7 @@
         <v>1140</v>
       </c>
       <c r="I188">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11338,7 +11338,7 @@
         <v>1140</v>
       </c>
       <c r="I189">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11382,7 +11382,7 @@
         <v>1140</v>
       </c>
       <c r="I190">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K190" t="s">
         <v>1146</v>
@@ -11420,7 +11420,7 @@
         <v>1140</v>
       </c>
       <c r="I191">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11464,7 +11464,7 @@
         <v>1140</v>
       </c>
       <c r="I192">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K192" t="s">
         <v>1144</v>
@@ -11502,7 +11502,7 @@
         <v>1140</v>
       </c>
       <c r="I193">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K193" t="s">
         <v>1149</v>
@@ -11572,7 +11572,7 @@
         <v>1140</v>
       </c>
       <c r="I195">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K195" t="s">
         <v>1146</v>
@@ -11706,7 +11706,7 @@
         <v>1140</v>
       </c>
       <c r="I199">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -11750,7 +11750,7 @@
         <v>1140</v>
       </c>
       <c r="I200">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K200" t="s">
         <v>1146</v>
@@ -11788,7 +11788,7 @@
         <v>1140</v>
       </c>
       <c r="I201">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K201" t="s">
         <v>1144</v>
@@ -11826,7 +11826,7 @@
         <v>1140</v>
       </c>
       <c r="I202">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K202" t="s">
         <v>1144</v>
@@ -11864,7 +11864,7 @@
         <v>1140</v>
       </c>
       <c r="I203">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K203" t="s">
         <v>1144</v>
@@ -11902,7 +11902,7 @@
         <v>1140</v>
       </c>
       <c r="I204">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K204" t="s">
         <v>1143</v>
@@ -11940,7 +11940,7 @@
         <v>1140</v>
       </c>
       <c r="I205">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K205" t="s">
         <v>1143</v>
@@ -12013,7 +12013,7 @@
         <v>1140</v>
       </c>
       <c r="I207">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12057,7 +12057,7 @@
         <v>1140</v>
       </c>
       <c r="I208">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12101,7 +12101,7 @@
         <v>1140</v>
       </c>
       <c r="I209">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12145,7 +12145,7 @@
         <v>1140</v>
       </c>
       <c r="I210">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K210" t="s">
         <v>1147</v>
@@ -12253,7 +12253,7 @@
         <v>1140</v>
       </c>
       <c r="I213">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K213" t="s">
         <v>1144</v>
@@ -12291,7 +12291,7 @@
         <v>1140</v>
       </c>
       <c r="I214">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12338,7 +12338,7 @@
         <v>1140</v>
       </c>
       <c r="I215">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K215" t="s">
         <v>1144</v>
@@ -12405,7 +12405,7 @@
         <v>1140</v>
       </c>
       <c r="I217">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12449,7 +12449,7 @@
         <v>1140</v>
       </c>
       <c r="I218">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K218" t="s">
         <v>1146</v>
@@ -12487,7 +12487,7 @@
         <v>1140</v>
       </c>
       <c r="I219">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K219" t="s">
         <v>1146</v>
@@ -12525,7 +12525,7 @@
         <v>1140</v>
       </c>
       <c r="I220">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K220" t="s">
         <v>1146</v>
@@ -12601,7 +12601,7 @@
         <v>1140</v>
       </c>
       <c r="I222">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K222" t="s">
         <v>1144</v>
@@ -12639,7 +12639,7 @@
         <v>1140</v>
       </c>
       <c r="I223">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K223" t="s">
         <v>1144</v>
@@ -12677,7 +12677,7 @@
         <v>1140</v>
       </c>
       <c r="I224">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K224" t="s">
         <v>1144</v>
@@ -12715,7 +12715,7 @@
         <v>1140</v>
       </c>
       <c r="I225">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K225" t="s">
         <v>1144</v>
@@ -12753,7 +12753,7 @@
         <v>1140</v>
       </c>
       <c r="I226">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K226" t="s">
         <v>1144</v>
@@ -12791,7 +12791,7 @@
         <v>1140</v>
       </c>
       <c r="I227">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K227" t="s">
         <v>1144</v>
@@ -12829,7 +12829,7 @@
         <v>1140</v>
       </c>
       <c r="I228">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K228" t="s">
         <v>1144</v>
@@ -12902,7 +12902,7 @@
         <v>1140</v>
       </c>
       <c r="I230">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K230" t="s">
         <v>1147</v>
@@ -12940,7 +12940,7 @@
         <v>1140</v>
       </c>
       <c r="I231">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13054,7 +13054,7 @@
         <v>1140</v>
       </c>
       <c r="I234">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13101,7 +13101,7 @@
         <v>1140</v>
       </c>
       <c r="I235">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13148,7 +13148,7 @@
         <v>1140</v>
       </c>
       <c r="I236">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13192,7 +13192,7 @@
         <v>1140</v>
       </c>
       <c r="I237">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K237" t="s">
         <v>1144</v>
@@ -13259,7 +13259,7 @@
         <v>1140</v>
       </c>
       <c r="I239">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K239" t="s">
         <v>1117</v>
@@ -13370,7 +13370,7 @@
         <v>1140</v>
       </c>
       <c r="I242">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K242" t="s">
         <v>1143</v>
@@ -13440,7 +13440,7 @@
         <v>1140</v>
       </c>
       <c r="I244">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K244" t="s">
         <v>1146</v>
@@ -13478,7 +13478,7 @@
         <v>1140</v>
       </c>
       <c r="I245">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K245" t="s">
         <v>1146</v>
@@ -13516,7 +13516,7 @@
         <v>1140</v>
       </c>
       <c r="I246">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13621,7 +13621,7 @@
         <v>1140</v>
       </c>
       <c r="I249">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K249" t="s">
         <v>1144</v>
@@ -13659,7 +13659,7 @@
         <v>1140</v>
       </c>
       <c r="I250">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K250" t="s">
         <v>1146</v>
@@ -13767,7 +13767,7 @@
         <v>1140</v>
       </c>
       <c r="I253">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K253" t="s">
         <v>1147</v>
@@ -13805,7 +13805,7 @@
         <v>1140</v>
       </c>
       <c r="I254">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K254" t="s">
         <v>1147</v>
@@ -13843,7 +13843,7 @@
         <v>1140</v>
       </c>
       <c r="I255">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K255" t="s">
         <v>1146</v>
@@ -13881,7 +13881,7 @@
         <v>1140</v>
       </c>
       <c r="I256">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K256" t="s">
         <v>1144</v>
@@ -13980,7 +13980,7 @@
         <v>1140</v>
       </c>
       <c r="I259">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K259" t="s">
         <v>1146</v>
@@ -14018,7 +14018,7 @@
         <v>1140</v>
       </c>
       <c r="I260">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K260" t="s">
         <v>1146</v>
@@ -14056,7 +14056,7 @@
         <v>1140</v>
       </c>
       <c r="I261">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K261" t="s">
         <v>1147</v>
@@ -14094,7 +14094,7 @@
         <v>1140</v>
       </c>
       <c r="I262">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14179,7 +14179,7 @@
         <v>1140</v>
       </c>
       <c r="I264">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K264" t="s">
         <v>1147</v>
@@ -14217,7 +14217,7 @@
         <v>1140</v>
       </c>
       <c r="I265">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K265" t="s">
         <v>1147</v>
@@ -14255,7 +14255,7 @@
         <v>1140</v>
       </c>
       <c r="I266">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K266" t="s">
         <v>1146</v>
@@ -14293,7 +14293,7 @@
         <v>1140</v>
       </c>
       <c r="I267">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K267" t="s">
         <v>1147</v>
@@ -14331,7 +14331,7 @@
         <v>1140</v>
       </c>
       <c r="I268">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K268" t="s">
         <v>1144</v>
@@ -14366,7 +14366,7 @@
         <v>1140</v>
       </c>
       <c r="I269">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K269" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1140</v>
       </c>
       <c r="I270">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K270" t="s">
         <v>1147</v>
@@ -14442,7 +14442,7 @@
         <v>1140</v>
       </c>
       <c r="I271">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K271" t="s">
         <v>1147</v>
@@ -14480,7 +14480,7 @@
         <v>1140</v>
       </c>
       <c r="I272">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14562,7 +14562,7 @@
         <v>1140</v>
       </c>
       <c r="I274">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K274" t="s">
         <v>1144</v>
@@ -14635,7 +14635,7 @@
         <v>1140</v>
       </c>
       <c r="I276">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K276" t="s">
         <v>1148</v>
@@ -14673,7 +14673,7 @@
         <v>1140</v>
       </c>
       <c r="I277">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K277" t="s">
         <v>1144</v>
@@ -14711,7 +14711,7 @@
         <v>1140</v>
       </c>
       <c r="I278">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K278" t="s">
         <v>1147</v>
@@ -14749,7 +14749,7 @@
         <v>1140</v>
       </c>
       <c r="I279">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K279" t="s">
         <v>1146</v>
@@ -14790,7 +14790,7 @@
         <v>1140</v>
       </c>
       <c r="I280">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K280" t="s">
         <v>1144</v>
@@ -14828,7 +14828,7 @@
         <v>1140</v>
       </c>
       <c r="I281">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K281" t="s">
         <v>1144</v>
@@ -14866,7 +14866,7 @@
         <v>1140</v>
       </c>
       <c r="I282">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K282" t="s">
         <v>1144</v>
@@ -15073,7 +15073,7 @@
         <v>1140</v>
       </c>
       <c r="I288">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K288" t="s">
         <v>1147</v>
@@ -15140,7 +15140,7 @@
         <v>1140</v>
       </c>
       <c r="I290">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15181,7 +15181,7 @@
         <v>1140</v>
       </c>
       <c r="I291">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K291" t="s">
         <v>1146</v>
@@ -15219,7 +15219,7 @@
         <v>1140</v>
       </c>
       <c r="I292">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K292" t="s">
         <v>1147</v>
@@ -15257,7 +15257,7 @@
         <v>1140</v>
       </c>
       <c r="I293">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K293" t="s">
         <v>1148</v>
@@ -15295,7 +15295,7 @@
         <v>1140</v>
       </c>
       <c r="I294">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K294" t="s">
         <v>1150</v>
@@ -15330,7 +15330,7 @@
         <v>1140</v>
       </c>
       <c r="I295">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K295" t="s">
         <v>1150</v>
@@ -15365,7 +15365,7 @@
         <v>1140</v>
       </c>
       <c r="I296">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K296" t="s">
         <v>1150</v>
@@ -15435,7 +15435,7 @@
         <v>1140</v>
       </c>
       <c r="I298">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K298" t="s">
         <v>1144</v>
@@ -15473,7 +15473,7 @@
         <v>1140</v>
       </c>
       <c r="I299">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K299" t="s">
         <v>1147</v>
@@ -15511,7 +15511,7 @@
         <v>1140</v>
       </c>
       <c r="I300">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K300" t="s">
         <v>1147</v>
@@ -15549,7 +15549,7 @@
         <v>1140</v>
       </c>
       <c r="I301">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K301" t="s">
         <v>1147</v>
@@ -15587,7 +15587,7 @@
         <v>1140</v>
       </c>
       <c r="I302">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K302" t="s">
         <v>1147</v>
@@ -15625,7 +15625,7 @@
         <v>1140</v>
       </c>
       <c r="I303">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K303" t="s">
         <v>1144</v>
@@ -15663,7 +15663,7 @@
         <v>1140</v>
       </c>
       <c r="I304">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K304" t="s">
         <v>1147</v>
@@ -15701,7 +15701,7 @@
         <v>1140</v>
       </c>
       <c r="I305">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -15745,7 +15745,7 @@
         <v>1140</v>
       </c>
       <c r="I306">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -15789,7 +15789,7 @@
         <v>1140</v>
       </c>
       <c r="I307">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K307" t="s">
         <v>1143</v>
@@ -15827,7 +15827,7 @@
         <v>1140</v>
       </c>
       <c r="I308">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K308" t="s">
         <v>1143</v>
@@ -15865,7 +15865,7 @@
         <v>1140</v>
       </c>
       <c r="I309">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K309" t="s">
         <v>1143</v>
@@ -15903,7 +15903,7 @@
         <v>1140</v>
       </c>
       <c r="I310">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K310" t="s">
         <v>1144</v>
@@ -15941,7 +15941,7 @@
         <v>1140</v>
       </c>
       <c r="I311">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K311" t="s">
         <v>1143</v>
@@ -15979,7 +15979,7 @@
         <v>1140</v>
       </c>
       <c r="I312">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K312" t="s">
         <v>1144</v>
@@ -16052,7 +16052,7 @@
         <v>1140</v>
       </c>
       <c r="I314">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K314" t="s">
         <v>1144</v>
@@ -16090,7 +16090,7 @@
         <v>1140</v>
       </c>
       <c r="I315">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K315" t="s">
         <v>1144</v>
@@ -16128,7 +16128,7 @@
         <v>1140</v>
       </c>
       <c r="I316">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K316" t="s">
         <v>1144</v>
@@ -16166,7 +16166,7 @@
         <v>1140</v>
       </c>
       <c r="I317">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K317" t="s">
         <v>1144</v>
@@ -16277,7 +16277,7 @@
         <v>1140</v>
       </c>
       <c r="I320">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K320" t="s">
         <v>1148</v>
@@ -16315,7 +16315,7 @@
         <v>1140</v>
       </c>
       <c r="I321">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K321" t="s">
         <v>1144</v>
@@ -16353,7 +16353,7 @@
         <v>1140</v>
       </c>
       <c r="I322">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16397,7 +16397,7 @@
         <v>1140</v>
       </c>
       <c r="I323">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K323" t="s">
         <v>1144</v>
@@ -16435,7 +16435,7 @@
         <v>1140</v>
       </c>
       <c r="I324">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K324" t="s">
         <v>1144</v>
@@ -16473,7 +16473,7 @@
         <v>1140</v>
       </c>
       <c r="I325">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16517,7 +16517,7 @@
         <v>1140</v>
       </c>
       <c r="I326">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K326" t="s">
         <v>1144</v>
@@ -16555,7 +16555,7 @@
         <v>1140</v>
       </c>
       <c r="I327">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16599,7 +16599,7 @@
         <v>1140</v>
       </c>
       <c r="I328">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16643,7 +16643,7 @@
         <v>1140</v>
       </c>
       <c r="I329">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16687,7 +16687,7 @@
         <v>1140</v>
       </c>
       <c r="I330">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -16731,7 +16731,7 @@
         <v>1140</v>
       </c>
       <c r="I331">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K331" t="s">
         <v>1143</v>
@@ -16769,7 +16769,7 @@
         <v>1140</v>
       </c>
       <c r="I332">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K332" t="s">
         <v>1144</v>
@@ -16807,7 +16807,7 @@
         <v>1140</v>
       </c>
       <c r="I333">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K333" t="s">
         <v>1147</v>
@@ -16845,7 +16845,7 @@
         <v>1140</v>
       </c>
       <c r="I334">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K334" t="s">
         <v>1144</v>
@@ -16924,7 +16924,7 @@
         <v>1140</v>
       </c>
       <c r="I336">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K336" t="s">
         <v>1146</v>
@@ -17003,7 +17003,7 @@
         <v>1140</v>
       </c>
       <c r="I338">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K338" t="s">
         <v>1146</v>
@@ -17070,7 +17070,7 @@
         <v>1140</v>
       </c>
       <c r="I340">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K340" t="s">
         <v>1143</v>
@@ -17108,7 +17108,7 @@
         <v>1140</v>
       </c>
       <c r="I341">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K341" t="s">
         <v>1143</v>
@@ -17146,7 +17146,7 @@
         <v>1140</v>
       </c>
       <c r="I342">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K342" t="s">
         <v>1143</v>
@@ -17184,7 +17184,7 @@
         <v>1140</v>
       </c>
       <c r="I343">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K343" t="s">
         <v>1144</v>
@@ -17222,7 +17222,7 @@
         <v>1140</v>
       </c>
       <c r="I344">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K344" t="s">
         <v>1144</v>
@@ -17260,7 +17260,7 @@
         <v>1140</v>
       </c>
       <c r="I345">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K345" t="s">
         <v>1143</v>
@@ -17298,7 +17298,7 @@
         <v>1140</v>
       </c>
       <c r="I346">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K346" t="s">
         <v>1144</v>
@@ -17336,7 +17336,7 @@
         <v>1140</v>
       </c>
       <c r="I347">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17380,7 +17380,7 @@
         <v>1140</v>
       </c>
       <c r="I348">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17424,7 +17424,7 @@
         <v>1140</v>
       </c>
       <c r="I349">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K349" t="s">
         <v>1148</v>
@@ -17462,7 +17462,7 @@
         <v>1140</v>
       </c>
       <c r="I350">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K350" t="s">
         <v>1150</v>
@@ -17497,7 +17497,7 @@
         <v>1140</v>
       </c>
       <c r="I351">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K351" t="s">
         <v>1148</v>
@@ -17535,7 +17535,7 @@
         <v>1140</v>
       </c>
       <c r="I352">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K352" t="s">
         <v>1148</v>
@@ -17573,7 +17573,7 @@
         <v>1140</v>
       </c>
       <c r="I353">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K353" t="s">
         <v>1147</v>
@@ -17611,7 +17611,7 @@
         <v>1140</v>
       </c>
       <c r="I354">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K354" t="s">
         <v>1147</v>
@@ -17649,7 +17649,7 @@
         <v>1140</v>
       </c>
       <c r="I355">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -17731,7 +17731,7 @@
         <v>1140</v>
       </c>
       <c r="I357">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K357" t="s">
         <v>1147</v>
@@ -17769,7 +17769,7 @@
         <v>1140</v>
       </c>
       <c r="I358">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K358" t="s">
         <v>1147</v>
@@ -17807,7 +17807,7 @@
         <v>1140</v>
       </c>
       <c r="I359">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K359" t="s">
         <v>1147</v>
@@ -17848,7 +17848,7 @@
         <v>1140</v>
       </c>
       <c r="I360">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K360" t="s">
         <v>1147</v>
@@ -17886,7 +17886,7 @@
         <v>1140</v>
       </c>
       <c r="I361">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K361" t="s">
         <v>1147</v>
@@ -17924,7 +17924,7 @@
         <v>1140</v>
       </c>
       <c r="I362">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K362" t="s">
         <v>1147</v>
@@ -17962,7 +17962,7 @@
         <v>1140</v>
       </c>
       <c r="I363">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K363" t="s">
         <v>1147</v>
@@ -18000,7 +18000,7 @@
         <v>1140</v>
       </c>
       <c r="I364">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K364" t="s">
         <v>1147</v>
@@ -18038,7 +18038,7 @@
         <v>1140</v>
       </c>
       <c r="I365">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K365" t="s">
         <v>1146</v>
@@ -18076,7 +18076,7 @@
         <v>1140</v>
       </c>
       <c r="I366">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K366" t="s">
         <v>1147</v>
@@ -18114,7 +18114,7 @@
         <v>1140</v>
       </c>
       <c r="I367">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K367" t="s">
         <v>1147</v>
@@ -18152,7 +18152,7 @@
         <v>1140</v>
       </c>
       <c r="I368">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K368" t="s">
         <v>1147</v>
@@ -18190,7 +18190,7 @@
         <v>1140</v>
       </c>
       <c r="I369">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K369" t="s">
         <v>1147</v>
@@ -18228,7 +18228,7 @@
         <v>1140</v>
       </c>
       <c r="I370">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K370" t="s">
         <v>1147</v>
@@ -18266,7 +18266,7 @@
         <v>1140</v>
       </c>
       <c r="I371">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18310,7 +18310,7 @@
         <v>1140</v>
       </c>
       <c r="I372">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18357,7 +18357,7 @@
         <v>1140</v>
       </c>
       <c r="I373">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K373" t="s">
         <v>1143</v>
@@ -18395,7 +18395,7 @@
         <v>1140</v>
       </c>
       <c r="I374">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K374" t="s">
         <v>1143</v>
@@ -18433,7 +18433,7 @@
         <v>1140</v>
       </c>
       <c r="I375">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K375" t="s">
         <v>1147</v>
@@ -18471,7 +18471,7 @@
         <v>1140</v>
       </c>
       <c r="I376">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K376" t="s">
         <v>1147</v>
@@ -18547,7 +18547,7 @@
         <v>1140</v>
       </c>
       <c r="I378">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K378" t="s">
         <v>1147</v>
@@ -18585,7 +18585,7 @@
         <v>1140</v>
       </c>
       <c r="I379">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18629,7 +18629,7 @@
         <v>1140</v>
       </c>
       <c r="I380">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K380" t="s">
         <v>1147</v>
@@ -18667,7 +18667,7 @@
         <v>1140</v>
       </c>
       <c r="I381">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K381" t="s">
         <v>1147</v>
@@ -18705,7 +18705,7 @@
         <v>1140</v>
       </c>
       <c r="I382">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K382" t="s">
         <v>1147</v>
@@ -18743,7 +18743,7 @@
         <v>1140</v>
       </c>
       <c r="I383">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K383" t="s">
         <v>1147</v>
@@ -18781,7 +18781,7 @@
         <v>1140</v>
       </c>
       <c r="I384">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K384" t="s">
         <v>1143</v>
@@ -18819,7 +18819,7 @@
         <v>1140</v>
       </c>
       <c r="I385">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K385" t="s">
         <v>1143</v>
@@ -18857,7 +18857,7 @@
         <v>1140</v>
       </c>
       <c r="I386">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K386" t="s">
         <v>1147</v>
@@ -18895,7 +18895,7 @@
         <v>1140</v>
       </c>
       <c r="I387">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K387" t="s">
         <v>1147</v>
@@ -18933,7 +18933,7 @@
         <v>1140</v>
       </c>
       <c r="I388">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K388" t="s">
         <v>1147</v>
@@ -18971,7 +18971,7 @@
         <v>1140</v>
       </c>
       <c r="I389">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K389" t="s">
         <v>1148</v>
@@ -19009,7 +19009,7 @@
         <v>1140</v>
       </c>
       <c r="I390">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19129,7 +19129,7 @@
         <v>1140</v>
       </c>
       <c r="I393">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K393" t="s">
         <v>1147</v>
@@ -19167,7 +19167,7 @@
         <v>1140</v>
       </c>
       <c r="I394">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K394" t="s">
         <v>1147</v>
@@ -19205,7 +19205,7 @@
         <v>1140</v>
       </c>
       <c r="I395">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K395" t="s">
         <v>1147</v>
@@ -19243,7 +19243,7 @@
         <v>1140</v>
       </c>
       <c r="I396">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K396" t="s">
         <v>1147</v>
@@ -19281,7 +19281,7 @@
         <v>1140</v>
       </c>
       <c r="I397">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K397" t="s">
         <v>1147</v>
@@ -19319,7 +19319,7 @@
         <v>1140</v>
       </c>
       <c r="I398">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K398" t="s">
         <v>1147</v>
@@ -19395,7 +19395,7 @@
         <v>1140</v>
       </c>
       <c r="I400">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K400" t="s">
         <v>1147</v>
@@ -19433,7 +19433,7 @@
         <v>1140</v>
       </c>
       <c r="I401">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K401" t="s">
         <v>1147</v>
@@ -19471,7 +19471,7 @@
         <v>1140</v>
       </c>
       <c r="I402">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K402" t="s">
         <v>1147</v>
@@ -19509,7 +19509,7 @@
         <v>1140</v>
       </c>
       <c r="I403">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K403" t="s">
         <v>1150</v>
@@ -19544,7 +19544,7 @@
         <v>1140</v>
       </c>
       <c r="I404">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K404" t="s">
         <v>1150</v>
@@ -19608,7 +19608,7 @@
         <v>1140</v>
       </c>
       <c r="I406">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19640,7 +19640,7 @@
         <v>1140</v>
       </c>
       <c r="I407">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19672,7 +19672,7 @@
         <v>1140</v>
       </c>
       <c r="I408">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19704,7 +19704,7 @@
         <v>1140</v>
       </c>
       <c r="I409">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -19736,7 +19736,7 @@
         <v>1140</v>
       </c>
       <c r="I410">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -19768,7 +19768,7 @@
         <v>1140</v>
       </c>
       <c r="I411">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -19800,7 +19800,7 @@
         <v>1140</v>
       </c>
       <c r="I412">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -19832,7 +19832,7 @@
         <v>1140</v>
       </c>
       <c r="I413">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -19864,7 +19864,7 @@
         <v>1140</v>
       </c>
       <c r="I414">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -19896,7 +19896,7 @@
         <v>1140</v>
       </c>
       <c r="I415">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -19928,7 +19928,7 @@
         <v>1140</v>
       </c>
       <c r="I416">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -19960,7 +19960,7 @@
         <v>1140</v>
       </c>
       <c r="I417">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -19992,7 +19992,7 @@
         <v>1140</v>
       </c>
       <c r="I418">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20024,7 +20024,7 @@
         <v>1140</v>
       </c>
       <c r="I419">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20056,7 +20056,7 @@
         <v>1140</v>
       </c>
       <c r="I420">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20088,7 +20088,7 @@
         <v>1140</v>
       </c>
       <c r="I421">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20120,7 +20120,7 @@
         <v>1140</v>
       </c>
       <c r="I422">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20152,7 +20152,7 @@
         <v>1140</v>
       </c>
       <c r="I423">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20184,7 +20184,7 @@
         <v>1140</v>
       </c>
       <c r="I424">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20216,7 +20216,7 @@
         <v>1140</v>
       </c>
       <c r="I425">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20248,7 +20248,7 @@
         <v>1140</v>
       </c>
       <c r="I426">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20280,7 +20280,7 @@
         <v>1140</v>
       </c>
       <c r="I427">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20312,7 +20312,7 @@
         <v>1140</v>
       </c>
       <c r="I428">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20344,7 +20344,7 @@
         <v>1140</v>
       </c>
       <c r="I429">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20376,7 +20376,7 @@
         <v>1140</v>
       </c>
       <c r="I430">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20408,7 +20408,7 @@
         <v>1140</v>
       </c>
       <c r="I431">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20440,7 +20440,7 @@
         <v>1140</v>
       </c>
       <c r="I432">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20472,7 +20472,7 @@
         <v>1140</v>
       </c>
       <c r="I433">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20504,7 +20504,7 @@
         <v>1140</v>
       </c>
       <c r="I434">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20536,7 +20536,7 @@
         <v>1140</v>
       </c>
       <c r="I435">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20568,7 +20568,7 @@
         <v>1140</v>
       </c>
       <c r="I436">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20600,7 +20600,7 @@
         <v>1142</v>
       </c>
       <c r="I437">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20632,7 +20632,7 @@
         <v>1142</v>
       </c>
       <c r="I438">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20664,7 +20664,7 @@
         <v>1140</v>
       </c>
       <c r="I439">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20696,7 +20696,7 @@
         <v>1140</v>
       </c>
       <c r="I440">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -20728,7 +20728,7 @@
         <v>1140</v>
       </c>
       <c r="I441">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -20760,7 +20760,7 @@
         <v>1140</v>
       </c>
       <c r="I442">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -20792,7 +20792,7 @@
         <v>1140</v>
       </c>
       <c r="I443">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -20824,7 +20824,7 @@
         <v>1140</v>
       </c>
       <c r="I444">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -20856,7 +20856,7 @@
         <v>1140</v>
       </c>
       <c r="I445">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -20888,7 +20888,7 @@
         <v>1140</v>
       </c>
       <c r="I446">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -20920,7 +20920,7 @@
         <v>1140</v>
       </c>
       <c r="I447">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (29/07/2026 13:14)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4253,7 +4253,7 @@
         <v>1140</v>
       </c>
       <c r="I2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K2" t="s">
         <v>1143</v>
@@ -4291,7 +4291,7 @@
         <v>1140</v>
       </c>
       <c r="I3">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="K3" t="s">
         <v>1144</v>
@@ -4329,7 +4329,7 @@
         <v>1140</v>
       </c>
       <c r="I4">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="K4" t="s">
         <v>1144</v>
@@ -4367,7 +4367,7 @@
         <v>1140</v>
       </c>
       <c r="I5">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4411,7 +4411,7 @@
         <v>1140</v>
       </c>
       <c r="I6">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4455,7 +4455,7 @@
         <v>1140</v>
       </c>
       <c r="I7">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4531,7 +4531,7 @@
         <v>1140</v>
       </c>
       <c r="I9">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4578,7 +4578,7 @@
         <v>1140</v>
       </c>
       <c r="I10">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4625,7 +4625,7 @@
         <v>1140</v>
       </c>
       <c r="I11">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4672,7 +4672,7 @@
         <v>1140</v>
       </c>
       <c r="I12">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -4751,7 +4751,7 @@
         <v>1140</v>
       </c>
       <c r="I14">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -4795,7 +4795,7 @@
         <v>1140</v>
       </c>
       <c r="I15">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K15" t="s">
         <v>1146</v>
@@ -4833,7 +4833,7 @@
         <v>1140</v>
       </c>
       <c r="I16">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K16" t="s">
         <v>1143</v>
@@ -4871,7 +4871,7 @@
         <v>1140</v>
       </c>
       <c r="I17">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -4915,7 +4915,7 @@
         <v>1140</v>
       </c>
       <c r="I18">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -4994,7 +4994,7 @@
         <v>1140</v>
       </c>
       <c r="I20">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5073,7 +5073,7 @@
         <v>1140</v>
       </c>
       <c r="I22">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K22" t="s">
         <v>1147</v>
@@ -5111,7 +5111,7 @@
         <v>1140</v>
       </c>
       <c r="I23">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5234,7 +5234,7 @@
         <v>1140</v>
       </c>
       <c r="I26">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5281,7 +5281,7 @@
         <v>1140</v>
       </c>
       <c r="I27">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K27" t="s">
         <v>1147</v>
@@ -5386,7 +5386,7 @@
         <v>1140</v>
       </c>
       <c r="I30">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5468,7 +5468,7 @@
         <v>1140</v>
       </c>
       <c r="I32">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K32" t="s">
         <v>1143</v>
@@ -5710,7 +5710,7 @@
         <v>1140</v>
       </c>
       <c r="I39">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K39" t="s">
         <v>1148</v>
@@ -5745,7 +5745,7 @@
         <v>1140</v>
       </c>
       <c r="I40">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K40" t="s">
         <v>1146</v>
@@ -5894,7 +5894,7 @@
         <v>1140</v>
       </c>
       <c r="I44">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -5941,7 +5941,7 @@
         <v>1140</v>
       </c>
       <c r="I45">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -5988,7 +5988,7 @@
         <v>1140</v>
       </c>
       <c r="I46">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K46" t="s">
         <v>1147</v>
@@ -6026,7 +6026,7 @@
         <v>1140</v>
       </c>
       <c r="I47">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6073,7 +6073,7 @@
         <v>1140</v>
       </c>
       <c r="I48">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K48" t="s">
         <v>1147</v>
@@ -6143,7 +6143,7 @@
         <v>1140</v>
       </c>
       <c r="I50">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K50" t="s">
         <v>1147</v>
@@ -6219,7 +6219,7 @@
         <v>1140</v>
       </c>
       <c r="I52">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K52" t="s">
         <v>1143</v>
@@ -6257,7 +6257,7 @@
         <v>1140</v>
       </c>
       <c r="I53">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K53" t="s">
         <v>1144</v>
@@ -6295,7 +6295,7 @@
         <v>1140</v>
       </c>
       <c r="I54">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K54" t="s">
         <v>1144</v>
@@ -6403,7 +6403,7 @@
         <v>1140</v>
       </c>
       <c r="I57">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K57" t="s">
         <v>1147</v>
@@ -6607,7 +6607,7 @@
         <v>1140</v>
       </c>
       <c r="I63">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6654,7 +6654,7 @@
         <v>1140</v>
       </c>
       <c r="I64">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -6885,7 +6885,7 @@
         <v>1140</v>
       </c>
       <c r="I70">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K70" t="s">
         <v>1144</v>
@@ -6923,7 +6923,7 @@
         <v>1140</v>
       </c>
       <c r="I71">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K71" t="s">
         <v>1150</v>
@@ -6993,7 +6993,7 @@
         <v>1140</v>
       </c>
       <c r="I73">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K73" t="s">
         <v>1143</v>
@@ -7069,7 +7069,7 @@
         <v>1140</v>
       </c>
       <c r="I75">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K75" t="s">
         <v>1144</v>
@@ -7107,7 +7107,7 @@
         <v>1140</v>
       </c>
       <c r="I76">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K76" t="s">
         <v>1150</v>
@@ -7215,7 +7215,7 @@
         <v>1140</v>
       </c>
       <c r="I79">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K79" t="s">
         <v>1150</v>
@@ -7250,7 +7250,7 @@
         <v>1140</v>
       </c>
       <c r="I80">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K80" t="s">
         <v>1144</v>
@@ -7326,7 +7326,7 @@
         <v>1140</v>
       </c>
       <c r="I82">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K82" t="s">
         <v>1147</v>
@@ -7399,7 +7399,7 @@
         <v>1140</v>
       </c>
       <c r="I84">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7446,7 +7446,7 @@
         <v>1140</v>
       </c>
       <c r="I85">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K85" t="s">
         <v>1144</v>
@@ -7484,7 +7484,7 @@
         <v>1140</v>
       </c>
       <c r="I86">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K86" t="s">
         <v>1144</v>
@@ -7522,7 +7522,7 @@
         <v>1140</v>
       </c>
       <c r="I87">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7639,7 +7639,7 @@
         <v>1140</v>
       </c>
       <c r="I90">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K90" t="s">
         <v>1117</v>
@@ -7680,7 +7680,7 @@
         <v>1140</v>
       </c>
       <c r="I91">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K91" t="s">
         <v>1146</v>
@@ -7747,7 +7747,7 @@
         <v>1140</v>
       </c>
       <c r="I93">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K93" t="s">
         <v>1146</v>
@@ -7785,7 +7785,7 @@
         <v>1140</v>
       </c>
       <c r="I94">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K94" t="s">
         <v>1147</v>
@@ -7823,7 +7823,7 @@
         <v>1140</v>
       </c>
       <c r="I95">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K95" t="s">
         <v>1146</v>
@@ -7861,7 +7861,7 @@
         <v>1140</v>
       </c>
       <c r="I96">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -7908,7 +7908,7 @@
         <v>1140</v>
       </c>
       <c r="I97">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K97" t="s">
         <v>1117</v>
@@ -7949,7 +7949,7 @@
         <v>1140</v>
       </c>
       <c r="I98">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K98" t="s">
         <v>1147</v>
@@ -8016,7 +8016,7 @@
         <v>1140</v>
       </c>
       <c r="I100">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K100" t="s">
         <v>1146</v>
@@ -8144,7 +8144,7 @@
         <v>1140</v>
       </c>
       <c r="I104">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K104" t="s">
         <v>1146</v>
@@ -8182,7 +8182,7 @@
         <v>1140</v>
       </c>
       <c r="I105">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K105" t="s">
         <v>1146</v>
@@ -8220,7 +8220,7 @@
         <v>1140</v>
       </c>
       <c r="I106">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8264,7 +8264,7 @@
         <v>1140</v>
       </c>
       <c r="I107">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8308,7 +8308,7 @@
         <v>1140</v>
       </c>
       <c r="I108">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K108" t="s">
         <v>1144</v>
@@ -8346,7 +8346,7 @@
         <v>1140</v>
       </c>
       <c r="I109">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K109" t="s">
         <v>1144</v>
@@ -8562,7 +8562,7 @@
         <v>1140</v>
       </c>
       <c r="I115">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K115" t="s">
         <v>1144</v>
@@ -8600,7 +8600,7 @@
         <v>1140</v>
       </c>
       <c r="I116">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K116" t="s">
         <v>1144</v>
@@ -8638,7 +8638,7 @@
         <v>1140</v>
       </c>
       <c r="I117">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K117" t="s">
         <v>1144</v>
@@ -8676,7 +8676,7 @@
         <v>1140</v>
       </c>
       <c r="I118">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K118" t="s">
         <v>1144</v>
@@ -8714,7 +8714,7 @@
         <v>1140</v>
       </c>
       <c r="I119">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K119" t="s">
         <v>1144</v>
@@ -8752,7 +8752,7 @@
         <v>1140</v>
       </c>
       <c r="I120">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K120" t="s">
         <v>1144</v>
@@ -8790,7 +8790,7 @@
         <v>1140</v>
       </c>
       <c r="I121">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -8837,7 +8837,7 @@
         <v>1140</v>
       </c>
       <c r="I122">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K122" t="s">
         <v>1144</v>
@@ -8904,7 +8904,7 @@
         <v>1140</v>
       </c>
       <c r="I124">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K124" t="s">
         <v>1144</v>
@@ -8942,7 +8942,7 @@
         <v>1140</v>
       </c>
       <c r="I125">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K125" t="s">
         <v>1150</v>
@@ -9047,7 +9047,7 @@
         <v>1140</v>
       </c>
       <c r="I128">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K128" t="s">
         <v>1144</v>
@@ -9085,7 +9085,7 @@
         <v>1140</v>
       </c>
       <c r="I129">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K129" t="s">
         <v>1143</v>
@@ -9123,7 +9123,7 @@
         <v>1140</v>
       </c>
       <c r="I130">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9205,7 +9205,7 @@
         <v>1140</v>
       </c>
       <c r="I132">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9281,7 +9281,7 @@
         <v>1140</v>
       </c>
       <c r="I134">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K134" t="s">
         <v>1143</v>
@@ -9412,7 +9412,7 @@
         <v>1140</v>
       </c>
       <c r="I138">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K138" t="s">
         <v>1144</v>
@@ -9741,7 +9741,7 @@
         <v>1140</v>
       </c>
       <c r="I148">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K148" t="s">
         <v>1144</v>
@@ -9779,7 +9779,7 @@
         <v>1140</v>
       </c>
       <c r="I149">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K149" t="s">
         <v>1150</v>
@@ -9814,7 +9814,7 @@
         <v>1140</v>
       </c>
       <c r="I150">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -9899,7 +9899,7 @@
         <v>1140</v>
       </c>
       <c r="I152">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -9943,7 +9943,7 @@
         <v>1140</v>
       </c>
       <c r="I153">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K153" t="s">
         <v>1144</v>
@@ -10016,7 +10016,7 @@
         <v>1140</v>
       </c>
       <c r="I155">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K155" t="s">
         <v>1150</v>
@@ -10051,7 +10051,7 @@
         <v>1140</v>
       </c>
       <c r="I156">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K156" t="s">
         <v>1144</v>
@@ -10089,7 +10089,7 @@
         <v>1140</v>
       </c>
       <c r="I157">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K157" t="s">
         <v>1146</v>
@@ -10127,7 +10127,7 @@
         <v>1140</v>
       </c>
       <c r="I158">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10171,7 +10171,7 @@
         <v>1140</v>
       </c>
       <c r="I159">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K159" t="s">
         <v>1144</v>
@@ -10209,7 +10209,7 @@
         <v>1140</v>
       </c>
       <c r="I160">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K160" t="s">
         <v>1144</v>
@@ -10247,7 +10247,7 @@
         <v>1140</v>
       </c>
       <c r="I161">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10294,7 +10294,7 @@
         <v>1140</v>
       </c>
       <c r="I162">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10338,7 +10338,7 @@
         <v>1140</v>
       </c>
       <c r="I163">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10382,7 +10382,7 @@
         <v>1142</v>
       </c>
       <c r="I164">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K164" t="s">
         <v>1151</v>
@@ -10417,7 +10417,7 @@
         <v>1140</v>
       </c>
       <c r="I165">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K165" t="s">
         <v>1144</v>
@@ -10525,7 +10525,7 @@
         <v>1140</v>
       </c>
       <c r="I168">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K168" t="s">
         <v>1147</v>
@@ -10566,7 +10566,7 @@
         <v>1140</v>
       </c>
       <c r="I169">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10648,7 +10648,7 @@
         <v>1140</v>
       </c>
       <c r="I171">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K171" t="s">
         <v>1144</v>
@@ -10794,7 +10794,7 @@
         <v>1140</v>
       </c>
       <c r="I175">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -10841,7 +10841,7 @@
         <v>1140</v>
       </c>
       <c r="I176">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K176" t="s">
         <v>1144</v>
@@ -10879,7 +10879,7 @@
         <v>1140</v>
       </c>
       <c r="I177">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -10926,7 +10926,7 @@
         <v>1140</v>
       </c>
       <c r="I178">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K178" t="s">
         <v>1143</v>
@@ -10993,7 +10993,7 @@
         <v>1140</v>
       </c>
       <c r="I180">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K180" t="s">
         <v>1143</v>
@@ -11098,7 +11098,7 @@
         <v>1140</v>
       </c>
       <c r="I183">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K183" t="s">
         <v>1144</v>
@@ -11133,7 +11133,7 @@
         <v>1140</v>
       </c>
       <c r="I184">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K184" t="s">
         <v>1150</v>
@@ -11168,7 +11168,7 @@
         <v>1140</v>
       </c>
       <c r="I185">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K185" t="s">
         <v>1144</v>
@@ -11206,7 +11206,7 @@
         <v>1140</v>
       </c>
       <c r="I186">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K186" t="s">
         <v>1144</v>
@@ -11244,7 +11244,7 @@
         <v>1140</v>
       </c>
       <c r="I187">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11291,7 +11291,7 @@
         <v>1140</v>
       </c>
       <c r="I188">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11338,7 +11338,7 @@
         <v>1140</v>
       </c>
       <c r="I189">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11382,7 +11382,7 @@
         <v>1140</v>
       </c>
       <c r="I190">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K190" t="s">
         <v>1146</v>
@@ -11420,7 +11420,7 @@
         <v>1140</v>
       </c>
       <c r="I191">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11464,7 +11464,7 @@
         <v>1140</v>
       </c>
       <c r="I192">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K192" t="s">
         <v>1144</v>
@@ -11502,7 +11502,7 @@
         <v>1140</v>
       </c>
       <c r="I193">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K193" t="s">
         <v>1149</v>
@@ -11572,7 +11572,7 @@
         <v>1140</v>
       </c>
       <c r="I195">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K195" t="s">
         <v>1146</v>
@@ -11706,7 +11706,7 @@
         <v>1140</v>
       </c>
       <c r="I199">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -11750,7 +11750,7 @@
         <v>1140</v>
       </c>
       <c r="I200">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K200" t="s">
         <v>1146</v>
@@ -11788,7 +11788,7 @@
         <v>1140</v>
       </c>
       <c r="I201">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K201" t="s">
         <v>1144</v>
@@ -11826,7 +11826,7 @@
         <v>1140</v>
       </c>
       <c r="I202">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K202" t="s">
         <v>1144</v>
@@ -11864,7 +11864,7 @@
         <v>1140</v>
       </c>
       <c r="I203">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K203" t="s">
         <v>1144</v>
@@ -11902,7 +11902,7 @@
         <v>1140</v>
       </c>
       <c r="I204">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K204" t="s">
         <v>1143</v>
@@ -11940,7 +11940,7 @@
         <v>1140</v>
       </c>
       <c r="I205">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K205" t="s">
         <v>1143</v>
@@ -12013,7 +12013,7 @@
         <v>1140</v>
       </c>
       <c r="I207">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12057,7 +12057,7 @@
         <v>1140</v>
       </c>
       <c r="I208">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12101,7 +12101,7 @@
         <v>1140</v>
       </c>
       <c r="I209">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12145,7 +12145,7 @@
         <v>1140</v>
       </c>
       <c r="I210">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K210" t="s">
         <v>1147</v>
@@ -12253,7 +12253,7 @@
         <v>1140</v>
       </c>
       <c r="I213">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K213" t="s">
         <v>1144</v>
@@ -12291,7 +12291,7 @@
         <v>1140</v>
       </c>
       <c r="I214">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12338,7 +12338,7 @@
         <v>1140</v>
       </c>
       <c r="I215">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K215" t="s">
         <v>1144</v>
@@ -12405,7 +12405,7 @@
         <v>1140</v>
       </c>
       <c r="I217">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12449,7 +12449,7 @@
         <v>1140</v>
       </c>
       <c r="I218">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K218" t="s">
         <v>1146</v>
@@ -12487,7 +12487,7 @@
         <v>1140</v>
       </c>
       <c r="I219">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K219" t="s">
         <v>1146</v>
@@ -12525,7 +12525,7 @@
         <v>1140</v>
       </c>
       <c r="I220">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K220" t="s">
         <v>1146</v>
@@ -12601,7 +12601,7 @@
         <v>1140</v>
       </c>
       <c r="I222">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K222" t="s">
         <v>1144</v>
@@ -12639,7 +12639,7 @@
         <v>1140</v>
       </c>
       <c r="I223">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K223" t="s">
         <v>1144</v>
@@ -12677,7 +12677,7 @@
         <v>1140</v>
       </c>
       <c r="I224">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K224" t="s">
         <v>1144</v>
@@ -12715,7 +12715,7 @@
         <v>1140</v>
       </c>
       <c r="I225">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K225" t="s">
         <v>1144</v>
@@ -12753,7 +12753,7 @@
         <v>1140</v>
       </c>
       <c r="I226">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K226" t="s">
         <v>1144</v>
@@ -12791,7 +12791,7 @@
         <v>1140</v>
       </c>
       <c r="I227">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K227" t="s">
         <v>1144</v>
@@ -12829,7 +12829,7 @@
         <v>1140</v>
       </c>
       <c r="I228">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K228" t="s">
         <v>1144</v>
@@ -12902,7 +12902,7 @@
         <v>1140</v>
       </c>
       <c r="I230">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K230" t="s">
         <v>1147</v>
@@ -12940,7 +12940,7 @@
         <v>1140</v>
       </c>
       <c r="I231">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13054,7 +13054,7 @@
         <v>1140</v>
       </c>
       <c r="I234">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13101,7 +13101,7 @@
         <v>1140</v>
       </c>
       <c r="I235">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13148,7 +13148,7 @@
         <v>1140</v>
       </c>
       <c r="I236">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13192,7 +13192,7 @@
         <v>1140</v>
       </c>
       <c r="I237">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K237" t="s">
         <v>1144</v>
@@ -13259,7 +13259,7 @@
         <v>1140</v>
       </c>
       <c r="I239">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K239" t="s">
         <v>1117</v>
@@ -13370,7 +13370,7 @@
         <v>1140</v>
       </c>
       <c r="I242">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K242" t="s">
         <v>1143</v>
@@ -13440,7 +13440,7 @@
         <v>1140</v>
       </c>
       <c r="I244">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K244" t="s">
         <v>1146</v>
@@ -13478,7 +13478,7 @@
         <v>1140</v>
       </c>
       <c r="I245">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K245" t="s">
         <v>1146</v>
@@ -13516,7 +13516,7 @@
         <v>1140</v>
       </c>
       <c r="I246">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13621,7 +13621,7 @@
         <v>1140</v>
       </c>
       <c r="I249">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K249" t="s">
         <v>1144</v>
@@ -13659,7 +13659,7 @@
         <v>1140</v>
       </c>
       <c r="I250">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K250" t="s">
         <v>1146</v>
@@ -13767,7 +13767,7 @@
         <v>1140</v>
       </c>
       <c r="I253">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K253" t="s">
         <v>1147</v>
@@ -13805,7 +13805,7 @@
         <v>1140</v>
       </c>
       <c r="I254">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K254" t="s">
         <v>1147</v>
@@ -13843,7 +13843,7 @@
         <v>1140</v>
       </c>
       <c r="I255">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K255" t="s">
         <v>1146</v>
@@ -13881,7 +13881,7 @@
         <v>1140</v>
       </c>
       <c r="I256">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K256" t="s">
         <v>1144</v>
@@ -13980,7 +13980,7 @@
         <v>1140</v>
       </c>
       <c r="I259">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K259" t="s">
         <v>1146</v>
@@ -14018,7 +14018,7 @@
         <v>1140</v>
       </c>
       <c r="I260">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K260" t="s">
         <v>1146</v>
@@ -14056,7 +14056,7 @@
         <v>1140</v>
       </c>
       <c r="I261">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K261" t="s">
         <v>1147</v>
@@ -14094,7 +14094,7 @@
         <v>1140</v>
       </c>
       <c r="I262">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14179,7 +14179,7 @@
         <v>1140</v>
       </c>
       <c r="I264">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K264" t="s">
         <v>1147</v>
@@ -14217,7 +14217,7 @@
         <v>1140</v>
       </c>
       <c r="I265">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K265" t="s">
         <v>1147</v>
@@ -14255,7 +14255,7 @@
         <v>1140</v>
       </c>
       <c r="I266">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K266" t="s">
         <v>1146</v>
@@ -14293,7 +14293,7 @@
         <v>1140</v>
       </c>
       <c r="I267">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K267" t="s">
         <v>1147</v>
@@ -14331,7 +14331,7 @@
         <v>1140</v>
       </c>
       <c r="I268">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K268" t="s">
         <v>1144</v>
@@ -14366,7 +14366,7 @@
         <v>1140</v>
       </c>
       <c r="I269">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K269" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1140</v>
       </c>
       <c r="I270">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K270" t="s">
         <v>1147</v>
@@ -14442,7 +14442,7 @@
         <v>1140</v>
       </c>
       <c r="I271">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K271" t="s">
         <v>1147</v>
@@ -14480,7 +14480,7 @@
         <v>1140</v>
       </c>
       <c r="I272">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14562,7 +14562,7 @@
         <v>1140</v>
       </c>
       <c r="I274">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K274" t="s">
         <v>1144</v>
@@ -14635,7 +14635,7 @@
         <v>1140</v>
       </c>
       <c r="I276">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K276" t="s">
         <v>1148</v>
@@ -14673,7 +14673,7 @@
         <v>1140</v>
       </c>
       <c r="I277">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K277" t="s">
         <v>1144</v>
@@ -14711,7 +14711,7 @@
         <v>1140</v>
       </c>
       <c r="I278">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K278" t="s">
         <v>1147</v>
@@ -14749,7 +14749,7 @@
         <v>1140</v>
       </c>
       <c r="I279">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K279" t="s">
         <v>1146</v>
@@ -14790,7 +14790,7 @@
         <v>1140</v>
       </c>
       <c r="I280">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K280" t="s">
         <v>1144</v>
@@ -14828,7 +14828,7 @@
         <v>1140</v>
       </c>
       <c r="I281">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K281" t="s">
         <v>1144</v>
@@ -14866,7 +14866,7 @@
         <v>1140</v>
       </c>
       <c r="I282">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K282" t="s">
         <v>1144</v>
@@ -15073,7 +15073,7 @@
         <v>1140</v>
       </c>
       <c r="I288">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K288" t="s">
         <v>1147</v>
@@ -15140,7 +15140,7 @@
         <v>1140</v>
       </c>
       <c r="I290">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15181,7 +15181,7 @@
         <v>1140</v>
       </c>
       <c r="I291">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K291" t="s">
         <v>1146</v>
@@ -15219,7 +15219,7 @@
         <v>1140</v>
       </c>
       <c r="I292">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K292" t="s">
         <v>1147</v>
@@ -15257,7 +15257,7 @@
         <v>1140</v>
       </c>
       <c r="I293">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K293" t="s">
         <v>1148</v>
@@ -15295,7 +15295,7 @@
         <v>1140</v>
       </c>
       <c r="I294">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K294" t="s">
         <v>1150</v>
@@ -15330,7 +15330,7 @@
         <v>1140</v>
       </c>
       <c r="I295">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K295" t="s">
         <v>1150</v>
@@ -15365,7 +15365,7 @@
         <v>1140</v>
       </c>
       <c r="I296">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K296" t="s">
         <v>1150</v>
@@ -15435,7 +15435,7 @@
         <v>1140</v>
       </c>
       <c r="I298">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K298" t="s">
         <v>1144</v>
@@ -15473,7 +15473,7 @@
         <v>1140</v>
       </c>
       <c r="I299">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K299" t="s">
         <v>1147</v>
@@ -15511,7 +15511,7 @@
         <v>1140</v>
       </c>
       <c r="I300">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K300" t="s">
         <v>1147</v>
@@ -15549,7 +15549,7 @@
         <v>1140</v>
       </c>
       <c r="I301">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K301" t="s">
         <v>1147</v>
@@ -15587,7 +15587,7 @@
         <v>1140</v>
       </c>
       <c r="I302">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K302" t="s">
         <v>1147</v>
@@ -15625,7 +15625,7 @@
         <v>1140</v>
       </c>
       <c r="I303">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K303" t="s">
         <v>1144</v>
@@ -15663,7 +15663,7 @@
         <v>1140</v>
       </c>
       <c r="I304">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K304" t="s">
         <v>1147</v>
@@ -15701,7 +15701,7 @@
         <v>1140</v>
       </c>
       <c r="I305">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -15745,7 +15745,7 @@
         <v>1140</v>
       </c>
       <c r="I306">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -15789,7 +15789,7 @@
         <v>1140</v>
       </c>
       <c r="I307">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K307" t="s">
         <v>1143</v>
@@ -15827,7 +15827,7 @@
         <v>1140</v>
       </c>
       <c r="I308">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K308" t="s">
         <v>1143</v>
@@ -15865,7 +15865,7 @@
         <v>1140</v>
       </c>
       <c r="I309">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K309" t="s">
         <v>1143</v>
@@ -15903,7 +15903,7 @@
         <v>1140</v>
       </c>
       <c r="I310">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K310" t="s">
         <v>1144</v>
@@ -15941,7 +15941,7 @@
         <v>1140</v>
       </c>
       <c r="I311">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K311" t="s">
         <v>1143</v>
@@ -15979,7 +15979,7 @@
         <v>1140</v>
       </c>
       <c r="I312">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K312" t="s">
         <v>1144</v>
@@ -16052,7 +16052,7 @@
         <v>1140</v>
       </c>
       <c r="I314">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K314" t="s">
         <v>1144</v>
@@ -16090,7 +16090,7 @@
         <v>1140</v>
       </c>
       <c r="I315">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K315" t="s">
         <v>1144</v>
@@ -16128,7 +16128,7 @@
         <v>1140</v>
       </c>
       <c r="I316">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K316" t="s">
         <v>1144</v>
@@ -16166,7 +16166,7 @@
         <v>1140</v>
       </c>
       <c r="I317">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K317" t="s">
         <v>1144</v>
@@ -16277,7 +16277,7 @@
         <v>1140</v>
       </c>
       <c r="I320">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K320" t="s">
         <v>1148</v>
@@ -16315,7 +16315,7 @@
         <v>1140</v>
       </c>
       <c r="I321">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K321" t="s">
         <v>1144</v>
@@ -16353,7 +16353,7 @@
         <v>1140</v>
       </c>
       <c r="I322">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16397,7 +16397,7 @@
         <v>1140</v>
       </c>
       <c r="I323">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K323" t="s">
         <v>1144</v>
@@ -16435,7 +16435,7 @@
         <v>1140</v>
       </c>
       <c r="I324">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K324" t="s">
         <v>1144</v>
@@ -16473,7 +16473,7 @@
         <v>1140</v>
       </c>
       <c r="I325">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16517,7 +16517,7 @@
         <v>1140</v>
       </c>
       <c r="I326">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K326" t="s">
         <v>1144</v>
@@ -16555,7 +16555,7 @@
         <v>1140</v>
       </c>
       <c r="I327">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16599,7 +16599,7 @@
         <v>1140</v>
       </c>
       <c r="I328">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16643,7 +16643,7 @@
         <v>1140</v>
       </c>
       <c r="I329">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16687,7 +16687,7 @@
         <v>1140</v>
       </c>
       <c r="I330">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -16731,7 +16731,7 @@
         <v>1140</v>
       </c>
       <c r="I331">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K331" t="s">
         <v>1143</v>
@@ -16769,7 +16769,7 @@
         <v>1140</v>
       </c>
       <c r="I332">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K332" t="s">
         <v>1144</v>
@@ -16807,7 +16807,7 @@
         <v>1140</v>
       </c>
       <c r="I333">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K333" t="s">
         <v>1147</v>
@@ -16845,7 +16845,7 @@
         <v>1140</v>
       </c>
       <c r="I334">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K334" t="s">
         <v>1144</v>
@@ -16924,7 +16924,7 @@
         <v>1140</v>
       </c>
       <c r="I336">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K336" t="s">
         <v>1146</v>
@@ -17003,7 +17003,7 @@
         <v>1140</v>
       </c>
       <c r="I338">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K338" t="s">
         <v>1146</v>
@@ -17070,7 +17070,7 @@
         <v>1140</v>
       </c>
       <c r="I340">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K340" t="s">
         <v>1143</v>
@@ -17108,7 +17108,7 @@
         <v>1140</v>
       </c>
       <c r="I341">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K341" t="s">
         <v>1143</v>
@@ -17146,7 +17146,7 @@
         <v>1140</v>
       </c>
       <c r="I342">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K342" t="s">
         <v>1143</v>
@@ -17184,7 +17184,7 @@
         <v>1140</v>
       </c>
       <c r="I343">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K343" t="s">
         <v>1144</v>
@@ -17222,7 +17222,7 @@
         <v>1140</v>
       </c>
       <c r="I344">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K344" t="s">
         <v>1144</v>
@@ -17260,7 +17260,7 @@
         <v>1140</v>
       </c>
       <c r="I345">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K345" t="s">
         <v>1143</v>
@@ -17298,7 +17298,7 @@
         <v>1140</v>
       </c>
       <c r="I346">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K346" t="s">
         <v>1144</v>
@@ -17336,7 +17336,7 @@
         <v>1140</v>
       </c>
       <c r="I347">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17380,7 +17380,7 @@
         <v>1140</v>
       </c>
       <c r="I348">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17424,7 +17424,7 @@
         <v>1140</v>
       </c>
       <c r="I349">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K349" t="s">
         <v>1148</v>
@@ -17462,7 +17462,7 @@
         <v>1140</v>
       </c>
       <c r="I350">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K350" t="s">
         <v>1150</v>
@@ -17497,7 +17497,7 @@
         <v>1140</v>
       </c>
       <c r="I351">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K351" t="s">
         <v>1148</v>
@@ -17535,7 +17535,7 @@
         <v>1140</v>
       </c>
       <c r="I352">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K352" t="s">
         <v>1148</v>
@@ -17573,7 +17573,7 @@
         <v>1140</v>
       </c>
       <c r="I353">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K353" t="s">
         <v>1147</v>
@@ -17611,7 +17611,7 @@
         <v>1140</v>
       </c>
       <c r="I354">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K354" t="s">
         <v>1147</v>
@@ -17649,7 +17649,7 @@
         <v>1140</v>
       </c>
       <c r="I355">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -17731,7 +17731,7 @@
         <v>1140</v>
       </c>
       <c r="I357">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K357" t="s">
         <v>1147</v>
@@ -17769,7 +17769,7 @@
         <v>1140</v>
       </c>
       <c r="I358">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K358" t="s">
         <v>1147</v>
@@ -17807,7 +17807,7 @@
         <v>1140</v>
       </c>
       <c r="I359">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K359" t="s">
         <v>1147</v>
@@ -17848,7 +17848,7 @@
         <v>1140</v>
       </c>
       <c r="I360">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K360" t="s">
         <v>1147</v>
@@ -17886,7 +17886,7 @@
         <v>1140</v>
       </c>
       <c r="I361">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K361" t="s">
         <v>1147</v>
@@ -17924,7 +17924,7 @@
         <v>1140</v>
       </c>
       <c r="I362">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K362" t="s">
         <v>1147</v>
@@ -17962,7 +17962,7 @@
         <v>1140</v>
       </c>
       <c r="I363">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K363" t="s">
         <v>1147</v>
@@ -18000,7 +18000,7 @@
         <v>1140</v>
       </c>
       <c r="I364">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K364" t="s">
         <v>1147</v>
@@ -18038,7 +18038,7 @@
         <v>1140</v>
       </c>
       <c r="I365">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K365" t="s">
         <v>1146</v>
@@ -18076,7 +18076,7 @@
         <v>1140</v>
       </c>
       <c r="I366">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K366" t="s">
         <v>1147</v>
@@ -18114,7 +18114,7 @@
         <v>1140</v>
       </c>
       <c r="I367">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K367" t="s">
         <v>1147</v>
@@ -18152,7 +18152,7 @@
         <v>1140</v>
       </c>
       <c r="I368">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K368" t="s">
         <v>1147</v>
@@ -18190,7 +18190,7 @@
         <v>1140</v>
       </c>
       <c r="I369">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K369" t="s">
         <v>1147</v>
@@ -18228,7 +18228,7 @@
         <v>1140</v>
       </c>
       <c r="I370">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K370" t="s">
         <v>1147</v>
@@ -18266,7 +18266,7 @@
         <v>1140</v>
       </c>
       <c r="I371">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18310,7 +18310,7 @@
         <v>1140</v>
       </c>
       <c r="I372">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18357,7 +18357,7 @@
         <v>1140</v>
       </c>
       <c r="I373">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K373" t="s">
         <v>1143</v>
@@ -18395,7 +18395,7 @@
         <v>1140</v>
       </c>
       <c r="I374">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K374" t="s">
         <v>1143</v>
@@ -18433,7 +18433,7 @@
         <v>1140</v>
       </c>
       <c r="I375">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K375" t="s">
         <v>1147</v>
@@ -18471,7 +18471,7 @@
         <v>1140</v>
       </c>
       <c r="I376">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K376" t="s">
         <v>1147</v>
@@ -18547,7 +18547,7 @@
         <v>1140</v>
       </c>
       <c r="I378">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K378" t="s">
         <v>1147</v>
@@ -18585,7 +18585,7 @@
         <v>1140</v>
       </c>
       <c r="I379">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18629,7 +18629,7 @@
         <v>1140</v>
       </c>
       <c r="I380">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K380" t="s">
         <v>1147</v>
@@ -18667,7 +18667,7 @@
         <v>1140</v>
       </c>
       <c r="I381">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K381" t="s">
         <v>1147</v>
@@ -18705,7 +18705,7 @@
         <v>1140</v>
       </c>
       <c r="I382">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K382" t="s">
         <v>1147</v>
@@ -18743,7 +18743,7 @@
         <v>1140</v>
       </c>
       <c r="I383">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K383" t="s">
         <v>1147</v>
@@ -18781,7 +18781,7 @@
         <v>1140</v>
       </c>
       <c r="I384">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K384" t="s">
         <v>1143</v>
@@ -18819,7 +18819,7 @@
         <v>1140</v>
       </c>
       <c r="I385">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K385" t="s">
         <v>1143</v>
@@ -18857,7 +18857,7 @@
         <v>1140</v>
       </c>
       <c r="I386">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K386" t="s">
         <v>1147</v>
@@ -18895,7 +18895,7 @@
         <v>1140</v>
       </c>
       <c r="I387">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K387" t="s">
         <v>1147</v>
@@ -18933,7 +18933,7 @@
         <v>1140</v>
       </c>
       <c r="I388">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K388" t="s">
         <v>1147</v>
@@ -18971,7 +18971,7 @@
         <v>1140</v>
       </c>
       <c r="I389">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K389" t="s">
         <v>1148</v>
@@ -19009,7 +19009,7 @@
         <v>1140</v>
       </c>
       <c r="I390">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19129,7 +19129,7 @@
         <v>1140</v>
       </c>
       <c r="I393">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K393" t="s">
         <v>1147</v>
@@ -19167,7 +19167,7 @@
         <v>1140</v>
       </c>
       <c r="I394">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K394" t="s">
         <v>1147</v>
@@ -19205,7 +19205,7 @@
         <v>1140</v>
       </c>
       <c r="I395">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K395" t="s">
         <v>1147</v>
@@ -19243,7 +19243,7 @@
         <v>1140</v>
       </c>
       <c r="I396">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K396" t="s">
         <v>1147</v>
@@ -19281,7 +19281,7 @@
         <v>1140</v>
       </c>
       <c r="I397">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K397" t="s">
         <v>1147</v>
@@ -19319,7 +19319,7 @@
         <v>1140</v>
       </c>
       <c r="I398">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K398" t="s">
         <v>1147</v>
@@ -19395,7 +19395,7 @@
         <v>1140</v>
       </c>
       <c r="I400">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K400" t="s">
         <v>1147</v>
@@ -19433,7 +19433,7 @@
         <v>1140</v>
       </c>
       <c r="I401">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K401" t="s">
         <v>1147</v>
@@ -19471,7 +19471,7 @@
         <v>1140</v>
       </c>
       <c r="I402">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K402" t="s">
         <v>1147</v>
@@ -19509,7 +19509,7 @@
         <v>1140</v>
       </c>
       <c r="I403">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K403" t="s">
         <v>1150</v>
@@ -19544,7 +19544,7 @@
         <v>1140</v>
       </c>
       <c r="I404">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K404" t="s">
         <v>1150</v>
@@ -19608,7 +19608,7 @@
         <v>1140</v>
       </c>
       <c r="I406">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19640,7 +19640,7 @@
         <v>1140</v>
       </c>
       <c r="I407">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19672,7 +19672,7 @@
         <v>1140</v>
       </c>
       <c r="I408">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19704,7 +19704,7 @@
         <v>1140</v>
       </c>
       <c r="I409">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -19736,7 +19736,7 @@
         <v>1140</v>
       </c>
       <c r="I410">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -19768,7 +19768,7 @@
         <v>1140</v>
       </c>
       <c r="I411">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -19800,7 +19800,7 @@
         <v>1140</v>
       </c>
       <c r="I412">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -19832,7 +19832,7 @@
         <v>1140</v>
       </c>
       <c r="I413">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -19864,7 +19864,7 @@
         <v>1140</v>
       </c>
       <c r="I414">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -19896,7 +19896,7 @@
         <v>1140</v>
       </c>
       <c r="I415">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -19928,7 +19928,7 @@
         <v>1140</v>
       </c>
       <c r="I416">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -19960,7 +19960,7 @@
         <v>1140</v>
       </c>
       <c r="I417">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -19992,7 +19992,7 @@
         <v>1140</v>
       </c>
       <c r="I418">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20024,7 +20024,7 @@
         <v>1140</v>
       </c>
       <c r="I419">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20056,7 +20056,7 @@
         <v>1140</v>
       </c>
       <c r="I420">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20088,7 +20088,7 @@
         <v>1140</v>
       </c>
       <c r="I421">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20120,7 +20120,7 @@
         <v>1140</v>
       </c>
       <c r="I422">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20152,7 +20152,7 @@
         <v>1140</v>
       </c>
       <c r="I423">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20184,7 +20184,7 @@
         <v>1140</v>
       </c>
       <c r="I424">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20216,7 +20216,7 @@
         <v>1140</v>
       </c>
       <c r="I425">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20248,7 +20248,7 @@
         <v>1140</v>
       </c>
       <c r="I426">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20280,7 +20280,7 @@
         <v>1140</v>
       </c>
       <c r="I427">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20312,7 +20312,7 @@
         <v>1140</v>
       </c>
       <c r="I428">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20344,7 +20344,7 @@
         <v>1140</v>
       </c>
       <c r="I429">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20376,7 +20376,7 @@
         <v>1140</v>
       </c>
       <c r="I430">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20408,7 +20408,7 @@
         <v>1140</v>
       </c>
       <c r="I431">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20440,7 +20440,7 @@
         <v>1140</v>
       </c>
       <c r="I432">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20472,7 +20472,7 @@
         <v>1140</v>
       </c>
       <c r="I433">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20504,7 +20504,7 @@
         <v>1140</v>
       </c>
       <c r="I434">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20536,7 +20536,7 @@
         <v>1140</v>
       </c>
       <c r="I435">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20568,7 +20568,7 @@
         <v>1140</v>
       </c>
       <c r="I436">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20600,7 +20600,7 @@
         <v>1142</v>
       </c>
       <c r="I437">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20632,7 +20632,7 @@
         <v>1142</v>
       </c>
       <c r="I438">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20664,7 +20664,7 @@
         <v>1140</v>
       </c>
       <c r="I439">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20696,7 +20696,7 @@
         <v>1140</v>
       </c>
       <c r="I440">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -20728,7 +20728,7 @@
         <v>1140</v>
       </c>
       <c r="I441">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -20760,7 +20760,7 @@
         <v>1140</v>
       </c>
       <c r="I442">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -20792,7 +20792,7 @@
         <v>1140</v>
       </c>
       <c r="I443">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -20824,7 +20824,7 @@
         <v>1140</v>
       </c>
       <c r="I444">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -20856,7 +20856,7 @@
         <v>1140</v>
       </c>
       <c r="I445">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -20888,7 +20888,7 @@
         <v>1140</v>
       </c>
       <c r="I446">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -20920,7 +20920,7 @@
         <v>1140</v>
       </c>
       <c r="I447">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (30/07/2026 13:20)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4253,7 +4253,7 @@
         <v>1140</v>
       </c>
       <c r="I2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K2" t="s">
         <v>1143</v>
@@ -4291,7 +4291,7 @@
         <v>1140</v>
       </c>
       <c r="I3">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K3" t="s">
         <v>1144</v>
@@ -4329,7 +4329,7 @@
         <v>1140</v>
       </c>
       <c r="I4">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K4" t="s">
         <v>1144</v>
@@ -4367,7 +4367,7 @@
         <v>1140</v>
       </c>
       <c r="I5">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4411,7 +4411,7 @@
         <v>1140</v>
       </c>
       <c r="I6">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4455,7 +4455,7 @@
         <v>1140</v>
       </c>
       <c r="I7">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4531,7 +4531,7 @@
         <v>1140</v>
       </c>
       <c r="I9">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4578,7 +4578,7 @@
         <v>1140</v>
       </c>
       <c r="I10">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4625,7 +4625,7 @@
         <v>1140</v>
       </c>
       <c r="I11">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4672,7 +4672,7 @@
         <v>1140</v>
       </c>
       <c r="I12">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -4751,7 +4751,7 @@
         <v>1140</v>
       </c>
       <c r="I14">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -4795,7 +4795,7 @@
         <v>1140</v>
       </c>
       <c r="I15">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K15" t="s">
         <v>1146</v>
@@ -4833,7 +4833,7 @@
         <v>1140</v>
       </c>
       <c r="I16">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K16" t="s">
         <v>1143</v>
@@ -4871,7 +4871,7 @@
         <v>1140</v>
       </c>
       <c r="I17">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -4915,7 +4915,7 @@
         <v>1140</v>
       </c>
       <c r="I18">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -4994,7 +4994,7 @@
         <v>1140</v>
       </c>
       <c r="I20">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5073,7 +5073,7 @@
         <v>1140</v>
       </c>
       <c r="I22">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K22" t="s">
         <v>1147</v>
@@ -5111,7 +5111,7 @@
         <v>1140</v>
       </c>
       <c r="I23">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5234,7 +5234,7 @@
         <v>1140</v>
       </c>
       <c r="I26">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5281,7 +5281,7 @@
         <v>1140</v>
       </c>
       <c r="I27">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K27" t="s">
         <v>1147</v>
@@ -5386,7 +5386,7 @@
         <v>1140</v>
       </c>
       <c r="I30">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5468,7 +5468,7 @@
         <v>1140</v>
       </c>
       <c r="I32">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K32" t="s">
         <v>1143</v>
@@ -5710,7 +5710,7 @@
         <v>1140</v>
       </c>
       <c r="I39">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K39" t="s">
         <v>1148</v>
@@ -5745,7 +5745,7 @@
         <v>1140</v>
       </c>
       <c r="I40">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K40" t="s">
         <v>1146</v>
@@ -5894,7 +5894,7 @@
         <v>1140</v>
       </c>
       <c r="I44">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -5941,7 +5941,7 @@
         <v>1140</v>
       </c>
       <c r="I45">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -5988,7 +5988,7 @@
         <v>1140</v>
       </c>
       <c r="I46">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K46" t="s">
         <v>1147</v>
@@ -6026,7 +6026,7 @@
         <v>1140</v>
       </c>
       <c r="I47">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6073,7 +6073,7 @@
         <v>1140</v>
       </c>
       <c r="I48">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K48" t="s">
         <v>1147</v>
@@ -6143,7 +6143,7 @@
         <v>1140</v>
       </c>
       <c r="I50">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K50" t="s">
         <v>1147</v>
@@ -6219,7 +6219,7 @@
         <v>1140</v>
       </c>
       <c r="I52">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K52" t="s">
         <v>1143</v>
@@ -6257,7 +6257,7 @@
         <v>1140</v>
       </c>
       <c r="I53">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K53" t="s">
         <v>1144</v>
@@ -6295,7 +6295,7 @@
         <v>1140</v>
       </c>
       <c r="I54">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K54" t="s">
         <v>1144</v>
@@ -6403,7 +6403,7 @@
         <v>1140</v>
       </c>
       <c r="I57">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K57" t="s">
         <v>1147</v>
@@ -6607,7 +6607,7 @@
         <v>1140</v>
       </c>
       <c r="I63">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6654,7 +6654,7 @@
         <v>1140</v>
       </c>
       <c r="I64">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -6885,7 +6885,7 @@
         <v>1140</v>
       </c>
       <c r="I70">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K70" t="s">
         <v>1144</v>
@@ -6923,7 +6923,7 @@
         <v>1140</v>
       </c>
       <c r="I71">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K71" t="s">
         <v>1150</v>
@@ -6993,7 +6993,7 @@
         <v>1140</v>
       </c>
       <c r="I73">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K73" t="s">
         <v>1143</v>
@@ -7069,7 +7069,7 @@
         <v>1140</v>
       </c>
       <c r="I75">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K75" t="s">
         <v>1144</v>
@@ -7107,7 +7107,7 @@
         <v>1140</v>
       </c>
       <c r="I76">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K76" t="s">
         <v>1150</v>
@@ -7215,7 +7215,7 @@
         <v>1140</v>
       </c>
       <c r="I79">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K79" t="s">
         <v>1150</v>
@@ -7250,7 +7250,7 @@
         <v>1140</v>
       </c>
       <c r="I80">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K80" t="s">
         <v>1144</v>
@@ -7326,7 +7326,7 @@
         <v>1140</v>
       </c>
       <c r="I82">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K82" t="s">
         <v>1147</v>
@@ -7399,7 +7399,7 @@
         <v>1140</v>
       </c>
       <c r="I84">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7446,7 +7446,7 @@
         <v>1140</v>
       </c>
       <c r="I85">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K85" t="s">
         <v>1144</v>
@@ -7484,7 +7484,7 @@
         <v>1140</v>
       </c>
       <c r="I86">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K86" t="s">
         <v>1144</v>
@@ -7522,7 +7522,7 @@
         <v>1140</v>
       </c>
       <c r="I87">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7639,7 +7639,7 @@
         <v>1140</v>
       </c>
       <c r="I90">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K90" t="s">
         <v>1117</v>
@@ -7680,7 +7680,7 @@
         <v>1140</v>
       </c>
       <c r="I91">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K91" t="s">
         <v>1146</v>
@@ -7747,7 +7747,7 @@
         <v>1140</v>
       </c>
       <c r="I93">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K93" t="s">
         <v>1146</v>
@@ -7785,7 +7785,7 @@
         <v>1140</v>
       </c>
       <c r="I94">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K94" t="s">
         <v>1147</v>
@@ -7823,7 +7823,7 @@
         <v>1140</v>
       </c>
       <c r="I95">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K95" t="s">
         <v>1146</v>
@@ -7861,7 +7861,7 @@
         <v>1140</v>
       </c>
       <c r="I96">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -7908,7 +7908,7 @@
         <v>1140</v>
       </c>
       <c r="I97">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K97" t="s">
         <v>1117</v>
@@ -7949,7 +7949,7 @@
         <v>1140</v>
       </c>
       <c r="I98">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K98" t="s">
         <v>1147</v>
@@ -8016,7 +8016,7 @@
         <v>1140</v>
       </c>
       <c r="I100">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K100" t="s">
         <v>1146</v>
@@ -8144,7 +8144,7 @@
         <v>1140</v>
       </c>
       <c r="I104">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K104" t="s">
         <v>1146</v>
@@ -8182,7 +8182,7 @@
         <v>1140</v>
       </c>
       <c r="I105">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K105" t="s">
         <v>1146</v>
@@ -8220,7 +8220,7 @@
         <v>1140</v>
       </c>
       <c r="I106">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8264,7 +8264,7 @@
         <v>1140</v>
       </c>
       <c r="I107">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8308,7 +8308,7 @@
         <v>1140</v>
       </c>
       <c r="I108">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K108" t="s">
         <v>1144</v>
@@ -8346,7 +8346,7 @@
         <v>1140</v>
       </c>
       <c r="I109">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K109" t="s">
         <v>1144</v>
@@ -8562,7 +8562,7 @@
         <v>1140</v>
       </c>
       <c r="I115">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K115" t="s">
         <v>1144</v>
@@ -8600,7 +8600,7 @@
         <v>1140</v>
       </c>
       <c r="I116">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K116" t="s">
         <v>1144</v>
@@ -8638,7 +8638,7 @@
         <v>1140</v>
       </c>
       <c r="I117">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K117" t="s">
         <v>1144</v>
@@ -8676,7 +8676,7 @@
         <v>1140</v>
       </c>
       <c r="I118">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K118" t="s">
         <v>1144</v>
@@ -8714,7 +8714,7 @@
         <v>1140</v>
       </c>
       <c r="I119">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K119" t="s">
         <v>1144</v>
@@ -8752,7 +8752,7 @@
         <v>1140</v>
       </c>
       <c r="I120">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K120" t="s">
         <v>1144</v>
@@ -8790,7 +8790,7 @@
         <v>1140</v>
       </c>
       <c r="I121">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -8837,7 +8837,7 @@
         <v>1140</v>
       </c>
       <c r="I122">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K122" t="s">
         <v>1144</v>
@@ -8904,7 +8904,7 @@
         <v>1140</v>
       </c>
       <c r="I124">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K124" t="s">
         <v>1144</v>
@@ -8942,7 +8942,7 @@
         <v>1140</v>
       </c>
       <c r="I125">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K125" t="s">
         <v>1150</v>
@@ -9047,7 +9047,7 @@
         <v>1140</v>
       </c>
       <c r="I128">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K128" t="s">
         <v>1144</v>
@@ -9085,7 +9085,7 @@
         <v>1140</v>
       </c>
       <c r="I129">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K129" t="s">
         <v>1143</v>
@@ -9123,7 +9123,7 @@
         <v>1140</v>
       </c>
       <c r="I130">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9205,7 +9205,7 @@
         <v>1140</v>
       </c>
       <c r="I132">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9281,7 +9281,7 @@
         <v>1140</v>
       </c>
       <c r="I134">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K134" t="s">
         <v>1143</v>
@@ -9412,7 +9412,7 @@
         <v>1140</v>
       </c>
       <c r="I138">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K138" t="s">
         <v>1144</v>
@@ -9741,7 +9741,7 @@
         <v>1140</v>
       </c>
       <c r="I148">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K148" t="s">
         <v>1144</v>
@@ -9779,7 +9779,7 @@
         <v>1140</v>
       </c>
       <c r="I149">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K149" t="s">
         <v>1150</v>
@@ -9814,7 +9814,7 @@
         <v>1140</v>
       </c>
       <c r="I150">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -9899,7 +9899,7 @@
         <v>1140</v>
       </c>
       <c r="I152">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -9943,7 +9943,7 @@
         <v>1140</v>
       </c>
       <c r="I153">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K153" t="s">
         <v>1144</v>
@@ -10016,7 +10016,7 @@
         <v>1140</v>
       </c>
       <c r="I155">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K155" t="s">
         <v>1150</v>
@@ -10051,7 +10051,7 @@
         <v>1140</v>
       </c>
       <c r="I156">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K156" t="s">
         <v>1144</v>
@@ -10089,7 +10089,7 @@
         <v>1140</v>
       </c>
       <c r="I157">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K157" t="s">
         <v>1146</v>
@@ -10127,7 +10127,7 @@
         <v>1140</v>
       </c>
       <c r="I158">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10171,7 +10171,7 @@
         <v>1140</v>
       </c>
       <c r="I159">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K159" t="s">
         <v>1144</v>
@@ -10209,7 +10209,7 @@
         <v>1140</v>
       </c>
       <c r="I160">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K160" t="s">
         <v>1144</v>
@@ -10247,7 +10247,7 @@
         <v>1140</v>
       </c>
       <c r="I161">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10294,7 +10294,7 @@
         <v>1140</v>
       </c>
       <c r="I162">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10338,7 +10338,7 @@
         <v>1140</v>
       </c>
       <c r="I163">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10382,7 +10382,7 @@
         <v>1142</v>
       </c>
       <c r="I164">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K164" t="s">
         <v>1151</v>
@@ -10417,7 +10417,7 @@
         <v>1140</v>
       </c>
       <c r="I165">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K165" t="s">
         <v>1144</v>
@@ -10525,7 +10525,7 @@
         <v>1140</v>
       </c>
       <c r="I168">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K168" t="s">
         <v>1147</v>
@@ -10566,7 +10566,7 @@
         <v>1140</v>
       </c>
       <c r="I169">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10648,7 +10648,7 @@
         <v>1140</v>
       </c>
       <c r="I171">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K171" t="s">
         <v>1144</v>
@@ -10794,7 +10794,7 @@
         <v>1140</v>
       </c>
       <c r="I175">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -10841,7 +10841,7 @@
         <v>1140</v>
       </c>
       <c r="I176">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K176" t="s">
         <v>1144</v>
@@ -10879,7 +10879,7 @@
         <v>1140</v>
       </c>
       <c r="I177">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -10926,7 +10926,7 @@
         <v>1140</v>
       </c>
       <c r="I178">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K178" t="s">
         <v>1143</v>
@@ -10993,7 +10993,7 @@
         <v>1140</v>
       </c>
       <c r="I180">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K180" t="s">
         <v>1143</v>
@@ -11098,7 +11098,7 @@
         <v>1140</v>
       </c>
       <c r="I183">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K183" t="s">
         <v>1144</v>
@@ -11133,7 +11133,7 @@
         <v>1140</v>
       </c>
       <c r="I184">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K184" t="s">
         <v>1150</v>
@@ -11168,7 +11168,7 @@
         <v>1140</v>
       </c>
       <c r="I185">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K185" t="s">
         <v>1144</v>
@@ -11206,7 +11206,7 @@
         <v>1140</v>
       </c>
       <c r="I186">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K186" t="s">
         <v>1144</v>
@@ -11244,7 +11244,7 @@
         <v>1140</v>
       </c>
       <c r="I187">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11291,7 +11291,7 @@
         <v>1140</v>
       </c>
       <c r="I188">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11338,7 +11338,7 @@
         <v>1140</v>
       </c>
       <c r="I189">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11382,7 +11382,7 @@
         <v>1140</v>
       </c>
       <c r="I190">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K190" t="s">
         <v>1146</v>
@@ -11420,7 +11420,7 @@
         <v>1140</v>
       </c>
       <c r="I191">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11464,7 +11464,7 @@
         <v>1140</v>
       </c>
       <c r="I192">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K192" t="s">
         <v>1144</v>
@@ -11502,7 +11502,7 @@
         <v>1140</v>
       </c>
       <c r="I193">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K193" t="s">
         <v>1149</v>
@@ -11572,7 +11572,7 @@
         <v>1140</v>
       </c>
       <c r="I195">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K195" t="s">
         <v>1146</v>
@@ -11706,7 +11706,7 @@
         <v>1140</v>
       </c>
       <c r="I199">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -11750,7 +11750,7 @@
         <v>1140</v>
       </c>
       <c r="I200">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K200" t="s">
         <v>1146</v>
@@ -11788,7 +11788,7 @@
         <v>1140</v>
       </c>
       <c r="I201">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K201" t="s">
         <v>1144</v>
@@ -11826,7 +11826,7 @@
         <v>1140</v>
       </c>
       <c r="I202">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K202" t="s">
         <v>1144</v>
@@ -11864,7 +11864,7 @@
         <v>1140</v>
       </c>
       <c r="I203">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K203" t="s">
         <v>1144</v>
@@ -11902,7 +11902,7 @@
         <v>1140</v>
       </c>
       <c r="I204">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K204" t="s">
         <v>1143</v>
@@ -11940,7 +11940,7 @@
         <v>1140</v>
       </c>
       <c r="I205">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K205" t="s">
         <v>1143</v>
@@ -12013,7 +12013,7 @@
         <v>1140</v>
       </c>
       <c r="I207">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12057,7 +12057,7 @@
         <v>1140</v>
       </c>
       <c r="I208">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12101,7 +12101,7 @@
         <v>1140</v>
       </c>
       <c r="I209">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12145,7 +12145,7 @@
         <v>1140</v>
       </c>
       <c r="I210">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K210" t="s">
         <v>1147</v>
@@ -12253,7 +12253,7 @@
         <v>1140</v>
       </c>
       <c r="I213">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K213" t="s">
         <v>1144</v>
@@ -12291,7 +12291,7 @@
         <v>1140</v>
       </c>
       <c r="I214">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12338,7 +12338,7 @@
         <v>1140</v>
       </c>
       <c r="I215">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K215" t="s">
         <v>1144</v>
@@ -12405,7 +12405,7 @@
         <v>1140</v>
       </c>
       <c r="I217">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12449,7 +12449,7 @@
         <v>1140</v>
       </c>
       <c r="I218">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K218" t="s">
         <v>1146</v>
@@ -12487,7 +12487,7 @@
         <v>1140</v>
       </c>
       <c r="I219">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K219" t="s">
         <v>1146</v>
@@ -12525,7 +12525,7 @@
         <v>1140</v>
       </c>
       <c r="I220">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K220" t="s">
         <v>1146</v>
@@ -12601,7 +12601,7 @@
         <v>1140</v>
       </c>
       <c r="I222">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K222" t="s">
         <v>1144</v>
@@ -12639,7 +12639,7 @@
         <v>1140</v>
       </c>
       <c r="I223">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K223" t="s">
         <v>1144</v>
@@ -12677,7 +12677,7 @@
         <v>1140</v>
       </c>
       <c r="I224">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K224" t="s">
         <v>1144</v>
@@ -12715,7 +12715,7 @@
         <v>1140</v>
       </c>
       <c r="I225">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K225" t="s">
         <v>1144</v>
@@ -12753,7 +12753,7 @@
         <v>1140</v>
       </c>
       <c r="I226">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K226" t="s">
         <v>1144</v>
@@ -12791,7 +12791,7 @@
         <v>1140</v>
       </c>
       <c r="I227">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K227" t="s">
         <v>1144</v>
@@ -12829,7 +12829,7 @@
         <v>1140</v>
       </c>
       <c r="I228">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K228" t="s">
         <v>1144</v>
@@ -12902,7 +12902,7 @@
         <v>1140</v>
       </c>
       <c r="I230">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K230" t="s">
         <v>1147</v>
@@ -12940,7 +12940,7 @@
         <v>1140</v>
       </c>
       <c r="I231">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13054,7 +13054,7 @@
         <v>1140</v>
       </c>
       <c r="I234">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13101,7 +13101,7 @@
         <v>1140</v>
       </c>
       <c r="I235">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13148,7 +13148,7 @@
         <v>1140</v>
       </c>
       <c r="I236">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13192,7 +13192,7 @@
         <v>1140</v>
       </c>
       <c r="I237">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K237" t="s">
         <v>1144</v>
@@ -13259,7 +13259,7 @@
         <v>1140</v>
       </c>
       <c r="I239">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K239" t="s">
         <v>1117</v>
@@ -13370,7 +13370,7 @@
         <v>1140</v>
       </c>
       <c r="I242">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K242" t="s">
         <v>1143</v>
@@ -13440,7 +13440,7 @@
         <v>1140</v>
       </c>
       <c r="I244">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K244" t="s">
         <v>1146</v>
@@ -13478,7 +13478,7 @@
         <v>1140</v>
       </c>
       <c r="I245">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K245" t="s">
         <v>1146</v>
@@ -13516,7 +13516,7 @@
         <v>1140</v>
       </c>
       <c r="I246">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13621,7 +13621,7 @@
         <v>1140</v>
       </c>
       <c r="I249">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K249" t="s">
         <v>1144</v>
@@ -13659,7 +13659,7 @@
         <v>1140</v>
       </c>
       <c r="I250">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K250" t="s">
         <v>1146</v>
@@ -13767,7 +13767,7 @@
         <v>1140</v>
       </c>
       <c r="I253">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K253" t="s">
         <v>1147</v>
@@ -13805,7 +13805,7 @@
         <v>1140</v>
       </c>
       <c r="I254">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K254" t="s">
         <v>1147</v>
@@ -13843,7 +13843,7 @@
         <v>1140</v>
       </c>
       <c r="I255">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K255" t="s">
         <v>1146</v>
@@ -13881,7 +13881,7 @@
         <v>1140</v>
       </c>
       <c r="I256">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K256" t="s">
         <v>1144</v>
@@ -13980,7 +13980,7 @@
         <v>1140</v>
       </c>
       <c r="I259">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K259" t="s">
         <v>1146</v>
@@ -14018,7 +14018,7 @@
         <v>1140</v>
       </c>
       <c r="I260">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K260" t="s">
         <v>1146</v>
@@ -14056,7 +14056,7 @@
         <v>1140</v>
       </c>
       <c r="I261">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K261" t="s">
         <v>1147</v>
@@ -14094,7 +14094,7 @@
         <v>1140</v>
       </c>
       <c r="I262">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14179,7 +14179,7 @@
         <v>1140</v>
       </c>
       <c r="I264">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K264" t="s">
         <v>1147</v>
@@ -14217,7 +14217,7 @@
         <v>1140</v>
       </c>
       <c r="I265">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K265" t="s">
         <v>1147</v>
@@ -14255,7 +14255,7 @@
         <v>1140</v>
       </c>
       <c r="I266">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K266" t="s">
         <v>1146</v>
@@ -14293,7 +14293,7 @@
         <v>1140</v>
       </c>
       <c r="I267">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K267" t="s">
         <v>1147</v>
@@ -14331,7 +14331,7 @@
         <v>1140</v>
       </c>
       <c r="I268">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K268" t="s">
         <v>1144</v>
@@ -14366,7 +14366,7 @@
         <v>1140</v>
       </c>
       <c r="I269">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K269" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1140</v>
       </c>
       <c r="I270">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K270" t="s">
         <v>1147</v>
@@ -14442,7 +14442,7 @@
         <v>1140</v>
       </c>
       <c r="I271">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K271" t="s">
         <v>1147</v>
@@ -14480,7 +14480,7 @@
         <v>1140</v>
       </c>
       <c r="I272">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14562,7 +14562,7 @@
         <v>1140</v>
       </c>
       <c r="I274">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K274" t="s">
         <v>1144</v>
@@ -14635,7 +14635,7 @@
         <v>1140</v>
       </c>
       <c r="I276">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K276" t="s">
         <v>1148</v>
@@ -14673,7 +14673,7 @@
         <v>1140</v>
       </c>
       <c r="I277">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K277" t="s">
         <v>1144</v>
@@ -14711,7 +14711,7 @@
         <v>1140</v>
       </c>
       <c r="I278">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K278" t="s">
         <v>1147</v>
@@ -14749,7 +14749,7 @@
         <v>1140</v>
       </c>
       <c r="I279">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K279" t="s">
         <v>1146</v>
@@ -14790,7 +14790,7 @@
         <v>1140</v>
       </c>
       <c r="I280">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K280" t="s">
         <v>1144</v>
@@ -14828,7 +14828,7 @@
         <v>1140</v>
       </c>
       <c r="I281">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K281" t="s">
         <v>1144</v>
@@ -14866,7 +14866,7 @@
         <v>1140</v>
       </c>
       <c r="I282">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="K282" t="s">
         <v>1144</v>
@@ -15073,7 +15073,7 @@
         <v>1140</v>
       </c>
       <c r="I288">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K288" t="s">
         <v>1147</v>
@@ -15140,7 +15140,7 @@
         <v>1140</v>
       </c>
       <c r="I290">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15181,7 +15181,7 @@
         <v>1140</v>
       </c>
       <c r="I291">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K291" t="s">
         <v>1146</v>
@@ -15219,7 +15219,7 @@
         <v>1140</v>
       </c>
       <c r="I292">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K292" t="s">
         <v>1147</v>
@@ -15257,7 +15257,7 @@
         <v>1140</v>
       </c>
       <c r="I293">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K293" t="s">
         <v>1148</v>
@@ -15295,7 +15295,7 @@
         <v>1140</v>
       </c>
       <c r="I294">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K294" t="s">
         <v>1150</v>
@@ -15330,7 +15330,7 @@
         <v>1140</v>
       </c>
       <c r="I295">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K295" t="s">
         <v>1150</v>
@@ -15365,7 +15365,7 @@
         <v>1140</v>
       </c>
       <c r="I296">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K296" t="s">
         <v>1150</v>
@@ -15435,7 +15435,7 @@
         <v>1140</v>
       </c>
       <c r="I298">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K298" t="s">
         <v>1144</v>
@@ -15473,7 +15473,7 @@
         <v>1140</v>
       </c>
       <c r="I299">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K299" t="s">
         <v>1147</v>
@@ -15511,7 +15511,7 @@
         <v>1140</v>
       </c>
       <c r="I300">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K300" t="s">
         <v>1147</v>
@@ -15549,7 +15549,7 @@
         <v>1140</v>
       </c>
       <c r="I301">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K301" t="s">
         <v>1147</v>
@@ -15587,7 +15587,7 @@
         <v>1140</v>
       </c>
       <c r="I302">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K302" t="s">
         <v>1147</v>
@@ -15625,7 +15625,7 @@
         <v>1140</v>
       </c>
       <c r="I303">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K303" t="s">
         <v>1144</v>
@@ -15663,7 +15663,7 @@
         <v>1140</v>
       </c>
       <c r="I304">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K304" t="s">
         <v>1147</v>
@@ -15701,7 +15701,7 @@
         <v>1140</v>
       </c>
       <c r="I305">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -15745,7 +15745,7 @@
         <v>1140</v>
       </c>
       <c r="I306">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -15789,7 +15789,7 @@
         <v>1140</v>
       </c>
       <c r="I307">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K307" t="s">
         <v>1143</v>
@@ -15827,7 +15827,7 @@
         <v>1140</v>
       </c>
       <c r="I308">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K308" t="s">
         <v>1143</v>
@@ -15865,7 +15865,7 @@
         <v>1140</v>
       </c>
       <c r="I309">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K309" t="s">
         <v>1143</v>
@@ -15903,7 +15903,7 @@
         <v>1140</v>
       </c>
       <c r="I310">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K310" t="s">
         <v>1144</v>
@@ -15941,7 +15941,7 @@
         <v>1140</v>
       </c>
       <c r="I311">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K311" t="s">
         <v>1143</v>
@@ -15979,7 +15979,7 @@
         <v>1140</v>
       </c>
       <c r="I312">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K312" t="s">
         <v>1144</v>
@@ -16052,7 +16052,7 @@
         <v>1140</v>
       </c>
       <c r="I314">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K314" t="s">
         <v>1144</v>
@@ -16090,7 +16090,7 @@
         <v>1140</v>
       </c>
       <c r="I315">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K315" t="s">
         <v>1144</v>
@@ -16128,7 +16128,7 @@
         <v>1140</v>
       </c>
       <c r="I316">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K316" t="s">
         <v>1144</v>
@@ -16166,7 +16166,7 @@
         <v>1140</v>
       </c>
       <c r="I317">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K317" t="s">
         <v>1144</v>
@@ -16277,7 +16277,7 @@
         <v>1140</v>
       </c>
       <c r="I320">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K320" t="s">
         <v>1148</v>
@@ -16315,7 +16315,7 @@
         <v>1140</v>
       </c>
       <c r="I321">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K321" t="s">
         <v>1144</v>
@@ -16353,7 +16353,7 @@
         <v>1140</v>
       </c>
       <c r="I322">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16397,7 +16397,7 @@
         <v>1140</v>
       </c>
       <c r="I323">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K323" t="s">
         <v>1144</v>
@@ -16435,7 +16435,7 @@
         <v>1140</v>
       </c>
       <c r="I324">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K324" t="s">
         <v>1144</v>
@@ -16473,7 +16473,7 @@
         <v>1140</v>
       </c>
       <c r="I325">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16517,7 +16517,7 @@
         <v>1140</v>
       </c>
       <c r="I326">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K326" t="s">
         <v>1144</v>
@@ -16555,7 +16555,7 @@
         <v>1140</v>
       </c>
       <c r="I327">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16599,7 +16599,7 @@
         <v>1140</v>
       </c>
       <c r="I328">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16643,7 +16643,7 @@
         <v>1140</v>
       </c>
       <c r="I329">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16687,7 +16687,7 @@
         <v>1140</v>
       </c>
       <c r="I330">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -16731,7 +16731,7 @@
         <v>1140</v>
       </c>
       <c r="I331">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K331" t="s">
         <v>1143</v>
@@ -16769,7 +16769,7 @@
         <v>1140</v>
       </c>
       <c r="I332">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K332" t="s">
         <v>1144</v>
@@ -16807,7 +16807,7 @@
         <v>1140</v>
       </c>
       <c r="I333">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K333" t="s">
         <v>1147</v>
@@ -16845,7 +16845,7 @@
         <v>1140</v>
       </c>
       <c r="I334">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K334" t="s">
         <v>1144</v>
@@ -16924,7 +16924,7 @@
         <v>1140</v>
       </c>
       <c r="I336">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K336" t="s">
         <v>1146</v>
@@ -17003,7 +17003,7 @@
         <v>1140</v>
       </c>
       <c r="I338">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K338" t="s">
         <v>1146</v>
@@ -17070,7 +17070,7 @@
         <v>1140</v>
       </c>
       <c r="I340">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K340" t="s">
         <v>1143</v>
@@ -17108,7 +17108,7 @@
         <v>1140</v>
       </c>
       <c r="I341">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K341" t="s">
         <v>1143</v>
@@ -17146,7 +17146,7 @@
         <v>1140</v>
       </c>
       <c r="I342">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K342" t="s">
         <v>1143</v>
@@ -17184,7 +17184,7 @@
         <v>1140</v>
       </c>
       <c r="I343">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K343" t="s">
         <v>1144</v>
@@ -17222,7 +17222,7 @@
         <v>1140</v>
       </c>
       <c r="I344">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K344" t="s">
         <v>1144</v>
@@ -17260,7 +17260,7 @@
         <v>1140</v>
       </c>
       <c r="I345">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K345" t="s">
         <v>1143</v>
@@ -17298,7 +17298,7 @@
         <v>1140</v>
       </c>
       <c r="I346">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K346" t="s">
         <v>1144</v>
@@ -17336,7 +17336,7 @@
         <v>1140</v>
       </c>
       <c r="I347">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17380,7 +17380,7 @@
         <v>1140</v>
       </c>
       <c r="I348">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17424,7 +17424,7 @@
         <v>1140</v>
       </c>
       <c r="I349">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K349" t="s">
         <v>1148</v>
@@ -17462,7 +17462,7 @@
         <v>1140</v>
       </c>
       <c r="I350">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K350" t="s">
         <v>1150</v>
@@ -17497,7 +17497,7 @@
         <v>1140</v>
       </c>
       <c r="I351">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K351" t="s">
         <v>1148</v>
@@ -17535,7 +17535,7 @@
         <v>1140</v>
       </c>
       <c r="I352">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K352" t="s">
         <v>1148</v>
@@ -17573,7 +17573,7 @@
         <v>1140</v>
       </c>
       <c r="I353">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K353" t="s">
         <v>1147</v>
@@ -17611,7 +17611,7 @@
         <v>1140</v>
       </c>
       <c r="I354">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K354" t="s">
         <v>1147</v>
@@ -17649,7 +17649,7 @@
         <v>1140</v>
       </c>
       <c r="I355">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -17731,7 +17731,7 @@
         <v>1140</v>
       </c>
       <c r="I357">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K357" t="s">
         <v>1147</v>
@@ -17769,7 +17769,7 @@
         <v>1140</v>
       </c>
       <c r="I358">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K358" t="s">
         <v>1147</v>
@@ -17807,7 +17807,7 @@
         <v>1140</v>
       </c>
       <c r="I359">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K359" t="s">
         <v>1147</v>
@@ -17848,7 +17848,7 @@
         <v>1140</v>
       </c>
       <c r="I360">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K360" t="s">
         <v>1147</v>
@@ -17886,7 +17886,7 @@
         <v>1140</v>
       </c>
       <c r="I361">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K361" t="s">
         <v>1147</v>
@@ -17924,7 +17924,7 @@
         <v>1140</v>
       </c>
       <c r="I362">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K362" t="s">
         <v>1147</v>
@@ -17962,7 +17962,7 @@
         <v>1140</v>
       </c>
       <c r="I363">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K363" t="s">
         <v>1147</v>
@@ -18000,7 +18000,7 @@
         <v>1140</v>
       </c>
       <c r="I364">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K364" t="s">
         <v>1147</v>
@@ -18038,7 +18038,7 @@
         <v>1140</v>
       </c>
       <c r="I365">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K365" t="s">
         <v>1146</v>
@@ -18076,7 +18076,7 @@
         <v>1140</v>
       </c>
       <c r="I366">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K366" t="s">
         <v>1147</v>
@@ -18114,7 +18114,7 @@
         <v>1140</v>
       </c>
       <c r="I367">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K367" t="s">
         <v>1147</v>
@@ -18152,7 +18152,7 @@
         <v>1140</v>
       </c>
       <c r="I368">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K368" t="s">
         <v>1147</v>
@@ -18190,7 +18190,7 @@
         <v>1140</v>
       </c>
       <c r="I369">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K369" t="s">
         <v>1147</v>
@@ -18228,7 +18228,7 @@
         <v>1140</v>
       </c>
       <c r="I370">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K370" t="s">
         <v>1147</v>
@@ -18266,7 +18266,7 @@
         <v>1140</v>
       </c>
       <c r="I371">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18310,7 +18310,7 @@
         <v>1140</v>
       </c>
       <c r="I372">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18357,7 +18357,7 @@
         <v>1140</v>
       </c>
       <c r="I373">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K373" t="s">
         <v>1143</v>
@@ -18395,7 +18395,7 @@
         <v>1140</v>
       </c>
       <c r="I374">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K374" t="s">
         <v>1143</v>
@@ -18433,7 +18433,7 @@
         <v>1140</v>
       </c>
       <c r="I375">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K375" t="s">
         <v>1147</v>
@@ -18471,7 +18471,7 @@
         <v>1140</v>
       </c>
       <c r="I376">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K376" t="s">
         <v>1147</v>
@@ -18547,7 +18547,7 @@
         <v>1140</v>
       </c>
       <c r="I378">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K378" t="s">
         <v>1147</v>
@@ -18585,7 +18585,7 @@
         <v>1140</v>
       </c>
       <c r="I379">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18629,7 +18629,7 @@
         <v>1140</v>
       </c>
       <c r="I380">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K380" t="s">
         <v>1147</v>
@@ -18667,7 +18667,7 @@
         <v>1140</v>
       </c>
       <c r="I381">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K381" t="s">
         <v>1147</v>
@@ -18705,7 +18705,7 @@
         <v>1140</v>
       </c>
       <c r="I382">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K382" t="s">
         <v>1147</v>
@@ -18743,7 +18743,7 @@
         <v>1140</v>
       </c>
       <c r="I383">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K383" t="s">
         <v>1147</v>
@@ -18781,7 +18781,7 @@
         <v>1140</v>
       </c>
       <c r="I384">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K384" t="s">
         <v>1143</v>
@@ -18819,7 +18819,7 @@
         <v>1140</v>
       </c>
       <c r="I385">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K385" t="s">
         <v>1143</v>
@@ -18857,7 +18857,7 @@
         <v>1140</v>
       </c>
       <c r="I386">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K386" t="s">
         <v>1147</v>
@@ -18895,7 +18895,7 @@
         <v>1140</v>
       </c>
       <c r="I387">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K387" t="s">
         <v>1147</v>
@@ -18933,7 +18933,7 @@
         <v>1140</v>
       </c>
       <c r="I388">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K388" t="s">
         <v>1147</v>
@@ -18971,7 +18971,7 @@
         <v>1140</v>
       </c>
       <c r="I389">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K389" t="s">
         <v>1148</v>
@@ -19009,7 +19009,7 @@
         <v>1140</v>
       </c>
       <c r="I390">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19129,7 +19129,7 @@
         <v>1140</v>
       </c>
       <c r="I393">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K393" t="s">
         <v>1147</v>
@@ -19167,7 +19167,7 @@
         <v>1140</v>
       </c>
       <c r="I394">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K394" t="s">
         <v>1147</v>
@@ -19205,7 +19205,7 @@
         <v>1140</v>
       </c>
       <c r="I395">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K395" t="s">
         <v>1147</v>
@@ -19243,7 +19243,7 @@
         <v>1140</v>
       </c>
       <c r="I396">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K396" t="s">
         <v>1147</v>
@@ -19281,7 +19281,7 @@
         <v>1140</v>
       </c>
       <c r="I397">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K397" t="s">
         <v>1147</v>
@@ -19319,7 +19319,7 @@
         <v>1140</v>
       </c>
       <c r="I398">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K398" t="s">
         <v>1147</v>
@@ -19395,7 +19395,7 @@
         <v>1140</v>
       </c>
       <c r="I400">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K400" t="s">
         <v>1147</v>
@@ -19433,7 +19433,7 @@
         <v>1140</v>
       </c>
       <c r="I401">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K401" t="s">
         <v>1147</v>
@@ -19471,7 +19471,7 @@
         <v>1140</v>
       </c>
       <c r="I402">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K402" t="s">
         <v>1147</v>
@@ -19509,7 +19509,7 @@
         <v>1140</v>
       </c>
       <c r="I403">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K403" t="s">
         <v>1150</v>
@@ -19544,7 +19544,7 @@
         <v>1140</v>
       </c>
       <c r="I404">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K404" t="s">
         <v>1150</v>
@@ -19608,7 +19608,7 @@
         <v>1140</v>
       </c>
       <c r="I406">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19640,7 +19640,7 @@
         <v>1140</v>
       </c>
       <c r="I407">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19672,7 +19672,7 @@
         <v>1140</v>
       </c>
       <c r="I408">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19704,7 +19704,7 @@
         <v>1140</v>
       </c>
       <c r="I409">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -19736,7 +19736,7 @@
         <v>1140</v>
       </c>
       <c r="I410">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -19768,7 +19768,7 @@
         <v>1140</v>
       </c>
       <c r="I411">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -19800,7 +19800,7 @@
         <v>1140</v>
       </c>
       <c r="I412">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -19832,7 +19832,7 @@
         <v>1140</v>
       </c>
       <c r="I413">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -19864,7 +19864,7 @@
         <v>1140</v>
       </c>
       <c r="I414">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -19896,7 +19896,7 @@
         <v>1140</v>
       </c>
       <c r="I415">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -19928,7 +19928,7 @@
         <v>1140</v>
       </c>
       <c r="I416">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -19960,7 +19960,7 @@
         <v>1140</v>
       </c>
       <c r="I417">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -19992,7 +19992,7 @@
         <v>1140</v>
       </c>
       <c r="I418">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20024,7 +20024,7 @@
         <v>1140</v>
       </c>
       <c r="I419">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20056,7 +20056,7 @@
         <v>1140</v>
       </c>
       <c r="I420">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20088,7 +20088,7 @@
         <v>1140</v>
       </c>
       <c r="I421">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20120,7 +20120,7 @@
         <v>1140</v>
       </c>
       <c r="I422">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20152,7 +20152,7 @@
         <v>1140</v>
       </c>
       <c r="I423">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20184,7 +20184,7 @@
         <v>1140</v>
       </c>
       <c r="I424">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20216,7 +20216,7 @@
         <v>1140</v>
       </c>
       <c r="I425">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20248,7 +20248,7 @@
         <v>1140</v>
       </c>
       <c r="I426">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20280,7 +20280,7 @@
         <v>1140</v>
       </c>
       <c r="I427">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20312,7 +20312,7 @@
         <v>1140</v>
       </c>
       <c r="I428">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20344,7 +20344,7 @@
         <v>1140</v>
       </c>
       <c r="I429">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20376,7 +20376,7 @@
         <v>1140</v>
       </c>
       <c r="I430">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20408,7 +20408,7 @@
         <v>1140</v>
       </c>
       <c r="I431">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20440,7 +20440,7 @@
         <v>1140</v>
       </c>
       <c r="I432">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20472,7 +20472,7 @@
         <v>1140</v>
       </c>
       <c r="I433">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20504,7 +20504,7 @@
         <v>1140</v>
       </c>
       <c r="I434">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20536,7 +20536,7 @@
         <v>1140</v>
       </c>
       <c r="I435">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20568,7 +20568,7 @@
         <v>1140</v>
       </c>
       <c r="I436">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20600,7 +20600,7 @@
         <v>1142</v>
       </c>
       <c r="I437">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20632,7 +20632,7 @@
         <v>1142</v>
       </c>
       <c r="I438">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20664,7 +20664,7 @@
         <v>1140</v>
       </c>
       <c r="I439">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20696,7 +20696,7 @@
         <v>1140</v>
       </c>
       <c r="I440">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -20728,7 +20728,7 @@
         <v>1140</v>
       </c>
       <c r="I441">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -20760,7 +20760,7 @@
         <v>1140</v>
       </c>
       <c r="I442">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -20792,7 +20792,7 @@
         <v>1140</v>
       </c>
       <c r="I443">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -20824,7 +20824,7 @@
         <v>1140</v>
       </c>
       <c r="I444">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -20856,7 +20856,7 @@
         <v>1140</v>
       </c>
       <c r="I445">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -20888,7 +20888,7 @@
         <v>1140</v>
       </c>
       <c r="I446">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -20920,7 +20920,7 @@
         <v>1140</v>
       </c>
       <c r="I447">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (31/07/2026 05:13)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4253,7 +4253,7 @@
         <v>1140</v>
       </c>
       <c r="I2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="K2" t="s">
         <v>1143</v>
@@ -4291,7 +4291,7 @@
         <v>1140</v>
       </c>
       <c r="I3">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K3" t="s">
         <v>1144</v>
@@ -4329,7 +4329,7 @@
         <v>1140</v>
       </c>
       <c r="I4">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K4" t="s">
         <v>1144</v>
@@ -4367,7 +4367,7 @@
         <v>1140</v>
       </c>
       <c r="I5">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4411,7 +4411,7 @@
         <v>1140</v>
       </c>
       <c r="I6">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4455,7 +4455,7 @@
         <v>1140</v>
       </c>
       <c r="I7">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4531,7 +4531,7 @@
         <v>1140</v>
       </c>
       <c r="I9">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4578,7 +4578,7 @@
         <v>1140</v>
       </c>
       <c r="I10">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4625,7 +4625,7 @@
         <v>1140</v>
       </c>
       <c r="I11">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4672,7 +4672,7 @@
         <v>1140</v>
       </c>
       <c r="I12">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -4751,7 +4751,7 @@
         <v>1140</v>
       </c>
       <c r="I14">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -4795,7 +4795,7 @@
         <v>1140</v>
       </c>
       <c r="I15">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K15" t="s">
         <v>1146</v>
@@ -4833,7 +4833,7 @@
         <v>1140</v>
       </c>
       <c r="I16">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K16" t="s">
         <v>1143</v>
@@ -4871,7 +4871,7 @@
         <v>1140</v>
       </c>
       <c r="I17">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -4915,7 +4915,7 @@
         <v>1140</v>
       </c>
       <c r="I18">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -4994,7 +4994,7 @@
         <v>1140</v>
       </c>
       <c r="I20">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5073,7 +5073,7 @@
         <v>1140</v>
       </c>
       <c r="I22">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K22" t="s">
         <v>1147</v>
@@ -5111,7 +5111,7 @@
         <v>1140</v>
       </c>
       <c r="I23">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5234,7 +5234,7 @@
         <v>1140</v>
       </c>
       <c r="I26">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5281,7 +5281,7 @@
         <v>1140</v>
       </c>
       <c r="I27">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K27" t="s">
         <v>1147</v>
@@ -5386,7 +5386,7 @@
         <v>1140</v>
       </c>
       <c r="I30">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5468,7 +5468,7 @@
         <v>1140</v>
       </c>
       <c r="I32">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K32" t="s">
         <v>1143</v>
@@ -5710,7 +5710,7 @@
         <v>1140</v>
       </c>
       <c r="I39">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K39" t="s">
         <v>1148</v>
@@ -5745,7 +5745,7 @@
         <v>1140</v>
       </c>
       <c r="I40">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K40" t="s">
         <v>1146</v>
@@ -5894,7 +5894,7 @@
         <v>1140</v>
       </c>
       <c r="I44">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -5941,7 +5941,7 @@
         <v>1140</v>
       </c>
       <c r="I45">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -5988,7 +5988,7 @@
         <v>1140</v>
       </c>
       <c r="I46">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K46" t="s">
         <v>1147</v>
@@ -6026,7 +6026,7 @@
         <v>1140</v>
       </c>
       <c r="I47">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6073,7 +6073,7 @@
         <v>1140</v>
       </c>
       <c r="I48">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K48" t="s">
         <v>1147</v>
@@ -6143,7 +6143,7 @@
         <v>1140</v>
       </c>
       <c r="I50">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K50" t="s">
         <v>1147</v>
@@ -6219,7 +6219,7 @@
         <v>1140</v>
       </c>
       <c r="I52">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K52" t="s">
         <v>1143</v>
@@ -6257,7 +6257,7 @@
         <v>1140</v>
       </c>
       <c r="I53">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K53" t="s">
         <v>1144</v>
@@ -6295,7 +6295,7 @@
         <v>1140</v>
       </c>
       <c r="I54">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K54" t="s">
         <v>1144</v>
@@ -6403,7 +6403,7 @@
         <v>1140</v>
       </c>
       <c r="I57">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K57" t="s">
         <v>1147</v>
@@ -6607,7 +6607,7 @@
         <v>1140</v>
       </c>
       <c r="I63">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6654,7 +6654,7 @@
         <v>1140</v>
       </c>
       <c r="I64">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -6885,7 +6885,7 @@
         <v>1140</v>
       </c>
       <c r="I70">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K70" t="s">
         <v>1144</v>
@@ -6923,7 +6923,7 @@
         <v>1140</v>
       </c>
       <c r="I71">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K71" t="s">
         <v>1150</v>
@@ -6993,7 +6993,7 @@
         <v>1140</v>
       </c>
       <c r="I73">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K73" t="s">
         <v>1143</v>
@@ -7069,7 +7069,7 @@
         <v>1140</v>
       </c>
       <c r="I75">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K75" t="s">
         <v>1144</v>
@@ -7107,7 +7107,7 @@
         <v>1140</v>
       </c>
       <c r="I76">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K76" t="s">
         <v>1150</v>
@@ -7215,7 +7215,7 @@
         <v>1140</v>
       </c>
       <c r="I79">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K79" t="s">
         <v>1150</v>
@@ -7250,7 +7250,7 @@
         <v>1140</v>
       </c>
       <c r="I80">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K80" t="s">
         <v>1144</v>
@@ -7326,7 +7326,7 @@
         <v>1140</v>
       </c>
       <c r="I82">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K82" t="s">
         <v>1147</v>
@@ -7399,7 +7399,7 @@
         <v>1140</v>
       </c>
       <c r="I84">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7446,7 +7446,7 @@
         <v>1140</v>
       </c>
       <c r="I85">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K85" t="s">
         <v>1144</v>
@@ -7484,7 +7484,7 @@
         <v>1140</v>
       </c>
       <c r="I86">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K86" t="s">
         <v>1144</v>
@@ -7522,7 +7522,7 @@
         <v>1140</v>
       </c>
       <c r="I87">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7639,7 +7639,7 @@
         <v>1140</v>
       </c>
       <c r="I90">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K90" t="s">
         <v>1117</v>
@@ -7680,7 +7680,7 @@
         <v>1140</v>
       </c>
       <c r="I91">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K91" t="s">
         <v>1146</v>
@@ -7747,7 +7747,7 @@
         <v>1140</v>
       </c>
       <c r="I93">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K93" t="s">
         <v>1146</v>
@@ -7785,7 +7785,7 @@
         <v>1140</v>
       </c>
       <c r="I94">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K94" t="s">
         <v>1147</v>
@@ -7823,7 +7823,7 @@
         <v>1140</v>
       </c>
       <c r="I95">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K95" t="s">
         <v>1146</v>
@@ -7861,7 +7861,7 @@
         <v>1140</v>
       </c>
       <c r="I96">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -7908,7 +7908,7 @@
         <v>1140</v>
       </c>
       <c r="I97">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K97" t="s">
         <v>1117</v>
@@ -7949,7 +7949,7 @@
         <v>1140</v>
       </c>
       <c r="I98">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K98" t="s">
         <v>1147</v>
@@ -8016,7 +8016,7 @@
         <v>1140</v>
       </c>
       <c r="I100">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K100" t="s">
         <v>1146</v>
@@ -8144,7 +8144,7 @@
         <v>1140</v>
       </c>
       <c r="I104">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K104" t="s">
         <v>1146</v>
@@ -8182,7 +8182,7 @@
         <v>1140</v>
       </c>
       <c r="I105">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K105" t="s">
         <v>1146</v>
@@ -8220,7 +8220,7 @@
         <v>1140</v>
       </c>
       <c r="I106">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8264,7 +8264,7 @@
         <v>1140</v>
       </c>
       <c r="I107">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8308,7 +8308,7 @@
         <v>1140</v>
       </c>
       <c r="I108">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K108" t="s">
         <v>1144</v>
@@ -8346,7 +8346,7 @@
         <v>1140</v>
       </c>
       <c r="I109">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K109" t="s">
         <v>1144</v>
@@ -8562,7 +8562,7 @@
         <v>1140</v>
       </c>
       <c r="I115">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K115" t="s">
         <v>1144</v>
@@ -8600,7 +8600,7 @@
         <v>1140</v>
       </c>
       <c r="I116">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K116" t="s">
         <v>1144</v>
@@ -8638,7 +8638,7 @@
         <v>1140</v>
       </c>
       <c r="I117">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K117" t="s">
         <v>1144</v>
@@ -8676,7 +8676,7 @@
         <v>1140</v>
       </c>
       <c r="I118">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K118" t="s">
         <v>1144</v>
@@ -8714,7 +8714,7 @@
         <v>1140</v>
       </c>
       <c r="I119">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K119" t="s">
         <v>1144</v>
@@ -8752,7 +8752,7 @@
         <v>1140</v>
       </c>
       <c r="I120">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K120" t="s">
         <v>1144</v>
@@ -8790,7 +8790,7 @@
         <v>1140</v>
       </c>
       <c r="I121">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -8837,7 +8837,7 @@
         <v>1140</v>
       </c>
       <c r="I122">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K122" t="s">
         <v>1144</v>
@@ -8904,7 +8904,7 @@
         <v>1140</v>
       </c>
       <c r="I124">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K124" t="s">
         <v>1144</v>
@@ -8942,7 +8942,7 @@
         <v>1140</v>
       </c>
       <c r="I125">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K125" t="s">
         <v>1150</v>
@@ -9047,7 +9047,7 @@
         <v>1140</v>
       </c>
       <c r="I128">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K128" t="s">
         <v>1144</v>
@@ -9085,7 +9085,7 @@
         <v>1140</v>
       </c>
       <c r="I129">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K129" t="s">
         <v>1143</v>
@@ -9123,7 +9123,7 @@
         <v>1140</v>
       </c>
       <c r="I130">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9205,7 +9205,7 @@
         <v>1140</v>
       </c>
       <c r="I132">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9281,7 +9281,7 @@
         <v>1140</v>
       </c>
       <c r="I134">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K134" t="s">
         <v>1143</v>
@@ -9412,7 +9412,7 @@
         <v>1140</v>
       </c>
       <c r="I138">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K138" t="s">
         <v>1144</v>
@@ -9741,7 +9741,7 @@
         <v>1140</v>
       </c>
       <c r="I148">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K148" t="s">
         <v>1144</v>
@@ -9779,7 +9779,7 @@
         <v>1140</v>
       </c>
       <c r="I149">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K149" t="s">
         <v>1150</v>
@@ -9814,7 +9814,7 @@
         <v>1140</v>
       </c>
       <c r="I150">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -9899,7 +9899,7 @@
         <v>1140</v>
       </c>
       <c r="I152">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -9943,7 +9943,7 @@
         <v>1140</v>
       </c>
       <c r="I153">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K153" t="s">
         <v>1144</v>
@@ -10016,7 +10016,7 @@
         <v>1140</v>
       </c>
       <c r="I155">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K155" t="s">
         <v>1150</v>
@@ -10051,7 +10051,7 @@
         <v>1140</v>
       </c>
       <c r="I156">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K156" t="s">
         <v>1144</v>
@@ -10089,7 +10089,7 @@
         <v>1140</v>
       </c>
       <c r="I157">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K157" t="s">
         <v>1146</v>
@@ -10127,7 +10127,7 @@
         <v>1140</v>
       </c>
       <c r="I158">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10171,7 +10171,7 @@
         <v>1140</v>
       </c>
       <c r="I159">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K159" t="s">
         <v>1144</v>
@@ -10209,7 +10209,7 @@
         <v>1140</v>
       </c>
       <c r="I160">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K160" t="s">
         <v>1144</v>
@@ -10247,7 +10247,7 @@
         <v>1140</v>
       </c>
       <c r="I161">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10294,7 +10294,7 @@
         <v>1140</v>
       </c>
       <c r="I162">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10338,7 +10338,7 @@
         <v>1140</v>
       </c>
       <c r="I163">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10382,7 +10382,7 @@
         <v>1142</v>
       </c>
       <c r="I164">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K164" t="s">
         <v>1151</v>
@@ -10417,7 +10417,7 @@
         <v>1140</v>
       </c>
       <c r="I165">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K165" t="s">
         <v>1144</v>
@@ -10525,7 +10525,7 @@
         <v>1140</v>
       </c>
       <c r="I168">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K168" t="s">
         <v>1147</v>
@@ -10566,7 +10566,7 @@
         <v>1140</v>
       </c>
       <c r="I169">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10648,7 +10648,7 @@
         <v>1140</v>
       </c>
       <c r="I171">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K171" t="s">
         <v>1144</v>
@@ -10794,7 +10794,7 @@
         <v>1140</v>
       </c>
       <c r="I175">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -10841,7 +10841,7 @@
         <v>1140</v>
       </c>
       <c r="I176">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K176" t="s">
         <v>1144</v>
@@ -10879,7 +10879,7 @@
         <v>1140</v>
       </c>
       <c r="I177">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -10926,7 +10926,7 @@
         <v>1140</v>
       </c>
       <c r="I178">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K178" t="s">
         <v>1143</v>
@@ -10993,7 +10993,7 @@
         <v>1140</v>
       </c>
       <c r="I180">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K180" t="s">
         <v>1143</v>
@@ -11098,7 +11098,7 @@
         <v>1140</v>
       </c>
       <c r="I183">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K183" t="s">
         <v>1144</v>
@@ -11133,7 +11133,7 @@
         <v>1140</v>
       </c>
       <c r="I184">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K184" t="s">
         <v>1150</v>
@@ -11168,7 +11168,7 @@
         <v>1140</v>
       </c>
       <c r="I185">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K185" t="s">
         <v>1144</v>
@@ -11206,7 +11206,7 @@
         <v>1140</v>
       </c>
       <c r="I186">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K186" t="s">
         <v>1144</v>
@@ -11244,7 +11244,7 @@
         <v>1140</v>
       </c>
       <c r="I187">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11291,7 +11291,7 @@
         <v>1140</v>
       </c>
       <c r="I188">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11338,7 +11338,7 @@
         <v>1140</v>
       </c>
       <c r="I189">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11382,7 +11382,7 @@
         <v>1140</v>
       </c>
       <c r="I190">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K190" t="s">
         <v>1146</v>
@@ -11420,7 +11420,7 @@
         <v>1140</v>
       </c>
       <c r="I191">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11464,7 +11464,7 @@
         <v>1140</v>
       </c>
       <c r="I192">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K192" t="s">
         <v>1144</v>
@@ -11502,7 +11502,7 @@
         <v>1140</v>
       </c>
       <c r="I193">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K193" t="s">
         <v>1149</v>
@@ -11572,7 +11572,7 @@
         <v>1140</v>
       </c>
       <c r="I195">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K195" t="s">
         <v>1146</v>
@@ -11706,7 +11706,7 @@
         <v>1140</v>
       </c>
       <c r="I199">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -11750,7 +11750,7 @@
         <v>1140</v>
       </c>
       <c r="I200">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K200" t="s">
         <v>1146</v>
@@ -11788,7 +11788,7 @@
         <v>1140</v>
       </c>
       <c r="I201">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K201" t="s">
         <v>1144</v>
@@ -11826,7 +11826,7 @@
         <v>1140</v>
       </c>
       <c r="I202">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K202" t="s">
         <v>1144</v>
@@ -11864,7 +11864,7 @@
         <v>1140</v>
       </c>
       <c r="I203">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K203" t="s">
         <v>1144</v>
@@ -11902,7 +11902,7 @@
         <v>1140</v>
       </c>
       <c r="I204">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K204" t="s">
         <v>1143</v>
@@ -11940,7 +11940,7 @@
         <v>1140</v>
       </c>
       <c r="I205">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K205" t="s">
         <v>1143</v>
@@ -12013,7 +12013,7 @@
         <v>1140</v>
       </c>
       <c r="I207">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12057,7 +12057,7 @@
         <v>1140</v>
       </c>
       <c r="I208">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12101,7 +12101,7 @@
         <v>1140</v>
       </c>
       <c r="I209">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12145,7 +12145,7 @@
         <v>1140</v>
       </c>
       <c r="I210">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K210" t="s">
         <v>1147</v>
@@ -12253,7 +12253,7 @@
         <v>1140</v>
       </c>
       <c r="I213">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K213" t="s">
         <v>1144</v>
@@ -12291,7 +12291,7 @@
         <v>1140</v>
       </c>
       <c r="I214">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12338,7 +12338,7 @@
         <v>1140</v>
       </c>
       <c r="I215">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K215" t="s">
         <v>1144</v>
@@ -12405,7 +12405,7 @@
         <v>1140</v>
       </c>
       <c r="I217">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12449,7 +12449,7 @@
         <v>1140</v>
       </c>
       <c r="I218">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K218" t="s">
         <v>1146</v>
@@ -12487,7 +12487,7 @@
         <v>1140</v>
       </c>
       <c r="I219">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K219" t="s">
         <v>1146</v>
@@ -12525,7 +12525,7 @@
         <v>1140</v>
       </c>
       <c r="I220">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K220" t="s">
         <v>1146</v>
@@ -12601,7 +12601,7 @@
         <v>1140</v>
       </c>
       <c r="I222">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K222" t="s">
         <v>1144</v>
@@ -12639,7 +12639,7 @@
         <v>1140</v>
       </c>
       <c r="I223">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K223" t="s">
         <v>1144</v>
@@ -12677,7 +12677,7 @@
         <v>1140</v>
       </c>
       <c r="I224">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K224" t="s">
         <v>1144</v>
@@ -12715,7 +12715,7 @@
         <v>1140</v>
       </c>
       <c r="I225">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K225" t="s">
         <v>1144</v>
@@ -12753,7 +12753,7 @@
         <v>1140</v>
       </c>
       <c r="I226">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K226" t="s">
         <v>1144</v>
@@ -12791,7 +12791,7 @@
         <v>1140</v>
       </c>
       <c r="I227">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K227" t="s">
         <v>1144</v>
@@ -12829,7 +12829,7 @@
         <v>1140</v>
       </c>
       <c r="I228">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K228" t="s">
         <v>1144</v>
@@ -12902,7 +12902,7 @@
         <v>1140</v>
       </c>
       <c r="I230">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K230" t="s">
         <v>1147</v>
@@ -12940,7 +12940,7 @@
         <v>1140</v>
       </c>
       <c r="I231">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13054,7 +13054,7 @@
         <v>1140</v>
       </c>
       <c r="I234">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13101,7 +13101,7 @@
         <v>1140</v>
       </c>
       <c r="I235">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13148,7 +13148,7 @@
         <v>1140</v>
       </c>
       <c r="I236">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13192,7 +13192,7 @@
         <v>1140</v>
       </c>
       <c r="I237">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K237" t="s">
         <v>1144</v>
@@ -13259,7 +13259,7 @@
         <v>1140</v>
       </c>
       <c r="I239">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K239" t="s">
         <v>1117</v>
@@ -13370,7 +13370,7 @@
         <v>1140</v>
       </c>
       <c r="I242">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K242" t="s">
         <v>1143</v>
@@ -13440,7 +13440,7 @@
         <v>1140</v>
       </c>
       <c r="I244">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K244" t="s">
         <v>1146</v>
@@ -13478,7 +13478,7 @@
         <v>1140</v>
       </c>
       <c r="I245">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K245" t="s">
         <v>1146</v>
@@ -13516,7 +13516,7 @@
         <v>1140</v>
       </c>
       <c r="I246">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13621,7 +13621,7 @@
         <v>1140</v>
       </c>
       <c r="I249">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K249" t="s">
         <v>1144</v>
@@ -13659,7 +13659,7 @@
         <v>1140</v>
       </c>
       <c r="I250">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K250" t="s">
         <v>1146</v>
@@ -13767,7 +13767,7 @@
         <v>1140</v>
       </c>
       <c r="I253">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K253" t="s">
         <v>1147</v>
@@ -13805,7 +13805,7 @@
         <v>1140</v>
       </c>
       <c r="I254">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K254" t="s">
         <v>1147</v>
@@ -13843,7 +13843,7 @@
         <v>1140</v>
       </c>
       <c r="I255">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K255" t="s">
         <v>1146</v>
@@ -13881,7 +13881,7 @@
         <v>1140</v>
       </c>
       <c r="I256">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K256" t="s">
         <v>1144</v>
@@ -13980,7 +13980,7 @@
         <v>1140</v>
       </c>
       <c r="I259">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K259" t="s">
         <v>1146</v>
@@ -14018,7 +14018,7 @@
         <v>1140</v>
       </c>
       <c r="I260">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K260" t="s">
         <v>1146</v>
@@ -14056,7 +14056,7 @@
         <v>1140</v>
       </c>
       <c r="I261">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K261" t="s">
         <v>1147</v>
@@ -14094,7 +14094,7 @@
         <v>1140</v>
       </c>
       <c r="I262">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14179,7 +14179,7 @@
         <v>1140</v>
       </c>
       <c r="I264">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K264" t="s">
         <v>1147</v>
@@ -14217,7 +14217,7 @@
         <v>1140</v>
       </c>
       <c r="I265">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K265" t="s">
         <v>1147</v>
@@ -14255,7 +14255,7 @@
         <v>1140</v>
       </c>
       <c r="I266">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K266" t="s">
         <v>1146</v>
@@ -14293,7 +14293,7 @@
         <v>1140</v>
       </c>
       <c r="I267">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K267" t="s">
         <v>1147</v>
@@ -14331,7 +14331,7 @@
         <v>1140</v>
       </c>
       <c r="I268">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K268" t="s">
         <v>1144</v>
@@ -14366,7 +14366,7 @@
         <v>1140</v>
       </c>
       <c r="I269">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K269" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1140</v>
       </c>
       <c r="I270">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K270" t="s">
         <v>1147</v>
@@ -14442,7 +14442,7 @@
         <v>1140</v>
       </c>
       <c r="I271">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K271" t="s">
         <v>1147</v>
@@ -14480,7 +14480,7 @@
         <v>1140</v>
       </c>
       <c r="I272">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14562,7 +14562,7 @@
         <v>1140</v>
       </c>
       <c r="I274">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K274" t="s">
         <v>1144</v>
@@ -14635,7 +14635,7 @@
         <v>1140</v>
       </c>
       <c r="I276">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K276" t="s">
         <v>1148</v>
@@ -14673,7 +14673,7 @@
         <v>1140</v>
       </c>
       <c r="I277">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K277" t="s">
         <v>1144</v>
@@ -14711,7 +14711,7 @@
         <v>1140</v>
       </c>
       <c r="I278">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K278" t="s">
         <v>1147</v>
@@ -14749,7 +14749,7 @@
         <v>1140</v>
       </c>
       <c r="I279">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K279" t="s">
         <v>1146</v>
@@ -14790,7 +14790,7 @@
         <v>1140</v>
       </c>
       <c r="I280">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K280" t="s">
         <v>1144</v>
@@ -14828,7 +14828,7 @@
         <v>1140</v>
       </c>
       <c r="I281">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K281" t="s">
         <v>1144</v>
@@ -14866,7 +14866,7 @@
         <v>1140</v>
       </c>
       <c r="I282">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K282" t="s">
         <v>1144</v>
@@ -15073,7 +15073,7 @@
         <v>1140</v>
       </c>
       <c r="I288">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K288" t="s">
         <v>1147</v>
@@ -15140,7 +15140,7 @@
         <v>1140</v>
       </c>
       <c r="I290">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15181,7 +15181,7 @@
         <v>1140</v>
       </c>
       <c r="I291">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K291" t="s">
         <v>1146</v>
@@ -15219,7 +15219,7 @@
         <v>1140</v>
       </c>
       <c r="I292">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K292" t="s">
         <v>1147</v>
@@ -15257,7 +15257,7 @@
         <v>1140</v>
       </c>
       <c r="I293">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K293" t="s">
         <v>1148</v>
@@ -15295,7 +15295,7 @@
         <v>1140</v>
       </c>
       <c r="I294">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K294" t="s">
         <v>1150</v>
@@ -15330,7 +15330,7 @@
         <v>1140</v>
       </c>
       <c r="I295">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K295" t="s">
         <v>1150</v>
@@ -15365,7 +15365,7 @@
         <v>1140</v>
       </c>
       <c r="I296">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K296" t="s">
         <v>1150</v>
@@ -15435,7 +15435,7 @@
         <v>1140</v>
       </c>
       <c r="I298">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K298" t="s">
         <v>1144</v>
@@ -15473,7 +15473,7 @@
         <v>1140</v>
       </c>
       <c r="I299">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K299" t="s">
         <v>1147</v>
@@ -15511,7 +15511,7 @@
         <v>1140</v>
       </c>
       <c r="I300">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K300" t="s">
         <v>1147</v>
@@ -15549,7 +15549,7 @@
         <v>1140</v>
       </c>
       <c r="I301">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K301" t="s">
         <v>1147</v>
@@ -15587,7 +15587,7 @@
         <v>1140</v>
       </c>
       <c r="I302">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K302" t="s">
         <v>1147</v>
@@ -15625,7 +15625,7 @@
         <v>1140</v>
       </c>
       <c r="I303">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K303" t="s">
         <v>1144</v>
@@ -15663,7 +15663,7 @@
         <v>1140</v>
       </c>
       <c r="I304">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K304" t="s">
         <v>1147</v>
@@ -15701,7 +15701,7 @@
         <v>1140</v>
       </c>
       <c r="I305">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -15745,7 +15745,7 @@
         <v>1140</v>
       </c>
       <c r="I306">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -15789,7 +15789,7 @@
         <v>1140</v>
       </c>
       <c r="I307">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K307" t="s">
         <v>1143</v>
@@ -15827,7 +15827,7 @@
         <v>1140</v>
       </c>
       <c r="I308">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K308" t="s">
         <v>1143</v>
@@ -15865,7 +15865,7 @@
         <v>1140</v>
       </c>
       <c r="I309">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K309" t="s">
         <v>1143</v>
@@ -15903,7 +15903,7 @@
         <v>1140</v>
       </c>
       <c r="I310">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K310" t="s">
         <v>1144</v>
@@ -15941,7 +15941,7 @@
         <v>1140</v>
       </c>
       <c r="I311">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K311" t="s">
         <v>1143</v>
@@ -15979,7 +15979,7 @@
         <v>1140</v>
       </c>
       <c r="I312">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K312" t="s">
         <v>1144</v>
@@ -16052,7 +16052,7 @@
         <v>1140</v>
       </c>
       <c r="I314">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K314" t="s">
         <v>1144</v>
@@ -16090,7 +16090,7 @@
         <v>1140</v>
       </c>
       <c r="I315">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K315" t="s">
         <v>1144</v>
@@ -16128,7 +16128,7 @@
         <v>1140</v>
       </c>
       <c r="I316">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K316" t="s">
         <v>1144</v>
@@ -16166,7 +16166,7 @@
         <v>1140</v>
       </c>
       <c r="I317">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K317" t="s">
         <v>1144</v>
@@ -16277,7 +16277,7 @@
         <v>1140</v>
       </c>
       <c r="I320">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K320" t="s">
         <v>1148</v>
@@ -16315,7 +16315,7 @@
         <v>1140</v>
       </c>
       <c r="I321">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K321" t="s">
         <v>1144</v>
@@ -16353,7 +16353,7 @@
         <v>1140</v>
       </c>
       <c r="I322">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16397,7 +16397,7 @@
         <v>1140</v>
       </c>
       <c r="I323">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K323" t="s">
         <v>1144</v>
@@ -16435,7 +16435,7 @@
         <v>1140</v>
       </c>
       <c r="I324">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K324" t="s">
         <v>1144</v>
@@ -16473,7 +16473,7 @@
         <v>1140</v>
       </c>
       <c r="I325">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16517,7 +16517,7 @@
         <v>1140</v>
       </c>
       <c r="I326">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K326" t="s">
         <v>1144</v>
@@ -16555,7 +16555,7 @@
         <v>1140</v>
       </c>
       <c r="I327">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16599,7 +16599,7 @@
         <v>1140</v>
       </c>
       <c r="I328">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16643,7 +16643,7 @@
         <v>1140</v>
       </c>
       <c r="I329">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16687,7 +16687,7 @@
         <v>1140</v>
       </c>
       <c r="I330">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -16731,7 +16731,7 @@
         <v>1140</v>
       </c>
       <c r="I331">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K331" t="s">
         <v>1143</v>
@@ -16769,7 +16769,7 @@
         <v>1140</v>
       </c>
       <c r="I332">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K332" t="s">
         <v>1144</v>
@@ -16807,7 +16807,7 @@
         <v>1140</v>
       </c>
       <c r="I333">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K333" t="s">
         <v>1147</v>
@@ -16845,7 +16845,7 @@
         <v>1140</v>
       </c>
       <c r="I334">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K334" t="s">
         <v>1144</v>
@@ -16924,7 +16924,7 @@
         <v>1140</v>
       </c>
       <c r="I336">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K336" t="s">
         <v>1146</v>
@@ -17003,7 +17003,7 @@
         <v>1140</v>
       </c>
       <c r="I338">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K338" t="s">
         <v>1146</v>
@@ -17070,7 +17070,7 @@
         <v>1140</v>
       </c>
       <c r="I340">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K340" t="s">
         <v>1143</v>
@@ -17108,7 +17108,7 @@
         <v>1140</v>
       </c>
       <c r="I341">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K341" t="s">
         <v>1143</v>
@@ -17146,7 +17146,7 @@
         <v>1140</v>
       </c>
       <c r="I342">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K342" t="s">
         <v>1143</v>
@@ -17184,7 +17184,7 @@
         <v>1140</v>
       </c>
       <c r="I343">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K343" t="s">
         <v>1144</v>
@@ -17222,7 +17222,7 @@
         <v>1140</v>
       </c>
       <c r="I344">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K344" t="s">
         <v>1144</v>
@@ -17260,7 +17260,7 @@
         <v>1140</v>
       </c>
       <c r="I345">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K345" t="s">
         <v>1143</v>
@@ -17298,7 +17298,7 @@
         <v>1140</v>
       </c>
       <c r="I346">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K346" t="s">
         <v>1144</v>
@@ -17336,7 +17336,7 @@
         <v>1140</v>
       </c>
       <c r="I347">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17380,7 +17380,7 @@
         <v>1140</v>
       </c>
       <c r="I348">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17424,7 +17424,7 @@
         <v>1140</v>
       </c>
       <c r="I349">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K349" t="s">
         <v>1148</v>
@@ -17462,7 +17462,7 @@
         <v>1140</v>
       </c>
       <c r="I350">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K350" t="s">
         <v>1150</v>
@@ -17497,7 +17497,7 @@
         <v>1140</v>
       </c>
       <c r="I351">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K351" t="s">
         <v>1148</v>
@@ -17535,7 +17535,7 @@
         <v>1140</v>
       </c>
       <c r="I352">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K352" t="s">
         <v>1148</v>
@@ -17573,7 +17573,7 @@
         <v>1140</v>
       </c>
       <c r="I353">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K353" t="s">
         <v>1147</v>
@@ -17611,7 +17611,7 @@
         <v>1140</v>
       </c>
       <c r="I354">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K354" t="s">
         <v>1147</v>
@@ -17649,7 +17649,7 @@
         <v>1140</v>
       </c>
       <c r="I355">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -17731,7 +17731,7 @@
         <v>1140</v>
       </c>
       <c r="I357">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K357" t="s">
         <v>1147</v>
@@ -17769,7 +17769,7 @@
         <v>1140</v>
       </c>
       <c r="I358">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K358" t="s">
         <v>1147</v>
@@ -17807,7 +17807,7 @@
         <v>1140</v>
       </c>
       <c r="I359">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K359" t="s">
         <v>1147</v>
@@ -17848,7 +17848,7 @@
         <v>1140</v>
       </c>
       <c r="I360">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K360" t="s">
         <v>1147</v>
@@ -17886,7 +17886,7 @@
         <v>1140</v>
       </c>
       <c r="I361">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K361" t="s">
         <v>1147</v>
@@ -17924,7 +17924,7 @@
         <v>1140</v>
       </c>
       <c r="I362">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K362" t="s">
         <v>1147</v>
@@ -17962,7 +17962,7 @@
         <v>1140</v>
       </c>
       <c r="I363">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K363" t="s">
         <v>1147</v>
@@ -18000,7 +18000,7 @@
         <v>1140</v>
       </c>
       <c r="I364">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K364" t="s">
         <v>1147</v>
@@ -18038,7 +18038,7 @@
         <v>1140</v>
       </c>
       <c r="I365">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K365" t="s">
         <v>1146</v>
@@ -18076,7 +18076,7 @@
         <v>1140</v>
       </c>
       <c r="I366">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K366" t="s">
         <v>1147</v>
@@ -18114,7 +18114,7 @@
         <v>1140</v>
       </c>
       <c r="I367">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K367" t="s">
         <v>1147</v>
@@ -18152,7 +18152,7 @@
         <v>1140</v>
       </c>
       <c r="I368">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K368" t="s">
         <v>1147</v>
@@ -18190,7 +18190,7 @@
         <v>1140</v>
       </c>
       <c r="I369">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K369" t="s">
         <v>1147</v>
@@ -18228,7 +18228,7 @@
         <v>1140</v>
       </c>
       <c r="I370">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K370" t="s">
         <v>1147</v>
@@ -18266,7 +18266,7 @@
         <v>1140</v>
       </c>
       <c r="I371">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18310,7 +18310,7 @@
         <v>1140</v>
       </c>
       <c r="I372">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18357,7 +18357,7 @@
         <v>1140</v>
       </c>
       <c r="I373">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K373" t="s">
         <v>1143</v>
@@ -18395,7 +18395,7 @@
         <v>1140</v>
       </c>
       <c r="I374">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K374" t="s">
         <v>1143</v>
@@ -18433,7 +18433,7 @@
         <v>1140</v>
       </c>
       <c r="I375">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K375" t="s">
         <v>1147</v>
@@ -18471,7 +18471,7 @@
         <v>1140</v>
       </c>
       <c r="I376">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K376" t="s">
         <v>1147</v>
@@ -18547,7 +18547,7 @@
         <v>1140</v>
       </c>
       <c r="I378">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K378" t="s">
         <v>1147</v>
@@ -18585,7 +18585,7 @@
         <v>1140</v>
       </c>
       <c r="I379">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18629,7 +18629,7 @@
         <v>1140</v>
       </c>
       <c r="I380">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K380" t="s">
         <v>1147</v>
@@ -18667,7 +18667,7 @@
         <v>1140</v>
       </c>
       <c r="I381">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K381" t="s">
         <v>1147</v>
@@ -18705,7 +18705,7 @@
         <v>1140</v>
       </c>
       <c r="I382">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K382" t="s">
         <v>1147</v>
@@ -18743,7 +18743,7 @@
         <v>1140</v>
       </c>
       <c r="I383">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K383" t="s">
         <v>1147</v>
@@ -18781,7 +18781,7 @@
         <v>1140</v>
       </c>
       <c r="I384">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K384" t="s">
         <v>1143</v>
@@ -18819,7 +18819,7 @@
         <v>1140</v>
       </c>
       <c r="I385">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K385" t="s">
         <v>1143</v>
@@ -18857,7 +18857,7 @@
         <v>1140</v>
       </c>
       <c r="I386">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K386" t="s">
         <v>1147</v>
@@ -18895,7 +18895,7 @@
         <v>1140</v>
       </c>
       <c r="I387">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K387" t="s">
         <v>1147</v>
@@ -18933,7 +18933,7 @@
         <v>1140</v>
       </c>
       <c r="I388">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K388" t="s">
         <v>1147</v>
@@ -18971,7 +18971,7 @@
         <v>1140</v>
       </c>
       <c r="I389">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K389" t="s">
         <v>1148</v>
@@ -19009,7 +19009,7 @@
         <v>1140</v>
       </c>
       <c r="I390">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19129,7 +19129,7 @@
         <v>1140</v>
       </c>
       <c r="I393">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K393" t="s">
         <v>1147</v>
@@ -19167,7 +19167,7 @@
         <v>1140</v>
       </c>
       <c r="I394">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K394" t="s">
         <v>1147</v>
@@ -19205,7 +19205,7 @@
         <v>1140</v>
       </c>
       <c r="I395">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K395" t="s">
         <v>1147</v>
@@ -19243,7 +19243,7 @@
         <v>1140</v>
       </c>
       <c r="I396">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K396" t="s">
         <v>1147</v>
@@ -19281,7 +19281,7 @@
         <v>1140</v>
       </c>
       <c r="I397">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K397" t="s">
         <v>1147</v>
@@ -19319,7 +19319,7 @@
         <v>1140</v>
       </c>
       <c r="I398">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K398" t="s">
         <v>1147</v>
@@ -19395,7 +19395,7 @@
         <v>1140</v>
       </c>
       <c r="I400">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K400" t="s">
         <v>1147</v>
@@ -19433,7 +19433,7 @@
         <v>1140</v>
       </c>
       <c r="I401">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K401" t="s">
         <v>1147</v>
@@ -19471,7 +19471,7 @@
         <v>1140</v>
       </c>
       <c r="I402">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K402" t="s">
         <v>1147</v>
@@ -19509,7 +19509,7 @@
         <v>1140</v>
       </c>
       <c r="I403">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K403" t="s">
         <v>1150</v>
@@ -19544,7 +19544,7 @@
         <v>1140</v>
       </c>
       <c r="I404">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K404" t="s">
         <v>1150</v>
@@ -19608,7 +19608,7 @@
         <v>1140</v>
       </c>
       <c r="I406">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19640,7 +19640,7 @@
         <v>1140</v>
       </c>
       <c r="I407">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19672,7 +19672,7 @@
         <v>1140</v>
       </c>
       <c r="I408">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19704,7 +19704,7 @@
         <v>1140</v>
       </c>
       <c r="I409">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -19736,7 +19736,7 @@
         <v>1140</v>
       </c>
       <c r="I410">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -19768,7 +19768,7 @@
         <v>1140</v>
       </c>
       <c r="I411">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -19800,7 +19800,7 @@
         <v>1140</v>
       </c>
       <c r="I412">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -19832,7 +19832,7 @@
         <v>1140</v>
       </c>
       <c r="I413">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -19864,7 +19864,7 @@
         <v>1140</v>
       </c>
       <c r="I414">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -19896,7 +19896,7 @@
         <v>1140</v>
       </c>
       <c r="I415">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -19928,7 +19928,7 @@
         <v>1140</v>
       </c>
       <c r="I416">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -19960,7 +19960,7 @@
         <v>1140</v>
       </c>
       <c r="I417">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -19992,7 +19992,7 @@
         <v>1140</v>
       </c>
       <c r="I418">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20024,7 +20024,7 @@
         <v>1140</v>
       </c>
       <c r="I419">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20056,7 +20056,7 @@
         <v>1140</v>
       </c>
       <c r="I420">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20088,7 +20088,7 @@
         <v>1140</v>
       </c>
       <c r="I421">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20120,7 +20120,7 @@
         <v>1140</v>
       </c>
       <c r="I422">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20152,7 +20152,7 @@
         <v>1140</v>
       </c>
       <c r="I423">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20184,7 +20184,7 @@
         <v>1140</v>
       </c>
       <c r="I424">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20216,7 +20216,7 @@
         <v>1140</v>
       </c>
       <c r="I425">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20248,7 +20248,7 @@
         <v>1140</v>
       </c>
       <c r="I426">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20280,7 +20280,7 @@
         <v>1140</v>
       </c>
       <c r="I427">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20312,7 +20312,7 @@
         <v>1140</v>
       </c>
       <c r="I428">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20344,7 +20344,7 @@
         <v>1140</v>
       </c>
       <c r="I429">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20376,7 +20376,7 @@
         <v>1140</v>
       </c>
       <c r="I430">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20408,7 +20408,7 @@
         <v>1140</v>
       </c>
       <c r="I431">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20440,7 +20440,7 @@
         <v>1140</v>
       </c>
       <c r="I432">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20472,7 +20472,7 @@
         <v>1140</v>
       </c>
       <c r="I433">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20504,7 +20504,7 @@
         <v>1140</v>
       </c>
       <c r="I434">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20536,7 +20536,7 @@
         <v>1140</v>
       </c>
       <c r="I435">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20568,7 +20568,7 @@
         <v>1140</v>
       </c>
       <c r="I436">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20600,7 +20600,7 @@
         <v>1142</v>
       </c>
       <c r="I437">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20632,7 +20632,7 @@
         <v>1142</v>
       </c>
       <c r="I438">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20664,7 +20664,7 @@
         <v>1140</v>
       </c>
       <c r="I439">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20696,7 +20696,7 @@
         <v>1140</v>
       </c>
       <c r="I440">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -20728,7 +20728,7 @@
         <v>1140</v>
       </c>
       <c r="I441">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -20760,7 +20760,7 @@
         <v>1140</v>
       </c>
       <c r="I442">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -20792,7 +20792,7 @@
         <v>1140</v>
       </c>
       <c r="I443">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -20824,7 +20824,7 @@
         <v>1140</v>
       </c>
       <c r="I444">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -20856,7 +20856,7 @@
         <v>1140</v>
       </c>
       <c r="I445">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -20888,7 +20888,7 @@
         <v>1140</v>
       </c>
       <c r="I446">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -20920,7 +20920,7 @@
         <v>1140</v>
       </c>
       <c r="I447">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (03/08/2026 14:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4253,7 +4253,7 @@
         <v>1140</v>
       </c>
       <c r="I2">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="K2" t="s">
         <v>1143</v>
@@ -4291,7 +4291,7 @@
         <v>1140</v>
       </c>
       <c r="I3">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="K3" t="s">
         <v>1144</v>
@@ -4329,7 +4329,7 @@
         <v>1140</v>
       </c>
       <c r="I4">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="K4" t="s">
         <v>1144</v>
@@ -4367,7 +4367,7 @@
         <v>1140</v>
       </c>
       <c r="I5">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4411,7 +4411,7 @@
         <v>1140</v>
       </c>
       <c r="I6">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4455,7 +4455,7 @@
         <v>1140</v>
       </c>
       <c r="I7">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4531,7 +4531,7 @@
         <v>1140</v>
       </c>
       <c r="I9">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4578,7 +4578,7 @@
         <v>1140</v>
       </c>
       <c r="I10">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4625,7 +4625,7 @@
         <v>1140</v>
       </c>
       <c r="I11">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4672,7 +4672,7 @@
         <v>1140</v>
       </c>
       <c r="I12">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -4751,7 +4751,7 @@
         <v>1140</v>
       </c>
       <c r="I14">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -4795,7 +4795,7 @@
         <v>1140</v>
       </c>
       <c r="I15">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K15" t="s">
         <v>1146</v>
@@ -4833,7 +4833,7 @@
         <v>1140</v>
       </c>
       <c r="I16">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K16" t="s">
         <v>1143</v>
@@ -4871,7 +4871,7 @@
         <v>1140</v>
       </c>
       <c r="I17">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -4915,7 +4915,7 @@
         <v>1140</v>
       </c>
       <c r="I18">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -4994,7 +4994,7 @@
         <v>1140</v>
       </c>
       <c r="I20">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5073,7 +5073,7 @@
         <v>1140</v>
       </c>
       <c r="I22">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K22" t="s">
         <v>1147</v>
@@ -5111,7 +5111,7 @@
         <v>1140</v>
       </c>
       <c r="I23">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5234,7 +5234,7 @@
         <v>1140</v>
       </c>
       <c r="I26">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5281,7 +5281,7 @@
         <v>1140</v>
       </c>
       <c r="I27">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K27" t="s">
         <v>1147</v>
@@ -5386,7 +5386,7 @@
         <v>1140</v>
       </c>
       <c r="I30">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5468,7 +5468,7 @@
         <v>1140</v>
       </c>
       <c r="I32">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K32" t="s">
         <v>1143</v>
@@ -5710,7 +5710,7 @@
         <v>1140</v>
       </c>
       <c r="I39">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K39" t="s">
         <v>1148</v>
@@ -5745,7 +5745,7 @@
         <v>1140</v>
       </c>
       <c r="I40">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K40" t="s">
         <v>1146</v>
@@ -5894,7 +5894,7 @@
         <v>1140</v>
       </c>
       <c r="I44">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -5941,7 +5941,7 @@
         <v>1140</v>
       </c>
       <c r="I45">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -5988,7 +5988,7 @@
         <v>1140</v>
       </c>
       <c r="I46">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K46" t="s">
         <v>1147</v>
@@ -6026,7 +6026,7 @@
         <v>1140</v>
       </c>
       <c r="I47">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6073,7 +6073,7 @@
         <v>1140</v>
       </c>
       <c r="I48">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K48" t="s">
         <v>1147</v>
@@ -6143,7 +6143,7 @@
         <v>1140</v>
       </c>
       <c r="I50">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K50" t="s">
         <v>1147</v>
@@ -6219,7 +6219,7 @@
         <v>1140</v>
       </c>
       <c r="I52">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K52" t="s">
         <v>1143</v>
@@ -6257,7 +6257,7 @@
         <v>1140</v>
       </c>
       <c r="I53">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K53" t="s">
         <v>1144</v>
@@ -6295,7 +6295,7 @@
         <v>1140</v>
       </c>
       <c r="I54">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K54" t="s">
         <v>1144</v>
@@ -6403,7 +6403,7 @@
         <v>1140</v>
       </c>
       <c r="I57">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K57" t="s">
         <v>1147</v>
@@ -6607,7 +6607,7 @@
         <v>1140</v>
       </c>
       <c r="I63">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6654,7 +6654,7 @@
         <v>1140</v>
       </c>
       <c r="I64">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -6885,7 +6885,7 @@
         <v>1140</v>
       </c>
       <c r="I70">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K70" t="s">
         <v>1144</v>
@@ -6923,7 +6923,7 @@
         <v>1140</v>
       </c>
       <c r="I71">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K71" t="s">
         <v>1150</v>
@@ -6993,7 +6993,7 @@
         <v>1140</v>
       </c>
       <c r="I73">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K73" t="s">
         <v>1143</v>
@@ -7069,7 +7069,7 @@
         <v>1140</v>
       </c>
       <c r="I75">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K75" t="s">
         <v>1144</v>
@@ -7107,7 +7107,7 @@
         <v>1140</v>
       </c>
       <c r="I76">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K76" t="s">
         <v>1150</v>
@@ -7215,7 +7215,7 @@
         <v>1140</v>
       </c>
       <c r="I79">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K79" t="s">
         <v>1150</v>
@@ -7250,7 +7250,7 @@
         <v>1140</v>
       </c>
       <c r="I80">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K80" t="s">
         <v>1144</v>
@@ -7326,7 +7326,7 @@
         <v>1140</v>
       </c>
       <c r="I82">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="K82" t="s">
         <v>1147</v>
@@ -7399,7 +7399,7 @@
         <v>1140</v>
       </c>
       <c r="I84">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7446,7 +7446,7 @@
         <v>1140</v>
       </c>
       <c r="I85">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="K85" t="s">
         <v>1144</v>
@@ -7484,7 +7484,7 @@
         <v>1140</v>
       </c>
       <c r="I86">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="K86" t="s">
         <v>1144</v>
@@ -7522,7 +7522,7 @@
         <v>1140</v>
       </c>
       <c r="I87">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7639,7 +7639,7 @@
         <v>1140</v>
       </c>
       <c r="I90">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="K90" t="s">
         <v>1117</v>
@@ -7680,7 +7680,7 @@
         <v>1140</v>
       </c>
       <c r="I91">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="K91" t="s">
         <v>1146</v>
@@ -7747,7 +7747,7 @@
         <v>1140</v>
       </c>
       <c r="I93">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="K93" t="s">
         <v>1146</v>
@@ -7785,7 +7785,7 @@
         <v>1140</v>
       </c>
       <c r="I94">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="K94" t="s">
         <v>1147</v>
@@ -7823,7 +7823,7 @@
         <v>1140</v>
       </c>
       <c r="I95">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="K95" t="s">
         <v>1146</v>
@@ -7861,7 +7861,7 @@
         <v>1140</v>
       </c>
       <c r="I96">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -7908,7 +7908,7 @@
         <v>1140</v>
       </c>
       <c r="I97">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K97" t="s">
         <v>1117</v>
@@ -7949,7 +7949,7 @@
         <v>1140</v>
       </c>
       <c r="I98">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K98" t="s">
         <v>1147</v>
@@ -8016,7 +8016,7 @@
         <v>1140</v>
       </c>
       <c r="I100">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K100" t="s">
         <v>1146</v>
@@ -8144,7 +8144,7 @@
         <v>1140</v>
       </c>
       <c r="I104">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K104" t="s">
         <v>1146</v>
@@ -8182,7 +8182,7 @@
         <v>1140</v>
       </c>
       <c r="I105">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K105" t="s">
         <v>1146</v>
@@ -8220,7 +8220,7 @@
         <v>1140</v>
       </c>
       <c r="I106">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8264,7 +8264,7 @@
         <v>1140</v>
       </c>
       <c r="I107">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8308,7 +8308,7 @@
         <v>1140</v>
       </c>
       <c r="I108">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K108" t="s">
         <v>1144</v>
@@ -8346,7 +8346,7 @@
         <v>1140</v>
       </c>
       <c r="I109">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K109" t="s">
         <v>1144</v>
@@ -8562,7 +8562,7 @@
         <v>1140</v>
       </c>
       <c r="I115">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K115" t="s">
         <v>1144</v>
@@ -8600,7 +8600,7 @@
         <v>1140</v>
       </c>
       <c r="I116">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K116" t="s">
         <v>1144</v>
@@ -8638,7 +8638,7 @@
         <v>1140</v>
       </c>
       <c r="I117">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K117" t="s">
         <v>1144</v>
@@ -8676,7 +8676,7 @@
         <v>1140</v>
       </c>
       <c r="I118">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K118" t="s">
         <v>1144</v>
@@ -8714,7 +8714,7 @@
         <v>1140</v>
       </c>
       <c r="I119">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K119" t="s">
         <v>1144</v>
@@ -8752,7 +8752,7 @@
         <v>1140</v>
       </c>
       <c r="I120">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="K120" t="s">
         <v>1144</v>
@@ -8790,7 +8790,7 @@
         <v>1140</v>
       </c>
       <c r="I121">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -8837,7 +8837,7 @@
         <v>1140</v>
       </c>
       <c r="I122">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="K122" t="s">
         <v>1144</v>
@@ -8904,7 +8904,7 @@
         <v>1140</v>
       </c>
       <c r="I124">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="K124" t="s">
         <v>1144</v>
@@ -8942,7 +8942,7 @@
         <v>1140</v>
       </c>
       <c r="I125">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="K125" t="s">
         <v>1150</v>
@@ -9047,7 +9047,7 @@
         <v>1140</v>
       </c>
       <c r="I128">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K128" t="s">
         <v>1144</v>
@@ -9085,7 +9085,7 @@
         <v>1140</v>
       </c>
       <c r="I129">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K129" t="s">
         <v>1143</v>
@@ -9123,7 +9123,7 @@
         <v>1140</v>
       </c>
       <c r="I130">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9205,7 +9205,7 @@
         <v>1140</v>
       </c>
       <c r="I132">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9281,7 +9281,7 @@
         <v>1140</v>
       </c>
       <c r="I134">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="K134" t="s">
         <v>1143</v>
@@ -9412,7 +9412,7 @@
         <v>1140</v>
       </c>
       <c r="I138">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K138" t="s">
         <v>1144</v>
@@ -9741,7 +9741,7 @@
         <v>1140</v>
       </c>
       <c r="I148">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K148" t="s">
         <v>1144</v>
@@ -9779,7 +9779,7 @@
         <v>1140</v>
       </c>
       <c r="I149">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K149" t="s">
         <v>1150</v>
@@ -9814,7 +9814,7 @@
         <v>1140</v>
       </c>
       <c r="I150">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -9899,7 +9899,7 @@
         <v>1140</v>
       </c>
       <c r="I152">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -9943,7 +9943,7 @@
         <v>1140</v>
       </c>
       <c r="I153">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K153" t="s">
         <v>1144</v>
@@ -10016,7 +10016,7 @@
         <v>1140</v>
       </c>
       <c r="I155">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K155" t="s">
         <v>1150</v>
@@ -10051,7 +10051,7 @@
         <v>1140</v>
       </c>
       <c r="I156">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K156" t="s">
         <v>1144</v>
@@ -10089,7 +10089,7 @@
         <v>1140</v>
       </c>
       <c r="I157">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K157" t="s">
         <v>1146</v>
@@ -10127,7 +10127,7 @@
         <v>1140</v>
       </c>
       <c r="I158">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10171,7 +10171,7 @@
         <v>1140</v>
       </c>
       <c r="I159">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="K159" t="s">
         <v>1144</v>
@@ -10209,7 +10209,7 @@
         <v>1140</v>
       </c>
       <c r="I160">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="K160" t="s">
         <v>1144</v>
@@ -10247,7 +10247,7 @@
         <v>1140</v>
       </c>
       <c r="I161">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10294,7 +10294,7 @@
         <v>1140</v>
       </c>
       <c r="I162">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10338,7 +10338,7 @@
         <v>1140</v>
       </c>
       <c r="I163">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10382,7 +10382,7 @@
         <v>1142</v>
       </c>
       <c r="I164">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="K164" t="s">
         <v>1151</v>
@@ -10417,7 +10417,7 @@
         <v>1140</v>
       </c>
       <c r="I165">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="K165" t="s">
         <v>1144</v>
@@ -10525,7 +10525,7 @@
         <v>1140</v>
       </c>
       <c r="I168">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="K168" t="s">
         <v>1147</v>
@@ -10566,7 +10566,7 @@
         <v>1140</v>
       </c>
       <c r="I169">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10648,7 +10648,7 @@
         <v>1140</v>
       </c>
       <c r="I171">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="K171" t="s">
         <v>1144</v>
@@ -10794,7 +10794,7 @@
         <v>1140</v>
       </c>
       <c r="I175">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -10841,7 +10841,7 @@
         <v>1140</v>
       </c>
       <c r="I176">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="K176" t="s">
         <v>1144</v>
@@ -10879,7 +10879,7 @@
         <v>1140</v>
       </c>
       <c r="I177">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -10926,7 +10926,7 @@
         <v>1140</v>
       </c>
       <c r="I178">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K178" t="s">
         <v>1143</v>
@@ -10993,7 +10993,7 @@
         <v>1140</v>
       </c>
       <c r="I180">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K180" t="s">
         <v>1143</v>
@@ -11098,7 +11098,7 @@
         <v>1140</v>
       </c>
       <c r="I183">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K183" t="s">
         <v>1144</v>
@@ -11133,7 +11133,7 @@
         <v>1140</v>
       </c>
       <c r="I184">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="K184" t="s">
         <v>1150</v>
@@ -11168,7 +11168,7 @@
         <v>1140</v>
       </c>
       <c r="I185">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="K185" t="s">
         <v>1144</v>
@@ -11206,7 +11206,7 @@
         <v>1140</v>
       </c>
       <c r="I186">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="K186" t="s">
         <v>1144</v>
@@ -11244,7 +11244,7 @@
         <v>1140</v>
       </c>
       <c r="I187">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11291,7 +11291,7 @@
         <v>1140</v>
       </c>
       <c r="I188">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11338,7 +11338,7 @@
         <v>1140</v>
       </c>
       <c r="I189">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11382,7 +11382,7 @@
         <v>1140</v>
       </c>
       <c r="I190">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="K190" t="s">
         <v>1146</v>
@@ -11420,7 +11420,7 @@
         <v>1140</v>
       </c>
       <c r="I191">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11464,7 +11464,7 @@
         <v>1140</v>
       </c>
       <c r="I192">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="K192" t="s">
         <v>1144</v>
@@ -11502,7 +11502,7 @@
         <v>1140</v>
       </c>
       <c r="I193">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="K193" t="s">
         <v>1149</v>
@@ -11572,7 +11572,7 @@
         <v>1140</v>
       </c>
       <c r="I195">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="K195" t="s">
         <v>1146</v>
@@ -11706,7 +11706,7 @@
         <v>1140</v>
       </c>
       <c r="I199">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -11750,7 +11750,7 @@
         <v>1140</v>
       </c>
       <c r="I200">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K200" t="s">
         <v>1146</v>
@@ -11788,7 +11788,7 @@
         <v>1140</v>
       </c>
       <c r="I201">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K201" t="s">
         <v>1144</v>
@@ -11826,7 +11826,7 @@
         <v>1140</v>
       </c>
       <c r="I202">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K202" t="s">
         <v>1144</v>
@@ -11864,7 +11864,7 @@
         <v>1140</v>
       </c>
       <c r="I203">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K203" t="s">
         <v>1144</v>
@@ -11902,7 +11902,7 @@
         <v>1140</v>
       </c>
       <c r="I204">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K204" t="s">
         <v>1143</v>
@@ -11940,7 +11940,7 @@
         <v>1140</v>
       </c>
       <c r="I205">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K205" t="s">
         <v>1143</v>
@@ -12013,7 +12013,7 @@
         <v>1140</v>
       </c>
       <c r="I207">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12057,7 +12057,7 @@
         <v>1140</v>
       </c>
       <c r="I208">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12101,7 +12101,7 @@
         <v>1140</v>
       </c>
       <c r="I209">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12145,7 +12145,7 @@
         <v>1140</v>
       </c>
       <c r="I210">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="K210" t="s">
         <v>1147</v>
@@ -12253,7 +12253,7 @@
         <v>1140</v>
       </c>
       <c r="I213">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="K213" t="s">
         <v>1144</v>
@@ -12291,7 +12291,7 @@
         <v>1140</v>
       </c>
       <c r="I214">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12338,7 +12338,7 @@
         <v>1140</v>
       </c>
       <c r="I215">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="K215" t="s">
         <v>1144</v>
@@ -12405,7 +12405,7 @@
         <v>1140</v>
       </c>
       <c r="I217">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12449,7 +12449,7 @@
         <v>1140</v>
       </c>
       <c r="I218">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="K218" t="s">
         <v>1146</v>
@@ -12487,7 +12487,7 @@
         <v>1140</v>
       </c>
       <c r="I219">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="K219" t="s">
         <v>1146</v>
@@ -12525,7 +12525,7 @@
         <v>1140</v>
       </c>
       <c r="I220">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="K220" t="s">
         <v>1146</v>
@@ -12601,7 +12601,7 @@
         <v>1140</v>
       </c>
       <c r="I222">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K222" t="s">
         <v>1144</v>
@@ -12639,7 +12639,7 @@
         <v>1140</v>
       </c>
       <c r="I223">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K223" t="s">
         <v>1144</v>
@@ -12677,7 +12677,7 @@
         <v>1140</v>
       </c>
       <c r="I224">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K224" t="s">
         <v>1144</v>
@@ -12715,7 +12715,7 @@
         <v>1140</v>
       </c>
       <c r="I225">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K225" t="s">
         <v>1144</v>
@@ -12753,7 +12753,7 @@
         <v>1140</v>
       </c>
       <c r="I226">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K226" t="s">
         <v>1144</v>
@@ -12791,7 +12791,7 @@
         <v>1140</v>
       </c>
       <c r="I227">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K227" t="s">
         <v>1144</v>
@@ -12829,7 +12829,7 @@
         <v>1140</v>
       </c>
       <c r="I228">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K228" t="s">
         <v>1144</v>
@@ -12902,7 +12902,7 @@
         <v>1140</v>
       </c>
       <c r="I230">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K230" t="s">
         <v>1147</v>
@@ -12940,7 +12940,7 @@
         <v>1140</v>
       </c>
       <c r="I231">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13054,7 +13054,7 @@
         <v>1140</v>
       </c>
       <c r="I234">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13101,7 +13101,7 @@
         <v>1140</v>
       </c>
       <c r="I235">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13148,7 +13148,7 @@
         <v>1140</v>
       </c>
       <c r="I236">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13192,7 +13192,7 @@
         <v>1140</v>
       </c>
       <c r="I237">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="K237" t="s">
         <v>1144</v>
@@ -13259,7 +13259,7 @@
         <v>1140</v>
       </c>
       <c r="I239">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="K239" t="s">
         <v>1117</v>
@@ -13370,7 +13370,7 @@
         <v>1140</v>
       </c>
       <c r="I242">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="K242" t="s">
         <v>1143</v>
@@ -13440,7 +13440,7 @@
         <v>1140</v>
       </c>
       <c r="I244">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="K244" t="s">
         <v>1146</v>
@@ -13478,7 +13478,7 @@
         <v>1140</v>
       </c>
       <c r="I245">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="K245" t="s">
         <v>1146</v>
@@ -13516,7 +13516,7 @@
         <v>1140</v>
       </c>
       <c r="I246">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13621,7 +13621,7 @@
         <v>1140</v>
       </c>
       <c r="I249">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="K249" t="s">
         <v>1144</v>
@@ -13659,7 +13659,7 @@
         <v>1140</v>
       </c>
       <c r="I250">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K250" t="s">
         <v>1146</v>
@@ -13767,7 +13767,7 @@
         <v>1140</v>
       </c>
       <c r="I253">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K253" t="s">
         <v>1147</v>
@@ -13805,7 +13805,7 @@
         <v>1140</v>
       </c>
       <c r="I254">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K254" t="s">
         <v>1147</v>
@@ -13843,7 +13843,7 @@
         <v>1140</v>
       </c>
       <c r="I255">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K255" t="s">
         <v>1146</v>
@@ -13881,7 +13881,7 @@
         <v>1140</v>
       </c>
       <c r="I256">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K256" t="s">
         <v>1144</v>
@@ -13980,7 +13980,7 @@
         <v>1140</v>
       </c>
       <c r="I259">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K259" t="s">
         <v>1146</v>
@@ -14018,7 +14018,7 @@
         <v>1140</v>
       </c>
       <c r="I260">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K260" t="s">
         <v>1146</v>
@@ -14056,7 +14056,7 @@
         <v>1140</v>
       </c>
       <c r="I261">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K261" t="s">
         <v>1147</v>
@@ -14094,7 +14094,7 @@
         <v>1140</v>
       </c>
       <c r="I262">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14179,7 +14179,7 @@
         <v>1140</v>
       </c>
       <c r="I264">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K264" t="s">
         <v>1147</v>
@@ -14217,7 +14217,7 @@
         <v>1140</v>
       </c>
       <c r="I265">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K265" t="s">
         <v>1147</v>
@@ -14255,7 +14255,7 @@
         <v>1140</v>
       </c>
       <c r="I266">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K266" t="s">
         <v>1146</v>
@@ -14293,7 +14293,7 @@
         <v>1140</v>
       </c>
       <c r="I267">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K267" t="s">
         <v>1147</v>
@@ -14331,7 +14331,7 @@
         <v>1140</v>
       </c>
       <c r="I268">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K268" t="s">
         <v>1144</v>
@@ -14366,7 +14366,7 @@
         <v>1140</v>
       </c>
       <c r="I269">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K269" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1140</v>
       </c>
       <c r="I270">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K270" t="s">
         <v>1147</v>
@@ -14442,7 +14442,7 @@
         <v>1140</v>
       </c>
       <c r="I271">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K271" t="s">
         <v>1147</v>
@@ -14480,7 +14480,7 @@
         <v>1140</v>
       </c>
       <c r="I272">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14562,7 +14562,7 @@
         <v>1140</v>
       </c>
       <c r="I274">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K274" t="s">
         <v>1144</v>
@@ -14635,7 +14635,7 @@
         <v>1140</v>
       </c>
       <c r="I276">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K276" t="s">
         <v>1148</v>
@@ -14673,7 +14673,7 @@
         <v>1140</v>
       </c>
       <c r="I277">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K277" t="s">
         <v>1144</v>
@@ -14711,7 +14711,7 @@
         <v>1140</v>
       </c>
       <c r="I278">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="K278" t="s">
         <v>1147</v>
@@ -14749,7 +14749,7 @@
         <v>1140</v>
       </c>
       <c r="I279">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="K279" t="s">
         <v>1146</v>
@@ -14790,7 +14790,7 @@
         <v>1140</v>
       </c>
       <c r="I280">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="K280" t="s">
         <v>1144</v>
@@ -14828,7 +14828,7 @@
         <v>1140</v>
       </c>
       <c r="I281">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="K281" t="s">
         <v>1144</v>
@@ -14866,7 +14866,7 @@
         <v>1140</v>
       </c>
       <c r="I282">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="K282" t="s">
         <v>1144</v>
@@ -15073,7 +15073,7 @@
         <v>1140</v>
       </c>
       <c r="I288">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K288" t="s">
         <v>1147</v>
@@ -15140,7 +15140,7 @@
         <v>1140</v>
       </c>
       <c r="I290">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15181,7 +15181,7 @@
         <v>1140</v>
       </c>
       <c r="I291">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K291" t="s">
         <v>1146</v>
@@ -15219,7 +15219,7 @@
         <v>1140</v>
       </c>
       <c r="I292">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="K292" t="s">
         <v>1147</v>
@@ -15257,7 +15257,7 @@
         <v>1140</v>
       </c>
       <c r="I293">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K293" t="s">
         <v>1148</v>
@@ -15295,7 +15295,7 @@
         <v>1140</v>
       </c>
       <c r="I294">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K294" t="s">
         <v>1150</v>
@@ -15330,7 +15330,7 @@
         <v>1140</v>
       </c>
       <c r="I295">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K295" t="s">
         <v>1150</v>
@@ -15365,7 +15365,7 @@
         <v>1140</v>
       </c>
       <c r="I296">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K296" t="s">
         <v>1150</v>
@@ -15435,7 +15435,7 @@
         <v>1140</v>
       </c>
       <c r="I298">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K298" t="s">
         <v>1144</v>
@@ -15473,7 +15473,7 @@
         <v>1140</v>
       </c>
       <c r="I299">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K299" t="s">
         <v>1147</v>
@@ -15511,7 +15511,7 @@
         <v>1140</v>
       </c>
       <c r="I300">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K300" t="s">
         <v>1147</v>
@@ -15549,7 +15549,7 @@
         <v>1140</v>
       </c>
       <c r="I301">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K301" t="s">
         <v>1147</v>
@@ -15587,7 +15587,7 @@
         <v>1140</v>
       </c>
       <c r="I302">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K302" t="s">
         <v>1147</v>
@@ -15625,7 +15625,7 @@
         <v>1140</v>
       </c>
       <c r="I303">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K303" t="s">
         <v>1144</v>
@@ -15663,7 +15663,7 @@
         <v>1140</v>
       </c>
       <c r="I304">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K304" t="s">
         <v>1147</v>
@@ -15701,7 +15701,7 @@
         <v>1140</v>
       </c>
       <c r="I305">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -15745,7 +15745,7 @@
         <v>1140</v>
       </c>
       <c r="I306">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -15789,7 +15789,7 @@
         <v>1140</v>
       </c>
       <c r="I307">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K307" t="s">
         <v>1143</v>
@@ -15827,7 +15827,7 @@
         <v>1140</v>
       </c>
       <c r="I308">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K308" t="s">
         <v>1143</v>
@@ -15865,7 +15865,7 @@
         <v>1140</v>
       </c>
       <c r="I309">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K309" t="s">
         <v>1143</v>
@@ -15903,7 +15903,7 @@
         <v>1140</v>
       </c>
       <c r="I310">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K310" t="s">
         <v>1144</v>
@@ -15941,7 +15941,7 @@
         <v>1140</v>
       </c>
       <c r="I311">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K311" t="s">
         <v>1143</v>
@@ -15979,7 +15979,7 @@
         <v>1140</v>
       </c>
       <c r="I312">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K312" t="s">
         <v>1144</v>
@@ -16052,7 +16052,7 @@
         <v>1140</v>
       </c>
       <c r="I314">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K314" t="s">
         <v>1144</v>
@@ -16090,7 +16090,7 @@
         <v>1140</v>
       </c>
       <c r="I315">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K315" t="s">
         <v>1144</v>
@@ -16128,7 +16128,7 @@
         <v>1140</v>
       </c>
       <c r="I316">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K316" t="s">
         <v>1144</v>
@@ -16166,7 +16166,7 @@
         <v>1140</v>
       </c>
       <c r="I317">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K317" t="s">
         <v>1144</v>
@@ -16277,7 +16277,7 @@
         <v>1140</v>
       </c>
       <c r="I320">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K320" t="s">
         <v>1148</v>
@@ -16315,7 +16315,7 @@
         <v>1140</v>
       </c>
       <c r="I321">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K321" t="s">
         <v>1144</v>
@@ -16353,7 +16353,7 @@
         <v>1140</v>
       </c>
       <c r="I322">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16397,7 +16397,7 @@
         <v>1140</v>
       </c>
       <c r="I323">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K323" t="s">
         <v>1144</v>
@@ -16435,7 +16435,7 @@
         <v>1140</v>
       </c>
       <c r="I324">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K324" t="s">
         <v>1144</v>
@@ -16473,7 +16473,7 @@
         <v>1140</v>
       </c>
       <c r="I325">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16517,7 +16517,7 @@
         <v>1140</v>
       </c>
       <c r="I326">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K326" t="s">
         <v>1144</v>
@@ -16555,7 +16555,7 @@
         <v>1140</v>
       </c>
       <c r="I327">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16599,7 +16599,7 @@
         <v>1140</v>
       </c>
       <c r="I328">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16643,7 +16643,7 @@
         <v>1140</v>
       </c>
       <c r="I329">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16687,7 +16687,7 @@
         <v>1140</v>
       </c>
       <c r="I330">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -16731,7 +16731,7 @@
         <v>1140</v>
       </c>
       <c r="I331">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K331" t="s">
         <v>1143</v>
@@ -16769,7 +16769,7 @@
         <v>1140</v>
       </c>
       <c r="I332">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K332" t="s">
         <v>1144</v>
@@ -16807,7 +16807,7 @@
         <v>1140</v>
       </c>
       <c r="I333">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K333" t="s">
         <v>1147</v>
@@ -16845,7 +16845,7 @@
         <v>1140</v>
       </c>
       <c r="I334">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K334" t="s">
         <v>1144</v>
@@ -16924,7 +16924,7 @@
         <v>1140</v>
       </c>
       <c r="I336">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="K336" t="s">
         <v>1146</v>
@@ -17003,7 +17003,7 @@
         <v>1140</v>
       </c>
       <c r="I338">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="K338" t="s">
         <v>1146</v>
@@ -17070,7 +17070,7 @@
         <v>1140</v>
       </c>
       <c r="I340">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K340" t="s">
         <v>1143</v>
@@ -17108,7 +17108,7 @@
         <v>1140</v>
       </c>
       <c r="I341">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K341" t="s">
         <v>1143</v>
@@ -17146,7 +17146,7 @@
         <v>1140</v>
       </c>
       <c r="I342">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K342" t="s">
         <v>1143</v>
@@ -17184,7 +17184,7 @@
         <v>1140</v>
       </c>
       <c r="I343">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K343" t="s">
         <v>1144</v>
@@ -17222,7 +17222,7 @@
         <v>1140</v>
       </c>
       <c r="I344">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K344" t="s">
         <v>1144</v>
@@ -17260,7 +17260,7 @@
         <v>1140</v>
       </c>
       <c r="I345">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K345" t="s">
         <v>1143</v>
@@ -17298,7 +17298,7 @@
         <v>1140</v>
       </c>
       <c r="I346">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K346" t="s">
         <v>1144</v>
@@ -17336,7 +17336,7 @@
         <v>1140</v>
       </c>
       <c r="I347">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17380,7 +17380,7 @@
         <v>1140</v>
       </c>
       <c r="I348">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17424,7 +17424,7 @@
         <v>1140</v>
       </c>
       <c r="I349">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K349" t="s">
         <v>1148</v>
@@ -17462,7 +17462,7 @@
         <v>1140</v>
       </c>
       <c r="I350">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K350" t="s">
         <v>1150</v>
@@ -17497,7 +17497,7 @@
         <v>1140</v>
       </c>
       <c r="I351">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K351" t="s">
         <v>1148</v>
@@ -17535,7 +17535,7 @@
         <v>1140</v>
       </c>
       <c r="I352">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K352" t="s">
         <v>1148</v>
@@ -17573,7 +17573,7 @@
         <v>1140</v>
       </c>
       <c r="I353">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K353" t="s">
         <v>1147</v>
@@ -17611,7 +17611,7 @@
         <v>1140</v>
       </c>
       <c r="I354">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K354" t="s">
         <v>1147</v>
@@ -17649,7 +17649,7 @@
         <v>1140</v>
       </c>
       <c r="I355">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -17731,7 +17731,7 @@
         <v>1140</v>
       </c>
       <c r="I357">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K357" t="s">
         <v>1147</v>
@@ -17769,7 +17769,7 @@
         <v>1140</v>
       </c>
       <c r="I358">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K358" t="s">
         <v>1147</v>
@@ -17807,7 +17807,7 @@
         <v>1140</v>
       </c>
       <c r="I359">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K359" t="s">
         <v>1147</v>
@@ -17848,7 +17848,7 @@
         <v>1140</v>
       </c>
       <c r="I360">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K360" t="s">
         <v>1147</v>
@@ -17886,7 +17886,7 @@
         <v>1140</v>
       </c>
       <c r="I361">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K361" t="s">
         <v>1147</v>
@@ -17924,7 +17924,7 @@
         <v>1140</v>
       </c>
       <c r="I362">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K362" t="s">
         <v>1147</v>
@@ -17962,7 +17962,7 @@
         <v>1140</v>
       </c>
       <c r="I363">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K363" t="s">
         <v>1147</v>
@@ -18000,7 +18000,7 @@
         <v>1140</v>
       </c>
       <c r="I364">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K364" t="s">
         <v>1147</v>
@@ -18038,7 +18038,7 @@
         <v>1140</v>
       </c>
       <c r="I365">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K365" t="s">
         <v>1146</v>
@@ -18076,7 +18076,7 @@
         <v>1140</v>
       </c>
       <c r="I366">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K366" t="s">
         <v>1147</v>
@@ -18114,7 +18114,7 @@
         <v>1140</v>
       </c>
       <c r="I367">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K367" t="s">
         <v>1147</v>
@@ -18152,7 +18152,7 @@
         <v>1140</v>
       </c>
       <c r="I368">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K368" t="s">
         <v>1147</v>
@@ -18190,7 +18190,7 @@
         <v>1140</v>
       </c>
       <c r="I369">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K369" t="s">
         <v>1147</v>
@@ -18228,7 +18228,7 @@
         <v>1140</v>
       </c>
       <c r="I370">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K370" t="s">
         <v>1147</v>
@@ -18266,7 +18266,7 @@
         <v>1140</v>
       </c>
       <c r="I371">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18310,7 +18310,7 @@
         <v>1140</v>
       </c>
       <c r="I372">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18357,7 +18357,7 @@
         <v>1140</v>
       </c>
       <c r="I373">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K373" t="s">
         <v>1143</v>
@@ -18395,7 +18395,7 @@
         <v>1140</v>
       </c>
       <c r="I374">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K374" t="s">
         <v>1143</v>
@@ -18433,7 +18433,7 @@
         <v>1140</v>
       </c>
       <c r="I375">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K375" t="s">
         <v>1147</v>
@@ -18471,7 +18471,7 @@
         <v>1140</v>
       </c>
       <c r="I376">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K376" t="s">
         <v>1147</v>
@@ -18547,7 +18547,7 @@
         <v>1140</v>
       </c>
       <c r="I378">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K378" t="s">
         <v>1147</v>
@@ -18585,7 +18585,7 @@
         <v>1140</v>
       </c>
       <c r="I379">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18629,7 +18629,7 @@
         <v>1140</v>
       </c>
       <c r="I380">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K380" t="s">
         <v>1147</v>
@@ -18667,7 +18667,7 @@
         <v>1140</v>
       </c>
       <c r="I381">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K381" t="s">
         <v>1147</v>
@@ -18705,7 +18705,7 @@
         <v>1140</v>
       </c>
       <c r="I382">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K382" t="s">
         <v>1147</v>
@@ -18743,7 +18743,7 @@
         <v>1140</v>
       </c>
       <c r="I383">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K383" t="s">
         <v>1147</v>
@@ -18781,7 +18781,7 @@
         <v>1140</v>
       </c>
       <c r="I384">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K384" t="s">
         <v>1143</v>
@@ -18819,7 +18819,7 @@
         <v>1140</v>
       </c>
       <c r="I385">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K385" t="s">
         <v>1143</v>
@@ -18857,7 +18857,7 @@
         <v>1140</v>
       </c>
       <c r="I386">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K386" t="s">
         <v>1147</v>
@@ -18895,7 +18895,7 @@
         <v>1140</v>
       </c>
       <c r="I387">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K387" t="s">
         <v>1147</v>
@@ -18933,7 +18933,7 @@
         <v>1140</v>
       </c>
       <c r="I388">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K388" t="s">
         <v>1147</v>
@@ -18971,7 +18971,7 @@
         <v>1140</v>
       </c>
       <c r="I389">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K389" t="s">
         <v>1148</v>
@@ -19009,7 +19009,7 @@
         <v>1140</v>
       </c>
       <c r="I390">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19129,7 +19129,7 @@
         <v>1140</v>
       </c>
       <c r="I393">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K393" t="s">
         <v>1147</v>
@@ -19167,7 +19167,7 @@
         <v>1140</v>
       </c>
       <c r="I394">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K394" t="s">
         <v>1147</v>
@@ -19205,7 +19205,7 @@
         <v>1140</v>
       </c>
       <c r="I395">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K395" t="s">
         <v>1147</v>
@@ -19243,7 +19243,7 @@
         <v>1140</v>
       </c>
       <c r="I396">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K396" t="s">
         <v>1147</v>
@@ -19281,7 +19281,7 @@
         <v>1140</v>
       </c>
       <c r="I397">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K397" t="s">
         <v>1147</v>
@@ -19319,7 +19319,7 @@
         <v>1140</v>
       </c>
       <c r="I398">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K398" t="s">
         <v>1147</v>
@@ -19395,7 +19395,7 @@
         <v>1140</v>
       </c>
       <c r="I400">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K400" t="s">
         <v>1147</v>
@@ -19433,7 +19433,7 @@
         <v>1140</v>
       </c>
       <c r="I401">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K401" t="s">
         <v>1147</v>
@@ -19471,7 +19471,7 @@
         <v>1140</v>
       </c>
       <c r="I402">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K402" t="s">
         <v>1147</v>
@@ -19509,7 +19509,7 @@
         <v>1140</v>
       </c>
       <c r="I403">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K403" t="s">
         <v>1150</v>
@@ -19544,7 +19544,7 @@
         <v>1140</v>
       </c>
       <c r="I404">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K404" t="s">
         <v>1150</v>
@@ -19608,7 +19608,7 @@
         <v>1140</v>
       </c>
       <c r="I406">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19640,7 +19640,7 @@
         <v>1140</v>
       </c>
       <c r="I407">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19672,7 +19672,7 @@
         <v>1140</v>
       </c>
       <c r="I408">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19704,7 +19704,7 @@
         <v>1140</v>
       </c>
       <c r="I409">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -19736,7 +19736,7 @@
         <v>1140</v>
       </c>
       <c r="I410">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -19768,7 +19768,7 @@
         <v>1140</v>
       </c>
       <c r="I411">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -19800,7 +19800,7 @@
         <v>1140</v>
       </c>
       <c r="I412">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -19832,7 +19832,7 @@
         <v>1140</v>
       </c>
       <c r="I413">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -19864,7 +19864,7 @@
         <v>1140</v>
       </c>
       <c r="I414">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -19896,7 +19896,7 @@
         <v>1140</v>
       </c>
       <c r="I415">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -19928,7 +19928,7 @@
         <v>1140</v>
       </c>
       <c r="I416">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -19960,7 +19960,7 @@
         <v>1140</v>
       </c>
       <c r="I417">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -19992,7 +19992,7 @@
         <v>1140</v>
       </c>
       <c r="I418">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20024,7 +20024,7 @@
         <v>1140</v>
       </c>
       <c r="I419">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20056,7 +20056,7 @@
         <v>1140</v>
       </c>
       <c r="I420">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20088,7 +20088,7 @@
         <v>1140</v>
       </c>
       <c r="I421">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20120,7 +20120,7 @@
         <v>1140</v>
       </c>
       <c r="I422">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20152,7 +20152,7 @@
         <v>1140</v>
       </c>
       <c r="I423">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20184,7 +20184,7 @@
         <v>1140</v>
       </c>
       <c r="I424">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20216,7 +20216,7 @@
         <v>1140</v>
       </c>
       <c r="I425">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20248,7 +20248,7 @@
         <v>1140</v>
       </c>
       <c r="I426">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20280,7 +20280,7 @@
         <v>1140</v>
       </c>
       <c r="I427">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20312,7 +20312,7 @@
         <v>1140</v>
       </c>
       <c r="I428">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20344,7 +20344,7 @@
         <v>1140</v>
       </c>
       <c r="I429">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20376,7 +20376,7 @@
         <v>1140</v>
       </c>
       <c r="I430">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20408,7 +20408,7 @@
         <v>1140</v>
       </c>
       <c r="I431">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20440,7 +20440,7 @@
         <v>1140</v>
       </c>
       <c r="I432">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20472,7 +20472,7 @@
         <v>1140</v>
       </c>
       <c r="I433">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20504,7 +20504,7 @@
         <v>1140</v>
       </c>
       <c r="I434">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20536,7 +20536,7 @@
         <v>1140</v>
       </c>
       <c r="I435">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20568,7 +20568,7 @@
         <v>1140</v>
       </c>
       <c r="I436">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20600,7 +20600,7 @@
         <v>1142</v>
       </c>
       <c r="I437">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20632,7 +20632,7 @@
         <v>1142</v>
       </c>
       <c r="I438">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20664,7 +20664,7 @@
         <v>1140</v>
       </c>
       <c r="I439">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20696,7 +20696,7 @@
         <v>1140</v>
       </c>
       <c r="I440">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -20728,7 +20728,7 @@
         <v>1140</v>
       </c>
       <c r="I441">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -20760,7 +20760,7 @@
         <v>1140</v>
       </c>
       <c r="I442">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -20792,7 +20792,7 @@
         <v>1140</v>
       </c>
       <c r="I443">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -20824,7 +20824,7 @@
         <v>1140</v>
       </c>
       <c r="I444">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -20856,7 +20856,7 @@
         <v>1140</v>
       </c>
       <c r="I445">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -20888,7 +20888,7 @@
         <v>1140</v>
       </c>
       <c r="I446">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -20920,7 +20920,7 @@
         <v>1140</v>
       </c>
       <c r="I447">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (04/08/2026 05:12)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4541,7 +4541,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4579,7 +4579,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4617,7 +4617,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4655,7 +4655,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4699,7 +4699,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4743,7 +4743,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4819,7 +4819,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4866,7 +4866,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4913,7 +4913,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4960,7 +4960,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5039,7 +5039,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5083,7 +5083,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5121,7 +5121,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5159,7 +5159,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5203,7 +5203,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5282,7 +5282,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5361,7 +5361,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5399,7 +5399,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5522,7 +5522,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5569,7 +5569,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5674,7 +5674,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5756,7 +5756,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -5998,7 +5998,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6033,7 +6033,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6182,7 +6182,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6229,7 +6229,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6276,7 +6276,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6314,7 +6314,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6361,7 +6361,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6431,7 +6431,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6507,7 +6507,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6545,7 +6545,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6583,7 +6583,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6691,7 +6691,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6895,7 +6895,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6942,7 +6942,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7173,7 +7173,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7211,7 +7211,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7281,7 +7281,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7357,7 +7357,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7395,7 +7395,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7503,7 +7503,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7538,7 +7538,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7614,7 +7614,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7687,7 +7687,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7734,7 +7734,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7772,7 +7772,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7810,7 +7810,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7927,7 +7927,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7968,7 +7968,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8035,7 +8035,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8073,7 +8073,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8111,7 +8111,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8149,7 +8149,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8196,7 +8196,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8237,7 +8237,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8304,7 +8304,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8432,7 +8432,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8470,7 +8470,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8508,7 +8508,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8552,7 +8552,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8596,7 +8596,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8634,7 +8634,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8850,7 +8850,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8888,7 +8888,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8926,7 +8926,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8964,7 +8964,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9002,7 +9002,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9040,7 +9040,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9078,7 +9078,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9125,7 +9125,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9192,7 +9192,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9230,7 +9230,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9335,7 +9335,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9373,7 +9373,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9411,7 +9411,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9493,7 +9493,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9569,7 +9569,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9700,7 +9700,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10029,7 +10029,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10067,7 +10067,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10102,7 +10102,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10187,7 +10187,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10231,7 +10231,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10304,7 +10304,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10339,7 +10339,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10377,7 +10377,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10415,7 +10415,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10459,7 +10459,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10497,7 +10497,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10535,7 +10535,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10582,7 +10582,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10626,7 +10626,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10670,7 +10670,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10810,7 +10810,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10851,7 +10851,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10933,7 +10933,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11079,7 +11079,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11126,7 +11126,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11164,7 +11164,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11211,7 +11211,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11278,7 +11278,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11383,7 +11383,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11418,7 +11418,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11453,7 +11453,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11491,7 +11491,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11529,7 +11529,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11576,7 +11576,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11623,7 +11623,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11667,7 +11667,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11705,7 +11705,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11749,7 +11749,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11787,7 +11787,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11857,7 +11857,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -11991,7 +11991,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12035,7 +12035,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12073,7 +12073,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12111,7 +12111,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12149,7 +12149,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12187,7 +12187,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12225,7 +12225,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12298,7 +12298,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12342,7 +12342,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12386,7 +12386,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12430,7 +12430,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12538,7 +12538,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12576,7 +12576,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12623,7 +12623,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12690,7 +12690,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12734,7 +12734,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12772,7 +12772,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12810,7 +12810,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12886,7 +12886,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12924,7 +12924,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12962,7 +12962,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13000,7 +13000,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13038,7 +13038,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13076,7 +13076,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13114,7 +13114,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13187,7 +13187,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13225,7 +13225,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13339,7 +13339,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13386,7 +13386,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13433,7 +13433,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13477,7 +13477,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13544,7 +13544,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13655,7 +13655,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13725,7 +13725,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13763,7 +13763,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13801,7 +13801,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13906,7 +13906,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13944,7 +13944,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14052,7 +14052,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14090,7 +14090,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14128,7 +14128,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14166,7 +14166,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14265,7 +14265,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14303,7 +14303,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14341,7 +14341,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14379,7 +14379,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14464,7 +14464,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14502,7 +14502,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14540,7 +14540,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14578,7 +14578,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14616,7 +14616,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14651,7 +14651,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14689,7 +14689,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14727,7 +14727,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14765,7 +14765,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14847,7 +14847,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14920,7 +14920,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14958,7 +14958,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -14996,7 +14996,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15034,7 +15034,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15075,7 +15075,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15113,7 +15113,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15151,7 +15151,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15358,7 +15358,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15425,7 +15425,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15466,7 +15466,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15504,7 +15504,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15542,7 +15542,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15580,7 +15580,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15615,7 +15615,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15650,7 +15650,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15720,7 +15720,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15758,7 +15758,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15796,7 +15796,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15834,7 +15834,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15872,7 +15872,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15910,7 +15910,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15948,7 +15948,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -15986,7 +15986,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16030,7 +16030,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16074,7 +16074,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16112,7 +16112,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16150,7 +16150,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16188,7 +16188,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16226,7 +16226,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16264,7 +16264,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16337,7 +16337,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16375,7 +16375,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16413,7 +16413,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16451,7 +16451,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16562,7 +16562,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16600,7 +16600,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16638,7 +16638,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16682,7 +16682,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16720,7 +16720,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16758,7 +16758,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16802,7 +16802,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16840,7 +16840,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16884,7 +16884,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16928,7 +16928,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16972,7 +16972,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17016,7 +17016,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17054,7 +17054,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17092,7 +17092,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17130,7 +17130,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17209,7 +17209,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17288,7 +17288,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17355,7 +17355,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17393,7 +17393,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17431,7 +17431,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17469,7 +17469,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17507,7 +17507,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17545,7 +17545,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17583,7 +17583,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17621,7 +17621,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17665,7 +17665,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17709,7 +17709,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17747,7 +17747,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17782,7 +17782,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17820,7 +17820,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17858,7 +17858,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17896,7 +17896,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17934,7 +17934,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18016,7 +18016,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18054,7 +18054,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18130,7 +18130,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18168,7 +18168,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18206,7 +18206,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18244,7 +18244,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18282,7 +18282,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18320,7 +18320,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18358,7 +18358,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18396,7 +18396,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18434,7 +18434,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18472,7 +18472,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18510,7 +18510,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18548,7 +18548,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18592,7 +18592,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18639,7 +18639,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18677,7 +18677,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18715,7 +18715,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18753,7 +18753,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18829,7 +18829,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18867,7 +18867,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18911,7 +18911,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18949,7 +18949,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -18987,7 +18987,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19025,7 +19025,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19063,7 +19063,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19101,7 +19101,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19139,7 +19139,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19177,7 +19177,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19215,7 +19215,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19253,7 +19253,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19291,7 +19291,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19411,7 +19411,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19449,7 +19449,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19487,7 +19487,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19525,7 +19525,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19563,7 +19563,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19601,7 +19601,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19677,7 +19677,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19715,7 +19715,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19753,7 +19753,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19791,7 +19791,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19826,7 +19826,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19890,7 +19890,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19922,7 +19922,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19954,7 +19954,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19986,7 +19986,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20018,7 +20018,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20050,7 +20050,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20082,7 +20082,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20114,7 +20114,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20146,7 +20146,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20178,7 +20178,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20210,7 +20210,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20242,7 +20242,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20274,7 +20274,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20306,7 +20306,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20338,7 +20338,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20370,7 +20370,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20402,7 +20402,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20434,7 +20434,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20466,7 +20466,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20498,7 +20498,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20530,7 +20530,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20562,7 +20562,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20594,7 +20594,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20626,7 +20626,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20658,7 +20658,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20690,7 +20690,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20722,7 +20722,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20754,7 +20754,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20786,7 +20786,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20818,7 +20818,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20850,7 +20850,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20882,7 +20882,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20914,7 +20914,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20946,7 +20946,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20978,7 +20978,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21010,7 +21010,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21042,7 +21042,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21074,7 +21074,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21106,7 +21106,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21138,7 +21138,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21170,7 +21170,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21202,7 +21202,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21234,7 +21234,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21266,7 +21266,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21298,7 +21298,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21330,7 +21330,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21362,7 +21362,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21394,7 +21394,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21426,7 +21426,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21458,7 +21458,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21490,7 +21490,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21522,7 +21522,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21554,7 +21554,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21586,7 +21586,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21618,7 +21618,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21650,7 +21650,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21682,7 +21682,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21714,7 +21714,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21746,7 +21746,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21778,7 +21778,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21810,7 +21810,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21842,7 +21842,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21874,7 +21874,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22322,7 +22322,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22354,7 +22354,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22386,7 +22386,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22418,7 +22418,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22450,7 +22450,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22482,7 +22482,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22514,7 +22514,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22546,7 +22546,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22578,7 +22578,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22610,7 +22610,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22642,7 +22642,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22674,7 +22674,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22706,7 +22706,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22738,7 +22738,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22770,7 +22770,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22802,7 +22802,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22834,7 +22834,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22866,7 +22866,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22898,7 +22898,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22930,7 +22930,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -22962,7 +22962,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -22994,7 +22994,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23026,7 +23026,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23058,7 +23058,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23090,7 +23090,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23122,7 +23122,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23154,7 +23154,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23186,7 +23186,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23218,7 +23218,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (05/08/2026 05:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4541,7 +4541,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4579,7 +4579,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4617,7 +4617,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4655,7 +4655,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4699,7 +4699,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4743,7 +4743,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4819,7 +4819,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4866,7 +4866,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4913,7 +4913,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4960,7 +4960,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5039,7 +5039,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5083,7 +5083,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5121,7 +5121,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5159,7 +5159,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5203,7 +5203,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5282,7 +5282,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5361,7 +5361,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5399,7 +5399,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5522,7 +5522,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5569,7 +5569,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5674,7 +5674,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5756,7 +5756,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -5998,7 +5998,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6033,7 +6033,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6182,7 +6182,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6229,7 +6229,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6276,7 +6276,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6314,7 +6314,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6361,7 +6361,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6431,7 +6431,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6507,7 +6507,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6545,7 +6545,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6583,7 +6583,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6691,7 +6691,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6895,7 +6895,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6942,7 +6942,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7173,7 +7173,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7211,7 +7211,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7281,7 +7281,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7357,7 +7357,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7395,7 +7395,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7503,7 +7503,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7538,7 +7538,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7614,7 +7614,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7687,7 +7687,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7734,7 +7734,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7772,7 +7772,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7810,7 +7810,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7927,7 +7927,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7968,7 +7968,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8035,7 +8035,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8073,7 +8073,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8111,7 +8111,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8149,7 +8149,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8196,7 +8196,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8237,7 +8237,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8304,7 +8304,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8432,7 +8432,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8470,7 +8470,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8508,7 +8508,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8552,7 +8552,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8596,7 +8596,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8634,7 +8634,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8850,7 +8850,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8888,7 +8888,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8926,7 +8926,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8964,7 +8964,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9002,7 +9002,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9040,7 +9040,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9078,7 +9078,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9125,7 +9125,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9192,7 +9192,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9230,7 +9230,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9335,7 +9335,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9373,7 +9373,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9411,7 +9411,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9493,7 +9493,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9569,7 +9569,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9700,7 +9700,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10029,7 +10029,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10067,7 +10067,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10102,7 +10102,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10187,7 +10187,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10231,7 +10231,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10304,7 +10304,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10339,7 +10339,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10377,7 +10377,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10415,7 +10415,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10459,7 +10459,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10497,7 +10497,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10535,7 +10535,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10582,7 +10582,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10626,7 +10626,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10670,7 +10670,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10810,7 +10810,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10851,7 +10851,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10933,7 +10933,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11079,7 +11079,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11126,7 +11126,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11164,7 +11164,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11211,7 +11211,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11278,7 +11278,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11383,7 +11383,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11418,7 +11418,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11453,7 +11453,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11491,7 +11491,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11529,7 +11529,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11576,7 +11576,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11623,7 +11623,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11667,7 +11667,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11705,7 +11705,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11749,7 +11749,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11787,7 +11787,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11857,7 +11857,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -11991,7 +11991,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12035,7 +12035,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12073,7 +12073,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12111,7 +12111,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12149,7 +12149,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12187,7 +12187,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12225,7 +12225,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12298,7 +12298,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12342,7 +12342,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12386,7 +12386,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12430,7 +12430,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12538,7 +12538,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12576,7 +12576,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12623,7 +12623,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12690,7 +12690,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12734,7 +12734,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12772,7 +12772,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12810,7 +12810,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12886,7 +12886,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12924,7 +12924,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12962,7 +12962,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13000,7 +13000,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13038,7 +13038,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13076,7 +13076,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13114,7 +13114,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13187,7 +13187,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13225,7 +13225,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13339,7 +13339,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13386,7 +13386,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13433,7 +13433,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13477,7 +13477,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13544,7 +13544,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13655,7 +13655,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13725,7 +13725,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13763,7 +13763,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13801,7 +13801,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13906,7 +13906,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13944,7 +13944,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14052,7 +14052,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14090,7 +14090,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14128,7 +14128,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14166,7 +14166,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14265,7 +14265,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14303,7 +14303,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14341,7 +14341,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14379,7 +14379,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14464,7 +14464,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14502,7 +14502,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14540,7 +14540,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14578,7 +14578,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14616,7 +14616,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14651,7 +14651,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14689,7 +14689,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14727,7 +14727,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14765,7 +14765,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14847,7 +14847,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14920,7 +14920,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14958,7 +14958,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -14996,7 +14996,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15034,7 +15034,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15075,7 +15075,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15113,7 +15113,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15151,7 +15151,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15358,7 +15358,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15425,7 +15425,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15466,7 +15466,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15504,7 +15504,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15542,7 +15542,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15580,7 +15580,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15615,7 +15615,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15650,7 +15650,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15720,7 +15720,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15758,7 +15758,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15796,7 +15796,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15834,7 +15834,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15872,7 +15872,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15910,7 +15910,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15948,7 +15948,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -15986,7 +15986,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16030,7 +16030,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16074,7 +16074,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16112,7 +16112,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16150,7 +16150,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16188,7 +16188,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16226,7 +16226,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16264,7 +16264,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16337,7 +16337,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16375,7 +16375,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16413,7 +16413,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16451,7 +16451,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16562,7 +16562,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16600,7 +16600,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16638,7 +16638,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16682,7 +16682,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16720,7 +16720,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16758,7 +16758,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16802,7 +16802,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16840,7 +16840,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16884,7 +16884,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16928,7 +16928,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16972,7 +16972,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17016,7 +17016,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17054,7 +17054,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17092,7 +17092,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17130,7 +17130,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17209,7 +17209,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17288,7 +17288,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17355,7 +17355,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17393,7 +17393,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17431,7 +17431,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17469,7 +17469,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17507,7 +17507,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17545,7 +17545,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17583,7 +17583,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17621,7 +17621,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17665,7 +17665,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17709,7 +17709,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17747,7 +17747,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17782,7 +17782,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17820,7 +17820,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17858,7 +17858,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17896,7 +17896,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17934,7 +17934,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18016,7 +18016,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18054,7 +18054,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18130,7 +18130,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18168,7 +18168,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18206,7 +18206,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18244,7 +18244,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18282,7 +18282,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18320,7 +18320,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18358,7 +18358,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18396,7 +18396,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18434,7 +18434,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18472,7 +18472,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18510,7 +18510,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18548,7 +18548,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18592,7 +18592,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18639,7 +18639,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18677,7 +18677,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18715,7 +18715,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18753,7 +18753,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18829,7 +18829,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18867,7 +18867,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18911,7 +18911,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18949,7 +18949,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -18987,7 +18987,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19025,7 +19025,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19063,7 +19063,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19101,7 +19101,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19139,7 +19139,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19177,7 +19177,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19215,7 +19215,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19253,7 +19253,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19291,7 +19291,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19411,7 +19411,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19449,7 +19449,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19487,7 +19487,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19525,7 +19525,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19563,7 +19563,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19601,7 +19601,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19677,7 +19677,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19715,7 +19715,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19753,7 +19753,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19791,7 +19791,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19826,7 +19826,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19890,7 +19890,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19922,7 +19922,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19954,7 +19954,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -19986,7 +19986,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20018,7 +20018,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20050,7 +20050,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20082,7 +20082,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20114,7 +20114,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20146,7 +20146,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20178,7 +20178,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20210,7 +20210,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20242,7 +20242,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20274,7 +20274,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20306,7 +20306,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20338,7 +20338,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20370,7 +20370,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20402,7 +20402,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20434,7 +20434,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20466,7 +20466,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20498,7 +20498,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20530,7 +20530,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20562,7 +20562,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20594,7 +20594,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20626,7 +20626,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20658,7 +20658,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20690,7 +20690,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20722,7 +20722,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20754,7 +20754,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20786,7 +20786,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20818,7 +20818,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20850,7 +20850,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20882,7 +20882,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20914,7 +20914,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20946,7 +20946,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20978,7 +20978,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21010,7 +21010,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21042,7 +21042,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21074,7 +21074,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21106,7 +21106,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21138,7 +21138,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21170,7 +21170,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21202,7 +21202,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21234,7 +21234,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21266,7 +21266,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21298,7 +21298,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21330,7 +21330,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21362,7 +21362,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21394,7 +21394,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21426,7 +21426,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21458,7 +21458,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21490,7 +21490,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21522,7 +21522,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21554,7 +21554,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21586,7 +21586,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21618,7 +21618,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21650,7 +21650,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21682,7 +21682,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21714,7 +21714,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21746,7 +21746,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21778,7 +21778,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21810,7 +21810,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21842,7 +21842,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21874,7 +21874,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22322,7 +22322,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22354,7 +22354,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22386,7 +22386,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22418,7 +22418,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22450,7 +22450,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22482,7 +22482,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22514,7 +22514,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22546,7 +22546,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22578,7 +22578,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22610,7 +22610,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22642,7 +22642,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22674,7 +22674,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22706,7 +22706,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22738,7 +22738,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22770,7 +22770,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22802,7 +22802,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22834,7 +22834,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22866,7 +22866,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22898,7 +22898,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22930,7 +22930,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -22962,7 +22962,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -22994,7 +22994,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23026,7 +23026,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23058,7 +23058,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23090,7 +23090,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23122,7 +23122,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23154,7 +23154,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23186,7 +23186,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23218,7 +23218,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (05/08/2026 10:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4120" uniqueCount="1370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4122" uniqueCount="1371">
   <si>
     <t>os</t>
   </si>
@@ -4124,6 +4124,9 @@
   </si>
   <si>
     <t>024/2026</t>
+  </si>
+  <si>
+    <t>088/2026</t>
   </si>
 </sst>
 </file>
@@ -19495,6 +19498,9 @@
       <c r="M395" t="s">
         <v>1337</v>
       </c>
+      <c r="P395" t="s">
+        <v>1370</v>
+      </c>
       <c r="Q395" t="b">
         <v>1</v>
       </c>
@@ -19608,6 +19614,9 @@
       </c>
       <c r="M398" t="s">
         <v>1337</v>
+      </c>
+      <c r="P398" t="s">
+        <v>1370</v>
       </c>
       <c r="Q398" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (05/08/2026 15:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4122" uniqueCount="1371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4123" uniqueCount="1372">
   <si>
     <t>os</t>
   </si>
@@ -4109,6 +4109,9 @@
   </si>
   <si>
     <t>037/2025</t>
+  </si>
+  <si>
+    <t>029/2026</t>
   </si>
   <si>
     <t>007/2026</t>
@@ -12783,6 +12786,9 @@
       <c r="M219" t="s">
         <v>1339</v>
       </c>
+      <c r="P219" t="s">
+        <v>1365</v>
+      </c>
       <c r="Q219" t="b">
         <v>1</v>
       </c>
@@ -13357,7 +13363,7 @@
         <v>46063</v>
       </c>
       <c r="P234" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="Q234" t="b">
         <v>1</v>
@@ -13404,7 +13410,7 @@
         <v>46063</v>
       </c>
       <c r="P235" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="Q235" t="b">
         <v>1</v>
@@ -14397,7 +14403,7 @@
         <v>46113</v>
       </c>
       <c r="P262" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="Q262" t="b">
         <v>1</v>
@@ -15046,7 +15052,7 @@
         <v>1339</v>
       </c>
       <c r="P279" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="Q279" t="b">
         <v>1</v>
@@ -18101,7 +18107,7 @@
         <v>1337</v>
       </c>
       <c r="P359" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="Q359" t="b">
         <v>0</v>
@@ -18610,7 +18616,7 @@
         <v>46113</v>
       </c>
       <c r="P372" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="Q372" t="b">
         <v>1</v>
@@ -18800,7 +18806,7 @@
         <v>1341</v>
       </c>
       <c r="P377" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="Q377" t="b">
         <v>0</v>
@@ -19344,7 +19350,7 @@
         <v>1337</v>
       </c>
       <c r="P391" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="Q391" t="b">
         <v>0</v>
@@ -19499,7 +19505,7 @@
         <v>1337</v>
       </c>
       <c r="P395" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="Q395" t="b">
         <v>1</v>
@@ -19616,7 +19622,7 @@
         <v>1337</v>
       </c>
       <c r="P398" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="Q398" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (06/08/2026 10:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4547,7 +4547,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4585,7 +4585,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4623,7 +4623,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4661,7 +4661,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4705,7 +4705,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4749,7 +4749,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4825,7 +4825,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4872,7 +4872,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4919,7 +4919,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4966,7 +4966,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5045,7 +5045,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5089,7 +5089,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5127,7 +5127,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5165,7 +5165,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5209,7 +5209,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5288,7 +5288,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5367,7 +5367,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5405,7 +5405,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5528,7 +5528,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5575,7 +5575,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5680,7 +5680,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5762,7 +5762,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -6004,7 +6004,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6039,7 +6039,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6188,7 +6188,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6235,7 +6235,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6282,7 +6282,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6320,7 +6320,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6367,7 +6367,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6437,7 +6437,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6513,7 +6513,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6551,7 +6551,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6589,7 +6589,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6697,7 +6697,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6901,7 +6901,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6948,7 +6948,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7179,7 +7179,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7217,7 +7217,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7287,7 +7287,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7363,7 +7363,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7401,7 +7401,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7509,7 +7509,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7544,7 +7544,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7620,7 +7620,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7693,7 +7693,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7740,7 +7740,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7778,7 +7778,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7816,7 +7816,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7933,7 +7933,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7974,7 +7974,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8041,7 +8041,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8079,7 +8079,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8117,7 +8117,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8155,7 +8155,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8202,7 +8202,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8243,7 +8243,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8310,7 +8310,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8438,7 +8438,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8476,7 +8476,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8514,7 +8514,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8558,7 +8558,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8602,7 +8602,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8640,7 +8640,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8856,7 +8856,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8894,7 +8894,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8932,7 +8932,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8970,7 +8970,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9008,7 +9008,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9046,7 +9046,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9084,7 +9084,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9131,7 +9131,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9198,7 +9198,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9236,7 +9236,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9341,7 +9341,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9379,7 +9379,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9417,7 +9417,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9499,7 +9499,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9575,7 +9575,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9706,7 +9706,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10035,7 +10035,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10073,7 +10073,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10108,7 +10108,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10193,7 +10193,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10237,7 +10237,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10310,7 +10310,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10345,7 +10345,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10383,7 +10383,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10421,7 +10421,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10465,7 +10465,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10503,7 +10503,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10541,7 +10541,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10588,7 +10588,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10632,7 +10632,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10676,7 +10676,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10816,7 +10816,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10857,7 +10857,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10939,7 +10939,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11085,7 +11085,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11132,7 +11132,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11170,7 +11170,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11217,7 +11217,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11284,7 +11284,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11389,7 +11389,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11424,7 +11424,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11459,7 +11459,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11497,7 +11497,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11535,7 +11535,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11582,7 +11582,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11629,7 +11629,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11673,7 +11673,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11711,7 +11711,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11755,7 +11755,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11793,7 +11793,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11863,7 +11863,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -11997,7 +11997,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12041,7 +12041,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12079,7 +12079,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12117,7 +12117,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12155,7 +12155,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12193,7 +12193,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12231,7 +12231,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12304,7 +12304,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12348,7 +12348,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12392,7 +12392,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12436,7 +12436,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12544,7 +12544,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12582,7 +12582,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12629,7 +12629,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12696,7 +12696,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12740,7 +12740,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12778,7 +12778,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12819,7 +12819,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12895,7 +12895,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12933,7 +12933,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12971,7 +12971,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13009,7 +13009,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13047,7 +13047,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13085,7 +13085,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13123,7 +13123,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13196,7 +13196,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13234,7 +13234,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13348,7 +13348,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13395,7 +13395,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13442,7 +13442,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13486,7 +13486,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13553,7 +13553,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13664,7 +13664,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13734,7 +13734,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13772,7 +13772,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13810,7 +13810,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13915,7 +13915,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13953,7 +13953,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14061,7 +14061,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14099,7 +14099,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14137,7 +14137,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14175,7 +14175,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14274,7 +14274,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14312,7 +14312,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14350,7 +14350,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14388,7 +14388,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14473,7 +14473,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14511,7 +14511,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14549,7 +14549,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14587,7 +14587,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14625,7 +14625,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14660,7 +14660,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14698,7 +14698,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14736,7 +14736,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14774,7 +14774,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14856,7 +14856,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14929,7 +14929,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14967,7 +14967,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -15005,7 +15005,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15043,7 +15043,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15084,7 +15084,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15122,7 +15122,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15160,7 +15160,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15367,7 +15367,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15434,7 +15434,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15475,7 +15475,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15513,7 +15513,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15551,7 +15551,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15589,7 +15589,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15624,7 +15624,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15659,7 +15659,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15729,7 +15729,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15767,7 +15767,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15805,7 +15805,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15843,7 +15843,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15881,7 +15881,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15919,7 +15919,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15957,7 +15957,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -15995,7 +15995,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16039,7 +16039,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16083,7 +16083,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16121,7 +16121,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16159,7 +16159,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16197,7 +16197,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16235,7 +16235,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16273,7 +16273,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16346,7 +16346,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16384,7 +16384,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16422,7 +16422,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16460,7 +16460,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16571,7 +16571,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16609,7 +16609,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16647,7 +16647,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16691,7 +16691,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16729,7 +16729,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16767,7 +16767,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16811,7 +16811,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16849,7 +16849,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16893,7 +16893,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16937,7 +16937,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16981,7 +16981,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17025,7 +17025,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17063,7 +17063,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17101,7 +17101,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17139,7 +17139,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17218,7 +17218,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17297,7 +17297,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17364,7 +17364,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17402,7 +17402,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17440,7 +17440,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17478,7 +17478,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17516,7 +17516,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17554,7 +17554,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17592,7 +17592,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17630,7 +17630,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17674,7 +17674,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17718,7 +17718,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17756,7 +17756,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17791,7 +17791,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17829,7 +17829,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17867,7 +17867,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17905,7 +17905,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17943,7 +17943,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18025,7 +18025,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18063,7 +18063,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18139,7 +18139,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18177,7 +18177,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18215,7 +18215,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18253,7 +18253,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18291,7 +18291,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18329,7 +18329,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18367,7 +18367,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18405,7 +18405,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18443,7 +18443,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18481,7 +18481,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18519,7 +18519,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18557,7 +18557,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18601,7 +18601,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18648,7 +18648,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18686,7 +18686,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18724,7 +18724,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18762,7 +18762,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18838,7 +18838,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18876,7 +18876,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18920,7 +18920,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18958,7 +18958,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -18996,7 +18996,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19034,7 +19034,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19072,7 +19072,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19110,7 +19110,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19148,7 +19148,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19186,7 +19186,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19224,7 +19224,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19262,7 +19262,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19300,7 +19300,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19420,7 +19420,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19458,7 +19458,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19496,7 +19496,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19537,7 +19537,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19575,7 +19575,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19613,7 +19613,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19692,7 +19692,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19730,7 +19730,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19768,7 +19768,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19806,7 +19806,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19841,7 +19841,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19905,7 +19905,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19937,7 +19937,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19969,7 +19969,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20001,7 +20001,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20033,7 +20033,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20065,7 +20065,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20097,7 +20097,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20129,7 +20129,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20161,7 +20161,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20193,7 +20193,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20225,7 +20225,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20257,7 +20257,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20289,7 +20289,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20321,7 +20321,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20353,7 +20353,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20385,7 +20385,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20417,7 +20417,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20449,7 +20449,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20481,7 +20481,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20513,7 +20513,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20545,7 +20545,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20577,7 +20577,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20609,7 +20609,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20641,7 +20641,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20673,7 +20673,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20705,7 +20705,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20737,7 +20737,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20769,7 +20769,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20801,7 +20801,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20833,7 +20833,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20865,7 +20865,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20897,7 +20897,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20929,7 +20929,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20961,7 +20961,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20993,7 +20993,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21025,7 +21025,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21441,7 +21441,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21473,7 +21473,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21505,7 +21505,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21537,7 +21537,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21569,7 +21569,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21601,7 +21601,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21633,7 +21633,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21665,7 +21665,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21697,7 +21697,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21729,7 +21729,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21761,7 +21761,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21793,7 +21793,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21825,7 +21825,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21857,7 +21857,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21889,7 +21889,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21921,7 +21921,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21953,7 +21953,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -21985,7 +21985,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22017,7 +22017,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22049,7 +22049,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22081,7 +22081,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22113,7 +22113,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22145,7 +22145,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22177,7 +22177,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22209,7 +22209,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22241,7 +22241,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22273,7 +22273,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22305,7 +22305,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22337,7 +22337,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22369,7 +22369,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22401,7 +22401,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22433,7 +22433,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22465,7 +22465,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22497,7 +22497,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22529,7 +22529,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22561,7 +22561,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22593,7 +22593,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22625,7 +22625,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22657,7 +22657,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22689,7 +22689,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22721,7 +22721,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22753,7 +22753,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22785,7 +22785,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22817,7 +22817,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22849,7 +22849,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22881,7 +22881,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22913,7 +22913,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22945,7 +22945,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -22977,7 +22977,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23009,7 +23009,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23041,7 +23041,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23073,7 +23073,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23105,7 +23105,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23137,7 +23137,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23169,7 +23169,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23201,7 +23201,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23233,7 +23233,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (07/08/2026 08:53)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4547,7 +4547,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4585,7 +4585,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4623,7 +4623,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4661,7 +4661,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4705,7 +4705,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4749,7 +4749,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4825,7 +4825,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4872,7 +4872,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4919,7 +4919,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4966,7 +4966,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5045,7 +5045,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5089,7 +5089,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5127,7 +5127,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5165,7 +5165,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5209,7 +5209,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5288,7 +5288,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5367,7 +5367,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5405,7 +5405,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5528,7 +5528,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5575,7 +5575,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5680,7 +5680,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5762,7 +5762,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -6004,7 +6004,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6039,7 +6039,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6188,7 +6188,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6235,7 +6235,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6282,7 +6282,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6320,7 +6320,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6367,7 +6367,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6437,7 +6437,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6513,7 +6513,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6551,7 +6551,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6589,7 +6589,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6697,7 +6697,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6901,7 +6901,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6948,7 +6948,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7179,7 +7179,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7217,7 +7217,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7287,7 +7287,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7363,7 +7363,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7401,7 +7401,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7509,7 +7509,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7544,7 +7544,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7620,7 +7620,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7693,7 +7693,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7740,7 +7740,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7778,7 +7778,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7816,7 +7816,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7933,7 +7933,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7974,7 +7974,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8041,7 +8041,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8079,7 +8079,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8117,7 +8117,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8155,7 +8155,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8202,7 +8202,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8243,7 +8243,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8310,7 +8310,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8438,7 +8438,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8476,7 +8476,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8514,7 +8514,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8558,7 +8558,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8602,7 +8602,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8640,7 +8640,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8856,7 +8856,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8894,7 +8894,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8932,7 +8932,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8970,7 +8970,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9008,7 +9008,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9046,7 +9046,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9084,7 +9084,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9131,7 +9131,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9198,7 +9198,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9236,7 +9236,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9341,7 +9341,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9379,7 +9379,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9417,7 +9417,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9499,7 +9499,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9575,7 +9575,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9706,7 +9706,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10035,7 +10035,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10073,7 +10073,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10108,7 +10108,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10193,7 +10193,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10237,7 +10237,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10310,7 +10310,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10345,7 +10345,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10383,7 +10383,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10421,7 +10421,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10465,7 +10465,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10503,7 +10503,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10541,7 +10541,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10588,7 +10588,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10632,7 +10632,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10676,7 +10676,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10816,7 +10816,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10857,7 +10857,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10939,7 +10939,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11085,7 +11085,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11132,7 +11132,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11170,7 +11170,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11217,7 +11217,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11284,7 +11284,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11389,7 +11389,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11424,7 +11424,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11459,7 +11459,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11497,7 +11497,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11535,7 +11535,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11582,7 +11582,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11629,7 +11629,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11673,7 +11673,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11711,7 +11711,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11755,7 +11755,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11793,7 +11793,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11863,7 +11863,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -11997,7 +11997,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12041,7 +12041,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12079,7 +12079,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12117,7 +12117,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12155,7 +12155,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12193,7 +12193,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12231,7 +12231,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12304,7 +12304,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12348,7 +12348,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12392,7 +12392,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12436,7 +12436,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12544,7 +12544,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12582,7 +12582,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12629,7 +12629,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12696,7 +12696,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12740,7 +12740,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12778,7 +12778,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12819,7 +12819,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12895,7 +12895,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12933,7 +12933,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12971,7 +12971,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13009,7 +13009,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13047,7 +13047,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13085,7 +13085,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13123,7 +13123,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13196,7 +13196,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13234,7 +13234,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13348,7 +13348,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13395,7 +13395,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13442,7 +13442,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13486,7 +13486,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13553,7 +13553,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13664,7 +13664,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13734,7 +13734,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13772,7 +13772,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13810,7 +13810,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13915,7 +13915,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13953,7 +13953,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14061,7 +14061,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14099,7 +14099,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14137,7 +14137,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14175,7 +14175,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14274,7 +14274,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14312,7 +14312,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14350,7 +14350,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14388,7 +14388,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14473,7 +14473,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14511,7 +14511,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14549,7 +14549,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14587,7 +14587,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14625,7 +14625,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14660,7 +14660,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14698,7 +14698,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14736,7 +14736,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14774,7 +14774,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14856,7 +14856,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14929,7 +14929,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14967,7 +14967,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -15005,7 +15005,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15043,7 +15043,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15084,7 +15084,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15122,7 +15122,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15160,7 +15160,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15367,7 +15367,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15434,7 +15434,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15475,7 +15475,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15513,7 +15513,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15551,7 +15551,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15589,7 +15589,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15624,7 +15624,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15659,7 +15659,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15729,7 +15729,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15767,7 +15767,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15805,7 +15805,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15843,7 +15843,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15881,7 +15881,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15919,7 +15919,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15957,7 +15957,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -15995,7 +15995,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16039,7 +16039,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16083,7 +16083,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16121,7 +16121,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16159,7 +16159,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16197,7 +16197,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16235,7 +16235,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16273,7 +16273,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16346,7 +16346,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16384,7 +16384,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16422,7 +16422,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16460,7 +16460,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16571,7 +16571,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16609,7 +16609,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16647,7 +16647,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16691,7 +16691,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16729,7 +16729,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16767,7 +16767,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16811,7 +16811,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16849,7 +16849,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16893,7 +16893,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16937,7 +16937,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16981,7 +16981,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17025,7 +17025,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17063,7 +17063,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17101,7 +17101,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17139,7 +17139,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17218,7 +17218,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17297,7 +17297,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17364,7 +17364,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17402,7 +17402,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17440,7 +17440,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17478,7 +17478,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17516,7 +17516,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17554,7 +17554,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17592,7 +17592,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17630,7 +17630,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17674,7 +17674,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17718,7 +17718,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17756,7 +17756,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17791,7 +17791,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17829,7 +17829,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17867,7 +17867,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17905,7 +17905,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17943,7 +17943,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18025,7 +18025,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18063,7 +18063,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18139,7 +18139,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18177,7 +18177,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18215,7 +18215,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18253,7 +18253,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18291,7 +18291,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18329,7 +18329,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18367,7 +18367,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18405,7 +18405,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18443,7 +18443,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18481,7 +18481,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18519,7 +18519,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18557,7 +18557,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18601,7 +18601,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18648,7 +18648,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18686,7 +18686,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18724,7 +18724,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18762,7 +18762,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18838,7 +18838,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18876,7 +18876,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18920,7 +18920,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18958,7 +18958,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -18996,7 +18996,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19034,7 +19034,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19072,7 +19072,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19110,7 +19110,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19148,7 +19148,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19186,7 +19186,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19224,7 +19224,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19262,7 +19262,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19300,7 +19300,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19420,7 +19420,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19458,7 +19458,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19496,7 +19496,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19537,7 +19537,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19575,7 +19575,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19613,7 +19613,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19692,7 +19692,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19730,7 +19730,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19768,7 +19768,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19806,7 +19806,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19841,7 +19841,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19905,7 +19905,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19937,7 +19937,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19969,7 +19969,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20001,7 +20001,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20033,7 +20033,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20065,7 +20065,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20097,7 +20097,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20129,7 +20129,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20161,7 +20161,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20193,7 +20193,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20225,7 +20225,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20257,7 +20257,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20289,7 +20289,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20321,7 +20321,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20353,7 +20353,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20385,7 +20385,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20417,7 +20417,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20449,7 +20449,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20481,7 +20481,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20513,7 +20513,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20545,7 +20545,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20577,7 +20577,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20609,7 +20609,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20641,7 +20641,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20673,7 +20673,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20705,7 +20705,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20737,7 +20737,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20769,7 +20769,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20801,7 +20801,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20833,7 +20833,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20865,7 +20865,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20897,7 +20897,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20929,7 +20929,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20961,7 +20961,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20993,7 +20993,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21025,7 +21025,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21441,7 +21441,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21473,7 +21473,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21505,7 +21505,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21537,7 +21537,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21569,7 +21569,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21601,7 +21601,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21633,7 +21633,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21665,7 +21665,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21697,7 +21697,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21729,7 +21729,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21761,7 +21761,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21793,7 +21793,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21825,7 +21825,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21857,7 +21857,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21889,7 +21889,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21921,7 +21921,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21953,7 +21953,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -21985,7 +21985,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22017,7 +22017,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22049,7 +22049,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22081,7 +22081,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22113,7 +22113,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22145,7 +22145,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22177,7 +22177,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22209,7 +22209,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22241,7 +22241,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22273,7 +22273,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22305,7 +22305,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22337,7 +22337,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22369,7 +22369,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22401,7 +22401,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22433,7 +22433,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22465,7 +22465,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22497,7 +22497,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22529,7 +22529,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22561,7 +22561,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22593,7 +22593,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22625,7 +22625,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22657,7 +22657,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22689,7 +22689,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22721,7 +22721,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22753,7 +22753,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22785,7 +22785,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22817,7 +22817,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22849,7 +22849,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22881,7 +22881,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22913,7 +22913,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22945,7 +22945,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -22977,7 +22977,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23009,7 +23009,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23041,7 +23041,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23073,7 +23073,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23105,7 +23105,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23137,7 +23137,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23169,7 +23169,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23201,7 +23201,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23233,7 +23233,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (07/08/2026 13:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4123" uniqueCount="1372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4124" uniqueCount="1373">
   <si>
     <t>os</t>
   </si>
@@ -4115,6 +4115,9 @@
   </si>
   <si>
     <t>007/2026</t>
+  </si>
+  <si>
+    <t>027/2026</t>
   </si>
   <si>
     <t>015/2026</t>
@@ -13494,6 +13497,9 @@
       <c r="M237" t="s">
         <v>1339</v>
       </c>
+      <c r="P237" t="s">
+        <v>1367</v>
+      </c>
       <c r="Q237" t="b">
         <v>1</v>
       </c>
@@ -14403,7 +14409,7 @@
         <v>46113</v>
       </c>
       <c r="P262" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="Q262" t="b">
         <v>1</v>
@@ -15052,7 +15058,7 @@
         <v>1339</v>
       </c>
       <c r="P279" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="Q279" t="b">
         <v>1</v>
@@ -18107,7 +18113,7 @@
         <v>1337</v>
       </c>
       <c r="P359" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="Q359" t="b">
         <v>0</v>
@@ -18616,7 +18622,7 @@
         <v>46113</v>
       </c>
       <c r="P372" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="Q372" t="b">
         <v>1</v>
@@ -18806,7 +18812,7 @@
         <v>1341</v>
       </c>
       <c r="P377" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="Q377" t="b">
         <v>0</v>
@@ -19350,7 +19356,7 @@
         <v>1337</v>
       </c>
       <c r="P391" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="Q391" t="b">
         <v>0</v>
@@ -19505,7 +19511,7 @@
         <v>1337</v>
       </c>
       <c r="P395" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="Q395" t="b">
         <v>1</v>
@@ -19622,7 +19628,7 @@
         <v>1337</v>
       </c>
       <c r="P398" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="Q398" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (10/08/2026 08:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4550,7 +4550,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4588,7 +4588,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4626,7 +4626,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4664,7 +4664,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4708,7 +4708,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4752,7 +4752,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4828,7 +4828,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4875,7 +4875,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4922,7 +4922,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4969,7 +4969,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5048,7 +5048,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5092,7 +5092,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5130,7 +5130,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5168,7 +5168,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5212,7 +5212,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5291,7 +5291,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5370,7 +5370,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5408,7 +5408,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5531,7 +5531,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5578,7 +5578,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5683,7 +5683,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5765,7 +5765,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -6007,7 +6007,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6042,7 +6042,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6191,7 +6191,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6238,7 +6238,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6285,7 +6285,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6323,7 +6323,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6370,7 +6370,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6440,7 +6440,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6516,7 +6516,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6554,7 +6554,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6592,7 +6592,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6700,7 +6700,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6904,7 +6904,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6951,7 +6951,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7182,7 +7182,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7220,7 +7220,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7290,7 +7290,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7366,7 +7366,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7404,7 +7404,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7512,7 +7512,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7547,7 +7547,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7623,7 +7623,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7696,7 +7696,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7743,7 +7743,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7781,7 +7781,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7819,7 +7819,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7936,7 +7936,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7977,7 +7977,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8044,7 +8044,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8082,7 +8082,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8120,7 +8120,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8158,7 +8158,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8205,7 +8205,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8246,7 +8246,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8313,7 +8313,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8441,7 +8441,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8479,7 +8479,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8517,7 +8517,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8561,7 +8561,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8605,7 +8605,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8643,7 +8643,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8859,7 +8859,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8897,7 +8897,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8935,7 +8935,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8973,7 +8973,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9011,7 +9011,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9049,7 +9049,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9087,7 +9087,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9134,7 +9134,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9201,7 +9201,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9239,7 +9239,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9344,7 +9344,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9382,7 +9382,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9420,7 +9420,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9502,7 +9502,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9578,7 +9578,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9709,7 +9709,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10038,7 +10038,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10076,7 +10076,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10111,7 +10111,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10196,7 +10196,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10240,7 +10240,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10313,7 +10313,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10348,7 +10348,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10386,7 +10386,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10424,7 +10424,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10468,7 +10468,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10506,7 +10506,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10544,7 +10544,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10591,7 +10591,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10635,7 +10635,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10679,7 +10679,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10819,7 +10819,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10860,7 +10860,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10942,7 +10942,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11088,7 +11088,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11135,7 +11135,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11173,7 +11173,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11220,7 +11220,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11287,7 +11287,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11392,7 +11392,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11427,7 +11427,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11462,7 +11462,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11500,7 +11500,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11538,7 +11538,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11585,7 +11585,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11632,7 +11632,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11676,7 +11676,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11714,7 +11714,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11758,7 +11758,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11796,7 +11796,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11866,7 +11866,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -12000,7 +12000,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12044,7 +12044,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12082,7 +12082,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12120,7 +12120,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12158,7 +12158,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12196,7 +12196,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12234,7 +12234,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12307,7 +12307,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12351,7 +12351,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12395,7 +12395,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12439,7 +12439,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12547,7 +12547,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12585,7 +12585,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12632,7 +12632,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12699,7 +12699,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12743,7 +12743,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12781,7 +12781,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12822,7 +12822,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12898,7 +12898,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12936,7 +12936,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12974,7 +12974,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13012,7 +13012,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13050,7 +13050,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13088,7 +13088,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13126,7 +13126,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13199,7 +13199,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13237,7 +13237,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13351,7 +13351,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13398,7 +13398,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13445,7 +13445,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13489,7 +13489,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13559,7 +13559,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13670,7 +13670,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13740,7 +13740,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13778,7 +13778,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13816,7 +13816,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13921,7 +13921,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13959,7 +13959,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14067,7 +14067,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14105,7 +14105,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14143,7 +14143,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14181,7 +14181,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14280,7 +14280,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14318,7 +14318,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14356,7 +14356,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14394,7 +14394,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14479,7 +14479,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14517,7 +14517,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14555,7 +14555,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14593,7 +14593,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14631,7 +14631,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14666,7 +14666,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14704,7 +14704,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14742,7 +14742,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14780,7 +14780,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14862,7 +14862,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14935,7 +14935,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14973,7 +14973,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -15011,7 +15011,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15049,7 +15049,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15090,7 +15090,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15128,7 +15128,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15166,7 +15166,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15373,7 +15373,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15440,7 +15440,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15481,7 +15481,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15519,7 +15519,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15557,7 +15557,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15595,7 +15595,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15630,7 +15630,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15665,7 +15665,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15735,7 +15735,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15773,7 +15773,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15811,7 +15811,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15849,7 +15849,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15887,7 +15887,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15925,7 +15925,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15963,7 +15963,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -16001,7 +16001,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16045,7 +16045,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16089,7 +16089,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16127,7 +16127,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16165,7 +16165,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16203,7 +16203,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16241,7 +16241,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16279,7 +16279,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16352,7 +16352,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16390,7 +16390,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16428,7 +16428,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16466,7 +16466,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16577,7 +16577,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16615,7 +16615,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16653,7 +16653,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16697,7 +16697,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16735,7 +16735,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16773,7 +16773,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16817,7 +16817,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16855,7 +16855,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16899,7 +16899,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16943,7 +16943,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -16987,7 +16987,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17031,7 +17031,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17069,7 +17069,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17107,7 +17107,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17145,7 +17145,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17224,7 +17224,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17303,7 +17303,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17370,7 +17370,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17408,7 +17408,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17446,7 +17446,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17484,7 +17484,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17522,7 +17522,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17560,7 +17560,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17598,7 +17598,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17636,7 +17636,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17680,7 +17680,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17724,7 +17724,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17762,7 +17762,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17797,7 +17797,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17835,7 +17835,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17873,7 +17873,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17911,7 +17911,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17949,7 +17949,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18031,7 +18031,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18069,7 +18069,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18145,7 +18145,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18183,7 +18183,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18221,7 +18221,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18259,7 +18259,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18297,7 +18297,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18335,7 +18335,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18373,7 +18373,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18411,7 +18411,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18449,7 +18449,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18487,7 +18487,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18525,7 +18525,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18563,7 +18563,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18607,7 +18607,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18654,7 +18654,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18692,7 +18692,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18730,7 +18730,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18768,7 +18768,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18844,7 +18844,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18882,7 +18882,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18926,7 +18926,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18964,7 +18964,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -19002,7 +19002,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19040,7 +19040,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19078,7 +19078,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19116,7 +19116,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19154,7 +19154,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19192,7 +19192,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19230,7 +19230,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19268,7 +19268,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19306,7 +19306,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19426,7 +19426,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19464,7 +19464,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19502,7 +19502,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19543,7 +19543,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19581,7 +19581,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19619,7 +19619,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19698,7 +19698,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19736,7 +19736,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19774,7 +19774,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19812,7 +19812,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19847,7 +19847,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19911,7 +19911,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19943,7 +19943,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -19975,7 +19975,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20007,7 +20007,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20039,7 +20039,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20071,7 +20071,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20103,7 +20103,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20135,7 +20135,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20167,7 +20167,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20199,7 +20199,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20231,7 +20231,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20263,7 +20263,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20295,7 +20295,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20327,7 +20327,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20359,7 +20359,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20391,7 +20391,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20423,7 +20423,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20455,7 +20455,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20487,7 +20487,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20519,7 +20519,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20551,7 +20551,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20583,7 +20583,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20615,7 +20615,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20647,7 +20647,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20679,7 +20679,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -20999,7 +20999,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21031,7 +21031,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21063,7 +21063,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21095,7 +21095,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21127,7 +21127,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21159,7 +21159,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21191,7 +21191,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21223,7 +21223,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21255,7 +21255,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21287,7 +21287,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21319,7 +21319,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21351,7 +21351,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21383,7 +21383,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21415,7 +21415,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21447,7 +21447,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21479,7 +21479,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21511,7 +21511,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21543,7 +21543,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21575,7 +21575,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21607,7 +21607,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21639,7 +21639,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21671,7 +21671,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21703,7 +21703,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21735,7 +21735,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21767,7 +21767,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21799,7 +21799,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21831,7 +21831,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21863,7 +21863,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21895,7 +21895,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21927,7 +21927,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21959,7 +21959,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -21991,7 +21991,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22023,7 +22023,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22055,7 +22055,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22087,7 +22087,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22119,7 +22119,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22151,7 +22151,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22183,7 +22183,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22215,7 +22215,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22247,7 +22247,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22279,7 +22279,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22311,7 +22311,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22343,7 +22343,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22375,7 +22375,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22407,7 +22407,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22439,7 +22439,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22471,7 +22471,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22503,7 +22503,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22535,7 +22535,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22567,7 +22567,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22599,7 +22599,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22631,7 +22631,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22663,7 +22663,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22695,7 +22695,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22727,7 +22727,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22759,7 +22759,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22791,7 +22791,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22823,7 +22823,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22855,7 +22855,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22887,7 +22887,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22919,7 +22919,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22951,7 +22951,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -22983,7 +22983,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23015,7 +23015,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23047,7 +23047,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23079,7 +23079,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23111,7 +23111,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23143,7 +23143,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23175,7 +23175,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23207,7 +23207,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23239,7 +23239,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (10/08/2026 11:25)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4124" uniqueCount="1373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4129" uniqueCount="1377">
   <si>
     <t>os</t>
   </si>
@@ -4120,19 +4120,31 @@
     <t>027/2026</t>
   </si>
   <si>
+    <t>019/2026</t>
+  </si>
+  <si>
     <t>015/2026</t>
   </si>
   <si>
     <t>006/2026</t>
   </si>
   <si>
+    <t>089/2026</t>
+  </si>
+  <si>
     <t>078/2026</t>
   </si>
   <si>
     <t>024/2026</t>
   </si>
   <si>
+    <t>018/2026</t>
+  </si>
+  <si>
     <t>088/2026</t>
+  </si>
+  <si>
+    <t>020/2026</t>
   </si>
 </sst>
 </file>
@@ -13967,6 +13979,9 @@
       <c r="M250" t="s">
         <v>1339</v>
       </c>
+      <c r="P250" t="s">
+        <v>1368</v>
+      </c>
       <c r="Q250" t="b">
         <v>1</v>
       </c>
@@ -14409,7 +14424,7 @@
         <v>46113</v>
       </c>
       <c r="P262" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="Q262" t="b">
         <v>1</v>
@@ -15058,7 +15073,7 @@
         <v>1339</v>
       </c>
       <c r="P279" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="Q279" t="b">
         <v>1</v>
@@ -18077,6 +18092,9 @@
       <c r="M358" t="s">
         <v>1337</v>
       </c>
+      <c r="P358" t="s">
+        <v>1371</v>
+      </c>
       <c r="Q358" t="b">
         <v>1</v>
       </c>
@@ -18113,7 +18131,7 @@
         <v>1337</v>
       </c>
       <c r="P359" t="s">
-        <v>1370</v>
+        <v>1372</v>
       </c>
       <c r="Q359" t="b">
         <v>0</v>
@@ -18622,7 +18640,7 @@
         <v>46113</v>
       </c>
       <c r="P372" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="Q372" t="b">
         <v>1</v>
@@ -18812,7 +18830,7 @@
         <v>1341</v>
       </c>
       <c r="P377" t="s">
-        <v>1371</v>
+        <v>1373</v>
       </c>
       <c r="Q377" t="b">
         <v>0</v>
@@ -19320,6 +19338,9 @@
       <c r="N390" s="1">
         <v>46191</v>
       </c>
+      <c r="P390" t="s">
+        <v>1374</v>
+      </c>
       <c r="Q390" t="b">
         <v>1</v>
       </c>
@@ -19356,7 +19377,7 @@
         <v>1337</v>
       </c>
       <c r="P391" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="Q391" t="b">
         <v>0</v>
@@ -19511,7 +19532,7 @@
         <v>1337</v>
       </c>
       <c r="P395" t="s">
-        <v>1372</v>
+        <v>1375</v>
       </c>
       <c r="Q395" t="b">
         <v>1</v>
@@ -19551,6 +19572,9 @@
       <c r="M396" t="s">
         <v>1337</v>
       </c>
+      <c r="P396" t="s">
+        <v>1374</v>
+      </c>
       <c r="Q396" t="b">
         <v>1</v>
       </c>
@@ -19628,7 +19652,7 @@
         <v>1337</v>
       </c>
       <c r="P398" t="s">
-        <v>1372</v>
+        <v>1375</v>
       </c>
       <c r="Q398" t="b">
         <v>1</v>
@@ -19743,6 +19767,9 @@
       </c>
       <c r="M401" t="s">
         <v>1337</v>
+      </c>
+      <c r="P401" t="s">
+        <v>1376</v>
       </c>
       <c r="Q401" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (11/08/2026 08:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4562,7 +4562,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4600,7 +4600,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4638,7 +4638,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4676,7 +4676,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4720,7 +4720,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4764,7 +4764,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4840,7 +4840,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4887,7 +4887,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4934,7 +4934,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4981,7 +4981,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5060,7 +5060,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5104,7 +5104,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5142,7 +5142,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5180,7 +5180,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5224,7 +5224,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5303,7 +5303,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5382,7 +5382,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5420,7 +5420,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5543,7 +5543,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5590,7 +5590,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5695,7 +5695,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5777,7 +5777,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -6019,7 +6019,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6054,7 +6054,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6203,7 +6203,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6250,7 +6250,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6297,7 +6297,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6335,7 +6335,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6382,7 +6382,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6452,7 +6452,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6528,7 +6528,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6566,7 +6566,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6604,7 +6604,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6712,7 +6712,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6916,7 +6916,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6963,7 +6963,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7194,7 +7194,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7232,7 +7232,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7302,7 +7302,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7378,7 +7378,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7416,7 +7416,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7524,7 +7524,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7559,7 +7559,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7635,7 +7635,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7708,7 +7708,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7755,7 +7755,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7793,7 +7793,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7831,7 +7831,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7948,7 +7948,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7989,7 +7989,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8056,7 +8056,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8094,7 +8094,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8132,7 +8132,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8170,7 +8170,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8217,7 +8217,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8258,7 +8258,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8325,7 +8325,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8453,7 +8453,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8491,7 +8491,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8529,7 +8529,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8573,7 +8573,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8617,7 +8617,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8655,7 +8655,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8871,7 +8871,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8909,7 +8909,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8947,7 +8947,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8985,7 +8985,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9023,7 +9023,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9061,7 +9061,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9099,7 +9099,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9146,7 +9146,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9213,7 +9213,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9251,7 +9251,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9356,7 +9356,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9394,7 +9394,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9432,7 +9432,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9514,7 +9514,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9590,7 +9590,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9721,7 +9721,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10050,7 +10050,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10088,7 +10088,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10123,7 +10123,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10208,7 +10208,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10252,7 +10252,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10325,7 +10325,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10360,7 +10360,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10398,7 +10398,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10436,7 +10436,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10480,7 +10480,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10518,7 +10518,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10556,7 +10556,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10603,7 +10603,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10647,7 +10647,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10691,7 +10691,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10831,7 +10831,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10872,7 +10872,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10954,7 +10954,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11100,7 +11100,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11147,7 +11147,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11185,7 +11185,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11232,7 +11232,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11299,7 +11299,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11404,7 +11404,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11439,7 +11439,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11474,7 +11474,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11512,7 +11512,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11550,7 +11550,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11597,7 +11597,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11644,7 +11644,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11688,7 +11688,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11726,7 +11726,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11770,7 +11770,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11808,7 +11808,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11878,7 +11878,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -12012,7 +12012,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12056,7 +12056,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12094,7 +12094,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12132,7 +12132,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12170,7 +12170,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12208,7 +12208,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12246,7 +12246,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12319,7 +12319,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12363,7 +12363,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12407,7 +12407,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12451,7 +12451,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12559,7 +12559,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12597,7 +12597,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12644,7 +12644,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12711,7 +12711,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12755,7 +12755,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12793,7 +12793,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12834,7 +12834,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12910,7 +12910,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12948,7 +12948,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12986,7 +12986,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13024,7 +13024,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13062,7 +13062,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13100,7 +13100,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13138,7 +13138,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13211,7 +13211,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13249,7 +13249,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13363,7 +13363,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13410,7 +13410,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13457,7 +13457,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13501,7 +13501,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13571,7 +13571,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13682,7 +13682,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13752,7 +13752,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13790,7 +13790,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13828,7 +13828,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13933,7 +13933,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13971,7 +13971,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14082,7 +14082,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14120,7 +14120,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14158,7 +14158,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14196,7 +14196,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14295,7 +14295,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14333,7 +14333,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14371,7 +14371,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14409,7 +14409,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14494,7 +14494,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14532,7 +14532,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14570,7 +14570,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14608,7 +14608,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14646,7 +14646,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14681,7 +14681,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14719,7 +14719,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14757,7 +14757,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14795,7 +14795,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14877,7 +14877,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14950,7 +14950,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14988,7 +14988,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -15026,7 +15026,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15064,7 +15064,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15105,7 +15105,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15143,7 +15143,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15181,7 +15181,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15388,7 +15388,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15455,7 +15455,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15496,7 +15496,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15534,7 +15534,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15572,7 +15572,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15610,7 +15610,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15645,7 +15645,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15680,7 +15680,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15750,7 +15750,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15788,7 +15788,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15826,7 +15826,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15864,7 +15864,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15902,7 +15902,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15940,7 +15940,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15978,7 +15978,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -16016,7 +16016,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16060,7 +16060,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16104,7 +16104,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16142,7 +16142,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16180,7 +16180,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16218,7 +16218,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16256,7 +16256,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16294,7 +16294,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16367,7 +16367,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16405,7 +16405,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16443,7 +16443,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16481,7 +16481,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16592,7 +16592,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16630,7 +16630,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16668,7 +16668,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16712,7 +16712,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16750,7 +16750,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16788,7 +16788,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16832,7 +16832,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16870,7 +16870,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16914,7 +16914,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16958,7 +16958,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17002,7 +17002,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17046,7 +17046,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17084,7 +17084,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17122,7 +17122,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17160,7 +17160,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17239,7 +17239,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17318,7 +17318,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17385,7 +17385,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17423,7 +17423,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17461,7 +17461,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17499,7 +17499,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17537,7 +17537,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17575,7 +17575,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17613,7 +17613,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17651,7 +17651,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17695,7 +17695,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17739,7 +17739,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17777,7 +17777,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17812,7 +17812,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17850,7 +17850,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17888,7 +17888,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17926,7 +17926,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17964,7 +17964,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18046,7 +18046,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18084,7 +18084,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18163,7 +18163,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18201,7 +18201,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18239,7 +18239,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18277,7 +18277,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18315,7 +18315,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18353,7 +18353,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18391,7 +18391,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18429,7 +18429,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18467,7 +18467,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18505,7 +18505,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18543,7 +18543,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18581,7 +18581,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18625,7 +18625,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18672,7 +18672,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18710,7 +18710,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18748,7 +18748,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18786,7 +18786,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18862,7 +18862,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18900,7 +18900,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18944,7 +18944,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18982,7 +18982,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -19020,7 +19020,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19058,7 +19058,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19096,7 +19096,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19134,7 +19134,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19172,7 +19172,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19210,7 +19210,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19248,7 +19248,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19286,7 +19286,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19324,7 +19324,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19447,7 +19447,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19485,7 +19485,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19523,7 +19523,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19564,7 +19564,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19605,7 +19605,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19643,7 +19643,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19722,7 +19722,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19760,7 +19760,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19801,7 +19801,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19839,7 +19839,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19874,7 +19874,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19938,7 +19938,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19970,7 +19970,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20002,7 +20002,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20034,7 +20034,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20066,7 +20066,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20098,7 +20098,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20130,7 +20130,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20162,7 +20162,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20194,7 +20194,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20226,7 +20226,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20258,7 +20258,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20290,7 +20290,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20322,7 +20322,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20354,7 +20354,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20386,7 +20386,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20418,7 +20418,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20450,7 +20450,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20482,7 +20482,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20514,7 +20514,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20546,7 +20546,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20578,7 +20578,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20610,7 +20610,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20642,7 +20642,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20674,7 +20674,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20706,7 +20706,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20738,7 +20738,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20770,7 +20770,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20802,7 +20802,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20834,7 +20834,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20866,7 +20866,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20898,7 +20898,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20930,7 +20930,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20962,7 +20962,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20994,7 +20994,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21026,7 +21026,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21058,7 +21058,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21090,7 +21090,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21122,7 +21122,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21154,7 +21154,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21186,7 +21186,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21218,7 +21218,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21250,7 +21250,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21282,7 +21282,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21314,7 +21314,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21346,7 +21346,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21378,7 +21378,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21410,7 +21410,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21442,7 +21442,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21474,7 +21474,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21506,7 +21506,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21538,7 +21538,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21570,7 +21570,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21602,7 +21602,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21634,7 +21634,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21666,7 +21666,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21698,7 +21698,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21730,7 +21730,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21762,7 +21762,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21794,7 +21794,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21826,7 +21826,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21858,7 +21858,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21890,7 +21890,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21922,7 +21922,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21954,7 +21954,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21986,7 +21986,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -22018,7 +22018,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22050,7 +22050,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22082,7 +22082,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22114,7 +22114,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22146,7 +22146,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22178,7 +22178,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22210,7 +22210,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22242,7 +22242,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22274,7 +22274,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22306,7 +22306,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22338,7 +22338,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22370,7 +22370,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22402,7 +22402,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22434,7 +22434,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22466,7 +22466,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22498,7 +22498,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22530,7 +22530,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22562,7 +22562,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22594,7 +22594,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22626,7 +22626,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22658,7 +22658,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22690,7 +22690,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22722,7 +22722,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22754,7 +22754,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22786,7 +22786,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22818,7 +22818,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22850,7 +22850,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22882,7 +22882,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22914,7 +22914,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22946,7 +22946,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22978,7 +22978,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23010,7 +23010,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23042,7 +23042,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23074,7 +23074,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23106,7 +23106,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23138,7 +23138,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23170,7 +23170,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23202,7 +23202,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23234,7 +23234,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23266,7 +23266,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (12/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4562,7 +4562,7 @@
         <v>1236</v>
       </c>
       <c r="I2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="K2" t="s">
         <v>1239</v>
@@ -4600,7 +4600,7 @@
         <v>1236</v>
       </c>
       <c r="I3">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K3" t="s">
         <v>1240</v>
@@ -4638,7 +4638,7 @@
         <v>1236</v>
       </c>
       <c r="I4">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K4" t="s">
         <v>1240</v>
@@ -4676,7 +4676,7 @@
         <v>1236</v>
       </c>
       <c r="I5">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -4720,7 +4720,7 @@
         <v>1236</v>
       </c>
       <c r="I6">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -4764,7 +4764,7 @@
         <v>1236</v>
       </c>
       <c r="I7">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -4840,7 +4840,7 @@
         <v>1236</v>
       </c>
       <c r="I9">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -4887,7 +4887,7 @@
         <v>1236</v>
       </c>
       <c r="I10">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -4934,7 +4934,7 @@
         <v>1236</v>
       </c>
       <c r="I11">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -4981,7 +4981,7 @@
         <v>1236</v>
       </c>
       <c r="I12">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5060,7 +5060,7 @@
         <v>1236</v>
       </c>
       <c r="I14">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5104,7 +5104,7 @@
         <v>1236</v>
       </c>
       <c r="I15">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K15" t="s">
         <v>1242</v>
@@ -5142,7 +5142,7 @@
         <v>1236</v>
       </c>
       <c r="I16">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K16" t="s">
         <v>1239</v>
@@ -5180,7 +5180,7 @@
         <v>1236</v>
       </c>
       <c r="I17">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5224,7 +5224,7 @@
         <v>1236</v>
       </c>
       <c r="I18">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5303,7 +5303,7 @@
         <v>1236</v>
       </c>
       <c r="I20">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5382,7 +5382,7 @@
         <v>1236</v>
       </c>
       <c r="I22">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K22" t="s">
         <v>1243</v>
@@ -5420,7 +5420,7 @@
         <v>1236</v>
       </c>
       <c r="I23">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5543,7 +5543,7 @@
         <v>1236</v>
       </c>
       <c r="I26">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5590,7 +5590,7 @@
         <v>1236</v>
       </c>
       <c r="I27">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K27" t="s">
         <v>1243</v>
@@ -5695,7 +5695,7 @@
         <v>1236</v>
       </c>
       <c r="I30">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -5777,7 +5777,7 @@
         <v>1236</v>
       </c>
       <c r="I32">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K32" t="s">
         <v>1239</v>
@@ -6019,7 +6019,7 @@
         <v>1236</v>
       </c>
       <c r="I39">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K39" t="s">
         <v>1244</v>
@@ -6054,7 +6054,7 @@
         <v>1236</v>
       </c>
       <c r="I40">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K40" t="s">
         <v>1242</v>
@@ -6203,7 +6203,7 @@
         <v>1236</v>
       </c>
       <c r="I44">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6250,7 +6250,7 @@
         <v>1236</v>
       </c>
       <c r="I45">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6297,7 +6297,7 @@
         <v>1236</v>
       </c>
       <c r="I46">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K46" t="s">
         <v>1243</v>
@@ -6335,7 +6335,7 @@
         <v>1236</v>
       </c>
       <c r="I47">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6382,7 +6382,7 @@
         <v>1236</v>
       </c>
       <c r="I48">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K48" t="s">
         <v>1243</v>
@@ -6452,7 +6452,7 @@
         <v>1236</v>
       </c>
       <c r="I50">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K50" t="s">
         <v>1243</v>
@@ -6528,7 +6528,7 @@
         <v>1236</v>
       </c>
       <c r="I52">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K52" t="s">
         <v>1239</v>
@@ -6566,7 +6566,7 @@
         <v>1236</v>
       </c>
       <c r="I53">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K53" t="s">
         <v>1240</v>
@@ -6604,7 +6604,7 @@
         <v>1236</v>
       </c>
       <c r="I54">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K54" t="s">
         <v>1240</v>
@@ -6712,7 +6712,7 @@
         <v>1236</v>
       </c>
       <c r="I57">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K57" t="s">
         <v>1243</v>
@@ -6916,7 +6916,7 @@
         <v>1236</v>
       </c>
       <c r="I63">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -6963,7 +6963,7 @@
         <v>1236</v>
       </c>
       <c r="I64">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7194,7 +7194,7 @@
         <v>1236</v>
       </c>
       <c r="I70">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K70" t="s">
         <v>1240</v>
@@ -7232,7 +7232,7 @@
         <v>1236</v>
       </c>
       <c r="I71">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K71" t="s">
         <v>1246</v>
@@ -7302,7 +7302,7 @@
         <v>1236</v>
       </c>
       <c r="I73">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K73" t="s">
         <v>1239</v>
@@ -7378,7 +7378,7 @@
         <v>1236</v>
       </c>
       <c r="I75">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K75" t="s">
         <v>1240</v>
@@ -7416,7 +7416,7 @@
         <v>1236</v>
       </c>
       <c r="I76">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K76" t="s">
         <v>1246</v>
@@ -7524,7 +7524,7 @@
         <v>1236</v>
       </c>
       <c r="I79">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K79" t="s">
         <v>1246</v>
@@ -7559,7 +7559,7 @@
         <v>1236</v>
       </c>
       <c r="I80">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K80" t="s">
         <v>1240</v>
@@ -7635,7 +7635,7 @@
         <v>1236</v>
       </c>
       <c r="I82">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K82" t="s">
         <v>1243</v>
@@ -7708,7 +7708,7 @@
         <v>1236</v>
       </c>
       <c r="I84">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7755,7 +7755,7 @@
         <v>1236</v>
       </c>
       <c r="I85">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K85" t="s">
         <v>1240</v>
@@ -7793,7 +7793,7 @@
         <v>1236</v>
       </c>
       <c r="I86">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K86" t="s">
         <v>1240</v>
@@ -7831,7 +7831,7 @@
         <v>1236</v>
       </c>
       <c r="I87">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -7948,7 +7948,7 @@
         <v>1236</v>
       </c>
       <c r="I90">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K90" t="s">
         <v>1213</v>
@@ -7989,7 +7989,7 @@
         <v>1236</v>
       </c>
       <c r="I91">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K91" t="s">
         <v>1242</v>
@@ -8056,7 +8056,7 @@
         <v>1236</v>
       </c>
       <c r="I93">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K93" t="s">
         <v>1242</v>
@@ -8094,7 +8094,7 @@
         <v>1236</v>
       </c>
       <c r="I94">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K94" t="s">
         <v>1243</v>
@@ -8132,7 +8132,7 @@
         <v>1236</v>
       </c>
       <c r="I95">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K95" t="s">
         <v>1242</v>
@@ -8170,7 +8170,7 @@
         <v>1236</v>
       </c>
       <c r="I96">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8217,7 +8217,7 @@
         <v>1236</v>
       </c>
       <c r="I97">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K97" t="s">
         <v>1213</v>
@@ -8258,7 +8258,7 @@
         <v>1236</v>
       </c>
       <c r="I98">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K98" t="s">
         <v>1243</v>
@@ -8325,7 +8325,7 @@
         <v>1236</v>
       </c>
       <c r="I100">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K100" t="s">
         <v>1242</v>
@@ -8453,7 +8453,7 @@
         <v>1236</v>
       </c>
       <c r="I104">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K104" t="s">
         <v>1242</v>
@@ -8491,7 +8491,7 @@
         <v>1236</v>
       </c>
       <c r="I105">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K105" t="s">
         <v>1242</v>
@@ -8529,7 +8529,7 @@
         <v>1236</v>
       </c>
       <c r="I106">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8573,7 +8573,7 @@
         <v>1236</v>
       </c>
       <c r="I107">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8617,7 +8617,7 @@
         <v>1236</v>
       </c>
       <c r="I108">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K108" t="s">
         <v>1240</v>
@@ -8655,7 +8655,7 @@
         <v>1236</v>
       </c>
       <c r="I109">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K109" t="s">
         <v>1240</v>
@@ -8871,7 +8871,7 @@
         <v>1236</v>
       </c>
       <c r="I115">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K115" t="s">
         <v>1240</v>
@@ -8909,7 +8909,7 @@
         <v>1236</v>
       </c>
       <c r="I116">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K116" t="s">
         <v>1240</v>
@@ -8947,7 +8947,7 @@
         <v>1236</v>
       </c>
       <c r="I117">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K117" t="s">
         <v>1240</v>
@@ -8985,7 +8985,7 @@
         <v>1236</v>
       </c>
       <c r="I118">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K118" t="s">
         <v>1240</v>
@@ -9023,7 +9023,7 @@
         <v>1236</v>
       </c>
       <c r="I119">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K119" t="s">
         <v>1240</v>
@@ -9061,7 +9061,7 @@
         <v>1236</v>
       </c>
       <c r="I120">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K120" t="s">
         <v>1240</v>
@@ -9099,7 +9099,7 @@
         <v>1236</v>
       </c>
       <c r="I121">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9146,7 +9146,7 @@
         <v>1236</v>
       </c>
       <c r="I122">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="K122" t="s">
         <v>1240</v>
@@ -9213,7 +9213,7 @@
         <v>1236</v>
       </c>
       <c r="I124">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K124" t="s">
         <v>1240</v>
@@ -9251,7 +9251,7 @@
         <v>1236</v>
       </c>
       <c r="I125">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K125" t="s">
         <v>1246</v>
@@ -9356,7 +9356,7 @@
         <v>1236</v>
       </c>
       <c r="I128">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K128" t="s">
         <v>1240</v>
@@ -9394,7 +9394,7 @@
         <v>1236</v>
       </c>
       <c r="I129">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K129" t="s">
         <v>1239</v>
@@ -9432,7 +9432,7 @@
         <v>1236</v>
       </c>
       <c r="I130">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9514,7 +9514,7 @@
         <v>1236</v>
       </c>
       <c r="I132">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9590,7 +9590,7 @@
         <v>1236</v>
       </c>
       <c r="I134">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K134" t="s">
         <v>1239</v>
@@ -9721,7 +9721,7 @@
         <v>1236</v>
       </c>
       <c r="I138">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K138" t="s">
         <v>1240</v>
@@ -10050,7 +10050,7 @@
         <v>1236</v>
       </c>
       <c r="I148">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K148" t="s">
         <v>1240</v>
@@ -10088,7 +10088,7 @@
         <v>1236</v>
       </c>
       <c r="I149">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K149" t="s">
         <v>1246</v>
@@ -10123,7 +10123,7 @@
         <v>1236</v>
       </c>
       <c r="I150">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10208,7 +10208,7 @@
         <v>1236</v>
       </c>
       <c r="I152">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10252,7 +10252,7 @@
         <v>1236</v>
       </c>
       <c r="I153">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K153" t="s">
         <v>1240</v>
@@ -10325,7 +10325,7 @@
         <v>1236</v>
       </c>
       <c r="I155">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K155" t="s">
         <v>1246</v>
@@ -10360,7 +10360,7 @@
         <v>1236</v>
       </c>
       <c r="I156">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K156" t="s">
         <v>1240</v>
@@ -10398,7 +10398,7 @@
         <v>1236</v>
       </c>
       <c r="I157">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K157" t="s">
         <v>1242</v>
@@ -10436,7 +10436,7 @@
         <v>1236</v>
       </c>
       <c r="I158">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10480,7 +10480,7 @@
         <v>1236</v>
       </c>
       <c r="I159">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K159" t="s">
         <v>1240</v>
@@ -10518,7 +10518,7 @@
         <v>1236</v>
       </c>
       <c r="I160">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K160" t="s">
         <v>1240</v>
@@ -10556,7 +10556,7 @@
         <v>1236</v>
       </c>
       <c r="I161">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10603,7 +10603,7 @@
         <v>1236</v>
       </c>
       <c r="I162">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10647,7 +10647,7 @@
         <v>1236</v>
       </c>
       <c r="I163">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10691,7 +10691,7 @@
         <v>1238</v>
       </c>
       <c r="I164">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K164" t="s">
         <v>1247</v>
@@ -10831,7 +10831,7 @@
         <v>1236</v>
       </c>
       <c r="I168">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K168" t="s">
         <v>1243</v>
@@ -10872,7 +10872,7 @@
         <v>1236</v>
       </c>
       <c r="I169">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J169">
         <v>-40</v>
@@ -10954,7 +10954,7 @@
         <v>1236</v>
       </c>
       <c r="I171">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K171" t="s">
         <v>1240</v>
@@ -11100,7 +11100,7 @@
         <v>1236</v>
       </c>
       <c r="I175">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11147,7 +11147,7 @@
         <v>1236</v>
       </c>
       <c r="I176">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K176" t="s">
         <v>1240</v>
@@ -11185,7 +11185,7 @@
         <v>1236</v>
       </c>
       <c r="I177">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11232,7 +11232,7 @@
         <v>1236</v>
       </c>
       <c r="I178">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K178" t="s">
         <v>1239</v>
@@ -11299,7 +11299,7 @@
         <v>1236</v>
       </c>
       <c r="I180">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K180" t="s">
         <v>1239</v>
@@ -11404,7 +11404,7 @@
         <v>1236</v>
       </c>
       <c r="I183">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K183" t="s">
         <v>1240</v>
@@ -11439,7 +11439,7 @@
         <v>1236</v>
       </c>
       <c r="I184">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K184" t="s">
         <v>1246</v>
@@ -11474,7 +11474,7 @@
         <v>1236</v>
       </c>
       <c r="I185">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K185" t="s">
         <v>1240</v>
@@ -11512,7 +11512,7 @@
         <v>1236</v>
       </c>
       <c r="I186">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K186" t="s">
         <v>1240</v>
@@ -11550,7 +11550,7 @@
         <v>1236</v>
       </c>
       <c r="I187">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11597,7 +11597,7 @@
         <v>1236</v>
       </c>
       <c r="I188">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11644,7 +11644,7 @@
         <v>1236</v>
       </c>
       <c r="I189">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11688,7 +11688,7 @@
         <v>1236</v>
       </c>
       <c r="I190">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K190" t="s">
         <v>1242</v>
@@ -11726,7 +11726,7 @@
         <v>1236</v>
       </c>
       <c r="I191">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11770,7 +11770,7 @@
         <v>1236</v>
       </c>
       <c r="I192">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K192" t="s">
         <v>1240</v>
@@ -11808,7 +11808,7 @@
         <v>1236</v>
       </c>
       <c r="I193">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K193" t="s">
         <v>1245</v>
@@ -11878,7 +11878,7 @@
         <v>1236</v>
       </c>
       <c r="I195">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K195" t="s">
         <v>1242</v>
@@ -12012,7 +12012,7 @@
         <v>1236</v>
       </c>
       <c r="I199">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12056,7 +12056,7 @@
         <v>1236</v>
       </c>
       <c r="I200">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K200" t="s">
         <v>1242</v>
@@ -12094,7 +12094,7 @@
         <v>1236</v>
       </c>
       <c r="I201">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K201" t="s">
         <v>1240</v>
@@ -12132,7 +12132,7 @@
         <v>1236</v>
       </c>
       <c r="I202">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K202" t="s">
         <v>1240</v>
@@ -12170,7 +12170,7 @@
         <v>1236</v>
       </c>
       <c r="I203">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K203" t="s">
         <v>1240</v>
@@ -12208,7 +12208,7 @@
         <v>1236</v>
       </c>
       <c r="I204">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K204" t="s">
         <v>1239</v>
@@ -12246,7 +12246,7 @@
         <v>1236</v>
       </c>
       <c r="I205">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K205" t="s">
         <v>1239</v>
@@ -12319,7 +12319,7 @@
         <v>1236</v>
       </c>
       <c r="I207">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12363,7 +12363,7 @@
         <v>1236</v>
       </c>
       <c r="I208">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12407,7 +12407,7 @@
         <v>1236</v>
       </c>
       <c r="I209">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12451,7 +12451,7 @@
         <v>1236</v>
       </c>
       <c r="I210">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K210" t="s">
         <v>1243</v>
@@ -12559,7 +12559,7 @@
         <v>1236</v>
       </c>
       <c r="I213">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K213" t="s">
         <v>1240</v>
@@ -12597,7 +12597,7 @@
         <v>1236</v>
       </c>
       <c r="I214">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12644,7 +12644,7 @@
         <v>1236</v>
       </c>
       <c r="I215">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K215" t="s">
         <v>1240</v>
@@ -12711,7 +12711,7 @@
         <v>1236</v>
       </c>
       <c r="I217">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12755,7 +12755,7 @@
         <v>1236</v>
       </c>
       <c r="I218">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K218" t="s">
         <v>1242</v>
@@ -12793,7 +12793,7 @@
         <v>1236</v>
       </c>
       <c r="I219">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K219" t="s">
         <v>1242</v>
@@ -12834,7 +12834,7 @@
         <v>1236</v>
       </c>
       <c r="I220">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K220" t="s">
         <v>1242</v>
@@ -12910,7 +12910,7 @@
         <v>1236</v>
       </c>
       <c r="I222">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K222" t="s">
         <v>1240</v>
@@ -12948,7 +12948,7 @@
         <v>1236</v>
       </c>
       <c r="I223">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K223" t="s">
         <v>1240</v>
@@ -12986,7 +12986,7 @@
         <v>1236</v>
       </c>
       <c r="I224">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K224" t="s">
         <v>1240</v>
@@ -13024,7 +13024,7 @@
         <v>1236</v>
       </c>
       <c r="I225">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K225" t="s">
         <v>1240</v>
@@ -13062,7 +13062,7 @@
         <v>1236</v>
       </c>
       <c r="I226">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K226" t="s">
         <v>1240</v>
@@ -13100,7 +13100,7 @@
         <v>1236</v>
       </c>
       <c r="I227">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K227" t="s">
         <v>1240</v>
@@ -13138,7 +13138,7 @@
         <v>1236</v>
       </c>
       <c r="I228">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K228" t="s">
         <v>1240</v>
@@ -13211,7 +13211,7 @@
         <v>1236</v>
       </c>
       <c r="I230">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K230" t="s">
         <v>1243</v>
@@ -13249,7 +13249,7 @@
         <v>1236</v>
       </c>
       <c r="I231">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13363,7 +13363,7 @@
         <v>1236</v>
       </c>
       <c r="I234">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13410,7 +13410,7 @@
         <v>1236</v>
       </c>
       <c r="I235">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13457,7 +13457,7 @@
         <v>1236</v>
       </c>
       <c r="I236">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13501,7 +13501,7 @@
         <v>1236</v>
       </c>
       <c r="I237">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K237" t="s">
         <v>1240</v>
@@ -13571,7 +13571,7 @@
         <v>1236</v>
       </c>
       <c r="I239">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K239" t="s">
         <v>1213</v>
@@ -13682,7 +13682,7 @@
         <v>1236</v>
       </c>
       <c r="I242">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K242" t="s">
         <v>1239</v>
@@ -13752,7 +13752,7 @@
         <v>1236</v>
       </c>
       <c r="I244">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K244" t="s">
         <v>1242</v>
@@ -13790,7 +13790,7 @@
         <v>1236</v>
       </c>
       <c r="I245">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K245" t="s">
         <v>1242</v>
@@ -13828,7 +13828,7 @@
         <v>1236</v>
       </c>
       <c r="I246">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J246">
         <v>141</v>
@@ -13933,7 +13933,7 @@
         <v>1236</v>
       </c>
       <c r="I249">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K249" t="s">
         <v>1240</v>
@@ -13971,7 +13971,7 @@
         <v>1236</v>
       </c>
       <c r="I250">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K250" t="s">
         <v>1242</v>
@@ -14082,7 +14082,7 @@
         <v>1236</v>
       </c>
       <c r="I253">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K253" t="s">
         <v>1243</v>
@@ -14120,7 +14120,7 @@
         <v>1236</v>
       </c>
       <c r="I254">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K254" t="s">
         <v>1243</v>
@@ -14158,7 +14158,7 @@
         <v>1236</v>
       </c>
       <c r="I255">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K255" t="s">
         <v>1242</v>
@@ -14196,7 +14196,7 @@
         <v>1236</v>
       </c>
       <c r="I256">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K256" t="s">
         <v>1240</v>
@@ -14295,7 +14295,7 @@
         <v>1236</v>
       </c>
       <c r="I259">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K259" t="s">
         <v>1242</v>
@@ -14333,7 +14333,7 @@
         <v>1236</v>
       </c>
       <c r="I260">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K260" t="s">
         <v>1242</v>
@@ -14371,7 +14371,7 @@
         <v>1236</v>
       </c>
       <c r="I261">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K261" t="s">
         <v>1243</v>
@@ -14409,7 +14409,7 @@
         <v>1236</v>
       </c>
       <c r="I262">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J262">
         <v>50</v>
@@ -14494,7 +14494,7 @@
         <v>1236</v>
       </c>
       <c r="I264">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K264" t="s">
         <v>1243</v>
@@ -14532,7 +14532,7 @@
         <v>1236</v>
       </c>
       <c r="I265">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K265" t="s">
         <v>1243</v>
@@ -14570,7 +14570,7 @@
         <v>1236</v>
       </c>
       <c r="I266">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K266" t="s">
         <v>1242</v>
@@ -14608,7 +14608,7 @@
         <v>1236</v>
       </c>
       <c r="I267">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K267" t="s">
         <v>1243</v>
@@ -14646,7 +14646,7 @@
         <v>1236</v>
       </c>
       <c r="I268">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K268" t="s">
         <v>1240</v>
@@ -14681,7 +14681,7 @@
         <v>1236</v>
       </c>
       <c r="I269">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K269" t="s">
         <v>1240</v>
@@ -14719,7 +14719,7 @@
         <v>1236</v>
       </c>
       <c r="I270">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K270" t="s">
         <v>1243</v>
@@ -14757,7 +14757,7 @@
         <v>1236</v>
       </c>
       <c r="I271">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K271" t="s">
         <v>1243</v>
@@ -14795,7 +14795,7 @@
         <v>1236</v>
       </c>
       <c r="I272">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J272">
         <v>122</v>
@@ -14877,7 +14877,7 @@
         <v>1236</v>
       </c>
       <c r="I274">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K274" t="s">
         <v>1240</v>
@@ -14950,7 +14950,7 @@
         <v>1236</v>
       </c>
       <c r="I276">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K276" t="s">
         <v>1244</v>
@@ -14988,7 +14988,7 @@
         <v>1236</v>
       </c>
       <c r="I277">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K277" t="s">
         <v>1240</v>
@@ -15026,7 +15026,7 @@
         <v>1236</v>
       </c>
       <c r="I278">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K278" t="s">
         <v>1243</v>
@@ -15064,7 +15064,7 @@
         <v>1236</v>
       </c>
       <c r="I279">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K279" t="s">
         <v>1242</v>
@@ -15105,7 +15105,7 @@
         <v>1236</v>
       </c>
       <c r="I280">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K280" t="s">
         <v>1240</v>
@@ -15143,7 +15143,7 @@
         <v>1236</v>
       </c>
       <c r="I281">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K281" t="s">
         <v>1240</v>
@@ -15181,7 +15181,7 @@
         <v>1236</v>
       </c>
       <c r="I282">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K282" t="s">
         <v>1240</v>
@@ -15388,7 +15388,7 @@
         <v>1236</v>
       </c>
       <c r="I288">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K288" t="s">
         <v>1243</v>
@@ -15455,7 +15455,7 @@
         <v>1236</v>
       </c>
       <c r="I290">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15496,7 +15496,7 @@
         <v>1236</v>
       </c>
       <c r="I291">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K291" t="s">
         <v>1242</v>
@@ -15534,7 +15534,7 @@
         <v>1236</v>
       </c>
       <c r="I292">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K292" t="s">
         <v>1243</v>
@@ -15572,7 +15572,7 @@
         <v>1236</v>
       </c>
       <c r="I293">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K293" t="s">
         <v>1244</v>
@@ -15610,7 +15610,7 @@
         <v>1236</v>
       </c>
       <c r="I294">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K294" t="s">
         <v>1246</v>
@@ -15645,7 +15645,7 @@
         <v>1236</v>
       </c>
       <c r="I295">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K295" t="s">
         <v>1246</v>
@@ -15680,7 +15680,7 @@
         <v>1236</v>
       </c>
       <c r="I296">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K296" t="s">
         <v>1246</v>
@@ -15750,7 +15750,7 @@
         <v>1236</v>
       </c>
       <c r="I298">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K298" t="s">
         <v>1240</v>
@@ -15788,7 +15788,7 @@
         <v>1236</v>
       </c>
       <c r="I299">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K299" t="s">
         <v>1243</v>
@@ -15826,7 +15826,7 @@
         <v>1236</v>
       </c>
       <c r="I300">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K300" t="s">
         <v>1243</v>
@@ -15864,7 +15864,7 @@
         <v>1236</v>
       </c>
       <c r="I301">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K301" t="s">
         <v>1243</v>
@@ -15902,7 +15902,7 @@
         <v>1236</v>
       </c>
       <c r="I302">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K302" t="s">
         <v>1243</v>
@@ -15940,7 +15940,7 @@
         <v>1236</v>
       </c>
       <c r="I303">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K303" t="s">
         <v>1240</v>
@@ -15978,7 +15978,7 @@
         <v>1236</v>
       </c>
       <c r="I304">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K304" t="s">
         <v>1243</v>
@@ -16016,7 +16016,7 @@
         <v>1236</v>
       </c>
       <c r="I305">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16060,7 +16060,7 @@
         <v>1236</v>
       </c>
       <c r="I306">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16104,7 +16104,7 @@
         <v>1236</v>
       </c>
       <c r="I307">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K307" t="s">
         <v>1239</v>
@@ -16142,7 +16142,7 @@
         <v>1236</v>
       </c>
       <c r="I308">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K308" t="s">
         <v>1239</v>
@@ -16180,7 +16180,7 @@
         <v>1236</v>
       </c>
       <c r="I309">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K309" t="s">
         <v>1239</v>
@@ -16218,7 +16218,7 @@
         <v>1236</v>
       </c>
       <c r="I310">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K310" t="s">
         <v>1240</v>
@@ -16256,7 +16256,7 @@
         <v>1236</v>
       </c>
       <c r="I311">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K311" t="s">
         <v>1239</v>
@@ -16294,7 +16294,7 @@
         <v>1236</v>
       </c>
       <c r="I312">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K312" t="s">
         <v>1240</v>
@@ -16367,7 +16367,7 @@
         <v>1236</v>
       </c>
       <c r="I314">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K314" t="s">
         <v>1240</v>
@@ -16405,7 +16405,7 @@
         <v>1236</v>
       </c>
       <c r="I315">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K315" t="s">
         <v>1240</v>
@@ -16443,7 +16443,7 @@
         <v>1236</v>
       </c>
       <c r="I316">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K316" t="s">
         <v>1240</v>
@@ -16481,7 +16481,7 @@
         <v>1236</v>
       </c>
       <c r="I317">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K317" t="s">
         <v>1240</v>
@@ -16592,7 +16592,7 @@
         <v>1236</v>
       </c>
       <c r="I320">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K320" t="s">
         <v>1244</v>
@@ -16630,7 +16630,7 @@
         <v>1236</v>
       </c>
       <c r="I321">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K321" t="s">
         <v>1240</v>
@@ -16668,7 +16668,7 @@
         <v>1236</v>
       </c>
       <c r="I322">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16712,7 +16712,7 @@
         <v>1236</v>
       </c>
       <c r="I323">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K323" t="s">
         <v>1240</v>
@@ -16750,7 +16750,7 @@
         <v>1236</v>
       </c>
       <c r="I324">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K324" t="s">
         <v>1240</v>
@@ -16788,7 +16788,7 @@
         <v>1236</v>
       </c>
       <c r="I325">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -16832,7 +16832,7 @@
         <v>1236</v>
       </c>
       <c r="I326">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K326" t="s">
         <v>1240</v>
@@ -16870,7 +16870,7 @@
         <v>1236</v>
       </c>
       <c r="I327">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -16914,7 +16914,7 @@
         <v>1236</v>
       </c>
       <c r="I328">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -16958,7 +16958,7 @@
         <v>1236</v>
       </c>
       <c r="I329">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17002,7 +17002,7 @@
         <v>1236</v>
       </c>
       <c r="I330">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17046,7 +17046,7 @@
         <v>1236</v>
       </c>
       <c r="I331">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K331" t="s">
         <v>1239</v>
@@ -17084,7 +17084,7 @@
         <v>1236</v>
       </c>
       <c r="I332">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K332" t="s">
         <v>1240</v>
@@ -17122,7 +17122,7 @@
         <v>1236</v>
       </c>
       <c r="I333">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K333" t="s">
         <v>1243</v>
@@ -17160,7 +17160,7 @@
         <v>1236</v>
       </c>
       <c r="I334">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K334" t="s">
         <v>1240</v>
@@ -17239,7 +17239,7 @@
         <v>1236</v>
       </c>
       <c r="I336">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K336" t="s">
         <v>1242</v>
@@ -17318,7 +17318,7 @@
         <v>1236</v>
       </c>
       <c r="I338">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K338" t="s">
         <v>1242</v>
@@ -17385,7 +17385,7 @@
         <v>1236</v>
       </c>
       <c r="I340">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K340" t="s">
         <v>1239</v>
@@ -17423,7 +17423,7 @@
         <v>1236</v>
       </c>
       <c r="I341">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K341" t="s">
         <v>1239</v>
@@ -17461,7 +17461,7 @@
         <v>1236</v>
       </c>
       <c r="I342">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K342" t="s">
         <v>1239</v>
@@ -17499,7 +17499,7 @@
         <v>1236</v>
       </c>
       <c r="I343">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K343" t="s">
         <v>1240</v>
@@ -17537,7 +17537,7 @@
         <v>1236</v>
       </c>
       <c r="I344">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K344" t="s">
         <v>1240</v>
@@ -17575,7 +17575,7 @@
         <v>1236</v>
       </c>
       <c r="I345">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K345" t="s">
         <v>1239</v>
@@ -17613,7 +17613,7 @@
         <v>1236</v>
       </c>
       <c r="I346">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K346" t="s">
         <v>1240</v>
@@ -17651,7 +17651,7 @@
         <v>1236</v>
       </c>
       <c r="I347">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17695,7 +17695,7 @@
         <v>1236</v>
       </c>
       <c r="I348">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17739,7 +17739,7 @@
         <v>1236</v>
       </c>
       <c r="I349">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K349" t="s">
         <v>1244</v>
@@ -17777,7 +17777,7 @@
         <v>1236</v>
       </c>
       <c r="I350">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K350" t="s">
         <v>1246</v>
@@ -17812,7 +17812,7 @@
         <v>1236</v>
       </c>
       <c r="I351">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K351" t="s">
         <v>1244</v>
@@ -17850,7 +17850,7 @@
         <v>1236</v>
       </c>
       <c r="I352">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K352" t="s">
         <v>1244</v>
@@ -17888,7 +17888,7 @@
         <v>1236</v>
       </c>
       <c r="I353">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K353" t="s">
         <v>1243</v>
@@ -17926,7 +17926,7 @@
         <v>1236</v>
       </c>
       <c r="I354">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K354" t="s">
         <v>1243</v>
@@ -17964,7 +17964,7 @@
         <v>1236</v>
       </c>
       <c r="I355">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18046,7 +18046,7 @@
         <v>1236</v>
       </c>
       <c r="I357">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K357" t="s">
         <v>1243</v>
@@ -18084,7 +18084,7 @@
         <v>1236</v>
       </c>
       <c r="I358">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K358" t="s">
         <v>1243</v>
@@ -18163,7 +18163,7 @@
         <v>1236</v>
       </c>
       <c r="I360">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K360" t="s">
         <v>1243</v>
@@ -18201,7 +18201,7 @@
         <v>1236</v>
       </c>
       <c r="I361">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K361" t="s">
         <v>1243</v>
@@ -18239,7 +18239,7 @@
         <v>1236</v>
       </c>
       <c r="I362">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K362" t="s">
         <v>1243</v>
@@ -18277,7 +18277,7 @@
         <v>1236</v>
       </c>
       <c r="I363">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K363" t="s">
         <v>1243</v>
@@ -18315,7 +18315,7 @@
         <v>1236</v>
       </c>
       <c r="I364">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K364" t="s">
         <v>1243</v>
@@ -18353,7 +18353,7 @@
         <v>1236</v>
       </c>
       <c r="I365">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K365" t="s">
         <v>1242</v>
@@ -18391,7 +18391,7 @@
         <v>1236</v>
       </c>
       <c r="I366">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K366" t="s">
         <v>1243</v>
@@ -18429,7 +18429,7 @@
         <v>1236</v>
       </c>
       <c r="I367">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K367" t="s">
         <v>1243</v>
@@ -18467,7 +18467,7 @@
         <v>1236</v>
       </c>
       <c r="I368">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K368" t="s">
         <v>1243</v>
@@ -18505,7 +18505,7 @@
         <v>1236</v>
       </c>
       <c r="I369">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K369" t="s">
         <v>1243</v>
@@ -18543,7 +18543,7 @@
         <v>1236</v>
       </c>
       <c r="I370">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K370" t="s">
         <v>1243</v>
@@ -18581,7 +18581,7 @@
         <v>1236</v>
       </c>
       <c r="I371">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18625,7 +18625,7 @@
         <v>1236</v>
       </c>
       <c r="I372">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J372">
         <v>-35</v>
@@ -18672,7 +18672,7 @@
         <v>1236</v>
       </c>
       <c r="I373">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K373" t="s">
         <v>1239</v>
@@ -18710,7 +18710,7 @@
         <v>1236</v>
       </c>
       <c r="I374">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K374" t="s">
         <v>1239</v>
@@ -18748,7 +18748,7 @@
         <v>1236</v>
       </c>
       <c r="I375">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K375" t="s">
         <v>1243</v>
@@ -18786,7 +18786,7 @@
         <v>1236</v>
       </c>
       <c r="I376">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K376" t="s">
         <v>1243</v>
@@ -18862,7 +18862,7 @@
         <v>1236</v>
       </c>
       <c r="I378">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K378" t="s">
         <v>1243</v>
@@ -18900,7 +18900,7 @@
         <v>1236</v>
       </c>
       <c r="I379">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -18944,7 +18944,7 @@
         <v>1236</v>
       </c>
       <c r="I380">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K380" t="s">
         <v>1243</v>
@@ -18982,7 +18982,7 @@
         <v>1236</v>
       </c>
       <c r="I381">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K381" t="s">
         <v>1243</v>
@@ -19020,7 +19020,7 @@
         <v>1236</v>
       </c>
       <c r="I382">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K382" t="s">
         <v>1243</v>
@@ -19058,7 +19058,7 @@
         <v>1236</v>
       </c>
       <c r="I383">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K383" t="s">
         <v>1243</v>
@@ -19096,7 +19096,7 @@
         <v>1236</v>
       </c>
       <c r="I384">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K384" t="s">
         <v>1239</v>
@@ -19134,7 +19134,7 @@
         <v>1236</v>
       </c>
       <c r="I385">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K385" t="s">
         <v>1239</v>
@@ -19172,7 +19172,7 @@
         <v>1236</v>
       </c>
       <c r="I386">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K386" t="s">
         <v>1243</v>
@@ -19210,7 +19210,7 @@
         <v>1236</v>
       </c>
       <c r="I387">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K387" t="s">
         <v>1243</v>
@@ -19248,7 +19248,7 @@
         <v>1236</v>
       </c>
       <c r="I388">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K388" t="s">
         <v>1243</v>
@@ -19286,7 +19286,7 @@
         <v>1236</v>
       </c>
       <c r="I389">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K389" t="s">
         <v>1244</v>
@@ -19324,7 +19324,7 @@
         <v>1236</v>
       </c>
       <c r="I390">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J390">
         <v>20</v>
@@ -19447,7 +19447,7 @@
         <v>1236</v>
       </c>
       <c r="I393">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K393" t="s">
         <v>1243</v>
@@ -19485,7 +19485,7 @@
         <v>1236</v>
       </c>
       <c r="I394">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K394" t="s">
         <v>1243</v>
@@ -19523,7 +19523,7 @@
         <v>1236</v>
       </c>
       <c r="I395">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K395" t="s">
         <v>1243</v>
@@ -19564,7 +19564,7 @@
         <v>1236</v>
       </c>
       <c r="I396">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K396" t="s">
         <v>1243</v>
@@ -19605,7 +19605,7 @@
         <v>1236</v>
       </c>
       <c r="I397">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K397" t="s">
         <v>1243</v>
@@ -19643,7 +19643,7 @@
         <v>1236</v>
       </c>
       <c r="I398">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K398" t="s">
         <v>1243</v>
@@ -19722,7 +19722,7 @@
         <v>1236</v>
       </c>
       <c r="I400">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K400" t="s">
         <v>1243</v>
@@ -19760,7 +19760,7 @@
         <v>1236</v>
       </c>
       <c r="I401">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K401" t="s">
         <v>1243</v>
@@ -19801,7 +19801,7 @@
         <v>1236</v>
       </c>
       <c r="I402">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K402" t="s">
         <v>1243</v>
@@ -19839,7 +19839,7 @@
         <v>1236</v>
       </c>
       <c r="I403">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K403" t="s">
         <v>1246</v>
@@ -19874,7 +19874,7 @@
         <v>1236</v>
       </c>
       <c r="I404">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K404" t="s">
         <v>1246</v>
@@ -19938,7 +19938,7 @@
         <v>1236</v>
       </c>
       <c r="I406">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -19970,7 +19970,7 @@
         <v>1236</v>
       </c>
       <c r="I407">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20002,7 +20002,7 @@
         <v>1236</v>
       </c>
       <c r="I408">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20034,7 +20034,7 @@
         <v>1236</v>
       </c>
       <c r="I409">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20066,7 +20066,7 @@
         <v>1236</v>
       </c>
       <c r="I410">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20098,7 +20098,7 @@
         <v>1236</v>
       </c>
       <c r="I411">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20130,7 +20130,7 @@
         <v>1236</v>
       </c>
       <c r="I412">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20162,7 +20162,7 @@
         <v>1236</v>
       </c>
       <c r="I413">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20194,7 +20194,7 @@
         <v>1236</v>
       </c>
       <c r="I414">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q414" t="b">
         <v>1</v>
@@ -20226,7 +20226,7 @@
         <v>1236</v>
       </c>
       <c r="I415">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q415" t="b">
         <v>1</v>
@@ -20258,7 +20258,7 @@
         <v>1236</v>
       </c>
       <c r="I416">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20290,7 +20290,7 @@
         <v>1236</v>
       </c>
       <c r="I417">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q417" t="b">
         <v>1</v>
@@ -20322,7 +20322,7 @@
         <v>1236</v>
       </c>
       <c r="I418">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q418" t="b">
         <v>1</v>
@@ -20354,7 +20354,7 @@
         <v>1236</v>
       </c>
       <c r="I419">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20386,7 +20386,7 @@
         <v>1236</v>
       </c>
       <c r="I420">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20418,7 +20418,7 @@
         <v>1236</v>
       </c>
       <c r="I421">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20450,7 +20450,7 @@
         <v>1236</v>
       </c>
       <c r="I422">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20482,7 +20482,7 @@
         <v>1236</v>
       </c>
       <c r="I423">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20514,7 +20514,7 @@
         <v>1236</v>
       </c>
       <c r="I424">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20546,7 +20546,7 @@
         <v>1236</v>
       </c>
       <c r="I425">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20578,7 +20578,7 @@
         <v>1236</v>
       </c>
       <c r="I426">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20610,7 +20610,7 @@
         <v>1236</v>
       </c>
       <c r="I427">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20642,7 +20642,7 @@
         <v>1236</v>
       </c>
       <c r="I428">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q428" t="b">
         <v>1</v>
@@ -20674,7 +20674,7 @@
         <v>1236</v>
       </c>
       <c r="I429">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q429" t="b">
         <v>1</v>
@@ -20706,7 +20706,7 @@
         <v>1236</v>
       </c>
       <c r="I430">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -20738,7 +20738,7 @@
         <v>1236</v>
       </c>
       <c r="I431">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -20770,7 +20770,7 @@
         <v>1236</v>
       </c>
       <c r="I432">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -20802,7 +20802,7 @@
         <v>1236</v>
       </c>
       <c r="I433">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -20834,7 +20834,7 @@
         <v>1236</v>
       </c>
       <c r="I434">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -20866,7 +20866,7 @@
         <v>1236</v>
       </c>
       <c r="I435">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -20898,7 +20898,7 @@
         <v>1236</v>
       </c>
       <c r="I436">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -20930,7 +20930,7 @@
         <v>1238</v>
       </c>
       <c r="I437">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -20962,7 +20962,7 @@
         <v>1238</v>
       </c>
       <c r="I438">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -20994,7 +20994,7 @@
         <v>1236</v>
       </c>
       <c r="I439">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21026,7 +21026,7 @@
         <v>1236</v>
       </c>
       <c r="I440">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21058,7 +21058,7 @@
         <v>1236</v>
       </c>
       <c r="I441">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21090,7 +21090,7 @@
         <v>1236</v>
       </c>
       <c r="I442">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q442" t="b">
         <v>1</v>
@@ -21122,7 +21122,7 @@
         <v>1236</v>
       </c>
       <c r="I443">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21154,7 +21154,7 @@
         <v>1236</v>
       </c>
       <c r="I444">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q444" t="b">
         <v>1</v>
@@ -21186,7 +21186,7 @@
         <v>1236</v>
       </c>
       <c r="I445">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q445" t="b">
         <v>1</v>
@@ -21218,7 +21218,7 @@
         <v>1236</v>
       </c>
       <c r="I446">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21250,7 +21250,7 @@
         <v>1236</v>
       </c>
       <c r="I447">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21282,7 +21282,7 @@
         <v>1236</v>
       </c>
       <c r="I448">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21314,7 +21314,7 @@
         <v>1236</v>
       </c>
       <c r="I449">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21346,7 +21346,7 @@
         <v>1236</v>
       </c>
       <c r="I450">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21378,7 +21378,7 @@
         <v>1236</v>
       </c>
       <c r="I451">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21410,7 +21410,7 @@
         <v>1236</v>
       </c>
       <c r="I452">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21442,7 +21442,7 @@
         <v>1236</v>
       </c>
       <c r="I453">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21474,7 +21474,7 @@
         <v>1236</v>
       </c>
       <c r="I454">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21506,7 +21506,7 @@
         <v>1236</v>
       </c>
       <c r="I455">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21538,7 +21538,7 @@
         <v>1236</v>
       </c>
       <c r="I456">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21570,7 +21570,7 @@
         <v>1236</v>
       </c>
       <c r="I457">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21602,7 +21602,7 @@
         <v>1236</v>
       </c>
       <c r="I458">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21634,7 +21634,7 @@
         <v>1236</v>
       </c>
       <c r="I459">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21666,7 +21666,7 @@
         <v>1236</v>
       </c>
       <c r="I460">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21698,7 +21698,7 @@
         <v>1236</v>
       </c>
       <c r="I461">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -21730,7 +21730,7 @@
         <v>1236</v>
       </c>
       <c r="I462">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -21762,7 +21762,7 @@
         <v>1236</v>
       </c>
       <c r="I463">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -21794,7 +21794,7 @@
         <v>1238</v>
       </c>
       <c r="I464">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -21826,7 +21826,7 @@
         <v>1238</v>
       </c>
       <c r="I465">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -21858,7 +21858,7 @@
         <v>1238</v>
       </c>
       <c r="I466">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -21890,7 +21890,7 @@
         <v>1238</v>
       </c>
       <c r="I467">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -21922,7 +21922,7 @@
         <v>1238</v>
       </c>
       <c r="I468">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -21954,7 +21954,7 @@
         <v>1238</v>
       </c>
       <c r="I469">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -21986,7 +21986,7 @@
         <v>1238</v>
       </c>
       <c r="I470">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q470" t="b">
         <v>1</v>
@@ -22018,7 +22018,7 @@
         <v>1238</v>
       </c>
       <c r="I471">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22050,7 +22050,7 @@
         <v>1238</v>
       </c>
       <c r="I472">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22082,7 +22082,7 @@
         <v>1238</v>
       </c>
       <c r="I473">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22114,7 +22114,7 @@
         <v>1238</v>
       </c>
       <c r="I474">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22146,7 +22146,7 @@
         <v>1238</v>
       </c>
       <c r="I475">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22178,7 +22178,7 @@
         <v>1238</v>
       </c>
       <c r="I476">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22210,7 +22210,7 @@
         <v>1238</v>
       </c>
       <c r="I477">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22242,7 +22242,7 @@
         <v>1238</v>
       </c>
       <c r="I478">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22274,7 +22274,7 @@
         <v>1238</v>
       </c>
       <c r="I479">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22306,7 +22306,7 @@
         <v>1238</v>
       </c>
       <c r="I480">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22338,7 +22338,7 @@
         <v>1238</v>
       </c>
       <c r="I481">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22370,7 +22370,7 @@
         <v>1238</v>
       </c>
       <c r="I482">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22402,7 +22402,7 @@
         <v>1238</v>
       </c>
       <c r="I483">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22434,7 +22434,7 @@
         <v>1238</v>
       </c>
       <c r="I484">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22466,7 +22466,7 @@
         <v>1238</v>
       </c>
       <c r="I485">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22498,7 +22498,7 @@
         <v>1238</v>
       </c>
       <c r="I486">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22530,7 +22530,7 @@
         <v>1238</v>
       </c>
       <c r="I487">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22562,7 +22562,7 @@
         <v>1238</v>
       </c>
       <c r="I488">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22594,7 +22594,7 @@
         <v>1238</v>
       </c>
       <c r="I489">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22626,7 +22626,7 @@
         <v>1238</v>
       </c>
       <c r="I490">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22658,7 +22658,7 @@
         <v>1238</v>
       </c>
       <c r="I491">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22690,7 +22690,7 @@
         <v>1238</v>
       </c>
       <c r="I492">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22722,7 +22722,7 @@
         <v>1238</v>
       </c>
       <c r="I493">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -22754,7 +22754,7 @@
         <v>1238</v>
       </c>
       <c r="I494">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -22786,7 +22786,7 @@
         <v>1238</v>
       </c>
       <c r="I495">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -22818,7 +22818,7 @@
         <v>1238</v>
       </c>
       <c r="I496">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -22850,7 +22850,7 @@
         <v>1238</v>
       </c>
       <c r="I497">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -22882,7 +22882,7 @@
         <v>1238</v>
       </c>
       <c r="I498">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -22914,7 +22914,7 @@
         <v>1238</v>
       </c>
       <c r="I499">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -22946,7 +22946,7 @@
         <v>1238</v>
       </c>
       <c r="I500">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -22978,7 +22978,7 @@
         <v>1238</v>
       </c>
       <c r="I501">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23010,7 +23010,7 @@
         <v>1238</v>
       </c>
       <c r="I502">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23042,7 +23042,7 @@
         <v>1238</v>
       </c>
       <c r="I503">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23074,7 +23074,7 @@
         <v>1238</v>
       </c>
       <c r="I504">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23106,7 +23106,7 @@
         <v>1238</v>
       </c>
       <c r="I505">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23138,7 +23138,7 @@
         <v>1238</v>
       </c>
       <c r="I506">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23170,7 +23170,7 @@
         <v>1238</v>
       </c>
       <c r="I507">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23202,7 +23202,7 @@
         <v>1238</v>
       </c>
       <c r="I508">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q508" t="b">
         <v>1</v>
@@ -23234,7 +23234,7 @@
         <v>1238</v>
       </c>
       <c r="I509">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23266,7 +23266,7 @@
         <v>1238</v>
       </c>
       <c r="I510">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (12/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4129" uniqueCount="1377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4009" uniqueCount="1345">
   <si>
     <t>os</t>
   </si>
@@ -3781,36 +3781,18 @@
     <t>045/C98/2025</t>
   </si>
   <si>
-    <t>1032/LS-C98/2025</t>
-  </si>
-  <si>
     <t>352/FAB/26</t>
   </si>
   <si>
-    <t>310/FAB/26</t>
-  </si>
-  <si>
     <t>1082/2025</t>
   </si>
   <si>
-    <t>252/FAB/26</t>
-  </si>
-  <si>
-    <t>1094/LS-C-98/2025</t>
-  </si>
-  <si>
     <t>1049/2025</t>
   </si>
   <si>
     <t>161/FAB/25</t>
   </si>
   <si>
-    <t>044/C98/2025</t>
-  </si>
-  <si>
-    <t>250/FAB/25</t>
-  </si>
-  <si>
     <t>1034/2025</t>
   </si>
   <si>
@@ -3820,27 +3802,12 @@
     <t>263/FAB/26</t>
   </si>
   <si>
-    <t>1019/LS-C98/2025</t>
-  </si>
-  <si>
-    <t>196/FAB/26</t>
-  </si>
-  <si>
     <t>176/FAB/26</t>
   </si>
   <si>
     <t>133/FAB/25</t>
   </si>
   <si>
-    <t>160/C98/2025</t>
-  </si>
-  <si>
-    <t>328/FAB/26</t>
-  </si>
-  <si>
-    <t>1022/LS-C98/2025</t>
-  </si>
-  <si>
     <t>108/C98/2025</t>
   </si>
   <si>
@@ -3859,30 +3826,12 @@
     <t>143/C98/2025</t>
   </si>
   <si>
-    <t>228/FAB/26</t>
-  </si>
-  <si>
-    <t>131/FAB/25</t>
-  </si>
-  <si>
-    <t>1063/LS-C98/2026</t>
-  </si>
-  <si>
     <t>083/FAB/25</t>
   </si>
   <si>
-    <t>1043/LS-C98/2025</t>
-  </si>
-  <si>
     <t>329/FAB/26</t>
   </si>
   <si>
-    <t>1059/LS-C98/2025</t>
-  </si>
-  <si>
-    <t>015/FAB/26</t>
-  </si>
-  <si>
     <t>162/FAB/25</t>
   </si>
   <si>
@@ -3892,9 +3841,6 @@
     <t>140/FAB/25</t>
   </si>
   <si>
-    <t>327/FAB/25</t>
-  </si>
-  <si>
     <t>MATERIAL VOLTOU EM GARANTIA</t>
   </si>
   <si>
@@ -3907,9 +3853,6 @@
     <t>198/FAB/25</t>
   </si>
   <si>
-    <t>332/FAB/26</t>
-  </si>
-  <si>
     <t>329/FAB/25</t>
   </si>
   <si>
@@ -3925,9 +3868,6 @@
     <t>1116/LS-C98/2026</t>
   </si>
   <si>
-    <t>317/FAB/26</t>
-  </si>
-  <si>
     <t>362/FAB/26</t>
   </si>
   <si>
@@ -3937,12 +3877,6 @@
     <t>490/FAB/26</t>
   </si>
   <si>
-    <t>1114/LS-C-98/2026</t>
-  </si>
-  <si>
-    <t>375/FAB/2026</t>
-  </si>
-  <si>
     <t>339/FAB/25</t>
   </si>
   <si>
@@ -3952,49 +3886,19 @@
     <t>195/FAB/26</t>
   </si>
   <si>
-    <t>075/FAB/26</t>
-  </si>
-  <si>
     <t>269/FAB/26</t>
   </si>
   <si>
     <t>063/FAB/26</t>
   </si>
   <si>
-    <t>256/FAB/26</t>
-  </si>
-  <si>
-    <t>367/FAB/2026</t>
-  </si>
-  <si>
     <t>485/FAB/26</t>
   </si>
   <si>
-    <t>153/FAB/26</t>
-  </si>
-  <si>
-    <t>143/FAB/2026</t>
-  </si>
-  <si>
     <t>261/FAB/26</t>
   </si>
   <si>
-    <t>232/FAB/26</t>
-  </si>
-  <si>
     <t>498/FAB/26</t>
-  </si>
-  <si>
-    <t>301/FAB/26</t>
-  </si>
-  <si>
-    <t>222/FAB/26</t>
-  </si>
-  <si>
-    <t>383/FAB/20286</t>
-  </si>
-  <si>
-    <t>448/FAB/2026</t>
   </si>
   <si>
     <t>392/FAB/26</t>
@@ -4568,7 +4472,7 @@
         <v>1239</v>
       </c>
       <c r="M2" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q2" t="b">
         <v>1</v>
@@ -4606,7 +4510,7 @@
         <v>1240</v>
       </c>
       <c r="M3" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
@@ -4644,7 +4548,7 @@
         <v>1240</v>
       </c>
       <c r="M4" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
@@ -4779,7 +4683,7 @@
         <v>45848</v>
       </c>
       <c r="O7" t="s">
-        <v>1346</v>
+        <v>1314</v>
       </c>
       <c r="Q7" t="b">
         <v>1</v>
@@ -4902,7 +4806,7 @@
         <v>46114</v>
       </c>
       <c r="O10" t="s">
-        <v>1347</v>
+        <v>1315</v>
       </c>
       <c r="Q10" t="b">
         <v>1</v>
@@ -4949,7 +4853,7 @@
         <v>45848</v>
       </c>
       <c r="O11" t="s">
-        <v>1348</v>
+        <v>1316</v>
       </c>
       <c r="Q11" t="b">
         <v>1</v>
@@ -5024,12 +4928,6 @@
       <c r="H13" t="s">
         <v>1237</v>
       </c>
-      <c r="L13" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M13" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
@@ -5110,7 +5008,7 @@
         <v>1242</v>
       </c>
       <c r="M15" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q15" t="b">
         <v>1</v>
@@ -5148,7 +5046,7 @@
         <v>1239</v>
       </c>
       <c r="M16" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q16" t="b">
         <v>1</v>
@@ -5267,12 +5165,6 @@
       <c r="H19" t="s">
         <v>1237</v>
       </c>
-      <c r="L19" t="s">
-        <v>1255</v>
-      </c>
-      <c r="M19" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q19" t="b">
         <v>0</v>
       </c>
@@ -5312,7 +5204,7 @@
         <v>1213</v>
       </c>
       <c r="L20" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="N20" s="1">
         <v>46135</v>
@@ -5346,12 +5238,6 @@
       <c r="H21" t="s">
         <v>1237</v>
       </c>
-      <c r="L21" t="s">
-        <v>1257</v>
-      </c>
-      <c r="M21" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q21" t="b">
         <v>0</v>
       </c>
@@ -5388,7 +5274,7 @@
         <v>1243</v>
       </c>
       <c r="M22" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q22" t="b">
         <v>1</v>
@@ -5429,13 +5315,13 @@
         <v>1209</v>
       </c>
       <c r="L23" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="N23" s="1">
         <v>45965</v>
       </c>
       <c r="P23" t="s">
-        <v>1355</v>
+        <v>1323</v>
       </c>
       <c r="Q23" t="b">
         <v>1</v>
@@ -5466,15 +5352,6 @@
       <c r="H24" t="s">
         <v>1237</v>
       </c>
-      <c r="J24">
-        <v>41</v>
-      </c>
-      <c r="L24" t="s">
-        <v>1259</v>
-      </c>
-      <c r="M24" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q24" t="b">
         <v>0</v>
       </c>
@@ -5504,15 +5381,6 @@
       <c r="H25" t="s">
         <v>1237</v>
       </c>
-      <c r="J25">
-        <v>140</v>
-      </c>
-      <c r="L25" t="s">
-        <v>1260</v>
-      </c>
-      <c r="M25" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q25" t="b">
         <v>0</v>
       </c>
@@ -5552,13 +5420,13 @@
         <v>1213</v>
       </c>
       <c r="L26" t="s">
-        <v>1261</v>
+        <v>1257</v>
       </c>
       <c r="N26" s="1">
         <v>45891</v>
       </c>
       <c r="P26" t="s">
-        <v>1356</v>
+        <v>1324</v>
       </c>
       <c r="Q26" t="b">
         <v>1</v>
@@ -5596,7 +5464,7 @@
         <v>1243</v>
       </c>
       <c r="M27" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q27" t="b">
         <v>1</v>
@@ -5656,15 +5524,6 @@
       <c r="H29" t="s">
         <v>1237</v>
       </c>
-      <c r="J29">
-        <v>113</v>
-      </c>
-      <c r="L29" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M29" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q29" t="b">
         <v>0</v>
       </c>
@@ -5704,7 +5563,7 @@
         <v>1212</v>
       </c>
       <c r="L30" t="s">
-        <v>1262</v>
+        <v>1258</v>
       </c>
       <c r="N30" s="1">
         <v>45945</v>
@@ -5738,15 +5597,6 @@
       <c r="H31" t="s">
         <v>1237</v>
       </c>
-      <c r="J31">
-        <v>33</v>
-      </c>
-      <c r="L31" t="s">
-        <v>1263</v>
-      </c>
-      <c r="M31" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q31" t="b">
         <v>0</v>
       </c>
@@ -5783,7 +5633,7 @@
         <v>1239</v>
       </c>
       <c r="M32" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q32" t="b">
         <v>1</v>
@@ -5814,12 +5664,6 @@
       <c r="H33" t="s">
         <v>1237</v>
       </c>
-      <c r="L33" t="s">
-        <v>1263</v>
-      </c>
-      <c r="M33" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q33" t="b">
         <v>0</v>
       </c>
@@ -5907,15 +5751,6 @@
       <c r="H36" t="s">
         <v>1237</v>
       </c>
-      <c r="J36">
-        <v>140</v>
-      </c>
-      <c r="L36" t="s">
-        <v>1264</v>
-      </c>
-      <c r="M36" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q36" t="b">
         <v>0</v>
       </c>
@@ -5945,15 +5780,6 @@
       <c r="H37" t="s">
         <v>1237</v>
       </c>
-      <c r="J37">
-        <v>225</v>
-      </c>
-      <c r="L37" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M37" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q37" t="b">
         <v>0</v>
       </c>
@@ -5983,15 +5809,6 @@
       <c r="H38" t="s">
         <v>1237</v>
       </c>
-      <c r="J38">
-        <v>127</v>
-      </c>
-      <c r="L38" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M38" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q38" t="b">
         <v>0</v>
       </c>
@@ -6025,7 +5842,7 @@
         <v>1244</v>
       </c>
       <c r="M39" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q39" t="b">
         <v>1</v>
@@ -6060,7 +5877,7 @@
         <v>1242</v>
       </c>
       <c r="M40" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q40" t="b">
         <v>1</v>
@@ -6091,15 +5908,6 @@
       <c r="H41" t="s">
         <v>1237</v>
       </c>
-      <c r="J41">
-        <v>124</v>
-      </c>
-      <c r="L41" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M41" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q41" t="b">
         <v>0</v>
       </c>
@@ -6129,15 +5937,6 @@
       <c r="H42" t="s">
         <v>1237</v>
       </c>
-      <c r="J42">
-        <v>127</v>
-      </c>
-      <c r="L42" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M42" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q42" t="b">
         <v>0</v>
       </c>
@@ -6171,7 +5970,7 @@
         <v>1245</v>
       </c>
       <c r="M43" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -6212,13 +6011,13 @@
         <v>1209</v>
       </c>
       <c r="L44" t="s">
-        <v>1265</v>
+        <v>1259</v>
       </c>
       <c r="N44" s="1">
         <v>45856</v>
       </c>
       <c r="P44" t="s">
-        <v>1357</v>
+        <v>1325</v>
       </c>
       <c r="Q44" t="b">
         <v>1</v>
@@ -6259,7 +6058,7 @@
         <v>1210</v>
       </c>
       <c r="L45" t="s">
-        <v>1266</v>
+        <v>1260</v>
       </c>
       <c r="N45" s="1">
         <v>46100</v>
@@ -6303,7 +6102,7 @@
         <v>1243</v>
       </c>
       <c r="M46" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q46" t="b">
         <v>1</v>
@@ -6344,13 +6143,13 @@
         <v>1221</v>
       </c>
       <c r="L47" t="s">
-        <v>1267</v>
+        <v>1261</v>
       </c>
       <c r="N47" s="1">
         <v>46113</v>
       </c>
       <c r="P47" t="s">
-        <v>1358</v>
+        <v>1326</v>
       </c>
       <c r="Q47" t="b">
         <v>1</v>
@@ -6388,7 +6187,7 @@
         <v>1243</v>
       </c>
       <c r="M48" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q48" t="b">
         <v>1</v>
@@ -6419,9 +6218,6 @@
       <c r="H49" t="s">
         <v>1237</v>
       </c>
-      <c r="J49">
-        <v>107</v>
-      </c>
       <c r="Q49" t="b">
         <v>0</v>
       </c>
@@ -6458,7 +6254,7 @@
         <v>1243</v>
       </c>
       <c r="M50" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q50" t="b">
         <v>1</v>
@@ -6489,15 +6285,6 @@
       <c r="H51" t="s">
         <v>1237</v>
       </c>
-      <c r="J51">
-        <v>69</v>
-      </c>
-      <c r="L51" t="s">
-        <v>1268</v>
-      </c>
-      <c r="M51" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q51" t="b">
         <v>0</v>
       </c>
@@ -6534,7 +6321,7 @@
         <v>1239</v>
       </c>
       <c r="M52" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q52" t="b">
         <v>1</v>
@@ -6572,7 +6359,7 @@
         <v>1240</v>
       </c>
       <c r="M53" t="s">
-        <v>1340</v>
+        <v>1308</v>
       </c>
       <c r="Q53" t="b">
         <v>1</v>
@@ -6610,7 +6397,7 @@
         <v>1240</v>
       </c>
       <c r="M54" t="s">
-        <v>1340</v>
+        <v>1308</v>
       </c>
       <c r="Q54" t="b">
         <v>1</v>
@@ -6641,9 +6428,6 @@
       <c r="H55" t="s">
         <v>1237</v>
       </c>
-      <c r="J55">
-        <v>45</v>
-      </c>
       <c r="Q55" t="b">
         <v>0</v>
       </c>
@@ -6673,15 +6457,6 @@
       <c r="H56" t="s">
         <v>1237</v>
       </c>
-      <c r="J56">
-        <v>120</v>
-      </c>
-      <c r="L56" t="s">
-        <v>1268</v>
-      </c>
-      <c r="M56" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q56" t="b">
         <v>0</v>
       </c>
@@ -6718,7 +6493,7 @@
         <v>1243</v>
       </c>
       <c r="M57" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q57" t="b">
         <v>1</v>
@@ -6749,9 +6524,6 @@
       <c r="H58" t="s">
         <v>1237</v>
       </c>
-      <c r="J58">
-        <v>120</v>
-      </c>
       <c r="Q58" t="b">
         <v>0</v>
       </c>
@@ -6781,12 +6553,6 @@
       <c r="H59" t="s">
         <v>1237</v>
       </c>
-      <c r="L59" t="s">
-        <v>1255</v>
-      </c>
-      <c r="M59" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q59" t="b">
         <v>0</v>
       </c>
@@ -6816,12 +6582,6 @@
       <c r="H60" t="s">
         <v>1237</v>
       </c>
-      <c r="L60" t="s">
-        <v>1269</v>
-      </c>
-      <c r="M60" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q60" t="b">
         <v>0</v>
       </c>
@@ -6851,9 +6611,6 @@
       <c r="H61" t="s">
         <v>1237</v>
       </c>
-      <c r="L61" t="s">
-        <v>1268</v>
-      </c>
       <c r="Q61" t="b">
         <v>0</v>
       </c>
@@ -6883,9 +6640,6 @@
       <c r="H62" t="s">
         <v>1237</v>
       </c>
-      <c r="J62">
-        <v>119</v>
-      </c>
       <c r="Q62" t="b">
         <v>0</v>
       </c>
@@ -6925,13 +6679,13 @@
         <v>1210</v>
       </c>
       <c r="L63" t="s">
-        <v>1270</v>
+        <v>1262</v>
       </c>
       <c r="N63" s="1">
         <v>46092</v>
       </c>
       <c r="P63" t="s">
-        <v>1359</v>
+        <v>1327</v>
       </c>
       <c r="Q63" t="b">
         <v>1</v>
@@ -6972,7 +6726,7 @@
         <v>1241</v>
       </c>
       <c r="L64" t="s">
-        <v>1271</v>
+        <v>1263</v>
       </c>
       <c r="N64" s="1">
         <v>46119</v>
@@ -7006,15 +6760,6 @@
       <c r="H65" t="s">
         <v>1237</v>
       </c>
-      <c r="J65">
-        <v>15</v>
-      </c>
-      <c r="L65" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M65" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q65" t="b">
         <v>0</v>
       </c>
@@ -7044,15 +6789,6 @@
       <c r="H66" t="s">
         <v>1237</v>
       </c>
-      <c r="J66">
-        <v>91</v>
-      </c>
-      <c r="L66" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M66" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q66" t="b">
         <v>0</v>
       </c>
@@ -7082,12 +6818,6 @@
       <c r="H67" t="s">
         <v>1237</v>
       </c>
-      <c r="L67" t="s">
-        <v>1271</v>
-      </c>
-      <c r="M67" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q67" t="b">
         <v>0</v>
       </c>
@@ -7117,15 +6847,6 @@
       <c r="H68" t="s">
         <v>1237</v>
       </c>
-      <c r="J68">
-        <v>91</v>
-      </c>
-      <c r="L68" t="s">
-        <v>1271</v>
-      </c>
-      <c r="M68" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q68" t="b">
         <v>0</v>
       </c>
@@ -7155,15 +6876,6 @@
       <c r="H69" t="s">
         <v>1237</v>
       </c>
-      <c r="J69">
-        <v>51</v>
-      </c>
-      <c r="L69" t="s">
-        <v>1272</v>
-      </c>
-      <c r="M69" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q69" t="b">
         <v>0</v>
       </c>
@@ -7200,7 +6912,7 @@
         <v>1240</v>
       </c>
       <c r="M70" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q70" t="b">
         <v>1</v>
@@ -7266,12 +6978,6 @@
       <c r="H72" t="s">
         <v>1237</v>
       </c>
-      <c r="L72" t="s">
-        <v>1272</v>
-      </c>
-      <c r="M72" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q72" t="b">
         <v>0</v>
       </c>
@@ -7308,7 +7014,7 @@
         <v>1239</v>
       </c>
       <c r="M73" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q73" t="b">
         <v>1</v>
@@ -7339,15 +7045,6 @@
       <c r="H74" t="s">
         <v>1237</v>
       </c>
-      <c r="J74">
-        <v>86</v>
-      </c>
-      <c r="L74" t="s">
-        <v>1272</v>
-      </c>
-      <c r="M74" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q74" t="b">
         <v>0</v>
       </c>
@@ -7384,7 +7081,7 @@
         <v>1240</v>
       </c>
       <c r="M75" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q75" t="b">
         <v>1</v>
@@ -7450,12 +7147,6 @@
       <c r="H77" t="s">
         <v>1237</v>
       </c>
-      <c r="L77" t="s">
-        <v>1272</v>
-      </c>
-      <c r="M77" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q77" t="b">
         <v>0</v>
       </c>
@@ -7485,15 +7176,6 @@
       <c r="H78" t="s">
         <v>1237</v>
       </c>
-      <c r="J78">
-        <v>57</v>
-      </c>
-      <c r="L78" t="s">
-        <v>1273</v>
-      </c>
-      <c r="M78" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q78" t="b">
         <v>0</v>
       </c>
@@ -7565,7 +7247,7 @@
         <v>1240</v>
       </c>
       <c r="M80" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q80" t="b">
         <v>1</v>
@@ -7596,15 +7278,6 @@
       <c r="H81" t="s">
         <v>1237</v>
       </c>
-      <c r="J81">
-        <v>50</v>
-      </c>
-      <c r="L81" t="s">
-        <v>1249</v>
-      </c>
-      <c r="M81" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q81" t="b">
         <v>0</v>
       </c>
@@ -7641,7 +7314,7 @@
         <v>1243</v>
       </c>
       <c r="M82" t="s">
-        <v>1341</v>
+        <v>1309</v>
       </c>
       <c r="Q82" t="b">
         <v>1</v>
@@ -7672,12 +7345,6 @@
       <c r="H83" t="s">
         <v>1237</v>
       </c>
-      <c r="L83" t="s">
-        <v>1274</v>
-      </c>
-      <c r="M83" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q83" t="b">
         <v>0</v>
       </c>
@@ -7717,7 +7384,7 @@
         <v>1213</v>
       </c>
       <c r="L84" t="s">
-        <v>1275</v>
+        <v>1264</v>
       </c>
       <c r="N84" s="1">
         <v>45853</v>
@@ -7761,7 +7428,7 @@
         <v>1240</v>
       </c>
       <c r="M85" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q85" t="b">
         <v>1</v>
@@ -7799,7 +7466,7 @@
         <v>1240</v>
       </c>
       <c r="O86" t="s">
-        <v>1349</v>
+        <v>1317</v>
       </c>
       <c r="Q86" t="b">
         <v>1</v>
@@ -7840,13 +7507,13 @@
         <v>1213</v>
       </c>
       <c r="L87" t="s">
-        <v>1276</v>
+        <v>1265</v>
       </c>
       <c r="N87" s="1">
         <v>45797</v>
       </c>
       <c r="O87" t="s">
-        <v>1350</v>
+        <v>1318</v>
       </c>
       <c r="Q87" t="b">
         <v>1</v>
@@ -7881,7 +7548,7 @@
         <v>1245</v>
       </c>
       <c r="M88" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q88" t="b">
         <v>0</v>
@@ -7916,7 +7583,7 @@
         <v>1245</v>
       </c>
       <c r="M89" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q89" t="b">
         <v>0</v>
@@ -7954,10 +7621,10 @@
         <v>1213</v>
       </c>
       <c r="L90" t="s">
-        <v>1277</v>
+        <v>1266</v>
       </c>
       <c r="P90" t="s">
-        <v>1360</v>
+        <v>1328</v>
       </c>
       <c r="Q90" t="b">
         <v>1</v>
@@ -7995,7 +7662,7 @@
         <v>1242</v>
       </c>
       <c r="M91" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q91" t="b">
         <v>1</v>
@@ -8023,9 +7690,6 @@
       <c r="H92" t="s">
         <v>1237</v>
       </c>
-      <c r="J92">
-        <v>218</v>
-      </c>
       <c r="Q92" t="b">
         <v>0</v>
       </c>
@@ -8062,7 +7726,7 @@
         <v>1242</v>
       </c>
       <c r="M93" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q93" t="b">
         <v>1</v>
@@ -8100,7 +7764,7 @@
         <v>1243</v>
       </c>
       <c r="M94" t="s">
-        <v>1342</v>
+        <v>1310</v>
       </c>
       <c r="Q94" t="b">
         <v>1</v>
@@ -8138,7 +7802,7 @@
         <v>1242</v>
       </c>
       <c r="M95" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q95" t="b">
         <v>1</v>
@@ -8185,7 +7849,7 @@
         <v>45848</v>
       </c>
       <c r="O96" t="s">
-        <v>1351</v>
+        <v>1319</v>
       </c>
       <c r="Q96" t="b">
         <v>1</v>
@@ -8223,10 +7887,10 @@
         <v>1213</v>
       </c>
       <c r="L97" t="s">
-        <v>1278</v>
+        <v>1267</v>
       </c>
       <c r="P97" t="s">
-        <v>1356</v>
+        <v>1324</v>
       </c>
       <c r="Q97" t="b">
         <v>1</v>
@@ -8264,7 +7928,7 @@
         <v>1243</v>
       </c>
       <c r="M98" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q98" t="b">
         <v>1</v>
@@ -8331,7 +7995,7 @@
         <v>1242</v>
       </c>
       <c r="M100" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q100" t="b">
         <v>1</v>
@@ -8362,9 +8026,6 @@
       <c r="H101" t="s">
         <v>1237</v>
       </c>
-      <c r="J101">
-        <v>131</v>
-      </c>
       <c r="Q101" t="b">
         <v>0</v>
       </c>
@@ -8459,7 +8120,7 @@
         <v>1242</v>
       </c>
       <c r="M104" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q104" t="b">
         <v>1</v>
@@ -8497,7 +8158,7 @@
         <v>1242</v>
       </c>
       <c r="M105" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q105" t="b">
         <v>1</v>
@@ -8538,7 +8199,7 @@
         <v>1241</v>
       </c>
       <c r="L106" t="s">
-        <v>1279</v>
+        <v>1268</v>
       </c>
       <c r="N106" s="1">
         <v>45889</v>
@@ -8582,7 +8243,7 @@
         <v>1241</v>
       </c>
       <c r="L107" t="s">
-        <v>1280</v>
+        <v>1269</v>
       </c>
       <c r="N107" s="1">
         <v>45876</v>
@@ -8623,7 +8284,7 @@
         <v>1240</v>
       </c>
       <c r="M108" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q108" t="b">
         <v>1</v>
@@ -8661,7 +8322,7 @@
         <v>1240</v>
       </c>
       <c r="M109" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q109" t="b">
         <v>1</v>
@@ -8692,12 +8353,6 @@
       <c r="H110" t="s">
         <v>1237</v>
       </c>
-      <c r="L110" t="s">
-        <v>1281</v>
-      </c>
-      <c r="M110" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q110" t="b">
         <v>0</v>
       </c>
@@ -8727,15 +8382,6 @@
       <c r="H111" t="s">
         <v>1237</v>
       </c>
-      <c r="J111">
-        <v>49</v>
-      </c>
-      <c r="L111" t="s">
-        <v>1271</v>
-      </c>
-      <c r="M111" t="s">
-        <v>1340</v>
-      </c>
       <c r="Q111" t="b">
         <v>0</v>
       </c>
@@ -8765,9 +8411,6 @@
       <c r="H112" t="s">
         <v>1237</v>
       </c>
-      <c r="J112">
-        <v>9</v>
-      </c>
       <c r="Q112" t="b">
         <v>0</v>
       </c>
@@ -8797,15 +8440,6 @@
       <c r="H113" t="s">
         <v>1237</v>
       </c>
-      <c r="J113">
-        <v>119</v>
-      </c>
-      <c r="L113" t="s">
-        <v>1281</v>
-      </c>
-      <c r="M113" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q113" t="b">
         <v>0</v>
       </c>
@@ -8835,12 +8469,6 @@
       <c r="H114" t="s">
         <v>1237</v>
       </c>
-      <c r="L114" t="s">
-        <v>1282</v>
-      </c>
-      <c r="M114" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q114" t="b">
         <v>0</v>
       </c>
@@ -8877,7 +8505,7 @@
         <v>1240</v>
       </c>
       <c r="M115" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q115" t="b">
         <v>1</v>
@@ -8915,7 +8543,7 @@
         <v>1240</v>
       </c>
       <c r="M116" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q116" t="b">
         <v>1</v>
@@ -8953,7 +8581,7 @@
         <v>1240</v>
       </c>
       <c r="M117" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q117" t="b">
         <v>1</v>
@@ -8991,7 +8619,7 @@
         <v>1240</v>
       </c>
       <c r="M118" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q118" t="b">
         <v>1</v>
@@ -9029,7 +8657,7 @@
         <v>1240</v>
       </c>
       <c r="M119" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q119" t="b">
         <v>1</v>
@@ -9067,7 +8695,7 @@
         <v>1240</v>
       </c>
       <c r="M120" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q120" t="b">
         <v>1</v>
@@ -9108,7 +8736,7 @@
         <v>1210</v>
       </c>
       <c r="L121" t="s">
-        <v>1266</v>
+        <v>1260</v>
       </c>
       <c r="N121" s="1">
         <v>46100</v>
@@ -9152,7 +8780,7 @@
         <v>1240</v>
       </c>
       <c r="M122" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q122" t="b">
         <v>1</v>
@@ -9219,7 +8847,7 @@
         <v>1240</v>
       </c>
       <c r="M124" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q124" t="b">
         <v>1</v>
@@ -9257,7 +8885,7 @@
         <v>1246</v>
       </c>
       <c r="O125" t="s">
-        <v>1352</v>
+        <v>1320</v>
       </c>
       <c r="Q125" t="b">
         <v>1</v>
@@ -9288,15 +8916,6 @@
       <c r="H126" t="s">
         <v>1237</v>
       </c>
-      <c r="J126">
-        <v>28</v>
-      </c>
-      <c r="L126" t="s">
-        <v>1283</v>
-      </c>
-      <c r="M126" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q126" t="b">
         <v>0</v>
       </c>
@@ -9362,7 +8981,7 @@
         <v>1240</v>
       </c>
       <c r="M128" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q128" t="b">
         <v>1</v>
@@ -9400,7 +9019,7 @@
         <v>1239</v>
       </c>
       <c r="M129" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q129" t="b">
         <v>1</v>
@@ -9441,7 +9060,7 @@
         <v>1210</v>
       </c>
       <c r="L130" t="s">
-        <v>1284</v>
+        <v>1270</v>
       </c>
       <c r="N130" s="1">
         <v>45916</v>
@@ -9478,12 +9097,6 @@
       <c r="H131" t="s">
         <v>1237</v>
       </c>
-      <c r="L131" t="s">
-        <v>1285</v>
-      </c>
-      <c r="M131" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q131" t="b">
         <v>0</v>
       </c>
@@ -9523,7 +9136,7 @@
         <v>1211</v>
       </c>
       <c r="L132" t="s">
-        <v>1286</v>
+        <v>1271</v>
       </c>
       <c r="N132" s="1">
         <v>46014</v>
@@ -9596,7 +9209,7 @@
         <v>1239</v>
       </c>
       <c r="M134" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q134" t="b">
         <v>1</v>
@@ -9627,9 +9240,6 @@
       <c r="H135" t="s">
         <v>1237</v>
       </c>
-      <c r="J135">
-        <v>50</v>
-      </c>
       <c r="Q135" t="b">
         <v>0</v>
       </c>
@@ -9688,9 +9298,6 @@
       <c r="H137" t="s">
         <v>1237</v>
       </c>
-      <c r="J137">
-        <v>111</v>
-      </c>
       <c r="Q137" t="b">
         <v>0</v>
       </c>
@@ -9727,7 +9334,7 @@
         <v>1240</v>
       </c>
       <c r="M138" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q138" t="b">
         <v>1</v>
@@ -9787,12 +9394,6 @@
       <c r="H140" t="s">
         <v>1237</v>
       </c>
-      <c r="L140" t="s">
-        <v>1287</v>
-      </c>
-      <c r="M140" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q140" t="b">
         <v>0</v>
       </c>
@@ -9822,9 +9423,6 @@
       <c r="H141" t="s">
         <v>1237</v>
       </c>
-      <c r="J141">
-        <v>18</v>
-      </c>
       <c r="Q141" t="b">
         <v>0</v>
       </c>
@@ -9854,9 +9452,6 @@
       <c r="H142" t="s">
         <v>1237</v>
       </c>
-      <c r="J142">
-        <v>80</v>
-      </c>
       <c r="Q142" t="b">
         <v>0</v>
       </c>
@@ -9915,9 +9510,6 @@
       <c r="H144" t="s">
         <v>1237</v>
       </c>
-      <c r="J144">
-        <v>-87</v>
-      </c>
       <c r="Q144" t="b">
         <v>0</v>
       </c>
@@ -9947,15 +9539,6 @@
       <c r="H145" t="s">
         <v>1237</v>
       </c>
-      <c r="J145">
-        <v>-87</v>
-      </c>
-      <c r="L145" t="s">
-        <v>1288</v>
-      </c>
-      <c r="M145" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q145" t="b">
         <v>0</v>
       </c>
@@ -10014,12 +9597,6 @@
       <c r="H147" t="s">
         <v>1237</v>
       </c>
-      <c r="L147" t="s">
-        <v>1288</v>
-      </c>
-      <c r="M147" t="s">
-        <v>1338</v>
-      </c>
       <c r="Q147" t="b">
         <v>0</v>
       </c>
@@ -10056,7 +9633,7 @@
         <v>1240</v>
       </c>
       <c r="M148" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q148" t="b">
         <v>1</v>
@@ -10132,13 +9709,13 @@
         <v>1210</v>
       </c>
       <c r="L150" t="s">
-        <v>1270</v>
+        <v>1262</v>
       </c>
       <c r="N150" s="1">
         <v>46092</v>
       </c>
       <c r="P150" t="s">
-        <v>1359</v>
+        <v>1327</v>
       </c>
       <c r="Q150" t="b">
         <v>1</v>
@@ -10169,15 +9746,6 @@
       <c r="H151" t="s">
         <v>1237</v>
       </c>
-      <c r="J151">
-        <v>-15</v>
-      </c>
-      <c r="L151" t="s">
-        <v>1273</v>
-      </c>
-      <c r="M151" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q151" t="b">
         <v>0</v>
       </c>
@@ -10217,7 +9785,7 @@
         <v>1241</v>
       </c>
       <c r="L152" t="s">
-        <v>1271</v>
+        <v>1263</v>
       </c>
       <c r="N152" s="1">
         <v>46119</v>
@@ -10258,7 +9826,7 @@
         <v>1240</v>
       </c>
       <c r="M153" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="Q153" t="b">
         <v>1</v>
@@ -10289,12 +9857,6 @@
       <c r="H154" t="s">
         <v>1237</v>
       </c>
-      <c r="L154" t="s">
-        <v>1273</v>
-      </c>
-      <c r="M154" t="s">
-        <v>1339</v>
-      </c>
       <c r="Q154" t="b">
         <v>0</v>
       </c>
@@ -10366,7 +9928,7 @@
         <v>1240</v>
       </c>
       <c r="M156" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q156" t="b">
         <v>1</v>
@@ -10404,7 +9966,7 @@
         <v>1242</v>
       </c>
       <c r="M157" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q157" t="b">
         <v>1</v>
@@ -10445,7 +10007,7 @@
         <v>1213</v>
       </c>
       <c r="L158" t="s">
-        <v>1289</v>
+        <v>1272</v>
       </c>
       <c r="N158" s="1">
         <v>45946</v>
@@ -10486,7 +10048,7 @@
         <v>1240</v>
       </c>
       <c r="M159" t="s">
-        <v>1338</v>
+        <v>1306</v>
       </c>
       <c r="Q159" t="b">
         <v>1</v>
@@ -10524,7 +10086,7 @@
         <v>1240</v>
       </c>
       <c r="M160" t="s">
-        <v>1337</v>
+        <v>1305</v>
       </c>
       <c r="Q160" t="b">
         <v>1</v>
@@ -10565,13 +10127,13 @@
         <v>1210</v>
       </c>
       <c r="L161" t="s">
-        <v>1290</v>
+        <v>1273</v>
       </c>
       <c r="N161" s="1">
         <v>45953</v>
       </c>
       <c r="O161" t="s">
-        <v>1353</v>
+        <v>1321</v>
       </c>
       <c r="Q161" t="b">
         <v>1</v>
@@ -10612,7 +10174,7 @@
         <v>1213</v>
       </c>
       <c r="L162" t="s">
-        <v>1291</v>
+        <v>1274</v>
       </c>
       <c r="N162" s="1">
         <v>45940</v>
@@ -10656,7 +10218,7 @@
         <v>1213</v>
       </c>
       <c r="L163" t="s">
-        <v>1291</v>
+        <v>1274</v>
       </c>
       <c r="N163" s="1">
         <v>45940</v>
@@ -10729,10 +10291,10 @@
         <v>1240</v>
       </c>
       <c r="M165" t="s">
-        <v>1339</v>
+        <v>1307</v>
       </c>
       <c r="P165" t="s">
-        <v>1361</v>
+        <v>1329</v>
       </c>
       <c r="Q165" t="b">
        